<commit_message>
Update workforce capacity data for improved analytics
Updated the capacity_dashboard.xlsx file to enhance the accuracy of workforce capacity data within the analytics engine.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: debe8ea6-a4b7-4b45-bd4c-d101bf085400
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/debe8ea6-a4b7-4b45-bd4c-d101bf085400/PSmR3tL
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3300,13 +3300,13 @@
         <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="G2" t="str">
-        <v>50.17</v>
+        <v>-13.83</v>
       </c>
       <c r="H2" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="3">
@@ -3326,13 +3326,13 @@
         <v>9</v>
       </c>
       <c r="F3" t="str">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="G3" t="str">
-        <v>83.8</v>
+        <v>-14.2</v>
       </c>
       <c r="H3" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="4">
@@ -3352,13 +3352,13 @@
         <v>9</v>
       </c>
       <c r="F4" t="str">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="G4" t="str">
-        <v>79.47</v>
+        <v>-25.53</v>
       </c>
       <c r="H4" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="5">
@@ -3378,13 +3378,13 @@
         <v>9</v>
       </c>
       <c r="F5" t="str">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="G5" t="str">
-        <v>80.8</v>
+        <v>-16.2</v>
       </c>
       <c r="H5" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="6">
@@ -3404,10 +3404,10 @@
         <v>9</v>
       </c>
       <c r="F6" t="str">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="G6" t="str">
-        <v>72.13</v>
+        <v>13.13</v>
       </c>
       <c r="H6" t="str">
         <v>Sufficient</v>
@@ -3430,13 +3430,13 @@
         <v>9</v>
       </c>
       <c r="F7" t="str">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="G7" t="str">
-        <v>33.67</v>
+        <v>-10.33</v>
       </c>
       <c r="H7" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="8">
@@ -3456,10 +3456,10 @@
         <v>0</v>
       </c>
       <c r="F8" t="str">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="G8" t="str">
-        <v>47</v>
+        <v>7</v>
       </c>
       <c r="H8" t="str">
         <v>Sufficient</v>

</xml_diff>

<commit_message>
Improve data display by showing all available days
Update the dashboard to correctly display the full range of daily data, ensuring all seven days are visible and accurate.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: debe8ea6-a4b7-4b45-bd4c-d101bf085400
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/debe8ea6-a4b7-4b45-bd4c-d101bf085400/WNJCh19
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3268,7 +3268,7 @@
         <v>Net Capacity</v>
       </c>
       <c r="D1" t="str">
-        <v>Sickness</v>
+        <v>Unavailability</v>
       </c>
       <c r="E1" t="str">
         <v>Holidays</v>
@@ -3294,7 +3294,7 @@
         <v>50.17</v>
       </c>
       <c r="D2" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="E2" t="str">
         <v>0</v>
@@ -3320,7 +3320,7 @@
         <v>83.8</v>
       </c>
       <c r="D3" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E3" t="str">
         <v>9</v>
@@ -3346,7 +3346,7 @@
         <v>79.47</v>
       </c>
       <c r="D4" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E4" t="str">
         <v>9</v>
@@ -3398,7 +3398,7 @@
         <v>72.13</v>
       </c>
       <c r="D6" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6" t="str">
         <v>9</v>

</xml_diff>

<commit_message>
Improve data logging for capacity analysis debugging
Add detailed logging for date fields in guaranteed hours processing to aid in debugging time window issues.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ae21854f-56f0-4406-b430-4b525fbb8b36
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/ae21854f-56f0-4406-b430-4b525fbb8b36/LrepN0o
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3301,13 +3301,13 @@
         <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="G2" t="str">
-        <v>57</v>
+        <v>-12</v>
       </c>
       <c r="H2" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="3">
@@ -3327,10 +3327,10 @@
         <v>0</v>
       </c>
       <c r="F3" t="str">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="G3" t="str">
-        <v>70.5</v>
+        <v>2.5</v>
       </c>
       <c r="H3" t="str">
         <v>Sufficient</v>
@@ -3353,13 +3353,13 @@
         <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="G4" t="str">
-        <v>74</v>
+        <v>-8</v>
       </c>
       <c r="H4" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="5">
@@ -3379,10 +3379,10 @@
         <v>0</v>
       </c>
       <c r="F5" t="str">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="G5" t="str">
-        <v>86.66</v>
+        <v>15.66</v>
       </c>
       <c r="H5" t="str">
         <v>Sufficient</v>
@@ -3405,10 +3405,10 @@
         <v>12.43</v>
       </c>
       <c r="F6" t="str">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="G6" t="str">
-        <v>71.56</v>
+        <v>16.56</v>
       </c>
       <c r="H6" t="str">
         <v>Sufficient</v>
@@ -3431,13 +3431,13 @@
         <v>12.43</v>
       </c>
       <c r="F7" t="str">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="G7" t="str">
-        <v>30.17</v>
+        <v>-12.83</v>
       </c>
       <c r="H7" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="8">
@@ -3457,13 +3457,13 @@
         <v>3.43</v>
       </c>
       <c r="F8" t="str">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="G8" t="str">
-        <v>40.83</v>
+        <v>-0.17</v>
       </c>
       <c r="H8" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improve employee data processing for clearer capacity reporting
Refactor employee data aggregation in pipeline.ts to consolidate entries by employee name, calculate total unavailability hours, and accurately track the presence of 'Available' statuses, enhancing the accuracy of capacity dashboard calculations.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ae21854f-56f0-4406-b430-4b525fbb8b36
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/ae21854f-56f0-4406-b430-4b525fbb8b36/LrepN0o
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -447,7 +447,7 @@
         <v>Holiday</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G2" t="str">
         <v>9</v>
@@ -476,7 +476,7 @@
         <v>Holiday</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G3" t="str">
         <v>9</v>
@@ -505,7 +505,7 @@
         <v>Holiday</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>09:15-17:00</v>
       </c>
       <c r="G4" t="str">
         <v>3.43</v>
@@ -534,7 +534,7 @@
         <v>Holiday</v>
       </c>
       <c r="F5" t="str">
-        <v/>
+        <v>09:15-17:00</v>
       </c>
       <c r="G5" t="str">
         <v>3.43</v>
@@ -563,7 +563,7 @@
         <v>Holiday</v>
       </c>
       <c r="F6" t="str">
-        <v/>
+        <v>09:15-17:00</v>
       </c>
       <c r="G6" t="str">
         <v>3.43</v>
@@ -592,7 +592,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F7" t="str">
-        <v/>
+        <v>08:00-15:00</v>
       </c>
       <c r="G7" t="str">
         <v>7</v>
@@ -622,7 +622,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>10:30-12:30</v>
       </c>
       <c r="G8" t="str">
         <v>2</v>
@@ -651,7 +651,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F9" t="str">
-        <v/>
+        <v>10:30-12:30</v>
       </c>
       <c r="G9" t="str">
         <v>2</v>
@@ -681,7 +681,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F10" t="str">
-        <v/>
+        <v>10:30-12:30</v>
       </c>
       <c r="G10" t="str">
         <v>2</v>
@@ -711,7 +711,7 @@
         <v>Pre-Agreed Appointment</v>
       </c>
       <c r="F11" t="str">
-        <v/>
+        <v>10:20-12:50</v>
       </c>
       <c r="G11" t="str">
         <v>2.5</v>
@@ -740,7 +740,7 @@
         <v>Available</v>
       </c>
       <c r="F12" t="str">
-        <v/>
+        <v>10:30-14:00</v>
       </c>
       <c r="G12" t="str">
         <v>3.2</v>
@@ -769,7 +769,7 @@
         <v>Available</v>
       </c>
       <c r="F13" t="str">
-        <v/>
+        <v>09:15-15:15</v>
       </c>
       <c r="G13" t="str">
         <v>3.2</v>
@@ -798,7 +798,7 @@
         <v>Available</v>
       </c>
       <c r="F14" t="str">
-        <v/>
+        <v>09:15-15:15</v>
       </c>
       <c r="G14" t="str">
         <v>3.2</v>
@@ -827,7 +827,7 @@
         <v>Available</v>
       </c>
       <c r="F15" t="str">
-        <v/>
+        <v>09:15-15:15</v>
       </c>
       <c r="G15" t="str">
         <v>3.2</v>
@@ -856,7 +856,7 @@
         <v>Available</v>
       </c>
       <c r="F16" t="str">
-        <v/>
+        <v>10:30-14:00</v>
       </c>
       <c r="G16" t="str">
         <v>3.2</v>
@@ -885,7 +885,7 @@
         <v>Available</v>
       </c>
       <c r="F17" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G17" t="str">
         <v>0.17</v>
@@ -914,7 +914,7 @@
         <v>Available</v>
       </c>
       <c r="F18" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G18" t="str">
         <v>2.67</v>
@@ -943,7 +943,7 @@
         <v>Available</v>
       </c>
       <c r="F19" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G19" t="str">
         <v>2.67</v>
@@ -972,7 +972,7 @@
         <v>Available</v>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G20" t="str">
         <v>2.67</v>
@@ -1001,7 +1001,7 @@
         <v>Available</v>
       </c>
       <c r="F21" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G21" t="str">
         <v>2.67</v>
@@ -1030,7 +1030,7 @@
         <v>Available</v>
       </c>
       <c r="F22" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G22" t="str">
         <v>2.67</v>
@@ -1059,7 +1059,7 @@
         <v>Available</v>
       </c>
       <c r="F23" t="str">
-        <v/>
+        <v>08:00-15:15</v>
       </c>
       <c r="G23" t="str">
         <v>7.5</v>
@@ -1088,7 +1088,7 @@
         <v>Available</v>
       </c>
       <c r="F24" t="str">
-        <v/>
+        <v>08:00-15:15</v>
       </c>
       <c r="G24" t="str">
         <v>0.5</v>
@@ -1117,7 +1117,7 @@
         <v>Available</v>
       </c>
       <c r="F25" t="str">
-        <v/>
+        <v>08:30-21:30</v>
       </c>
       <c r="G25" t="str">
         <v>7.5</v>
@@ -1146,7 +1146,7 @@
         <v>Available</v>
       </c>
       <c r="F26" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G26" t="str">
         <v>7.5</v>
@@ -1175,7 +1175,7 @@
         <v>Available</v>
       </c>
       <c r="F27" t="str">
-        <v/>
+        <v>08:30-14:30</v>
       </c>
       <c r="G27" t="str">
         <v>7.5</v>
@@ -1205,7 +1205,7 @@
         <v>Available</v>
       </c>
       <c r="F28" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G28" t="str">
         <v>4</v>
@@ -1234,7 +1234,7 @@
         <v>Available</v>
       </c>
       <c r="F29" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G29" t="str">
         <v>4</v>
@@ -1263,7 +1263,7 @@
         <v>Available</v>
       </c>
       <c r="F30" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G30" t="str">
         <v>4</v>
@@ -1292,7 +1292,7 @@
         <v>Available</v>
       </c>
       <c r="F31" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G31" t="str">
         <v>4</v>
@@ -1321,7 +1321,7 @@
         <v>Available</v>
       </c>
       <c r="F32" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G32" t="str">
         <v>4</v>
@@ -1350,7 +1350,7 @@
         <v>Available</v>
       </c>
       <c r="F33" t="str">
-        <v/>
+        <v>09:15-14:45</v>
       </c>
       <c r="G33" t="str">
         <v>2.8</v>
@@ -1379,7 +1379,7 @@
         <v>Available</v>
       </c>
       <c r="F34" t="str">
-        <v/>
+        <v>09:15-11:30</v>
       </c>
       <c r="G34" t="str">
         <v>2.8</v>
@@ -1408,7 +1408,7 @@
         <v>Available</v>
       </c>
       <c r="F35" t="str">
-        <v/>
+        <v>09:15-14:45</v>
       </c>
       <c r="G35" t="str">
         <v>2.8</v>
@@ -1437,7 +1437,7 @@
         <v>Available</v>
       </c>
       <c r="F36" t="str">
-        <v/>
+        <v>09:15-11:30</v>
       </c>
       <c r="G36" t="str">
         <v>2.8</v>
@@ -1466,7 +1466,7 @@
         <v>Available</v>
       </c>
       <c r="F37" t="str">
-        <v/>
+        <v>09:15-10:15</v>
       </c>
       <c r="G37" t="str">
         <v>2.8</v>
@@ -1495,7 +1495,7 @@
         <v>Available</v>
       </c>
       <c r="F38" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G38" t="str">
         <v>10</v>
@@ -1524,7 +1524,7 @@
         <v>Available</v>
       </c>
       <c r="F39" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G39" t="str">
         <v>10</v>
@@ -1553,7 +1553,7 @@
         <v>Available</v>
       </c>
       <c r="F40" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G40" t="str">
         <v>7.5</v>
@@ -1582,7 +1582,7 @@
         <v>Available</v>
       </c>
       <c r="F41" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G41" t="str">
         <v>7.5</v>
@@ -1611,7 +1611,7 @@
         <v>Available</v>
       </c>
       <c r="F42" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G42" t="str">
         <v>7.5</v>
@@ -1640,7 +1640,7 @@
         <v>Available</v>
       </c>
       <c r="F43" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G43" t="str">
         <v>7.5</v>
@@ -1669,7 +1669,7 @@
         <v>Available</v>
       </c>
       <c r="F44" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G44" t="str">
         <v>5.33</v>
@@ -1698,7 +1698,7 @@
         <v>Available</v>
       </c>
       <c r="F45" t="str">
-        <v/>
+        <v>08:00-17:45</v>
       </c>
       <c r="G45" t="str">
         <v>5.33</v>
@@ -1727,7 +1727,7 @@
         <v>Available</v>
       </c>
       <c r="F46" t="str">
-        <v/>
+        <v>08:00-17:45</v>
       </c>
       <c r="G46" t="str">
         <v>5.33</v>
@@ -1756,7 +1756,7 @@
         <v>Available</v>
       </c>
       <c r="F47" t="str">
-        <v/>
+        <v>08:00-15:15</v>
       </c>
       <c r="G47" t="str">
         <v>4</v>
@@ -1785,7 +1785,7 @@
         <v>Available</v>
       </c>
       <c r="F48" t="str">
-        <v/>
+        <v>08:00-15:15</v>
       </c>
       <c r="G48" t="str">
         <v>4</v>
@@ -1814,7 +1814,7 @@
         <v>Available</v>
       </c>
       <c r="F49" t="str">
-        <v/>
+        <v>08:00-15:15</v>
       </c>
       <c r="G49" t="str">
         <v>4</v>
@@ -1843,7 +1843,7 @@
         <v>Available</v>
       </c>
       <c r="F50" t="str">
-        <v/>
+        <v>08:00-15:15</v>
       </c>
       <c r="G50" t="str">
         <v>4</v>
@@ -1872,7 +1872,7 @@
         <v>Available</v>
       </c>
       <c r="F51" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G51" t="str">
         <v>10</v>
@@ -1901,7 +1901,7 @@
         <v>Available</v>
       </c>
       <c r="F52" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G52" t="str">
         <v>10</v>
@@ -1930,7 +1930,7 @@
         <v>Available</v>
       </c>
       <c r="F53" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G53" t="str">
         <v>9</v>
@@ -1959,7 +1959,7 @@
         <v>Available</v>
       </c>
       <c r="F54" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G54" t="str">
         <v>9</v>
@@ -1988,7 +1988,7 @@
         <v>Available</v>
       </c>
       <c r="F55" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G55" t="str">
         <v>9</v>
@@ -2017,7 +2017,7 @@
         <v>Available</v>
       </c>
       <c r="F56" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G56" t="str">
         <v>0</v>
@@ -2046,7 +2046,7 @@
         <v>Available</v>
       </c>
       <c r="F57" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G57" t="str">
         <v>0</v>
@@ -2075,7 +2075,7 @@
         <v>Available</v>
       </c>
       <c r="F58" t="str">
-        <v/>
+        <v>16:45-21:30</v>
       </c>
       <c r="G58" t="str">
         <v>7.5</v>
@@ -2104,7 +2104,7 @@
         <v>Available</v>
       </c>
       <c r="F59" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G59" t="str">
         <v>7.5</v>
@@ -2133,7 +2133,7 @@
         <v>Available</v>
       </c>
       <c r="F60" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G60" t="str">
         <v>7.5</v>
@@ -2162,7 +2162,7 @@
         <v>Available</v>
       </c>
       <c r="F61" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G61" t="str">
         <v>7.5</v>
@@ -2191,7 +2191,7 @@
         <v>Available</v>
       </c>
       <c r="F62" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G62" t="str">
         <v>7.5</v>
@@ -2220,7 +2220,7 @@
         <v>Available</v>
       </c>
       <c r="F63" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G63" t="str">
         <v>7.5</v>
@@ -2249,7 +2249,7 @@
         <v>Available</v>
       </c>
       <c r="F64" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G64" t="str">
         <v>7.5</v>
@@ -2278,7 +2278,7 @@
         <v>Available</v>
       </c>
       <c r="F65" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G65" t="str">
         <v>7.5</v>
@@ -2307,7 +2307,7 @@
         <v>Available</v>
       </c>
       <c r="F66" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G66" t="str">
         <v>6</v>
@@ -2336,7 +2336,7 @@
         <v>Available</v>
       </c>
       <c r="F67" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G67" t="str">
         <v>6</v>
@@ -2365,7 +2365,7 @@
         <v>Available</v>
       </c>
       <c r="F68" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G68" t="str">
         <v>6</v>
@@ -2394,7 +2394,7 @@
         <v>Available</v>
       </c>
       <c r="F69" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G69" t="str">
         <v>6</v>
@@ -2423,7 +2423,7 @@
         <v>Available</v>
       </c>
       <c r="F70" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G70" t="str">
         <v>6</v>
@@ -2452,7 +2452,7 @@
         <v>Available</v>
       </c>
       <c r="F71" t="str">
-        <v/>
+        <v>09:15-15:00</v>
       </c>
       <c r="G71" t="str">
         <v>3.2</v>
@@ -2481,7 +2481,7 @@
         <v>Available</v>
       </c>
       <c r="F72" t="str">
-        <v/>
+        <v>09:15-15:00</v>
       </c>
       <c r="G72" t="str">
         <v>3.2</v>
@@ -2510,7 +2510,7 @@
         <v>Available</v>
       </c>
       <c r="F73" t="str">
-        <v/>
+        <v>09:15-15:00</v>
       </c>
       <c r="G73" t="str">
         <v>3.2</v>
@@ -2539,7 +2539,7 @@
         <v>Available</v>
       </c>
       <c r="F74" t="str">
-        <v/>
+        <v>09:15-15:00</v>
       </c>
       <c r="G74" t="str">
         <v>3.2</v>
@@ -2568,7 +2568,7 @@
         <v>Available</v>
       </c>
       <c r="F75" t="str">
-        <v/>
+        <v>09:15-15:00</v>
       </c>
       <c r="G75" t="str">
         <v>3.2</v>
@@ -2597,7 +2597,7 @@
         <v>Available</v>
       </c>
       <c r="F76" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G76" t="str">
         <v>6</v>
@@ -2626,7 +2626,7 @@
         <v>Available</v>
       </c>
       <c r="F77" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G77" t="str">
         <v>6</v>
@@ -2655,7 +2655,7 @@
         <v>Available</v>
       </c>
       <c r="F78" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G78" t="str">
         <v>6</v>
@@ -2684,7 +2684,7 @@
         <v>Available</v>
       </c>
       <c r="F79" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G79" t="str">
         <v>6</v>
@@ -2713,7 +2713,7 @@
         <v>Available</v>
       </c>
       <c r="F80" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G80" t="str">
         <v>6</v>
@@ -2742,7 +2742,7 @@
         <v>Available</v>
       </c>
       <c r="F81" t="str">
-        <v/>
+        <v>08:00-17:15</v>
       </c>
       <c r="G81" t="str">
         <v>5.33</v>
@@ -2771,7 +2771,7 @@
         <v>Available</v>
       </c>
       <c r="F82" t="str">
-        <v/>
+        <v>08:00-13:00</v>
       </c>
       <c r="G82" t="str">
         <v>5.33</v>
@@ -2800,7 +2800,7 @@
         <v>Available</v>
       </c>
       <c r="F83" t="str">
-        <v/>
+        <v>08:00-18:00</v>
       </c>
       <c r="G83" t="str">
         <v>5.33</v>
@@ -2829,7 +2829,7 @@
         <v>Available</v>
       </c>
       <c r="F84" t="str">
-        <v/>
+        <v>09:15-21:30</v>
       </c>
       <c r="G84" t="str">
         <v>3.2</v>
@@ -2858,7 +2858,7 @@
         <v>Available</v>
       </c>
       <c r="F85" t="str">
-        <v/>
+        <v>16:45-21:30</v>
       </c>
       <c r="G85" t="str">
         <v>3.2</v>
@@ -2887,7 +2887,7 @@
         <v>Available</v>
       </c>
       <c r="F86" t="str">
-        <v/>
+        <v>16:45-21:30</v>
       </c>
       <c r="G86" t="str">
         <v>3.2</v>
@@ -2916,7 +2916,7 @@
         <v>Available</v>
       </c>
       <c r="F87" t="str">
-        <v/>
+        <v>16:45-21:30</v>
       </c>
       <c r="G87" t="str">
         <v>3.2</v>
@@ -2945,7 +2945,7 @@
         <v>Available</v>
       </c>
       <c r="F88" t="str">
-        <v/>
+        <v>16:45-21:30</v>
       </c>
       <c r="G88" t="str">
         <v>3.2</v>
@@ -2974,7 +2974,7 @@
         <v>Available</v>
       </c>
       <c r="F89" t="str">
-        <v/>
+        <v>09:15-10:15</v>
       </c>
       <c r="G89" t="str">
         <v>3.43</v>
@@ -3003,7 +3003,7 @@
         <v>Available</v>
       </c>
       <c r="F90" t="str">
-        <v/>
+        <v>09:15-16:15</v>
       </c>
       <c r="G90" t="str">
         <v>1.43</v>
@@ -3032,7 +3032,7 @@
         <v>Available</v>
       </c>
       <c r="F91" t="str">
-        <v/>
+        <v>09:15-16:30</v>
       </c>
       <c r="G91" t="str">
         <v>1.43</v>
@@ -3061,7 +3061,7 @@
         <v>Available</v>
       </c>
       <c r="F92" t="str">
-        <v/>
+        <v>09:15-16:15</v>
       </c>
       <c r="G92" t="str">
         <v>3.43</v>
@@ -3090,7 +3090,7 @@
         <v>Available</v>
       </c>
       <c r="F93" t="str">
-        <v/>
+        <v>09:15-17:00</v>
       </c>
       <c r="G93" t="str">
         <v>0</v>
@@ -3119,7 +3119,7 @@
         <v>Available</v>
       </c>
       <c r="F94" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G94" t="str">
         <v>6</v>
@@ -3148,7 +3148,7 @@
         <v>Available</v>
       </c>
       <c r="F95" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G95" t="str">
         <v>6</v>
@@ -3177,7 +3177,7 @@
         <v>Available</v>
       </c>
       <c r="F96" t="str">
-        <v/>
+        <v>09:15-15:00</v>
       </c>
       <c r="G96" t="str">
         <v>6</v>
@@ -3206,7 +3206,7 @@
         <v>Available</v>
       </c>
       <c r="F97" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G97" t="str">
         <v>6</v>
@@ -3235,7 +3235,7 @@
         <v>Available</v>
       </c>
       <c r="F98" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="G98" t="str">
         <v>6</v>
@@ -3514,7 +3514,7 @@
         <v>Available</v>
       </c>
       <c r="D2" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E2" t="str">
         <v>7.5</v>
@@ -3540,7 +3540,7 @@
         <v>Available</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E3" t="str">
         <v>4</v>
@@ -3566,7 +3566,7 @@
         <v>Available</v>
       </c>
       <c r="D4" t="str">
-        <v/>
+        <v>08:00-17:45</v>
       </c>
       <c r="E4" t="str">
         <v>5.33</v>
@@ -3592,7 +3592,7 @@
         <v>Holiday</v>
       </c>
       <c r="D5" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E5" t="str">
         <v>9</v>
@@ -3618,7 +3618,7 @@
         <v>Available</v>
       </c>
       <c r="D6" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E6" t="str">
         <v>9</v>
@@ -3644,7 +3644,7 @@
         <v>Available</v>
       </c>
       <c r="D7" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E7" t="str">
         <v>10</v>
@@ -3670,7 +3670,7 @@
         <v>Available</v>
       </c>
       <c r="D8" t="str">
-        <v/>
+        <v>10:30-14:00</v>
       </c>
       <c r="E8" t="str">
         <v>3.2</v>
@@ -3696,7 +3696,7 @@
         <v>Available</v>
       </c>
       <c r="D9" t="str">
-        <v/>
+        <v>09:15-10:15</v>
       </c>
       <c r="E9" t="str">
         <v>2.8</v>
@@ -3722,7 +3722,7 @@
         <v>Available</v>
       </c>
       <c r="D10" t="str">
-        <v/>
+        <v>08:30-14:30</v>
       </c>
       <c r="E10" t="str">
         <v>7.5</v>
@@ -3749,7 +3749,7 @@
         <v>Available</v>
       </c>
       <c r="D11" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E11" t="str">
         <v>6</v>
@@ -3775,7 +3775,7 @@
         <v>Available</v>
       </c>
       <c r="D12" t="str">
-        <v/>
+        <v>09:15-15:00</v>
       </c>
       <c r="E12" t="str">
         <v>3.2</v>
@@ -3801,7 +3801,7 @@
         <v>Holiday</v>
       </c>
       <c r="D13" t="str">
-        <v/>
+        <v>09:15-17:00</v>
       </c>
       <c r="E13" t="str">
         <v>3.43</v>
@@ -3827,7 +3827,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D14" t="str">
-        <v/>
+        <v>10:30-12:30</v>
       </c>
       <c r="E14" t="str">
         <v>3.43</v>
@@ -3854,7 +3854,7 @@
         <v>Available</v>
       </c>
       <c r="D15" t="str">
-        <v/>
+        <v>09:15-17:00</v>
       </c>
       <c r="E15" t="str">
         <v>3.43</v>
@@ -3880,7 +3880,7 @@
         <v>Available</v>
       </c>
       <c r="D16" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E16" t="str">
         <v>7.5</v>
@@ -3906,7 +3906,7 @@
         <v>Available</v>
       </c>
       <c r="D17" t="str">
-        <v/>
+        <v>16:45-21:30</v>
       </c>
       <c r="E17" t="str">
         <v>3.2</v>
@@ -3932,7 +3932,7 @@
         <v>Available</v>
       </c>
       <c r="D18" t="str">
-        <v/>
+        <v>08:00-13:00</v>
       </c>
       <c r="E18" t="str">
         <v>5.33</v>
@@ -3958,7 +3958,7 @@
         <v>Available</v>
       </c>
       <c r="D19" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E19" t="str">
         <v>6</v>
@@ -3984,7 +3984,7 @@
         <v>Available</v>
       </c>
       <c r="D20" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E20" t="str">
         <v>7.5</v>
@@ -4010,7 +4010,7 @@
         <v>Holiday</v>
       </c>
       <c r="D21" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E21" t="str">
         <v>9</v>
@@ -4036,7 +4036,7 @@
         <v>Available</v>
       </c>
       <c r="D22" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E22" t="str">
         <v>9</v>
@@ -4062,7 +4062,7 @@
         <v>Available</v>
       </c>
       <c r="D23" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E23" t="str">
         <v>6</v>
@@ -4088,7 +4088,7 @@
         <v>Holiday</v>
       </c>
       <c r="D24" t="str">
-        <v/>
+        <v>09:15-17:00</v>
       </c>
       <c r="E24" t="str">
         <v>3.43</v>
@@ -4114,7 +4114,7 @@
         <v>Available</v>
       </c>
       <c r="D25" t="str">
-        <v/>
+        <v>08:00-15:15</v>
       </c>
       <c r="E25" t="str">
         <v>4</v>
@@ -4140,7 +4140,7 @@
         <v>Available</v>
       </c>
       <c r="D26" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E26" t="str">
         <v>2.67</v>
@@ -4166,7 +4166,7 @@
         <v>Available</v>
       </c>
       <c r="D27" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E27" t="str">
         <v>10</v>
@@ -4192,7 +4192,7 @@
         <v>Available</v>
       </c>
       <c r="D28" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E28" t="str">
         <v>7.5</v>
@@ -4218,7 +4218,7 @@
         <v>Available</v>
       </c>
       <c r="D29" t="str">
-        <v/>
+        <v>08:00-17:45</v>
       </c>
       <c r="E29" t="str">
         <v>5.33</v>
@@ -4244,7 +4244,7 @@
         <v>Available</v>
       </c>
       <c r="D30" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E30" t="str">
         <v>6</v>
@@ -4270,7 +4270,7 @@
         <v>Holiday</v>
       </c>
       <c r="D31" t="str">
-        <v/>
+        <v>09:15-17:00</v>
       </c>
       <c r="E31" t="str">
         <v>3.43</v>
@@ -4296,7 +4296,7 @@
         <v>Available</v>
       </c>
       <c r="D32" t="str">
-        <v/>
+        <v>08:00-15:15</v>
       </c>
       <c r="E32" t="str">
         <v>4</v>
@@ -4322,7 +4322,7 @@
         <v>Available</v>
       </c>
       <c r="D33" t="str">
-        <v/>
+        <v>08:00-18:00</v>
       </c>
       <c r="E33" t="str">
         <v>5.33</v>
@@ -4348,7 +4348,7 @@
         <v>Available</v>
       </c>
       <c r="D34" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E34" t="str">
         <v>2.67</v>
@@ -4374,7 +4374,7 @@
         <v>Available</v>
       </c>
       <c r="D35" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E35" t="str">
         <v>10</v>
@@ -4400,7 +4400,7 @@
         <v>Available</v>
       </c>
       <c r="D36" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E36" t="str">
         <v>7.5</v>
@@ -4426,7 +4426,7 @@
         <v>Available</v>
       </c>
       <c r="D37" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E37" t="str">
         <v>4</v>
@@ -4452,7 +4452,7 @@
         <v>Available</v>
       </c>
       <c r="D38" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E38" t="str">
         <v>7.5</v>
@@ -4478,7 +4478,7 @@
         <v>Available</v>
       </c>
       <c r="D39" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E39" t="str">
         <v>9</v>
@@ -4504,7 +4504,7 @@
         <v>Available</v>
       </c>
       <c r="D40" t="str">
-        <v/>
+        <v>09:15-15:15</v>
       </c>
       <c r="E40" t="str">
         <v>3.2</v>
@@ -4530,7 +4530,7 @@
         <v>Available</v>
       </c>
       <c r="D41" t="str">
-        <v/>
+        <v>09:15-11:30</v>
       </c>
       <c r="E41" t="str">
         <v>2.8</v>
@@ -4556,7 +4556,7 @@
         <v>Available</v>
       </c>
       <c r="D42" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E42" t="str">
         <v>6</v>
@@ -4582,7 +4582,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D43" t="str">
-        <v/>
+        <v>08:00-15:00</v>
       </c>
       <c r="E43" t="str">
         <v>7.5</v>
@@ -4609,7 +4609,7 @@
         <v>Available</v>
       </c>
       <c r="D44" t="str">
-        <v/>
+        <v>08:00-15:15</v>
       </c>
       <c r="E44" t="str">
         <v>7.5</v>
@@ -4635,7 +4635,7 @@
         <v>Available</v>
       </c>
       <c r="D45" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E45" t="str">
         <v>6</v>
@@ -4661,7 +4661,7 @@
         <v>Available</v>
       </c>
       <c r="D46" t="str">
-        <v/>
+        <v>09:15-15:00</v>
       </c>
       <c r="E46" t="str">
         <v>3.2</v>
@@ -4687,7 +4687,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D47" t="str">
-        <v/>
+        <v>10:30-12:30</v>
       </c>
       <c r="E47" t="str">
         <v>3.43</v>
@@ -4713,7 +4713,7 @@
         <v>Available</v>
       </c>
       <c r="D48" t="str">
-        <v/>
+        <v>09:15-16:15</v>
       </c>
       <c r="E48" t="str">
         <v>3.43</v>
@@ -4739,7 +4739,7 @@
         <v>Available</v>
       </c>
       <c r="D49" t="str">
-        <v/>
+        <v>16:45-21:30</v>
       </c>
       <c r="E49" t="str">
         <v>7.5</v>
@@ -4765,7 +4765,7 @@
         <v>Available</v>
       </c>
       <c r="D50" t="str">
-        <v/>
+        <v>16:45-21:30</v>
       </c>
       <c r="E50" t="str">
         <v>3.2</v>
@@ -4791,7 +4791,7 @@
         <v>Available</v>
       </c>
       <c r="D51" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E51" t="str">
         <v>2.67</v>
@@ -4817,7 +4817,7 @@
         <v>Available</v>
       </c>
       <c r="D52" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E52" t="str">
         <v>6</v>
@@ -4843,7 +4843,7 @@
         <v>Available</v>
       </c>
       <c r="D53" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E53" t="str">
         <v>7.5</v>
@@ -4869,7 +4869,7 @@
         <v>Available</v>
       </c>
       <c r="D54" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E54" t="str">
         <v>4</v>
@@ -4895,7 +4895,7 @@
         <v>Available</v>
       </c>
       <c r="D55" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E55" t="str">
         <v>9</v>
@@ -4921,7 +4921,7 @@
         <v>Available</v>
       </c>
       <c r="D56" t="str">
-        <v/>
+        <v>09:15-15:15</v>
       </c>
       <c r="E56" t="str">
         <v>3.2</v>
@@ -4947,7 +4947,7 @@
         <v>Available</v>
       </c>
       <c r="D57" t="str">
-        <v/>
+        <v>09:15-14:45</v>
       </c>
       <c r="E57" t="str">
         <v>2.8</v>
@@ -4973,7 +4973,7 @@
         <v>Available</v>
       </c>
       <c r="D58" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E58" t="str">
         <v>6</v>
@@ -4999,7 +4999,7 @@
         <v>Available</v>
       </c>
       <c r="D59" t="str">
-        <v/>
+        <v>08:30-21:30</v>
       </c>
       <c r="E59" t="str">
         <v>7.5</v>
@@ -5025,7 +5025,7 @@
         <v>Available</v>
       </c>
       <c r="D60" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E60" t="str">
         <v>6</v>
@@ -5051,7 +5051,7 @@
         <v>Available</v>
       </c>
       <c r="D61" t="str">
-        <v/>
+        <v>09:15-15:00</v>
       </c>
       <c r="E61" t="str">
         <v>3.2</v>
@@ -5077,7 +5077,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D62" t="str">
-        <v/>
+        <v>10:30-12:30</v>
       </c>
       <c r="E62" t="str">
         <v>3.43</v>
@@ -5104,7 +5104,7 @@
         <v>Available</v>
       </c>
       <c r="D63" t="str">
-        <v/>
+        <v>09:15-16:30</v>
       </c>
       <c r="E63" t="str">
         <v>3.43</v>
@@ -5130,7 +5130,7 @@
         <v>Available</v>
       </c>
       <c r="D64" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E64" t="str">
         <v>7.5</v>
@@ -5156,7 +5156,7 @@
         <v>Available</v>
       </c>
       <c r="D65" t="str">
-        <v/>
+        <v>08:00-15:15</v>
       </c>
       <c r="E65" t="str">
         <v>4</v>
@@ -5182,7 +5182,7 @@
         <v>Available</v>
       </c>
       <c r="D66" t="str">
-        <v/>
+        <v>16:45-21:30</v>
       </c>
       <c r="E66" t="str">
         <v>3.2</v>
@@ -5208,7 +5208,7 @@
         <v>Available</v>
       </c>
       <c r="D67" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E67" t="str">
         <v>2.67</v>
@@ -5234,7 +5234,7 @@
         <v>Available</v>
       </c>
       <c r="D68" t="str">
-        <v/>
+        <v>09:15-15:00</v>
       </c>
       <c r="E68" t="str">
         <v>6</v>
@@ -5260,7 +5260,7 @@
         <v>Available</v>
       </c>
       <c r="D69" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E69" t="str">
         <v>4</v>
@@ -5286,7 +5286,7 @@
         <v>Available</v>
       </c>
       <c r="D70" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E70" t="str">
         <v>7.5</v>
@@ -5312,7 +5312,7 @@
         <v>Available</v>
       </c>
       <c r="D71" t="str">
-        <v/>
+        <v>10:30-14:00</v>
       </c>
       <c r="E71" t="str">
         <v>3.2</v>
@@ -5338,7 +5338,7 @@
         <v>Available</v>
       </c>
       <c r="D72" t="str">
-        <v/>
+        <v>09:15-14:45</v>
       </c>
       <c r="E72" t="str">
         <v>2.8</v>
@@ -5364,7 +5364,7 @@
         <v>Available</v>
       </c>
       <c r="D73" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E73" t="str">
         <v>6</v>
@@ -5390,7 +5390,7 @@
         <v>Available</v>
       </c>
       <c r="D74" t="str">
-        <v/>
+        <v>08:00-15:15</v>
       </c>
       <c r="E74" t="str">
         <v>7.5</v>
@@ -5416,7 +5416,7 @@
         <v>Available</v>
       </c>
       <c r="D75" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E75" t="str">
         <v>6</v>
@@ -5442,7 +5442,7 @@
         <v>Available</v>
       </c>
       <c r="D76" t="str">
-        <v/>
+        <v>09:15-15:00</v>
       </c>
       <c r="E76" t="str">
         <v>3.2</v>
@@ -5468,7 +5468,7 @@
         <v>Available</v>
       </c>
       <c r="D77" t="str">
-        <v/>
+        <v>09:15-10:15</v>
       </c>
       <c r="E77" t="str">
         <v>3.43</v>
@@ -5494,7 +5494,7 @@
         <v>Available</v>
       </c>
       <c r="D78" t="str">
-        <v/>
+        <v>08:00-15:15</v>
       </c>
       <c r="E78" t="str">
         <v>4</v>
@@ -5520,7 +5520,7 @@
         <v>Available</v>
       </c>
       <c r="D79" t="str">
-        <v/>
+        <v>09:15-21:30</v>
       </c>
       <c r="E79" t="str">
         <v>3.2</v>
@@ -5546,7 +5546,7 @@
         <v>Pre-Agreed Appointment</v>
       </c>
       <c r="D80" t="str">
-        <v/>
+        <v>10:20-12:50</v>
       </c>
       <c r="E80" t="str">
         <v>2.67</v>
@@ -5572,7 +5572,7 @@
         <v>Available</v>
       </c>
       <c r="D81" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E81" t="str">
         <v>2.67</v>
@@ -5598,7 +5598,7 @@
         <v>Available</v>
       </c>
       <c r="D82" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E82" t="str">
         <v>6</v>
@@ -5624,7 +5624,7 @@
         <v>Available</v>
       </c>
       <c r="D83" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E83" t="str">
         <v>7.5</v>
@@ -5650,7 +5650,7 @@
         <v>Available</v>
       </c>
       <c r="D84" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E84" t="str">
         <v>4</v>
@@ -5676,7 +5676,7 @@
         <v>Available</v>
       </c>
       <c r="D85" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E85" t="str">
         <v>5.33</v>
@@ -5702,7 +5702,7 @@
         <v>Available</v>
       </c>
       <c r="D86" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E86" t="str">
         <v>9</v>
@@ -5728,7 +5728,7 @@
         <v>Available</v>
       </c>
       <c r="D87" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E87" t="str">
         <v>10</v>
@@ -5754,7 +5754,7 @@
         <v>Available</v>
       </c>
       <c r="D88" t="str">
-        <v/>
+        <v>09:15-15:15</v>
       </c>
       <c r="E88" t="str">
         <v>3.2</v>
@@ -5780,7 +5780,7 @@
         <v>Available</v>
       </c>
       <c r="D89" t="str">
-        <v/>
+        <v>09:15-11:30</v>
       </c>
       <c r="E89" t="str">
         <v>2.8</v>
@@ -5806,7 +5806,7 @@
         <v>Available</v>
       </c>
       <c r="D90" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E90" t="str">
         <v>6</v>
@@ -5832,7 +5832,7 @@
         <v>Available</v>
       </c>
       <c r="D91" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E91" t="str">
         <v>7.5</v>
@@ -5858,7 +5858,7 @@
         <v>Available</v>
       </c>
       <c r="D92" t="str">
-        <v/>
+        <v>09:15-15:00</v>
       </c>
       <c r="E92" t="str">
         <v>3.2</v>
@@ -5884,7 +5884,7 @@
         <v>Available</v>
       </c>
       <c r="D93" t="str">
-        <v/>
+        <v>09:15-16:15</v>
       </c>
       <c r="E93" t="str">
         <v>3.43</v>
@@ -5910,7 +5910,7 @@
         <v>Available</v>
       </c>
       <c r="D94" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E94" t="str">
         <v>7.5</v>
@@ -5936,7 +5936,7 @@
         <v>Available</v>
       </c>
       <c r="D95" t="str">
-        <v/>
+        <v>16:45-21:30</v>
       </c>
       <c r="E95" t="str">
         <v>3.2</v>
@@ -5962,7 +5962,7 @@
         <v>Available</v>
       </c>
       <c r="D96" t="str">
-        <v/>
+        <v>08:00-17:15</v>
       </c>
       <c r="E96" t="str">
         <v>5.33</v>
@@ -5988,7 +5988,7 @@
         <v>Available</v>
       </c>
       <c r="D97" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E97" t="str">
         <v>2.67</v>
@@ -6014,7 +6014,7 @@
         <v>Available</v>
       </c>
       <c r="D98" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E98" t="str">
         <v>6</v>

</xml_diff>

<commit_message>
Improve calculation of total scheduled hours for employees on specific dates
Update the logic in `server/pipeline.ts` to correctly sum all scheduled hours for an employee on a given date by iterating through the `scheduledHoursMap` in `getScheduledHoursForEmployeeAndDate`, addressing an issue where only the first entry was considered.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ae21854f-56f0-4406-b430-4b525fbb8b36
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/ae21854f-56f0-4406-b430-4b525fbb8b36/LrepN0o
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3289,10 +3289,10 @@
         <v>2025-09-01</v>
       </c>
       <c r="B2" t="str">
-        <v>57</v>
+        <v>56.83</v>
       </c>
       <c r="C2" t="str">
-        <v>57</v>
+        <v>56.83</v>
       </c>
       <c r="D2" t="str">
         <v>2.5</v>
@@ -3304,7 +3304,7 @@
         <v>69</v>
       </c>
       <c r="G2" t="str">
-        <v>-12</v>
+        <v>-12.17</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -3315,10 +3315,10 @@
         <v>2025-09-02</v>
       </c>
       <c r="B3" t="str">
-        <v>70.5</v>
+        <v>68.57</v>
       </c>
       <c r="C3" t="str">
-        <v>70.5</v>
+        <v>68.57</v>
       </c>
       <c r="D3" t="str">
         <v>9</v>
@@ -3330,7 +3330,7 @@
         <v>68</v>
       </c>
       <c r="G3" t="str">
-        <v>2.5</v>
+        <v>0.57</v>
       </c>
       <c r="H3" t="str">
         <v>Sufficient</v>
@@ -3341,10 +3341,10 @@
         <v>2025-09-03</v>
       </c>
       <c r="B4" t="str">
-        <v>74</v>
+        <v>72.57</v>
       </c>
       <c r="C4" t="str">
-        <v>74</v>
+        <v>72.57</v>
       </c>
       <c r="D4" t="str">
         <v>2</v>
@@ -3356,7 +3356,7 @@
         <v>82</v>
       </c>
       <c r="G4" t="str">
-        <v>-8</v>
+        <v>-9.43</v>
       </c>
       <c r="H4" t="str">
         <v>Shortage</v>

</xml_diff>

<commit_message>
Improve accuracy of required hours calculation by debugging filtering logic
Add detailed console logging to the `parseExcelFiles` function in `server/pipeline.ts` to trace data processing and identify discrepancies in required hours calculation, particularly for specific dates like Monday.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ae21854f-56f0-4406-b430-4b525fbb8b36
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/ae21854f-56f0-4406-b430-4b525fbb8b36/RN3t8ei
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -34,7 +34,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="5">
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
   </numFmts>
   <fonts count="1">
@@ -399,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I98"/>
+  <dimension ref="A1:I99"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -711,74 +715,74 @@
         <v>Pre-Agreed Appointment</v>
       </c>
       <c r="F11" t="str">
-        <v>10:20-12:50</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G11" t="str">
-        <v>2.5</v>
+        <v>2.67</v>
       </c>
       <c r="H11" t="str">
         <v>0</v>
       </c>
       <c r="I11" t="str">
-        <v>Brooke has an appointment to get bloods taken at 11.45 - MT</v>
+        <v>Brooke has a colonoscopy appointment - MT</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Forbes (NL) (GH), Amanda</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="B12" t="str">
         <v>16</v>
       </c>
       <c r="C12" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="D12" t="str">
-        <v>2025-09-01</v>
+        <v>2025-09-02</v>
       </c>
       <c r="E12" t="str">
-        <v>Available</v>
+        <v>Pre-Agreed Appointment</v>
       </c>
       <c r="F12" t="str">
-        <v>10:30-14:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G12" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="H12" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="I12" t="str">
-        <v>Confirmed at induction with MT</v>
+        <v>Brooke has a colonoscopy appointment - MT</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Forbes (NL) (GH), Amanda</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="B13" t="str">
         <v>16</v>
       </c>
       <c r="C13" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="D13" t="str">
-        <v>2025-09-02</v>
+        <v>2025-09-07</v>
       </c>
       <c r="E13" t="str">
-        <v>Available</v>
+        <v>Pre-Agreed Appointment</v>
       </c>
       <c r="F13" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G13" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="H13" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="I13" t="str">
-        <v/>
+        <v>Brooke advised that her previous appointment was cancelled and that it has been rescheduled. SM</v>
       </c>
     </row>
     <row r="14">
@@ -792,13 +796,13 @@
         <v>3.2</v>
       </c>
       <c r="D14" t="str">
-        <v>2025-09-03</v>
+        <v>2025-09-01</v>
       </c>
       <c r="E14" t="str">
         <v>Available</v>
       </c>
       <c r="F14" t="str">
-        <v>09:15-15:15</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="G14" t="str">
         <v>3.2</v>
@@ -807,7 +811,7 @@
         <v>3.2</v>
       </c>
       <c r="I14" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="15">
@@ -821,7 +825,7 @@
         <v>3.2</v>
       </c>
       <c r="D15" t="str">
-        <v>2025-09-04</v>
+        <v>2025-09-02</v>
       </c>
       <c r="E15" t="str">
         <v>Available</v>
@@ -850,13 +854,13 @@
         <v>3.2</v>
       </c>
       <c r="D16" t="str">
-        <v>2025-09-05</v>
+        <v>2025-09-03</v>
       </c>
       <c r="E16" t="str">
         <v>Available</v>
       </c>
       <c r="F16" t="str">
-        <v>10:30-14:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G16" t="str">
         <v>3.2</v>
@@ -865,65 +869,65 @@
         <v>3.2</v>
       </c>
       <c r="I16" t="str">
-        <v>Confirmed at induction with MT</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Forbes (NL) (GH), Amanda</v>
       </c>
       <c r="B17" t="str">
         <v>16</v>
       </c>
       <c r="C17" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="D17" t="str">
-        <v>2025-09-01</v>
+        <v>2025-09-04</v>
       </c>
       <c r="E17" t="str">
         <v>Available</v>
       </c>
       <c r="F17" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G17" t="str">
-        <v>0.17</v>
+        <v>3.2</v>
       </c>
       <c r="H17" t="str">
-        <v>0.17</v>
+        <v>3.2</v>
       </c>
       <c r="I17" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Forbes (NL) (GH), Amanda</v>
       </c>
       <c r="B18" t="str">
         <v>16</v>
       </c>
       <c r="C18" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="D18" t="str">
-        <v>2025-09-02</v>
+        <v>2025-09-05</v>
       </c>
       <c r="E18" t="str">
         <v>Available</v>
       </c>
       <c r="F18" t="str">
-        <v>09:15-14:00</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="G18" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="H18" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="I18" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="19">
@@ -937,7 +941,7 @@
         <v>2.67</v>
       </c>
       <c r="D19" t="str">
-        <v>2025-09-03</v>
+        <v>2025-09-01</v>
       </c>
       <c r="E19" t="str">
         <v>Available</v>
@@ -946,10 +950,10 @@
         <v>09:15-14:00</v>
       </c>
       <c r="G19" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="H19" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="I19" t="str">
         <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
@@ -966,7 +970,7 @@
         <v>2.67</v>
       </c>
       <c r="D20" t="str">
-        <v>2025-09-04</v>
+        <v>2025-09-02</v>
       </c>
       <c r="E20" t="str">
         <v>Available</v>
@@ -975,13 +979,13 @@
         <v>09:15-14:00</v>
       </c>
       <c r="G20" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="H20" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="I20" t="str">
-        <v/>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="21">
@@ -995,13 +999,13 @@
         <v>2.67</v>
       </c>
       <c r="D21" t="str">
-        <v>2025-09-06</v>
+        <v>2025-09-03</v>
       </c>
       <c r="E21" t="str">
         <v>Available</v>
       </c>
       <c r="F21" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G21" t="str">
         <v>2.67</v>
@@ -1010,7 +1014,7 @@
         <v>2.67</v>
       </c>
       <c r="I21" t="str">
-        <v/>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="22">
@@ -1024,7 +1028,7 @@
         <v>2.67</v>
       </c>
       <c r="D22" t="str">
-        <v>2025-09-07</v>
+        <v>2025-09-04</v>
       </c>
       <c r="E22" t="str">
         <v>Available</v>
@@ -1044,28 +1048,28 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Hume (NL) (GH), Chelsi-Anne</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="B23" t="str">
-        <v>37.5</v>
+        <v>16</v>
       </c>
       <c r="C23" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="D23" t="str">
-        <v>2025-09-01</v>
+        <v>2025-09-06</v>
       </c>
       <c r="E23" t="str">
         <v>Available</v>
       </c>
       <c r="F23" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G23" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="H23" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="I23" t="str">
         <v/>
@@ -1073,28 +1077,28 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Hume (NL) (GH), Chelsi-Anne</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="B24" t="str">
-        <v>37.5</v>
+        <v>16</v>
       </c>
       <c r="C24" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="D24" t="str">
-        <v>2025-09-02</v>
+        <v>2025-09-07</v>
       </c>
       <c r="E24" t="str">
         <v>Available</v>
       </c>
       <c r="F24" t="str">
-        <v>08:00-15:15</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G24" t="str">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H24" t="str">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I24" t="str">
         <v/>
@@ -1111,13 +1115,13 @@
         <v>7.5</v>
       </c>
       <c r="D25" t="str">
-        <v>2025-09-03</v>
+        <v>2025-09-01</v>
       </c>
       <c r="E25" t="str">
         <v>Available</v>
       </c>
       <c r="F25" t="str">
-        <v>08:30-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="G25" t="str">
         <v>7.5</v>
@@ -1140,25 +1144,25 @@
         <v>7.5</v>
       </c>
       <c r="D26" t="str">
-        <v>2025-09-04</v>
+        <v>2025-09-02</v>
       </c>
       <c r="E26" t="str">
         <v>Available</v>
       </c>
       <c r="F26" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="G26" t="str">
-        <v>7.5</v>
+        <v>0.5</v>
       </c>
       <c r="H26" t="str">
-        <v>7.5</v>
+        <v>0.5</v>
       </c>
       <c r="I26" t="str">
         <v/>
       </c>
     </row>
-    <row r="27" xml:space="preserve">
+    <row r="27">
       <c r="A27" t="str">
         <v>Hume (NL) (GH), Chelsi-Anne</v>
       </c>
@@ -1169,81 +1173,81 @@
         <v>7.5</v>
       </c>
       <c r="D27" t="str">
+        <v>2025-09-03</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F27" t="str">
+        <v>08:30-21:30</v>
+      </c>
+      <c r="G27" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="H27" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Hume (NL) (GH), Chelsi-Anne</v>
+      </c>
+      <c r="B28" t="str">
+        <v>37.5</v>
+      </c>
+      <c r="C28" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D28" t="str">
+        <v>2025-09-04</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F28" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G28" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="H28" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>Hume (NL) (GH), Chelsi-Anne</v>
+      </c>
+      <c r="B29" t="str">
+        <v>37.5</v>
+      </c>
+      <c r="C29" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D29" t="str">
         <v>2025-09-05</v>
       </c>
-      <c r="E27" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F27" t="str">
+      <c r="E29" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F29" t="str">
         <v>08:30-14:30</v>
       </c>
-      <c r="G27" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H27" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="I27" t="str" xml:space="preserve">
+      <c r="G29" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="H29" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="I29" t="str" xml:space="preserve">
         <v xml:space="preserve">Office hours
 Eilidh 27/08/2025</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Asokhia (NL), Deborah</v>
-      </c>
-      <c r="B28" t="str">
-        <v>20</v>
-      </c>
-      <c r="C28" t="str">
-        <v>4</v>
-      </c>
-      <c r="D28" t="str">
-        <v>2025-09-01</v>
-      </c>
-      <c r="E28" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F28" t="str">
-        <v>09:15-14:00</v>
-      </c>
-      <c r="G28" t="str">
-        <v>4</v>
-      </c>
-      <c r="H28" t="str">
-        <v>4</v>
-      </c>
-      <c r="I28" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>Asokhia (NL), Deborah</v>
-      </c>
-      <c r="B29" t="str">
-        <v>20</v>
-      </c>
-      <c r="C29" t="str">
-        <v>4</v>
-      </c>
-      <c r="D29" t="str">
-        <v>2025-09-02</v>
-      </c>
-      <c r="E29" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F29" t="str">
-        <v>09:15-14:00</v>
-      </c>
-      <c r="G29" t="str">
-        <v>4</v>
-      </c>
-      <c r="H29" t="str">
-        <v>4</v>
-      </c>
-      <c r="I29" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="30">
@@ -1257,7 +1261,7 @@
         <v>4</v>
       </c>
       <c r="D30" t="str">
-        <v>2025-09-03</v>
+        <v>2025-09-01</v>
       </c>
       <c r="E30" t="str">
         <v>Available</v>
@@ -1286,7 +1290,7 @@
         <v>4</v>
       </c>
       <c r="D31" t="str">
-        <v>2025-09-04</v>
+        <v>2025-09-02</v>
       </c>
       <c r="E31" t="str">
         <v>Available</v>
@@ -1315,7 +1319,7 @@
         <v>4</v>
       </c>
       <c r="D32" t="str">
-        <v>2025-09-05</v>
+        <v>2025-09-03</v>
       </c>
       <c r="E32" t="str">
         <v>Available</v>
@@ -1335,60 +1339,60 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Gabillard (NL), Donna</v>
+        <v>Asokhia (NL), Deborah</v>
       </c>
       <c r="B33" t="str">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C33" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="D33" t="str">
-        <v>2025-09-01</v>
+        <v>2025-09-04</v>
       </c>
       <c r="E33" t="str">
         <v>Available</v>
       </c>
       <c r="F33" t="str">
-        <v>09:15-14:45</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G33" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="H33" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="I33" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Gabillard (NL), Donna</v>
+        <v>Asokhia (NL), Deborah</v>
       </c>
       <c r="B34" t="str">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C34" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="D34" t="str">
-        <v>2025-09-02</v>
+        <v>2025-09-05</v>
       </c>
       <c r="E34" t="str">
         <v>Available</v>
       </c>
       <c r="F34" t="str">
-        <v>09:15-11:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G34" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="H34" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="I34" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="35">
@@ -1402,7 +1406,7 @@
         <v>2.8</v>
       </c>
       <c r="D35" t="str">
-        <v>2025-09-03</v>
+        <v>2025-09-01</v>
       </c>
       <c r="E35" t="str">
         <v>Available</v>
@@ -1431,7 +1435,7 @@
         <v>2.8</v>
       </c>
       <c r="D36" t="str">
-        <v>2025-09-04</v>
+        <v>2025-09-02</v>
       </c>
       <c r="E36" t="str">
         <v>Available</v>
@@ -1460,13 +1464,13 @@
         <v>2.8</v>
       </c>
       <c r="D37" t="str">
-        <v>2025-09-05</v>
+        <v>2025-09-03</v>
       </c>
       <c r="E37" t="str">
         <v>Available</v>
       </c>
       <c r="F37" t="str">
-        <v>09:15-10:15</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="G37" t="str">
         <v>2.8</v>
@@ -1480,74 +1484,74 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Shawcross (NL), Emma</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="B38" t="str">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C38" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="D38" t="str">
-        <v>2025-09-06</v>
+        <v>2025-09-04</v>
       </c>
       <c r="E38" t="str">
         <v>Available</v>
       </c>
       <c r="F38" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-11:30</v>
       </c>
       <c r="G38" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="H38" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="I38" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Shawcross (NL), Emma</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="B39" t="str">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C39" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="D39" t="str">
-        <v>2025-09-07</v>
+        <v>2025-09-05</v>
       </c>
       <c r="E39" t="str">
         <v>Available</v>
       </c>
       <c r="F39" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G39" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="H39" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="I39" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Shawcross (NL), Emma</v>
       </c>
       <c r="B40" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C40" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="D40" t="str">
-        <v>2025-09-01</v>
+        <v>2025-09-06</v>
       </c>
       <c r="E40" t="str">
         <v>Available</v>
@@ -1556,27 +1560,27 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G40" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="H40" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="I40" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Shawcross (NL), Emma</v>
       </c>
       <c r="B41" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C41" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="D41" t="str">
-        <v>2025-09-02</v>
+        <v>2025-09-07</v>
       </c>
       <c r="E41" t="str">
         <v>Available</v>
@@ -1585,13 +1589,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G41" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="H41" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="I41" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="42">
@@ -1605,7 +1609,7 @@
         <v>7.5</v>
       </c>
       <c r="D42" t="str">
-        <v>2025-09-06</v>
+        <v>2025-09-01</v>
       </c>
       <c r="E42" t="str">
         <v>Available</v>
@@ -1634,7 +1638,7 @@
         <v>7.5</v>
       </c>
       <c r="D43" t="str">
-        <v>2025-09-07</v>
+        <v>2025-09-02</v>
       </c>
       <c r="E43" t="str">
         <v>Available</v>
@@ -1654,16 +1658,16 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Duncan (NL), Madison</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="B44" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C44" t="str">
-        <v>5.33</v>
+        <v>7.5</v>
       </c>
       <c r="D44" t="str">
-        <v>2025-09-04</v>
+        <v>2025-09-06</v>
       </c>
       <c r="E44" t="str">
         <v>Available</v>
@@ -1672,10 +1676,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G44" t="str">
-        <v>5.33</v>
+        <v>7.5</v>
       </c>
       <c r="H44" t="str">
-        <v>5.33</v>
+        <v>7.5</v>
       </c>
       <c r="I44" t="str">
         <v/>
@@ -1683,28 +1687,28 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Duncan (NL), Madison</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="B45" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C45" t="str">
-        <v>5.33</v>
+        <v>7.5</v>
       </c>
       <c r="D45" t="str">
-        <v>2025-09-05</v>
+        <v>2025-09-07</v>
       </c>
       <c r="E45" t="str">
         <v>Available</v>
       </c>
       <c r="F45" t="str">
-        <v>08:00-17:45</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G45" t="str">
-        <v>5.33</v>
+        <v>7.5</v>
       </c>
       <c r="H45" t="str">
-        <v>5.33</v>
+        <v>7.5</v>
       </c>
       <c r="I45" t="str">
         <v/>
@@ -1712,28 +1716,28 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Duncan (NL), Madison</v>
+        <v>Mcewan (NL) (GH), Makala</v>
       </c>
       <c r="B46" t="str">
         <v>16</v>
       </c>
       <c r="C46" t="str">
-        <v>5.33</v>
+        <v>4</v>
       </c>
       <c r="D46" t="str">
-        <v>2025-09-07</v>
+        <v>2025-09-01</v>
       </c>
       <c r="E46" t="str">
         <v>Available</v>
       </c>
       <c r="F46" t="str">
-        <v>08:00-17:45</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="G46" t="str">
-        <v>5.33</v>
+        <v>4</v>
       </c>
       <c r="H46" t="str">
-        <v>5.33</v>
+        <v>4</v>
       </c>
       <c r="I46" t="str">
         <v/>
@@ -1750,7 +1754,7 @@
         <v>4</v>
       </c>
       <c r="D47" t="str">
-        <v>2025-09-01</v>
+        <v>2025-09-03</v>
       </c>
       <c r="E47" t="str">
         <v>Available</v>
@@ -1779,7 +1783,7 @@
         <v>4</v>
       </c>
       <c r="D48" t="str">
-        <v>2025-09-03</v>
+        <v>2025-09-06</v>
       </c>
       <c r="E48" t="str">
         <v>Available</v>
@@ -1808,7 +1812,7 @@
         <v>4</v>
       </c>
       <c r="D49" t="str">
-        <v>2025-09-06</v>
+        <v>2025-09-07</v>
       </c>
       <c r="E49" t="str">
         <v>Available</v>
@@ -1828,28 +1832,28 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Mcewan (NL) (GH), Makala</v>
+        <v>Ferris, Marykate</v>
       </c>
       <c r="B50" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C50" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="D50" t="str">
-        <v>2025-09-07</v>
+        <v>2025-09-02</v>
       </c>
       <c r="E50" t="str">
         <v>Available</v>
       </c>
       <c r="F50" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="G50" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="H50" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="I50" t="str">
         <v/>
@@ -1863,7 +1867,7 @@
         <v>20</v>
       </c>
       <c r="C51" t="str">
-        <v>10</v>
+        <v>6.67</v>
       </c>
       <c r="D51" t="str">
         <v>2025-09-04</v>
@@ -1875,10 +1879,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G51" t="str">
-        <v>10</v>
+        <v>6.67</v>
       </c>
       <c r="H51" t="str">
-        <v>10</v>
+        <v>6.67</v>
       </c>
       <c r="I51" t="str">
         <v/>
@@ -1892,7 +1896,7 @@
         <v>20</v>
       </c>
       <c r="C52" t="str">
-        <v>10</v>
+        <v>6.67</v>
       </c>
       <c r="D52" t="str">
         <v>2025-09-05</v>
@@ -1904,10 +1908,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G52" t="str">
-        <v>10</v>
+        <v>6.67</v>
       </c>
       <c r="H52" t="str">
-        <v>10</v>
+        <v>6.67</v>
       </c>
       <c r="I52" t="str">
         <v/>
@@ -3247,9 +3251,38 @@
         <v/>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Wylie (NL), Lori</v>
+      </c>
+      <c r="B99" t="str">
+        <v>30</v>
+      </c>
+      <c r="C99" t="str">
+        <v>6</v>
+      </c>
+      <c r="D99" t="str">
+        <v>2025-09-02</v>
+      </c>
+      <c r="E99" t="str">
+        <v>Dependant Leave</v>
+      </c>
+      <c r="F99" t="str">
+        <v>09:15-15:00</v>
+      </c>
+      <c r="G99" t="str">
+        <v>5.75</v>
+      </c>
+      <c r="H99" t="str">
+        <v>0</v>
+      </c>
+      <c r="I99" t="str">
+        <v>Lori's little boy has an abscess and isn't able to go to school - MT</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I98"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I99"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3295,16 +3328,16 @@
         <v>56.83</v>
       </c>
       <c r="D2" t="str">
-        <v>2.5</v>
+        <v>2.67</v>
       </c>
       <c r="E2" t="str">
         <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>69</v>
+        <v>77.55</v>
       </c>
       <c r="G2" t="str">
-        <v>-12.17</v>
+        <v>-20.72</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -3315,25 +3348,25 @@
         <v>2025-09-02</v>
       </c>
       <c r="B3" t="str">
-        <v>68.57</v>
+        <v>66.57</v>
       </c>
       <c r="C3" t="str">
-        <v>68.57</v>
+        <v>72.57</v>
       </c>
       <c r="D3" t="str">
-        <v>9</v>
+        <v>11.67</v>
       </c>
       <c r="E3" t="str">
         <v>0</v>
       </c>
       <c r="F3" t="str">
-        <v>68</v>
+        <v>78.36</v>
       </c>
       <c r="G3" t="str">
-        <v>0.57</v>
+        <v>-5.79</v>
       </c>
       <c r="H3" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="4">
@@ -3353,13 +3386,13 @@
         <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>82</v>
+        <v>69.07</v>
       </c>
       <c r="G4" t="str">
-        <v>-9.43</v>
+        <v>3.5</v>
       </c>
       <c r="H4" t="str">
-        <v>Shortage</v>
+        <v>Sufficient</v>
       </c>
     </row>
     <row r="5">
@@ -3367,10 +3400,10 @@
         <v>2025-09-04</v>
       </c>
       <c r="B5" t="str">
-        <v>86.66</v>
+        <v>78</v>
       </c>
       <c r="C5" t="str">
-        <v>86.66</v>
+        <v>78</v>
       </c>
       <c r="D5" t="str">
         <v>0</v>
@@ -3379,10 +3412,10 @@
         <v>0</v>
       </c>
       <c r="F5" t="str">
-        <v>71</v>
+        <v>66.58</v>
       </c>
       <c r="G5" t="str">
-        <v>15.66</v>
+        <v>11.42</v>
       </c>
       <c r="H5" t="str">
         <v>Sufficient</v>
@@ -3393,10 +3426,10 @@
         <v>2025-09-05</v>
       </c>
       <c r="B6" t="str">
-        <v>71.56</v>
+        <v>62.9</v>
       </c>
       <c r="C6" t="str">
-        <v>71.56</v>
+        <v>62.9</v>
       </c>
       <c r="D6" t="str">
         <v>2</v>
@@ -3405,10 +3438,10 @@
         <v>12.43</v>
       </c>
       <c r="F6" t="str">
-        <v>55</v>
+        <v>51.5</v>
       </c>
       <c r="G6" t="str">
-        <v>16.56</v>
+        <v>11.4</v>
       </c>
       <c r="H6" t="str">
         <v>Sufficient</v>
@@ -3431,10 +3464,10 @@
         <v>12.43</v>
       </c>
       <c r="F7" t="str">
-        <v>43</v>
+        <v>42.75</v>
       </c>
       <c r="G7" t="str">
-        <v>-12.83</v>
+        <v>-12.58</v>
       </c>
       <c r="H7" t="str">
         <v>Shortage</v>
@@ -3445,22 +3478,22 @@
         <v>2025-09-07</v>
       </c>
       <c r="B8" t="str">
-        <v>40.83</v>
+        <v>32.83</v>
       </c>
       <c r="C8" t="str">
-        <v>40.83</v>
+        <v>32.83</v>
       </c>
       <c r="D8" t="str">
-        <v>0</v>
+        <v>2.67</v>
       </c>
       <c r="E8" t="str">
         <v>3.43</v>
       </c>
       <c r="F8" t="str">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G8" t="str">
-        <v>-0.17</v>
+        <v>-7.17</v>
       </c>
       <c r="H8" t="str">
         <v>Shortage</v>
@@ -3475,7 +3508,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H98"/>
+  <dimension ref="A1:H99"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3560,25 +3593,25 @@
         <v>2025-09-05</v>
       </c>
       <c r="B4" t="str">
-        <v>Duncan (NL), Madison</v>
+        <v>Fayaz GH, Shafiya</v>
       </c>
       <c r="C4" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D4" t="str">
-        <v>08:00-17:45</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E4" t="str">
-        <v>5.33</v>
+        <v>9</v>
       </c>
       <c r="F4" t="str">
-        <v>5.33</v>
+        <v>9</v>
       </c>
       <c r="G4" t="str">
-        <v>5.33</v>
+        <v>0</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="5">
@@ -3589,7 +3622,7 @@
         <v>Fayaz GH, Shafiya</v>
       </c>
       <c r="C5" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D5" t="str">
         <v>08:00-21:30</v>
@@ -3598,13 +3631,13 @@
         <v>9</v>
       </c>
       <c r="F5" t="str">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G5" t="str">
         <v>0</v>
       </c>
       <c r="H5" t="str">
-        <v>Created by new vacation process.</v>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -3612,7 +3645,7 @@
         <v>2025-09-05</v>
       </c>
       <c r="B6" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Ferris, Marykate</v>
       </c>
       <c r="C6" t="str">
         <v>Available</v>
@@ -3621,13 +3654,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E6" t="str">
-        <v>9</v>
+        <v>6.67</v>
       </c>
       <c r="F6" t="str">
-        <v>0</v>
+        <v>6.67</v>
       </c>
       <c r="G6" t="str">
-        <v>0</v>
+        <v>6.67</v>
       </c>
       <c r="H6" t="str">
         <v/>
@@ -3638,25 +3671,25 @@
         <v>2025-09-05</v>
       </c>
       <c r="B7" t="str">
-        <v>Ferris, Marykate</v>
+        <v>Forbes (NL) (GH), Amanda</v>
       </c>
       <c r="C7" t="str">
         <v>Available</v>
       </c>
       <c r="D7" t="str">
-        <v>08:00-21:30</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="E7" t="str">
-        <v>10</v>
+        <v>3.2</v>
       </c>
       <c r="F7" t="str">
-        <v>10</v>
+        <v>3.2</v>
       </c>
       <c r="G7" t="str">
-        <v>10</v>
+        <v>3.2</v>
       </c>
       <c r="H7" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="8">
@@ -3664,78 +3697,78 @@
         <v>2025-09-05</v>
       </c>
       <c r="B8" t="str">
-        <v>Forbes (NL) (GH), Amanda</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="C8" t="str">
         <v>Available</v>
       </c>
       <c r="D8" t="str">
-        <v>10:30-14:00</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E8" t="str">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="F8" t="str">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="G8" t="str">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="H8" t="str">
-        <v>Confirmed at induction with MT</v>
-      </c>
-    </row>
-    <row r="9">
+        <v/>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
       <c r="A9" t="str">
         <v>2025-09-05</v>
       </c>
       <c r="B9" t="str">
-        <v>Gabillard (NL), Donna</v>
+        <v>Hume (NL) (GH), Chelsi-Anne</v>
       </c>
       <c r="C9" t="str">
         <v>Available</v>
       </c>
       <c r="D9" t="str">
-        <v>09:15-10:15</v>
+        <v>08:30-14:30</v>
       </c>
       <c r="E9" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="F9" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="G9" t="str">
-        <v>2.8</v>
-      </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="10" xml:space="preserve">
+        <v>7.5</v>
+      </c>
+      <c r="H9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Office hours
+Eilidh 27/08/2025</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" t="str">
         <v>2025-09-05</v>
       </c>
       <c r="B10" t="str">
-        <v>Hume (NL) (GH), Chelsi-Anne</v>
+        <v>Hussain (NL) (GH), Mustansar</v>
       </c>
       <c r="C10" t="str">
         <v>Available</v>
       </c>
       <c r="D10" t="str">
-        <v>08:30-14:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E10" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F10" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G10" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H10" t="str" xml:space="preserve">
-        <v xml:space="preserve">Office hours
-Eilidh 27/08/2025</v>
+        <v>6</v>
+      </c>
+      <c r="H10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -3743,25 +3776,25 @@
         <v>2025-09-05</v>
       </c>
       <c r="B11" t="str">
-        <v>Hussain (NL) (GH), Mustansar</v>
+        <v>Ibrahim (NL), Olusegun Isaac</v>
       </c>
       <c r="C11" t="str">
         <v>Available</v>
       </c>
       <c r="D11" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="E11" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="F11" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="G11" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H11" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="12">
@@ -3769,28 +3802,28 @@
         <v>2025-09-05</v>
       </c>
       <c r="B12" t="str">
-        <v>Ibrahim (NL), Olusegun Isaac</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="C12" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D12" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-17:00</v>
       </c>
       <c r="E12" t="str">
-        <v>3.2</v>
+        <v>3.43</v>
       </c>
       <c r="F12" t="str">
-        <v>3.2</v>
+        <v>3.43</v>
       </c>
       <c r="G12" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H12" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>Created by new vacation process.</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
       <c r="A13" t="str">
         <v>2025-09-05</v>
       </c>
@@ -3798,25 +3831,26 @@
         <v>Jack (NL), Sharon</v>
       </c>
       <c r="C13" t="str">
-        <v>Holiday</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D13" t="str">
-        <v>09:15-17:00</v>
+        <v>10:30-12:30</v>
       </c>
       <c r="E13" t="str">
         <v>3.43</v>
       </c>
       <c r="F13" t="str">
-        <v>3.43</v>
+        <v>2</v>
       </c>
       <c r="G13" t="str">
         <v>0</v>
       </c>
-      <c r="H13" t="str">
-        <v>Created by new vacation process.</v>
-      </c>
-    </row>
-    <row r="14" xml:space="preserve">
+      <c r="H13" t="str" xml:space="preserve">
+        <v xml:space="preserve">Wants this as a break. 
+Eilidh 29/05/2025</v>
+      </c>
+    </row>
+    <row r="14">
       <c r="A14" t="str">
         <v>2025-09-05</v>
       </c>
@@ -3824,23 +3858,22 @@
         <v>Jack (NL), Sharon</v>
       </c>
       <c r="C14" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D14" t="str">
-        <v>10:30-12:30</v>
+        <v>09:15-17:00</v>
       </c>
       <c r="E14" t="str">
         <v>3.43</v>
       </c>
       <c r="F14" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G14" t="str">
         <v>0</v>
       </c>
-      <c r="H14" t="str" xml:space="preserve">
-        <v xml:space="preserve">Wants this as a break. 
-Eilidh 29/05/2025</v>
+      <c r="H14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -3848,22 +3881,22 @@
         <v>2025-09-05</v>
       </c>
       <c r="B15" t="str">
-        <v>Jack (NL), Sharon</v>
+        <v>Lamont (NL) (GH), Sophie</v>
       </c>
       <c r="C15" t="str">
         <v>Available</v>
       </c>
       <c r="D15" t="str">
-        <v>09:15-17:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E15" t="str">
-        <v>3.43</v>
+        <v>7.5</v>
       </c>
       <c r="F15" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="G15" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H15" t="str">
         <v/>
@@ -3874,22 +3907,22 @@
         <v>2025-09-05</v>
       </c>
       <c r="B16" t="str">
-        <v>Lamont (NL) (GH), Sophie</v>
+        <v>McGhie (NL) (GH), Cheryl</v>
       </c>
       <c r="C16" t="str">
         <v>Available</v>
       </c>
       <c r="D16" t="str">
-        <v>08:00-21:30</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E16" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="F16" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="G16" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="H16" t="str">
         <v/>
@@ -3900,22 +3933,22 @@
         <v>2025-09-05</v>
       </c>
       <c r="B17" t="str">
-        <v>McGhie (NL) (GH), Cheryl</v>
+        <v>Nelson (NL), Anne</v>
       </c>
       <c r="C17" t="str">
         <v>Available</v>
       </c>
       <c r="D17" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-13:00</v>
       </c>
       <c r="E17" t="str">
-        <v>3.2</v>
+        <v>5.33</v>
       </c>
       <c r="F17" t="str">
-        <v>3.2</v>
+        <v>5.33</v>
       </c>
       <c r="G17" t="str">
-        <v>3.2</v>
+        <v>5.33</v>
       </c>
       <c r="H17" t="str">
         <v/>
@@ -3926,22 +3959,22 @@
         <v>2025-09-05</v>
       </c>
       <c r="B18" t="str">
-        <v>Nelson (NL), Anne</v>
+        <v>Wylie (NL), Lori</v>
       </c>
       <c r="C18" t="str">
         <v>Available</v>
       </c>
       <c r="D18" t="str">
-        <v>08:00-13:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E18" t="str">
-        <v>5.33</v>
+        <v>6</v>
       </c>
       <c r="F18" t="str">
-        <v>5.33</v>
+        <v>6</v>
       </c>
       <c r="G18" t="str">
-        <v>5.33</v>
+        <v>6</v>
       </c>
       <c r="H18" t="str">
         <v/>
@@ -3949,25 +3982,25 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2025-09-05</v>
+        <v>2025-09-06</v>
       </c>
       <c r="B19" t="str">
-        <v>Wylie (NL), Lori</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="C19" t="str">
         <v>Available</v>
       </c>
       <c r="D19" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E19" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="F19" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="G19" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="H19" t="str">
         <v/>
@@ -3978,25 +4011,25 @@
         <v>2025-09-06</v>
       </c>
       <c r="B20" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Fayaz GH, Shafiya</v>
       </c>
       <c r="C20" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D20" t="str">
         <v>08:00-21:30</v>
       </c>
       <c r="E20" t="str">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="F20" t="str">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="G20" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H20" t="str">
-        <v/>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="21">
@@ -4007,7 +4040,7 @@
         <v>Fayaz GH, Shafiya</v>
       </c>
       <c r="C21" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D21" t="str">
         <v>08:00-21:30</v>
@@ -4016,13 +4049,13 @@
         <v>9</v>
       </c>
       <c r="F21" t="str">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G21" t="str">
         <v>0</v>
       </c>
       <c r="H21" t="str">
-        <v>Created by new vacation process.</v>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -4030,7 +4063,7 @@
         <v>2025-09-06</v>
       </c>
       <c r="B22" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Hussain (NL) (GH), Mustansar</v>
       </c>
       <c r="C22" t="str">
         <v>Available</v>
@@ -4039,13 +4072,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E22" t="str">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F22" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G22" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H22" t="str">
         <v/>
@@ -4056,25 +4089,25 @@
         <v>2025-09-06</v>
       </c>
       <c r="B23" t="str">
-        <v>Hussain (NL) (GH), Mustansar</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="C23" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D23" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-17:00</v>
       </c>
       <c r="E23" t="str">
-        <v>6</v>
+        <v>3.43</v>
       </c>
       <c r="F23" t="str">
-        <v>6</v>
+        <v>3.43</v>
       </c>
       <c r="G23" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H23" t="str">
-        <v/>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="24">
@@ -4082,25 +4115,25 @@
         <v>2025-09-06</v>
       </c>
       <c r="B24" t="str">
-        <v>Jack (NL), Sharon</v>
+        <v>Mcewan (NL) (GH), Makala</v>
       </c>
       <c r="C24" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D24" t="str">
-        <v>09:15-17:00</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="E24" t="str">
-        <v>3.43</v>
+        <v>4</v>
       </c>
       <c r="F24" t="str">
-        <v>3.43</v>
+        <v>4</v>
       </c>
       <c r="G24" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H24" t="str">
-        <v>Created by new vacation process.</v>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -4108,22 +4141,22 @@
         <v>2025-09-06</v>
       </c>
       <c r="B25" t="str">
-        <v>Mcewan (NL) (GH), Makala</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C25" t="str">
         <v>Available</v>
       </c>
       <c r="D25" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E25" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="F25" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="G25" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="H25" t="str">
         <v/>
@@ -4134,7 +4167,7 @@
         <v>2025-09-06</v>
       </c>
       <c r="B26" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Shawcross (NL), Emma</v>
       </c>
       <c r="C26" t="str">
         <v>Available</v>
@@ -4143,24 +4176,24 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E26" t="str">
-        <v>2.67</v>
+        <v>10</v>
       </c>
       <c r="F26" t="str">
-        <v>2.67</v>
+        <v>10</v>
       </c>
       <c r="G26" t="str">
-        <v>2.67</v>
+        <v>10</v>
       </c>
       <c r="H26" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2025-09-06</v>
+        <v>2025-09-07</v>
       </c>
       <c r="B27" t="str">
-        <v>Shawcross (NL), Emma</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="C27" t="str">
         <v>Available</v>
@@ -4169,16 +4202,16 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E27" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="F27" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="G27" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="H27" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -4186,7 +4219,7 @@
         <v>2025-09-07</v>
       </c>
       <c r="B28" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Griffiths (NL), Wayne (GH)</v>
       </c>
       <c r="C28" t="str">
         <v>Available</v>
@@ -4195,13 +4228,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E28" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F28" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G28" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -4212,25 +4245,25 @@
         <v>2025-09-07</v>
       </c>
       <c r="B29" t="str">
-        <v>Duncan (NL), Madison</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="C29" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D29" t="str">
-        <v>08:00-17:45</v>
+        <v>09:15-17:00</v>
       </c>
       <c r="E29" t="str">
-        <v>5.33</v>
+        <v>3.43</v>
       </c>
       <c r="F29" t="str">
-        <v>5.33</v>
+        <v>3.43</v>
       </c>
       <c r="G29" t="str">
-        <v>5.33</v>
+        <v>0</v>
       </c>
       <c r="H29" t="str">
-        <v/>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="30">
@@ -4238,22 +4271,22 @@
         <v>2025-09-07</v>
       </c>
       <c r="B30" t="str">
-        <v>Griffiths (NL), Wayne (GH)</v>
+        <v>Mcewan (NL) (GH), Makala</v>
       </c>
       <c r="C30" t="str">
         <v>Available</v>
       </c>
       <c r="D30" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="E30" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F30" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G30" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H30" t="str">
         <v/>
@@ -4264,25 +4297,25 @@
         <v>2025-09-07</v>
       </c>
       <c r="B31" t="str">
-        <v>Jack (NL), Sharon</v>
+        <v>Nelson (NL), Anne</v>
       </c>
       <c r="C31" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D31" t="str">
-        <v>09:15-17:00</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E31" t="str">
-        <v>3.43</v>
+        <v>5.33</v>
       </c>
       <c r="F31" t="str">
-        <v>3.43</v>
+        <v>5.33</v>
       </c>
       <c r="G31" t="str">
-        <v>0</v>
+        <v>5.33</v>
       </c>
       <c r="H31" t="str">
-        <v>Created by new vacation process.</v>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -4290,25 +4323,25 @@
         <v>2025-09-07</v>
       </c>
       <c r="B32" t="str">
-        <v>Mcewan (NL) (GH), Makala</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C32" t="str">
-        <v>Available</v>
+        <v>Pre-Agreed Appointment</v>
       </c>
       <c r="D32" t="str">
-        <v>08:00-15:15</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E32" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="F32" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="G32" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H32" t="str">
-        <v/>
+        <v>Brooke advised that her previous appointment was cancelled and that it has been rescheduled. SM</v>
       </c>
     </row>
     <row r="33">
@@ -4316,22 +4349,22 @@
         <v>2025-09-07</v>
       </c>
       <c r="B33" t="str">
-        <v>Nelson (NL), Anne</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C33" t="str">
         <v>Available</v>
       </c>
       <c r="D33" t="str">
-        <v>08:00-18:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E33" t="str">
-        <v>5.33</v>
+        <v>2.67</v>
       </c>
       <c r="F33" t="str">
-        <v>5.33</v>
+        <v>0</v>
       </c>
       <c r="G33" t="str">
-        <v>5.33</v>
+        <v>0</v>
       </c>
       <c r="H33" t="str">
         <v/>
@@ -4342,33 +4375,33 @@
         <v>2025-09-07</v>
       </c>
       <c r="B34" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Shawcross (NL), Emma</v>
       </c>
       <c r="C34" t="str">
         <v>Available</v>
       </c>
       <c r="D34" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E34" t="str">
-        <v>2.67</v>
+        <v>10</v>
       </c>
       <c r="F34" t="str">
-        <v>2.67</v>
+        <v>10</v>
       </c>
       <c r="G34" t="str">
-        <v>2.67</v>
+        <v>10</v>
       </c>
       <c r="H34" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2025-09-07</v>
+        <v>2025-09-02</v>
       </c>
       <c r="B35" t="str">
-        <v>Shawcross (NL), Emma</v>
+        <v>Adeyanju (NL) (GH), Adedayo</v>
       </c>
       <c r="C35" t="str">
         <v>Available</v>
@@ -4377,16 +4410,16 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E35" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="F35" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="G35" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="H35" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -4394,25 +4427,25 @@
         <v>2025-09-02</v>
       </c>
       <c r="B36" t="str">
-        <v>Adeyanju (NL) (GH), Adedayo</v>
+        <v>Asokhia (NL), Deborah</v>
       </c>
       <c r="C36" t="str">
         <v>Available</v>
       </c>
       <c r="D36" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E36" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="F36" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="G36" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="H36" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="37">
@@ -4420,25 +4453,25 @@
         <v>2025-09-02</v>
       </c>
       <c r="B37" t="str">
-        <v>Asokhia (NL), Deborah</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="C37" t="str">
         <v>Available</v>
       </c>
       <c r="D37" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E37" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="F37" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="G37" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="H37" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -4446,7 +4479,7 @@
         <v>2025-09-02</v>
       </c>
       <c r="B38" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Fayaz GH, Shafiya</v>
       </c>
       <c r="C38" t="str">
         <v>Available</v>
@@ -4455,13 +4488,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E38" t="str">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="F38" t="str">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="G38" t="str">
-        <v>7.5</v>
+        <v>9</v>
       </c>
       <c r="H38" t="str">
         <v/>
@@ -4472,22 +4505,22 @@
         <v>2025-09-02</v>
       </c>
       <c r="B39" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Ferris, Marykate</v>
       </c>
       <c r="C39" t="str">
         <v>Available</v>
       </c>
       <c r="D39" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E39" t="str">
-        <v>9</v>
+        <v>6.67</v>
       </c>
       <c r="F39" t="str">
-        <v>9</v>
+        <v>6.67</v>
       </c>
       <c r="G39" t="str">
-        <v>9</v>
+        <v>6.67</v>
       </c>
       <c r="H39" t="str">
         <v/>
@@ -4788,7 +4821,7 @@
         <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C51" t="str">
-        <v>Available</v>
+        <v>Pre-Agreed Appointment</v>
       </c>
       <c r="D51" t="str">
         <v>09:15-14:00</v>
@@ -4800,10 +4833,10 @@
         <v>2.67</v>
       </c>
       <c r="G51" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="H51" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v>Brooke has a colonoscopy appointment - MT</v>
       </c>
     </row>
     <row r="52">
@@ -4811,7 +4844,7 @@
         <v>2025-09-02</v>
       </c>
       <c r="B52" t="str">
-        <v>Wylie (NL), Lori</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C52" t="str">
         <v>Available</v>
@@ -4820,39 +4853,39 @@
         <v>09:15-14:00</v>
       </c>
       <c r="E52" t="str">
-        <v>6</v>
+        <v>2.67</v>
       </c>
       <c r="F52" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G52" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H52" t="str">
-        <v/>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2025-09-03</v>
+        <v>2025-09-02</v>
       </c>
       <c r="B53" t="str">
-        <v>Adeyanju (NL) (GH), Adedayo</v>
+        <v>Wylie (NL), Lori</v>
       </c>
       <c r="C53" t="str">
         <v>Available</v>
       </c>
       <c r="D53" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E53" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F53" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G53" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H53" t="str">
         <v/>
@@ -4860,28 +4893,28 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2025-09-03</v>
+        <v>2025-09-02</v>
       </c>
       <c r="B54" t="str">
-        <v>Asokhia (NL), Deborah</v>
+        <v>Wylie (NL), Lori</v>
       </c>
       <c r="C54" t="str">
-        <v>Available</v>
+        <v>Dependant Leave</v>
       </c>
       <c r="D54" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="E54" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F54" t="str">
-        <v>4</v>
+        <v>5.75</v>
       </c>
       <c r="G54" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H54" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v>Lori's little boy has an abscess and isn't able to go to school - MT</v>
       </c>
     </row>
     <row r="55">
@@ -4889,7 +4922,7 @@
         <v>2025-09-03</v>
       </c>
       <c r="B55" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Adeyanju (NL) (GH), Adedayo</v>
       </c>
       <c r="C55" t="str">
         <v>Available</v>
@@ -4898,13 +4931,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E55" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="F55" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="G55" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H55" t="str">
         <v/>
@@ -4915,25 +4948,25 @@
         <v>2025-09-03</v>
       </c>
       <c r="B56" t="str">
-        <v>Forbes (NL) (GH), Amanda</v>
+        <v>Asokhia (NL), Deborah</v>
       </c>
       <c r="C56" t="str">
         <v>Available</v>
       </c>
       <c r="D56" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E56" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="F56" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="G56" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="H56" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="57">
@@ -4941,22 +4974,22 @@
         <v>2025-09-03</v>
       </c>
       <c r="B57" t="str">
-        <v>Gabillard (NL), Donna</v>
+        <v>Fayaz GH, Shafiya</v>
       </c>
       <c r="C57" t="str">
         <v>Available</v>
       </c>
       <c r="D57" t="str">
-        <v>09:15-14:45</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E57" t="str">
-        <v>2.8</v>
+        <v>9</v>
       </c>
       <c r="F57" t="str">
-        <v>2.8</v>
+        <v>9</v>
       </c>
       <c r="G57" t="str">
-        <v>2.8</v>
+        <v>9</v>
       </c>
       <c r="H57" t="str">
         <v/>
@@ -4967,22 +5000,22 @@
         <v>2025-09-03</v>
       </c>
       <c r="B58" t="str">
-        <v>Griffiths (NL), Wayne (GH)</v>
+        <v>Forbes (NL) (GH), Amanda</v>
       </c>
       <c r="C58" t="str">
         <v>Available</v>
       </c>
       <c r="D58" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E58" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="F58" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="G58" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H58" t="str">
         <v/>
@@ -4993,22 +5026,22 @@
         <v>2025-09-03</v>
       </c>
       <c r="B59" t="str">
-        <v>Hume (NL) (GH), Chelsi-Anne</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="C59" t="str">
         <v>Available</v>
       </c>
       <c r="D59" t="str">
-        <v>08:30-21:30</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="E59" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="F59" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="G59" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="H59" t="str">
         <v/>
@@ -5019,7 +5052,7 @@
         <v>2025-09-03</v>
       </c>
       <c r="B60" t="str">
-        <v>Hussain (NL) (GH), Mustansar</v>
+        <v>Griffiths (NL), Wayne (GH)</v>
       </c>
       <c r="C60" t="str">
         <v>Available</v>
@@ -5045,52 +5078,51 @@
         <v>2025-09-03</v>
       </c>
       <c r="B61" t="str">
-        <v>Ibrahim (NL), Olusegun Isaac</v>
+        <v>Hume (NL) (GH), Chelsi-Anne</v>
       </c>
       <c r="C61" t="str">
         <v>Available</v>
       </c>
       <c r="D61" t="str">
-        <v>09:15-15:00</v>
+        <v>08:30-21:30</v>
       </c>
       <c r="E61" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F61" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G61" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H61" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
-      </c>
-    </row>
-    <row r="62" xml:space="preserve">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
       <c r="A62" t="str">
         <v>2025-09-03</v>
       </c>
       <c r="B62" t="str">
-        <v>Jack (NL), Sharon</v>
+        <v>Hussain (NL) (GH), Mustansar</v>
       </c>
       <c r="C62" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D62" t="str">
-        <v>10:30-12:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E62" t="str">
-        <v>3.43</v>
+        <v>6</v>
       </c>
       <c r="F62" t="str">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G62" t="str">
-        <v>0</v>
-      </c>
-      <c r="H62" t="str" xml:space="preserve">
-        <v xml:space="preserve">Wants this as a break. 
-Eilidh 29/05/2025</v>
+        <v>6</v>
+      </c>
+      <c r="H62" t="str">
+        <v/>
       </c>
     </row>
     <row r="63">
@@ -5098,51 +5130,52 @@
         <v>2025-09-03</v>
       </c>
       <c r="B63" t="str">
-        <v>Jack (NL), Sharon</v>
+        <v>Ibrahim (NL), Olusegun Isaac</v>
       </c>
       <c r="C63" t="str">
         <v>Available</v>
       </c>
       <c r="D63" t="str">
-        <v>09:15-16:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="E63" t="str">
-        <v>3.43</v>
+        <v>3.2</v>
       </c>
       <c r="F63" t="str">
-        <v>1.43</v>
+        <v>3.2</v>
       </c>
       <c r="G63" t="str">
-        <v>1.43</v>
+        <v>3.2</v>
       </c>
       <c r="H63" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="64">
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+      </c>
+    </row>
+    <row r="64" xml:space="preserve">
       <c r="A64" t="str">
         <v>2025-09-03</v>
       </c>
       <c r="B64" t="str">
-        <v>Lamont (NL) (GH), Sophie</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="C64" t="str">
-        <v>Available</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D64" t="str">
-        <v>08:00-21:30</v>
+        <v>10:30-12:30</v>
       </c>
       <c r="E64" t="str">
-        <v>7.5</v>
+        <v>3.43</v>
       </c>
       <c r="F64" t="str">
-        <v>7.5</v>
+        <v>2</v>
       </c>
       <c r="G64" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H64" t="str">
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="H64" t="str" xml:space="preserve">
+        <v xml:space="preserve">Wants this as a break. 
+Eilidh 29/05/2025</v>
       </c>
     </row>
     <row r="65">
@@ -5150,22 +5183,22 @@
         <v>2025-09-03</v>
       </c>
       <c r="B65" t="str">
-        <v>Mcewan (NL) (GH), Makala</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="C65" t="str">
         <v>Available</v>
       </c>
       <c r="D65" t="str">
-        <v>08:00-15:15</v>
+        <v>09:15-16:30</v>
       </c>
       <c r="E65" t="str">
-        <v>4</v>
+        <v>3.43</v>
       </c>
       <c r="F65" t="str">
-        <v>4</v>
+        <v>1.43</v>
       </c>
       <c r="G65" t="str">
-        <v>4</v>
+        <v>1.43</v>
       </c>
       <c r="H65" t="str">
         <v/>
@@ -5176,22 +5209,22 @@
         <v>2025-09-03</v>
       </c>
       <c r="B66" t="str">
-        <v>McGhie (NL) (GH), Cheryl</v>
+        <v>Lamont (NL) (GH), Sophie</v>
       </c>
       <c r="C66" t="str">
         <v>Available</v>
       </c>
       <c r="D66" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E66" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F66" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G66" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H66" t="str">
         <v/>
@@ -5202,25 +5235,25 @@
         <v>2025-09-03</v>
       </c>
       <c r="B67" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Mcewan (NL) (GH), Makala</v>
       </c>
       <c r="C67" t="str">
         <v>Available</v>
       </c>
       <c r="D67" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="E67" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="F67" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="G67" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="H67" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="68">
@@ -5228,22 +5261,22 @@
         <v>2025-09-03</v>
       </c>
       <c r="B68" t="str">
-        <v>Wylie (NL), Lori</v>
+        <v>McGhie (NL) (GH), Cheryl</v>
       </c>
       <c r="C68" t="str">
         <v>Available</v>
       </c>
       <c r="D68" t="str">
-        <v>09:15-15:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E68" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="F68" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="G68" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H68" t="str">
         <v/>
@@ -5251,10 +5284,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2025-09-01</v>
+        <v>2025-09-03</v>
       </c>
       <c r="B69" t="str">
-        <v>Asokhia (NL), Deborah</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C69" t="str">
         <v>Available</v>
@@ -5263,39 +5296,39 @@
         <v>09:15-14:00</v>
       </c>
       <c r="E69" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="F69" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="G69" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="H69" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2025-09-01</v>
+        <v>2025-09-03</v>
       </c>
       <c r="B70" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Wylie (NL), Lori</v>
       </c>
       <c r="C70" t="str">
         <v>Available</v>
       </c>
       <c r="D70" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="E70" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F70" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G70" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H70" t="str">
         <v/>
@@ -5306,25 +5339,25 @@
         <v>2025-09-01</v>
       </c>
       <c r="B71" t="str">
-        <v>Forbes (NL) (GH), Amanda</v>
+        <v>Asokhia (NL), Deborah</v>
       </c>
       <c r="C71" t="str">
         <v>Available</v>
       </c>
       <c r="D71" t="str">
-        <v>10:30-14:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E71" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="F71" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="G71" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="H71" t="str">
-        <v>Confirmed at induction with MT</v>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="72">
@@ -5332,22 +5365,22 @@
         <v>2025-09-01</v>
       </c>
       <c r="B72" t="str">
-        <v>Gabillard (NL), Donna</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="C72" t="str">
         <v>Available</v>
       </c>
       <c r="D72" t="str">
-        <v>09:15-14:45</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E72" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="F72" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="G72" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="H72" t="str">
         <v/>
@@ -5358,25 +5391,25 @@
         <v>2025-09-01</v>
       </c>
       <c r="B73" t="str">
-        <v>Griffiths (NL), Wayne (GH)</v>
+        <v>Forbes (NL) (GH), Amanda</v>
       </c>
       <c r="C73" t="str">
         <v>Available</v>
       </c>
       <c r="D73" t="str">
-        <v>08:00-21:30</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="E73" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="F73" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="G73" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H73" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="74">
@@ -5384,22 +5417,22 @@
         <v>2025-09-01</v>
       </c>
       <c r="B74" t="str">
-        <v>Hume (NL) (GH), Chelsi-Anne</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="C74" t="str">
         <v>Available</v>
       </c>
       <c r="D74" t="str">
-        <v>08:00-15:15</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="E74" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="F74" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="G74" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="H74" t="str">
         <v/>
@@ -5410,7 +5443,7 @@
         <v>2025-09-01</v>
       </c>
       <c r="B75" t="str">
-        <v>Hussain (NL) (GH), Mustansar</v>
+        <v>Griffiths (NL), Wayne (GH)</v>
       </c>
       <c r="C75" t="str">
         <v>Available</v>
@@ -5436,25 +5469,25 @@
         <v>2025-09-01</v>
       </c>
       <c r="B76" t="str">
-        <v>Ibrahim (NL), Olusegun Isaac</v>
+        <v>Hume (NL) (GH), Chelsi-Anne</v>
       </c>
       <c r="C76" t="str">
         <v>Available</v>
       </c>
       <c r="D76" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="E76" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F76" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G76" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H76" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="77">
@@ -5462,22 +5495,22 @@
         <v>2025-09-01</v>
       </c>
       <c r="B77" t="str">
-        <v>Jack (NL), Sharon</v>
+        <v>Hussain (NL) (GH), Mustansar</v>
       </c>
       <c r="C77" t="str">
         <v>Available</v>
       </c>
       <c r="D77" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E77" t="str">
-        <v>3.43</v>
+        <v>6</v>
       </c>
       <c r="F77" t="str">
-        <v>3.43</v>
+        <v>6</v>
       </c>
       <c r="G77" t="str">
-        <v>3.43</v>
+        <v>6</v>
       </c>
       <c r="H77" t="str">
         <v/>
@@ -5488,25 +5521,25 @@
         <v>2025-09-01</v>
       </c>
       <c r="B78" t="str">
-        <v>Mcewan (NL) (GH), Makala</v>
+        <v>Ibrahim (NL), Olusegun Isaac</v>
       </c>
       <c r="C78" t="str">
         <v>Available</v>
       </c>
       <c r="D78" t="str">
-        <v>08:00-15:15</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="E78" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="F78" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="G78" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="H78" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="79">
@@ -5514,25 +5547,25 @@
         <v>2025-09-01</v>
       </c>
       <c r="B79" t="str">
-        <v>McGhie (NL) (GH), Cheryl</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="C79" t="str">
         <v>Available</v>
       </c>
       <c r="D79" t="str">
-        <v>09:15-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E79" t="str">
-        <v>3.2</v>
+        <v>3.43</v>
       </c>
       <c r="F79" t="str">
-        <v>3.2</v>
+        <v>3.43</v>
       </c>
       <c r="G79" t="str">
-        <v>3.2</v>
+        <v>3.43</v>
       </c>
       <c r="H79" t="str">
-        <v>Cheryl has agreed to extend her availability via email 02/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="80">
@@ -5540,25 +5573,25 @@
         <v>2025-09-01</v>
       </c>
       <c r="B80" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Mcewan (NL) (GH), Makala</v>
       </c>
       <c r="C80" t="str">
-        <v>Pre-Agreed Appointment</v>
+        <v>Available</v>
       </c>
       <c r="D80" t="str">
-        <v>10:20-12:50</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="E80" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="F80" t="str">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="G80" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H80" t="str">
-        <v>Brooke has an appointment to get bloods taken at 11.45 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="81">
@@ -5566,25 +5599,25 @@
         <v>2025-09-01</v>
       </c>
       <c r="B81" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>McGhie (NL) (GH), Cheryl</v>
       </c>
       <c r="C81" t="str">
         <v>Available</v>
       </c>
       <c r="D81" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-21:30</v>
       </c>
       <c r="E81" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="F81" t="str">
-        <v>0.17</v>
+        <v>3.2</v>
       </c>
       <c r="G81" t="str">
-        <v>0.17</v>
+        <v>3.2</v>
       </c>
       <c r="H81" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v>Cheryl has agreed to extend her availability via email 02/04/2025 - MT</v>
       </c>
     </row>
     <row r="82">
@@ -5592,59 +5625,59 @@
         <v>2025-09-01</v>
       </c>
       <c r="B82" t="str">
-        <v>Wylie (NL), Lori</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C82" t="str">
-        <v>Available</v>
+        <v>Pre-Agreed Appointment</v>
       </c>
       <c r="D82" t="str">
         <v>09:15-14:00</v>
       </c>
       <c r="E82" t="str">
-        <v>6</v>
+        <v>2.67</v>
       </c>
       <c r="F82" t="str">
-        <v>6</v>
+        <v>2.67</v>
       </c>
       <c r="G82" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H82" t="str">
-        <v/>
+        <v>Brooke has a colonoscopy appointment - MT</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2025-09-04</v>
+        <v>2025-09-01</v>
       </c>
       <c r="B83" t="str">
-        <v>Adeyanju (NL) (GH), Adedayo</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C83" t="str">
         <v>Available</v>
       </c>
       <c r="D83" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E83" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="F83" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G83" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H83" t="str">
-        <v/>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2025-09-04</v>
+        <v>2025-09-01</v>
       </c>
       <c r="B84" t="str">
-        <v>Asokhia (NL), Deborah</v>
+        <v>Wylie (NL), Lori</v>
       </c>
       <c r="C84" t="str">
         <v>Available</v>
@@ -5653,16 +5686,16 @@
         <v>09:15-14:00</v>
       </c>
       <c r="E84" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F84" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G84" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H84" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="85">
@@ -5670,7 +5703,7 @@
         <v>2025-09-04</v>
       </c>
       <c r="B85" t="str">
-        <v>Duncan (NL), Madison</v>
+        <v>Adeyanju (NL) (GH), Adedayo</v>
       </c>
       <c r="C85" t="str">
         <v>Available</v>
@@ -5679,13 +5712,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E85" t="str">
-        <v>5.33</v>
+        <v>7.5</v>
       </c>
       <c r="F85" t="str">
-        <v>5.33</v>
+        <v>7.5</v>
       </c>
       <c r="G85" t="str">
-        <v>5.33</v>
+        <v>7.5</v>
       </c>
       <c r="H85" t="str">
         <v/>
@@ -5696,25 +5729,25 @@
         <v>2025-09-04</v>
       </c>
       <c r="B86" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Asokhia (NL), Deborah</v>
       </c>
       <c r="C86" t="str">
         <v>Available</v>
       </c>
       <c r="D86" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E86" t="str">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F86" t="str">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G86" t="str">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H86" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="87">
@@ -5722,7 +5755,7 @@
         <v>2025-09-04</v>
       </c>
       <c r="B87" t="str">
-        <v>Ferris, Marykate</v>
+        <v>Fayaz GH, Shafiya</v>
       </c>
       <c r="C87" t="str">
         <v>Available</v>
@@ -5731,13 +5764,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E87" t="str">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F87" t="str">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G87" t="str">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H87" t="str">
         <v/>
@@ -5748,22 +5781,22 @@
         <v>2025-09-04</v>
       </c>
       <c r="B88" t="str">
-        <v>Forbes (NL) (GH), Amanda</v>
+        <v>Ferris, Marykate</v>
       </c>
       <c r="C88" t="str">
         <v>Available</v>
       </c>
       <c r="D88" t="str">
-        <v>09:15-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E88" t="str">
-        <v>3.2</v>
+        <v>6.67</v>
       </c>
       <c r="F88" t="str">
-        <v>3.2</v>
+        <v>6.67</v>
       </c>
       <c r="G88" t="str">
-        <v>3.2</v>
+        <v>6.67</v>
       </c>
       <c r="H88" t="str">
         <v/>
@@ -5774,22 +5807,22 @@
         <v>2025-09-04</v>
       </c>
       <c r="B89" t="str">
-        <v>Gabillard (NL), Donna</v>
+        <v>Forbes (NL) (GH), Amanda</v>
       </c>
       <c r="C89" t="str">
         <v>Available</v>
       </c>
       <c r="D89" t="str">
-        <v>09:15-11:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E89" t="str">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="F89" t="str">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="G89" t="str">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="H89" t="str">
         <v/>
@@ -5800,22 +5833,22 @@
         <v>2025-09-04</v>
       </c>
       <c r="B90" t="str">
-        <v>Griffiths (NL), Wayne (GH)</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="C90" t="str">
         <v>Available</v>
       </c>
       <c r="D90" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-11:30</v>
       </c>
       <c r="E90" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="F90" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="G90" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="H90" t="str">
         <v/>
@@ -5826,7 +5859,7 @@
         <v>2025-09-04</v>
       </c>
       <c r="B91" t="str">
-        <v>Hume (NL) (GH), Chelsi-Anne</v>
+        <v>Griffiths (NL), Wayne (GH)</v>
       </c>
       <c r="C91" t="str">
         <v>Available</v>
@@ -5835,13 +5868,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E91" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F91" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G91" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H91" t="str">
         <v/>
@@ -5852,25 +5885,25 @@
         <v>2025-09-04</v>
       </c>
       <c r="B92" t="str">
-        <v>Ibrahim (NL), Olusegun Isaac</v>
+        <v>Hume (NL) (GH), Chelsi-Anne</v>
       </c>
       <c r="C92" t="str">
         <v>Available</v>
       </c>
       <c r="D92" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E92" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F92" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G92" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H92" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="93">
@@ -5878,25 +5911,25 @@
         <v>2025-09-04</v>
       </c>
       <c r="B93" t="str">
-        <v>Jack (NL), Sharon</v>
+        <v>Ibrahim (NL), Olusegun Isaac</v>
       </c>
       <c r="C93" t="str">
         <v>Available</v>
       </c>
       <c r="D93" t="str">
-        <v>09:15-16:15</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="E93" t="str">
-        <v>3.43</v>
+        <v>3.2</v>
       </c>
       <c r="F93" t="str">
-        <v>3.43</v>
+        <v>3.2</v>
       </c>
       <c r="G93" t="str">
-        <v>3.43</v>
+        <v>3.2</v>
       </c>
       <c r="H93" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="94">
@@ -5904,22 +5937,22 @@
         <v>2025-09-04</v>
       </c>
       <c r="B94" t="str">
-        <v>Lamont (NL) (GH), Sophie</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="C94" t="str">
         <v>Available</v>
       </c>
       <c r="D94" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-16:15</v>
       </c>
       <c r="E94" t="str">
-        <v>7.5</v>
+        <v>3.43</v>
       </c>
       <c r="F94" t="str">
-        <v>7.5</v>
+        <v>3.43</v>
       </c>
       <c r="G94" t="str">
-        <v>7.5</v>
+        <v>3.43</v>
       </c>
       <c r="H94" t="str">
         <v/>
@@ -5930,22 +5963,22 @@
         <v>2025-09-04</v>
       </c>
       <c r="B95" t="str">
-        <v>McGhie (NL) (GH), Cheryl</v>
+        <v>Lamont (NL) (GH), Sophie</v>
       </c>
       <c r="C95" t="str">
         <v>Available</v>
       </c>
       <c r="D95" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E95" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F95" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G95" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H95" t="str">
         <v/>
@@ -5956,22 +5989,22 @@
         <v>2025-09-04</v>
       </c>
       <c r="B96" t="str">
-        <v>Nelson (NL), Anne</v>
+        <v>McGhie (NL) (GH), Cheryl</v>
       </c>
       <c r="C96" t="str">
         <v>Available</v>
       </c>
       <c r="D96" t="str">
-        <v>08:00-17:15</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E96" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="F96" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="G96" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="H96" t="str">
         <v/>
@@ -5982,22 +6015,22 @@
         <v>2025-09-04</v>
       </c>
       <c r="B97" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Nelson (NL), Anne</v>
       </c>
       <c r="C97" t="str">
         <v>Available</v>
       </c>
       <c r="D97" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-17:15</v>
       </c>
       <c r="E97" t="str">
-        <v>2.67</v>
+        <v>5.33</v>
       </c>
       <c r="F97" t="str">
-        <v>2.67</v>
+        <v>5.33</v>
       </c>
       <c r="G97" t="str">
-        <v>2.67</v>
+        <v>5.33</v>
       </c>
       <c r="H97" t="str">
         <v/>
@@ -6008,7 +6041,7 @@
         <v>2025-09-04</v>
       </c>
       <c r="B98" t="str">
-        <v>Wylie (NL), Lori</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C98" t="str">
         <v>Available</v>
@@ -6017,21 +6050,47 @@
         <v>09:15-14:00</v>
       </c>
       <c r="E98" t="str">
-        <v>6</v>
+        <v>2.67</v>
       </c>
       <c r="F98" t="str">
-        <v>6</v>
+        <v>2.67</v>
       </c>
       <c r="G98" t="str">
-        <v>6</v>
+        <v>2.67</v>
       </c>
       <c r="H98" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>2025-09-04</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Wylie (NL), Lori</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D99" t="str">
+        <v>09:15-14:00</v>
+      </c>
+      <c r="E99" t="str">
+        <v>6</v>
+      </c>
+      <c r="F99" t="str">
+        <v>6</v>
+      </c>
+      <c r="G99" t="str">
+        <v>6</v>
+      </c>
+      <c r="H99" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H98"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H99"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adjust data processing to match exact total hours
Update server/pipeline.ts to remove proportional scaling of demand hours and log total demand hours from filtering for verification against the expected 400.33.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ae21854f-56f0-4406-b430-4b525fbb8b36
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/ae21854f-56f0-4406-b430-4b525fbb8b36/FXftk5h
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3334,10 +3334,10 @@
         <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>77.55</v>
+        <v>72.91</v>
       </c>
       <c r="G2" t="str">
-        <v>-20.72</v>
+        <v>-16.08</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -3360,10 +3360,10 @@
         <v>0</v>
       </c>
       <c r="F3" t="str">
-        <v>78.36</v>
+        <v>73.67</v>
       </c>
       <c r="G3" t="str">
-        <v>-5.79</v>
+        <v>-1.1</v>
       </c>
       <c r="H3" t="str">
         <v>Shortage</v>
@@ -3386,10 +3386,10 @@
         <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>69.07</v>
+        <v>64.94</v>
       </c>
       <c r="G4" t="str">
-        <v>3.5</v>
+        <v>7.63</v>
       </c>
       <c r="H4" t="str">
         <v>Sufficient</v>
@@ -3412,10 +3412,10 @@
         <v>0</v>
       </c>
       <c r="F5" t="str">
-        <v>66.58</v>
+        <v>62.6</v>
       </c>
       <c r="G5" t="str">
-        <v>11.42</v>
+        <v>15.4</v>
       </c>
       <c r="H5" t="str">
         <v>Sufficient</v>
@@ -3438,10 +3438,10 @@
         <v>12.43</v>
       </c>
       <c r="F6" t="str">
-        <v>51.5</v>
+        <v>48.42</v>
       </c>
       <c r="G6" t="str">
-        <v>11.4</v>
+        <v>14.48</v>
       </c>
       <c r="H6" t="str">
         <v>Sufficient</v>
@@ -3464,10 +3464,10 @@
         <v>12.43</v>
       </c>
       <c r="F7" t="str">
-        <v>42.75</v>
+        <v>40.19</v>
       </c>
       <c r="G7" t="str">
-        <v>-12.58</v>
+        <v>-10.02</v>
       </c>
       <c r="H7" t="str">
         <v>Shortage</v>
@@ -3490,10 +3490,10 @@
         <v>3.43</v>
       </c>
       <c r="F8" t="str">
-        <v>40</v>
+        <v>37.61</v>
       </c>
       <c r="G8" t="str">
-        <v>-7.17</v>
+        <v>-4.78</v>
       </c>
       <c r="H8" t="str">
         <v>Shortage</v>

</xml_diff>

<commit_message>
Improve service delivery data processing for better insights
Add logging to the service delivery parsing function in `server/pipeline.ts` to display service types and details of the first 5 records for debugging purposes.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ae21854f-56f0-4406-b430-4b525fbb8b36
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/ae21854f-56f0-4406-b430-4b525fbb8b36/sfjbFC1
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3334,10 +3334,10 @@
         <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>72.91</v>
+        <v>77.55</v>
       </c>
       <c r="G2" t="str">
-        <v>-16.08</v>
+        <v>-20.72</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -3360,10 +3360,10 @@
         <v>0</v>
       </c>
       <c r="F3" t="str">
-        <v>73.67</v>
+        <v>78.36</v>
       </c>
       <c r="G3" t="str">
-        <v>-1.1</v>
+        <v>-5.79</v>
       </c>
       <c r="H3" t="str">
         <v>Shortage</v>
@@ -3386,10 +3386,10 @@
         <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>64.94</v>
+        <v>69.07</v>
       </c>
       <c r="G4" t="str">
-        <v>7.63</v>
+        <v>3.5</v>
       </c>
       <c r="H4" t="str">
         <v>Sufficient</v>
@@ -3412,10 +3412,10 @@
         <v>0</v>
       </c>
       <c r="F5" t="str">
-        <v>62.6</v>
+        <v>66.58</v>
       </c>
       <c r="G5" t="str">
-        <v>15.4</v>
+        <v>11.42</v>
       </c>
       <c r="H5" t="str">
         <v>Sufficient</v>
@@ -3438,10 +3438,10 @@
         <v>12.43</v>
       </c>
       <c r="F6" t="str">
-        <v>48.42</v>
+        <v>51.5</v>
       </c>
       <c r="G6" t="str">
-        <v>14.48</v>
+        <v>11.4</v>
       </c>
       <c r="H6" t="str">
         <v>Sufficient</v>
@@ -3464,10 +3464,10 @@
         <v>12.43</v>
       </c>
       <c r="F7" t="str">
-        <v>40.19</v>
+        <v>42.75</v>
       </c>
       <c r="G7" t="str">
-        <v>-10.02</v>
+        <v>-12.58</v>
       </c>
       <c r="H7" t="str">
         <v>Shortage</v>
@@ -3490,10 +3490,10 @@
         <v>3.43</v>
       </c>
       <c r="F8" t="str">
-        <v>37.61</v>
+        <v>40</v>
       </c>
       <c r="G8" t="str">
-        <v>-4.78</v>
+        <v>-7.17</v>
       </c>
       <c r="H8" t="str">
         <v>Shortage</v>

</xml_diff>

<commit_message>
Update capacity dashboard spreadsheet
Updated the capacity dashboard spreadsheet with new data.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ae21854f-56f0-4406-b430-4b525fbb8b36
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/ae21854f-56f0-4406-b430-4b525fbb8b36/VZ5bqQe
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3334,10 +3334,10 @@
         <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>77.55</v>
+        <v>64.5</v>
       </c>
       <c r="G2" t="str">
-        <v>-20.72</v>
+        <v>-7.67</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -3360,13 +3360,13 @@
         <v>0</v>
       </c>
       <c r="F3" t="str">
-        <v>78.36</v>
+        <v>65.25</v>
       </c>
       <c r="G3" t="str">
-        <v>-5.79</v>
+        <v>7.32</v>
       </c>
       <c r="H3" t="str">
-        <v>Shortage</v>
+        <v>Sufficient</v>
       </c>
     </row>
     <row r="4">
@@ -3386,10 +3386,10 @@
         <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>69.07</v>
+        <v>69.75</v>
       </c>
       <c r="G4" t="str">
-        <v>3.5</v>
+        <v>2.82</v>
       </c>
       <c r="H4" t="str">
         <v>Sufficient</v>

</xml_diff>

<commit_message>
Improve data filtering and processing for guaranteed hours
Update filtering logic for guaranteed hours data to accurately exclude cancelled entries and specific secondary care types, and refine timestamp resolution using a fallback priority system (Service Requirement, Actual, Planned).

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a879ae68-84fc-4594-b56e-c187951a080e
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/a879ae68-84fc-4594-b56e-c187951a080e/WqNP8CB
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3092,10 +3092,10 @@
         <v>0</v>
       </c>
       <c r="F5" t="str">
-        <v>57.75</v>
+        <v>28.88</v>
       </c>
       <c r="G5" t="str">
-        <v>3.02</v>
+        <v>31.89</v>
       </c>
       <c r="H5" t="str">
         <v>Sufficient</v>

</xml_diff>

<commit_message>
Restore previous rules and configurations for capacity dashboard data
Revert changes made to the capacity_dashboard.xlsx file, restoring original rules and configurations.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a879ae68-84fc-4594-b56e-c187951a080e
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/a879ae68-84fc-4594-b56e-c187951a080e/WqNP8CB
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3092,10 +3092,10 @@
         <v>0</v>
       </c>
       <c r="F5" t="str">
-        <v>28.88</v>
+        <v>57.75</v>
       </c>
       <c r="G5" t="str">
-        <v>31.89</v>
+        <v>3.02</v>
       </c>
       <c r="H5" t="str">
         <v>Sufficient</v>

</xml_diff>

<commit_message>
Hide available hours column in employee details view
Removes the 'Available Hours' column and its corresponding cell data from the employee details table in the dashboard, adjusting the column span for the 'no data' message.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: a082e99a-71e6-4dbf-affd-374f87ef8d86
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/a082e99a-71e6-4dbf-affd-374f87ef8d86/QF1IHiD
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -436,350 +436,349 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="B2" t="str">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C2" t="str">
-        <v>2.67</v>
+        <v>4.8</v>
       </c>
       <c r="D2" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E2" t="str">
-        <v>Sick</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="F2" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-16:15</v>
       </c>
       <c r="G2" t="str">
-        <v>2.67</v>
+        <v>2</v>
       </c>
       <c r="H2" t="str">
         <v>0</v>
       </c>
       <c r="I2" t="str">
-        <v>Brooke advised that her previous appointment was cancelled and that it has been rescheduled. SM; Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM; Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>Sharon has advised she is unable to work between 10.30 and 12.30 on Tuesday's - MT</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
       <c r="A3" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="B3" t="str">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C3" t="str">
-        <v>2.67</v>
+        <v>4.8</v>
       </c>
       <c r="D3" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E3" t="str">
-        <v>Sick</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="F3" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-16:30</v>
       </c>
       <c r="G3" t="str">
-        <v>2.67</v>
+        <v>2</v>
       </c>
       <c r="H3" t="str">
         <v>0</v>
       </c>
-      <c r="I3" t="str">
-        <v>Brooke advised that her previous appointment was cancelled and that it has been rescheduled. SM; Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM; Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
-      </c>
-    </row>
-    <row r="4">
+      <c r="I3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Wants this as a break. 
+Eilidh 29/05/2025</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
       <c r="A4" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="B4" t="str">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C4" t="str">
-        <v>2.67</v>
+        <v>4.8</v>
       </c>
       <c r="D4" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E4" t="str">
-        <v>Sick</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="F4" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-17:00</v>
       </c>
       <c r="G4" t="str">
-        <v>2.67</v>
+        <v>2</v>
       </c>
       <c r="H4" t="str">
         <v>0</v>
       </c>
-      <c r="I4" t="str">
-        <v>Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM; Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
-      </c>
-    </row>
-    <row r="5" xml:space="preserve">
+      <c r="I4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Wants this as a break. 
+Eilidh 29/05/2025</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" t="str">
-        <v>Asokhia (NL), Deborah</v>
+        <v>Forbes (NL) (GH), Amanda</v>
       </c>
       <c r="B5" t="str">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C5" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="D5" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E5" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="F5" t="str">
-        <v>08:00-15:00</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="G5" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="H5" t="str">
-        <v>0</v>
-      </c>
-      <c r="I5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Agreed at induction with MT and SM - 09/05/2025; Has appointment and is unable to work 
-Eilidh 22/08/2025</v>
-      </c>
-    </row>
-    <row r="6" xml:space="preserve">
+        <v>3.2</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Confirmed at induction with MT</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" t="str">
-        <v>Mcewan (NL) (GH), Makala</v>
+        <v>Forbes (NL) (GH), Amanda</v>
       </c>
       <c r="B6" t="str">
         <v>16</v>
       </c>
       <c r="C6" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="D6" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E6" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="F6" t="str">
-        <v>08:00-15:15</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G6" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="H6" t="str">
-        <v>0</v>
-      </c>
-      <c r="I6" t="str" xml:space="preserve">
-        <v xml:space="preserve">Family event
-Eilidh 01/09/2025</v>
-      </c>
-    </row>
-    <row r="7" xml:space="preserve">
+        <v>3.2</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" t="str">
-        <v>Ferris (NL), Marykate</v>
+        <v>Forbes (NL) (GH), Amanda</v>
       </c>
       <c r="B7" t="str">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C7" t="str">
-        <v>6.67</v>
+        <v>3.2</v>
       </c>
       <c r="D7" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E7" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="F7" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G7" t="str">
-        <v>6.67</v>
+        <v>3.2</v>
       </c>
       <c r="H7" t="str">
-        <v>0</v>
-      </c>
-      <c r="I7" t="str" xml:space="preserve">
-        <v xml:space="preserve">Away for a family members birthday, tickets were already bought before checking
-Eilidh 01/09/2025</v>
+        <v>3.2</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Griffiths (NL), Wayne (GH)</v>
+        <v>Forbes (NL) (GH), Amanda</v>
       </c>
       <c r="B8" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C8" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D8" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E8" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="F8" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G8" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H8" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="I8" t="str">
-        <v>Wayne called to advise that his car had broke down and that he would not be returning until his car situation was sorted. SM</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Griffiths (NL), Wayne (GH)</v>
+        <v>Forbes (NL) (GH), Amanda</v>
       </c>
       <c r="B9" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C9" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D9" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E9" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="F9" t="str">
-        <v>08:00-21:30</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="G9" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H9" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="I9" t="str">
-        <v>Wayne called to advise that his car had broke down and that he would not be returning until his car situation was sorted. SM</v>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Forbes (NL) (GH), Amanda</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="B10" t="str">
         <v>16</v>
       </c>
       <c r="C10" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="D10" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E10" t="str">
         <v>Available</v>
       </c>
       <c r="F10" t="str">
-        <v>10:30-14:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G10" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="H10" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="I10" t="str">
-        <v>Confirmed at induction with MT</v>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Forbes (NL) (GH), Amanda</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="B11" t="str">
         <v>16</v>
       </c>
       <c r="C11" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="D11" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E11" t="str">
         <v>Available</v>
       </c>
       <c r="F11" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G11" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="H11" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="I11" t="str">
-        <v/>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Forbes (NL) (GH), Amanda</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="B12" t="str">
         <v>16</v>
       </c>
       <c r="C12" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="D12" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E12" t="str">
         <v>Available</v>
       </c>
       <c r="F12" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G12" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="H12" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Forbes (NL) (GH), Amanda</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="B13" t="str">
         <v>16</v>
       </c>
       <c r="C13" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="D13" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E13" t="str">
         <v>Available</v>
       </c>
       <c r="F13" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G13" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="H13" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="I13" t="str">
         <v/>
@@ -787,31 +786,31 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Forbes (NL) (GH), Amanda</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="B14" t="str">
         <v>16</v>
       </c>
       <c r="C14" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="D14" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-20</v>
       </c>
       <c r="E14" t="str">
         <v>Available</v>
       </c>
       <c r="F14" t="str">
-        <v>10:30-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G14" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="H14" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="I14" t="str">
-        <v>Confirmed at induction with MT</v>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -825,7 +824,7 @@
         <v>2.67</v>
       </c>
       <c r="D15" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-21</v>
       </c>
       <c r="E15" t="str">
         <v>Available</v>
@@ -845,16 +844,16 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Asokhia (NL), Deborah</v>
       </c>
       <c r="B16" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C16" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="D16" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E16" t="str">
         <v>Available</v>
@@ -863,42 +862,42 @@
         <v>09:15-14:00</v>
       </c>
       <c r="G16" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="H16" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="I16" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Asokhia (NL), Deborah</v>
       </c>
       <c r="B17" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C17" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="D17" t="str">
-        <v>2025-09-13</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E17" t="str">
         <v>Available</v>
       </c>
       <c r="F17" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G17" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="H17" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="I17" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="18">
@@ -912,7 +911,7 @@
         <v>4</v>
       </c>
       <c r="D18" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E18" t="str">
         <v>Available</v>
@@ -941,7 +940,7 @@
         <v>4</v>
       </c>
       <c r="D19" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E19" t="str">
         <v>Available</v>
@@ -970,7 +969,7 @@
         <v>4</v>
       </c>
       <c r="D20" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E20" t="str">
         <v>Available</v>
@@ -990,115 +989,115 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Asokhia (NL), Deborah</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="B21" t="str">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C21" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="D21" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E21" t="str">
         <v>Available</v>
       </c>
       <c r="F21" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="G21" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="H21" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="I21" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Shawcross (NL), Emma</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="B22" t="str">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C22" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="D22" t="str">
-        <v>2025-09-13</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E22" t="str">
         <v>Available</v>
       </c>
       <c r="F22" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-11:30</v>
       </c>
       <c r="G22" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="H22" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="I22" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Shawcross (NL), Emma</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="B23" t="str">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C23" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="D23" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E23" t="str">
         <v>Available</v>
       </c>
       <c r="F23" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="G23" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="H23" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="I23" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="B24" t="str">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="C24" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="D24" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E24" t="str">
         <v>Available</v>
       </c>
       <c r="F24" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-11:30</v>
       </c>
       <c r="G24" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="H24" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="I24" t="str">
         <v/>
@@ -1106,28 +1105,28 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="B25" t="str">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="C25" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="D25" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E25" t="str">
         <v>Available</v>
       </c>
       <c r="F25" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G25" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="H25" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="I25" t="str">
         <v/>
@@ -1135,16 +1134,16 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Shawcross (NL), Emma</v>
       </c>
       <c r="B26" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C26" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="D26" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-20</v>
       </c>
       <c r="E26" t="str">
         <v>Available</v>
@@ -1153,27 +1152,27 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G26" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="H26" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="I26" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Shawcross (NL), Emma</v>
       </c>
       <c r="B27" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C27" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="D27" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-21</v>
       </c>
       <c r="E27" t="str">
         <v>Available</v>
@@ -1182,39 +1181,39 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G27" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="H27" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="I27" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Duncan (NL), Madison</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="B28" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C28" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="D28" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E28" t="str">
         <v>Available</v>
       </c>
       <c r="F28" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G28" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="H28" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="I28" t="str">
         <v/>
@@ -1222,28 +1221,28 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Duncan (NL), Madison</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="B29" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C29" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="D29" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E29" t="str">
         <v>Available</v>
       </c>
       <c r="F29" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G29" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="H29" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="I29" t="str">
         <v/>
@@ -1251,28 +1250,28 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Mcewan (NL) (GH), Makala</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="B30" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C30" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="D30" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-20</v>
       </c>
       <c r="E30" t="str">
         <v>Available</v>
       </c>
       <c r="F30" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G30" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="H30" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="I30" t="str">
         <v/>
@@ -1280,28 +1279,28 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Mcewan (NL) (GH), Makala</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="B31" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C31" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="D31" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-21</v>
       </c>
       <c r="E31" t="str">
         <v>Available</v>
       </c>
       <c r="F31" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G31" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="H31" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="I31" t="str">
         <v/>
@@ -1318,7 +1317,7 @@
         <v>4</v>
       </c>
       <c r="D32" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E32" t="str">
         <v>Available</v>
@@ -1338,28 +1337,28 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Ferris (NL), Marykate</v>
+        <v>Mcewan (NL) (GH), Makala</v>
       </c>
       <c r="B33" t="str">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C33" t="str">
-        <v>6.67</v>
+        <v>4</v>
       </c>
       <c r="D33" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E33" t="str">
         <v>Available</v>
       </c>
       <c r="F33" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="G33" t="str">
-        <v>6.67</v>
+        <v>4</v>
       </c>
       <c r="H33" t="str">
-        <v>6.67</v>
+        <v>4</v>
       </c>
       <c r="I33" t="str">
         <v/>
@@ -1367,28 +1366,28 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Ferris (NL), Marykate</v>
+        <v>Mcewan (NL) (GH), Makala</v>
       </c>
       <c r="B34" t="str">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C34" t="str">
-        <v>6.67</v>
+        <v>4</v>
       </c>
       <c r="D34" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-20</v>
       </c>
       <c r="E34" t="str">
         <v>Available</v>
       </c>
       <c r="F34" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="G34" t="str">
-        <v>6.67</v>
+        <v>4</v>
       </c>
       <c r="H34" t="str">
-        <v>6.67</v>
+        <v>4</v>
       </c>
       <c r="I34" t="str">
         <v/>
@@ -1396,28 +1395,28 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Mcewan (NL) (GH), Makala</v>
       </c>
       <c r="B35" t="str">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="C35" t="str">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D35" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-21</v>
       </c>
       <c r="E35" t="str">
         <v>Available</v>
       </c>
       <c r="F35" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="G35" t="str">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H35" t="str">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I35" t="str">
         <v/>
@@ -1425,28 +1424,28 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Lamont (NL) (GH), Sophie</v>
       </c>
       <c r="B36" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C36" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="D36" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E36" t="str">
         <v>Available</v>
       </c>
       <c r="F36" t="str">
-        <v>08:00-21:30</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G36" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H36" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="I36" t="str">
         <v/>
@@ -1454,16 +1453,16 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Lamont (NL) (GH), Sophie</v>
       </c>
       <c r="B37" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C37" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="D37" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E37" t="str">
         <v>Available</v>
@@ -1472,10 +1471,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G37" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H37" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="I37" t="str">
         <v/>
@@ -1483,16 +1482,16 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Lamont (NL) (GH), Sophie</v>
       </c>
       <c r="B38" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C38" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="D38" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E38" t="str">
         <v>Available</v>
@@ -1501,10 +1500,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G38" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H38" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="I38" t="str">
         <v/>
@@ -1512,16 +1511,16 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Lamont (NL) (GH), Sophie</v>
       </c>
       <c r="B39" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C39" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="D39" t="str">
-        <v>2025-09-13</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E39" t="str">
         <v>Available</v>
@@ -1530,10 +1529,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G39" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H39" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="I39" t="str">
         <v/>
@@ -1541,7 +1540,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Lamont (NL) (GH), Sophie</v>
+        <v>Adeyanju (NL) (GH), Adedayo</v>
       </c>
       <c r="B40" t="str">
         <v>30</v>
@@ -1550,7 +1549,7 @@
         <v>7.5</v>
       </c>
       <c r="D40" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E40" t="str">
         <v>Available</v>
@@ -1570,7 +1569,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Lamont (NL) (GH), Sophie</v>
+        <v>Adeyanju (NL) (GH), Adedayo</v>
       </c>
       <c r="B41" t="str">
         <v>30</v>
@@ -1579,13 +1578,13 @@
         <v>7.5</v>
       </c>
       <c r="D41" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E41" t="str">
         <v>Available</v>
       </c>
       <c r="F41" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G41" t="str">
         <v>7.5</v>
@@ -1599,7 +1598,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Lamont (NL) (GH), Sophie</v>
+        <v>Adeyanju (NL) (GH), Adedayo</v>
       </c>
       <c r="B42" t="str">
         <v>30</v>
@@ -1608,7 +1607,7 @@
         <v>7.5</v>
       </c>
       <c r="D42" t="str">
-        <v>2025-09-13</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E42" t="str">
         <v>Available</v>
@@ -1628,7 +1627,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Lamont (NL) (GH), Sophie</v>
+        <v>Adeyanju (NL) (GH), Adedayo</v>
       </c>
       <c r="B43" t="str">
         <v>30</v>
@@ -1637,7 +1636,7 @@
         <v>7.5</v>
       </c>
       <c r="D43" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E43" t="str">
         <v>Available</v>
@@ -1657,16 +1656,16 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Adeyanju (NL) (GH), Adedayo</v>
+        <v>Hussain (NL) (GH), Mustansar</v>
       </c>
       <c r="B44" t="str">
         <v>30</v>
       </c>
       <c r="C44" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D44" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E44" t="str">
         <v>Available</v>
@@ -1675,10 +1674,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G44" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H44" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="I44" t="str">
         <v/>
@@ -1686,16 +1685,16 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Adeyanju (NL) (GH), Adedayo</v>
+        <v>Hussain (NL) (GH), Mustansar</v>
       </c>
       <c r="B45" t="str">
         <v>30</v>
       </c>
       <c r="C45" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D45" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E45" t="str">
         <v>Available</v>
@@ -1704,10 +1703,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G45" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H45" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="I45" t="str">
         <v/>
@@ -1715,16 +1714,16 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Adeyanju (NL) (GH), Adedayo</v>
+        <v>Hussain (NL) (GH), Mustansar</v>
       </c>
       <c r="B46" t="str">
         <v>30</v>
       </c>
       <c r="C46" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D46" t="str">
-        <v>2025-09-13</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E46" t="str">
         <v>Available</v>
@@ -1733,10 +1732,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G46" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H46" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="I46" t="str">
         <v/>
@@ -1744,16 +1743,16 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Adeyanju (NL) (GH), Adedayo</v>
+        <v>Hussain (NL) (GH), Mustansar</v>
       </c>
       <c r="B47" t="str">
         <v>30</v>
       </c>
       <c r="C47" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D47" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E47" t="str">
         <v>Available</v>
@@ -1762,10 +1761,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G47" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H47" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="I47" t="str">
         <v/>
@@ -1782,7 +1781,7 @@
         <v>6</v>
       </c>
       <c r="D48" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-20</v>
       </c>
       <c r="E48" t="str">
         <v>Available</v>
@@ -1802,118 +1801,118 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Hussain (NL) (GH), Mustansar</v>
+        <v>Ibrahim (NL), Olusegun Isaac</v>
       </c>
       <c r="B49" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C49" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D49" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E49" t="str">
         <v>Available</v>
       </c>
       <c r="F49" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="G49" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H49" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I49" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Hussain (NL) (GH), Mustansar</v>
+        <v>Ibrahim (NL), Olusegun Isaac</v>
       </c>
       <c r="B50" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C50" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D50" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E50" t="str">
         <v>Available</v>
       </c>
       <c r="F50" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="G50" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H50" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I50" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Hussain (NL) (GH), Mustansar</v>
+        <v>Ibrahim (NL), Olusegun Isaac</v>
       </c>
       <c r="B51" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C51" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D51" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E51" t="str">
         <v>Available</v>
       </c>
       <c r="F51" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="G51" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H51" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I51" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Hussain (NL) (GH), Mustansar</v>
+        <v>Ibrahim (NL), Olusegun Isaac</v>
       </c>
       <c r="B52" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C52" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D52" t="str">
-        <v>2025-09-13</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E52" t="str">
         <v>Available</v>
       </c>
       <c r="F52" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="G52" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H52" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I52" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="53">
@@ -1927,7 +1926,7 @@
         <v>3.2</v>
       </c>
       <c r="D53" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E53" t="str">
         <v>Available</v>
@@ -1947,118 +1946,118 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Ibrahim (NL), Olusegun Isaac</v>
+        <v>Griffiths (NL), Wayne (GH)</v>
       </c>
       <c r="B54" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C54" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="D54" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E54" t="str">
         <v>Available</v>
       </c>
       <c r="F54" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G54" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H54" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="I54" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Ibrahim (NL), Olusegun Isaac</v>
+        <v>Griffiths (NL), Wayne (GH)</v>
       </c>
       <c r="B55" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C55" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="D55" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E55" t="str">
         <v>Available</v>
       </c>
       <c r="F55" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G55" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H55" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="I55" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Ibrahim (NL), Olusegun Isaac</v>
+        <v>Griffiths (NL), Wayne (GH)</v>
       </c>
       <c r="B56" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C56" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="D56" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E56" t="str">
         <v>Available</v>
       </c>
       <c r="F56" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G56" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H56" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="I56" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Ibrahim (NL), Olusegun Isaac</v>
+        <v>Griffiths (NL), Wayne (GH)</v>
       </c>
       <c r="B57" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C57" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="D57" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E57" t="str">
         <v>Available</v>
       </c>
       <c r="F57" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G57" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H57" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="I57" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="58">
@@ -2072,7 +2071,7 @@
         <v>6</v>
       </c>
       <c r="D58" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-21</v>
       </c>
       <c r="E58" t="str">
         <v>Available</v>
@@ -2092,28 +2091,28 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Griffiths (NL), Wayne (GH)</v>
+        <v>Nelson (NL), Anne</v>
       </c>
       <c r="B59" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C59" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="D59" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E59" t="str">
         <v>Available</v>
       </c>
       <c r="F59" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-17:15</v>
       </c>
       <c r="G59" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="H59" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="I59" t="str">
         <v/>
@@ -2121,28 +2120,28 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Griffiths (NL), Wayne (GH)</v>
+        <v>Nelson (NL), Anne</v>
       </c>
       <c r="B60" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C60" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="D60" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E60" t="str">
         <v>Available</v>
       </c>
       <c r="F60" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-13:00</v>
       </c>
       <c r="G60" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="H60" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="I60" t="str">
         <v/>
@@ -2159,13 +2158,13 @@
         <v>5.33</v>
       </c>
       <c r="D61" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-21</v>
       </c>
       <c r="E61" t="str">
         <v>Available</v>
       </c>
       <c r="F61" t="str">
-        <v>08:00-17:15</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="G61" t="str">
         <v>5.33</v>
@@ -2179,28 +2178,28 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Nelson (NL), Anne</v>
+        <v>McGhie (NL) (GH), Cheryl</v>
       </c>
       <c r="B62" t="str">
         <v>16</v>
       </c>
       <c r="C62" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="D62" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E62" t="str">
         <v>Available</v>
       </c>
       <c r="F62" t="str">
-        <v>08:00-13:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G62" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="H62" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="I62" t="str">
         <v/>
@@ -2208,28 +2207,28 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Nelson (NL), Anne</v>
+        <v>McGhie (NL) (GH), Cheryl</v>
       </c>
       <c r="B63" t="str">
         <v>16</v>
       </c>
       <c r="C63" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="D63" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E63" t="str">
         <v>Available</v>
       </c>
       <c r="F63" t="str">
-        <v>08:00-18:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G63" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="H63" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="I63" t="str">
         <v/>
@@ -2246,7 +2245,7 @@
         <v>3.2</v>
       </c>
       <c r="D64" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E64" t="str">
         <v>Available</v>
@@ -2275,7 +2274,7 @@
         <v>3.2</v>
       </c>
       <c r="D65" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E65" t="str">
         <v>Available</v>
@@ -2304,7 +2303,7 @@
         <v>3.2</v>
       </c>
       <c r="D66" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E66" t="str">
         <v>Available</v>
@@ -2324,28 +2323,28 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>McGhie (NL) (GH), Cheryl</v>
+        <v>Mooney (NL), Lynsey (GH)</v>
       </c>
       <c r="B67" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C67" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="D67" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E67" t="str">
         <v>Available</v>
       </c>
       <c r="F67" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="G67" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="H67" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="I67" t="str">
         <v/>
@@ -2353,28 +2352,28 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>McGhie (NL) (GH), Cheryl</v>
+        <v>Mooney (NL), Lynsey (GH)</v>
       </c>
       <c r="B68" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C68" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="D68" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E68" t="str">
         <v>Available</v>
       </c>
       <c r="F68" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="G68" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="H68" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="I68" t="str">
         <v/>
@@ -2391,7 +2390,7 @@
         <v>4</v>
       </c>
       <c r="D69" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E69" t="str">
         <v>Available</v>
@@ -2420,7 +2419,7 @@
         <v>4</v>
       </c>
       <c r="D70" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E70" t="str">
         <v>Available</v>
@@ -2449,13 +2448,13 @@
         <v>4</v>
       </c>
       <c r="D71" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E71" t="str">
         <v>Available</v>
       </c>
       <c r="F71" t="str">
-        <v>08:00-14:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="G71" t="str">
         <v>4</v>
@@ -2469,28 +2468,28 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Mooney (NL), Lynsey (GH)</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="B72" t="str">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C72" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="D72" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E72" t="str">
         <v>Available</v>
       </c>
       <c r="F72" t="str">
-        <v>08:00-15:00</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G72" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="H72" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="I72" t="str">
         <v/>
@@ -2498,28 +2497,28 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Mooney (NL), Lynsey (GH)</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="B73" t="str">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C73" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="D73" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E73" t="str">
         <v>Available</v>
       </c>
       <c r="F73" t="str">
-        <v>08:00-14:00</v>
+        <v>09:15-16:15</v>
       </c>
       <c r="G73" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="H73" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="I73" t="str">
         <v/>
@@ -2536,7 +2535,7 @@
         <v>6</v>
       </c>
       <c r="D74" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E74" t="str">
         <v>Available</v>
@@ -2565,7 +2564,7 @@
         <v>6</v>
       </c>
       <c r="D75" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E75" t="str">
         <v>Available</v>
@@ -2594,7 +2593,7 @@
         <v>6</v>
       </c>
       <c r="D76" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E76" t="str">
         <v>Available</v>
@@ -2623,7 +2622,7 @@
         <v>6</v>
       </c>
       <c r="D77" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E77" t="str">
         <v>Available</v>
@@ -2652,7 +2651,7 @@
         <v>6</v>
       </c>
       <c r="D78" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E78" t="str">
         <v>Available</v>
@@ -2709,25 +2708,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B2" t="str">
-        <v>52.6</v>
+        <v>57.37</v>
       </c>
       <c r="C2" t="str">
-        <v>52.6</v>
+        <v>57.37</v>
       </c>
       <c r="D2" t="str">
-        <v>8.67</v>
+        <v>0</v>
       </c>
       <c r="E2" t="str">
         <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>58.75</v>
+        <v>63.25</v>
       </c>
       <c r="G2" t="str">
-        <v>-6.15</v>
+        <v>-5.88</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -2735,51 +2734,51 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B3" t="str">
-        <v>69.1</v>
+        <v>63.57</v>
       </c>
       <c r="C3" t="str">
-        <v>69.1</v>
+        <v>63.57</v>
       </c>
       <c r="D3" t="str">
-        <v>8.67</v>
+        <v>2</v>
       </c>
       <c r="E3" t="str">
         <v>0</v>
       </c>
       <c r="F3" t="str">
-        <v>59.75</v>
+        <v>66.75</v>
       </c>
       <c r="G3" t="str">
-        <v>9.35</v>
+        <v>-3.18</v>
       </c>
       <c r="H3" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B4" t="str">
-        <v>62.77</v>
+        <v>60.07</v>
       </c>
       <c r="C4" t="str">
-        <v>62.77</v>
+        <v>60.07</v>
       </c>
       <c r="D4" t="str">
-        <v>2.67</v>
+        <v>2</v>
       </c>
       <c r="E4" t="str">
         <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>69.75</v>
+        <v>71.25</v>
       </c>
       <c r="G4" t="str">
-        <v>-6.98</v>
+        <v>-11.18</v>
       </c>
       <c r="H4" t="str">
         <v>Shortage</v>
@@ -2787,65 +2786,65 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B5" t="str">
-        <v>60.77</v>
+        <v>60.2</v>
       </c>
       <c r="C5" t="str">
-        <v>60.77</v>
+        <v>60.2</v>
       </c>
       <c r="D5" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E5" t="str">
         <v>0</v>
       </c>
       <c r="F5" t="str">
-        <v>57.75</v>
+        <v>61.75</v>
       </c>
       <c r="G5" t="str">
-        <v>3.02</v>
+        <v>-1.55</v>
       </c>
       <c r="H5" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-19</v>
       </c>
       <c r="B6" t="str">
-        <v>54.1</v>
+        <v>52.73</v>
       </c>
       <c r="C6" t="str">
-        <v>54.1</v>
+        <v>52.73</v>
       </c>
       <c r="D6" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E6" t="str">
         <v>0</v>
       </c>
       <c r="F6" t="str">
-        <v>53.75</v>
+        <v>56.75</v>
       </c>
       <c r="G6" t="str">
-        <v>0.35</v>
+        <v>-4.02</v>
       </c>
       <c r="H6" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2025-09-13</v>
+        <v>2025-09-20</v>
       </c>
       <c r="B7" t="str">
-        <v>42.67</v>
+        <v>30.17</v>
       </c>
       <c r="C7" t="str">
-        <v>42.67</v>
+        <v>30.17</v>
       </c>
       <c r="D7" t="str">
         <v>0</v>
@@ -2854,10 +2853,10 @@
         <v>0</v>
       </c>
       <c r="F7" t="str">
-        <v>46.75</v>
+        <v>45.75</v>
       </c>
       <c r="G7" t="str">
-        <v>-4.08</v>
+        <v>-15.58</v>
       </c>
       <c r="H7" t="str">
         <v>Shortage</v>
@@ -2865,16 +2864,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-21</v>
       </c>
       <c r="B8" t="str">
-        <v>40.33</v>
+        <v>35.5</v>
       </c>
       <c r="C8" t="str">
-        <v>40.33</v>
+        <v>35.5</v>
       </c>
       <c r="D8" t="str">
-        <v>6.67</v>
+        <v>0</v>
       </c>
       <c r="E8" t="str">
         <v>0</v>
@@ -2883,7 +2882,7 @@
         <v>43</v>
       </c>
       <c r="G8" t="str">
-        <v>-2.67</v>
+        <v>-7.5</v>
       </c>
       <c r="H8" t="str">
         <v>Shortage</v>
@@ -2928,7 +2927,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B2" t="str">
         <v>Adeyanju (NL) (GH), Adedayo</v>
@@ -2954,7 +2953,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B3" t="str">
         <v>Asokhia (NL), Deborah</v>
@@ -2980,25 +2979,25 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B4" t="str">
-        <v>Duncan (NL), Madison</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="C4" t="str">
         <v>Available</v>
       </c>
       <c r="D4" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E4" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="F4" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="G4" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="H4" t="str">
         <v/>
@@ -3006,7 +3005,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B5" t="str">
         <v>Forbes (NL) (GH), Amanda</v>
@@ -3015,7 +3014,7 @@
         <v>Available</v>
       </c>
       <c r="D5" t="str">
-        <v>10:30-14:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E5" t="str">
         <v>3.2</v>
@@ -3027,41 +3026,41 @@
         <v>3.2</v>
       </c>
       <c r="H5" t="str">
-        <v>Confirmed at induction with MT</v>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B6" t="str">
-        <v>Griffiths (NL), Wayne (GH)</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="C6" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D6" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-11:30</v>
       </c>
       <c r="E6" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="F6" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="G6" t="str">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="H6" t="str">
-        <v>Wayne called to advise that his car had broke down and that he would not be returning until his car situation was sorted. SM</v>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B7" t="str">
-        <v>Hussain (NL) (GH), Mustansar</v>
+        <v>Griffiths (NL), Wayne (GH)</v>
       </c>
       <c r="C7" t="str">
         <v>Available</v>
@@ -3084,103 +3083,103 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B8" t="str">
-        <v>Ibrahim (NL), Olusegun Isaac</v>
+        <v>Hussain (NL) (GH), Mustansar</v>
       </c>
       <c r="C8" t="str">
         <v>Available</v>
       </c>
       <c r="D8" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E8" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="F8" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="G8" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H8" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B9" t="str">
-        <v>Lamont (NL) (GH), Sophie</v>
+        <v>Ibrahim (NL), Olusegun Isaac</v>
       </c>
       <c r="C9" t="str">
         <v>Available</v>
       </c>
       <c r="D9" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="E9" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="F9" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="G9" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="H9" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B10" t="str">
-        <v>McGhie (NL) (GH), Cheryl</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="C10" t="str">
-        <v>Available</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D10" t="str">
-        <v>16:45-21:30</v>
+        <v>09:15-16:15</v>
       </c>
       <c r="E10" t="str">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="F10" t="str">
-        <v>3.2</v>
+        <v>2</v>
       </c>
       <c r="G10" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H10" t="str">
-        <v/>
+        <v>Sharon has advised she is unable to work between 10.30 and 12.30 on Tuesday's - MT</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B11" t="str">
-        <v>Mooney (NL), Lynsey (GH)</v>
+        <v>Lamont (NL) (GH), Sophie</v>
       </c>
       <c r="C11" t="str">
         <v>Available</v>
       </c>
       <c r="D11" t="str">
-        <v>08:00-15:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E11" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="F11" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="G11" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -3188,51 +3187,51 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B12" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>McGhie (NL) (GH), Cheryl</v>
       </c>
       <c r="C12" t="str">
-        <v>Sick</v>
+        <v>Available</v>
       </c>
       <c r="D12" t="str">
-        <v>08:00-21:30</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E12" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="F12" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="G12" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H12" t="str">
-        <v>Brooke advised that her previous appointment was cancelled and that it has been rescheduled. SM; Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM; Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2025-09-08</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B13" t="str">
-        <v>Wylie (NL), Lori</v>
+        <v>Mooney (NL), Lynsey (GH)</v>
       </c>
       <c r="C13" t="str">
         <v>Available</v>
       </c>
       <c r="D13" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E13" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F13" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G13" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H13" t="str">
         <v/>
@@ -3240,36 +3239,36 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B14" t="str">
-        <v>Adeyanju (NL) (GH), Adedayo</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C14" t="str">
         <v>Available</v>
       </c>
       <c r="D14" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E14" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="F14" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="G14" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-16</v>
       </c>
       <c r="B15" t="str">
-        <v>Asokhia (NL), Deborah</v>
+        <v>Wylie (NL), Lori</v>
       </c>
       <c r="C15" t="str">
         <v>Available</v>
@@ -3278,24 +3277,24 @@
         <v>09:15-14:00</v>
       </c>
       <c r="E15" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F15" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G15" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H15" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B16" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Adeyanju (NL) (GH), Adedayo</v>
       </c>
       <c r="C16" t="str">
         <v>Available</v>
@@ -3318,51 +3317,51 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B17" t="str">
-        <v>Duncan (NL), Madison</v>
+        <v>Asokhia (NL), Deborah</v>
       </c>
       <c r="C17" t="str">
         <v>Available</v>
       </c>
       <c r="D17" t="str">
-        <v>08:00-18:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E17" t="str">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F17" t="str">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G17" t="str">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H17" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B18" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Forbes (NL) (GH), Amanda</v>
       </c>
       <c r="C18" t="str">
         <v>Available</v>
       </c>
       <c r="D18" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E18" t="str">
-        <v>9</v>
+        <v>3.2</v>
       </c>
       <c r="F18" t="str">
-        <v>9</v>
+        <v>3.2</v>
       </c>
       <c r="G18" t="str">
-        <v>9</v>
+        <v>3.2</v>
       </c>
       <c r="H18" t="str">
         <v/>
@@ -3370,25 +3369,25 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B19" t="str">
-        <v>Forbes (NL) (GH), Amanda</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="C19" t="str">
         <v>Available</v>
       </c>
       <c r="D19" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="E19" t="str">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="F19" t="str">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="G19" t="str">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="H19" t="str">
         <v/>
@@ -3396,13 +3395,13 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B20" t="str">
         <v>Griffiths (NL), Wayne (GH)</v>
       </c>
       <c r="C20" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D20" t="str">
         <v>08:00-21:30</v>
@@ -3414,15 +3413,15 @@
         <v>6</v>
       </c>
       <c r="G20" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H20" t="str">
-        <v>Wayne called to advise that his car had broke down and that he would not be returning until his car situation was sorted. SM</v>
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B21" t="str">
         <v>Hussain (NL) (GH), Mustansar</v>
@@ -3448,7 +3447,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B22" t="str">
         <v>Ibrahim (NL), Olusegun Isaac</v>
@@ -3472,53 +3471,54 @@
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" xml:space="preserve">
       <c r="A23" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B23" t="str">
-        <v>Lamont (NL) (GH), Sophie</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="C23" t="str">
-        <v>Available</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D23" t="str">
-        <v>08:00-15:15</v>
+        <v>09:15-16:30</v>
       </c>
       <c r="E23" t="str">
-        <v>7.5</v>
+        <v>4.8</v>
       </c>
       <c r="F23" t="str">
-        <v>7.5</v>
+        <v>2</v>
       </c>
       <c r="G23" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H23" t="str">
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="H23" t="str" xml:space="preserve">
+        <v xml:space="preserve">Wants this as a break. 
+Eilidh 29/05/2025</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B24" t="str">
-        <v>McGhie (NL) (GH), Cheryl</v>
+        <v>Lamont (NL) (GH), Sophie</v>
       </c>
       <c r="C24" t="str">
         <v>Available</v>
       </c>
       <c r="D24" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E24" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F24" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G24" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H24" t="str">
         <v/>
@@ -3526,16 +3526,16 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B25" t="str">
-        <v>Mooney (NL), Lynsey (GH)</v>
+        <v>Mcewan (NL) (GH), Makala</v>
       </c>
       <c r="C25" t="str">
         <v>Available</v>
       </c>
       <c r="D25" t="str">
-        <v>08:00-15:00</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="E25" t="str">
         <v>4</v>
@@ -3552,51 +3552,51 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B26" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>McGhie (NL) (GH), Cheryl</v>
       </c>
       <c r="C26" t="str">
-        <v>Sick</v>
+        <v>Available</v>
       </c>
       <c r="D26" t="str">
-        <v>08:00-21:30</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E26" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="F26" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="G26" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H26" t="str">
-        <v>Brooke advised that her previous appointment was cancelled and that it has been rescheduled. SM; Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM; Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2025-09-09</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B27" t="str">
-        <v>Wylie (NL), Lori</v>
+        <v>Mooney (NL), Lynsey (GH)</v>
       </c>
       <c r="C27" t="str">
         <v>Available</v>
       </c>
       <c r="D27" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E27" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F27" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G27" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H27" t="str">
         <v/>
@@ -3604,10 +3604,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B28" t="str">
-        <v>Asokhia (NL), Deborah</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C28" t="str">
         <v>Available</v>
@@ -3616,39 +3616,39 @@
         <v>09:15-14:00</v>
       </c>
       <c r="E28" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="F28" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="G28" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="H28" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-17</v>
       </c>
       <c r="B29" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Wylie (NL), Lori</v>
       </c>
       <c r="C29" t="str">
         <v>Available</v>
       </c>
       <c r="D29" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="E29" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F29" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G29" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -3656,10 +3656,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="B30" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Adeyanju (NL) (GH), Adedayo</v>
       </c>
       <c r="C30" t="str">
         <v>Available</v>
@@ -3668,13 +3668,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E30" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="F30" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="G30" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H30" t="str">
         <v/>
@@ -3682,33 +3682,33 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="B31" t="str">
-        <v>Ferris (NL), Marykate</v>
+        <v>Asokhia (NL), Deborah</v>
       </c>
       <c r="C31" t="str">
         <v>Available</v>
       </c>
       <c r="D31" t="str">
-        <v>16:45-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E31" t="str">
-        <v>6.67</v>
+        <v>4</v>
       </c>
       <c r="F31" t="str">
-        <v>6.67</v>
+        <v>4</v>
       </c>
       <c r="G31" t="str">
-        <v>6.67</v>
+        <v>4</v>
       </c>
       <c r="H31" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="B32" t="str">
         <v>Forbes (NL) (GH), Amanda</v>
@@ -3717,7 +3717,7 @@
         <v>Available</v>
       </c>
       <c r="D32" t="str">
-        <v>09:15-15:15</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="E32" t="str">
         <v>3.2</v>
@@ -3729,30 +3729,30 @@
         <v>3.2</v>
       </c>
       <c r="H32" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="B33" t="str">
-        <v>Griffiths (NL), Wayne (GH)</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="C33" t="str">
         <v>Available</v>
       </c>
       <c r="D33" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E33" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="F33" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="G33" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="H33" t="str">
         <v/>
@@ -3760,7 +3760,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="B34" t="str">
         <v>Hussain (NL) (GH), Mustansar</v>
@@ -3786,7 +3786,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="B35" t="str">
         <v>Ibrahim (NL), Olusegun Isaac</v>
@@ -3810,53 +3810,54 @@
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" xml:space="preserve">
       <c r="A36" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="B36" t="str">
-        <v>Mcewan (NL) (GH), Makala</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="C36" t="str">
-        <v>Available</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D36" t="str">
-        <v>08:00-15:15</v>
+        <v>09:15-17:00</v>
       </c>
       <c r="E36" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="F36" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G36" t="str">
-        <v>4</v>
-      </c>
-      <c r="H36" t="str">
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="H36" t="str" xml:space="preserve">
+        <v xml:space="preserve">Wants this as a break. 
+Eilidh 29/05/2025</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="B37" t="str">
-        <v>McGhie (NL) (GH), Cheryl</v>
+        <v>Lamont (NL) (GH), Sophie</v>
       </c>
       <c r="C37" t="str">
         <v>Available</v>
       </c>
       <c r="D37" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E37" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F37" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G37" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H37" t="str">
         <v/>
@@ -3864,25 +3865,25 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="B38" t="str">
-        <v>Mooney (NL), Lynsey (GH)</v>
+        <v>McGhie (NL) (GH), Cheryl</v>
       </c>
       <c r="C38" t="str">
         <v>Available</v>
       </c>
       <c r="D38" t="str">
-        <v>08:00-14:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E38" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="F38" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="G38" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="H38" t="str">
         <v/>
@@ -3890,115 +3891,114 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="B39" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Mooney (NL), Lynsey (GH)</v>
       </c>
       <c r="C39" t="str">
-        <v>Sick</v>
+        <v>Available</v>
       </c>
       <c r="D39" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E39" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="F39" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="G39" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H39" t="str">
-        <v>Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM; Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2025-09-10</v>
+        <v>2025-09-19</v>
       </c>
       <c r="B40" t="str">
+        <v>Nelson (NL), Anne</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D40" t="str">
+        <v>08:00-13:00</v>
+      </c>
+      <c r="E40" t="str">
+        <v>5.33</v>
+      </c>
+      <c r="F40" t="str">
+        <v>5.33</v>
+      </c>
+      <c r="G40" t="str">
+        <v>5.33</v>
+      </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>2025-09-19</v>
+      </c>
+      <c r="B41" t="str">
         <v>Wylie (NL), Lori</v>
       </c>
-      <c r="C40" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D40" t="str">
-        <v>09:15-15:00</v>
-      </c>
-      <c r="E40" t="str">
-        <v>6</v>
-      </c>
-      <c r="F40" t="str">
-        <v>6</v>
-      </c>
-      <c r="G40" t="str">
-        <v>6</v>
-      </c>
-      <c r="H40" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="41" xml:space="preserve">
-      <c r="A41" t="str">
-        <v>2025-09-12</v>
-      </c>
-      <c r="B41" t="str">
-        <v>Asokhia (NL), Deborah</v>
-      </c>
       <c r="C41" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D41" t="str">
-        <v>08:00-15:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E41" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F41" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G41" t="str">
-        <v>0</v>
-      </c>
-      <c r="H41" t="str" xml:space="preserve">
-        <v xml:space="preserve">Agreed at induction with MT and SM - 09/05/2025; Has appointment and is unable to work 
-Eilidh 22/08/2025</v>
+        <v>6</v>
+      </c>
+      <c r="H41" t="str">
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B42" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Asokhia (NL), Deborah</v>
       </c>
       <c r="C42" t="str">
         <v>Available</v>
       </c>
       <c r="D42" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E42" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="F42" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="G42" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="H42" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B43" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="C43" t="str">
         <v>Available</v>
@@ -4007,13 +4007,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E43" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="F43" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="G43" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -4021,7 +4021,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B44" t="str">
         <v>Forbes (NL) (GH), Amanda</v>
@@ -4047,25 +4047,25 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B45" t="str">
-        <v>Hussain (NL) (GH), Mustansar</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="C45" t="str">
         <v>Available</v>
       </c>
       <c r="D45" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="E45" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="F45" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="G45" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="H45" t="str">
         <v/>
@@ -4073,51 +4073,51 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B46" t="str">
-        <v>Ibrahim (NL), Olusegun Isaac</v>
+        <v>Griffiths (NL), Wayne (GH)</v>
       </c>
       <c r="C46" t="str">
         <v>Available</v>
       </c>
       <c r="D46" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E46" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="F46" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="G46" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H46" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B47" t="str">
-        <v>Mcewan (NL) (GH), Makala</v>
+        <v>Hussain (NL) (GH), Mustansar</v>
       </c>
       <c r="C47" t="str">
         <v>Available</v>
       </c>
       <c r="D47" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E47" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F47" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G47" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H47" t="str">
         <v/>
@@ -4125,16 +4125,16 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B48" t="str">
-        <v>McGhie (NL) (GH), Cheryl</v>
+        <v>Ibrahim (NL), Olusegun Isaac</v>
       </c>
       <c r="C48" t="str">
         <v>Available</v>
       </c>
       <c r="D48" t="str">
-        <v>16:45-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="E48" t="str">
         <v>3.2</v>
@@ -4146,30 +4146,30 @@
         <v>3.2</v>
       </c>
       <c r="H48" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B49" t="str">
-        <v>Mooney (NL), Lynsey (GH)</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="C49" t="str">
         <v>Available</v>
       </c>
       <c r="D49" t="str">
-        <v>08:00-14:00</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E49" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="F49" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="G49" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="H49" t="str">
         <v/>
@@ -4177,25 +4177,25 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B50" t="str">
-        <v>Nelson (NL), Anne</v>
+        <v>Mcewan (NL) (GH), Makala</v>
       </c>
       <c r="C50" t="str">
         <v>Available</v>
       </c>
       <c r="D50" t="str">
-        <v>08:00-13:00</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="E50" t="str">
-        <v>5.33</v>
+        <v>4</v>
       </c>
       <c r="F50" t="str">
-        <v>5.33</v>
+        <v>4</v>
       </c>
       <c r="G50" t="str">
-        <v>5.33</v>
+        <v>4</v>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -4203,25 +4203,25 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B51" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>McGhie (NL) (GH), Cheryl</v>
       </c>
       <c r="C51" t="str">
         <v>Available</v>
       </c>
       <c r="D51" t="str">
-        <v>09:15-14:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E51" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="F51" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="G51" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="H51" t="str">
         <v/>
@@ -4229,25 +4229,25 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2025-09-12</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B52" t="str">
-        <v>Wylie (NL), Lori</v>
+        <v>Mooney (NL), Lynsey (GH)</v>
       </c>
       <c r="C52" t="str">
         <v>Available</v>
       </c>
       <c r="D52" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E52" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F52" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G52" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H52" t="str">
         <v/>
@@ -4255,10 +4255,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B53" t="str">
-        <v>Asokhia (NL), Deborah</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C53" t="str">
         <v>Available</v>
@@ -4267,39 +4267,39 @@
         <v>09:15-14:00</v>
       </c>
       <c r="E53" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="F53" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="G53" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="H53" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B54" t="str">
-        <v>Barton (NL) (GH), Kaitlyn</v>
+        <v>Wylie (NL), Lori</v>
       </c>
       <c r="C54" t="str">
         <v>Available</v>
       </c>
       <c r="D54" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E54" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F54" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G54" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H54" t="str">
         <v/>
@@ -4307,10 +4307,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B55" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Adeyanju (NL) (GH), Adedayo</v>
       </c>
       <c r="C55" t="str">
         <v>Available</v>
@@ -4319,13 +4319,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E55" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="F55" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="G55" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H55" t="str">
         <v/>
@@ -4333,33 +4333,33 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B56" t="str">
-        <v>Ferris (NL), Marykate</v>
+        <v>Asokhia (NL), Deborah</v>
       </c>
       <c r="C56" t="str">
         <v>Available</v>
       </c>
       <c r="D56" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E56" t="str">
-        <v>6.67</v>
+        <v>4</v>
       </c>
       <c r="F56" t="str">
-        <v>6.67</v>
+        <v>4</v>
       </c>
       <c r="G56" t="str">
-        <v>6.67</v>
+        <v>4</v>
       </c>
       <c r="H56" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B57" t="str">
         <v>Forbes (NL) (GH), Amanda</v>
@@ -4385,25 +4385,25 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B58" t="str">
-        <v>Griffiths (NL), Wayne (GH)</v>
+        <v>Gabillard (NL), Donna</v>
       </c>
       <c r="C58" t="str">
         <v>Available</v>
       </c>
       <c r="D58" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-11:30</v>
       </c>
       <c r="E58" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="F58" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="G58" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="H58" t="str">
         <v/>
@@ -4411,78 +4411,77 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B59" t="str">
+        <v>Griffiths (NL), Wayne (GH)</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D59" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E59" t="str">
+        <v>6</v>
+      </c>
+      <c r="F59" t="str">
+        <v>6</v>
+      </c>
+      <c r="G59" t="str">
+        <v>6</v>
+      </c>
+      <c r="H59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>2025-09-18</v>
+      </c>
+      <c r="B60" t="str">
         <v>Ibrahim (NL), Olusegun Isaac</v>
       </c>
-      <c r="C59" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D59" t="str">
+      <c r="C60" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D60" t="str">
         <v>09:15-15:00</v>
       </c>
-      <c r="E59" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="F59" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="G59" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H59" t="str">
+      <c r="E60" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="F60" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="G60" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H60" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
-      </c>
-    </row>
-    <row r="60" xml:space="preserve">
-      <c r="A60" t="str">
-        <v>2025-09-11</v>
-      </c>
-      <c r="B60" t="str">
-        <v>Mcewan (NL) (GH), Makala</v>
-      </c>
-      <c r="C60" t="str">
-        <v>Other Unavailable</v>
-      </c>
-      <c r="D60" t="str">
-        <v>08:00-15:15</v>
-      </c>
-      <c r="E60" t="str">
-        <v>4</v>
-      </c>
-      <c r="F60" t="str">
-        <v>4</v>
-      </c>
-      <c r="G60" t="str">
-        <v>0</v>
-      </c>
-      <c r="H60" t="str" xml:space="preserve">
-        <v xml:space="preserve">Family event
-Eilidh 01/09/2025</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B61" t="str">
-        <v>McGhie (NL) (GH), Cheryl</v>
+        <v>Jack (NL), Sharon</v>
       </c>
       <c r="C61" t="str">
         <v>Available</v>
       </c>
       <c r="D61" t="str">
-        <v>16:45-21:30</v>
+        <v>09:15-16:15</v>
       </c>
       <c r="E61" t="str">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="F61" t="str">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="G61" t="str">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="H61" t="str">
         <v/>
@@ -4490,25 +4489,25 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B62" t="str">
-        <v>Mooney (NL), Lynsey (GH)</v>
+        <v>Lamont (NL) (GH), Sophie</v>
       </c>
       <c r="C62" t="str">
         <v>Available</v>
       </c>
       <c r="D62" t="str">
-        <v>08:00-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E62" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="F62" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="G62" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="H62" t="str">
         <v/>
@@ -4516,25 +4515,25 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B63" t="str">
-        <v>Nelson (NL), Anne</v>
+        <v>McGhie (NL) (GH), Cheryl</v>
       </c>
       <c r="C63" t="str">
         <v>Available</v>
       </c>
       <c r="D63" t="str">
-        <v>08:00-17:15</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E63" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="F63" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="G63" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="H63" t="str">
         <v/>
@@ -4542,25 +4541,25 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B64" t="str">
-        <v>O'Brien (NL) (GH), Brooke</v>
+        <v>Mooney (NL), Lynsey (GH)</v>
       </c>
       <c r="C64" t="str">
         <v>Available</v>
       </c>
       <c r="D64" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E64" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="F64" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="G64" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="H64" t="str">
         <v/>
@@ -4568,25 +4567,25 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2025-09-11</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B65" t="str">
-        <v>Wylie (NL), Lori</v>
+        <v>Nelson (NL), Anne</v>
       </c>
       <c r="C65" t="str">
         <v>Available</v>
       </c>
       <c r="D65" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-17:15</v>
       </c>
       <c r="E65" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="F65" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="G65" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="H65" t="str">
         <v/>
@@ -4594,63 +4593,62 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B66" t="str">
-        <v>Adeyanju (NL) (GH), Adedayo</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C66" t="str">
         <v>Available</v>
       </c>
       <c r="D66" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E66" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="F66" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="G66" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="H66" t="str">
         <v/>
       </c>
     </row>
-    <row r="67" xml:space="preserve">
+    <row r="67">
       <c r="A67" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B67" t="str">
-        <v>Ferris (NL), Marykate</v>
+        <v>Wylie (NL), Lori</v>
       </c>
       <c r="C67" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D67" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E67" t="str">
-        <v>6.67</v>
+        <v>6</v>
       </c>
       <c r="F67" t="str">
-        <v>6.67</v>
+        <v>6</v>
       </c>
       <c r="G67" t="str">
-        <v>0</v>
-      </c>
-      <c r="H67" t="str" xml:space="preserve">
-        <v xml:space="preserve">Away for a family members birthday, tickets were already bought before checking
-Eilidh 01/09/2025</v>
+        <v>6</v>
+      </c>
+      <c r="H67" t="str">
+        <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-20</v>
       </c>
       <c r="B68" t="str">
-        <v>Griffiths (NL), Wayne (GH)</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="C68" t="str">
         <v>Available</v>
@@ -4659,13 +4657,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E68" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="F68" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="G68" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="H68" t="str">
         <v/>
@@ -4673,10 +4671,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-20</v>
       </c>
       <c r="B69" t="str">
-        <v>Lamont (NL) (GH), Sophie</v>
+        <v>Hussain (NL) (GH), Mustansar</v>
       </c>
       <c r="C69" t="str">
         <v>Available</v>
@@ -4685,13 +4683,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E69" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F69" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G69" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H69" t="str">
         <v/>
@@ -4699,7 +4697,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-20</v>
       </c>
       <c r="B70" t="str">
         <v>Mcewan (NL) (GH), Makala</v>
@@ -4725,25 +4723,25 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-20</v>
       </c>
       <c r="B71" t="str">
-        <v>Nelson (NL), Anne</v>
+        <v>O'Brien (NL) (GH), Brooke</v>
       </c>
       <c r="C71" t="str">
         <v>Available</v>
       </c>
       <c r="D71" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E71" t="str">
-        <v>5.33</v>
+        <v>2.67</v>
       </c>
       <c r="F71" t="str">
-        <v>5.33</v>
+        <v>2.67</v>
       </c>
       <c r="G71" t="str">
-        <v>5.33</v>
+        <v>2.67</v>
       </c>
       <c r="H71" t="str">
         <v/>
@@ -4751,7 +4749,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2025-09-14</v>
+        <v>2025-09-20</v>
       </c>
       <c r="B72" t="str">
         <v>Shawcross (NL), Emma</v>
@@ -4777,10 +4775,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2025-09-13</v>
+        <v>2025-09-21</v>
       </c>
       <c r="B73" t="str">
-        <v>Adeyanju (NL) (GH), Adedayo</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="C73" t="str">
         <v>Available</v>
@@ -4803,10 +4801,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2025-09-13</v>
+        <v>2025-09-21</v>
       </c>
       <c r="B74" t="str">
-        <v>Fayaz GH, Shafiya</v>
+        <v>Griffiths (NL), Wayne (GH)</v>
       </c>
       <c r="C74" t="str">
         <v>Available</v>
@@ -4815,13 +4813,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E74" t="str">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F74" t="str">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G74" t="str">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="H74" t="str">
         <v/>
@@ -4829,25 +4827,25 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2025-09-13</v>
+        <v>2025-09-21</v>
       </c>
       <c r="B75" t="str">
-        <v>Hussain (NL) (GH), Mustansar</v>
+        <v>Mcewan (NL) (GH), Makala</v>
       </c>
       <c r="C75" t="str">
         <v>Available</v>
       </c>
       <c r="D75" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="E75" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F75" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G75" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H75" t="str">
         <v/>
@@ -4855,25 +4853,25 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2025-09-13</v>
+        <v>2025-09-21</v>
       </c>
       <c r="B76" t="str">
-        <v>Lamont (NL) (GH), Sophie</v>
+        <v>Nelson (NL), Anne</v>
       </c>
       <c r="C76" t="str">
         <v>Available</v>
       </c>
       <c r="D76" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E76" t="str">
-        <v>7.5</v>
+        <v>5.33</v>
       </c>
       <c r="F76" t="str">
-        <v>7.5</v>
+        <v>5.33</v>
       </c>
       <c r="G76" t="str">
-        <v>7.5</v>
+        <v>5.33</v>
       </c>
       <c r="H76" t="str">
         <v/>
@@ -4881,7 +4879,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2025-09-13</v>
+        <v>2025-09-21</v>
       </c>
       <c r="B77" t="str">
         <v>O'Brien (NL) (GH), Brooke</v>
@@ -4890,7 +4888,7 @@
         <v>Available</v>
       </c>
       <c r="D77" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E77" t="str">
         <v>2.67</v>
@@ -4907,7 +4905,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2025-09-13</v>
+        <v>2025-09-21</v>
       </c>
       <c r="B78" t="str">
         <v>Shawcross (NL), Emma</v>

</xml_diff>

<commit_message>
Saved your changes before starting work
Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 0c2388b3-ddae-4cae-ac15-2ad61d8fe7fc
Replit-Commit-Checkpoint-Type: full_checkpoint
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -1608,7 +1608,7 @@
         <v>3.2</v>
       </c>
       <c r="H41" t="str">
-        <v>3.2</v>
+        <v>1.2</v>
       </c>
       <c r="I41" t="str">
         <v>Confirmed at induction with MT</v>
@@ -1637,7 +1637,7 @@
         <v>3.2</v>
       </c>
       <c r="H42" t="str">
-        <v>3.2</v>
+        <v>1.2</v>
       </c>
       <c r="I42" t="str">
         <v/>
@@ -1666,7 +1666,7 @@
         <v>3.2</v>
       </c>
       <c r="H43" t="str">
-        <v>3.2</v>
+        <v>0.2</v>
       </c>
       <c r="I43" t="str">
         <v/>
@@ -1695,7 +1695,7 @@
         <v>3.2</v>
       </c>
       <c r="H44" t="str">
-        <v>3.2</v>
+        <v>0.2</v>
       </c>
       <c r="I44" t="str">
         <v/>
@@ -1724,7 +1724,7 @@
         <v>3.2</v>
       </c>
       <c r="H45" t="str">
-        <v>3.2</v>
+        <v>0.2</v>
       </c>
       <c r="I45" t="str">
         <v>Confirmed at induction with MT</v>
@@ -1753,7 +1753,7 @@
         <v>2.67</v>
       </c>
       <c r="H46" t="str">
-        <v>2.67</v>
+        <v>1.67</v>
       </c>
       <c r="I46" t="str">
         <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
@@ -1782,7 +1782,7 @@
         <v>2.67</v>
       </c>
       <c r="H47" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="I47" t="str">
         <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
@@ -1811,7 +1811,7 @@
         <v>2.67</v>
       </c>
       <c r="H48" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="I48" t="str">
         <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
@@ -1869,7 +1869,7 @@
         <v>2.67</v>
       </c>
       <c r="H50" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="I50" t="str">
         <v/>
@@ -1898,7 +1898,7 @@
         <v>2.67</v>
       </c>
       <c r="H51" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="I51" t="str">
         <v/>
@@ -1927,7 +1927,7 @@
         <v>4</v>
       </c>
       <c r="H52" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I52" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
@@ -1956,7 +1956,7 @@
         <v>4</v>
       </c>
       <c r="H53" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I53" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
@@ -1985,7 +1985,7 @@
         <v>4</v>
       </c>
       <c r="H54" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I54" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
@@ -2014,7 +2014,7 @@
         <v>4</v>
       </c>
       <c r="H55" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I55" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
@@ -2043,7 +2043,7 @@
         <v>4</v>
       </c>
       <c r="H56" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I56" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
@@ -2072,7 +2072,7 @@
         <v>2.8</v>
       </c>
       <c r="H57" t="str">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="I57" t="str">
         <v/>
@@ -2101,7 +2101,7 @@
         <v>2.8</v>
       </c>
       <c r="H58" t="str">
-        <v>2.8</v>
+        <v>0.8</v>
       </c>
       <c r="I58" t="str">
         <v/>
@@ -2130,7 +2130,7 @@
         <v>2.8</v>
       </c>
       <c r="H59" t="str">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="I59" t="str">
         <v/>
@@ -2159,7 +2159,7 @@
         <v>2.8</v>
       </c>
       <c r="H60" t="str">
-        <v>2.8</v>
+        <v>1.8</v>
       </c>
       <c r="I60" t="str">
         <v/>
@@ -2188,7 +2188,7 @@
         <v>2.8</v>
       </c>
       <c r="H61" t="str">
-        <v>2.8</v>
+        <v>1.8</v>
       </c>
       <c r="I61" t="str">
         <v/>
@@ -2217,7 +2217,7 @@
         <v>10</v>
       </c>
       <c r="H62" t="str">
-        <v>10</v>
+        <v>1.25</v>
       </c>
       <c r="I62" t="str">
         <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
@@ -2246,7 +2246,7 @@
         <v>10</v>
       </c>
       <c r="H63" t="str">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I63" t="str">
         <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
@@ -2275,7 +2275,7 @@
         <v>7.5</v>
       </c>
       <c r="H64" t="str">
-        <v>7.5</v>
+        <v>1.5</v>
       </c>
       <c r="I64" t="str">
         <v/>
@@ -2304,7 +2304,7 @@
         <v>7.5</v>
       </c>
       <c r="H65" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I65" t="str">
         <v/>
@@ -2333,7 +2333,7 @@
         <v>7.5</v>
       </c>
       <c r="H66" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I66" t="str">
         <v/>
@@ -2362,7 +2362,7 @@
         <v>7.5</v>
       </c>
       <c r="H67" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I67" t="str">
         <v/>
@@ -2391,7 +2391,7 @@
         <v>4</v>
       </c>
       <c r="H68" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I68" t="str">
         <v/>
@@ -2420,7 +2420,7 @@
         <v>4</v>
       </c>
       <c r="H69" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I69" t="str">
         <v/>
@@ -2449,7 +2449,7 @@
         <v>4</v>
       </c>
       <c r="H70" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I70" t="str">
         <v/>
@@ -2478,7 +2478,7 @@
         <v>4</v>
       </c>
       <c r="H71" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I71" t="str">
         <v/>
@@ -2507,7 +2507,7 @@
         <v>7.5</v>
       </c>
       <c r="H72" t="str">
-        <v>7.5</v>
+        <v>3.5</v>
       </c>
       <c r="I72" t="str">
         <v/>
@@ -2536,7 +2536,7 @@
         <v>7.5</v>
       </c>
       <c r="H73" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I73" t="str">
         <v/>
@@ -2565,7 +2565,7 @@
         <v>7.5</v>
       </c>
       <c r="H74" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I74" t="str">
         <v/>
@@ -2594,7 +2594,7 @@
         <v>7.5</v>
       </c>
       <c r="H75" t="str">
-        <v>7.5</v>
+        <v>0.5</v>
       </c>
       <c r="I75" t="str">
         <v/>
@@ -2623,7 +2623,7 @@
         <v>7.5</v>
       </c>
       <c r="H76" t="str">
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
       <c r="I76" t="str">
         <v/>
@@ -2652,7 +2652,7 @@
         <v>7.5</v>
       </c>
       <c r="H77" t="str">
-        <v>7.5</v>
+        <v>4.5</v>
       </c>
       <c r="I77" t="str">
         <v/>
@@ -2681,7 +2681,7 @@
         <v>7.5</v>
       </c>
       <c r="H78" t="str">
-        <v>7.5</v>
+        <v>4.5</v>
       </c>
       <c r="I78" t="str">
         <v/>
@@ -2710,7 +2710,7 @@
         <v>7.5</v>
       </c>
       <c r="H79" t="str">
-        <v>7.5</v>
+        <v>3.5</v>
       </c>
       <c r="I79" t="str">
         <v/>
@@ -2768,7 +2768,7 @@
         <v>6</v>
       </c>
       <c r="H81" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I81" t="str">
         <v/>
@@ -2797,7 +2797,7 @@
         <v>6</v>
       </c>
       <c r="H82" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I82" t="str">
         <v/>
@@ -2826,7 +2826,7 @@
         <v>6</v>
       </c>
       <c r="H83" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I83" t="str">
         <v/>
@@ -2855,7 +2855,7 @@
         <v>6</v>
       </c>
       <c r="H84" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I84" t="str">
         <v/>
@@ -2884,7 +2884,7 @@
         <v>6</v>
       </c>
       <c r="H85" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I85" t="str">
         <v/>
@@ -2913,7 +2913,7 @@
         <v>3.2</v>
       </c>
       <c r="H86" t="str">
-        <v>3.2</v>
+        <v>0.2</v>
       </c>
       <c r="I86" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
@@ -2942,7 +2942,7 @@
         <v>3.2</v>
       </c>
       <c r="H87" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="I87" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
@@ -2971,7 +2971,7 @@
         <v>3.2</v>
       </c>
       <c r="H88" t="str">
-        <v>3.2</v>
+        <v>1.2</v>
       </c>
       <c r="I88" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
@@ -3000,7 +3000,7 @@
         <v>3.2</v>
       </c>
       <c r="H89" t="str">
-        <v>3.2</v>
+        <v>1.2</v>
       </c>
       <c r="I89" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
@@ -3058,7 +3058,7 @@
         <v>6</v>
       </c>
       <c r="H91" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I91" t="str">
         <v/>
@@ -3087,7 +3087,7 @@
         <v>6</v>
       </c>
       <c r="H92" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I92" t="str">
         <v/>
@@ -3116,7 +3116,7 @@
         <v>6</v>
       </c>
       <c r="H93" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I93" t="str">
         <v/>
@@ -3145,7 +3145,7 @@
         <v>6</v>
       </c>
       <c r="H94" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I94" t="str">
         <v/>
@@ -3174,7 +3174,7 @@
         <v>6</v>
       </c>
       <c r="H95" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I95" t="str">
         <v/>
@@ -3203,7 +3203,7 @@
         <v>5.33</v>
       </c>
       <c r="H96" t="str">
-        <v>5.33</v>
+        <v>0</v>
       </c>
       <c r="I96" t="str">
         <v/>
@@ -3232,7 +3232,7 @@
         <v>5.33</v>
       </c>
       <c r="H97" t="str">
-        <v>5.33</v>
+        <v>1.33</v>
       </c>
       <c r="I97" t="str">
         <v/>
@@ -3261,7 +3261,7 @@
         <v>5.33</v>
       </c>
       <c r="H98" t="str">
-        <v>5.33</v>
+        <v>0</v>
       </c>
       <c r="I98" t="str">
         <v/>
@@ -3290,7 +3290,7 @@
         <v>3.2</v>
       </c>
       <c r="H99" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="I99" t="str">
         <v/>
@@ -3319,7 +3319,7 @@
         <v>3.2</v>
       </c>
       <c r="H100" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="I100" t="str">
         <v/>
@@ -3348,7 +3348,7 @@
         <v>3.2</v>
       </c>
       <c r="H101" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="I101" t="str">
         <v/>
@@ -3377,7 +3377,7 @@
         <v>3.2</v>
       </c>
       <c r="H102" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="I102" t="str">
         <v/>
@@ -3406,7 +3406,7 @@
         <v>3.2</v>
       </c>
       <c r="H103" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="I103" t="str">
         <v/>
@@ -3435,7 +3435,7 @@
         <v>4</v>
       </c>
       <c r="H104" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I104" t="str">
         <v/>
@@ -3464,7 +3464,7 @@
         <v>4</v>
       </c>
       <c r="H105" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I105" t="str">
         <v/>
@@ -3493,7 +3493,7 @@
         <v>4</v>
       </c>
       <c r="H106" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I106" t="str">
         <v/>
@@ -3522,7 +3522,7 @@
         <v>4</v>
       </c>
       <c r="H107" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I107" t="str">
         <v/>
@@ -3551,7 +3551,7 @@
         <v>4</v>
       </c>
       <c r="H108" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I108" t="str">
         <v/>
@@ -3580,7 +3580,7 @@
         <v>4.8</v>
       </c>
       <c r="H109" t="str">
-        <v>4.8</v>
+        <v>3.8</v>
       </c>
       <c r="I109" t="str">
         <v/>
@@ -3609,7 +3609,7 @@
         <v>4.8</v>
       </c>
       <c r="H110" t="str">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="I110" t="str">
         <v/>
@@ -3638,7 +3638,7 @@
         <v>6</v>
       </c>
       <c r="H111" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I111" t="str">
         <v/>
@@ -3667,7 +3667,7 @@
         <v>6</v>
       </c>
       <c r="H112" t="str">
-        <v>6</v>
+        <v>1.25</v>
       </c>
       <c r="I112" t="str">
         <v/>
@@ -3696,7 +3696,7 @@
         <v>6</v>
       </c>
       <c r="H113" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I113" t="str">
         <v/>
@@ -3725,7 +3725,7 @@
         <v>6</v>
       </c>
       <c r="H114" t="str">
-        <v>6</v>
+        <v>1.25</v>
       </c>
       <c r="I114" t="str">
         <v/>
@@ -3754,7 +3754,7 @@
         <v>6</v>
       </c>
       <c r="H115" t="str">
-        <v>6</v>
+        <v>1.25</v>
       </c>
       <c r="I115" t="str">
         <v/>
@@ -3805,7 +3805,7 @@
         <v>57.37</v>
       </c>
       <c r="C2" t="str">
-        <v>57.37</v>
+        <v>12.37</v>
       </c>
       <c r="D2" t="str">
         <v>12.65</v>
@@ -3817,7 +3817,7 @@
         <v>63.25</v>
       </c>
       <c r="G2" t="str">
-        <v>-5.88</v>
+        <v>-50.88</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -3831,7 +3831,7 @@
         <v>63.57</v>
       </c>
       <c r="C3" t="str">
-        <v>63.57</v>
+        <v>15.25</v>
       </c>
       <c r="D3" t="str">
         <v>31.15</v>
@@ -3843,7 +3843,7 @@
         <v>66.75</v>
       </c>
       <c r="G3" t="str">
-        <v>-3.18</v>
+        <v>-51.5</v>
       </c>
       <c r="H3" t="str">
         <v>Shortage</v>
@@ -3857,7 +3857,7 @@
         <v>60.07</v>
       </c>
       <c r="C4" t="str">
-        <v>60.07</v>
+        <v>8.9</v>
       </c>
       <c r="D4" t="str">
         <v>31.15</v>
@@ -3869,7 +3869,7 @@
         <v>71.25</v>
       </c>
       <c r="G4" t="str">
-        <v>-11.18</v>
+        <v>-62.35</v>
       </c>
       <c r="H4" t="str">
         <v>Shortage</v>
@@ -3883,7 +3883,7 @@
         <v>60.2</v>
       </c>
       <c r="C5" t="str">
-        <v>60.2</v>
+        <v>13.62</v>
       </c>
       <c r="D5" t="str">
         <v>29.15</v>
@@ -3895,7 +3895,7 @@
         <v>61.75</v>
       </c>
       <c r="G5" t="str">
-        <v>-1.55</v>
+        <v>-48.13</v>
       </c>
       <c r="H5" t="str">
         <v>Shortage</v>
@@ -3909,7 +3909,7 @@
         <v>60.23</v>
       </c>
       <c r="C6" t="str">
-        <v>60.23</v>
+        <v>21.28</v>
       </c>
       <c r="D6" t="str">
         <v>23.65</v>
@@ -3921,10 +3921,10 @@
         <v>56.75</v>
       </c>
       <c r="G6" t="str">
-        <v>3.48</v>
+        <v>-35.47</v>
       </c>
       <c r="H6" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="7">
@@ -3935,7 +3935,7 @@
         <v>30.17</v>
       </c>
       <c r="C7" t="str">
-        <v>30.17</v>
+        <v>2.25</v>
       </c>
       <c r="D7" t="str">
         <v>21.65</v>
@@ -3947,7 +3947,7 @@
         <v>45.75</v>
       </c>
       <c r="G7" t="str">
-        <v>-15.58</v>
+        <v>-43.5</v>
       </c>
       <c r="H7" t="str">
         <v>Shortage</v>
@@ -3961,7 +3961,7 @@
         <v>35.5</v>
       </c>
       <c r="C8" t="str">
-        <v>35.5</v>
+        <v>2</v>
       </c>
       <c r="D8" t="str">
         <v>12.65</v>
@@ -3973,7 +3973,7 @@
         <v>43</v>
       </c>
       <c r="G8" t="str">
-        <v>-7.5</v>
+        <v>-41</v>
       </c>
       <c r="H8" t="str">
         <v>Shortage</v>
@@ -4036,7 +4036,7 @@
         <v>7.5</v>
       </c>
       <c r="G2" t="str">
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -4062,7 +4062,7 @@
         <v>3.2</v>
       </c>
       <c r="G3" t="str">
-        <v>3.2</v>
+        <v>1.2</v>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -4141,7 +4141,7 @@
         <v>2.67</v>
       </c>
       <c r="G6" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="H6" t="str">
         <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
@@ -4167,7 +4167,7 @@
         <v>3.2</v>
       </c>
       <c r="G7" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -4193,7 +4193,7 @@
         <v>4</v>
       </c>
       <c r="G8" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H8" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
@@ -4219,7 +4219,7 @@
         <v>2.8</v>
       </c>
       <c r="G9" t="str">
-        <v>2.8</v>
+        <v>0.8</v>
       </c>
       <c r="H9" t="str">
         <v/>
@@ -4271,7 +4271,7 @@
         <v>7.5</v>
       </c>
       <c r="G11" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -4297,7 +4297,7 @@
         <v>6</v>
       </c>
       <c r="G12" t="str">
-        <v>6</v>
+        <v>1.25</v>
       </c>
       <c r="H12" t="str">
         <v/>
@@ -4323,7 +4323,7 @@
         <v>4</v>
       </c>
       <c r="G13" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H13" t="str">
         <v/>
@@ -4402,7 +4402,7 @@
         <v>6</v>
       </c>
       <c r="G16" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H16" t="str">
         <v/>
@@ -4428,7 +4428,7 @@
         <v>3.2</v>
       </c>
       <c r="G17" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H17" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
@@ -4507,7 +4507,7 @@
         <v>7.5</v>
       </c>
       <c r="G20" t="str">
-        <v>7.5</v>
+        <v>3.5</v>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -4533,7 +4533,7 @@
         <v>6</v>
       </c>
       <c r="G21" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H21" t="str">
         <v/>
@@ -4559,7 +4559,7 @@
         <v>7.5</v>
       </c>
       <c r="G22" t="str">
-        <v>7.5</v>
+        <v>4.5</v>
       </c>
       <c r="H22" t="str">
         <v/>
@@ -4585,7 +4585,7 @@
         <v>3.2</v>
       </c>
       <c r="G23" t="str">
-        <v>3.2</v>
+        <v>0.2</v>
       </c>
       <c r="H23" t="str">
         <v/>
@@ -4664,7 +4664,7 @@
         <v>2.67</v>
       </c>
       <c r="G26" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="H26" t="str">
         <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
@@ -4690,7 +4690,7 @@
         <v>3.2</v>
       </c>
       <c r="G27" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H27" t="str">
         <v/>
@@ -4716,7 +4716,7 @@
         <v>4</v>
       </c>
       <c r="G28" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H28" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
@@ -4742,7 +4742,7 @@
         <v>2.8</v>
       </c>
       <c r="G29" t="str">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -4794,7 +4794,7 @@
         <v>6</v>
       </c>
       <c r="G31" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H31" t="str">
         <v/>
@@ -4820,7 +4820,7 @@
         <v>4</v>
       </c>
       <c r="G32" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H32" t="str">
         <v/>
@@ -4872,7 +4872,7 @@
         <v>4</v>
       </c>
       <c r="G34" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H34" t="str">
         <v/>
@@ -4925,7 +4925,7 @@
         <v>6</v>
       </c>
       <c r="G36" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H36" t="str">
         <v/>
@@ -4951,7 +4951,7 @@
         <v>3.2</v>
       </c>
       <c r="G37" t="str">
-        <v>3.2</v>
+        <v>1.2</v>
       </c>
       <c r="H37" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
@@ -5031,7 +5031,7 @@
         <v>7.5</v>
       </c>
       <c r="G40" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H40" t="str">
         <v/>
@@ -5057,7 +5057,7 @@
         <v>6</v>
       </c>
       <c r="G41" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H41" t="str">
         <v/>
@@ -5083,7 +5083,7 @@
         <v>7.5</v>
       </c>
       <c r="G42" t="str">
-        <v>7.5</v>
+        <v>4.5</v>
       </c>
       <c r="H42" t="str">
         <v/>
@@ -5109,7 +5109,7 @@
         <v>3.2</v>
       </c>
       <c r="G43" t="str">
-        <v>3.2</v>
+        <v>0.2</v>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -5135,7 +5135,7 @@
         <v>5.33</v>
       </c>
       <c r="G44" t="str">
-        <v>5.33</v>
+        <v>0</v>
       </c>
       <c r="H44" t="str">
         <v/>
@@ -5240,7 +5240,7 @@
         <v>3.2</v>
       </c>
       <c r="G48" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H48" t="str">
         <v/>
@@ -5266,7 +5266,7 @@
         <v>4</v>
       </c>
       <c r="G49" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H49" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
@@ -5292,7 +5292,7 @@
         <v>2.8</v>
       </c>
       <c r="G50" t="str">
-        <v>2.8</v>
+        <v>1.8</v>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -5344,7 +5344,7 @@
         <v>6</v>
       </c>
       <c r="G52" t="str">
-        <v>6</v>
+        <v>1.25</v>
       </c>
       <c r="H52" t="str">
         <v/>
@@ -5370,7 +5370,7 @@
         <v>4</v>
       </c>
       <c r="G53" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H53" t="str">
         <v/>
@@ -5449,7 +5449,7 @@
         <v>3.2</v>
       </c>
       <c r="G56" t="str">
-        <v>3.2</v>
+        <v>1.2</v>
       </c>
       <c r="H56" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
@@ -5502,7 +5502,7 @@
         <v>4.8</v>
       </c>
       <c r="G58" t="str">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="H58" t="str">
         <v/>
@@ -5528,7 +5528,7 @@
         <v>7.5</v>
       </c>
       <c r="G59" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H59" t="str">
         <v/>
@@ -5554,7 +5554,7 @@
         <v>6</v>
       </c>
       <c r="G60" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H60" t="str">
         <v/>
@@ -5580,7 +5580,7 @@
         <v>7.5</v>
       </c>
       <c r="G61" t="str">
-        <v>7.5</v>
+        <v>3.5</v>
       </c>
       <c r="H61" t="str">
         <v/>
@@ -5606,7 +5606,7 @@
         <v>3.2</v>
       </c>
       <c r="G62" t="str">
-        <v>3.2</v>
+        <v>0.2</v>
       </c>
       <c r="H62" t="str">
         <v>Confirmed at induction with MT</v>
@@ -5632,7 +5632,7 @@
         <v>5.33</v>
       </c>
       <c r="G63" t="str">
-        <v>5.33</v>
+        <v>1.33</v>
       </c>
       <c r="H63" t="str">
         <v/>
@@ -5711,7 +5711,7 @@
         <v>3.2</v>
       </c>
       <c r="G66" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H66" t="str">
         <v/>
@@ -5737,7 +5737,7 @@
         <v>4</v>
       </c>
       <c r="G67" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H67" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
@@ -5763,7 +5763,7 @@
         <v>2.8</v>
       </c>
       <c r="G68" t="str">
-        <v>2.8</v>
+        <v>1.8</v>
       </c>
       <c r="H68" t="str">
         <v/>
@@ -5815,7 +5815,7 @@
         <v>6</v>
       </c>
       <c r="G70" t="str">
-        <v>6</v>
+        <v>1.25</v>
       </c>
       <c r="H70" t="str">
         <v/>
@@ -5841,7 +5841,7 @@
         <v>4</v>
       </c>
       <c r="G71" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H71" t="str">
         <v/>
@@ -5920,7 +5920,7 @@
         <v>6</v>
       </c>
       <c r="G74" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H74" t="str">
         <v/>
@@ -6026,7 +6026,7 @@
         <v>7.5</v>
       </c>
       <c r="G78" t="str">
-        <v>7.5</v>
+        <v>0.5</v>
       </c>
       <c r="H78" t="str">
         <v/>
@@ -6105,7 +6105,7 @@
         <v>2.67</v>
       </c>
       <c r="G81" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="H81" t="str">
         <v/>
@@ -6131,7 +6131,7 @@
         <v>10</v>
       </c>
       <c r="G82" t="str">
-        <v>10</v>
+        <v>1.25</v>
       </c>
       <c r="H82" t="str">
         <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
@@ -6157,7 +6157,7 @@
         <v>7.5</v>
       </c>
       <c r="G83" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H83" t="str">
         <v/>
@@ -6209,7 +6209,7 @@
         <v>4</v>
       </c>
       <c r="G85" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H85" t="str">
         <v/>
@@ -6262,7 +6262,7 @@
         <v>6</v>
       </c>
       <c r="G87" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H87" t="str">
         <v/>
@@ -6315,7 +6315,7 @@
         <v>3.2</v>
       </c>
       <c r="G89" t="str">
-        <v>3.2</v>
+        <v>1.2</v>
       </c>
       <c r="H89" t="str">
         <v>Confirmed at induction with MT</v>
@@ -6367,7 +6367,7 @@
         <v>2.67</v>
       </c>
       <c r="G91" t="str">
-        <v>2.67</v>
+        <v>1.67</v>
       </c>
       <c r="H91" t="str">
         <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
@@ -6393,7 +6393,7 @@
         <v>3.2</v>
       </c>
       <c r="G92" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H92" t="str">
         <v/>
@@ -6419,7 +6419,7 @@
         <v>4</v>
       </c>
       <c r="G93" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H93" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
@@ -6445,7 +6445,7 @@
         <v>2.8</v>
       </c>
       <c r="G94" t="str">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="H94" t="str">
         <v/>
@@ -6497,7 +6497,7 @@
         <v>7.5</v>
       </c>
       <c r="G96" t="str">
-        <v>7.5</v>
+        <v>1.5</v>
       </c>
       <c r="H96" t="str">
         <v/>
@@ -6523,7 +6523,7 @@
         <v>6</v>
       </c>
       <c r="G97" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H97" t="str">
         <v/>
@@ -6549,7 +6549,7 @@
         <v>4</v>
       </c>
       <c r="G98" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H98" t="str">
         <v/>
@@ -6601,7 +6601,7 @@
         <v>4</v>
       </c>
       <c r="G100" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H100" t="str">
         <v/>
@@ -6654,7 +6654,7 @@
         <v>6</v>
       </c>
       <c r="G102" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H102" t="str">
         <v/>
@@ -6680,7 +6680,7 @@
         <v>3.2</v>
       </c>
       <c r="G103" t="str">
-        <v>3.2</v>
+        <v>0.2</v>
       </c>
       <c r="H103" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
@@ -6706,7 +6706,7 @@
         <v>4.8</v>
       </c>
       <c r="G104" t="str">
-        <v>4.8</v>
+        <v>3.8</v>
       </c>
       <c r="H104" t="str">
         <v/>
@@ -6732,7 +6732,7 @@
         <v>6</v>
       </c>
       <c r="G105" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H105" t="str">
         <v/>
@@ -6758,7 +6758,7 @@
         <v>5.33</v>
       </c>
       <c r="G106" t="str">
-        <v>5.33</v>
+        <v>0</v>
       </c>
       <c r="H106" t="str">
         <v/>
@@ -6810,7 +6810,7 @@
         <v>2.67</v>
       </c>
       <c r="G108" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="H108" t="str">
         <v/>
@@ -6836,7 +6836,7 @@
         <v>10</v>
       </c>
       <c r="G109" t="str">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H109" t="str">
         <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
@@ -6888,7 +6888,7 @@
         <v>7.5</v>
       </c>
       <c r="G111" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H111" t="str">
         <v/>
@@ -6940,7 +6940,7 @@
         <v>4</v>
       </c>
       <c r="G113" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H113" t="str">
         <v/>
@@ -6993,7 +6993,7 @@
         <v>6</v>
       </c>
       <c r="G115" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H115" t="str">
         <v/>

</xml_diff>

<commit_message>
Update capacity dashboard with new data and insights
Updated the capacity_dashboard.xlsx file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 2c4a1858-c1f5-4437-b570-0c310a178a38
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/2c4a1858-c1f5-4437-b570-0c310a178a38/WqFSwcU
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3691,7 +3691,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:H108"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4822,25 +4822,25 @@
         <v>2025-09-18</v>
       </c>
       <c r="B44" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="C44" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D44" t="str">
-        <v>09:15-14:00</v>
+        <v>16:45-20:15</v>
       </c>
       <c r="E44" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="F44" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="G44" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="H44" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="45">
@@ -4848,22 +4848,22 @@
         <v>2025-09-18</v>
       </c>
       <c r="B45" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C45" t="str">
         <v>Available</v>
       </c>
       <c r="D45" t="str">
-        <v>16:45-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E45" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="F45" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="G45" t="str">
-        <v>3.2</v>
+        <v>2.67</v>
       </c>
       <c r="H45" t="str">
         <v/>
@@ -4874,25 +4874,25 @@
         <v>2025-09-18</v>
       </c>
       <c r="B46" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="C46" t="str">
         <v>Available</v>
       </c>
       <c r="D46" t="str">
-        <v>09:15-14:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E46" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="F46" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="G46" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="H46" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -4900,25 +4900,25 @@
         <v>2025-09-18</v>
       </c>
       <c r="B47" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="C47" t="str">
         <v>Available</v>
       </c>
       <c r="D47" t="str">
-        <v>09:15-11:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E47" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="F47" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="G47" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="H47" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="48">
@@ -4926,22 +4926,22 @@
         <v>2025-09-18</v>
       </c>
       <c r="B48" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="C48" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D48" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-11:30</v>
       </c>
       <c r="E48" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="F48" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="G48" t="str">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="H48" t="str">
         <v/>
@@ -4952,22 +4952,22 @@
         <v>2025-09-18</v>
       </c>
       <c r="B49" t="str">
-        <v>Lori Wylie (NL)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="C49" t="str">
-        <v>Available</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D49" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E49" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="F49" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="G49" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H49" t="str">
         <v/>
@@ -4978,22 +4978,22 @@
         <v>2025-09-18</v>
       </c>
       <c r="B50" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="C50" t="str">
         <v>Available</v>
       </c>
       <c r="D50" t="str">
-        <v>08:00-15:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E50" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F50" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G50" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -5004,22 +5004,22 @@
         <v>2025-09-18</v>
       </c>
       <c r="B51" t="str">
-        <v>Marykate Ferris (NL)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="C51" t="str">
         <v>Available</v>
       </c>
       <c r="D51" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E51" t="str">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F51" t="str">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G51" t="str">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H51" t="str">
         <v/>
@@ -5030,78 +5030,78 @@
         <v>2025-09-18</v>
       </c>
       <c r="B52" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="C52" t="str">
         <v>Available</v>
       </c>
       <c r="D52" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E52" t="str">
-        <v>3.2</v>
+        <v>10</v>
       </c>
       <c r="F52" t="str">
-        <v>3.2</v>
+        <v>10</v>
       </c>
       <c r="G52" t="str">
-        <v>3.2</v>
+        <v>10</v>
       </c>
       <c r="H52" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
-      </c>
-    </row>
-    <row r="53" xml:space="preserve">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
       <c r="A53" t="str">
         <v>2025-09-18</v>
       </c>
       <c r="B53" t="str">
+        <v>Olusegun Isaac Ibrahim (NL)</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D53" t="str">
+        <v>09:15-15:00</v>
+      </c>
+      <c r="E53" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="F53" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="G53" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H53" t="str">
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+      </c>
+    </row>
+    <row r="54" xml:space="preserve">
+      <c r="A54" t="str">
+        <v>2025-09-18</v>
+      </c>
+      <c r="B54" t="str">
         <v>Shafiya Fayaz GH</v>
       </c>
-      <c r="C53" t="str">
+      <c r="C54" t="str">
         <v>Other Unavailable</v>
       </c>
-      <c r="D53" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E53" t="str">
+      <c r="D54" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E54" t="str">
         <v>9</v>
       </c>
-      <c r="F53" t="str">
+      <c r="F54" t="str">
         <v>9</v>
       </c>
-      <c r="G53" t="str">
+      <c r="G54" t="str">
         <v>0</v>
       </c>
-      <c r="H53" t="str" xml:space="preserve">
+      <c r="H54" t="str" xml:space="preserve">
         <v xml:space="preserve">Megan approved 
 Eilidh 02/07/2025</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="str">
-        <v>2025-09-18</v>
-      </c>
-      <c r="B54" t="str">
-        <v>Sharon Jack (NL)</v>
-      </c>
-      <c r="C54" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D54" t="str">
-        <v>09:15-16:15</v>
-      </c>
-      <c r="E54" t="str">
-        <v>4.8</v>
-      </c>
-      <c r="F54" t="str">
-        <v>4.8</v>
-      </c>
-      <c r="G54" t="str">
-        <v>4.8</v>
-      </c>
-      <c r="H54" t="str">
-        <v/>
       </c>
     </row>
     <row r="55">
@@ -5109,22 +5109,22 @@
         <v>2025-09-18</v>
       </c>
       <c r="B55" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
+        <v>Sharon Jack (NL)</v>
       </c>
       <c r="C55" t="str">
         <v>Available</v>
       </c>
       <c r="D55" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-16:15</v>
       </c>
       <c r="E55" t="str">
-        <v>7.5</v>
+        <v>4.8</v>
       </c>
       <c r="F55" t="str">
-        <v>7.5</v>
+        <v>4.8</v>
       </c>
       <c r="G55" t="str">
-        <v>7.5</v>
+        <v>4.8</v>
       </c>
       <c r="H55" t="str">
         <v/>
@@ -5135,7 +5135,7 @@
         <v>2025-09-18</v>
       </c>
       <c r="B56" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="C56" t="str">
         <v>Available</v>
@@ -5144,13 +5144,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E56" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="F56" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="G56" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="H56" t="str">
         <v/>
@@ -5158,10 +5158,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2025-09-19</v>
+        <v>2025-09-18</v>
       </c>
       <c r="B57" t="str">
-        <v>Adedayo Adeyanju (NL) (GH)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="C57" t="str">
         <v>Available</v>
@@ -5170,13 +5170,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E57" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F57" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G57" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H57" t="str">
         <v/>
@@ -5187,25 +5187,25 @@
         <v>2025-09-19</v>
       </c>
       <c r="B58" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
+        <v>Adedayo Adeyanju (NL) (GH)</v>
       </c>
       <c r="C58" t="str">
         <v>Available</v>
       </c>
       <c r="D58" t="str">
-        <v>10:30-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E58" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F58" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G58" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H58" t="str">
-        <v>Confirmed at induction with MT</v>
+        <v/>
       </c>
     </row>
     <row r="59">
@@ -5213,25 +5213,25 @@
         <v>2025-09-19</v>
       </c>
       <c r="B59" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="C59" t="str">
         <v>Available</v>
       </c>
       <c r="D59" t="str">
-        <v>08:00-13:00</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="E59" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="F59" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="G59" t="str">
-        <v>5.33</v>
+        <v>3.2</v>
       </c>
       <c r="H59" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="60">
@@ -5239,78 +5239,78 @@
         <v>2025-09-19</v>
       </c>
       <c r="B60" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
+        <v>Anne Nelson (NL)</v>
       </c>
       <c r="C60" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D60" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-13:00</v>
       </c>
       <c r="E60" t="str">
-        <v>2.29</v>
+        <v>5.33</v>
       </c>
       <c r="F60" t="str">
-        <v>2.29</v>
+        <v>5.33</v>
       </c>
       <c r="G60" t="str">
-        <v>0</v>
+        <v>5.33</v>
       </c>
       <c r="H60" t="str">
         <v/>
       </c>
     </row>
-    <row r="61" xml:space="preserve">
+    <row r="61">
       <c r="A61" t="str">
         <v>2025-09-19</v>
       </c>
       <c r="B61" t="str">
-        <v>Ayoola Ajibade (GH) (NL)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C61" t="str">
         <v>Maternity/Paternity</v>
       </c>
       <c r="D61" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E61" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="F61" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="G61" t="str">
         <v>0</v>
       </c>
-      <c r="H61" t="str" xml:space="preserve">
+      <c r="H61" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="62" xml:space="preserve">
+      <c r="A62" t="str">
+        <v>2025-09-19</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Ayoola Ajibade (GH) (NL)</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Maternity/Paternity</v>
+      </c>
+      <c r="D62" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E62" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="F62" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="G62" t="str">
+        <v>0</v>
+      </c>
+      <c r="H62" t="str" xml:space="preserve">
         <v xml:space="preserve">Morning sickness
 Eilidh 31/03/2025</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="str">
-        <v>2025-09-19</v>
-      </c>
-      <c r="B62" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
-      </c>
-      <c r="C62" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D62" t="str">
-        <v>16:45-21:30</v>
-      </c>
-      <c r="E62" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="F62" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="G62" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H62" t="str">
-        <v/>
       </c>
     </row>
     <row r="63">
@@ -5318,25 +5318,25 @@
         <v>2025-09-19</v>
       </c>
       <c r="B63" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Barton (NL) (GH), Kaitlyn</v>
       </c>
       <c r="C63" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D63" t="str">
-        <v>09:15-14:00</v>
+        <v>16:45-17:44; 19:14-21:29</v>
       </c>
       <c r="E63" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F63" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G63" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H63" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="64">
@@ -5344,22 +5344,22 @@
         <v>2025-09-19</v>
       </c>
       <c r="B64" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="C64" t="str">
         <v>Available</v>
       </c>
       <c r="D64" t="str">
-        <v>09:15-10:15</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E64" t="str">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="F64" t="str">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="G64" t="str">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="H64" t="str">
         <v/>
@@ -5370,25 +5370,25 @@
         <v>2025-09-19</v>
       </c>
       <c r="B65" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="C65" t="str">
         <v>Available</v>
       </c>
       <c r="D65" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E65" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="F65" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="G65" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="H65" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="66">
@@ -5396,22 +5396,22 @@
         <v>2025-09-19</v>
       </c>
       <c r="B66" t="str">
-        <v>Lori Wylie (NL)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="C66" t="str">
         <v>Available</v>
       </c>
       <c r="D66" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E66" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="F66" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="G66" t="str">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="H66" t="str">
         <v/>
@@ -5422,22 +5422,22 @@
         <v>2025-09-19</v>
       </c>
       <c r="B67" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="C67" t="str">
         <v>Available</v>
       </c>
       <c r="D67" t="str">
-        <v>08:00-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E67" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="F67" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="G67" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="H67" t="str">
         <v/>
@@ -5448,22 +5448,22 @@
         <v>2025-09-19</v>
       </c>
       <c r="B68" t="str">
-        <v>Marykate Ferris (NL)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="C68" t="str">
         <v>Available</v>
       </c>
       <c r="D68" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E68" t="str">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F68" t="str">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G68" t="str">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H68" t="str">
         <v/>
@@ -5474,22 +5474,22 @@
         <v>2025-09-19</v>
       </c>
       <c r="B69" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="C69" t="str">
         <v>Available</v>
       </c>
       <c r="D69" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E69" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F69" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G69" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H69" t="str">
         <v/>
@@ -5500,142 +5500,142 @@
         <v>2025-09-19</v>
       </c>
       <c r="B70" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="C70" t="str">
         <v>Available</v>
       </c>
       <c r="D70" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E70" t="str">
-        <v>3.2</v>
+        <v>10</v>
       </c>
       <c r="F70" t="str">
-        <v>3.2</v>
+        <v>10</v>
       </c>
       <c r="G70" t="str">
-        <v>3.2</v>
+        <v>10</v>
       </c>
       <c r="H70" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
-      </c>
-    </row>
-    <row r="71" xml:space="preserve">
+        <v/>
+      </c>
+    </row>
+    <row r="71">
       <c r="A71" t="str">
         <v>2025-09-19</v>
       </c>
       <c r="B71" t="str">
+        <v>Mustansar Hussain (NL) (GH)</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D71" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E71" t="str">
+        <v>6</v>
+      </c>
+      <c r="F71" t="str">
+        <v>6</v>
+      </c>
+      <c r="G71" t="str">
+        <v>6</v>
+      </c>
+      <c r="H71" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>2025-09-19</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Olusegun Isaac Ibrahim (NL)</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D72" t="str">
+        <v>09:15-15:00</v>
+      </c>
+      <c r="E72" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="F72" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="G72" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H72" t="str">
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+      </c>
+    </row>
+    <row r="73" xml:space="preserve">
+      <c r="A73" t="str">
+        <v>2025-09-19</v>
+      </c>
+      <c r="B73" t="str">
         <v>Shafiya Fayaz GH</v>
       </c>
-      <c r="C71" t="str">
+      <c r="C73" t="str">
         <v>Other Unavailable</v>
       </c>
-      <c r="D71" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E71" t="str">
+      <c r="D73" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E73" t="str">
         <v>9</v>
       </c>
-      <c r="F71" t="str">
+      <c r="F73" t="str">
         <v>9</v>
       </c>
-      <c r="G71" t="str">
+      <c r="G73" t="str">
         <v>0</v>
       </c>
-      <c r="H71" t="str" xml:space="preserve">
+      <c r="H73" t="str" xml:space="preserve">
         <v xml:space="preserve">Megan approved 
 Eilidh 02/07/2025</v>
       </c>
     </row>
-    <row r="72" xml:space="preserve">
-      <c r="A72" t="str">
+    <row r="74" xml:space="preserve">
+      <c r="A74" t="str">
         <v>2025-09-19</v>
       </c>
-      <c r="B72" t="str">
+      <c r="B74" t="str">
         <v>Sharon Jack (NL)</v>
       </c>
-      <c r="C72" t="str">
+      <c r="C74" t="str">
         <v>Other Unavailable</v>
       </c>
-      <c r="D72" t="str">
+      <c r="D74" t="str">
         <v>09:15-17:00</v>
       </c>
-      <c r="E72" t="str">
+      <c r="E74" t="str">
         <v>4.8</v>
       </c>
-      <c r="F72" t="str">
+      <c r="F74" t="str">
         <v>2</v>
       </c>
-      <c r="G72" t="str">
+      <c r="G74" t="str">
         <v>0</v>
       </c>
-      <c r="H72" t="str" xml:space="preserve">
+      <c r="H74" t="str" xml:space="preserve">
         <v xml:space="preserve">Wants this as a break. 
 Eilidh 29/05/2025</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="str">
+    <row r="75">
+      <c r="A75" t="str">
         <v>2025-09-19</v>
       </c>
-      <c r="B73" t="str">
+      <c r="B75" t="str">
         <v>Sophie Lamont (NL) (GH)</v>
       </c>
-      <c r="C73" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D73" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E73" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="F73" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="G73" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H73" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="str">
-        <v>2025-09-20</v>
-      </c>
-      <c r="B74" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
-      </c>
-      <c r="C74" t="str">
-        <v>Maternity/Paternity</v>
-      </c>
-      <c r="D74" t="str">
-        <v>08:00-15:30</v>
-      </c>
-      <c r="E74" t="str">
-        <v>2.29</v>
-      </c>
-      <c r="F74" t="str">
-        <v>2.29</v>
-      </c>
-      <c r="G74" t="str">
-        <v>0</v>
-      </c>
-      <c r="H74" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="75" xml:space="preserve">
-      <c r="A75" t="str">
-        <v>2025-09-20</v>
-      </c>
-      <c r="B75" t="str">
-        <v>Ayoola Ajibade (GH) (NL)</v>
-      </c>
       <c r="C75" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D75" t="str">
         <v>08:00-21:30</v>
@@ -5647,11 +5647,10 @@
         <v>7.5</v>
       </c>
       <c r="G75" t="str">
-        <v>0</v>
-      </c>
-      <c r="H75" t="str" xml:space="preserve">
-        <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025</v>
+        <v>7.5</v>
+      </c>
+      <c r="H75" t="str">
+        <v/>
       </c>
     </row>
     <row r="76">
@@ -5659,51 +5658,52 @@
         <v>2025-09-20</v>
       </c>
       <c r="B76" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C76" t="str">
-        <v>Available</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D76" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E76" t="str">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="F76" t="str">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="G76" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="H76" t="str">
         <v/>
       </c>
     </row>
-    <row r="77">
+    <row r="77" xml:space="preserve">
       <c r="A77" t="str">
         <v>2025-09-20</v>
       </c>
       <c r="B77" t="str">
-        <v>Emma Shawcross (NL)</v>
+        <v>Ayoola Ajibade (GH) (NL)</v>
       </c>
       <c r="C77" t="str">
-        <v>Available</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D77" t="str">
         <v>08:00-21:30</v>
       </c>
       <c r="E77" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="F77" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="G77" t="str">
-        <v>10</v>
-      </c>
-      <c r="H77" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v>0</v>
+      </c>
+      <c r="H77" t="str" xml:space="preserve">
+        <v xml:space="preserve">Morning sickness
+Eilidh 31/03/2025</v>
       </c>
     </row>
     <row r="78">
@@ -5711,7 +5711,7 @@
         <v>2025-09-20</v>
       </c>
       <c r="B78" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C78" t="str">
         <v>Available</v>
@@ -5720,13 +5720,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E78" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="F78" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="G78" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="H78" t="str">
         <v/>
@@ -5737,25 +5737,25 @@
         <v>2025-09-20</v>
       </c>
       <c r="B79" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Emma Shawcross (NL)</v>
       </c>
       <c r="C79" t="str">
         <v>Available</v>
       </c>
       <c r="D79" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E79" t="str">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F79" t="str">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G79" t="str">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H79" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="80">
@@ -5763,7 +5763,7 @@
         <v>2025-09-20</v>
       </c>
       <c r="B80" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Kaitlyn Barton (NL) (GH)</v>
       </c>
       <c r="C80" t="str">
         <v>Available</v>
@@ -5772,95 +5772,95 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E80" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="F80" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="G80" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="H80" t="str">
         <v/>
       </c>
     </row>
-    <row r="81" xml:space="preserve">
+    <row r="81">
       <c r="A81" t="str">
         <v>2025-09-20</v>
       </c>
       <c r="B81" t="str">
+        <v>Makala Mcewan (NL) (GH)</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D81" t="str">
+        <v>08:00-15:15</v>
+      </c>
+      <c r="E81" t="str">
+        <v>4</v>
+      </c>
+      <c r="F81" t="str">
+        <v>4</v>
+      </c>
+      <c r="G81" t="str">
+        <v>4</v>
+      </c>
+      <c r="H81" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>2025-09-20</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Mustansar Hussain (NL) (GH)</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D82" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E82" t="str">
+        <v>6</v>
+      </c>
+      <c r="F82" t="str">
+        <v>6</v>
+      </c>
+      <c r="G82" t="str">
+        <v>6</v>
+      </c>
+      <c r="H82" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="83" xml:space="preserve">
+      <c r="A83" t="str">
+        <v>2025-09-20</v>
+      </c>
+      <c r="B83" t="str">
         <v>Shafiya Fayaz GH</v>
       </c>
-      <c r="C81" t="str">
+      <c r="C83" t="str">
         <v>Other Unavailable</v>
       </c>
-      <c r="D81" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E81" t="str">
+      <c r="D83" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E83" t="str">
         <v>9</v>
       </c>
-      <c r="F81" t="str">
+      <c r="F83" t="str">
         <v>9</v>
       </c>
-      <c r="G81" t="str">
+      <c r="G83" t="str">
         <v>0</v>
       </c>
-      <c r="H81" t="str" xml:space="preserve">
+      <c r="H83" t="str" xml:space="preserve">
         <v xml:space="preserve">Megan approved 
 Eilidh 02/07/2025</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="str">
-        <v>2025-09-15</v>
-      </c>
-      <c r="B82" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
-      </c>
-      <c r="C82" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D82" t="str">
-        <v>10:30-14:00</v>
-      </c>
-      <c r="E82" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="F82" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="G82" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H82" t="str">
-        <v>Confirmed at induction with MT</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="str">
-        <v>2025-09-15</v>
-      </c>
-      <c r="B83" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
-      </c>
-      <c r="C83" t="str">
-        <v>Maternity/Paternity</v>
-      </c>
-      <c r="D83" t="str">
-        <v>08:00-15:30</v>
-      </c>
-      <c r="E83" t="str">
-        <v>2.29</v>
-      </c>
-      <c r="F83" t="str">
-        <v>2.29</v>
-      </c>
-      <c r="G83" t="str">
-        <v>0</v>
-      </c>
-      <c r="H83" t="str">
-        <v/>
       </c>
     </row>
     <row r="84">
@@ -5868,25 +5868,25 @@
         <v>2025-09-15</v>
       </c>
       <c r="B84" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="C84" t="str">
         <v>Available</v>
       </c>
       <c r="D84" t="str">
-        <v>09:15-14:00</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="E84" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="F84" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="G84" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="H84" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="85">
@@ -5894,22 +5894,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B85" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C85" t="str">
-        <v>Available</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D85" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E85" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="F85" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="G85" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H85" t="str">
         <v/>
@@ -5920,7 +5920,7 @@
         <v>2025-09-15</v>
       </c>
       <c r="B86" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C86" t="str">
         <v>Available</v>
@@ -5929,16 +5929,16 @@
         <v>09:15-14:00</v>
       </c>
       <c r="E86" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="F86" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="G86" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="H86" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="87">
@@ -5946,22 +5946,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B87" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="C87" t="str">
         <v>Available</v>
       </c>
       <c r="D87" t="str">
-        <v>09:15-14:45</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E87" t="str">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="F87" t="str">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="G87" t="str">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="H87" t="str">
         <v/>
@@ -5972,25 +5972,25 @@
         <v>2025-09-15</v>
       </c>
       <c r="B88" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="C88" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D88" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E88" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="F88" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="G88" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H88" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="89">
@@ -5998,22 +5998,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B89" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="C89" t="str">
         <v>Available</v>
       </c>
       <c r="D89" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="E89" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="F89" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="G89" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="H89" t="str">
         <v/>
@@ -6024,22 +6024,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B90" t="str">
-        <v>Lori Wylie (NL)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="C90" t="str">
-        <v>Available</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D90" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E90" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="F90" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="G90" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H90" t="str">
         <v/>
@@ -6050,22 +6050,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B91" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Kaitlyn Barton (NL) (GH)</v>
       </c>
       <c r="C91" t="str">
         <v>Available</v>
       </c>
       <c r="D91" t="str">
-        <v>08:00-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E91" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="F91" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="G91" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="H91" t="str">
         <v/>
@@ -6076,22 +6076,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B92" t="str">
-        <v>Madison Duncan (NL)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="C92" t="str">
         <v>Available</v>
       </c>
       <c r="D92" t="str">
-        <v>08:00-18:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E92" t="str">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F92" t="str">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G92" t="str">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H92" t="str">
         <v/>
@@ -6102,13 +6102,13 @@
         <v>2025-09-15</v>
       </c>
       <c r="B93" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="C93" t="str">
         <v>Available</v>
       </c>
       <c r="D93" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E93" t="str">
         <v>4</v>
@@ -6128,22 +6128,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B94" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Madison Duncan (NL)</v>
       </c>
       <c r="C94" t="str">
         <v>Available</v>
       </c>
       <c r="D94" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E94" t="str">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F94" t="str">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G94" t="str">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H94" t="str">
         <v/>
@@ -6154,25 +6154,25 @@
         <v>2025-09-15</v>
       </c>
       <c r="B95" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Makala Mcewan (NL) (GH)</v>
       </c>
       <c r="C95" t="str">
         <v>Available</v>
       </c>
       <c r="D95" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="E95" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="F95" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="G95" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="H95" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="96">
@@ -6180,22 +6180,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B96" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="C96" t="str">
         <v>Available</v>
       </c>
       <c r="D96" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E96" t="str">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="F96" t="str">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="G96" t="str">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="H96" t="str">
         <v/>
@@ -6206,48 +6206,48 @@
         <v>2025-09-15</v>
       </c>
       <c r="B97" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="C97" t="str">
         <v>Available</v>
       </c>
       <c r="D97" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="E97" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="F97" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="G97" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H97" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>2025-09-21</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B98" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Sharon Jack (NL)</v>
       </c>
       <c r="C98" t="str">
         <v>Available</v>
       </c>
       <c r="D98" t="str">
-        <v>08:00-18:00</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E98" t="str">
-        <v>5.33</v>
+        <v>4.8</v>
       </c>
       <c r="F98" t="str">
-        <v>5.33</v>
+        <v>4.8</v>
       </c>
       <c r="G98" t="str">
-        <v>5.33</v>
+        <v>4.8</v>
       </c>
       <c r="H98" t="str">
         <v/>
@@ -6255,25 +6255,25 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>2025-09-21</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B99" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="C99" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D99" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E99" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="F99" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="G99" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H99" t="str">
         <v/>
@@ -6284,22 +6284,22 @@
         <v>2025-09-21</v>
       </c>
       <c r="B100" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Anne Nelson (NL)</v>
       </c>
       <c r="C100" t="str">
         <v>Available</v>
       </c>
       <c r="D100" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E100" t="str">
-        <v>2.67</v>
+        <v>5.33</v>
       </c>
       <c r="F100" t="str">
-        <v>2.67</v>
+        <v>5.33</v>
       </c>
       <c r="G100" t="str">
-        <v>2.67</v>
+        <v>5.33</v>
       </c>
       <c r="H100" t="str">
         <v/>
@@ -6310,25 +6310,25 @@
         <v>2025-09-21</v>
       </c>
       <c r="B101" t="str">
-        <v>Emma Shawcross (NL)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C101" t="str">
-        <v>Available</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D101" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E101" t="str">
-        <v>10</v>
+        <v>2.29</v>
       </c>
       <c r="F101" t="str">
-        <v>10</v>
+        <v>2.29</v>
       </c>
       <c r="G101" t="str">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H101" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="102">
@@ -6336,22 +6336,22 @@
         <v>2025-09-21</v>
       </c>
       <c r="B102" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C102" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D102" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E102" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="F102" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="G102" t="str">
-        <v>0</v>
+        <v>2.67</v>
       </c>
       <c r="H102" t="str">
         <v/>
@@ -6362,25 +6362,25 @@
         <v>2025-09-21</v>
       </c>
       <c r="B103" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Duncan (NL), Madison</v>
       </c>
       <c r="C103" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D103" t="str">
-        <v>08:00-21:30</v>
+        <v>16:45-19:00</v>
       </c>
       <c r="E103" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="F103" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G103" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H103" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="104">
@@ -6388,25 +6388,25 @@
         <v>2025-09-21</v>
       </c>
       <c r="B104" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Emma Shawcross (NL)</v>
       </c>
       <c r="C104" t="str">
         <v>Available</v>
       </c>
       <c r="D104" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E104" t="str">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F104" t="str">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G104" t="str">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H104" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="105">
@@ -6414,30 +6414,108 @@
         <v>2025-09-21</v>
       </c>
       <c r="B105" t="str">
+        <v>Hamza Nafees (NL) (GH)</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Other Unavailable</v>
+      </c>
+      <c r="D105" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E105" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="F105" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="G105" t="str">
+        <v>0</v>
+      </c>
+      <c r="H105" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>2025-09-21</v>
+      </c>
+      <c r="B106" t="str">
+        <v>Kaitlyn Barton (NL) (GH)</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D106" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E106" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="F106" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="G106" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="H106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>2025-09-21</v>
+      </c>
+      <c r="B107" t="str">
+        <v>Makala Mcewan (NL) (GH)</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D107" t="str">
+        <v>08:00-15:15</v>
+      </c>
+      <c r="E107" t="str">
+        <v>4</v>
+      </c>
+      <c r="F107" t="str">
+        <v>4</v>
+      </c>
+      <c r="G107" t="str">
+        <v>4</v>
+      </c>
+      <c r="H107" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>2025-09-21</v>
+      </c>
+      <c r="B108" t="str">
         <v>Wayne (GH) Griffiths (NL)</v>
       </c>
-      <c r="C105" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D105" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E105" t="str">
-        <v>6</v>
-      </c>
-      <c r="F105" t="str">
-        <v>6</v>
-      </c>
-      <c r="G105" t="str">
-        <v>6</v>
-      </c>
-      <c r="H105" t="str">
+      <c r="C108" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D108" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E108" t="str">
+        <v>6</v>
+      </c>
+      <c r="F108" t="str">
+        <v>6</v>
+      </c>
+      <c r="G108" t="str">
+        <v>6</v>
+      </c>
+      <c r="H108" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H105"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H108"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Improve data storage and retrieval for weekly capacity analysis
Introduce unique constraints and indexes on week start and end dates for the capacity_analyses table. Add helper functions to determine canonical week boundaries for accurate data processing and querying.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 1bf77d94-6174-484a-826e-43c760e37b4c
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/1bf77d94-6174-484a-826e-43c760e37b4c/wUlw99X
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I105"/>
+  <dimension ref="A1:I106"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -790,644 +790,649 @@
     </row>
     <row r="14" xml:space="preserve">
       <c r="A14" t="str">
+        <v>Brooke O'Brien (NL) (GH)</v>
+      </c>
+      <c r="B14" t="str">
+        <v>16</v>
+      </c>
+      <c r="C14" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="D14" t="str">
+        <v>2025-09-15</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Sick</v>
+      </c>
+      <c r="F14" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G14" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="H14" t="str">
+        <v>0</v>
+      </c>
+      <c r="I14" t="str" xml:space="preserve">
+        <v xml:space="preserve">Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM
+New sick line 11/09 for 1 week - MT; Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>Brooke O'Brien (NL) (GH)</v>
+      </c>
+      <c r="B15" t="str">
+        <v>16</v>
+      </c>
+      <c r="C15" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="D15" t="str">
+        <v>2025-09-16</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Sick</v>
+      </c>
+      <c r="F15" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G15" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="H15" t="str">
+        <v>0</v>
+      </c>
+      <c r="I15" t="str" xml:space="preserve">
+        <v xml:space="preserve">Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM
+New sick line 11/09 for 1 week - MT; Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>Brooke O'Brien (NL) (GH)</v>
+      </c>
+      <c r="B16" t="str">
+        <v>16</v>
+      </c>
+      <c r="C16" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="D16" t="str">
+        <v>2025-09-17</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Sick</v>
+      </c>
+      <c r="F16" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G16" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="H16" t="str">
+        <v>0</v>
+      </c>
+      <c r="I16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM
+New sick line 11/09 for 1 week - MT; Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>Brooke O'Brien (NL) (GH)</v>
+      </c>
+      <c r="B17" t="str">
+        <v>16</v>
+      </c>
+      <c r="C17" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="D17" t="str">
+        <v>2025-09-18</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Sick</v>
+      </c>
+      <c r="F17" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G17" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="H17" t="str">
+        <v>0</v>
+      </c>
+      <c r="I17" t="str" xml:space="preserve">
+        <v xml:space="preserve">Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM
+New sick line 11/09 for 1 week - MT</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>Brooke O'Brien (NL) (GH)</v>
+      </c>
+      <c r="B18" t="str">
+        <v>16</v>
+      </c>
+      <c r="C18" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="D18" t="str">
+        <v>2025-09-19</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Sick</v>
+      </c>
+      <c r="F18" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G18" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="H18" t="str">
+        <v>0</v>
+      </c>
+      <c r="I18" t="str" xml:space="preserve">
+        <v xml:space="preserve">Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM
+New sick line 11/09 for 1 week - MT</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Makala Mcewan (NL) (GH)</v>
+      </c>
+      <c r="B19" t="str">
+        <v>16</v>
+      </c>
+      <c r="C19" t="str">
+        <v>4</v>
+      </c>
+      <c r="D19" t="str">
+        <v>2025-09-15</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Compassionate Leave</v>
+      </c>
+      <c r="F19" t="str">
+        <v>08:00-15:15</v>
+      </c>
+      <c r="G19" t="str">
+        <v>4</v>
+      </c>
+      <c r="H19" t="str">
+        <v>0</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Makala called to advise her papa has passed away today - MT</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
         <v>Shafiya Fayaz GH</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B20" t="str">
         <v>45</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C20" t="str">
         <v>9</v>
       </c>
-      <c r="D14" t="str">
+      <c r="D20" t="str">
         <v>2025-09-16</v>
       </c>
-      <c r="E14" t="str">
+      <c r="E20" t="str">
         <v>Other Unavailable</v>
       </c>
-      <c r="F14" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="G14" t="str">
+      <c r="F20" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G20" t="str">
         <v>9</v>
       </c>
-      <c r="H14" t="str">
-        <v>0</v>
-      </c>
-      <c r="I14" t="str" xml:space="preserve">
+      <c r="H20" t="str">
+        <v>0</v>
+      </c>
+      <c r="I20" t="str" xml:space="preserve">
         <v xml:space="preserve">Megan approved 
 Eilidh 02/07/2025</v>
       </c>
     </row>
-    <row r="15" xml:space="preserve">
-      <c r="A15" t="str">
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
         <v>Shafiya Fayaz GH</v>
       </c>
-      <c r="B15" t="str">
+      <c r="B21" t="str">
         <v>45</v>
       </c>
-      <c r="C15" t="str">
+      <c r="C21" t="str">
         <v>9</v>
       </c>
-      <c r="D15" t="str">
+      <c r="D21" t="str">
         <v>2025-09-17</v>
       </c>
-      <c r="E15" t="str">
+      <c r="E21" t="str">
         <v>Other Unavailable</v>
       </c>
-      <c r="F15" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="G15" t="str">
+      <c r="F21" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G21" t="str">
         <v>9</v>
       </c>
-      <c r="H15" t="str">
-        <v>0</v>
-      </c>
-      <c r="I15" t="str" xml:space="preserve">
+      <c r="H21" t="str">
+        <v>0</v>
+      </c>
+      <c r="I21" t="str" xml:space="preserve">
         <v xml:space="preserve">Megan approved 
 Eilidh 02/07/2025</v>
       </c>
     </row>
-    <row r="16" xml:space="preserve">
-      <c r="A16" t="str">
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
         <v>Shafiya Fayaz GH</v>
       </c>
-      <c r="B16" t="str">
+      <c r="B22" t="str">
         <v>45</v>
       </c>
-      <c r="C16" t="str">
+      <c r="C22" t="str">
         <v>9</v>
       </c>
-      <c r="D16" t="str">
+      <c r="D22" t="str">
         <v>2025-09-18</v>
       </c>
-      <c r="E16" t="str">
+      <c r="E22" t="str">
         <v>Other Unavailable</v>
       </c>
-      <c r="F16" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="G16" t="str">
+      <c r="F22" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G22" t="str">
         <v>9</v>
       </c>
-      <c r="H16" t="str">
-        <v>0</v>
-      </c>
-      <c r="I16" t="str" xml:space="preserve">
+      <c r="H22" t="str">
+        <v>0</v>
+      </c>
+      <c r="I22" t="str" xml:space="preserve">
         <v xml:space="preserve">Megan approved 
 Eilidh 02/07/2025</v>
       </c>
     </row>
-    <row r="17" xml:space="preserve">
-      <c r="A17" t="str">
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
         <v>Shafiya Fayaz GH</v>
       </c>
-      <c r="B17" t="str">
+      <c r="B23" t="str">
         <v>45</v>
       </c>
-      <c r="C17" t="str">
+      <c r="C23" t="str">
         <v>9</v>
       </c>
-      <c r="D17" t="str">
+      <c r="D23" t="str">
         <v>2025-09-19</v>
       </c>
-      <c r="E17" t="str">
+      <c r="E23" t="str">
         <v>Other Unavailable</v>
       </c>
-      <c r="F17" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="G17" t="str">
+      <c r="F23" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G23" t="str">
         <v>9</v>
       </c>
-      <c r="H17" t="str">
-        <v>0</v>
-      </c>
-      <c r="I17" t="str" xml:space="preserve">
+      <c r="H23" t="str">
+        <v>0</v>
+      </c>
+      <c r="I23" t="str" xml:space="preserve">
         <v xml:space="preserve">Megan approved 
 Eilidh 02/07/2025</v>
       </c>
     </row>
-    <row r="18" xml:space="preserve">
-      <c r="A18" t="str">
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
         <v>Shafiya Fayaz GH</v>
       </c>
-      <c r="B18" t="str">
+      <c r="B24" t="str">
         <v>45</v>
       </c>
-      <c r="C18" t="str">
+      <c r="C24" t="str">
         <v>9</v>
       </c>
-      <c r="D18" t="str">
+      <c r="D24" t="str">
         <v>2025-09-20</v>
       </c>
-      <c r="E18" t="str">
+      <c r="E24" t="str">
         <v>Other Unavailable</v>
       </c>
-      <c r="F18" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="G18" t="str">
+      <c r="F24" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G24" t="str">
         <v>9</v>
       </c>
-      <c r="H18" t="str">
-        <v>0</v>
-      </c>
-      <c r="I18" t="str" xml:space="preserve">
+      <c r="H24" t="str">
+        <v>0</v>
+      </c>
+      <c r="I24" t="str" xml:space="preserve">
         <v xml:space="preserve">Megan approved 
 Eilidh 02/07/2025</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="str">
+    <row r="25">
+      <c r="A25" t="str">
         <v>Hamza Nafees (NL) (GH)</v>
       </c>
-      <c r="B19" t="str">
+      <c r="B25" t="str">
         <v>45</v>
       </c>
-      <c r="C19" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="D19" t="str">
+      <c r="C25" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D25" t="str">
         <v>2025-09-15</v>
-      </c>
-      <c r="E19" t="str">
-        <v>Other Unavailable</v>
-      </c>
-      <c r="F19" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="G19" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H19" t="str">
-        <v>0</v>
-      </c>
-      <c r="I19" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
-      </c>
-      <c r="B20" t="str">
-        <v>45</v>
-      </c>
-      <c r="C20" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="D20" t="str">
-        <v>2025-09-16</v>
-      </c>
-      <c r="E20" t="str">
-        <v>Other Unavailable</v>
-      </c>
-      <c r="F20" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="G20" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H20" t="str">
-        <v>0</v>
-      </c>
-      <c r="I20" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
-      </c>
-      <c r="B21" t="str">
-        <v>45</v>
-      </c>
-      <c r="C21" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="D21" t="str">
-        <v>2025-09-17</v>
-      </c>
-      <c r="E21" t="str">
-        <v>Other Unavailable</v>
-      </c>
-      <c r="F21" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="G21" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H21" t="str">
-        <v>0</v>
-      </c>
-      <c r="I21" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
-      </c>
-      <c r="B22" t="str">
-        <v>45</v>
-      </c>
-      <c r="C22" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="D22" t="str">
-        <v>2025-09-18</v>
-      </c>
-      <c r="E22" t="str">
-        <v>Other Unavailable</v>
-      </c>
-      <c r="F22" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="G22" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H22" t="str">
-        <v>0</v>
-      </c>
-      <c r="I22" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
-      </c>
-      <c r="B23" t="str">
-        <v>45</v>
-      </c>
-      <c r="C23" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="D23" t="str">
-        <v>2025-09-21</v>
-      </c>
-      <c r="E23" t="str">
-        <v>Other Unavailable</v>
-      </c>
-      <c r="F23" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="G23" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H23" t="str">
-        <v>0</v>
-      </c>
-      <c r="I23" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>Sharon Jack (NL)</v>
-      </c>
-      <c r="B24" t="str">
-        <v>24</v>
-      </c>
-      <c r="C24" t="str">
-        <v>4.8</v>
-      </c>
-      <c r="D24" t="str">
-        <v>2025-09-16</v>
-      </c>
-      <c r="E24" t="str">
-        <v>Other Unavailable</v>
-      </c>
-      <c r="F24" t="str">
-        <v>09:15-16:15</v>
-      </c>
-      <c r="G24" t="str">
-        <v>2</v>
-      </c>
-      <c r="H24" t="str">
-        <v>0</v>
-      </c>
-      <c r="I24" t="str">
-        <v>Sharon has advised she is unable to work between 10.30 and 12.30 on Tuesday's - MT</v>
-      </c>
-    </row>
-    <row r="25" xml:space="preserve">
-      <c r="A25" t="str">
-        <v>Sharon Jack (NL)</v>
-      </c>
-      <c r="B25" t="str">
-        <v>24</v>
-      </c>
-      <c r="C25" t="str">
-        <v>4.8</v>
-      </c>
-      <c r="D25" t="str">
-        <v>2025-09-17</v>
       </c>
       <c r="E25" t="str">
         <v>Other Unavailable</v>
       </c>
       <c r="F25" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G25" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="H25" t="str">
+        <v>0</v>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Hamza Nafees (NL) (GH)</v>
+      </c>
+      <c r="B26" t="str">
+        <v>45</v>
+      </c>
+      <c r="C26" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D26" t="str">
+        <v>2025-09-16</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Other Unavailable</v>
+      </c>
+      <c r="F26" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G26" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="H26" t="str">
+        <v>0</v>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Hamza Nafees (NL) (GH)</v>
+      </c>
+      <c r="B27" t="str">
+        <v>45</v>
+      </c>
+      <c r="C27" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D27" t="str">
+        <v>2025-09-17</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Other Unavailable</v>
+      </c>
+      <c r="F27" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G27" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="H27" t="str">
+        <v>0</v>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Hamza Nafees (NL) (GH)</v>
+      </c>
+      <c r="B28" t="str">
+        <v>45</v>
+      </c>
+      <c r="C28" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D28" t="str">
+        <v>2025-09-18</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Other Unavailable</v>
+      </c>
+      <c r="F28" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G28" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="H28" t="str">
+        <v>0</v>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Hamza Nafees (NL) (GH)</v>
+      </c>
+      <c r="B29" t="str">
+        <v>45</v>
+      </c>
+      <c r="C29" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D29" t="str">
+        <v>2025-09-21</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Other Unavailable</v>
+      </c>
+      <c r="F29" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="G29" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="H29" t="str">
+        <v>0</v>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Sharon Jack (NL)</v>
+      </c>
+      <c r="B30" t="str">
+        <v>24</v>
+      </c>
+      <c r="C30" t="str">
+        <v>4.8</v>
+      </c>
+      <c r="D30" t="str">
+        <v>2025-09-16</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Other Unavailable</v>
+      </c>
+      <c r="F30" t="str">
+        <v>09:15-16:15</v>
+      </c>
+      <c r="G30" t="str">
+        <v>2</v>
+      </c>
+      <c r="H30" t="str">
+        <v>0</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Sharon has advised she is unable to work between 10.30 and 12.30 on Tuesday's - MT</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
+        <v>Sharon Jack (NL)</v>
+      </c>
+      <c r="B31" t="str">
+        <v>24</v>
+      </c>
+      <c r="C31" t="str">
+        <v>4.8</v>
+      </c>
+      <c r="D31" t="str">
+        <v>2025-09-17</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Other Unavailable</v>
+      </c>
+      <c r="F31" t="str">
         <v>09:15-16:30</v>
       </c>
-      <c r="G25" t="str">
+      <c r="G31" t="str">
         <v>2</v>
       </c>
-      <c r="H25" t="str">
-        <v>0</v>
-      </c>
-      <c r="I25" t="str" xml:space="preserve">
+      <c r="H31" t="str">
+        <v>0</v>
+      </c>
+      <c r="I31" t="str" xml:space="preserve">
         <v xml:space="preserve">Wants this as a break. 
 Eilidh 29/05/2025</v>
       </c>
     </row>
-    <row r="26" xml:space="preserve">
-      <c r="A26" t="str">
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
         <v>Sharon Jack (NL)</v>
       </c>
-      <c r="B26" t="str">
+      <c r="B32" t="str">
         <v>24</v>
       </c>
-      <c r="C26" t="str">
+      <c r="C32" t="str">
         <v>4.8</v>
       </c>
-      <c r="D26" t="str">
+      <c r="D32" t="str">
         <v>2025-09-19</v>
       </c>
-      <c r="E26" t="str">
+      <c r="E32" t="str">
         <v>Other Unavailable</v>
       </c>
-      <c r="F26" t="str">
+      <c r="F32" t="str">
         <v>09:15-17:00</v>
       </c>
-      <c r="G26" t="str">
+      <c r="G32" t="str">
         <v>2</v>
       </c>
-      <c r="H26" t="str">
-        <v>0</v>
-      </c>
-      <c r="I26" t="str" xml:space="preserve">
+      <c r="H32" t="str">
+        <v>0</v>
+      </c>
+      <c r="I32" t="str" xml:space="preserve">
         <v xml:space="preserve">Wants this as a break. 
 Eilidh 29/05/2025</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
-      </c>
-      <c r="B27" t="str">
-        <v>16</v>
-      </c>
-      <c r="C27" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D27" t="str">
-        <v>2025-09-15</v>
-      </c>
-      <c r="E27" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F27" t="str">
-        <v>10:30-14:00</v>
-      </c>
-      <c r="G27" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H27" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I27" t="str">
-        <v>Confirmed at induction with MT</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
-      </c>
-      <c r="B28" t="str">
-        <v>16</v>
-      </c>
-      <c r="C28" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D28" t="str">
-        <v>2025-09-16</v>
-      </c>
-      <c r="E28" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F28" t="str">
-        <v>09:15-15:15</v>
-      </c>
-      <c r="G28" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H28" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I28" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
-      </c>
-      <c r="B29" t="str">
-        <v>16</v>
-      </c>
-      <c r="C29" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D29" t="str">
-        <v>2025-09-17</v>
-      </c>
-      <c r="E29" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F29" t="str">
-        <v>09:15-15:15</v>
-      </c>
-      <c r="G29" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H29" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I29" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
-      </c>
-      <c r="B30" t="str">
-        <v>16</v>
-      </c>
-      <c r="C30" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D30" t="str">
-        <v>2025-09-18</v>
-      </c>
-      <c r="E30" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F30" t="str">
-        <v>09:15-15:15</v>
-      </c>
-      <c r="G30" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H30" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I30" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
-      </c>
-      <c r="B31" t="str">
-        <v>16</v>
-      </c>
-      <c r="C31" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D31" t="str">
-        <v>2025-09-19</v>
-      </c>
-      <c r="E31" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F31" t="str">
-        <v>10:30-14:00</v>
-      </c>
-      <c r="G31" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H31" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I31" t="str">
-        <v>Confirmed at induction with MT</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
-      </c>
-      <c r="B32" t="str">
-        <v>16</v>
-      </c>
-      <c r="C32" t="str">
-        <v>2.67</v>
-      </c>
-      <c r="D32" t="str">
-        <v>2025-09-15</v>
-      </c>
-      <c r="E32" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F32" t="str">
-        <v>09:15-14:00</v>
-      </c>
-      <c r="G32" t="str">
-        <v>2.67</v>
-      </c>
-      <c r="H32" t="str">
-        <v>2.67</v>
-      </c>
-      <c r="I32" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
-      </c>
-    </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="B33" t="str">
         <v>16</v>
       </c>
       <c r="C33" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="D33" t="str">
-        <v>2025-09-16</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E33" t="str">
         <v>Available</v>
       </c>
       <c r="F33" t="str">
-        <v>09:15-14:00</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="G33" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="H33" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="I33" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="B34" t="str">
         <v>16</v>
       </c>
       <c r="C34" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="D34" t="str">
-        <v>2025-09-17</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E34" t="str">
         <v>Available</v>
       </c>
       <c r="F34" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G34" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="H34" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="I34" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="B35" t="str">
         <v>16</v>
       </c>
       <c r="C35" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="D35" t="str">
-        <v>2025-09-18</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E35" t="str">
         <v>Available</v>
       </c>
       <c r="F35" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G35" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="H35" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="I35" t="str">
         <v/>
@@ -1435,28 +1440,28 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="B36" t="str">
         <v>16</v>
       </c>
       <c r="C36" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="D36" t="str">
-        <v>2025-09-20</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E36" t="str">
         <v>Available</v>
       </c>
       <c r="F36" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G36" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="H36" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="I36" t="str">
         <v/>
@@ -1464,74 +1469,74 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="B37" t="str">
         <v>16</v>
       </c>
       <c r="C37" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="D37" t="str">
-        <v>2025-09-21</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E37" t="str">
         <v>Available</v>
       </c>
       <c r="F37" t="str">
-        <v>09:15-14:00</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="G37" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="H37" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="I37" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="B38" t="str">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C38" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="D38" t="str">
-        <v>2025-09-15</v>
+        <v>2025-09-20</v>
       </c>
       <c r="E38" t="str">
         <v>Available</v>
       </c>
       <c r="F38" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G38" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="H38" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="I38" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="B39" t="str">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C39" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="D39" t="str">
-        <v>2025-09-16</v>
+        <v>2025-09-21</v>
       </c>
       <c r="E39" t="str">
         <v>Available</v>
@@ -1540,13 +1545,13 @@
         <v>09:15-14:00</v>
       </c>
       <c r="G39" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="H39" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="I39" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -1560,7 +1565,7 @@
         <v>4</v>
       </c>
       <c r="D40" t="str">
-        <v>2025-09-17</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E40" t="str">
         <v>Available</v>
@@ -1589,7 +1594,7 @@
         <v>4</v>
       </c>
       <c r="D41" t="str">
-        <v>2025-09-18</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E41" t="str">
         <v>Available</v>
@@ -1618,7 +1623,7 @@
         <v>4</v>
       </c>
       <c r="D42" t="str">
-        <v>2025-09-19</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E42" t="str">
         <v>Available</v>
@@ -1638,60 +1643,60 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="B43" t="str">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C43" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="D43" t="str">
-        <v>2025-09-15</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E43" t="str">
         <v>Available</v>
       </c>
       <c r="F43" t="str">
-        <v>09:15-14:45</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G43" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="H43" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="I43" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="B44" t="str">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C44" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="D44" t="str">
-        <v>2025-09-16</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E44" t="str">
         <v>Available</v>
       </c>
       <c r="F44" t="str">
-        <v>09:15-11:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G44" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="H44" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="I44" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="45">
@@ -1705,7 +1710,7 @@
         <v>2.8</v>
       </c>
       <c r="D45" t="str">
-        <v>2025-09-17</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E45" t="str">
         <v>Available</v>
@@ -1734,7 +1739,7 @@
         <v>2.8</v>
       </c>
       <c r="D46" t="str">
-        <v>2025-09-18</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E46" t="str">
         <v>Available</v>
@@ -1763,13 +1768,13 @@
         <v>2.8</v>
       </c>
       <c r="D47" t="str">
-        <v>2025-09-19</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E47" t="str">
         <v>Available</v>
       </c>
       <c r="F47" t="str">
-        <v>09:15-10:15</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="G47" t="str">
         <v>2.8</v>
@@ -1783,74 +1788,74 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Emma Shawcross (NL)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="B48" t="str">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C48" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="D48" t="str">
-        <v>2025-09-20</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E48" t="str">
         <v>Available</v>
       </c>
       <c r="F48" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-11:30</v>
       </c>
       <c r="G48" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="H48" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="I48" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Emma Shawcross (NL)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="B49" t="str">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C49" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="D49" t="str">
-        <v>2025-09-21</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E49" t="str">
         <v>Available</v>
       </c>
       <c r="F49" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G49" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="H49" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="I49" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Emma Shawcross (NL)</v>
       </c>
       <c r="B50" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C50" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="D50" t="str">
-        <v>2025-09-15</v>
+        <v>2025-09-20</v>
       </c>
       <c r="E50" t="str">
         <v>Available</v>
@@ -1859,27 +1864,27 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G50" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="H50" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="I50" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Emma Shawcross (NL)</v>
       </c>
       <c r="B51" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C51" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="D51" t="str">
-        <v>2025-09-16</v>
+        <v>2025-09-21</v>
       </c>
       <c r="E51" t="str">
         <v>Available</v>
@@ -1888,13 +1893,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G51" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="H51" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="I51" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="52">
@@ -1908,7 +1913,7 @@
         <v>7.5</v>
       </c>
       <c r="D52" t="str">
-        <v>2025-09-20</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E52" t="str">
         <v>Available</v>
@@ -1937,7 +1942,7 @@
         <v>7.5</v>
       </c>
       <c r="D53" t="str">
-        <v>2025-09-21</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E53" t="str">
         <v>Available</v>
@@ -1957,28 +1962,28 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Madison Duncan (NL)</v>
+        <v>Kaitlyn Barton (NL) (GH)</v>
       </c>
       <c r="B54" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C54" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="D54" t="str">
-        <v>2025-09-15</v>
+        <v>2025-09-20</v>
       </c>
       <c r="E54" t="str">
         <v>Available</v>
       </c>
       <c r="F54" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G54" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="H54" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="I54" t="str">
         <v/>
@@ -1986,28 +1991,28 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Madison Duncan (NL)</v>
+        <v>Kaitlyn Barton (NL) (GH)</v>
       </c>
       <c r="B55" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C55" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="D55" t="str">
-        <v>2025-09-16</v>
+        <v>2025-09-21</v>
       </c>
       <c r="E55" t="str">
         <v>Available</v>
       </c>
       <c r="F55" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G55" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="H55" t="str">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="I55" t="str">
         <v/>
@@ -2015,13 +2020,13 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Madison Duncan (NL)</v>
       </c>
       <c r="B56" t="str">
         <v>16</v>
       </c>
       <c r="C56" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D56" t="str">
         <v>2025-09-15</v>
@@ -2030,13 +2035,13 @@
         <v>Available</v>
       </c>
       <c r="F56" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="G56" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H56" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I56" t="str">
         <v/>
@@ -2044,28 +2049,28 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Madison Duncan (NL)</v>
       </c>
       <c r="B57" t="str">
         <v>16</v>
       </c>
       <c r="C57" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D57" t="str">
-        <v>2025-09-17</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E57" t="str">
         <v>Available</v>
       </c>
       <c r="F57" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="G57" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H57" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I57" t="str">
         <v/>
@@ -2082,7 +2087,7 @@
         <v>4</v>
       </c>
       <c r="D58" t="str">
-        <v>2025-09-20</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E58" t="str">
         <v>Available</v>
@@ -2111,7 +2116,7 @@
         <v>4</v>
       </c>
       <c r="D59" t="str">
-        <v>2025-09-21</v>
+        <v>2025-09-20</v>
       </c>
       <c r="E59" t="str">
         <v>Available</v>
@@ -2131,28 +2136,28 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Marykate Ferris (NL)</v>
+        <v>Makala Mcewan (NL) (GH)</v>
       </c>
       <c r="B60" t="str">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C60" t="str">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D60" t="str">
-        <v>2025-09-18</v>
+        <v>2025-09-21</v>
       </c>
       <c r="E60" t="str">
         <v>Available</v>
       </c>
       <c r="F60" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="G60" t="str">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H60" t="str">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I60" t="str">
         <v/>
@@ -2169,7 +2174,7 @@
         <v>10</v>
       </c>
       <c r="D61" t="str">
-        <v>2025-09-19</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E61" t="str">
         <v>Available</v>
@@ -2189,28 +2194,28 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="B62" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C62" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="D62" t="str">
-        <v>2025-09-16</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E62" t="str">
         <v>Available</v>
       </c>
       <c r="F62" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G62" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="H62" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="I62" t="str">
         <v/>
@@ -2227,13 +2232,13 @@
         <v>7.5</v>
       </c>
       <c r="D63" t="str">
-        <v>2025-09-17</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E63" t="str">
         <v>Available</v>
       </c>
       <c r="F63" t="str">
-        <v>08:00-21:30</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G63" t="str">
         <v>7.5</v>
@@ -2256,7 +2261,7 @@
         <v>7.5</v>
       </c>
       <c r="D64" t="str">
-        <v>2025-09-18</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E64" t="str">
         <v>Available</v>
@@ -2285,7 +2290,7 @@
         <v>7.5</v>
       </c>
       <c r="D65" t="str">
-        <v>2025-09-19</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E65" t="str">
         <v>Available</v>
@@ -2305,7 +2310,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Adedayo Adeyanju (NL) (GH)</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="B66" t="str">
         <v>30</v>
@@ -2314,7 +2319,7 @@
         <v>7.5</v>
       </c>
       <c r="D66" t="str">
-        <v>2025-09-16</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E66" t="str">
         <v>Available</v>
@@ -2343,7 +2348,7 @@
         <v>7.5</v>
       </c>
       <c r="D67" t="str">
-        <v>2025-09-17</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E67" t="str">
         <v>Available</v>
@@ -2372,7 +2377,7 @@
         <v>7.5</v>
       </c>
       <c r="D68" t="str">
-        <v>2025-09-18</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E68" t="str">
         <v>Available</v>
@@ -2401,7 +2406,7 @@
         <v>7.5</v>
       </c>
       <c r="D69" t="str">
-        <v>2025-09-19</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E69" t="str">
         <v>Available</v>
@@ -2421,10 +2426,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Adedayo Adeyanju (NL) (GH)</v>
       </c>
       <c r="B70" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C70" t="str">
         <v>7.5</v>
@@ -2450,16 +2455,16 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="B71" t="str">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C71" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="D71" t="str">
-        <v>2025-09-15</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E71" t="str">
         <v>Available</v>
@@ -2468,10 +2473,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G71" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="H71" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="I71" t="str">
         <v/>
@@ -2488,7 +2493,7 @@
         <v>6</v>
       </c>
       <c r="D72" t="str">
-        <v>2025-09-16</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E72" t="str">
         <v>Available</v>
@@ -2517,7 +2522,7 @@
         <v>6</v>
       </c>
       <c r="D73" t="str">
-        <v>2025-09-17</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E73" t="str">
         <v>Available</v>
@@ -2546,7 +2551,7 @@
         <v>6</v>
       </c>
       <c r="D74" t="str">
-        <v>2025-09-19</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E74" t="str">
         <v>Available</v>
@@ -2575,7 +2580,7 @@
         <v>6</v>
       </c>
       <c r="D75" t="str">
-        <v>2025-09-20</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E75" t="str">
         <v>Available</v>
@@ -2595,31 +2600,31 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="B76" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C76" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="D76" t="str">
-        <v>2025-09-15</v>
+        <v>2025-09-20</v>
       </c>
       <c r="E76" t="str">
         <v>Available</v>
       </c>
       <c r="F76" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G76" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H76" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="I76" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="77">
@@ -2633,7 +2638,7 @@
         <v>3.2</v>
       </c>
       <c r="D77" t="str">
-        <v>2025-09-16</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E77" t="str">
         <v>Available</v>
@@ -2662,7 +2667,7 @@
         <v>3.2</v>
       </c>
       <c r="D78" t="str">
-        <v>2025-09-17</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E78" t="str">
         <v>Available</v>
@@ -2691,7 +2696,7 @@
         <v>3.2</v>
       </c>
       <c r="D79" t="str">
-        <v>2025-09-18</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E79" t="str">
         <v>Available</v>
@@ -2720,7 +2725,7 @@
         <v>3.2</v>
       </c>
       <c r="D80" t="str">
-        <v>2025-09-19</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E80" t="str">
         <v>Available</v>
@@ -2740,31 +2745,31 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="B81" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C81" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D81" t="str">
-        <v>2025-09-15</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E81" t="str">
         <v>Available</v>
       </c>
       <c r="F81" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="G81" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H81" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I81" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="82">
@@ -2778,7 +2783,7 @@
         <v>6</v>
       </c>
       <c r="D82" t="str">
-        <v>2025-09-16</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E82" t="str">
         <v>Available</v>
@@ -2807,7 +2812,7 @@
         <v>6</v>
       </c>
       <c r="D83" t="str">
-        <v>2025-09-17</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E83" t="str">
         <v>Available</v>
@@ -2836,7 +2841,7 @@
         <v>6</v>
       </c>
       <c r="D84" t="str">
-        <v>2025-09-18</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E84" t="str">
         <v>Available</v>
@@ -2865,7 +2870,7 @@
         <v>6</v>
       </c>
       <c r="D85" t="str">
-        <v>2025-09-21</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E85" t="str">
         <v>Available</v>
@@ -2885,28 +2890,28 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="B86" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C86" t="str">
-        <v>5.33</v>
+        <v>6</v>
       </c>
       <c r="D86" t="str">
-        <v>2025-09-18</v>
+        <v>2025-09-21</v>
       </c>
       <c r="E86" t="str">
         <v>Available</v>
       </c>
       <c r="F86" t="str">
-        <v>08:00-17:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G86" t="str">
-        <v>5.33</v>
+        <v>6</v>
       </c>
       <c r="H86" t="str">
-        <v>5.33</v>
+        <v>6</v>
       </c>
       <c r="I86" t="str">
         <v/>
@@ -2923,13 +2928,13 @@
         <v>5.33</v>
       </c>
       <c r="D87" t="str">
-        <v>2025-09-19</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E87" t="str">
         <v>Available</v>
       </c>
       <c r="F87" t="str">
-        <v>08:00-13:00</v>
+        <v>08:00-17:15</v>
       </c>
       <c r="G87" t="str">
         <v>5.33</v>
@@ -2952,13 +2957,13 @@
         <v>5.33</v>
       </c>
       <c r="D88" t="str">
-        <v>2025-09-21</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E88" t="str">
         <v>Available</v>
       </c>
       <c r="F88" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-13:00</v>
       </c>
       <c r="G88" t="str">
         <v>5.33</v>
@@ -2972,28 +2977,28 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Anne Nelson (NL)</v>
       </c>
       <c r="B89" t="str">
         <v>16</v>
       </c>
       <c r="C89" t="str">
-        <v>3.2</v>
+        <v>5.33</v>
       </c>
       <c r="D89" t="str">
-        <v>2025-09-15</v>
+        <v>2025-09-21</v>
       </c>
       <c r="E89" t="str">
         <v>Available</v>
       </c>
       <c r="F89" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="G89" t="str">
-        <v>3.2</v>
+        <v>5.33</v>
       </c>
       <c r="H89" t="str">
-        <v>3.2</v>
+        <v>5.33</v>
       </c>
       <c r="I89" t="str">
         <v/>
@@ -3010,7 +3015,7 @@
         <v>3.2</v>
       </c>
       <c r="D90" t="str">
-        <v>2025-09-16</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E90" t="str">
         <v>Available</v>
@@ -3039,7 +3044,7 @@
         <v>3.2</v>
       </c>
       <c r="D91" t="str">
-        <v>2025-09-17</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E91" t="str">
         <v>Available</v>
@@ -3068,7 +3073,7 @@
         <v>3.2</v>
       </c>
       <c r="D92" t="str">
-        <v>2025-09-18</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E92" t="str">
         <v>Available</v>
@@ -3097,7 +3102,7 @@
         <v>3.2</v>
       </c>
       <c r="D93" t="str">
-        <v>2025-09-19</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E93" t="str">
         <v>Available</v>
@@ -3117,28 +3122,28 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="B94" t="str">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C94" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="D94" t="str">
-        <v>2025-09-15</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E94" t="str">
         <v>Available</v>
       </c>
       <c r="F94" t="str">
-        <v>08:00-15:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G94" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="H94" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="I94" t="str">
         <v/>
@@ -3155,7 +3160,7 @@
         <v>4</v>
       </c>
       <c r="D95" t="str">
-        <v>2025-09-16</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E95" t="str">
         <v>Available</v>
@@ -3184,7 +3189,7 @@
         <v>4</v>
       </c>
       <c r="D96" t="str">
-        <v>2025-09-17</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E96" t="str">
         <v>Available</v>
@@ -3213,7 +3218,7 @@
         <v>4</v>
       </c>
       <c r="D97" t="str">
-        <v>2025-09-18</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E97" t="str">
         <v>Available</v>
@@ -3242,7 +3247,7 @@
         <v>4</v>
       </c>
       <c r="D98" t="str">
-        <v>2025-09-19</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E98" t="str">
         <v>Available</v>
@@ -3262,28 +3267,28 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="B99" t="str">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C99" t="str">
-        <v>4.8</v>
+        <v>4</v>
       </c>
       <c r="D99" t="str">
-        <v>2025-09-15</v>
+        <v>2025-09-19</v>
       </c>
       <c r="E99" t="str">
         <v>Available</v>
       </c>
       <c r="F99" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="G99" t="str">
-        <v>4.8</v>
+        <v>4</v>
       </c>
       <c r="H99" t="str">
-        <v>4.8</v>
+        <v>4</v>
       </c>
       <c r="I99" t="str">
         <v/>
@@ -3300,13 +3305,13 @@
         <v>4.8</v>
       </c>
       <c r="D100" t="str">
-        <v>2025-09-18</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E100" t="str">
         <v>Available</v>
       </c>
       <c r="F100" t="str">
-        <v>09:15-16:15</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G100" t="str">
         <v>4.8</v>
@@ -3320,28 +3325,28 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Lori Wylie (NL)</v>
+        <v>Sharon Jack (NL)</v>
       </c>
       <c r="B101" t="str">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C101" t="str">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="D101" t="str">
-        <v>2025-09-15</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E101" t="str">
         <v>Available</v>
       </c>
       <c r="F101" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-16:15</v>
       </c>
       <c r="G101" t="str">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="H101" t="str">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="I101" t="str">
         <v/>
@@ -3358,7 +3363,7 @@
         <v>6</v>
       </c>
       <c r="D102" t="str">
-        <v>2025-09-16</v>
+        <v>2025-09-15</v>
       </c>
       <c r="E102" t="str">
         <v>Available</v>
@@ -3387,13 +3392,13 @@
         <v>6</v>
       </c>
       <c r="D103" t="str">
-        <v>2025-09-17</v>
+        <v>2025-09-16</v>
       </c>
       <c r="E103" t="str">
         <v>Available</v>
       </c>
       <c r="F103" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G103" t="str">
         <v>6</v>
@@ -3416,13 +3421,13 @@
         <v>6</v>
       </c>
       <c r="D104" t="str">
-        <v>2025-09-18</v>
+        <v>2025-09-17</v>
       </c>
       <c r="E104" t="str">
         <v>Available</v>
       </c>
       <c r="F104" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="G104" t="str">
         <v>6</v>
@@ -3445,7 +3450,7 @@
         <v>6</v>
       </c>
       <c r="D105" t="str">
-        <v>2025-09-19</v>
+        <v>2025-09-18</v>
       </c>
       <c r="E105" t="str">
         <v>Available</v>
@@ -3463,9 +3468,38 @@
         <v/>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>Lori Wylie (NL)</v>
+      </c>
+      <c r="B106" t="str">
+        <v>30</v>
+      </c>
+      <c r="C106" t="str">
+        <v>6</v>
+      </c>
+      <c r="D106" t="str">
+        <v>2025-09-19</v>
+      </c>
+      <c r="E106" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F106" t="str">
+        <v>09:15-14:00</v>
+      </c>
+      <c r="G106" t="str">
+        <v>6</v>
+      </c>
+      <c r="H106" t="str">
+        <v>6</v>
+      </c>
+      <c r="I106" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I105"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I106"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3505,25 +3539,25 @@
         <v>2025-09-15</v>
       </c>
       <c r="B2" t="str">
-        <v>65.37</v>
+        <v>58.7</v>
       </c>
       <c r="C2" t="str">
-        <v>65.37</v>
+        <v>58.7</v>
       </c>
       <c r="D2" t="str">
-        <v>9.79</v>
+        <v>16.08</v>
       </c>
       <c r="E2" t="str">
         <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>63.25</v>
+        <v>68</v>
       </c>
       <c r="G2" t="str">
-        <v>2.12</v>
+        <v>-9.3</v>
       </c>
       <c r="H2" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="3">
@@ -3531,13 +3565,13 @@
         <v>2025-09-16</v>
       </c>
       <c r="B3" t="str">
-        <v>71.57</v>
+        <v>68.9</v>
       </c>
       <c r="C3" t="str">
-        <v>71.57</v>
+        <v>68.9</v>
       </c>
       <c r="D3" t="str">
-        <v>28.29</v>
+        <v>30.58</v>
       </c>
       <c r="E3" t="str">
         <v>0</v>
@@ -3546,7 +3580,7 @@
         <v>66.75</v>
       </c>
       <c r="G3" t="str">
-        <v>4.82</v>
+        <v>2.15</v>
       </c>
       <c r="H3" t="str">
         <v>Sufficient</v>
@@ -3557,22 +3591,22 @@
         <v>2025-09-17</v>
       </c>
       <c r="B4" t="str">
-        <v>60.07</v>
+        <v>57.4</v>
       </c>
       <c r="C4" t="str">
-        <v>60.07</v>
+        <v>57.4</v>
       </c>
       <c r="D4" t="str">
-        <v>28.29</v>
+        <v>30.58</v>
       </c>
       <c r="E4" t="str">
         <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>71.25</v>
+        <v>73.25</v>
       </c>
       <c r="G4" t="str">
-        <v>-11.18</v>
+        <v>-15.85</v>
       </c>
       <c r="H4" t="str">
         <v>Shortage</v>
@@ -3583,25 +3617,25 @@
         <v>2025-09-18</v>
       </c>
       <c r="B5" t="str">
-        <v>70.2</v>
+        <v>67.53</v>
       </c>
       <c r="C5" t="str">
-        <v>70.2</v>
+        <v>67.53</v>
       </c>
       <c r="D5" t="str">
-        <v>26.29</v>
+        <v>28.58</v>
       </c>
       <c r="E5" t="str">
         <v>0</v>
       </c>
       <c r="F5" t="str">
-        <v>63.75</v>
+        <v>68.5</v>
       </c>
       <c r="G5" t="str">
-        <v>6.45</v>
+        <v>-0.97</v>
       </c>
       <c r="H5" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="6">
@@ -3615,16 +3649,16 @@
         <v>70.23</v>
       </c>
       <c r="D6" t="str">
-        <v>20.79</v>
+        <v>23.08</v>
       </c>
       <c r="E6" t="str">
         <v>0</v>
       </c>
       <c r="F6" t="str">
-        <v>54.75</v>
+        <v>59.5</v>
       </c>
       <c r="G6" t="str">
-        <v>15.48</v>
+        <v>10.73</v>
       </c>
       <c r="H6" t="str">
         <v>Sufficient</v>
@@ -3635,10 +3669,10 @@
         <v>2025-09-20</v>
       </c>
       <c r="B7" t="str">
-        <v>30.17</v>
+        <v>29.79</v>
       </c>
       <c r="C7" t="str">
-        <v>30.17</v>
+        <v>29.79</v>
       </c>
       <c r="D7" t="str">
         <v>18.79</v>
@@ -3647,10 +3681,10 @@
         <v>0</v>
       </c>
       <c r="F7" t="str">
-        <v>44.75</v>
+        <v>45.75</v>
       </c>
       <c r="G7" t="str">
-        <v>-14.58</v>
+        <v>-15.96</v>
       </c>
       <c r="H7" t="str">
         <v>Shortage</v>
@@ -3661,10 +3695,10 @@
         <v>2025-09-21</v>
       </c>
       <c r="B8" t="str">
-        <v>35.5</v>
+        <v>35.12</v>
       </c>
       <c r="C8" t="str">
-        <v>35.5</v>
+        <v>35.12</v>
       </c>
       <c r="D8" t="str">
         <v>9.79</v>
@@ -3676,7 +3710,7 @@
         <v>42</v>
       </c>
       <c r="G8" t="str">
-        <v>-6.5</v>
+        <v>-6.88</v>
       </c>
       <c r="H8" t="str">
         <v>Shortage</v>
@@ -3691,7 +3725,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H109"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3824,7 +3858,7 @@
 Eilidh 31/03/2025</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" xml:space="preserve">
       <c r="A6" t="str">
         <v>2025-09-16</v>
       </c>
@@ -3832,22 +3866,23 @@
         <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C6" t="str">
-        <v>Available</v>
+        <v>Sick</v>
       </c>
       <c r="D6" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E6" t="str">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="F6" t="str">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="G6" t="str">
-        <v>2.67</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v>0</v>
+      </c>
+      <c r="H6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM
+New sick line 11/09 for 1 week - MT; Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="7">
@@ -4320,7 +4355,7 @@
 Eilidh 31/03/2025</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" xml:space="preserve">
       <c r="A25" t="str">
         <v>2025-09-17</v>
       </c>
@@ -4328,22 +4363,23 @@
         <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C25" t="str">
-        <v>Available</v>
+        <v>Sick</v>
       </c>
       <c r="D25" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E25" t="str">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="F25" t="str">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="G25" t="str">
-        <v>2.67</v>
-      </c>
-      <c r="H25" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v>0</v>
+      </c>
+      <c r="H25" t="str" xml:space="preserve">
+        <v xml:space="preserve">Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM
+New sick line 11/09 for 1 week - MT; Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="26">
@@ -4843,7 +4879,7 @@
         <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" xml:space="preserve">
       <c r="A45" t="str">
         <v>2025-09-18</v>
       </c>
@@ -4851,22 +4887,23 @@
         <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C45" t="str">
-        <v>Available</v>
+        <v>Sick</v>
       </c>
       <c r="D45" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E45" t="str">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="F45" t="str">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="G45" t="str">
-        <v>2.67</v>
-      </c>
-      <c r="H45" t="str">
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="H45" t="str" xml:space="preserve">
+        <v xml:space="preserve">Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM
+New sick line 11/09 for 1 week - MT</v>
       </c>
     </row>
     <row r="46">
@@ -5339,30 +5376,31 @@
         <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" xml:space="preserve">
       <c r="A64" t="str">
         <v>2025-09-19</v>
       </c>
       <c r="B64" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C64" t="str">
-        <v>Available</v>
+        <v>Sick</v>
       </c>
       <c r="D64" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E64" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="F64" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="G64" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H64" t="str">
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="H64" t="str" xml:space="preserve">
+        <v xml:space="preserve">Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM
+New sick line 11/09 for 1 week - MT</v>
       </c>
     </row>
     <row r="65">
@@ -5370,25 +5408,25 @@
         <v>2025-09-19</v>
       </c>
       <c r="B65" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="C65" t="str">
         <v>Available</v>
       </c>
       <c r="D65" t="str">
-        <v>09:15-14:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E65" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="F65" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="G65" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="H65" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="66">
@@ -5396,25 +5434,25 @@
         <v>2025-09-19</v>
       </c>
       <c r="B66" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="C66" t="str">
         <v>Available</v>
       </c>
       <c r="D66" t="str">
-        <v>09:15-10:15</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E66" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="F66" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="G66" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="H66" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="67">
@@ -5422,22 +5460,22 @@
         <v>2025-09-19</v>
       </c>
       <c r="B67" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="C67" t="str">
         <v>Available</v>
       </c>
       <c r="D67" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E67" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="F67" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="G67" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="H67" t="str">
         <v/>
@@ -5448,22 +5486,22 @@
         <v>2025-09-19</v>
       </c>
       <c r="B68" t="str">
-        <v>Lori Wylie (NL)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="C68" t="str">
         <v>Available</v>
       </c>
       <c r="D68" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E68" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="F68" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="G68" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="H68" t="str">
         <v/>
@@ -5474,22 +5512,22 @@
         <v>2025-09-19</v>
       </c>
       <c r="B69" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="C69" t="str">
         <v>Available</v>
       </c>
       <c r="D69" t="str">
-        <v>08:00-15:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E69" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F69" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G69" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H69" t="str">
         <v/>
@@ -5500,22 +5538,22 @@
         <v>2025-09-19</v>
       </c>
       <c r="B70" t="str">
-        <v>Marykate Ferris (NL)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="C70" t="str">
         <v>Available</v>
       </c>
       <c r="D70" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E70" t="str">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F70" t="str">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G70" t="str">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H70" t="str">
         <v/>
@@ -5526,7 +5564,7 @@
         <v>2025-09-19</v>
       </c>
       <c r="B71" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="C71" t="str">
         <v>Available</v>
@@ -5535,13 +5573,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E71" t="str">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F71" t="str">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G71" t="str">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H71" t="str">
         <v/>
@@ -5552,52 +5590,51 @@
         <v>2025-09-19</v>
       </c>
       <c r="B72" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="C72" t="str">
         <v>Available</v>
       </c>
       <c r="D72" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E72" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="F72" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="G72" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H72" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
-      </c>
-    </row>
-    <row r="73" xml:space="preserve">
+        <v/>
+      </c>
+    </row>
+    <row r="73">
       <c r="A73" t="str">
         <v>2025-09-19</v>
       </c>
       <c r="B73" t="str">
-        <v>Shafiya Fayaz GH</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="C73" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D73" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="E73" t="str">
-        <v>9</v>
+        <v>3.2</v>
       </c>
       <c r="F73" t="str">
-        <v>9</v>
+        <v>3.2</v>
       </c>
       <c r="G73" t="str">
-        <v>0</v>
-      </c>
-      <c r="H73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Megan approved 
-Eilidh 02/07/2025</v>
+        <v>3.2</v>
+      </c>
+      <c r="H73" t="str">
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="74" xml:space="preserve">
@@ -5605,131 +5642,132 @@
         <v>2025-09-19</v>
       </c>
       <c r="B74" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Shafiya Fayaz GH</v>
       </c>
       <c r="C74" t="str">
         <v>Other Unavailable</v>
       </c>
       <c r="D74" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E74" t="str">
+        <v>9</v>
+      </c>
+      <c r="F74" t="str">
+        <v>9</v>
+      </c>
+      <c r="G74" t="str">
+        <v>0</v>
+      </c>
+      <c r="H74" t="str" xml:space="preserve">
+        <v xml:space="preserve">Megan approved 
+Eilidh 02/07/2025</v>
+      </c>
+    </row>
+    <row r="75" xml:space="preserve">
+      <c r="A75" t="str">
+        <v>2025-09-19</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Sharon Jack (NL)</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Other Unavailable</v>
+      </c>
+      <c r="D75" t="str">
         <v>09:15-17:00</v>
       </c>
-      <c r="E74" t="str">
+      <c r="E75" t="str">
         <v>4.8</v>
       </c>
-      <c r="F74" t="str">
+      <c r="F75" t="str">
         <v>2</v>
       </c>
-      <c r="G74" t="str">
-        <v>0</v>
-      </c>
-      <c r="H74" t="str" xml:space="preserve">
+      <c r="G75" t="str">
+        <v>0</v>
+      </c>
+      <c r="H75" t="str" xml:space="preserve">
         <v xml:space="preserve">Wants this as a break. 
 Eilidh 29/05/2025</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="str">
-        <v>2025-09-19</v>
-      </c>
-      <c r="B75" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
-      </c>
-      <c r="C75" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D75" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E75" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="F75" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="G75" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H75" t="str">
-        <v/>
-      </c>
-    </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2025-09-20</v>
+        <v>2025-09-19</v>
       </c>
       <c r="B76" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="C76" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D76" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E76" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="F76" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="G76" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H76" t="str">
         <v/>
       </c>
     </row>
-    <row r="77" xml:space="preserve">
+    <row r="77">
       <c r="A77" t="str">
         <v>2025-09-20</v>
       </c>
       <c r="B77" t="str">
-        <v>Ayoola Ajibade (GH) (NL)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C77" t="str">
         <v>Maternity/Paternity</v>
       </c>
       <c r="D77" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E77" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="F77" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="G77" t="str">
         <v>0</v>
       </c>
-      <c r="H77" t="str" xml:space="preserve">
+      <c r="H77" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="78" xml:space="preserve">
+      <c r="A78" t="str">
+        <v>2025-09-20</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Ayoola Ajibade (GH) (NL)</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Maternity/Paternity</v>
+      </c>
+      <c r="D78" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E78" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="F78" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="G78" t="str">
+        <v>0</v>
+      </c>
+      <c r="H78" t="str" xml:space="preserve">
         <v xml:space="preserve">Morning sickness
 Eilidh 31/03/2025</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="str">
-        <v>2025-09-20</v>
-      </c>
-      <c r="B78" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
-      </c>
-      <c r="C78" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D78" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E78" t="str">
-        <v>2.67</v>
-      </c>
-      <c r="F78" t="str">
-        <v>2.67</v>
-      </c>
-      <c r="G78" t="str">
-        <v>2.67</v>
-      </c>
-      <c r="H78" t="str">
-        <v/>
       </c>
     </row>
     <row r="79">
@@ -5737,7 +5775,7 @@
         <v>2025-09-20</v>
       </c>
       <c r="B79" t="str">
-        <v>Emma Shawcross (NL)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C79" t="str">
         <v>Available</v>
@@ -5746,16 +5784,16 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E79" t="str">
-        <v>10</v>
+        <v>2.29</v>
       </c>
       <c r="F79" t="str">
-        <v>10</v>
+        <v>2.29</v>
       </c>
       <c r="G79" t="str">
-        <v>10</v>
+        <v>2.29</v>
       </c>
       <c r="H79" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="80">
@@ -5763,7 +5801,7 @@
         <v>2025-09-20</v>
       </c>
       <c r="B80" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Emma Shawcross (NL)</v>
       </c>
       <c r="C80" t="str">
         <v>Available</v>
@@ -5772,16 +5810,16 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E80" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="F80" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="G80" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="H80" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="81">
@@ -5789,22 +5827,22 @@
         <v>2025-09-20</v>
       </c>
       <c r="B81" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Kaitlyn Barton (NL) (GH)</v>
       </c>
       <c r="C81" t="str">
         <v>Available</v>
       </c>
       <c r="D81" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E81" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="F81" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="G81" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="H81" t="str">
         <v/>
@@ -5815,78 +5853,78 @@
         <v>2025-09-20</v>
       </c>
       <c r="B82" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Makala Mcewan (NL) (GH)</v>
       </c>
       <c r="C82" t="str">
         <v>Available</v>
       </c>
       <c r="D82" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="E82" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F82" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G82" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H82" t="str">
         <v/>
       </c>
     </row>
-    <row r="83" xml:space="preserve">
+    <row r="83">
       <c r="A83" t="str">
         <v>2025-09-20</v>
       </c>
       <c r="B83" t="str">
+        <v>Mustansar Hussain (NL) (GH)</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D83" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E83" t="str">
+        <v>6</v>
+      </c>
+      <c r="F83" t="str">
+        <v>6</v>
+      </c>
+      <c r="G83" t="str">
+        <v>6</v>
+      </c>
+      <c r="H83" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="84" xml:space="preserve">
+      <c r="A84" t="str">
+        <v>2025-09-20</v>
+      </c>
+      <c r="B84" t="str">
         <v>Shafiya Fayaz GH</v>
       </c>
-      <c r="C83" t="str">
+      <c r="C84" t="str">
         <v>Other Unavailable</v>
       </c>
-      <c r="D83" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E83" t="str">
+      <c r="D84" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E84" t="str">
         <v>9</v>
       </c>
-      <c r="F83" t="str">
+      <c r="F84" t="str">
         <v>9</v>
       </c>
-      <c r="G83" t="str">
-        <v>0</v>
-      </c>
-      <c r="H83" t="str" xml:space="preserve">
+      <c r="G84" t="str">
+        <v>0</v>
+      </c>
+      <c r="H84" t="str" xml:space="preserve">
         <v xml:space="preserve">Megan approved 
 Eilidh 02/07/2025</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="str">
-        <v>2025-09-15</v>
-      </c>
-      <c r="B84" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
-      </c>
-      <c r="C84" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D84" t="str">
-        <v>10:30-14:00</v>
-      </c>
-      <c r="E84" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="F84" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="G84" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H84" t="str">
-        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="85">
@@ -5894,25 +5932,25 @@
         <v>2025-09-15</v>
       </c>
       <c r="B85" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="C85" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D85" t="str">
-        <v>08:00-15:30</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="E85" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="F85" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="G85" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H85" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="86">
@@ -5920,51 +5958,52 @@
         <v>2025-09-15</v>
       </c>
       <c r="B86" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C86" t="str">
-        <v>Available</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D86" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E86" t="str">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="F86" t="str">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="G86" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="H86" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
-      </c>
-    </row>
-    <row r="87">
+        <v/>
+      </c>
+    </row>
+    <row r="87" xml:space="preserve">
       <c r="A87" t="str">
         <v>2025-09-15</v>
       </c>
       <c r="B87" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C87" t="str">
-        <v>Available</v>
+        <v>Sick</v>
       </c>
       <c r="D87" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E87" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="F87" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="G87" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H87" t="str">
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="H87" t="str" xml:space="preserve">
+        <v xml:space="preserve">Brooke called to advise that she has been given a sick line due to multiple health problems at the moment. SM
+New sick line 11/09 for 1 week - MT; Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="88">
@@ -5972,25 +6011,25 @@
         <v>2025-09-15</v>
       </c>
       <c r="B88" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="C88" t="str">
         <v>Available</v>
       </c>
       <c r="D88" t="str">
-        <v>09:15-14:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E88" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="F88" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="G88" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="H88" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="89">
@@ -5998,25 +6037,25 @@
         <v>2025-09-15</v>
       </c>
       <c r="B89" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="C89" t="str">
         <v>Available</v>
       </c>
       <c r="D89" t="str">
-        <v>09:15-14:45</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E89" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="F89" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="G89" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="H89" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="90">
@@ -6024,22 +6063,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B90" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="C90" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D90" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="E90" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="F90" t="str">
-        <v>7.5</v>
+        <v>2.8</v>
       </c>
       <c r="G90" t="str">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="H90" t="str">
         <v/>
@@ -6050,10 +6089,10 @@
         <v>2025-09-15</v>
       </c>
       <c r="B91" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="C91" t="str">
-        <v>Available</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D91" t="str">
         <v>08:00-21:30</v>
@@ -6065,7 +6104,7 @@
         <v>7.5</v>
       </c>
       <c r="G91" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H91" t="str">
         <v/>
@@ -6076,22 +6115,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B92" t="str">
-        <v>Lori Wylie (NL)</v>
+        <v>Kaitlyn Barton (NL) (GH)</v>
       </c>
       <c r="C92" t="str">
         <v>Available</v>
       </c>
       <c r="D92" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E92" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="F92" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="G92" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="H92" t="str">
         <v/>
@@ -6102,22 +6141,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B93" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="C93" t="str">
         <v>Available</v>
       </c>
       <c r="D93" t="str">
-        <v>08:00-15:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E93" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F93" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G93" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H93" t="str">
         <v/>
@@ -6128,22 +6167,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B94" t="str">
-        <v>Madison Duncan (NL)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="C94" t="str">
         <v>Available</v>
       </c>
       <c r="D94" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E94" t="str">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F94" t="str">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G94" t="str">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H94" t="str">
         <v/>
@@ -6154,22 +6193,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B95" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Madison Duncan (NL)</v>
       </c>
       <c r="C95" t="str">
         <v>Available</v>
       </c>
       <c r="D95" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E95" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F95" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G95" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H95" t="str">
         <v/>
@@ -6180,25 +6219,25 @@
         <v>2025-09-15</v>
       </c>
       <c r="B96" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Makala Mcewan (NL) (GH)</v>
       </c>
       <c r="C96" t="str">
-        <v>Available</v>
+        <v>Compassionate Leave</v>
       </c>
       <c r="D96" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="E96" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F96" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G96" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H96" t="str">
-        <v/>
+        <v>Makala called to advise her papa has passed away today - MT</v>
       </c>
     </row>
     <row r="97">
@@ -6206,25 +6245,25 @@
         <v>2025-09-15</v>
       </c>
       <c r="B97" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="C97" t="str">
         <v>Available</v>
       </c>
       <c r="D97" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E97" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="F97" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="G97" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H97" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="98">
@@ -6232,25 +6271,25 @@
         <v>2025-09-15</v>
       </c>
       <c r="B98" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="C98" t="str">
         <v>Available</v>
       </c>
       <c r="D98" t="str">
-        <v>09:15-10:15</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="E98" t="str">
-        <v>4.8</v>
+        <v>3.2</v>
       </c>
       <c r="F98" t="str">
-        <v>4.8</v>
+        <v>3.2</v>
       </c>
       <c r="G98" t="str">
-        <v>4.8</v>
+        <v>3.2</v>
       </c>
       <c r="H98" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="99">
@@ -6258,22 +6297,22 @@
         <v>2025-09-15</v>
       </c>
       <c r="B99" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Sharon Jack (NL)</v>
       </c>
       <c r="C99" t="str">
         <v>Available</v>
       </c>
       <c r="D99" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E99" t="str">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="F99" t="str">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="G99" t="str">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="H99" t="str">
         <v/>
@@ -6281,25 +6320,25 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>2025-09-21</v>
+        <v>2025-09-15</v>
       </c>
       <c r="B100" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="C100" t="str">
         <v>Available</v>
       </c>
       <c r="D100" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E100" t="str">
-        <v>5.33</v>
+        <v>6</v>
       </c>
       <c r="F100" t="str">
-        <v>5.33</v>
+        <v>6</v>
       </c>
       <c r="G100" t="str">
-        <v>5.33</v>
+        <v>6</v>
       </c>
       <c r="H100" t="str">
         <v/>
@@ -6310,22 +6349,22 @@
         <v>2025-09-21</v>
       </c>
       <c r="B101" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
+        <v>Anne Nelson (NL)</v>
       </c>
       <c r="C101" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D101" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E101" t="str">
-        <v>2.29</v>
+        <v>5.33</v>
       </c>
       <c r="F101" t="str">
-        <v>2.29</v>
+        <v>5.33</v>
       </c>
       <c r="G101" t="str">
-        <v>0</v>
+        <v>5.33</v>
       </c>
       <c r="H101" t="str">
         <v/>
@@ -6336,22 +6375,22 @@
         <v>2025-09-21</v>
       </c>
       <c r="B102" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C102" t="str">
-        <v>Available</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D102" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E102" t="str">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="F102" t="str">
-        <v>2.67</v>
+        <v>2.29</v>
       </c>
       <c r="G102" t="str">
-        <v>2.67</v>
+        <v>0</v>
       </c>
       <c r="H102" t="str">
         <v/>
@@ -6362,25 +6401,25 @@
         <v>2025-09-21</v>
       </c>
       <c r="B103" t="str">
-        <v>Duncan (NL), Madison</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C103" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D103" t="str">
-        <v>16:45-19:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E103" t="str">
-        <v>0</v>
+        <v>2.29</v>
       </c>
       <c r="F103" t="str">
-        <v>0</v>
+        <v>2.29</v>
       </c>
       <c r="G103" t="str">
-        <v>0</v>
+        <v>2.29</v>
       </c>
       <c r="H103" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="104">
@@ -6388,25 +6427,25 @@
         <v>2025-09-21</v>
       </c>
       <c r="B104" t="str">
-        <v>Emma Shawcross (NL)</v>
+        <v>Duncan (NL), Madison</v>
       </c>
       <c r="C104" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D104" t="str">
-        <v>08:00-21:30</v>
+        <v>16:45-19:00</v>
       </c>
       <c r="E104" t="str">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F104" t="str">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G104" t="str">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H104" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="105">
@@ -6414,25 +6453,25 @@
         <v>2025-09-21</v>
       </c>
       <c r="B105" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Emma Shawcross (NL)</v>
       </c>
       <c r="C105" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D105" t="str">
         <v>08:00-21:30</v>
       </c>
       <c r="E105" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="F105" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="G105" t="str">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H105" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="106">
@@ -6440,10 +6479,10 @@
         <v>2025-09-21</v>
       </c>
       <c r="B106" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="C106" t="str">
-        <v>Available</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D106" t="str">
         <v>08:00-21:30</v>
@@ -6455,7 +6494,7 @@
         <v>7.5</v>
       </c>
       <c r="G106" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H106" t="str">
         <v/>
@@ -6466,22 +6505,22 @@
         <v>2025-09-21</v>
       </c>
       <c r="B107" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Kaitlyn Barton (NL) (GH)</v>
       </c>
       <c r="C107" t="str">
         <v>Available</v>
       </c>
       <c r="D107" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E107" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="F107" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="G107" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="H107" t="str">
         <v/>
@@ -6492,30 +6531,56 @@
         <v>2025-09-21</v>
       </c>
       <c r="B108" t="str">
+        <v>Makala Mcewan (NL) (GH)</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D108" t="str">
+        <v>08:00-15:15</v>
+      </c>
+      <c r="E108" t="str">
+        <v>4</v>
+      </c>
+      <c r="F108" t="str">
+        <v>4</v>
+      </c>
+      <c r="G108" t="str">
+        <v>4</v>
+      </c>
+      <c r="H108" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>2025-09-21</v>
+      </c>
+      <c r="B109" t="str">
         <v>Wayne (GH) Griffiths (NL)</v>
       </c>
-      <c r="C108" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D108" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E108" t="str">
-        <v>6</v>
-      </c>
-      <c r="F108" t="str">
-        <v>6</v>
-      </c>
-      <c r="G108" t="str">
-        <v>6</v>
-      </c>
-      <c r="H108" t="str">
+      <c r="C109" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D109" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E109" t="str">
+        <v>6</v>
+      </c>
+      <c r="F109" t="str">
+        <v>6</v>
+      </c>
+      <c r="G109" t="str">
+        <v>6</v>
+      </c>
+      <c r="H109" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H108"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H109"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adjust time window calculations and add new status policies
Update logic to precisely calculate time windows by removing gap tolerance and implement new policies for day-killers and time-killers, ensuring a minimum duration of 60 minutes for valid time blocks.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: faa34da4-36c5-42e2-9a7d-dfe321980219
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/faa34da4-36c5-42e2-9a7d-dfe321980219/RusRgGA
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I107"/>
+  <dimension ref="A1:I106"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -446,7 +446,7 @@
         <v>7.5</v>
       </c>
       <c r="D2" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E2" t="str">
         <v>Maternity/Paternity</v>
@@ -476,7 +476,7 @@
         <v>7.5</v>
       </c>
       <c r="D3" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E3" t="str">
         <v>Maternity/Paternity</v>
@@ -506,7 +506,7 @@
         <v>7.5</v>
       </c>
       <c r="D4" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E4" t="str">
         <v>Maternity/Paternity</v>
@@ -536,7 +536,7 @@
         <v>7.5</v>
       </c>
       <c r="D5" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E5" t="str">
         <v>Maternity/Paternity</v>
@@ -566,7 +566,7 @@
         <v>7.5</v>
       </c>
       <c r="D6" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-11</v>
       </c>
       <c r="E6" t="str">
         <v>Maternity/Paternity</v>
@@ -596,7 +596,7 @@
         <v>2.29</v>
       </c>
       <c r="D7" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E7" t="str">
         <v>Maternity/Paternity</v>
@@ -625,7 +625,7 @@
         <v>2.29</v>
       </c>
       <c r="D8" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E8" t="str">
         <v>Maternity/Paternity</v>
@@ -654,7 +654,7 @@
         <v>2.29</v>
       </c>
       <c r="D9" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E9" t="str">
         <v>Maternity/Paternity</v>
@@ -683,7 +683,7 @@
         <v>2.29</v>
       </c>
       <c r="D10" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E10" t="str">
         <v>Maternity/Paternity</v>
@@ -712,7 +712,7 @@
         <v>2.29</v>
       </c>
       <c r="D11" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E11" t="str">
         <v>Maternity/Paternity</v>
@@ -741,7 +741,7 @@
         <v>2.29</v>
       </c>
       <c r="D12" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-11</v>
       </c>
       <c r="E12" t="str">
         <v>Maternity/Paternity</v>
@@ -770,7 +770,7 @@
         <v>2.29</v>
       </c>
       <c r="D13" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-12</v>
       </c>
       <c r="E13" t="str">
         <v>Maternity/Paternity</v>
@@ -790,25 +790,25 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Madison Duncan (NL)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="B14" t="str">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C14" t="str">
-        <v>8</v>
+        <v>2.8</v>
       </c>
       <c r="D14" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E14" t="str">
         <v>Holiday</v>
       </c>
       <c r="F14" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="G14" t="str">
-        <v>8</v>
+        <v>2.8</v>
       </c>
       <c r="H14" t="str">
         <v>0</v>
@@ -819,25 +819,25 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Madison Duncan (NL)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="B15" t="str">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C15" t="str">
-        <v>8</v>
+        <v>2.8</v>
       </c>
       <c r="D15" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E15" t="str">
         <v>Holiday</v>
       </c>
       <c r="F15" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:15</v>
       </c>
       <c r="G15" t="str">
-        <v>8</v>
+        <v>2.8</v>
       </c>
       <c r="H15" t="str">
         <v>0</v>
@@ -848,25 +848,25 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="B16" t="str">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C16" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="D16" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E16" t="str">
         <v>Holiday</v>
       </c>
       <c r="F16" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="G16" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="H16" t="str">
         <v>0</v>
@@ -877,25 +877,25 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="B17" t="str">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C17" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="D17" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E17" t="str">
         <v>Holiday</v>
       </c>
       <c r="F17" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:15</v>
       </c>
       <c r="G17" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="H17" t="str">
         <v>0</v>
@@ -906,25 +906,25 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="B18" t="str">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C18" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="D18" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E18" t="str">
         <v>Holiday</v>
       </c>
       <c r="F18" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:15</v>
       </c>
       <c r="G18" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="H18" t="str">
         <v>0</v>
@@ -935,25 +935,25 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Madison Duncan (NL)</v>
       </c>
       <c r="B19" t="str">
         <v>16</v>
       </c>
       <c r="C19" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D19" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E19" t="str">
         <v>Holiday</v>
       </c>
       <c r="F19" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="G19" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H19" t="str">
         <v>0</v>
@@ -962,92 +962,91 @@
         <v>Created by new vacation process.</v>
       </c>
     </row>
-    <row r="20" xml:space="preserve">
+    <row r="20">
       <c r="A20" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Madison Duncan (NL)</v>
       </c>
       <c r="B20" t="str">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C20" t="str">
-        <v>4.8</v>
+        <v>8</v>
       </c>
       <c r="D20" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E20" t="str">
         <v>Holiday</v>
       </c>
       <c r="F20" t="str">
-        <v>09:15-17:00</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="G20" t="str">
-        <v>4.8</v>
+        <v>8</v>
       </c>
       <c r="H20" t="str">
         <v>0</v>
       </c>
-      <c r="I20" t="str" xml:space="preserve">
-        <v xml:space="preserve">Created by new vacation process.; Wants this as a break. 
-Eilidh 29/05/2025</v>
+      <c r="I20" t="str">
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="B21" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C21" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D21" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E21" t="str">
-        <v>Other Unavailable</v>
+        <v>Holiday</v>
       </c>
       <c r="F21" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-17:45</v>
       </c>
       <c r="G21" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H21" t="str">
         <v>0</v>
       </c>
       <c r="I21" t="str">
-        <v/>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="B22" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C22" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D22" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E22" t="str">
-        <v>Other Unavailable</v>
+        <v>Holiday</v>
       </c>
       <c r="F22" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-17:45</v>
       </c>
       <c r="G22" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H22" t="str">
         <v>0</v>
       </c>
       <c r="I22" t="str">
-        <v/>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="23">
@@ -1061,7 +1060,7 @@
         <v>7.5</v>
       </c>
       <c r="D23" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E23" t="str">
         <v>Other Unavailable</v>
@@ -1090,7 +1089,7 @@
         <v>7.5</v>
       </c>
       <c r="D24" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E24" t="str">
         <v>Other Unavailable</v>
@@ -1119,7 +1118,7 @@
         <v>7.5</v>
       </c>
       <c r="D25" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E25" t="str">
         <v>Other Unavailable</v>
@@ -1137,66 +1136,65 @@
         <v/>
       </c>
     </row>
-    <row r="26" xml:space="preserve">
+    <row r="26">
       <c r="A26" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="B26" t="str">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="C26" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="D26" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E26" t="str">
         <v>Other Unavailable</v>
       </c>
       <c r="F26" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G26" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H26" t="str">
         <v>0</v>
       </c>
-      <c r="I26" t="str" xml:space="preserve">
-        <v xml:space="preserve">Cheryl emailed to advise she is away for the September weekend 
-Eilidh 15/09/2025</v>
+      <c r="I26" t="str">
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="B27" t="str">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="C27" t="str">
-        <v>4.8</v>
+        <v>7.5</v>
       </c>
       <c r="D27" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-12</v>
       </c>
       <c r="E27" t="str">
         <v>Other Unavailable</v>
       </c>
       <c r="F27" t="str">
-        <v>09:15-16:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G27" t="str">
-        <v>2</v>
+        <v>7.5</v>
       </c>
       <c r="H27" t="str">
         <v>0</v>
       </c>
       <c r="I27" t="str">
-        <v>Sharon has advised she is unable to work between 10.30 and 12.30 on Tuesday's - MT</v>
-      </c>
-    </row>
-    <row r="28" xml:space="preserve">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
       <c r="A28" t="str">
         <v>Sharon Jack (NL)</v>
       </c>
@@ -1207,13 +1205,13 @@
         <v>4.8</v>
       </c>
       <c r="D28" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E28" t="str">
         <v>Other Unavailable</v>
       </c>
       <c r="F28" t="str">
-        <v>09:15-16:30</v>
+        <v>09:15-16:15</v>
       </c>
       <c r="G28" t="str">
         <v>2</v>
@@ -1221,67 +1219,68 @@
       <c r="H28" t="str">
         <v>0</v>
       </c>
-      <c r="I28" t="str" xml:space="preserve">
+      <c r="I28" t="str">
+        <v>Sharon has advised she is unable to work between 10.30 and 12.30 on Tuesday's - MT</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>Sharon Jack (NL)</v>
+      </c>
+      <c r="B29" t="str">
+        <v>24</v>
+      </c>
+      <c r="C29" t="str">
+        <v>4.8</v>
+      </c>
+      <c r="D29" t="str">
+        <v>2025-10-08</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Other Unavailable</v>
+      </c>
+      <c r="F29" t="str">
+        <v>09:15-16:30</v>
+      </c>
+      <c r="G29" t="str">
+        <v>2</v>
+      </c>
+      <c r="H29" t="str">
+        <v>0</v>
+      </c>
+      <c r="I29" t="str" xml:space="preserve">
         <v xml:space="preserve">Wants this as a break. 
 Eilidh 29/05/2025</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
-      </c>
-      <c r="B29" t="str">
-        <v>16</v>
-      </c>
-      <c r="C29" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D29" t="str">
-        <v>2025-09-22</v>
-      </c>
-      <c r="E29" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F29" t="str">
-        <v>10:30-14:00</v>
-      </c>
-      <c r="G29" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H29" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I29" t="str">
-        <v>Confirmed at induction with MT</v>
-      </c>
-    </row>
-    <row r="30">
+    <row r="30" xml:space="preserve">
       <c r="A30" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
+        <v>Sharon Jack (NL)</v>
       </c>
       <c r="B30" t="str">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C30" t="str">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="D30" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E30" t="str">
-        <v>Available</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="F30" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-17:00</v>
       </c>
       <c r="G30" t="str">
-        <v>3.2</v>
+        <v>2</v>
       </c>
       <c r="H30" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I30" t="str">
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="I30" t="str" xml:space="preserve">
+        <v xml:space="preserve">Wants this as a break. 
+Eilidh 29/05/2025</v>
       </c>
     </row>
     <row r="31">
@@ -1295,13 +1294,13 @@
         <v>3.2</v>
       </c>
       <c r="D31" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E31" t="str">
         <v>Available</v>
       </c>
       <c r="F31" t="str">
-        <v>09:15-15:15</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="G31" t="str">
         <v>3.2</v>
@@ -1310,7 +1309,7 @@
         <v>3.2</v>
       </c>
       <c r="I31" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="32">
@@ -1324,7 +1323,7 @@
         <v>3.2</v>
       </c>
       <c r="D32" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E32" t="str">
         <v>Available</v>
@@ -1353,13 +1352,13 @@
         <v>3.2</v>
       </c>
       <c r="D33" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E33" t="str">
         <v>Available</v>
       </c>
       <c r="F33" t="str">
-        <v>10:30-14:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G33" t="str">
         <v>3.2</v>
@@ -1368,65 +1367,65 @@
         <v>3.2</v>
       </c>
       <c r="I33" t="str">
-        <v>Confirmed at induction with MT</v>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="B34" t="str">
         <v>16</v>
       </c>
       <c r="C34" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="D34" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E34" t="str">
         <v>Available</v>
       </c>
       <c r="F34" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G34" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="H34" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="I34" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="B35" t="str">
         <v>16</v>
       </c>
       <c r="C35" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="D35" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E35" t="str">
         <v>Available</v>
       </c>
       <c r="F35" t="str">
-        <v>09:15-14:00</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="G35" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="H35" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="I35" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="36">
@@ -1440,7 +1439,7 @@
         <v>2.67</v>
       </c>
       <c r="D36" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E36" t="str">
         <v>Available</v>
@@ -1469,7 +1468,7 @@
         <v>2.67</v>
       </c>
       <c r="D37" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E37" t="str">
         <v>Available</v>
@@ -1484,7 +1483,7 @@
         <v>2.67</v>
       </c>
       <c r="I37" t="str">
-        <v/>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="38">
@@ -1498,7 +1497,7 @@
         <v>2.67</v>
       </c>
       <c r="D38" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E38" t="str">
         <v>Available</v>
@@ -1513,7 +1512,7 @@
         <v>2.67</v>
       </c>
       <c r="I38" t="str">
-        <v/>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="39">
@@ -1527,13 +1526,13 @@
         <v>2.67</v>
       </c>
       <c r="D39" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E39" t="str">
         <v>Available</v>
       </c>
       <c r="F39" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G39" t="str">
         <v>2.67</v>
@@ -1547,16 +1546,16 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="B40" t="str">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C40" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="D40" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E40" t="str">
         <v>Available</v>
@@ -1565,42 +1564,42 @@
         <v>09:15-14:00</v>
       </c>
       <c r="G40" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="H40" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="I40" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="B41" t="str">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C41" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="D41" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-11</v>
       </c>
       <c r="E41" t="str">
         <v>Available</v>
       </c>
       <c r="F41" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G41" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="H41" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="I41" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -1614,7 +1613,7 @@
         <v>4</v>
       </c>
       <c r="D42" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E42" t="str">
         <v>Available</v>
@@ -1643,7 +1642,7 @@
         <v>4</v>
       </c>
       <c r="D43" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E43" t="str">
         <v>Available</v>
@@ -1672,7 +1671,7 @@
         <v>4</v>
       </c>
       <c r="D44" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E44" t="str">
         <v>Available</v>
@@ -1692,144 +1691,144 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="B45" t="str">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C45" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="D45" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E45" t="str">
         <v>Available</v>
       </c>
       <c r="F45" t="str">
-        <v>09:15-14:45</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G45" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="H45" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="I45" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="B46" t="str">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C46" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="D46" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E46" t="str">
         <v>Available</v>
       </c>
       <c r="F46" t="str">
-        <v>09:15-11:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G46" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="H46" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="I46" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Emma Shawcross (NL)</v>
       </c>
       <c r="B47" t="str">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C47" t="str">
-        <v>2.8</v>
+        <v>10</v>
       </c>
       <c r="D47" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-11</v>
       </c>
       <c r="E47" t="str">
         <v>Available</v>
       </c>
       <c r="F47" t="str">
-        <v>09:15-14:45</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G47" t="str">
-        <v>2.8</v>
+        <v>10</v>
       </c>
       <c r="H47" t="str">
-        <v>2.8</v>
+        <v>10</v>
       </c>
       <c r="I47" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Emma Shawcross (NL)</v>
       </c>
       <c r="B48" t="str">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C48" t="str">
-        <v>2.8</v>
+        <v>10</v>
       </c>
       <c r="D48" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-12</v>
       </c>
       <c r="E48" t="str">
         <v>Available</v>
       </c>
       <c r="F48" t="str">
-        <v>09:15-11:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G48" t="str">
-        <v>2.8</v>
+        <v>10</v>
       </c>
       <c r="H48" t="str">
-        <v>2.8</v>
+        <v>10</v>
       </c>
       <c r="I48" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Kaitlyn Barton (NL) (GH)</v>
       </c>
       <c r="B49" t="str">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="C49" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="D49" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E49" t="str">
         <v>Available</v>
       </c>
       <c r="F49" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G49" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="H49" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="I49" t="str">
         <v/>
@@ -1837,16 +1836,16 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Emma Shawcross (NL)</v>
+        <v>Kaitlyn Barton (NL) (GH)</v>
       </c>
       <c r="B50" t="str">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C50" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="D50" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E50" t="str">
         <v>Available</v>
@@ -1855,27 +1854,27 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G50" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="H50" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="I50" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Emma Shawcross (NL)</v>
+        <v>Kaitlyn Barton (NL) (GH)</v>
       </c>
       <c r="B51" t="str">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C51" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="D51" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E51" t="str">
         <v>Available</v>
@@ -1884,13 +1883,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G51" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="H51" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="I51" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="52">
@@ -1904,7 +1903,7 @@
         <v>7.5</v>
       </c>
       <c r="D52" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E52" t="str">
         <v>Available</v>
@@ -1924,28 +1923,28 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Makala Mcewan (NL) (GH)</v>
       </c>
       <c r="B53" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C53" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="D53" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E53" t="str">
         <v>Available</v>
       </c>
       <c r="F53" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="G53" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="H53" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="I53" t="str">
         <v/>
@@ -1953,28 +1952,28 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Makala Mcewan (NL) (GH)</v>
       </c>
       <c r="B54" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C54" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="D54" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E54" t="str">
         <v>Available</v>
       </c>
       <c r="F54" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="G54" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="H54" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="I54" t="str">
         <v/>
@@ -1982,28 +1981,28 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Makala Mcewan (NL) (GH)</v>
       </c>
       <c r="B55" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C55" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="D55" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E55" t="str">
         <v>Available</v>
       </c>
       <c r="F55" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="G55" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="H55" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="I55" t="str">
         <v/>
@@ -2020,7 +2019,7 @@
         <v>4</v>
       </c>
       <c r="D56" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-12</v>
       </c>
       <c r="E56" t="str">
         <v>Available</v>
@@ -2040,28 +2039,28 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="B57" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C57" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="D57" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E57" t="str">
         <v>Available</v>
       </c>
       <c r="F57" t="str">
-        <v>08:00-15:15</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G57" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="H57" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="I57" t="str">
         <v/>
@@ -2069,28 +2068,28 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="B58" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C58" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="D58" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E58" t="str">
         <v>Available</v>
       </c>
       <c r="F58" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G58" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="H58" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="I58" t="str">
         <v/>
@@ -2098,28 +2097,28 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="B59" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C59" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="D59" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-12</v>
       </c>
       <c r="E59" t="str">
         <v>Available</v>
       </c>
       <c r="F59" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G59" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="H59" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="I59" t="str">
         <v/>
@@ -2127,28 +2126,28 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Marykate Ferris (NL)</v>
+        <v>Shafiya Fayaz GH</v>
       </c>
       <c r="B60" t="str">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C60" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="D60" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E60" t="str">
         <v>Available</v>
       </c>
       <c r="F60" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G60" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="H60" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="I60" t="str">
         <v/>
@@ -2156,16 +2155,16 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Marykate Ferris (NL)</v>
+        <v>Shafiya Fayaz GH</v>
       </c>
       <c r="B61" t="str">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C61" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="D61" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E61" t="str">
         <v>Available</v>
@@ -2174,10 +2173,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G61" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="H61" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="I61" t="str">
         <v/>
@@ -2185,16 +2184,16 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Marykate Ferris (NL)</v>
+        <v>Shafiya Fayaz GH</v>
       </c>
       <c r="B62" t="str">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C62" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="D62" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E62" t="str">
         <v>Available</v>
@@ -2203,10 +2202,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G62" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="H62" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="I62" t="str">
         <v/>
@@ -2223,7 +2222,7 @@
         <v>9</v>
       </c>
       <c r="D63" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E63" t="str">
         <v>Available</v>
@@ -2252,7 +2251,7 @@
         <v>9</v>
       </c>
       <c r="D64" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-11</v>
       </c>
       <c r="E64" t="str">
         <v>Available</v>
@@ -2272,16 +2271,16 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Shafiya Fayaz GH</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="B65" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C65" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="D65" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E65" t="str">
         <v>Available</v>
@@ -2290,10 +2289,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G65" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H65" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="I65" t="str">
         <v/>
@@ -2301,28 +2300,28 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Shafiya Fayaz GH</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="B66" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C66" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="D66" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E66" t="str">
         <v>Available</v>
       </c>
       <c r="F66" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="G66" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H66" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="I66" t="str">
         <v/>
@@ -2330,16 +2329,16 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Shafiya Fayaz GH</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="B67" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C67" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="D67" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-11</v>
       </c>
       <c r="E67" t="str">
         <v>Available</v>
@@ -2348,10 +2347,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G67" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H67" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="I67" t="str">
         <v/>
@@ -2368,7 +2367,7 @@
         <v>7.5</v>
       </c>
       <c r="D68" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-12</v>
       </c>
       <c r="E68" t="str">
         <v>Available</v>
@@ -2388,7 +2387,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
+        <v>Adedayo Adeyanju (NL) (GH)</v>
       </c>
       <c r="B69" t="str">
         <v>30</v>
@@ -2397,13 +2396,13 @@
         <v>7.5</v>
       </c>
       <c r="D69" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E69" t="str">
         <v>Available</v>
       </c>
       <c r="F69" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G69" t="str">
         <v>7.5</v>
@@ -2417,7 +2416,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
+        <v>Adedayo Adeyanju (NL) (GH)</v>
       </c>
       <c r="B70" t="str">
         <v>30</v>
@@ -2426,7 +2425,7 @@
         <v>7.5</v>
       </c>
       <c r="D70" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E70" t="str">
         <v>Available</v>
@@ -2446,7 +2445,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
+        <v>Adedayo Adeyanju (NL) (GH)</v>
       </c>
       <c r="B71" t="str">
         <v>30</v>
@@ -2455,7 +2454,7 @@
         <v>7.5</v>
       </c>
       <c r="D71" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-11</v>
       </c>
       <c r="E71" t="str">
         <v>Available</v>
@@ -2484,7 +2483,7 @@
         <v>7.5</v>
       </c>
       <c r="D72" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-12</v>
       </c>
       <c r="E72" t="str">
         <v>Available</v>
@@ -2504,16 +2503,16 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Adedayo Adeyanju (NL) (GH)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="B73" t="str">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C73" t="str">
         <v>7.5</v>
       </c>
       <c r="D73" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E73" t="str">
         <v>Available</v>
@@ -2533,16 +2532,16 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Adedayo Adeyanju (NL) (GH)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="B74" t="str">
         <v>30</v>
       </c>
       <c r="C74" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D74" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E74" t="str">
         <v>Available</v>
@@ -2551,10 +2550,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G74" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H74" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="I74" t="str">
         <v/>
@@ -2562,16 +2561,16 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Adedayo Adeyanju (NL) (GH)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="B75" t="str">
         <v>30</v>
       </c>
       <c r="C75" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D75" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E75" t="str">
         <v>Available</v>
@@ -2580,10 +2579,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G75" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H75" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="I75" t="str">
         <v/>
@@ -2591,16 +2590,16 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="B76" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C76" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D76" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E76" t="str">
         <v>Available</v>
@@ -2609,10 +2608,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G76" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H76" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="I76" t="str">
         <v/>
@@ -2629,7 +2628,7 @@
         <v>6</v>
       </c>
       <c r="D77" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E77" t="str">
         <v>Available</v>
@@ -2658,7 +2657,7 @@
         <v>6</v>
       </c>
       <c r="D78" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-11</v>
       </c>
       <c r="E78" t="str">
         <v>Available</v>
@@ -2678,89 +2677,89 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="B79" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C79" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D79" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E79" t="str">
         <v>Available</v>
       </c>
       <c r="F79" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="G79" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H79" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I79" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="B80" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C80" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D80" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E80" t="str">
         <v>Available</v>
       </c>
       <c r="F80" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="G80" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H80" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I80" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="B81" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C81" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D81" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E81" t="str">
         <v>Available</v>
       </c>
       <c r="F81" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="G81" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H81" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I81" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="82">
@@ -2774,7 +2773,7 @@
         <v>3.2</v>
       </c>
       <c r="D82" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E82" t="str">
         <v>Available</v>
@@ -2803,7 +2802,7 @@
         <v>3.2</v>
       </c>
       <c r="D83" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E83" t="str">
         <v>Available</v>
@@ -2823,89 +2822,89 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="B84" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C84" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="D84" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E84" t="str">
         <v>Available</v>
       </c>
       <c r="F84" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G84" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H84" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="I84" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="B85" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C85" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="D85" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E85" t="str">
         <v>Available</v>
       </c>
       <c r="F85" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G85" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H85" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="I85" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="B86" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C86" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="D86" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E86" t="str">
         <v>Available</v>
       </c>
       <c r="F86" t="str">
-        <v>09:15-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G86" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H86" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="I86" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="87">
@@ -2919,7 +2918,7 @@
         <v>6</v>
       </c>
       <c r="D87" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E87" t="str">
         <v>Available</v>
@@ -2948,7 +2947,7 @@
         <v>6</v>
       </c>
       <c r="D88" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-12</v>
       </c>
       <c r="E88" t="str">
         <v>Available</v>
@@ -2968,28 +2967,28 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Anne Nelson (NL)</v>
       </c>
       <c r="B89" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C89" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="D89" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E89" t="str">
         <v>Available</v>
       </c>
       <c r="F89" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-17:15</v>
       </c>
       <c r="G89" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="H89" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="I89" t="str">
         <v/>
@@ -2997,28 +2996,28 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Anne Nelson (NL)</v>
       </c>
       <c r="B90" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C90" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="D90" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E90" t="str">
         <v>Available</v>
       </c>
       <c r="F90" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-13:00</v>
       </c>
       <c r="G90" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="H90" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="I90" t="str">
         <v/>
@@ -3026,28 +3025,28 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Anne Nelson (NL)</v>
       </c>
       <c r="B91" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C91" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="D91" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-12</v>
       </c>
       <c r="E91" t="str">
         <v>Available</v>
       </c>
       <c r="F91" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="G91" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="H91" t="str">
-        <v>6</v>
+        <v>5.33</v>
       </c>
       <c r="I91" t="str">
         <v/>
@@ -3064,7 +3063,7 @@
         <v>3.2</v>
       </c>
       <c r="D92" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E92" t="str">
         <v>Available</v>
@@ -3093,7 +3092,7 @@
         <v>3.2</v>
       </c>
       <c r="D93" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E93" t="str">
         <v>Available</v>
@@ -3122,7 +3121,7 @@
         <v>3.2</v>
       </c>
       <c r="D94" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E94" t="str">
         <v>Available</v>
@@ -3151,7 +3150,7 @@
         <v>3.2</v>
       </c>
       <c r="D95" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E95" t="str">
         <v>Available</v>
@@ -3171,28 +3170,28 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="B96" t="str">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C96" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="D96" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E96" t="str">
         <v>Available</v>
       </c>
       <c r="F96" t="str">
-        <v>08:00-15:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G96" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="H96" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="I96" t="str">
         <v/>
@@ -3209,7 +3208,7 @@
         <v>4</v>
       </c>
       <c r="D97" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E97" t="str">
         <v>Available</v>
@@ -3238,13 +3237,13 @@
         <v>4</v>
       </c>
       <c r="D98" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E98" t="str">
         <v>Available</v>
       </c>
       <c r="F98" t="str">
-        <v>08:00-14:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="G98" t="str">
         <v>4</v>
@@ -3267,13 +3266,13 @@
         <v>4</v>
       </c>
       <c r="D99" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-08</v>
       </c>
       <c r="E99" t="str">
         <v>Available</v>
       </c>
       <c r="F99" t="str">
-        <v>08:00-15:00</v>
+        <v>08:00-14:00</v>
       </c>
       <c r="G99" t="str">
         <v>4</v>
@@ -3296,13 +3295,13 @@
         <v>4</v>
       </c>
       <c r="D100" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E100" t="str">
         <v>Available</v>
       </c>
       <c r="F100" t="str">
-        <v>08:00-14:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="G100" t="str">
         <v>4</v>
@@ -3316,28 +3315,28 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="B101" t="str">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C101" t="str">
-        <v>4.8</v>
+        <v>4</v>
       </c>
       <c r="D101" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E101" t="str">
         <v>Available</v>
       </c>
       <c r="F101" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-14:00</v>
       </c>
       <c r="G101" t="str">
-        <v>4.8</v>
+        <v>4</v>
       </c>
       <c r="H101" t="str">
-        <v>4.8</v>
+        <v>4</v>
       </c>
       <c r="I101" t="str">
         <v/>
@@ -3354,13 +3353,13 @@
         <v>4.8</v>
       </c>
       <c r="D102" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E102" t="str">
         <v>Available</v>
       </c>
       <c r="F102" t="str">
-        <v>09:15-16:15</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G102" t="str">
         <v>4.8</v>
@@ -3374,28 +3373,28 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>Lori Wylie (NL)</v>
+        <v>Sharon Jack (NL)</v>
       </c>
       <c r="B103" t="str">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C103" t="str">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="D103" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-09</v>
       </c>
       <c r="E103" t="str">
         <v>Available</v>
       </c>
       <c r="F103" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-16:15</v>
       </c>
       <c r="G103" t="str">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="H103" t="str">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="I103" t="str">
         <v/>
@@ -3412,7 +3411,7 @@
         <v>6</v>
       </c>
       <c r="D104" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-06</v>
       </c>
       <c r="E104" t="str">
         <v>Available</v>
@@ -3441,13 +3440,13 @@
         <v>6</v>
       </c>
       <c r="D105" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-07</v>
       </c>
       <c r="E105" t="str">
         <v>Available</v>
       </c>
       <c r="F105" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G105" t="str">
         <v>6</v>
@@ -3470,7 +3469,7 @@
         <v>6</v>
       </c>
       <c r="D106" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-10</v>
       </c>
       <c r="E106" t="str">
         <v>Available</v>
@@ -3488,38 +3487,9 @@
         <v/>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" t="str">
-        <v>Lori Wylie (NL)</v>
-      </c>
-      <c r="B107" t="str">
-        <v>30</v>
-      </c>
-      <c r="C107" t="str">
-        <v>6</v>
-      </c>
-      <c r="D107" t="str">
-        <v>2025-09-26</v>
-      </c>
-      <c r="E107" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F107" t="str">
-        <v>09:15-14:00</v>
-      </c>
-      <c r="G107" t="str">
-        <v>6</v>
-      </c>
-      <c r="H107" t="str">
-        <v>6</v>
-      </c>
-      <c r="I107" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I107"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I106"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3556,25 +3526,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B2" t="str">
-        <v>60.87</v>
+        <v>58.07</v>
       </c>
       <c r="C2" t="str">
-        <v>60.87</v>
+        <v>58.07</v>
       </c>
       <c r="D2" t="str">
         <v>9.79</v>
       </c>
       <c r="E2" t="str">
-        <v>8</v>
+        <v>10.8</v>
       </c>
       <c r="F2" t="str">
-        <v>65.5</v>
+        <v>61.75</v>
       </c>
       <c r="G2" t="str">
-        <v>-4.63</v>
+        <v>-3.68</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -3582,25 +3552,25 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B3" t="str">
-        <v>72.57</v>
+        <v>69.77</v>
       </c>
       <c r="C3" t="str">
-        <v>72.57</v>
+        <v>69.77</v>
       </c>
       <c r="D3" t="str">
         <v>19.29</v>
       </c>
       <c r="E3" t="str">
-        <v>8</v>
+        <v>10.8</v>
       </c>
       <c r="F3" t="str">
-        <v>55.25</v>
+        <v>64.25</v>
       </c>
       <c r="G3" t="str">
-        <v>17.32</v>
+        <v>5.52</v>
       </c>
       <c r="H3" t="str">
         <v>Sufficient</v>
@@ -3608,51 +3578,51 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B4" t="str">
-        <v>68.24</v>
+        <v>59.44</v>
       </c>
       <c r="C4" t="str">
-        <v>68.24</v>
+        <v>59.44</v>
       </c>
       <c r="D4" t="str">
         <v>19.29</v>
       </c>
       <c r="E4" t="str">
-        <v>0</v>
+        <v>8.8</v>
       </c>
       <c r="F4" t="str">
-        <v>65.5</v>
+        <v>86.5</v>
       </c>
       <c r="G4" t="str">
-        <v>2.74</v>
+        <v>-27.06</v>
       </c>
       <c r="H4" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B5" t="str">
-        <v>67.04</v>
+        <v>63.57</v>
       </c>
       <c r="C5" t="str">
-        <v>67.04</v>
+        <v>63.57</v>
       </c>
       <c r="D5" t="str">
         <v>17.29</v>
       </c>
       <c r="E5" t="str">
-        <v>4</v>
+        <v>8.8</v>
       </c>
       <c r="F5" t="str">
-        <v>54.5</v>
+        <v>63.5</v>
       </c>
       <c r="G5" t="str">
-        <v>12.54</v>
+        <v>0.07</v>
       </c>
       <c r="H5" t="str">
         <v>Sufficient</v>
@@ -3660,25 +3630,25 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B6" t="str">
-        <v>59.87</v>
+        <v>65.6</v>
       </c>
       <c r="C6" t="str">
-        <v>59.87</v>
+        <v>65.6</v>
       </c>
       <c r="D6" t="str">
-        <v>12.99</v>
+        <v>11.79</v>
       </c>
       <c r="E6" t="str">
-        <v>8.8</v>
+        <v>2.8</v>
       </c>
       <c r="F6" t="str">
-        <v>47.5</v>
+        <v>59.5</v>
       </c>
       <c r="G6" t="str">
-        <v>12.37</v>
+        <v>6.1</v>
       </c>
       <c r="H6" t="str">
         <v>Sufficient</v>
@@ -3686,7 +3656,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-11</v>
       </c>
       <c r="B7" t="str">
         <v>42.67</v>
@@ -3698,39 +3668,39 @@
         <v>9.79</v>
       </c>
       <c r="E7" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F7" t="str">
-        <v>37.75</v>
+        <v>42.75</v>
       </c>
       <c r="G7" t="str">
-        <v>4.92</v>
+        <v>-0.08</v>
       </c>
       <c r="H7" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-12</v>
       </c>
       <c r="B8" t="str">
-        <v>41.67</v>
+        <v>47</v>
       </c>
       <c r="C8" t="str">
-        <v>41.67</v>
+        <v>47</v>
       </c>
       <c r="D8" t="str">
         <v>9.79</v>
       </c>
       <c r="E8" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F8" t="str">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="G8" t="str">
-        <v>6.67</v>
+        <v>5</v>
       </c>
       <c r="H8" t="str">
         <v>Sufficient</v>
@@ -3745,7 +3715,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H107"/>
+  <dimension ref="A1:H106"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3775,7 +3745,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B2" t="str">
         <v>Adedayo Adeyanju (NL) (GH)</v>
@@ -3801,7 +3771,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B3" t="str">
         <v>Amanda Forbes (NL) (GH)</v>
@@ -3827,7 +3797,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B4" t="str">
         <v>Ashleigh Graham (GH) (NL)</v>
@@ -3853,7 +3823,7 @@
     </row>
     <row r="5" xml:space="preserve">
       <c r="A5" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B5" t="str">
         <v>Ayoola Ajibade (GH) (NL)</v>
@@ -3880,7 +3850,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B6" t="str">
         <v>Brooke O'Brien (NL) (GH)</v>
@@ -3906,7 +3876,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B7" t="str">
         <v>Cheryl McGhie (NL) (GH)</v>
@@ -3932,7 +3902,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B8" t="str">
         <v>Deborah Asokhia (NL)</v>
@@ -3958,16 +3928,16 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B9" t="str">
         <v>Donna Gabillard (NL)</v>
       </c>
       <c r="C9" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D9" t="str">
-        <v>09:15-11:30</v>
+        <v>09:15-14:15</v>
       </c>
       <c r="E9" t="str">
         <v>2.8</v>
@@ -3976,15 +3946,15 @@
         <v>2.8</v>
       </c>
       <c r="G9" t="str">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="H9" t="str">
-        <v/>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B10" t="str">
         <v>Hamza Nafees (NL) (GH)</v>
@@ -4010,7 +3980,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B11" t="str">
         <v>Kaitlyn Barton (NL) (GH)</v>
@@ -4036,7 +4006,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B12" t="str">
         <v>Lori Wylie (NL)</v>
@@ -4062,7 +4032,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B13" t="str">
         <v>Lynsey (GH) Mooney (NL)</v>
@@ -4088,7 +4058,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B14" t="str">
         <v>Madison Duncan (NL)</v>
@@ -4097,7 +4067,7 @@
         <v>Holiday</v>
       </c>
       <c r="D14" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E14" t="str">
         <v>8</v>
@@ -4114,7 +4084,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B15" t="str">
         <v>Mustansar Hussain (NL) (GH)</v>
@@ -4140,7 +4110,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B16" t="str">
         <v>Olusegun Isaac Ibrahim (NL)</v>
@@ -4166,7 +4136,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B17" t="str">
         <v>Shafiya Fayaz GH</v>
@@ -4192,7 +4162,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B18" t="str">
         <v>Sharon Jack (NL)</v>
@@ -4218,7 +4188,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B19" t="str">
         <v>Sophie Lamont (NL) (GH)</v>
@@ -4244,7 +4214,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2025-09-23</v>
+        <v>2025-10-07</v>
       </c>
       <c r="B20" t="str">
         <v>Wayne (GH) Griffiths (NL)</v>
@@ -4270,7 +4240,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B21" t="str">
         <v>Amanda Forbes (NL) (GH)</v>
@@ -4296,7 +4266,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B22" t="str">
         <v>Ashleigh Graham (GH) (NL)</v>
@@ -4322,7 +4292,7 @@
     </row>
     <row r="23" xml:space="preserve">
       <c r="A23" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B23" t="str">
         <v>Ayoola Ajibade (GH) (NL)</v>
@@ -4349,7 +4319,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B24" t="str">
         <v>Brooke O'Brien (NL) (GH)</v>
@@ -4375,7 +4345,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B25" t="str">
         <v>Cheryl McGhie (NL) (GH)</v>
@@ -4401,7 +4371,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B26" t="str">
         <v>Deborah Asokhia (NL)</v>
@@ -4427,13 +4397,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B27" t="str">
         <v>Donna Gabillard (NL)</v>
       </c>
       <c r="C27" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D27" t="str">
         <v>09:15-14:45</v>
@@ -4445,15 +4415,15 @@
         <v>2.8</v>
       </c>
       <c r="G27" t="str">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="H27" t="str">
-        <v/>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B28" t="str">
         <v>Hamza Nafees (NL) (GH)</v>
@@ -4479,7 +4449,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B29" t="str">
         <v>Kaitlyn Barton (NL) (GH)</v>
@@ -4505,16 +4475,16 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B30" t="str">
         <v>Lori Wylie (NL)</v>
       </c>
       <c r="C30" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D30" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-17:45</v>
       </c>
       <c r="E30" t="str">
         <v>6</v>
@@ -4523,15 +4493,15 @@
         <v>6</v>
       </c>
       <c r="G30" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H30" t="str">
-        <v/>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B31" t="str">
         <v>Lynsey (GH) Mooney (NL)</v>
@@ -4557,7 +4527,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B32" t="str">
         <v>Makala Mcewan (NL) (GH)</v>
@@ -4583,7 +4553,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B33" t="str">
         <v>Marykate Ferris (NL)</v>
@@ -4609,7 +4579,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B34" t="str">
         <v>Mustansar Hussain (NL) (GH)</v>
@@ -4635,7 +4605,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B35" t="str">
         <v>Olusegun Isaac Ibrahim (NL)</v>
@@ -4661,7 +4631,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B36" t="str">
         <v>Shafiya Fayaz GH</v>
@@ -4687,7 +4657,7 @@
     </row>
     <row r="37" xml:space="preserve">
       <c r="A37" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B37" t="str">
         <v>Sharon Jack (NL)</v>
@@ -4714,7 +4684,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2025-09-24</v>
+        <v>2025-10-08</v>
       </c>
       <c r="B38" t="str">
         <v>Wayne (GH) Griffiths (NL)</v>
@@ -4740,7 +4710,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B39" t="str">
         <v>Amanda Forbes (NL) (GH)</v>
@@ -4766,33 +4736,33 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B40" t="str">
         <v>Anne Nelson (NL)</v>
       </c>
       <c r="C40" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D40" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-17:15</v>
       </c>
       <c r="E40" t="str">
-        <v>4</v>
+        <v>5.33</v>
       </c>
       <c r="F40" t="str">
-        <v>4</v>
+        <v>5.33</v>
       </c>
       <c r="G40" t="str">
-        <v>0</v>
+        <v>5.33</v>
       </c>
       <c r="H40" t="str">
-        <v>Created by new vacation process.</v>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B41" t="str">
         <v>Ashleigh Graham (GH) (NL)</v>
@@ -4818,7 +4788,7 @@
     </row>
     <row r="42" xml:space="preserve">
       <c r="A42" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B42" t="str">
         <v>Ayoola Ajibade (GH) (NL)</v>
@@ -4845,7 +4815,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B43" t="str">
         <v>Brooke O'Brien (NL) (GH)</v>
@@ -4871,7 +4841,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B44" t="str">
         <v>Cheryl McGhie (NL) (GH)</v>
@@ -4897,7 +4867,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B45" t="str">
         <v>Deborah Asokhia (NL)</v>
@@ -4923,16 +4893,16 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B46" t="str">
         <v>Donna Gabillard (NL)</v>
       </c>
       <c r="C46" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D46" t="str">
-        <v>09:15-11:30</v>
+        <v>09:15-14:15</v>
       </c>
       <c r="E46" t="str">
         <v>2.8</v>
@@ -4941,15 +4911,15 @@
         <v>2.8</v>
       </c>
       <c r="G46" t="str">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="H46" t="str">
-        <v/>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B47" t="str">
         <v>Hamza Nafees (NL) (GH)</v>
@@ -4975,7 +4945,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B48" t="str">
         <v>Kaitlyn Barton (NL) (GH)</v>
@@ -5001,16 +4971,16 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B49" t="str">
         <v>Lori Wylie (NL)</v>
       </c>
       <c r="C49" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D49" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-17:45</v>
       </c>
       <c r="E49" t="str">
         <v>6</v>
@@ -5019,15 +4989,15 @@
         <v>6</v>
       </c>
       <c r="G49" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H49" t="str">
-        <v/>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B50" t="str">
         <v>Lynsey (GH) Mooney (NL)</v>
@@ -5053,7 +5023,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B51" t="str">
         <v>Makala Mcewan (NL) (GH)</v>
@@ -5079,7 +5049,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B52" t="str">
         <v>Marykate Ferris (NL)</v>
@@ -5105,7 +5075,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B53" t="str">
         <v>Olusegun Isaac Ibrahim (NL)</v>
@@ -5131,7 +5101,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B54" t="str">
         <v>Shafiya Fayaz GH</v>
@@ -5157,7 +5127,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B55" t="str">
         <v>Sharon Jack (NL)</v>
@@ -5183,7 +5153,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2025-09-25</v>
+        <v>2025-10-09</v>
       </c>
       <c r="B56" t="str">
         <v>Wayne (GH) Griffiths (NL)</v>
@@ -5209,7 +5179,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B57" t="str">
         <v>Amanda Forbes (NL) (GH)</v>
@@ -5235,33 +5205,33 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B58" t="str">
         <v>Anne Nelson (NL)</v>
       </c>
       <c r="C58" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D58" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-13:00</v>
       </c>
       <c r="E58" t="str">
-        <v>4</v>
+        <v>5.33</v>
       </c>
       <c r="F58" t="str">
-        <v>4</v>
+        <v>5.33</v>
       </c>
       <c r="G58" t="str">
-        <v>0</v>
+        <v>5.33</v>
       </c>
       <c r="H58" t="str">
-        <v>Created by new vacation process.</v>
+        <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B59" t="str">
         <v>Ashleigh Graham (GH) (NL)</v>
@@ -5287,7 +5257,7 @@
     </row>
     <row r="60" xml:space="preserve">
       <c r="A60" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B60" t="str">
         <v>Ayoola Ajibade (GH) (NL)</v>
@@ -5314,7 +5284,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B61" t="str">
         <v>Brooke O'Brien (NL) (GH)</v>
@@ -5338,15 +5308,15 @@
         <v/>
       </c>
     </row>
-    <row r="62" xml:space="preserve">
+    <row r="62">
       <c r="A62" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B62" t="str">
         <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="C62" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D62" t="str">
         <v>16:45-21:30</v>
@@ -5358,16 +5328,15 @@
         <v>3.2</v>
       </c>
       <c r="G62" t="str">
-        <v>0</v>
-      </c>
-      <c r="H62" t="str" xml:space="preserve">
-        <v xml:space="preserve">Cheryl emailed to advise she is away for the September weekend 
-Eilidh 15/09/2025</v>
+        <v>3.2</v>
+      </c>
+      <c r="H62" t="str">
+        <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B63" t="str">
         <v>Deborah Asokhia (NL)</v>
@@ -5393,16 +5362,16 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B64" t="str">
         <v>Donna Gabillard (NL)</v>
       </c>
       <c r="C64" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D64" t="str">
-        <v>09:15-10:15</v>
+        <v>09:15-14:15</v>
       </c>
       <c r="E64" t="str">
         <v>2.8</v>
@@ -5411,15 +5380,15 @@
         <v>2.8</v>
       </c>
       <c r="G64" t="str">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="H64" t="str">
-        <v/>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B65" t="str">
         <v>Hamza Nafees (NL) (GH)</v>
@@ -5445,7 +5414,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B66" t="str">
         <v>Kaitlyn Barton (NL) (GH)</v>
@@ -5471,7 +5440,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B67" t="str">
         <v>Lori Wylie (NL)</v>
@@ -5497,7 +5466,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B68" t="str">
         <v>Lynsey (GH) Mooney (NL)</v>
@@ -5523,7 +5492,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B69" t="str">
         <v>Makala Mcewan (NL) (GH)</v>
@@ -5549,7 +5518,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B70" t="str">
         <v>Mustansar Hussain (NL) (GH)</v>
@@ -5575,7 +5544,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B71" t="str">
         <v>Olusegun Isaac Ibrahim (NL)</v>
@@ -5601,7 +5570,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B72" t="str">
         <v>Shafiya Fayaz GH</v>
@@ -5627,13 +5596,13 @@
     </row>
     <row r="73" xml:space="preserve">
       <c r="A73" t="str">
-        <v>2025-09-26</v>
+        <v>2025-10-10</v>
       </c>
       <c r="B73" t="str">
         <v>Sharon Jack (NL)</v>
       </c>
       <c r="C73" t="str">
-        <v>Holiday</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D73" t="str">
         <v>09:15-17:00</v>
@@ -5642,19 +5611,19 @@
         <v>4.8</v>
       </c>
       <c r="F73" t="str">
-        <v>4.8</v>
+        <v>2</v>
       </c>
       <c r="G73" t="str">
         <v>0</v>
       </c>
       <c r="H73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Created by new vacation process.; Wants this as a break. 
+        <v xml:space="preserve">Wants this as a break. 
 Eilidh 29/05/2025</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-11</v>
       </c>
       <c r="B74" t="str">
         <v>Adedayo Adeyanju (NL) (GH)</v>
@@ -5680,89 +5649,89 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-11</v>
       </c>
       <c r="B75" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C75" t="str">
-        <v>Holiday</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D75" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E75" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="F75" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="G75" t="str">
         <v>0</v>
       </c>
       <c r="H75" t="str">
-        <v>Created by new vacation process.</v>
-      </c>
-    </row>
-    <row r="76">
+        <v/>
+      </c>
+    </row>
+    <row r="76" xml:space="preserve">
       <c r="A76" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-11</v>
       </c>
       <c r="B76" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
+        <v>Ayoola Ajibade (GH) (NL)</v>
       </c>
       <c r="C76" t="str">
         <v>Maternity/Paternity</v>
       </c>
       <c r="D76" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E76" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="F76" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="G76" t="str">
         <v>0</v>
       </c>
-      <c r="H76" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="77" xml:space="preserve">
-      <c r="A77" t="str">
-        <v>2025-09-27</v>
-      </c>
-      <c r="B77" t="str">
-        <v>Ayoola Ajibade (GH) (NL)</v>
-      </c>
-      <c r="C77" t="str">
-        <v>Maternity/Paternity</v>
-      </c>
-      <c r="D77" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E77" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="F77" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="G77" t="str">
-        <v>0</v>
-      </c>
-      <c r="H77" t="str" xml:space="preserve">
+      <c r="H76" t="str" xml:space="preserve">
         <v xml:space="preserve">Morning sickness
 Eilidh 31/03/2025</v>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>2025-10-11</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Brooke O'Brien (NL) (GH)</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D77" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E77" t="str">
+        <v>2.67</v>
+      </c>
+      <c r="F77" t="str">
+        <v>2.67</v>
+      </c>
+      <c r="G77" t="str">
+        <v>2.67</v>
+      </c>
+      <c r="H77" t="str">
+        <v/>
+      </c>
+    </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-11</v>
       </c>
       <c r="B78" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Emma Shawcross (NL)</v>
       </c>
       <c r="C78" t="str">
         <v>Available</v>
@@ -5771,24 +5740,24 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E78" t="str">
-        <v>2.67</v>
+        <v>10</v>
       </c>
       <c r="F78" t="str">
-        <v>2.67</v>
+        <v>10</v>
       </c>
       <c r="G78" t="str">
-        <v>2.67</v>
+        <v>10</v>
       </c>
       <c r="H78" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-11</v>
       </c>
       <c r="B79" t="str">
-        <v>Emma Shawcross (NL)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="C79" t="str">
         <v>Available</v>
@@ -5797,24 +5766,24 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E79" t="str">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F79" t="str">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G79" t="str">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H79" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-11</v>
       </c>
       <c r="B80" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Shafiya Fayaz GH</v>
       </c>
       <c r="C80" t="str">
         <v>Available</v>
@@ -5823,13 +5792,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E80" t="str">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F80" t="str">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G80" t="str">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H80" t="str">
         <v/>
@@ -5837,10 +5806,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-11</v>
       </c>
       <c r="B81" t="str">
-        <v>Shafiya Fayaz GH</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="C81" t="str">
         <v>Available</v>
@@ -5849,13 +5818,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E81" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="F81" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="G81" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H81" t="str">
         <v/>
@@ -5863,10 +5832,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2025-09-27</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B82" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
+        <v>Adedayo Adeyanju (NL) (GH)</v>
       </c>
       <c r="C82" t="str">
         <v>Available</v>
@@ -5889,181 +5858,181 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B83" t="str">
-        <v>Adedayo Adeyanju (NL) (GH)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="C83" t="str">
         <v>Available</v>
       </c>
       <c r="D83" t="str">
-        <v>08:00-21:30</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="E83" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="F83" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="G83" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="H83" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B84" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C84" t="str">
-        <v>Available</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D84" t="str">
-        <v>10:30-14:00</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E84" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="F84" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="G84" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H84" t="str">
-        <v>Confirmed at induction with MT</v>
+        <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B85" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C85" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D85" t="str">
-        <v>08:00-15:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E85" t="str">
-        <v>2.29</v>
+        <v>2.67</v>
       </c>
       <c r="F85" t="str">
-        <v>2.29</v>
+        <v>2.67</v>
       </c>
       <c r="G85" t="str">
-        <v>0</v>
+        <v>2.67</v>
       </c>
       <c r="H85" t="str">
-        <v/>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B86" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="C86" t="str">
         <v>Available</v>
       </c>
       <c r="D86" t="str">
-        <v>09:15-14:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E86" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="F86" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="G86" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="H86" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B87" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="C87" t="str">
         <v>Available</v>
       </c>
       <c r="D87" t="str">
-        <v>16:45-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E87" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="F87" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="G87" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="H87" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B88" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="C88" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D88" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="E88" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="F88" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="G88" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H88" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B89" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="C89" t="str">
-        <v>Available</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D89" t="str">
-        <v>09:15-14:45</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E89" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="F89" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="G89" t="str">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="H89" t="str">
         <v/>
@@ -6071,25 +6040,25 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B90" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="C90" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D90" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E90" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F90" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G90" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H90" t="str">
         <v/>
@@ -6097,25 +6066,25 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B91" t="str">
-        <v>Lori Wylie (NL)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="C91" t="str">
         <v>Available</v>
       </c>
       <c r="D91" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E91" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F91" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G91" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H91" t="str">
         <v/>
@@ -6123,129 +6092,129 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B92" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Madison Duncan (NL)</v>
       </c>
       <c r="C92" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D92" t="str">
-        <v>08:00-15:00</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E92" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F92" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G92" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H92" t="str">
-        <v/>
+        <v>Created by new vacation process.</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B93" t="str">
-        <v>Madison Duncan (NL)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="C93" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D93" t="str">
         <v>08:00-21:30</v>
       </c>
       <c r="E93" t="str">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F93" t="str">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G93" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H93" t="str">
-        <v>Created by new vacation process.</v>
+        <v/>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B94" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="C94" t="str">
         <v>Available</v>
       </c>
       <c r="D94" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:00</v>
       </c>
       <c r="E94" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="F94" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="G94" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H94" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B95" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Sharon Jack (NL)</v>
       </c>
       <c r="C95" t="str">
         <v>Available</v>
       </c>
       <c r="D95" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E95" t="str">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="F95" t="str">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="G95" t="str">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="H95" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B96" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="C96" t="str">
         <v>Available</v>
       </c>
       <c r="D96" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E96" t="str">
-        <v>4.8</v>
+        <v>7.5</v>
       </c>
       <c r="F96" t="str">
-        <v>4.8</v>
+        <v>7.5</v>
       </c>
       <c r="G96" t="str">
-        <v>4.8</v>
+        <v>7.5</v>
       </c>
       <c r="H96" t="str">
         <v/>
@@ -6253,10 +6222,10 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-06</v>
       </c>
       <c r="B97" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="C97" t="str">
         <v>Available</v>
@@ -6265,13 +6234,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E97" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F97" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G97" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H97" t="str">
         <v/>
@@ -6279,10 +6248,10 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>2025-09-22</v>
+        <v>2025-10-12</v>
       </c>
       <c r="B98" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Adedayo Adeyanju (NL) (GH)</v>
       </c>
       <c r="C98" t="str">
         <v>Available</v>
@@ -6291,13 +6260,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E98" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="F98" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="G98" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="H98" t="str">
         <v/>
@@ -6305,25 +6274,25 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-12</v>
       </c>
       <c r="B99" t="str">
-        <v>Adedayo Adeyanju (NL) (GH)</v>
+        <v>Anne Nelson (NL)</v>
       </c>
       <c r="C99" t="str">
         <v>Available</v>
       </c>
       <c r="D99" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E99" t="str">
-        <v>7.5</v>
+        <v>5.33</v>
       </c>
       <c r="F99" t="str">
-        <v>7.5</v>
+        <v>5.33</v>
       </c>
       <c r="G99" t="str">
-        <v>7.5</v>
+        <v>5.33</v>
       </c>
       <c r="H99" t="str">
         <v/>
@@ -6331,103 +6300,103 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-12</v>
       </c>
       <c r="B100" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C100" t="str">
-        <v>Holiday</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D100" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E100" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="F100" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="G100" t="str">
         <v>0</v>
       </c>
       <c r="H100" t="str">
-        <v>Created by new vacation process.</v>
+        <v/>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-12</v>
       </c>
       <c r="B101" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
+        <v>Emma Shawcross (NL)</v>
       </c>
       <c r="C101" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D101" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E101" t="str">
-        <v>2.29</v>
+        <v>10</v>
       </c>
       <c r="F101" t="str">
-        <v>2.29</v>
+        <v>10</v>
       </c>
       <c r="G101" t="str">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H101" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-12</v>
       </c>
       <c r="B102" t="str">
-        <v>Emma Shawcross (NL)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="C102" t="str">
-        <v>Available</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D102" t="str">
         <v>08:00-21:30</v>
       </c>
       <c r="E102" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="F102" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="G102" t="str">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H102" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-12</v>
       </c>
       <c r="B103" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Makala Mcewan (NL) (GH)</v>
       </c>
       <c r="C103" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D103" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="E103" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="F103" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="G103" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H103" t="str">
         <v/>
@@ -6435,25 +6404,25 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-12</v>
       </c>
       <c r="B104" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="C104" t="str">
         <v>Available</v>
       </c>
       <c r="D104" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E104" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="F104" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="G104" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="H104" t="str">
         <v/>
@@ -6461,10 +6430,10 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-12</v>
       </c>
       <c r="B105" t="str">
-        <v>Marykate Ferris (NL)</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="C105" t="str">
         <v>Available</v>
@@ -6473,13 +6442,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E105" t="str">
-        <v>6.67</v>
+        <v>7.5</v>
       </c>
       <c r="F105" t="str">
-        <v>6.67</v>
+        <v>7.5</v>
       </c>
       <c r="G105" t="str">
-        <v>6.67</v>
+        <v>7.5</v>
       </c>
       <c r="H105" t="str">
         <v/>
@@ -6487,10 +6456,10 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>2025-09-28</v>
+        <v>2025-10-12</v>
       </c>
       <c r="B106" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="C106" t="str">
         <v>Available</v>
@@ -6499,47 +6468,21 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E106" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F106" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G106" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H106" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="str">
-        <v>2025-09-28</v>
-      </c>
-      <c r="B107" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
-      </c>
-      <c r="C107" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D107" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E107" t="str">
-        <v>6</v>
-      </c>
-      <c r="F107" t="str">
-        <v>6</v>
-      </c>
-      <c r="G107" t="str">
-        <v>6</v>
-      </c>
-      <c r="H107" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H107"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H106"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add partial availability status to improve capacity calculations
Update server/pipeline.ts to include "Partial Availability" in STATUS_PRIORITY and adjust logic for calculating net capacity based on time blockers and employee availability.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: faa34da4-36c5-42e2-9a7d-dfe321980219
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/faa34da4-36c5-42e2-9a7d-dfe321980219/Bt6CaEz
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -452,7 +452,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="F2" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G2" t="str">
         <v>7.5</v>
@@ -462,7 +462,7 @@
       </c>
       <c r="I2" t="str" xml:space="preserve">
         <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025</v>
+Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -482,7 +482,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="F3" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G3" t="str">
         <v>7.5</v>
@@ -492,7 +492,7 @@
       </c>
       <c r="I3" t="str" xml:space="preserve">
         <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025</v>
+Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -512,7 +512,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="F4" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G4" t="str">
         <v>7.5</v>
@@ -522,7 +522,7 @@
       </c>
       <c r="I4" t="str" xml:space="preserve">
         <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025</v>
+Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
@@ -542,7 +542,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="F5" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G5" t="str">
         <v>7.5</v>
@@ -552,7 +552,7 @@
       </c>
       <c r="I5" t="str" xml:space="preserve">
         <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025</v>
+Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
@@ -572,7 +572,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="F6" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G6" t="str">
         <v>7.5</v>
@@ -582,7 +582,7 @@
       </c>
       <c r="I6" t="str" xml:space="preserve">
         <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025</v>
+Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="7">
@@ -602,7 +602,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="F7" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="G7" t="str">
         <v>2.29</v>
@@ -611,7 +611,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="8">
@@ -631,7 +631,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="F8" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="G8" t="str">
         <v>2.29</v>
@@ -640,7 +640,7 @@
         <v>0</v>
       </c>
       <c r="I8" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="9">
@@ -660,7 +660,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="F9" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="G9" t="str">
         <v>2.29</v>
@@ -669,7 +669,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="10">
@@ -689,7 +689,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="F10" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="G10" t="str">
         <v>2.29</v>
@@ -698,7 +698,7 @@
         <v>0</v>
       </c>
       <c r="I10" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="11">
@@ -718,7 +718,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="F11" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="G11" t="str">
         <v>2.29</v>
@@ -727,7 +727,7 @@
         <v>0</v>
       </c>
       <c r="I11" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="12">
@@ -747,7 +747,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="F12" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="G12" t="str">
         <v>2.29</v>
@@ -756,7 +756,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="13">
@@ -776,7 +776,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="F13" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="G13" t="str">
         <v>2.29</v>
@@ -785,7 +785,7 @@
         <v>0</v>
       </c>
       <c r="I13" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="14">
@@ -805,7 +805,7 @@
         <v>Holiday</v>
       </c>
       <c r="F14" t="str">
-        <v>09:15-14:45</v>
+        <v/>
       </c>
       <c r="G14" t="str">
         <v>2.8</v>
@@ -814,7 +814,7 @@
         <v>0</v>
       </c>
       <c r="I14" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="15">
@@ -834,7 +834,7 @@
         <v>Holiday</v>
       </c>
       <c r="F15" t="str">
-        <v>09:15-14:15</v>
+        <v/>
       </c>
       <c r="G15" t="str">
         <v>2.8</v>
@@ -843,7 +843,7 @@
         <v>0</v>
       </c>
       <c r="I15" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="16">
@@ -863,7 +863,7 @@
         <v>Holiday</v>
       </c>
       <c r="F16" t="str">
-        <v>09:15-14:45</v>
+        <v/>
       </c>
       <c r="G16" t="str">
         <v>2.8</v>
@@ -872,7 +872,7 @@
         <v>0</v>
       </c>
       <c r="I16" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="17">
@@ -892,7 +892,7 @@
         <v>Holiday</v>
       </c>
       <c r="F17" t="str">
-        <v>09:15-14:15</v>
+        <v/>
       </c>
       <c r="G17" t="str">
         <v>2.8</v>
@@ -901,7 +901,7 @@
         <v>0</v>
       </c>
       <c r="I17" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="18">
@@ -921,7 +921,7 @@
         <v>Holiday</v>
       </c>
       <c r="F18" t="str">
-        <v>09:15-14:15</v>
+        <v/>
       </c>
       <c r="G18" t="str">
         <v>2.8</v>
@@ -930,7 +930,7 @@
         <v>0</v>
       </c>
       <c r="I18" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="19">
@@ -950,7 +950,7 @@
         <v>Holiday</v>
       </c>
       <c r="F19" t="str">
-        <v>08:00-18:00</v>
+        <v/>
       </c>
       <c r="G19" t="str">
         <v>8</v>
@@ -959,7 +959,7 @@
         <v>0</v>
       </c>
       <c r="I19" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="20">
@@ -979,7 +979,7 @@
         <v>Holiday</v>
       </c>
       <c r="F20" t="str">
-        <v>08:00-18:00</v>
+        <v/>
       </c>
       <c r="G20" t="str">
         <v>8</v>
@@ -988,7 +988,7 @@
         <v>0</v>
       </c>
       <c r="I20" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="21">
@@ -1008,7 +1008,7 @@
         <v>Holiday</v>
       </c>
       <c r="F21" t="str">
-        <v>09:15-17:45</v>
+        <v/>
       </c>
       <c r="G21" t="str">
         <v>6</v>
@@ -1017,7 +1017,7 @@
         <v>0</v>
       </c>
       <c r="I21" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="22">
@@ -1037,7 +1037,7 @@
         <v>Holiday</v>
       </c>
       <c r="F22" t="str">
-        <v>09:15-17:45</v>
+        <v/>
       </c>
       <c r="G22" t="str">
         <v>6</v>
@@ -1046,7 +1046,7 @@
         <v>0</v>
       </c>
       <c r="I22" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="23">
@@ -1066,7 +1066,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F23" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G23" t="str">
         <v>7.5</v>
@@ -1095,7 +1095,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F24" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G24" t="str">
         <v>7.5</v>
@@ -1124,7 +1124,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F25" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G25" t="str">
         <v>7.5</v>
@@ -1153,7 +1153,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F26" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G26" t="str">
         <v>7.5</v>
@@ -1182,7 +1182,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F27" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G27" t="str">
         <v>7.5</v>
@@ -1211,7 +1211,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F28" t="str">
-        <v>09:15-16:15</v>
+        <v>09:15-10:30; 12:30-16:15</v>
       </c>
       <c r="G28" t="str">
         <v>2</v>
@@ -1240,7 +1240,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F29" t="str">
-        <v>09:15-16:30</v>
+        <v>09:15-10:30; 12:30-16:30</v>
       </c>
       <c r="G29" t="str">
         <v>2</v>
@@ -1270,7 +1270,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F30" t="str">
-        <v>09:15-17:00</v>
+        <v>09:15-10:30; 12:30-17:00</v>
       </c>
       <c r="G30" t="str">
         <v>2</v>
@@ -3806,7 +3806,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="D4" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="E4" t="str">
         <v>2.29</v>
@@ -3818,7 +3818,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
@@ -3832,7 +3832,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="D5" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E5" t="str">
         <v>7.5</v>
@@ -3845,7 +3845,7 @@
       </c>
       <c r="H5" t="str" xml:space="preserve">
         <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025</v>
+Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="6">
@@ -3937,7 +3937,7 @@
         <v>Holiday</v>
       </c>
       <c r="D9" t="str">
-        <v>09:15-14:15</v>
+        <v/>
       </c>
       <c r="E9" t="str">
         <v>2.8</v>
@@ -3949,7 +3949,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="10">
@@ -3963,7 +3963,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D10" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E10" t="str">
         <v>7.5</v>
@@ -4067,7 +4067,7 @@
         <v>Holiday</v>
       </c>
       <c r="D14" t="str">
-        <v>08:00-18:00</v>
+        <v/>
       </c>
       <c r="E14" t="str">
         <v>8</v>
@@ -4079,7 +4079,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="15">
@@ -4171,7 +4171,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D18" t="str">
-        <v>09:15-16:15</v>
+        <v>09:15-10:30; 12:30-16:15</v>
       </c>
       <c r="E18" t="str">
         <v>4.8</v>
@@ -4275,7 +4275,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="D22" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="E22" t="str">
         <v>2.29</v>
@@ -4287,7 +4287,7 @@
         <v>0</v>
       </c>
       <c r="H22" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="23" xml:space="preserve">
@@ -4301,7 +4301,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="D23" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E23" t="str">
         <v>7.5</v>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="H23" t="str" xml:space="preserve">
         <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025</v>
+Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="24">
@@ -4406,7 +4406,7 @@
         <v>Holiday</v>
       </c>
       <c r="D27" t="str">
-        <v>09:15-14:45</v>
+        <v/>
       </c>
       <c r="E27" t="str">
         <v>2.8</v>
@@ -4418,7 +4418,7 @@
         <v>0</v>
       </c>
       <c r="H27" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="28">
@@ -4432,7 +4432,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D28" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E28" t="str">
         <v>7.5</v>
@@ -4484,7 +4484,7 @@
         <v>Holiday</v>
       </c>
       <c r="D30" t="str">
-        <v>09:15-17:45</v>
+        <v/>
       </c>
       <c r="E30" t="str">
         <v>6</v>
@@ -4496,7 +4496,7 @@
         <v>0</v>
       </c>
       <c r="H30" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="31">
@@ -4666,7 +4666,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D37" t="str">
-        <v>09:15-16:30</v>
+        <v>09:15-10:30; 12:30-16:30</v>
       </c>
       <c r="E37" t="str">
         <v>4.8</v>
@@ -4771,7 +4771,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="D41" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="E41" t="str">
         <v>2.29</v>
@@ -4783,7 +4783,7 @@
         <v>0</v>
       </c>
       <c r="H41" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="42" xml:space="preserve">
@@ -4797,7 +4797,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="D42" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E42" t="str">
         <v>7.5</v>
@@ -4810,7 +4810,7 @@
       </c>
       <c r="H42" t="str" xml:space="preserve">
         <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025</v>
+Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="43">
@@ -4902,7 +4902,7 @@
         <v>Holiday</v>
       </c>
       <c r="D46" t="str">
-        <v>09:15-14:15</v>
+        <v/>
       </c>
       <c r="E46" t="str">
         <v>2.8</v>
@@ -4914,7 +4914,7 @@
         <v>0</v>
       </c>
       <c r="H46" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="47">
@@ -4928,7 +4928,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D47" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E47" t="str">
         <v>7.5</v>
@@ -4980,7 +4980,7 @@
         <v>Holiday</v>
       </c>
       <c r="D49" t="str">
-        <v>09:15-17:45</v>
+        <v/>
       </c>
       <c r="E49" t="str">
         <v>6</v>
@@ -4992,7 +4992,7 @@
         <v>0</v>
       </c>
       <c r="H49" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="50">
@@ -5240,7 +5240,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="D59" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="E59" t="str">
         <v>2.29</v>
@@ -5252,7 +5252,7 @@
         <v>0</v>
       </c>
       <c r="H59" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="60" xml:space="preserve">
@@ -5266,7 +5266,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="D60" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E60" t="str">
         <v>7.5</v>
@@ -5279,7 +5279,7 @@
       </c>
       <c r="H60" t="str" xml:space="preserve">
         <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025</v>
+Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="61">
@@ -5371,7 +5371,7 @@
         <v>Holiday</v>
       </c>
       <c r="D64" t="str">
-        <v>09:15-14:15</v>
+        <v/>
       </c>
       <c r="E64" t="str">
         <v>2.8</v>
@@ -5383,7 +5383,7 @@
         <v>0</v>
       </c>
       <c r="H64" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="65">
@@ -5605,7 +5605,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D73" t="str">
-        <v>09:15-17:00</v>
+        <v>09:15-10:30; 12:30-17:00</v>
       </c>
       <c r="E73" t="str">
         <v>4.8</v>
@@ -5658,7 +5658,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="D75" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="E75" t="str">
         <v>2.29</v>
@@ -5670,7 +5670,7 @@
         <v>0</v>
       </c>
       <c r="H75" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="76" xml:space="preserve">
@@ -5684,7 +5684,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="D76" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E76" t="str">
         <v>7.5</v>
@@ -5697,7 +5697,7 @@
       </c>
       <c r="H76" t="str" xml:space="preserve">
         <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025</v>
+Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="77">
@@ -5893,7 +5893,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="D84" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="E84" t="str">
         <v>2.29</v>
@@ -5905,7 +5905,7 @@
         <v>0</v>
       </c>
       <c r="H84" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="85">
@@ -5997,7 +5997,7 @@
         <v>Holiday</v>
       </c>
       <c r="D88" t="str">
-        <v>09:15-14:45</v>
+        <v/>
       </c>
       <c r="E88" t="str">
         <v>2.8</v>
@@ -6009,7 +6009,7 @@
         <v>0</v>
       </c>
       <c r="H88" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="89">
@@ -6023,7 +6023,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D89" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E89" t="str">
         <v>7.5</v>
@@ -6101,7 +6101,7 @@
         <v>Holiday</v>
       </c>
       <c r="D92" t="str">
-        <v>08:00-18:00</v>
+        <v/>
       </c>
       <c r="E92" t="str">
         <v>8</v>
@@ -6113,7 +6113,7 @@
         <v>0</v>
       </c>
       <c r="H92" t="str">
-        <v>Created by new vacation process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="93">
@@ -6309,7 +6309,7 @@
         <v>Maternity/Paternity</v>
       </c>
       <c r="D100" t="str">
-        <v>08:00-15:30</v>
+        <v/>
       </c>
       <c r="E100" t="str">
         <v>2.29</v>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="H100" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="101">
@@ -6361,7 +6361,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D102" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E102" t="str">
         <v>7.5</v>

</xml_diff>

<commit_message>
Update capacity dashboard data for better workforce insights
Updated capacity_dashboard.xlsx with new data to enhance workforce management and employee wellness analytics.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: faa34da4-36c5-42e2-9a7d-dfe321980219
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/faa34da4-36c5-42e2-9a7d-dfe321980219/r5Zgp9T
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -1240,7 +1240,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F29" t="str">
-        <v>09:15-10:30; 12:30-16:30</v>
+        <v>09:15-10:30; 12:30-17:15</v>
       </c>
       <c r="G29" t="str">
         <v>2</v>
@@ -1270,7 +1270,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="F30" t="str">
-        <v>09:15-10:30; 12:30-17:00</v>
+        <v>09:15-10:30; 12:30-18:15</v>
       </c>
       <c r="G30" t="str">
         <v>2</v>
@@ -1300,7 +1300,7 @@
         <v>Available</v>
       </c>
       <c r="F31" t="str">
-        <v>10:30-14:00</v>
+        <v>10:30-15:15</v>
       </c>
       <c r="G31" t="str">
         <v>3.2</v>
@@ -1329,7 +1329,7 @@
         <v>Available</v>
       </c>
       <c r="F32" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-15:15; 20:30-21:30</v>
       </c>
       <c r="G32" t="str">
         <v>3.2</v>
@@ -1338,7 +1338,7 @@
         <v>3.2</v>
       </c>
       <c r="I32" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="33">
@@ -1358,7 +1358,7 @@
         <v>Available</v>
       </c>
       <c r="F33" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-15:15; 20:30-21:30</v>
       </c>
       <c r="G33" t="str">
         <v>3.2</v>
@@ -1367,7 +1367,7 @@
         <v>3.2</v>
       </c>
       <c r="I33" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="34">
@@ -1387,7 +1387,7 @@
         <v>Available</v>
       </c>
       <c r="F34" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-15:15; 20:30-21:30</v>
       </c>
       <c r="G34" t="str">
         <v>3.2</v>
@@ -1396,7 +1396,7 @@
         <v>3.2</v>
       </c>
       <c r="I34" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="35">
@@ -2692,7 +2692,7 @@
         <v>Available</v>
       </c>
       <c r="F79" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G79" t="str">
         <v>3.2</v>
@@ -2721,7 +2721,7 @@
         <v>Available</v>
       </c>
       <c r="F80" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G80" t="str">
         <v>3.2</v>
@@ -2750,7 +2750,7 @@
         <v>Available</v>
       </c>
       <c r="F81" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G81" t="str">
         <v>3.2</v>
@@ -2779,7 +2779,7 @@
         <v>Available</v>
       </c>
       <c r="F82" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G82" t="str">
         <v>3.2</v>
@@ -2808,7 +2808,7 @@
         <v>Available</v>
       </c>
       <c r="F83" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G83" t="str">
         <v>3.2</v>
@@ -3272,7 +3272,7 @@
         <v>Available</v>
       </c>
       <c r="F99" t="str">
-        <v>08:00-14:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="G99" t="str">
         <v>4</v>
@@ -3330,7 +3330,7 @@
         <v>Available</v>
       </c>
       <c r="F101" t="str">
-        <v>08:00-14:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="G101" t="str">
         <v>4</v>
@@ -3417,7 +3417,7 @@
         <v>Available</v>
       </c>
       <c r="F104" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-15:15; 16:45-21:30</v>
       </c>
       <c r="G104" t="str">
         <v>6</v>
@@ -3426,7 +3426,7 @@
         <v>6</v>
       </c>
       <c r="I104" t="str">
-        <v/>
+        <v>Lori has agreed to extend her availability via email on 02/04/2025 - MT</v>
       </c>
     </row>
     <row r="105">
@@ -3446,7 +3446,7 @@
         <v>Available</v>
       </c>
       <c r="F105" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G105" t="str">
         <v>6</v>
@@ -3780,7 +3780,7 @@
         <v>Available</v>
       </c>
       <c r="D3" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-15:15; 20:30-21:30</v>
       </c>
       <c r="E3" t="str">
         <v>3.2</v>
@@ -3792,7 +3792,7 @@
         <v>3.2</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="4">
@@ -4015,7 +4015,7 @@
         <v>Available</v>
       </c>
       <c r="D12" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E12" t="str">
         <v>6</v>
@@ -4119,7 +4119,7 @@
         <v>Available</v>
       </c>
       <c r="D16" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E16" t="str">
         <v>3.2</v>
@@ -4249,7 +4249,7 @@
         <v>Available</v>
       </c>
       <c r="D21" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-15:15; 20:30-21:30</v>
       </c>
       <c r="E21" t="str">
         <v>3.2</v>
@@ -4261,7 +4261,7 @@
         <v>3.2</v>
       </c>
       <c r="H21" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="22">
@@ -4510,7 +4510,7 @@
         <v>Available</v>
       </c>
       <c r="D31" t="str">
-        <v>08:00-14:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E31" t="str">
         <v>4</v>
@@ -4614,7 +4614,7 @@
         <v>Available</v>
       </c>
       <c r="D35" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E35" t="str">
         <v>3.2</v>
@@ -4666,7 +4666,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D37" t="str">
-        <v>09:15-10:30; 12:30-16:30</v>
+        <v>09:15-10:30; 12:30-17:15</v>
       </c>
       <c r="E37" t="str">
         <v>4.8</v>
@@ -4719,7 +4719,7 @@
         <v>Available</v>
       </c>
       <c r="D39" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-15:15; 20:30-21:30</v>
       </c>
       <c r="E39" t="str">
         <v>3.2</v>
@@ -4731,7 +4731,7 @@
         <v>3.2</v>
       </c>
       <c r="H39" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="40">
@@ -5084,7 +5084,7 @@
         <v>Available</v>
       </c>
       <c r="D53" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E53" t="str">
         <v>3.2</v>
@@ -5475,7 +5475,7 @@
         <v>Available</v>
       </c>
       <c r="D68" t="str">
-        <v>08:00-14:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E68" t="str">
         <v>4</v>
@@ -5553,7 +5553,7 @@
         <v>Available</v>
       </c>
       <c r="D71" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E71" t="str">
         <v>3.2</v>
@@ -5605,7 +5605,7 @@
         <v>Other Unavailable</v>
       </c>
       <c r="D73" t="str">
-        <v>09:15-10:30; 12:30-17:00</v>
+        <v>09:15-10:30; 12:30-18:15</v>
       </c>
       <c r="E73" t="str">
         <v>4.8</v>
@@ -5867,7 +5867,7 @@
         <v>Available</v>
       </c>
       <c r="D83" t="str">
-        <v>10:30-14:00</v>
+        <v>10:30-15:15</v>
       </c>
       <c r="E83" t="str">
         <v>3.2</v>
@@ -6049,7 +6049,7 @@
         <v>Available</v>
       </c>
       <c r="D90" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-15:15; 16:45-21:30</v>
       </c>
       <c r="E90" t="str">
         <v>6</v>
@@ -6061,7 +6061,7 @@
         <v>6</v>
       </c>
       <c r="H90" t="str">
-        <v/>
+        <v>Lori has agreed to extend her availability via email on 02/04/2025 - MT</v>
       </c>
     </row>
     <row r="91">
@@ -6153,7 +6153,7 @@
         <v>Available</v>
       </c>
       <c r="D94" t="str">
-        <v>09:15-15:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E94" t="str">
         <v>3.2</v>

</xml_diff>

<commit_message>
Update dashboard documentation to reflect current features and capabilities
Refactor replit.md to accurately describe the enhanced capacity dashboard functionality, including advanced data processing, new dashboard tabs, workforce features, and UI improvements.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: faa34da4-36c5-42e2-9a7d-dfe321980219
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/faa34da4-36c5-42e2-9a7d-dfe321980219/YhdqmBQ
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -1208,16 +1208,16 @@
         <v>2025-10-07</v>
       </c>
       <c r="E28" t="str">
-        <v>Other Unavailable</v>
+        <v>Partial Availability</v>
       </c>
       <c r="F28" t="str">
         <v>09:15-10:30; 12:30-16:15</v>
       </c>
       <c r="G28" t="str">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="H28" t="str">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="I28" t="str">
         <v>Sharon has advised she is unable to work between 10.30 and 12.30 on Tuesday's - MT</v>
@@ -1237,16 +1237,16 @@
         <v>2025-10-08</v>
       </c>
       <c r="E29" t="str">
-        <v>Other Unavailable</v>
+        <v>Partial Availability</v>
       </c>
       <c r="F29" t="str">
         <v>09:15-10:30; 12:30-17:15</v>
       </c>
       <c r="G29" t="str">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="H29" t="str">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="I29" t="str" xml:space="preserve">
         <v xml:space="preserve">Wants this as a break. 
@@ -1267,16 +1267,16 @@
         <v>2025-10-10</v>
       </c>
       <c r="E30" t="str">
-        <v>Other Unavailable</v>
+        <v>Partial Availability</v>
       </c>
       <c r="F30" t="str">
         <v>09:15-10:30; 12:30-18:15</v>
       </c>
       <c r="G30" t="str">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="H30" t="str">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="I30" t="str" xml:space="preserve">
         <v xml:space="preserve">Wants this as a break. 
@@ -3558,10 +3558,10 @@
         <v>69.77</v>
       </c>
       <c r="C3" t="str">
-        <v>69.77</v>
+        <v>72.57</v>
       </c>
       <c r="D3" t="str">
-        <v>19.29</v>
+        <v>20.09</v>
       </c>
       <c r="E3" t="str">
         <v>10.8</v>
@@ -3570,7 +3570,7 @@
         <v>64.25</v>
       </c>
       <c r="G3" t="str">
-        <v>5.52</v>
+        <v>8.32</v>
       </c>
       <c r="H3" t="str">
         <v>Sufficient</v>
@@ -3584,10 +3584,10 @@
         <v>59.44</v>
       </c>
       <c r="C4" t="str">
-        <v>59.44</v>
+        <v>62.24</v>
       </c>
       <c r="D4" t="str">
-        <v>19.29</v>
+        <v>20.09</v>
       </c>
       <c r="E4" t="str">
         <v>8.8</v>
@@ -3596,7 +3596,7 @@
         <v>86.5</v>
       </c>
       <c r="G4" t="str">
-        <v>-27.06</v>
+        <v>-24.26</v>
       </c>
       <c r="H4" t="str">
         <v>Shortage</v>
@@ -3636,10 +3636,10 @@
         <v>65.6</v>
       </c>
       <c r="C6" t="str">
-        <v>65.6</v>
+        <v>68.4</v>
       </c>
       <c r="D6" t="str">
-        <v>11.79</v>
+        <v>12.59</v>
       </c>
       <c r="E6" t="str">
         <v>2.8</v>
@@ -3648,7 +3648,7 @@
         <v>59.5</v>
       </c>
       <c r="G6" t="str">
-        <v>6.1</v>
+        <v>8.9</v>
       </c>
       <c r="H6" t="str">
         <v>Sufficient</v>
@@ -4168,7 +4168,7 @@
         <v>Sharon Jack (NL)</v>
       </c>
       <c r="C18" t="str">
-        <v>Other Unavailable</v>
+        <v>Partial Availability</v>
       </c>
       <c r="D18" t="str">
         <v>09:15-10:30; 12:30-16:15</v>
@@ -4177,10 +4177,10 @@
         <v>4.8</v>
       </c>
       <c r="F18" t="str">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="G18" t="str">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="H18" t="str">
         <v>Sharon has advised she is unable to work between 10.30 and 12.30 on Tuesday's - MT</v>
@@ -4663,7 +4663,7 @@
         <v>Sharon Jack (NL)</v>
       </c>
       <c r="C37" t="str">
-        <v>Other Unavailable</v>
+        <v>Partial Availability</v>
       </c>
       <c r="D37" t="str">
         <v>09:15-10:30; 12:30-17:15</v>
@@ -4672,10 +4672,10 @@
         <v>4.8</v>
       </c>
       <c r="F37" t="str">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="G37" t="str">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="H37" t="str" xml:space="preserve">
         <v xml:space="preserve">Wants this as a break. 
@@ -5602,7 +5602,7 @@
         <v>Sharon Jack (NL)</v>
       </c>
       <c r="C73" t="str">
-        <v>Other Unavailable</v>
+        <v>Partial Availability</v>
       </c>
       <c r="D73" t="str">
         <v>09:15-10:30; 12:30-18:15</v>
@@ -5611,10 +5611,10 @@
         <v>4.8</v>
       </c>
       <c r="F73" t="str">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="G73" t="str">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="H73" t="str" xml:space="preserve">
         <v xml:space="preserve">Wants this as a break. 

</xml_diff>

<commit_message>
Add capacity dashboard data for workforce planning
Add capacity_dashboard.xlsx file to the repository.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: faa34da4-36c5-42e2-9a7d-dfe321980219
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/faa34da4-36c5-42e2-9a7d-dfe321980219/dOz1sph
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I107"/>
+  <dimension ref="A1:I103"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -819,31 +819,31 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Madison Duncan (NL)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="B15" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C15" t="str">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D15" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E15" t="str">
-        <v>Holiday</v>
+        <v>Sick</v>
       </c>
       <c r="F15" t="str">
         <v/>
       </c>
       <c r="G15" t="str">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H15" t="str">
         <v>0</v>
       </c>
       <c r="I15" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v>Sciatica flare up - MT [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="16">
@@ -857,7 +857,7 @@
         <v>8</v>
       </c>
       <c r="D16" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E16" t="str">
         <v>Holiday</v>
@@ -877,16 +877,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Madison Duncan (NL)</v>
       </c>
       <c r="B17" t="str">
         <v>16</v>
       </c>
       <c r="C17" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D17" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E17" t="str">
         <v>Holiday</v>
@@ -895,7 +895,7 @@
         <v/>
       </c>
       <c r="G17" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H17" t="str">
         <v>0</v>
@@ -915,7 +915,7 @@
         <v>4</v>
       </c>
       <c r="D18" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E18" t="str">
         <v>Holiday</v>
@@ -944,7 +944,7 @@
         <v>4</v>
       </c>
       <c r="D19" t="str">
-        <v>2025-09-27</v>
+        <v>2025-09-26</v>
       </c>
       <c r="E19" t="str">
         <v>Holiday</v>
@@ -973,7 +973,7 @@
         <v>4</v>
       </c>
       <c r="D20" t="str">
-        <v>2025-09-28</v>
+        <v>2025-09-27</v>
       </c>
       <c r="E20" t="str">
         <v>Holiday</v>
@@ -991,18 +991,18 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
-    <row r="21" xml:space="preserve">
+    <row r="21">
       <c r="A21" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Anne Nelson (NL)</v>
       </c>
       <c r="B21" t="str">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C21" t="str">
-        <v>4.8</v>
+        <v>4</v>
       </c>
       <c r="D21" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-28</v>
       </c>
       <c r="E21" t="str">
         <v>Holiday</v>
@@ -1011,43 +1011,43 @@
         <v/>
       </c>
       <c r="G21" t="str">
-        <v>4.8</v>
+        <v>4</v>
       </c>
       <c r="H21" t="str">
         <v>0</v>
       </c>
-      <c r="I21" t="str" xml:space="preserve">
+      <c r="I21" t="str">
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>Sharon Jack (NL)</v>
+      </c>
+      <c r="B22" t="str">
+        <v>24</v>
+      </c>
+      <c r="C22" t="str">
+        <v>4.8</v>
+      </c>
+      <c r="D22" t="str">
+        <v>2025-09-26</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Holiday</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v>4.8</v>
+      </c>
+      <c r="H22" t="str">
+        <v>0</v>
+      </c>
+      <c r="I22" t="str" xml:space="preserve">
         <v xml:space="preserve">Created by new vacation process.; Wants this as a break. 
 Eilidh 29/05/2025 [availability ignored due to day-level leave]</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
-      </c>
-      <c r="B22" t="str">
-        <v>45</v>
-      </c>
-      <c r="C22" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="D22" t="str">
-        <v>2025-09-22</v>
-      </c>
-      <c r="E22" t="str">
-        <v>Other Unavailable</v>
-      </c>
-      <c r="F22" t="str">
-        <v/>
-      </c>
-      <c r="G22" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H22" t="str">
-        <v>0</v>
-      </c>
-      <c r="I22" t="str">
-        <v/>
       </c>
     </row>
     <row r="23">
@@ -1061,7 +1061,7 @@
         <v>7.5</v>
       </c>
       <c r="D23" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E23" t="str">
         <v>Other Unavailable</v>
@@ -1090,7 +1090,7 @@
         <v>7.5</v>
       </c>
       <c r="D24" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E24" t="str">
         <v>Other Unavailable</v>
@@ -1119,7 +1119,7 @@
         <v>7.5</v>
       </c>
       <c r="D25" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E25" t="str">
         <v>Other Unavailable</v>
@@ -1148,7 +1148,7 @@
         <v>7.5</v>
       </c>
       <c r="D26" t="str">
-        <v>2025-09-28</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E26" t="str">
         <v>Other Unavailable</v>
@@ -1166,18 +1166,18 @@
         <v/>
       </c>
     </row>
-    <row r="27" xml:space="preserve">
+    <row r="27">
       <c r="A27" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="B27" t="str">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="C27" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="D27" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-28</v>
       </c>
       <c r="E27" t="str">
         <v>Other Unavailable</v>
@@ -1186,46 +1186,46 @@
         <v/>
       </c>
       <c r="G27" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H27" t="str">
         <v>0</v>
       </c>
-      <c r="I27" t="str" xml:space="preserve">
+      <c r="I27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>Cheryl McGhie (NL) (GH)</v>
+      </c>
+      <c r="B28" t="str">
+        <v>16</v>
+      </c>
+      <c r="C28" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="D28" t="str">
+        <v>2025-09-26</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Other Unavailable</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H28" t="str">
+        <v>0</v>
+      </c>
+      <c r="I28" t="str" xml:space="preserve">
         <v xml:space="preserve">Cheryl emailed to advise she is away for the September weekend 
 Eilidh 15/09/2025</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Sharon Jack (NL)</v>
-      </c>
-      <c r="B28" t="str">
-        <v>24</v>
-      </c>
-      <c r="C28" t="str">
-        <v>4.8</v>
-      </c>
-      <c r="D28" t="str">
-        <v>2025-09-23</v>
-      </c>
-      <c r="E28" t="str">
-        <v>Partial Availability</v>
-      </c>
-      <c r="F28" t="str">
-        <v>09:15-10:30; 12:30-16:15</v>
-      </c>
-      <c r="G28" t="str">
-        <v>2.8</v>
-      </c>
-      <c r="H28" t="str">
-        <v>2.8</v>
-      </c>
-      <c r="I28" t="str">
-        <v>Sharon has advised she is unable to work between 10.30 and 12.30 on Tuesday's - MT</v>
-      </c>
-    </row>
-    <row r="29" xml:space="preserve">
+    <row r="29">
       <c r="A29" t="str">
         <v>Sharon Jack (NL)</v>
       </c>
@@ -1236,13 +1236,13 @@
         <v>4.8</v>
       </c>
       <c r="D29" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E29" t="str">
         <v>Partial Availability</v>
       </c>
       <c r="F29" t="str">
-        <v>09:15-10:30; 12:30-17:15</v>
+        <v>09:15-10:30; 12:30-16:15</v>
       </c>
       <c r="G29" t="str">
         <v>2.8</v>
@@ -1250,38 +1250,38 @@
       <c r="H29" t="str">
         <v>2.8</v>
       </c>
-      <c r="I29" t="str" xml:space="preserve">
+      <c r="I29" t="str">
+        <v>Sharon has advised she is unable to work between 10.30 and 12.30 on Tuesday's - MT</v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>Sharon Jack (NL)</v>
+      </c>
+      <c r="B30" t="str">
+        <v>24</v>
+      </c>
+      <c r="C30" t="str">
+        <v>4.8</v>
+      </c>
+      <c r="D30" t="str">
+        <v>2025-09-24</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Partial Availability</v>
+      </c>
+      <c r="F30" t="str">
+        <v>09:15-10:30; 12:30-17:15</v>
+      </c>
+      <c r="G30" t="str">
+        <v>2.8</v>
+      </c>
+      <c r="H30" t="str">
+        <v>2.8</v>
+      </c>
+      <c r="I30" t="str" xml:space="preserve">
         <v xml:space="preserve">Wants this as a break. 
 Eilidh 29/05/2025</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
-      </c>
-      <c r="B30" t="str">
-        <v>16</v>
-      </c>
-      <c r="C30" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D30" t="str">
-        <v>2025-09-22</v>
-      </c>
-      <c r="E30" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F30" t="str">
-        <v>10:30-15:15</v>
-      </c>
-      <c r="G30" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H30" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I30" t="str">
-        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="31">
@@ -1295,13 +1295,13 @@
         <v>3.2</v>
       </c>
       <c r="D31" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E31" t="str">
         <v>Available</v>
       </c>
       <c r="F31" t="str">
-        <v>09:15-15:15; 20:30-21:30</v>
+        <v>10:30-15:15</v>
       </c>
       <c r="G31" t="str">
         <v>3.2</v>
@@ -1324,7 +1324,7 @@
         <v>3.2</v>
       </c>
       <c r="D32" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E32" t="str">
         <v>Available</v>
@@ -1353,7 +1353,7 @@
         <v>3.2</v>
       </c>
       <c r="D33" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E33" t="str">
         <v>Available</v>
@@ -1382,13 +1382,13 @@
         <v>3.2</v>
       </c>
       <c r="D34" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E34" t="str">
         <v>Available</v>
       </c>
       <c r="F34" t="str">
-        <v>10:30-14:00</v>
+        <v>09:15-15:15; 20:30-21:30</v>
       </c>
       <c r="G34" t="str">
         <v>3.2</v>
@@ -1402,31 +1402,31 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="B35" t="str">
         <v>16</v>
       </c>
       <c r="C35" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="D35" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-26</v>
       </c>
       <c r="E35" t="str">
         <v>Available</v>
       </c>
       <c r="F35" t="str">
-        <v>09:15-14:00</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="G35" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="H35" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="I35" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="36">
@@ -1440,7 +1440,7 @@
         <v>2.67</v>
       </c>
       <c r="D36" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E36" t="str">
         <v>Available</v>
@@ -1469,7 +1469,7 @@
         <v>2.67</v>
       </c>
       <c r="D37" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E37" t="str">
         <v>Available</v>
@@ -1498,7 +1498,7 @@
         <v>2.67</v>
       </c>
       <c r="D38" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E38" t="str">
         <v>Available</v>
@@ -1513,7 +1513,7 @@
         <v>2.67</v>
       </c>
       <c r="I38" t="str">
-        <v/>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="39">
@@ -1527,7 +1527,7 @@
         <v>2.67</v>
       </c>
       <c r="D39" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E39" t="str">
         <v>Available</v>
@@ -1556,13 +1556,13 @@
         <v>2.67</v>
       </c>
       <c r="D40" t="str">
-        <v>2025-09-27</v>
+        <v>2025-09-26</v>
       </c>
       <c r="E40" t="str">
         <v>Available</v>
       </c>
       <c r="F40" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G40" t="str">
         <v>2.67</v>
@@ -1576,31 +1576,31 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="B41" t="str">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C41" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="D41" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-27</v>
       </c>
       <c r="E41" t="str">
         <v>Available</v>
       </c>
       <c r="F41" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G41" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="H41" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="I41" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -1614,7 +1614,7 @@
         <v>4</v>
       </c>
       <c r="D42" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E42" t="str">
         <v>Available</v>
@@ -1643,7 +1643,7 @@
         <v>4</v>
       </c>
       <c r="D43" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E43" t="str">
         <v>Available</v>
@@ -1672,7 +1672,7 @@
         <v>4</v>
       </c>
       <c r="D44" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E44" t="str">
         <v>Available</v>
@@ -1701,7 +1701,7 @@
         <v>4</v>
       </c>
       <c r="D45" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E45" t="str">
         <v>Available</v>
@@ -1721,31 +1721,31 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="B46" t="str">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C46" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="D46" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-26</v>
       </c>
       <c r="E46" t="str">
         <v>Available</v>
       </c>
       <c r="F46" t="str">
-        <v>09:15-14:45</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G46" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="H46" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="I46" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="47">
@@ -1759,13 +1759,13 @@
         <v>2.8</v>
       </c>
       <c r="D47" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E47" t="str">
         <v>Available</v>
       </c>
       <c r="F47" t="str">
-        <v>09:15-11:30</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="G47" t="str">
         <v>2.8</v>
@@ -1788,13 +1788,13 @@
         <v>2.8</v>
       </c>
       <c r="D48" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E48" t="str">
         <v>Available</v>
       </c>
       <c r="F48" t="str">
-        <v>09:15-14:45</v>
+        <v>09:15-11:30</v>
       </c>
       <c r="G48" t="str">
         <v>2.8</v>
@@ -1803,7 +1803,7 @@
         <v>2.8</v>
       </c>
       <c r="I48" t="str">
-        <v/>
+        <v>Donna's daughter was sick on the way to school - MT</v>
       </c>
     </row>
     <row r="49">
@@ -1817,13 +1817,13 @@
         <v>2.8</v>
       </c>
       <c r="D49" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E49" t="str">
         <v>Available</v>
       </c>
       <c r="F49" t="str">
-        <v>09:15-11:30</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="G49" t="str">
         <v>2.8</v>
@@ -1846,13 +1846,13 @@
         <v>2.8</v>
       </c>
       <c r="D50" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E50" t="str">
         <v>Available</v>
       </c>
       <c r="F50" t="str">
-        <v>09:15-10:15</v>
+        <v>09:15-11:30</v>
       </c>
       <c r="G50" t="str">
         <v>2.8</v>
@@ -1866,31 +1866,31 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Emma Shawcross (NL)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="B51" t="str">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C51" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="D51" t="str">
-        <v>2025-09-27</v>
+        <v>2025-09-26</v>
       </c>
       <c r="E51" t="str">
         <v>Available</v>
       </c>
       <c r="F51" t="str">
-        <v>09:15-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G51" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="H51" t="str">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="I51" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="52">
@@ -1904,7 +1904,7 @@
         <v>10</v>
       </c>
       <c r="D52" t="str">
-        <v>2025-09-28</v>
+        <v>2025-09-27</v>
       </c>
       <c r="E52" t="str">
         <v>Available</v>
@@ -1924,31 +1924,31 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Emma Shawcross (NL)</v>
       </c>
       <c r="B53" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C53" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="D53" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-28</v>
       </c>
       <c r="E53" t="str">
         <v>Available</v>
       </c>
       <c r="F53" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-21:30</v>
       </c>
       <c r="G53" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="H53" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="I53" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="54">
@@ -1962,7 +1962,7 @@
         <v>7.5</v>
       </c>
       <c r="D54" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E54" t="str">
         <v>Available</v>
@@ -1991,7 +1991,7 @@
         <v>7.5</v>
       </c>
       <c r="D55" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E55" t="str">
         <v>Available</v>
@@ -2020,7 +2020,7 @@
         <v>7.5</v>
       </c>
       <c r="D56" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E56" t="str">
         <v>Available</v>
@@ -2040,28 +2040,28 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Kaitlyn Barton (NL) (GH)</v>
       </c>
       <c r="B57" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C57" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="D57" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-26</v>
       </c>
       <c r="E57" t="str">
         <v>Available</v>
       </c>
       <c r="F57" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G57" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="H57" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="I57" t="str">
         <v/>
@@ -2069,28 +2069,28 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="B58" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C58" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="D58" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E58" t="str">
         <v>Available</v>
       </c>
       <c r="F58" t="str">
-        <v>08:00-15:15</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G58" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="H58" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="I58" t="str">
         <v/>
@@ -2098,28 +2098,28 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="B59" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C59" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="D59" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E59" t="str">
         <v>Available</v>
       </c>
       <c r="F59" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G59" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="H59" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="I59" t="str">
         <v/>
@@ -2127,13 +2127,13 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="B60" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C60" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="D60" t="str">
         <v>2025-09-28</v>
@@ -2142,13 +2142,13 @@
         <v>Available</v>
       </c>
       <c r="F60" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G60" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="H60" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="I60" t="str">
         <v/>
@@ -2156,28 +2156,28 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Marykate Ferris (NL)</v>
+        <v>Shafiya Fayaz GH</v>
       </c>
       <c r="B61" t="str">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C61" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="D61" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E61" t="str">
         <v>Available</v>
       </c>
       <c r="F61" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G61" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="H61" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="I61" t="str">
         <v/>
@@ -2185,16 +2185,16 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Marykate Ferris (NL)</v>
+        <v>Shafiya Fayaz GH</v>
       </c>
       <c r="B62" t="str">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C62" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="D62" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E62" t="str">
         <v>Available</v>
@@ -2203,10 +2203,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G62" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="H62" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="I62" t="str">
         <v/>
@@ -2214,16 +2214,16 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Marykate Ferris (NL)</v>
+        <v>Shafiya Fayaz GH</v>
       </c>
       <c r="B63" t="str">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C63" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="D63" t="str">
-        <v>2025-09-28</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E63" t="str">
         <v>Available</v>
@@ -2232,10 +2232,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G63" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="H63" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="I63" t="str">
         <v/>
@@ -2252,7 +2252,7 @@
         <v>9</v>
       </c>
       <c r="D64" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-26</v>
       </c>
       <c r="E64" t="str">
         <v>Available</v>
@@ -2281,7 +2281,7 @@
         <v>9</v>
       </c>
       <c r="D65" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-27</v>
       </c>
       <c r="E65" t="str">
         <v>Available</v>
@@ -2301,16 +2301,16 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Shafiya Fayaz GH</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="B66" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C66" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="D66" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E66" t="str">
         <v>Available</v>
@@ -2319,10 +2319,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G66" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H66" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="I66" t="str">
         <v/>
@@ -2330,28 +2330,28 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Shafiya Fayaz GH</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="B67" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C67" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="D67" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E67" t="str">
         <v>Available</v>
       </c>
       <c r="F67" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:15</v>
       </c>
       <c r="G67" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H67" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="I67" t="str">
         <v/>
@@ -2359,13 +2359,13 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Shafiya Fayaz GH</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="B68" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C68" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="D68" t="str">
         <v>2025-09-27</v>
@@ -2377,10 +2377,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G68" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="H68" t="str">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="I68" t="str">
         <v/>
@@ -2397,7 +2397,7 @@
         <v>7.5</v>
       </c>
       <c r="D69" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-28</v>
       </c>
       <c r="E69" t="str">
         <v>Available</v>
@@ -2417,7 +2417,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
+        <v>Adedayo Adeyanju (NL) (GH)</v>
       </c>
       <c r="B70" t="str">
         <v>30</v>
@@ -2426,13 +2426,13 @@
         <v>7.5</v>
       </c>
       <c r="D70" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E70" t="str">
         <v>Available</v>
       </c>
       <c r="F70" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G70" t="str">
         <v>7.5</v>
@@ -2446,7 +2446,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
+        <v>Adedayo Adeyanju (NL) (GH)</v>
       </c>
       <c r="B71" t="str">
         <v>30</v>
@@ -2455,7 +2455,7 @@
         <v>7.5</v>
       </c>
       <c r="D71" t="str">
-        <v>2025-09-27</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E71" t="str">
         <v>Available</v>
@@ -2475,7 +2475,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
+        <v>Adedayo Adeyanju (NL) (GH)</v>
       </c>
       <c r="B72" t="str">
         <v>30</v>
@@ -2484,7 +2484,7 @@
         <v>7.5</v>
       </c>
       <c r="D72" t="str">
-        <v>2025-09-28</v>
+        <v>2025-09-27</v>
       </c>
       <c r="E72" t="str">
         <v>Available</v>
@@ -2513,7 +2513,7 @@
         <v>7.5</v>
       </c>
       <c r="D73" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-28</v>
       </c>
       <c r="E73" t="str">
         <v>Available</v>
@@ -2533,16 +2533,16 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Adedayo Adeyanju (NL) (GH)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="B74" t="str">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C74" t="str">
         <v>7.5</v>
       </c>
       <c r="D74" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-26</v>
       </c>
       <c r="E74" t="str">
         <v>Available</v>
@@ -2562,16 +2562,16 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Adedayo Adeyanju (NL) (GH)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="B75" t="str">
         <v>30</v>
       </c>
       <c r="C75" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D75" t="str">
-        <v>2025-09-27</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E75" t="str">
         <v>Available</v>
@@ -2580,10 +2580,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G75" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H75" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="I75" t="str">
         <v/>
@@ -2591,16 +2591,16 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Adedayo Adeyanju (NL) (GH)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="B76" t="str">
         <v>30</v>
       </c>
       <c r="C76" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D76" t="str">
-        <v>2025-09-28</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E76" t="str">
         <v>Available</v>
@@ -2609,10 +2609,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G76" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H76" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="I76" t="str">
         <v/>
@@ -2620,16 +2620,16 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="B77" t="str">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C77" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D77" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E77" t="str">
         <v>Available</v>
@@ -2638,10 +2638,10 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G77" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H77" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="I77" t="str">
         <v/>
@@ -2658,7 +2658,7 @@
         <v>6</v>
       </c>
       <c r="D78" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-26</v>
       </c>
       <c r="E78" t="str">
         <v>Available</v>
@@ -2687,7 +2687,7 @@
         <v>6</v>
       </c>
       <c r="D79" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-27</v>
       </c>
       <c r="E79" t="str">
         <v>Available</v>
@@ -2707,89 +2707,89 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="B80" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C80" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D80" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E80" t="str">
         <v>Available</v>
       </c>
       <c r="F80" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G80" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H80" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I80" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="B81" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C81" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D81" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E81" t="str">
         <v>Available</v>
       </c>
       <c r="F81" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G81" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H81" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I81" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="B82" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C82" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D82" t="str">
-        <v>2025-09-27</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E82" t="str">
         <v>Available</v>
       </c>
       <c r="F82" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G82" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H82" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I82" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="83">
@@ -2803,7 +2803,7 @@
         <v>3.2</v>
       </c>
       <c r="D83" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E83" t="str">
         <v>Available</v>
@@ -2832,7 +2832,7 @@
         <v>3.2</v>
       </c>
       <c r="D84" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-26</v>
       </c>
       <c r="E84" t="str">
         <v>Available</v>
@@ -2852,89 +2852,89 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="B85" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C85" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="D85" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E85" t="str">
         <v>Available</v>
       </c>
       <c r="F85" t="str">
-        <v>09:15-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G85" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H85" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="I85" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="B86" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C86" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="D86" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E86" t="str">
         <v>Available</v>
       </c>
       <c r="F86" t="str">
-        <v>09:15-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G86" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H86" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="I86" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="B87" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C87" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="D87" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E87" t="str">
         <v>Available</v>
       </c>
       <c r="F87" t="str">
-        <v>09:15-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G87" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H87" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="I87" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="88">
@@ -2948,7 +2948,7 @@
         <v>6</v>
       </c>
       <c r="D88" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E88" t="str">
         <v>Available</v>
@@ -2977,7 +2977,7 @@
         <v>6</v>
       </c>
       <c r="D89" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-28</v>
       </c>
       <c r="E89" t="str">
         <v>Available</v>
@@ -2997,28 +2997,28 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="B90" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C90" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D90" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E90" t="str">
         <v>Available</v>
       </c>
       <c r="F90" t="str">
-        <v>08:00-21:30</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G90" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H90" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I90" t="str">
         <v/>
@@ -3026,28 +3026,28 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="B91" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C91" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D91" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E91" t="str">
         <v>Available</v>
       </c>
       <c r="F91" t="str">
-        <v>08:00-21:30</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G91" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H91" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I91" t="str">
         <v/>
@@ -3055,28 +3055,28 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="B92" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C92" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="D92" t="str">
-        <v>2025-09-28</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E92" t="str">
         <v>Available</v>
       </c>
       <c r="F92" t="str">
-        <v>08:00-21:30</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G92" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H92" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="I92" t="str">
         <v/>
@@ -3093,7 +3093,7 @@
         <v>3.2</v>
       </c>
       <c r="D93" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E93" t="str">
         <v>Available</v>
@@ -3113,28 +3113,28 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="B94" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C94" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="D94" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E94" t="str">
         <v>Available</v>
       </c>
       <c r="F94" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="G94" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="H94" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="I94" t="str">
         <v/>
@@ -3142,28 +3142,28 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="B95" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C95" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="D95" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E95" t="str">
         <v>Available</v>
       </c>
       <c r="F95" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="G95" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="H95" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="I95" t="str">
         <v/>
@@ -3171,28 +3171,28 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="B96" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C96" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="D96" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-26</v>
       </c>
       <c r="E96" t="str">
         <v>Available</v>
       </c>
       <c r="F96" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="G96" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="H96" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="I96" t="str">
         <v/>
@@ -3200,28 +3200,28 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Sharon Jack (NL)</v>
       </c>
       <c r="B97" t="str">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C97" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="D97" t="str">
-        <v>2025-09-23</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E97" t="str">
         <v>Available</v>
       </c>
       <c r="F97" t="str">
-        <v>08:00-15:00</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G97" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="H97" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="I97" t="str">
         <v/>
@@ -3229,28 +3229,28 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Sharon Jack (NL)</v>
       </c>
       <c r="B98" t="str">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C98" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="D98" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-25</v>
       </c>
       <c r="E98" t="str">
         <v>Available</v>
       </c>
       <c r="F98" t="str">
-        <v>08:00-15:00</v>
+        <v>09:15-16:15</v>
       </c>
       <c r="G98" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="H98" t="str">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="I98" t="str">
         <v/>
@@ -3258,57 +3258,57 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="B99" t="str">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C99" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D99" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-22</v>
       </c>
       <c r="E99" t="str">
         <v>Available</v>
       </c>
       <c r="F99" t="str">
-        <v>08:00-15:00</v>
+        <v>09:15-15:15; 16:45-21:30</v>
       </c>
       <c r="G99" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H99" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I99" t="str">
-        <v/>
+        <v>Lori has agreed to extend her availability via email on 02/04/2025 - MT</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="B100" t="str">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C100" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D100" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-23</v>
       </c>
       <c r="E100" t="str">
         <v>Available</v>
       </c>
       <c r="F100" t="str">
-        <v>08:00-15:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G100" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H100" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I100" t="str">
         <v/>
@@ -3316,28 +3316,28 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="B101" t="str">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C101" t="str">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="D101" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-24</v>
       </c>
       <c r="E101" t="str">
         <v>Available</v>
       </c>
       <c r="F101" t="str">
-        <v>09:15-10:15</v>
+        <v>09:15-17:45</v>
       </c>
       <c r="G101" t="str">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="H101" t="str">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="I101" t="str">
         <v/>
@@ -3345,13 +3345,13 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="B102" t="str">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C102" t="str">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="D102" t="str">
         <v>2025-09-25</v>
@@ -3360,13 +3360,13 @@
         <v>Available</v>
       </c>
       <c r="F102" t="str">
-        <v>09:15-16:15</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G102" t="str">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="H102" t="str">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="I102" t="str">
         <v/>
@@ -3383,13 +3383,13 @@
         <v>6</v>
       </c>
       <c r="D103" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-26</v>
       </c>
       <c r="E103" t="str">
         <v>Available</v>
       </c>
       <c r="F103" t="str">
-        <v>09:15-15:15; 16:45-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G103" t="str">
         <v>6</v>
@@ -3398,128 +3398,12 @@
         <v>6</v>
       </c>
       <c r="I103" t="str">
-        <v>Lori has agreed to extend her availability via email on 02/04/2025 - MT</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="str">
-        <v>Lori Wylie (NL)</v>
-      </c>
-      <c r="B104" t="str">
-        <v>30</v>
-      </c>
-      <c r="C104" t="str">
-        <v>6</v>
-      </c>
-      <c r="D104" t="str">
-        <v>2025-09-23</v>
-      </c>
-      <c r="E104" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F104" t="str">
-        <v>09:15-15:15</v>
-      </c>
-      <c r="G104" t="str">
-        <v>6</v>
-      </c>
-      <c r="H104" t="str">
-        <v>6</v>
-      </c>
-      <c r="I104" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="str">
-        <v>Lori Wylie (NL)</v>
-      </c>
-      <c r="B105" t="str">
-        <v>30</v>
-      </c>
-      <c r="C105" t="str">
-        <v>6</v>
-      </c>
-      <c r="D105" t="str">
-        <v>2025-09-24</v>
-      </c>
-      <c r="E105" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F105" t="str">
-        <v>09:15-17:45</v>
-      </c>
-      <c r="G105" t="str">
-        <v>6</v>
-      </c>
-      <c r="H105" t="str">
-        <v>6</v>
-      </c>
-      <c r="I105" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="str">
-        <v>Lori Wylie (NL)</v>
-      </c>
-      <c r="B106" t="str">
-        <v>30</v>
-      </c>
-      <c r="C106" t="str">
-        <v>6</v>
-      </c>
-      <c r="D106" t="str">
-        <v>2025-09-25</v>
-      </c>
-      <c r="E106" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F106" t="str">
-        <v>09:15-14:00</v>
-      </c>
-      <c r="G106" t="str">
-        <v>6</v>
-      </c>
-      <c r="H106" t="str">
-        <v>6</v>
-      </c>
-      <c r="I106" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="str">
-        <v>Lori Wylie (NL)</v>
-      </c>
-      <c r="B107" t="str">
-        <v>30</v>
-      </c>
-      <c r="C107" t="str">
-        <v>6</v>
-      </c>
-      <c r="D107" t="str">
-        <v>2025-09-26</v>
-      </c>
-      <c r="E107" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F107" t="str">
-        <v>09:15-14:00</v>
-      </c>
-      <c r="G107" t="str">
-        <v>6</v>
-      </c>
-      <c r="H107" t="str">
-        <v>6</v>
-      </c>
-      <c r="I107" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I107"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I103"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3571,10 +3455,10 @@
         <v>8</v>
       </c>
       <c r="F2" t="str">
-        <v>64.5</v>
+        <v>65.5</v>
       </c>
       <c r="G2" t="str">
-        <v>-7.63</v>
+        <v>-8.63</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -3585,22 +3469,22 @@
         <v>2025-09-23</v>
       </c>
       <c r="B3" t="str">
-        <v>72.57</v>
+        <v>68.57</v>
       </c>
       <c r="C3" t="str">
-        <v>75.37</v>
+        <v>71.37</v>
       </c>
       <c r="D3" t="str">
-        <v>20.09</v>
+        <v>24.09</v>
       </c>
       <c r="E3" t="str">
         <v>8</v>
       </c>
       <c r="F3" t="str">
-        <v>55.25</v>
+        <v>52.75</v>
       </c>
       <c r="G3" t="str">
-        <v>20.12</v>
+        <v>18.62</v>
       </c>
       <c r="H3" t="str">
         <v>Sufficient</v>
@@ -3611,10 +3495,10 @@
         <v>2025-09-24</v>
       </c>
       <c r="B4" t="str">
-        <v>68.24</v>
+        <v>64.24</v>
       </c>
       <c r="C4" t="str">
-        <v>71.04</v>
+        <v>67.04</v>
       </c>
       <c r="D4" t="str">
         <v>20.09</v>
@@ -3623,10 +3507,10 @@
         <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>63.5</v>
+        <v>62.5</v>
       </c>
       <c r="G4" t="str">
-        <v>7.54</v>
+        <v>4.54</v>
       </c>
       <c r="H4" t="str">
         <v>Sufficient</v>
@@ -3637,10 +3521,10 @@
         <v>2025-09-25</v>
       </c>
       <c r="B5" t="str">
-        <v>67.04</v>
+        <v>63.04</v>
       </c>
       <c r="C5" t="str">
-        <v>67.04</v>
+        <v>63.04</v>
       </c>
       <c r="D5" t="str">
         <v>17.29</v>
@@ -3649,10 +3533,10 @@
         <v>4</v>
       </c>
       <c r="F5" t="str">
-        <v>54.5</v>
+        <v>56.5</v>
       </c>
       <c r="G5" t="str">
-        <v>12.54</v>
+        <v>6.54</v>
       </c>
       <c r="H5" t="str">
         <v>Sufficient</v>
@@ -3663,10 +3547,10 @@
         <v>2025-09-26</v>
       </c>
       <c r="B6" t="str">
-        <v>59.87</v>
+        <v>55.87</v>
       </c>
       <c r="C6" t="str">
-        <v>59.87</v>
+        <v>55.87</v>
       </c>
       <c r="D6" t="str">
         <v>12.99</v>
@@ -3675,10 +3559,10 @@
         <v>8.8</v>
       </c>
       <c r="F6" t="str">
-        <v>48.5</v>
+        <v>54.5</v>
       </c>
       <c r="G6" t="str">
-        <v>11.37</v>
+        <v>1.37</v>
       </c>
       <c r="H6" t="str">
         <v>Sufficient</v>
@@ -3701,10 +3585,10 @@
         <v>4</v>
       </c>
       <c r="F7" t="str">
-        <v>37.75</v>
+        <v>34.75</v>
       </c>
       <c r="G7" t="str">
-        <v>4.92</v>
+        <v>7.92</v>
       </c>
       <c r="H7" t="str">
         <v>Sufficient</v>
@@ -3715,10 +3599,10 @@
         <v>2025-09-28</v>
       </c>
       <c r="B8" t="str">
-        <v>41.67</v>
+        <v>37.67</v>
       </c>
       <c r="C8" t="str">
-        <v>41.67</v>
+        <v>37.67</v>
       </c>
       <c r="D8" t="str">
         <v>9.79</v>
@@ -3727,10 +3611,10 @@
         <v>4</v>
       </c>
       <c r="F8" t="str">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G8" t="str">
-        <v>6.67</v>
+        <v>4.67</v>
       </c>
       <c r="H8" t="str">
         <v>Sufficient</v>
@@ -3745,7 +3629,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H107"/>
+  <dimension ref="A1:H103"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3979,7 +3863,7 @@
         <v>2.8</v>
       </c>
       <c r="H9" t="str">
-        <v/>
+        <v>Donna's daughter was sick on the way to school - MT</v>
       </c>
     </row>
     <row r="10">
@@ -4068,10 +3952,10 @@
         <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="C13" t="str">
-        <v>Available</v>
+        <v>Sick</v>
       </c>
       <c r="D13" t="str">
-        <v>08:00-15:00</v>
+        <v/>
       </c>
       <c r="E13" t="str">
         <v>4</v>
@@ -4080,10 +3964,10 @@
         <v>4</v>
       </c>
       <c r="G13" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H13" t="str">
-        <v/>
+        <v>Sciatica flare up - MT [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="14">
@@ -4560,22 +4444,22 @@
         <v>2025-09-24</v>
       </c>
       <c r="B32" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="C32" t="str">
         <v>Available</v>
       </c>
       <c r="D32" t="str">
-        <v>08:00-15:15</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E32" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="F32" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="G32" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="H32" t="str">
         <v/>
@@ -4586,22 +4470,22 @@
         <v>2025-09-24</v>
       </c>
       <c r="B33" t="str">
-        <v>Marykate Ferris (NL)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="C33" t="str">
         <v>Available</v>
       </c>
       <c r="D33" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E33" t="str">
-        <v>6.67</v>
+        <v>6</v>
       </c>
       <c r="F33" t="str">
-        <v>6.67</v>
+        <v>6</v>
       </c>
       <c r="G33" t="str">
-        <v>6.67</v>
+        <v>6</v>
       </c>
       <c r="H33" t="str">
         <v/>
@@ -4612,25 +4496,25 @@
         <v>2025-09-24</v>
       </c>
       <c r="B34" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="C34" t="str">
         <v>Available</v>
       </c>
       <c r="D34" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E34" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="F34" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="G34" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H34" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="35">
@@ -4638,104 +4522,104 @@
         <v>2025-09-24</v>
       </c>
       <c r="B35" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Shafiya Fayaz GH</v>
       </c>
       <c r="C35" t="str">
         <v>Available</v>
       </c>
       <c r="D35" t="str">
-        <v>09:15-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E35" t="str">
-        <v>3.2</v>
+        <v>9</v>
       </c>
       <c r="F35" t="str">
-        <v>3.2</v>
+        <v>9</v>
       </c>
       <c r="G35" t="str">
-        <v>3.2</v>
+        <v>9</v>
       </c>
       <c r="H35" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
-      </c>
-    </row>
-    <row r="36">
+        <v/>
+      </c>
+    </row>
+    <row r="36" xml:space="preserve">
       <c r="A36" t="str">
         <v>2025-09-24</v>
       </c>
       <c r="B36" t="str">
-        <v>Shafiya Fayaz GH</v>
+        <v>Sharon Jack (NL)</v>
       </c>
       <c r="C36" t="str">
-        <v>Available</v>
+        <v>Partial Availability</v>
       </c>
       <c r="D36" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:30; 12:30-17:15</v>
       </c>
       <c r="E36" t="str">
-        <v>9</v>
+        <v>4.8</v>
       </c>
       <c r="F36" t="str">
-        <v>9</v>
+        <v>2.8</v>
       </c>
       <c r="G36" t="str">
-        <v>9</v>
-      </c>
-      <c r="H36" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="37" xml:space="preserve">
+        <v>2.8</v>
+      </c>
+      <c r="H36" t="str" xml:space="preserve">
+        <v xml:space="preserve">Wants this as a break. 
+Eilidh 29/05/2025</v>
+      </c>
+    </row>
+    <row r="37">
       <c r="A37" t="str">
         <v>2025-09-24</v>
       </c>
       <c r="B37" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="C37" t="str">
-        <v>Partial Availability</v>
+        <v>Available</v>
       </c>
       <c r="D37" t="str">
-        <v>09:15-10:30; 12:30-17:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E37" t="str">
-        <v>4.8</v>
+        <v>6</v>
       </c>
       <c r="F37" t="str">
-        <v>2.8</v>
+        <v>6</v>
       </c>
       <c r="G37" t="str">
-        <v>2.8</v>
-      </c>
-      <c r="H37" t="str" xml:space="preserve">
-        <v xml:space="preserve">Wants this as a break. 
-Eilidh 29/05/2025</v>
+        <v>6</v>
+      </c>
+      <c r="H37" t="str">
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2025-09-24</v>
+        <v>2025-09-25</v>
       </c>
       <c r="B38" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="C38" t="str">
         <v>Available</v>
       </c>
       <c r="D38" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:15; 20:30-21:30</v>
       </c>
       <c r="E38" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="F38" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="G38" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H38" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="39">
@@ -4743,25 +4627,25 @@
         <v>2025-09-25</v>
       </c>
       <c r="B39" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
+        <v>Anne Nelson (NL)</v>
       </c>
       <c r="C39" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D39" t="str">
-        <v>09:15-15:15; 20:30-21:30</v>
+        <v/>
       </c>
       <c r="E39" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="F39" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="G39" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H39" t="str">
-        <v>Confirmed at induction with MT</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="40">
@@ -4769,33 +4653,33 @@
         <v>2025-09-25</v>
       </c>
       <c r="B40" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C40" t="str">
-        <v>Holiday</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D40" t="str">
         <v/>
       </c>
       <c r="E40" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="F40" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="G40" t="str">
         <v>0</v>
       </c>
       <c r="H40" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
-      </c>
-    </row>
-    <row r="41">
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
+      </c>
+    </row>
+    <row r="41" xml:space="preserve">
       <c r="A41" t="str">
         <v>2025-09-25</v>
       </c>
       <c r="B41" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
+        <v>Ayoola Ajibade (GH) (NL)</v>
       </c>
       <c r="C41" t="str">
         <v>Maternity/Paternity</v>
@@ -4804,43 +4688,43 @@
         <v/>
       </c>
       <c r="E41" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="F41" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="G41" t="str">
         <v>0</v>
       </c>
-      <c r="H41" t="str">
-        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
-      </c>
-    </row>
-    <row r="42" xml:space="preserve">
+      <c r="H41" t="str" xml:space="preserve">
+        <v xml:space="preserve">Morning sickness
+Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
+      </c>
+    </row>
+    <row r="42">
       <c r="A42" t="str">
         <v>2025-09-25</v>
       </c>
       <c r="B42" t="str">
-        <v>Ayoola Ajibade (GH) (NL)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C42" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D42" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E42" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="F42" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="G42" t="str">
-        <v>0</v>
-      </c>
-      <c r="H42" t="str" xml:space="preserve">
-        <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
+        <v>2.67</v>
+      </c>
+      <c r="H42" t="str">
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -4848,22 +4732,22 @@
         <v>2025-09-25</v>
       </c>
       <c r="B43" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="C43" t="str">
         <v>Available</v>
       </c>
       <c r="D43" t="str">
-        <v>09:15-14:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E43" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="F43" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="G43" t="str">
-        <v>2.67</v>
+        <v>3.2</v>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -4874,25 +4758,25 @@
         <v>2025-09-25</v>
       </c>
       <c r="B44" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="C44" t="str">
         <v>Available</v>
       </c>
       <c r="D44" t="str">
-        <v>16:45-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E44" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="F44" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="G44" t="str">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="H44" t="str">
-        <v/>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="45">
@@ -4900,25 +4784,25 @@
         <v>2025-09-25</v>
       </c>
       <c r="B45" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="C45" t="str">
         <v>Available</v>
       </c>
       <c r="D45" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-11:30</v>
       </c>
       <c r="E45" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="F45" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="G45" t="str">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="H45" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -4926,22 +4810,22 @@
         <v>2025-09-25</v>
       </c>
       <c r="B46" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="C46" t="str">
-        <v>Available</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D46" t="str">
-        <v>09:15-11:30</v>
+        <v/>
       </c>
       <c r="E46" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="F46" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="G46" t="str">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="H46" t="str">
         <v/>
@@ -4952,13 +4836,13 @@
         <v>2025-09-25</v>
       </c>
       <c r="B47" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Kaitlyn Barton (NL) (GH)</v>
       </c>
       <c r="C47" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D47" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E47" t="str">
         <v>7.5</v>
@@ -4967,7 +4851,7 @@
         <v>7.5</v>
       </c>
       <c r="G47" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H47" t="str">
         <v/>
@@ -4978,22 +4862,22 @@
         <v>2025-09-25</v>
       </c>
       <c r="B48" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="C48" t="str">
         <v>Available</v>
       </c>
       <c r="D48" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E48" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F48" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G48" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H48" t="str">
         <v/>
@@ -5004,22 +4888,22 @@
         <v>2025-09-25</v>
       </c>
       <c r="B49" t="str">
-        <v>Lori Wylie (NL)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="C49" t="str">
         <v>Available</v>
       </c>
       <c r="D49" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E49" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F49" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G49" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H49" t="str">
         <v/>
@@ -5030,22 +4914,22 @@
         <v>2025-09-25</v>
       </c>
       <c r="B50" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="C50" t="str">
         <v>Available</v>
       </c>
       <c r="D50" t="str">
-        <v>08:00-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E50" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="F50" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="G50" t="str">
-        <v>4</v>
+        <v>6.67</v>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -5056,25 +4940,25 @@
         <v>2025-09-25</v>
       </c>
       <c r="B51" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="C51" t="str">
         <v>Available</v>
       </c>
       <c r="D51" t="str">
-        <v>08:00-15:15</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E51" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="F51" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="G51" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="H51" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="52">
@@ -5082,7 +4966,7 @@
         <v>2025-09-25</v>
       </c>
       <c r="B52" t="str">
-        <v>Marykate Ferris (NL)</v>
+        <v>Shafiya Fayaz GH</v>
       </c>
       <c r="C52" t="str">
         <v>Available</v>
@@ -5091,13 +4975,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E52" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="F52" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="G52" t="str">
-        <v>6.67</v>
+        <v>9</v>
       </c>
       <c r="H52" t="str">
         <v/>
@@ -5108,25 +4992,25 @@
         <v>2025-09-25</v>
       </c>
       <c r="B53" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Sharon Jack (NL)</v>
       </c>
       <c r="C53" t="str">
         <v>Available</v>
       </c>
       <c r="D53" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-16:15</v>
       </c>
       <c r="E53" t="str">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="F53" t="str">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="G53" t="str">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="H53" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="54">
@@ -5134,7 +5018,7 @@
         <v>2025-09-25</v>
       </c>
       <c r="B54" t="str">
-        <v>Shafiya Fayaz GH</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="C54" t="str">
         <v>Available</v>
@@ -5143,13 +5027,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E54" t="str">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F54" t="str">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G54" t="str">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="H54" t="str">
         <v/>
@@ -5157,54 +5041,54 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-26</v>
       </c>
       <c r="B55" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="C55" t="str">
         <v>Available</v>
       </c>
       <c r="D55" t="str">
-        <v>09:15-16:15</v>
+        <v>10:30-14:00</v>
       </c>
       <c r="E55" t="str">
-        <v>4.8</v>
+        <v>3.2</v>
       </c>
       <c r="F55" t="str">
-        <v>4.8</v>
+        <v>3.2</v>
       </c>
       <c r="G55" t="str">
-        <v>4.8</v>
+        <v>3.2</v>
       </c>
       <c r="H55" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2025-09-25</v>
+        <v>2025-09-26</v>
       </c>
       <c r="B56" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Anne Nelson (NL)</v>
       </c>
       <c r="C56" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D56" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E56" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F56" t="str">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G56" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H56" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="57">
@@ -5212,51 +5096,52 @@
         <v>2025-09-26</v>
       </c>
       <c r="B57" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C57" t="str">
-        <v>Available</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D57" t="str">
-        <v>10:30-14:00</v>
+        <v/>
       </c>
       <c r="E57" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="F57" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="G57" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H57" t="str">
-        <v>Confirmed at induction with MT</v>
-      </c>
-    </row>
-    <row r="58">
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
+      </c>
+    </row>
+    <row r="58" xml:space="preserve">
       <c r="A58" t="str">
         <v>2025-09-26</v>
       </c>
       <c r="B58" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Ayoola Ajibade (GH) (NL)</v>
       </c>
       <c r="C58" t="str">
-        <v>Holiday</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D58" t="str">
         <v/>
       </c>
       <c r="E58" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="F58" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="G58" t="str">
         <v>0</v>
       </c>
-      <c r="H58" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+      <c r="H58" t="str" xml:space="preserve">
+        <v xml:space="preserve">Morning sickness
+Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="59">
@@ -5264,25 +5149,25 @@
         <v>2025-09-26</v>
       </c>
       <c r="B59" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C59" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D59" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E59" t="str">
-        <v>2.29</v>
+        <v>2.67</v>
       </c>
       <c r="F59" t="str">
-        <v>2.29</v>
+        <v>2.67</v>
       </c>
       <c r="G59" t="str">
-        <v>0</v>
+        <v>2.67</v>
       </c>
       <c r="H59" t="str">
-        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="60" xml:space="preserve">
@@ -5290,26 +5175,26 @@
         <v>2025-09-26</v>
       </c>
       <c r="B60" t="str">
-        <v>Ayoola Ajibade (GH) (NL)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="C60" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D60" t="str">
         <v/>
       </c>
       <c r="E60" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="F60" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="G60" t="str">
         <v>0</v>
       </c>
       <c r="H60" t="str" xml:space="preserve">
-        <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
+        <v xml:space="preserve">Cheryl emailed to advise she is away for the September weekend 
+Eilidh 15/09/2025</v>
       </c>
     </row>
     <row r="61">
@@ -5317,7 +5202,7 @@
         <v>2025-09-26</v>
       </c>
       <c r="B61" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="C61" t="str">
         <v>Available</v>
@@ -5326,43 +5211,42 @@
         <v>09:15-14:00</v>
       </c>
       <c r="E61" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="F61" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="G61" t="str">
-        <v>2.67</v>
+        <v>4</v>
       </c>
       <c r="H61" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="62" xml:space="preserve">
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+      </c>
+    </row>
+    <row r="62">
       <c r="A62" t="str">
         <v>2025-09-26</v>
       </c>
       <c r="B62" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="C62" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D62" t="str">
-        <v/>
+        <v>09:15-10:15</v>
       </c>
       <c r="E62" t="str">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="F62" t="str">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="G62" t="str">
-        <v>0</v>
-      </c>
-      <c r="H62" t="str" xml:space="preserve">
-        <v xml:space="preserve">Cheryl emailed to advise she is away for the September weekend 
-Eilidh 15/09/2025</v>
+        <v>2.8</v>
+      </c>
+      <c r="H62" t="str">
+        <v/>
       </c>
     </row>
     <row r="63">
@@ -5370,25 +5254,25 @@
         <v>2025-09-26</v>
       </c>
       <c r="B63" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="C63" t="str">
         <v>Available</v>
       </c>
       <c r="D63" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E63" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="F63" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="G63" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="H63" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v/>
       </c>
     </row>
     <row r="64">
@@ -5396,22 +5280,22 @@
         <v>2025-09-26</v>
       </c>
       <c r="B64" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Kaitlyn Barton (NL) (GH)</v>
       </c>
       <c r="C64" t="str">
         <v>Available</v>
       </c>
       <c r="D64" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E64" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="F64" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="G64" t="str">
-        <v>2.8</v>
+        <v>7.5</v>
       </c>
       <c r="H64" t="str">
         <v/>
@@ -5422,22 +5306,22 @@
         <v>2025-09-26</v>
       </c>
       <c r="B65" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="C65" t="str">
         <v>Available</v>
       </c>
       <c r="D65" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E65" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F65" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G65" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="H65" t="str">
         <v/>
@@ -5448,22 +5332,22 @@
         <v>2025-09-26</v>
       </c>
       <c r="B66" t="str">
-        <v>Kaitlyn Barton (NL) (GH)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="C66" t="str">
         <v>Available</v>
       </c>
       <c r="D66" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:00</v>
       </c>
       <c r="E66" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="F66" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="G66" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="H66" t="str">
         <v/>
@@ -5474,13 +5358,13 @@
         <v>2025-09-26</v>
       </c>
       <c r="B67" t="str">
-        <v>Lori Wylie (NL)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="C67" t="str">
         <v>Available</v>
       </c>
       <c r="D67" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E67" t="str">
         <v>6</v>
@@ -5500,25 +5384,25 @@
         <v>2025-09-26</v>
       </c>
       <c r="B68" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="C68" t="str">
         <v>Available</v>
       </c>
       <c r="D68" t="str">
-        <v>08:00-15:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E68" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="F68" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="G68" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="H68" t="str">
-        <v/>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="69">
@@ -5526,144 +5410,144 @@
         <v>2025-09-26</v>
       </c>
       <c r="B69" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
+        <v>Shafiya Fayaz GH</v>
       </c>
       <c r="C69" t="str">
         <v>Available</v>
       </c>
       <c r="D69" t="str">
-        <v>08:00-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E69" t="str">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F69" t="str">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G69" t="str">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H69" t="str">
         <v/>
       </c>
     </row>
-    <row r="70">
+    <row r="70" xml:space="preserve">
       <c r="A70" t="str">
         <v>2025-09-26</v>
       </c>
       <c r="B70" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Sharon Jack (NL)</v>
       </c>
       <c r="C70" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D70" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E70" t="str">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="F70" t="str">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="G70" t="str">
-        <v>6</v>
-      </c>
-      <c r="H70" t="str">
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="H70" t="str" xml:space="preserve">
+        <v xml:space="preserve">Created by new vacation process.; Wants this as a break. 
+Eilidh 29/05/2025 [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-27</v>
       </c>
       <c r="B71" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Adedayo Adeyanju (NL) (GH)</v>
       </c>
       <c r="C71" t="str">
         <v>Available</v>
       </c>
       <c r="D71" t="str">
-        <v>09:15-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E71" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F71" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G71" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H71" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-27</v>
       </c>
       <c r="B72" t="str">
-        <v>Shafiya Fayaz GH</v>
+        <v>Anne Nelson (NL)</v>
       </c>
       <c r="C72" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D72" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E72" t="str">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F72" t="str">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G72" t="str">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H72" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="73" xml:space="preserve">
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+      </c>
+    </row>
+    <row r="73">
       <c r="A73" t="str">
-        <v>2025-09-26</v>
+        <v>2025-09-27</v>
       </c>
       <c r="B73" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C73" t="str">
-        <v>Holiday</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D73" t="str">
         <v/>
       </c>
       <c r="E73" t="str">
-        <v>4.8</v>
+        <v>2.29</v>
       </c>
       <c r="F73" t="str">
-        <v>4.8</v>
+        <v>2.29</v>
       </c>
       <c r="G73" t="str">
         <v>0</v>
       </c>
-      <c r="H73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Created by new vacation process.; Wants this as a break. 
-Eilidh 29/05/2025 [availability ignored due to day-level leave]</v>
-      </c>
-    </row>
-    <row r="74">
+      <c r="H73" t="str">
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
+      </c>
+    </row>
+    <row r="74" xml:space="preserve">
       <c r="A74" t="str">
         <v>2025-09-27</v>
       </c>
       <c r="B74" t="str">
-        <v>Adedayo Adeyanju (NL) (GH)</v>
+        <v>Ayoola Ajibade (GH) (NL)</v>
       </c>
       <c r="C74" t="str">
-        <v>Available</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D74" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E74" t="str">
         <v>7.5</v>
@@ -5672,10 +5556,11 @@
         <v>7.5</v>
       </c>
       <c r="G74" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H74" t="str">
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="H74" t="str" xml:space="preserve">
+        <v xml:space="preserve">Morning sickness
+Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="75">
@@ -5683,25 +5568,25 @@
         <v>2025-09-27</v>
       </c>
       <c r="B75" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C75" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D75" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E75" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="F75" t="str">
-        <v>4</v>
+        <v>2.67</v>
       </c>
       <c r="G75" t="str">
-        <v>0</v>
+        <v>2.67</v>
       </c>
       <c r="H75" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="76">
@@ -5709,52 +5594,51 @@
         <v>2025-09-27</v>
       </c>
       <c r="B76" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
+        <v>Emma Shawcross (NL)</v>
       </c>
       <c r="C76" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D76" t="str">
-        <v/>
+        <v>09:15-21:30</v>
       </c>
       <c r="E76" t="str">
-        <v>2.29</v>
+        <v>10</v>
       </c>
       <c r="F76" t="str">
-        <v>2.29</v>
+        <v>10</v>
       </c>
       <c r="G76" t="str">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H76" t="str">
-        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
-      </c>
-    </row>
-    <row r="77" xml:space="preserve">
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+      </c>
+    </row>
+    <row r="77">
       <c r="A77" t="str">
         <v>2025-09-27</v>
       </c>
       <c r="B77" t="str">
-        <v>Ayoola Ajibade (GH) (NL)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="C77" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D77" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E77" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F77" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G77" t="str">
-        <v>0</v>
-      </c>
-      <c r="H77" t="str" xml:space="preserve">
-        <v xml:space="preserve">Morning sickness
-Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
+        <v>6</v>
+      </c>
+      <c r="H77" t="str">
+        <v/>
       </c>
     </row>
     <row r="78">
@@ -5762,7 +5646,7 @@
         <v>2025-09-27</v>
       </c>
       <c r="B78" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Shafiya Fayaz GH</v>
       </c>
       <c r="C78" t="str">
         <v>Available</v>
@@ -5771,13 +5655,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E78" t="str">
-        <v>2.67</v>
+        <v>9</v>
       </c>
       <c r="F78" t="str">
-        <v>2.67</v>
+        <v>9</v>
       </c>
       <c r="G78" t="str">
-        <v>2.67</v>
+        <v>9</v>
       </c>
       <c r="H78" t="str">
         <v/>
@@ -5788,33 +5672,33 @@
         <v>2025-09-27</v>
       </c>
       <c r="B79" t="str">
-        <v>Emma Shawcross (NL)</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="C79" t="str">
         <v>Available</v>
       </c>
       <c r="D79" t="str">
-        <v>09:15-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E79" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="F79" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="G79" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="H79" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2025-09-27</v>
+        <v>2025-09-22</v>
       </c>
       <c r="B80" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Adedayo Adeyanju (NL) (GH)</v>
       </c>
       <c r="C80" t="str">
         <v>Available</v>
@@ -5823,13 +5707,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E80" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="F80" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="G80" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="H80" t="str">
         <v/>
@@ -5837,54 +5721,54 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2025-09-27</v>
+        <v>2025-09-22</v>
       </c>
       <c r="B81" t="str">
-        <v>Shafiya Fayaz GH</v>
+        <v>Amanda Forbes (NL) (GH)</v>
       </c>
       <c r="C81" t="str">
         <v>Available</v>
       </c>
       <c r="D81" t="str">
-        <v>08:00-21:30</v>
+        <v>10:30-15:15</v>
       </c>
       <c r="E81" t="str">
-        <v>9</v>
+        <v>3.2</v>
       </c>
       <c r="F81" t="str">
-        <v>9</v>
+        <v>3.2</v>
       </c>
       <c r="G81" t="str">
-        <v>9</v>
+        <v>3.2</v>
       </c>
       <c r="H81" t="str">
-        <v/>
+        <v>Confirmed at induction with MT</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2025-09-27</v>
+        <v>2025-09-22</v>
       </c>
       <c r="B82" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C82" t="str">
-        <v>Available</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D82" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E82" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="F82" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="G82" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H82" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="83">
@@ -5892,25 +5776,25 @@
         <v>2025-09-22</v>
       </c>
       <c r="B83" t="str">
-        <v>Adedayo Adeyanju (NL) (GH)</v>
+        <v>Brooke O'Brien (NL) (GH)</v>
       </c>
       <c r="C83" t="str">
         <v>Available</v>
       </c>
       <c r="D83" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E83" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="F83" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="G83" t="str">
-        <v>7.5</v>
+        <v>2.67</v>
       </c>
       <c r="H83" t="str">
-        <v/>
+        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
     </row>
     <row r="84">
@@ -5918,13 +5802,13 @@
         <v>2025-09-22</v>
       </c>
       <c r="B84" t="str">
-        <v>Amanda Forbes (NL) (GH)</v>
+        <v>Cheryl McGhie (NL) (GH)</v>
       </c>
       <c r="C84" t="str">
         <v>Available</v>
       </c>
       <c r="D84" t="str">
-        <v>10:30-15:15</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E84" t="str">
         <v>3.2</v>
@@ -5936,7 +5820,7 @@
         <v>3.2</v>
       </c>
       <c r="H84" t="str">
-        <v>Confirmed at induction with MT</v>
+        <v/>
       </c>
     </row>
     <row r="85">
@@ -5944,25 +5828,25 @@
         <v>2025-09-22</v>
       </c>
       <c r="B85" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
+        <v>Deborah Asokhia (NL)</v>
       </c>
       <c r="C85" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D85" t="str">
-        <v/>
+        <v>09:15-14:00</v>
       </c>
       <c r="E85" t="str">
-        <v>2.29</v>
+        <v>4</v>
       </c>
       <c r="F85" t="str">
-        <v>2.29</v>
+        <v>4</v>
       </c>
       <c r="G85" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H85" t="str">
-        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
+        <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
     </row>
     <row r="86">
@@ -5970,25 +5854,25 @@
         <v>2025-09-22</v>
       </c>
       <c r="B86" t="str">
-        <v>Brooke O'Brien (NL) (GH)</v>
+        <v>Donna Gabillard (NL)</v>
       </c>
       <c r="C86" t="str">
         <v>Available</v>
       </c>
       <c r="D86" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-14:45</v>
       </c>
       <c r="E86" t="str">
-        <v>2.67</v>
+        <v>2.8</v>
       </c>
       <c r="F86" t="str">
-        <v>2.67</v>
+        <v>2.8</v>
       </c>
       <c r="G86" t="str">
-        <v>2.67</v>
+        <v>2.8</v>
       </c>
       <c r="H86" t="str">
-        <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="87">
@@ -5996,22 +5880,22 @@
         <v>2025-09-22</v>
       </c>
       <c r="B87" t="str">
-        <v>Cheryl McGhie (NL) (GH)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="C87" t="str">
-        <v>Available</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D87" t="str">
-        <v>16:45-21:30</v>
+        <v/>
       </c>
       <c r="E87" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F87" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G87" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H87" t="str">
         <v/>
@@ -6022,25 +5906,25 @@
         <v>2025-09-22</v>
       </c>
       <c r="B88" t="str">
-        <v>Deborah Asokhia (NL)</v>
+        <v>Lori Wylie (NL)</v>
       </c>
       <c r="C88" t="str">
         <v>Available</v>
       </c>
       <c r="D88" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-15:15; 16:45-21:30</v>
       </c>
       <c r="E88" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F88" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G88" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H88" t="str">
-        <v>Agreed at induction with MT and SM - 09/05/2025</v>
+        <v>Lori has agreed to extend her availability via email on 02/04/2025 - MT</v>
       </c>
     </row>
     <row r="89">
@@ -6048,25 +5932,25 @@
         <v>2025-09-22</v>
       </c>
       <c r="B89" t="str">
-        <v>Donna Gabillard (NL)</v>
+        <v>Lynsey (GH) Mooney (NL)</v>
       </c>
       <c r="C89" t="str">
-        <v>Available</v>
+        <v>Sick</v>
       </c>
       <c r="D89" t="str">
-        <v>09:15-14:45</v>
+        <v/>
       </c>
       <c r="E89" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="F89" t="str">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="G89" t="str">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="H89" t="str">
-        <v/>
+        <v>Sciatica flare up - MT [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="90">
@@ -6074,25 +5958,25 @@
         <v>2025-09-22</v>
       </c>
       <c r="B90" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Madison Duncan (NL)</v>
       </c>
       <c r="C90" t="str">
-        <v>Other Unavailable</v>
+        <v>Holiday</v>
       </c>
       <c r="D90" t="str">
         <v/>
       </c>
       <c r="E90" t="str">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="F90" t="str">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="G90" t="str">
         <v>0</v>
       </c>
       <c r="H90" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="91">
@@ -6100,13 +5984,13 @@
         <v>2025-09-22</v>
       </c>
       <c r="B91" t="str">
-        <v>Lori Wylie (NL)</v>
+        <v>Mustansar Hussain (NL) (GH)</v>
       </c>
       <c r="C91" t="str">
         <v>Available</v>
       </c>
       <c r="D91" t="str">
-        <v>09:15-15:15; 16:45-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E91" t="str">
         <v>6</v>
@@ -6118,7 +6002,7 @@
         <v>6</v>
       </c>
       <c r="H91" t="str">
-        <v>Lori has agreed to extend her availability via email on 02/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="92">
@@ -6126,25 +6010,25 @@
         <v>2025-09-22</v>
       </c>
       <c r="B92" t="str">
-        <v>Lynsey (GH) Mooney (NL)</v>
+        <v>Olusegun Isaac Ibrahim (NL)</v>
       </c>
       <c r="C92" t="str">
-        <v>Sick</v>
+        <v>Available</v>
       </c>
       <c r="D92" t="str">
-        <v/>
+        <v>09:15-15:15</v>
       </c>
       <c r="E92" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="F92" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="G92" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H92" t="str">
-        <v>Sciatica flare up - MT [availability ignored due to day-level leave]</v>
+        <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
     </row>
     <row r="93">
@@ -6152,25 +6036,25 @@
         <v>2025-09-22</v>
       </c>
       <c r="B93" t="str">
-        <v>Madison Duncan (NL)</v>
+        <v>Sharon Jack (NL)</v>
       </c>
       <c r="C93" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D93" t="str">
-        <v/>
+        <v>09:15-10:15</v>
       </c>
       <c r="E93" t="str">
-        <v>8</v>
+        <v>4.8</v>
       </c>
       <c r="F93" t="str">
-        <v>8</v>
+        <v>4.8</v>
       </c>
       <c r="G93" t="str">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="H93" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="94">
@@ -6178,7 +6062,7 @@
         <v>2025-09-22</v>
       </c>
       <c r="B94" t="str">
-        <v>Mustansar Hussain (NL) (GH)</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="C94" t="str">
         <v>Available</v>
@@ -6187,13 +6071,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E94" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="F94" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="G94" t="str">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="H94" t="str">
         <v/>
@@ -6204,48 +6088,48 @@
         <v>2025-09-22</v>
       </c>
       <c r="B95" t="str">
-        <v>Olusegun Isaac Ibrahim (NL)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="C95" t="str">
         <v>Available</v>
       </c>
       <c r="D95" t="str">
-        <v>09:15-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E95" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="F95" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="G95" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H95" t="str">
-        <v>Agreed at induction with SM 25/04/2025 - MT</v>
+        <v/>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-28</v>
       </c>
       <c r="B96" t="str">
-        <v>Sharon Jack (NL)</v>
+        <v>Adedayo Adeyanju (NL) (GH)</v>
       </c>
       <c r="C96" t="str">
         <v>Available</v>
       </c>
       <c r="D96" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E96" t="str">
-        <v>4.8</v>
+        <v>7.5</v>
       </c>
       <c r="F96" t="str">
-        <v>4.8</v>
+        <v>7.5</v>
       </c>
       <c r="G96" t="str">
-        <v>4.8</v>
+        <v>7.5</v>
       </c>
       <c r="H96" t="str">
         <v/>
@@ -6253,54 +6137,54 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-28</v>
       </c>
       <c r="B97" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
+        <v>Anne Nelson (NL)</v>
       </c>
       <c r="C97" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D97" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E97" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="F97" t="str">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="G97" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H97" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>2025-09-22</v>
+        <v>2025-09-28</v>
       </c>
       <c r="B98" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
+        <v>Ashleigh Graham (GH) (NL)</v>
       </c>
       <c r="C98" t="str">
-        <v>Available</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D98" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E98" t="str">
-        <v>6</v>
+        <v>2.29</v>
       </c>
       <c r="F98" t="str">
-        <v>6</v>
+        <v>2.29</v>
       </c>
       <c r="G98" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H98" t="str">
-        <v/>
+        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="99">
@@ -6308,25 +6192,25 @@
         <v>2025-09-28</v>
       </c>
       <c r="B99" t="str">
-        <v>Adedayo Adeyanju (NL) (GH)</v>
+        <v>Emma Shawcross (NL)</v>
       </c>
       <c r="C99" t="str">
         <v>Available</v>
       </c>
       <c r="D99" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-21:30</v>
       </c>
       <c r="E99" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="F99" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="G99" t="str">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="H99" t="str">
-        <v/>
+        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
     </row>
     <row r="100">
@@ -6334,25 +6218,25 @@
         <v>2025-09-28</v>
       </c>
       <c r="B100" t="str">
-        <v>Anne Nelson (NL)</v>
+        <v>Hamza Nafees (NL) (GH)</v>
       </c>
       <c r="C100" t="str">
-        <v>Holiday</v>
+        <v>Other Unavailable</v>
       </c>
       <c r="D100" t="str">
         <v/>
       </c>
       <c r="E100" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="F100" t="str">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="G100" t="str">
         <v>0</v>
       </c>
       <c r="H100" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="101">
@@ -6360,25 +6244,25 @@
         <v>2025-09-28</v>
       </c>
       <c r="B101" t="str">
-        <v>Ashleigh Graham (GH) (NL)</v>
+        <v>Marykate Ferris (NL)</v>
       </c>
       <c r="C101" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D101" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E101" t="str">
-        <v>2.29</v>
+        <v>6.67</v>
       </c>
       <c r="F101" t="str">
-        <v>2.29</v>
+        <v>6.67</v>
       </c>
       <c r="G101" t="str">
-        <v>0</v>
+        <v>6.67</v>
       </c>
       <c r="H101" t="str">
-        <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="102">
@@ -6386,25 +6270,25 @@
         <v>2025-09-28</v>
       </c>
       <c r="B102" t="str">
-        <v>Emma Shawcross (NL)</v>
+        <v>Sophie Lamont (NL) (GH)</v>
       </c>
       <c r="C102" t="str">
         <v>Available</v>
       </c>
       <c r="D102" t="str">
-        <v>09:15-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E102" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="F102" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="G102" t="str">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="H102" t="str">
-        <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
+        <v/>
       </c>
     </row>
     <row r="103">
@@ -6412,134 +6296,30 @@
         <v>2025-09-28</v>
       </c>
       <c r="B103" t="str">
-        <v>Hamza Nafees (NL) (GH)</v>
+        <v>Wayne (GH) Griffiths (NL)</v>
       </c>
       <c r="C103" t="str">
-        <v>Other Unavailable</v>
+        <v>Available</v>
       </c>
       <c r="D103" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E103" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="F103" t="str">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="G103" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H103" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="str">
-        <v>2025-09-28</v>
-      </c>
-      <c r="B104" t="str">
-        <v>Makala Mcewan (NL) (GH)</v>
-      </c>
-      <c r="C104" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D104" t="str">
-        <v>08:00-15:15</v>
-      </c>
-      <c r="E104" t="str">
-        <v>4</v>
-      </c>
-      <c r="F104" t="str">
-        <v>4</v>
-      </c>
-      <c r="G104" t="str">
-        <v>4</v>
-      </c>
-      <c r="H104" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="str">
-        <v>2025-09-28</v>
-      </c>
-      <c r="B105" t="str">
-        <v>Marykate Ferris (NL)</v>
-      </c>
-      <c r="C105" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D105" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E105" t="str">
-        <v>6.67</v>
-      </c>
-      <c r="F105" t="str">
-        <v>6.67</v>
-      </c>
-      <c r="G105" t="str">
-        <v>6.67</v>
-      </c>
-      <c r="H105" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="str">
-        <v>2025-09-28</v>
-      </c>
-      <c r="B106" t="str">
-        <v>Sophie Lamont (NL) (GH)</v>
-      </c>
-      <c r="C106" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D106" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E106" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="F106" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="G106" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H106" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="str">
-        <v>2025-09-28</v>
-      </c>
-      <c r="B107" t="str">
-        <v>Wayne (GH) Griffiths (NL)</v>
-      </c>
-      <c r="C107" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D107" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E107" t="str">
-        <v>6</v>
-      </c>
-      <c r="F107" t="str">
-        <v>6</v>
-      </c>
-      <c r="G107" t="str">
-        <v>6</v>
-      </c>
-      <c r="H107" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H107"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H103"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add post code information to the exported employee data
Includes the addition of a 'Post Code' column to the cleaned employee records and the Excel export, sourcing data from the CG Data file to map employee names to their respective post codes.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 363bae44-e195-49b5-807e-5e99a74dd028
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/363bae44-e195-49b5-807e-5e99a74dd028/wxVIgG1
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -6,6 +6,7 @@
     <sheet name="Cleaned" sheetId="1" r:id="rId1"/>
     <sheet name="DailySummary" sheetId="2" r:id="rId2"/>
     <sheet name="EmployeeDailyDetail" sheetId="3" r:id="rId3"/>
+    <sheet name="EmployeeMasterList" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -6322,4 +6323,475 @@
     <ignoredError numberStoredAsText="1" sqref="A1:H103"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F23"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Employee Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Weekly Hours</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Transport Mode</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Title</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Gender</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Post Code</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Adedayo Adeyanju (NL) (GH)</v>
+      </c>
+      <c r="B2" t="str">
+        <v>30</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Mr</v>
+      </c>
+      <c r="E2" t="str">
+        <v>male</v>
+      </c>
+      <c r="F2" t="str">
+        <v xml:space="preserve">ML1 3YG   </v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Ayoola Ajibade (GH) (NL)</v>
+      </c>
+      <c r="B3" t="str">
+        <v>37.5</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E3" t="str">
+        <v>female</v>
+      </c>
+      <c r="F3" t="str">
+        <v xml:space="preserve">G34 9QA   </v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Deborah Asokhia (NL)</v>
+      </c>
+      <c r="B4" t="str">
+        <v>20</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Walker</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E4" t="str">
+        <v>female</v>
+      </c>
+      <c r="F4" t="str">
+        <v xml:space="preserve">G67 2QH   </v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Kaitlyn Barton (NL) (GH)</v>
+      </c>
+      <c r="B5" t="str">
+        <v>30</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E5" t="str">
+        <v>female</v>
+      </c>
+      <c r="F5" t="str">
+        <v xml:space="preserve">G67 2DT   </v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Madison Duncan (NL)</v>
+      </c>
+      <c r="B6" t="str">
+        <v>16</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E6" t="str">
+        <v>female</v>
+      </c>
+      <c r="F6" t="str">
+        <v xml:space="preserve">ML5 5TG   </v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Shafiya Fayaz GH</v>
+      </c>
+      <c r="B7" t="str">
+        <v>45</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E7" t="str">
+        <v>female</v>
+      </c>
+      <c r="F7" t="str">
+        <v xml:space="preserve">G42 8NR   </v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Marykate Ferris (NL)</v>
+      </c>
+      <c r="B8" t="str">
+        <v>20</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Walker</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E8" t="str">
+        <v>female</v>
+      </c>
+      <c r="F8" t="str">
+        <v xml:space="preserve">G67 2BS   </v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Amanda Forbes (NL) (GH)</v>
+      </c>
+      <c r="B9" t="str">
+        <v>16</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E9" t="str">
+        <v>female</v>
+      </c>
+      <c r="F9" t="str">
+        <v xml:space="preserve">G69 9FS   </v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Donna Gabillard (NL)</v>
+      </c>
+      <c r="B10" t="str">
+        <v>14</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E10" t="str">
+        <v>female</v>
+      </c>
+      <c r="F10" t="str">
+        <v xml:space="preserve">ML6 7UN   </v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Ashleigh Graham (GH) (NL)</v>
+      </c>
+      <c r="B11" t="str">
+        <v>16</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Mrs</v>
+      </c>
+      <c r="E11" t="str">
+        <v>female</v>
+      </c>
+      <c r="F11" t="str">
+        <v xml:space="preserve">FK4 1LQ   </v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Wayne (GH) Griffiths (NL)</v>
+      </c>
+      <c r="B12" t="str">
+        <v>30</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Mr</v>
+      </c>
+      <c r="E12" t="str">
+        <v>male</v>
+      </c>
+      <c r="F12" t="str">
+        <v xml:space="preserve">ML6 8UX   </v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Mustansar Hussain (NL) (GH)</v>
+      </c>
+      <c r="B13" t="str">
+        <v>30</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Mr</v>
+      </c>
+      <c r="E13" t="str">
+        <v>male</v>
+      </c>
+      <c r="F13" t="str">
+        <v xml:space="preserve">G51 2TJ   </v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Olusegun Isaac Ibrahim (NL)</v>
+      </c>
+      <c r="B14" t="str">
+        <v>16</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Mr</v>
+      </c>
+      <c r="E14" t="str">
+        <v>male</v>
+      </c>
+      <c r="F14" t="str">
+        <v xml:space="preserve">G67 2LE   </v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Sharon Jack (NL)</v>
+      </c>
+      <c r="B15" t="str">
+        <v>24</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Mrs</v>
+      </c>
+      <c r="E15" t="str">
+        <v>female</v>
+      </c>
+      <c r="F15" t="str">
+        <v xml:space="preserve">G33 2AF   </v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Sophie Lamont (NL) (GH)</v>
+      </c>
+      <c r="B16" t="str">
+        <v>30</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E16" t="str">
+        <v>female</v>
+      </c>
+      <c r="F16" t="str">
+        <v xml:space="preserve">G67 3JS   </v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Cheryl McGhie (NL) (GH)</v>
+      </c>
+      <c r="B17" t="str">
+        <v>16</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Mrs</v>
+      </c>
+      <c r="E17" t="str">
+        <v>female</v>
+      </c>
+      <c r="F17" t="str">
+        <v xml:space="preserve">G67 1JE   </v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Lynsey (GH) Mooney (NL)</v>
+      </c>
+      <c r="B18" t="str">
+        <v>20</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Mrs</v>
+      </c>
+      <c r="E18" t="str">
+        <v>female</v>
+      </c>
+      <c r="F18" t="str">
+        <v xml:space="preserve">G67 3NR   </v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Hamza Nafees (NL) (GH)</v>
+      </c>
+      <c r="B19" t="str">
+        <v>45</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Mr</v>
+      </c>
+      <c r="E19" t="str">
+        <v>male</v>
+      </c>
+      <c r="F19" t="str">
+        <v xml:space="preserve">ML3 9RN   </v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Anne Nelson (NL)</v>
+      </c>
+      <c r="B20" t="str">
+        <v>16</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Mrs</v>
+      </c>
+      <c r="E20" t="str">
+        <v>female</v>
+      </c>
+      <c r="F20" t="str">
+        <v xml:space="preserve">ML6 9TY   </v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Brooke O'Brien (NL) (GH)</v>
+      </c>
+      <c r="B21" t="str">
+        <v>16</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E21" t="str">
+        <v>female</v>
+      </c>
+      <c r="F21" t="str">
+        <v xml:space="preserve">G67 1LL   </v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Emma Shawcross (NL)</v>
+      </c>
+      <c r="B22" t="str">
+        <v>20</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Walker</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E22" t="str">
+        <v>female</v>
+      </c>
+      <c r="F22" t="str">
+        <v xml:space="preserve">ML6 0JH   </v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Lori Wylie (NL)</v>
+      </c>
+      <c r="B23" t="str">
+        <v>30</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Ms</v>
+      </c>
+      <c r="E23" t="str">
+        <v>female</v>
+      </c>
+      <c r="F23" t="str">
+        <v xml:space="preserve">G68 9GH   </v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F23"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Include postcode information in the exported employee data
Add the 'Post Code' column to the 'Cleaned' sheet in the exported Excel file to include employee postcode information.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 363bae44-e195-49b5-807e-5e99a74dd028
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/363bae44-e195-49b5-807e-5e99a74dd028/wxVIgG1
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I103"/>
+  <dimension ref="A1:J103"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -435,6 +435,9 @@
       <c r="I1" t="str">
         <v>Notes</v>
       </c>
+      <c r="J1" t="str">
+        <v>Post Code</v>
+      </c>
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
@@ -465,6 +468,9 @@
         <v xml:space="preserve">Morning sickness
 Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J2" t="str">
+        <v xml:space="preserve">G34 9QA   </v>
+      </c>
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
@@ -495,6 +501,9 @@
         <v xml:space="preserve">Morning sickness
 Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J3" t="str">
+        <v xml:space="preserve">G34 9QA   </v>
+      </c>
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4" t="str">
@@ -525,6 +534,9 @@
         <v xml:space="preserve">Morning sickness
 Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J4" t="str">
+        <v xml:space="preserve">G34 9QA   </v>
+      </c>
     </row>
     <row r="5" xml:space="preserve">
       <c r="A5" t="str">
@@ -555,6 +567,9 @@
         <v xml:space="preserve">Morning sickness
 Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J5" t="str">
+        <v xml:space="preserve">G34 9QA   </v>
+      </c>
     </row>
     <row r="6" xml:space="preserve">
       <c r="A6" t="str">
@@ -585,6 +600,9 @@
         <v xml:space="preserve">Morning sickness
 Eilidh 31/03/2025 [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J6" t="str">
+        <v xml:space="preserve">G34 9QA   </v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -614,6 +632,9 @@
       <c r="I7" t="str">
         <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J7" t="str">
+        <v xml:space="preserve">FK4 1LQ   </v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -643,6 +664,9 @@
       <c r="I8" t="str">
         <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J8" t="str">
+        <v xml:space="preserve">FK4 1LQ   </v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -672,6 +696,9 @@
       <c r="I9" t="str">
         <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J9" t="str">
+        <v xml:space="preserve">FK4 1LQ   </v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -701,6 +728,9 @@
       <c r="I10" t="str">
         <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J10" t="str">
+        <v xml:space="preserve">FK4 1LQ   </v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -730,6 +760,9 @@
       <c r="I11" t="str">
         <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J11" t="str">
+        <v xml:space="preserve">FK4 1LQ   </v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -759,6 +792,9 @@
       <c r="I12" t="str">
         <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J12" t="str">
+        <v xml:space="preserve">FK4 1LQ   </v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -788,6 +824,9 @@
       <c r="I13" t="str">
         <v xml:space="preserve"> [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J13" t="str">
+        <v xml:space="preserve">FK4 1LQ   </v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -817,6 +856,9 @@
       <c r="I14" t="str">
         <v>Sciatica flare up - MT [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J14" t="str">
+        <v xml:space="preserve">G67 3NR   </v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -846,6 +888,9 @@
       <c r="I15" t="str">
         <v>Sciatica flare up - MT [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J15" t="str">
+        <v xml:space="preserve">G67 3NR   </v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -875,6 +920,9 @@
       <c r="I16" t="str">
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J16" t="str">
+        <v xml:space="preserve">ML5 5TG   </v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -904,6 +952,9 @@
       <c r="I17" t="str">
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J17" t="str">
+        <v xml:space="preserve">ML5 5TG   </v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -933,6 +984,9 @@
       <c r="I18" t="str">
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J18" t="str">
+        <v xml:space="preserve">ML6 9TY   </v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -962,6 +1016,9 @@
       <c r="I19" t="str">
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J19" t="str">
+        <v xml:space="preserve">ML6 9TY   </v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -991,6 +1048,9 @@
       <c r="I20" t="str">
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J20" t="str">
+        <v xml:space="preserve">ML6 9TY   </v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1020,6 +1080,9 @@
       <c r="I21" t="str">
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J21" t="str">
+        <v xml:space="preserve">ML6 9TY   </v>
+      </c>
     </row>
     <row r="22" xml:space="preserve">
       <c r="A22" t="str">
@@ -1050,6 +1113,9 @@
         <v xml:space="preserve">Created by new vacation process.; Wants this as a break. 
 Eilidh 29/05/2025 [availability ignored due to day-level leave]</v>
       </c>
+      <c r="J22" t="str">
+        <v xml:space="preserve">G33 2AF   </v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1079,6 +1145,9 @@
       <c r="I23" t="str">
         <v/>
       </c>
+      <c r="J23" t="str">
+        <v xml:space="preserve">ML3 9RN   </v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1108,6 +1177,9 @@
       <c r="I24" t="str">
         <v/>
       </c>
+      <c r="J24" t="str">
+        <v xml:space="preserve">ML3 9RN   </v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1137,6 +1209,9 @@
       <c r="I25" t="str">
         <v/>
       </c>
+      <c r="J25" t="str">
+        <v xml:space="preserve">ML3 9RN   </v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1166,6 +1241,9 @@
       <c r="I26" t="str">
         <v/>
       </c>
+      <c r="J26" t="str">
+        <v xml:space="preserve">ML3 9RN   </v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1195,6 +1273,9 @@
       <c r="I27" t="str">
         <v/>
       </c>
+      <c r="J27" t="str">
+        <v xml:space="preserve">ML3 9RN   </v>
+      </c>
     </row>
     <row r="28" xml:space="preserve">
       <c r="A28" t="str">
@@ -1225,6 +1306,9 @@
         <v xml:space="preserve">Cheryl emailed to advise she is away for the September weekend 
 Eilidh 15/09/2025</v>
       </c>
+      <c r="J28" t="str">
+        <v xml:space="preserve">G67 1JE   </v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1254,6 +1338,9 @@
       <c r="I29" t="str">
         <v>Sharon has advised she is unable to work between 10.30 and 12.30 on Tuesday's - MT</v>
       </c>
+      <c r="J29" t="str">
+        <v xml:space="preserve">G33 2AF   </v>
+      </c>
     </row>
     <row r="30" xml:space="preserve">
       <c r="A30" t="str">
@@ -1284,6 +1371,9 @@
         <v xml:space="preserve">Wants this as a break. 
 Eilidh 29/05/2025</v>
       </c>
+      <c r="J30" t="str">
+        <v xml:space="preserve">G33 2AF   </v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1313,6 +1403,9 @@
       <c r="I31" t="str">
         <v>Confirmed at induction with MT</v>
       </c>
+      <c r="J31" t="str">
+        <v xml:space="preserve">G69 9FS   </v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1342,6 +1435,9 @@
       <c r="I32" t="str">
         <v>Confirmed at induction with MT</v>
       </c>
+      <c r="J32" t="str">
+        <v xml:space="preserve">G69 9FS   </v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1371,6 +1467,9 @@
       <c r="I33" t="str">
         <v>Confirmed at induction with MT</v>
       </c>
+      <c r="J33" t="str">
+        <v xml:space="preserve">G69 9FS   </v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1400,6 +1499,9 @@
       <c r="I34" t="str">
         <v>Confirmed at induction with MT</v>
       </c>
+      <c r="J34" t="str">
+        <v xml:space="preserve">G69 9FS   </v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1429,6 +1531,9 @@
       <c r="I35" t="str">
         <v>Confirmed at induction with MT</v>
       </c>
+      <c r="J35" t="str">
+        <v xml:space="preserve">G69 9FS   </v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1458,6 +1563,9 @@
       <c r="I36" t="str">
         <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
+      <c r="J36" t="str">
+        <v xml:space="preserve">G67 1LL   </v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -1487,6 +1595,9 @@
       <c r="I37" t="str">
         <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
+      <c r="J37" t="str">
+        <v xml:space="preserve">G67 1LL   </v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -1516,6 +1627,9 @@
       <c r="I38" t="str">
         <v>Increased availability to 09.15am starts on Monday, Tuesday and Wednesday as of Monday 28/04 - MT</v>
       </c>
+      <c r="J38" t="str">
+        <v xml:space="preserve">G67 1LL   </v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1545,6 +1659,9 @@
       <c r="I39" t="str">
         <v/>
       </c>
+      <c r="J39" t="str">
+        <v xml:space="preserve">G67 1LL   </v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1574,6 +1691,9 @@
       <c r="I40" t="str">
         <v/>
       </c>
+      <c r="J40" t="str">
+        <v xml:space="preserve">G67 1LL   </v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1603,6 +1723,9 @@
       <c r="I41" t="str">
         <v/>
       </c>
+      <c r="J41" t="str">
+        <v xml:space="preserve">G67 1LL   </v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -1632,6 +1755,9 @@
       <c r="I42" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
+      <c r="J42" t="str">
+        <v xml:space="preserve">G67 2QH   </v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -1661,6 +1787,9 @@
       <c r="I43" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
+      <c r="J43" t="str">
+        <v xml:space="preserve">G67 2QH   </v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -1690,6 +1819,9 @@
       <c r="I44" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
+      <c r="J44" t="str">
+        <v xml:space="preserve">G67 2QH   </v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -1719,6 +1851,9 @@
       <c r="I45" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
+      <c r="J45" t="str">
+        <v xml:space="preserve">G67 2QH   </v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -1748,6 +1883,9 @@
       <c r="I46" t="str">
         <v>Agreed at induction with MT and SM - 09/05/2025</v>
       </c>
+      <c r="J46" t="str">
+        <v xml:space="preserve">G67 2QH   </v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -1777,6 +1915,9 @@
       <c r="I47" t="str">
         <v/>
       </c>
+      <c r="J47" t="str">
+        <v xml:space="preserve">ML6 7UN   </v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -1806,6 +1947,9 @@
       <c r="I48" t="str">
         <v>Donna's daughter was sick on the way to school - MT</v>
       </c>
+      <c r="J48" t="str">
+        <v xml:space="preserve">ML6 7UN   </v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -1835,6 +1979,9 @@
       <c r="I49" t="str">
         <v/>
       </c>
+      <c r="J49" t="str">
+        <v xml:space="preserve">ML6 7UN   </v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -1864,6 +2011,9 @@
       <c r="I50" t="str">
         <v/>
       </c>
+      <c r="J50" t="str">
+        <v xml:space="preserve">ML6 7UN   </v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -1893,6 +2043,9 @@
       <c r="I51" t="str">
         <v/>
       </c>
+      <c r="J51" t="str">
+        <v xml:space="preserve">ML6 7UN   </v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -1922,6 +2075,9 @@
       <c r="I52" t="str">
         <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
+      <c r="J52" t="str">
+        <v xml:space="preserve">ML6 0JH   </v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -1951,6 +2107,9 @@
       <c r="I53" t="str">
         <v>Can only do Airdrie and Coatbridge clients on a Sunday - MT</v>
       </c>
+      <c r="J53" t="str">
+        <v xml:space="preserve">ML6 0JH   </v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -1980,6 +2139,9 @@
       <c r="I54" t="str">
         <v/>
       </c>
+      <c r="J54" t="str">
+        <v xml:space="preserve">G67 2DT   </v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -2009,6 +2171,9 @@
       <c r="I55" t="str">
         <v/>
       </c>
+      <c r="J55" t="str">
+        <v xml:space="preserve">G67 2DT   </v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -2038,6 +2203,9 @@
       <c r="I56" t="str">
         <v/>
       </c>
+      <c r="J56" t="str">
+        <v xml:space="preserve">G67 2DT   </v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -2067,6 +2235,9 @@
       <c r="I57" t="str">
         <v/>
       </c>
+      <c r="J57" t="str">
+        <v xml:space="preserve">G67 2DT   </v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -2096,6 +2267,9 @@
       <c r="I58" t="str">
         <v/>
       </c>
+      <c r="J58" t="str">
+        <v xml:space="preserve">G67 2BS   </v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -2125,6 +2299,9 @@
       <c r="I59" t="str">
         <v/>
       </c>
+      <c r="J59" t="str">
+        <v xml:space="preserve">G67 2BS   </v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -2154,6 +2331,9 @@
       <c r="I60" t="str">
         <v/>
       </c>
+      <c r="J60" t="str">
+        <v xml:space="preserve">G67 2BS   </v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -2183,6 +2363,9 @@
       <c r="I61" t="str">
         <v/>
       </c>
+      <c r="J61" t="str">
+        <v xml:space="preserve">G42 8NR   </v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -2212,6 +2395,9 @@
       <c r="I62" t="str">
         <v/>
       </c>
+      <c r="J62" t="str">
+        <v xml:space="preserve">G42 8NR   </v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -2241,6 +2427,9 @@
       <c r="I63" t="str">
         <v/>
       </c>
+      <c r="J63" t="str">
+        <v xml:space="preserve">G42 8NR   </v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -2270,6 +2459,9 @@
       <c r="I64" t="str">
         <v/>
       </c>
+      <c r="J64" t="str">
+        <v xml:space="preserve">G42 8NR   </v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -2299,6 +2491,9 @@
       <c r="I65" t="str">
         <v/>
       </c>
+      <c r="J65" t="str">
+        <v xml:space="preserve">G42 8NR   </v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -2328,6 +2523,9 @@
       <c r="I66" t="str">
         <v/>
       </c>
+      <c r="J66" t="str">
+        <v xml:space="preserve">G67 3JS   </v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -2357,6 +2555,9 @@
       <c r="I67" t="str">
         <v/>
       </c>
+      <c r="J67" t="str">
+        <v xml:space="preserve">G67 3JS   </v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -2386,6 +2587,9 @@
       <c r="I68" t="str">
         <v/>
       </c>
+      <c r="J68" t="str">
+        <v xml:space="preserve">G67 3JS   </v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -2415,6 +2619,9 @@
       <c r="I69" t="str">
         <v/>
       </c>
+      <c r="J69" t="str">
+        <v xml:space="preserve">G67 3JS   </v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -2444,6 +2651,9 @@
       <c r="I70" t="str">
         <v/>
       </c>
+      <c r="J70" t="str">
+        <v xml:space="preserve">ML1 3YG   </v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -2473,6 +2683,9 @@
       <c r="I71" t="str">
         <v/>
       </c>
+      <c r="J71" t="str">
+        <v xml:space="preserve">ML1 3YG   </v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -2502,6 +2715,9 @@
       <c r="I72" t="str">
         <v/>
       </c>
+      <c r="J72" t="str">
+        <v xml:space="preserve">ML1 3YG   </v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -2531,6 +2747,9 @@
       <c r="I73" t="str">
         <v/>
       </c>
+      <c r="J73" t="str">
+        <v xml:space="preserve">ML1 3YG   </v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -2560,6 +2779,9 @@
       <c r="I74" t="str">
         <v/>
       </c>
+      <c r="J74" t="str">
+        <v xml:space="preserve">ML3 9RN   </v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -2589,6 +2811,9 @@
       <c r="I75" t="str">
         <v/>
       </c>
+      <c r="J75" t="str">
+        <v xml:space="preserve">G51 2TJ   </v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -2618,6 +2843,9 @@
       <c r="I76" t="str">
         <v/>
       </c>
+      <c r="J76" t="str">
+        <v xml:space="preserve">G51 2TJ   </v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -2647,6 +2875,9 @@
       <c r="I77" t="str">
         <v/>
       </c>
+      <c r="J77" t="str">
+        <v xml:space="preserve">G51 2TJ   </v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -2676,6 +2907,9 @@
       <c r="I78" t="str">
         <v/>
       </c>
+      <c r="J78" t="str">
+        <v xml:space="preserve">G51 2TJ   </v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -2705,6 +2939,9 @@
       <c r="I79" t="str">
         <v/>
       </c>
+      <c r="J79" t="str">
+        <v xml:space="preserve">G51 2TJ   </v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -2734,6 +2971,9 @@
       <c r="I80" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
+      <c r="J80" t="str">
+        <v xml:space="preserve">G67 2LE   </v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -2763,6 +3003,9 @@
       <c r="I81" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
+      <c r="J81" t="str">
+        <v xml:space="preserve">G67 2LE   </v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -2792,6 +3035,9 @@
       <c r="I82" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
+      <c r="J82" t="str">
+        <v xml:space="preserve">G67 2LE   </v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -2821,6 +3067,9 @@
       <c r="I83" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
+      <c r="J83" t="str">
+        <v xml:space="preserve">G67 2LE   </v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -2850,6 +3099,9 @@
       <c r="I84" t="str">
         <v>Agreed at induction with SM 25/04/2025 - MT</v>
       </c>
+      <c r="J84" t="str">
+        <v xml:space="preserve">G67 2LE   </v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -2879,6 +3131,9 @@
       <c r="I85" t="str">
         <v/>
       </c>
+      <c r="J85" t="str">
+        <v xml:space="preserve">ML6 8UX   </v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -2908,6 +3163,9 @@
       <c r="I86" t="str">
         <v/>
       </c>
+      <c r="J86" t="str">
+        <v xml:space="preserve">ML6 8UX   </v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -2937,6 +3195,9 @@
       <c r="I87" t="str">
         <v/>
       </c>
+      <c r="J87" t="str">
+        <v xml:space="preserve">ML6 8UX   </v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -2966,6 +3227,9 @@
       <c r="I88" t="str">
         <v/>
       </c>
+      <c r="J88" t="str">
+        <v xml:space="preserve">ML6 8UX   </v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -2995,6 +3259,9 @@
       <c r="I89" t="str">
         <v/>
       </c>
+      <c r="J89" t="str">
+        <v xml:space="preserve">ML6 8UX   </v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -3024,6 +3291,9 @@
       <c r="I90" t="str">
         <v/>
       </c>
+      <c r="J90" t="str">
+        <v xml:space="preserve">G67 1JE   </v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -3053,6 +3323,9 @@
       <c r="I91" t="str">
         <v/>
       </c>
+      <c r="J91" t="str">
+        <v xml:space="preserve">G67 1JE   </v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -3082,6 +3355,9 @@
       <c r="I92" t="str">
         <v/>
       </c>
+      <c r="J92" t="str">
+        <v xml:space="preserve">G67 1JE   </v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -3111,6 +3387,9 @@
       <c r="I93" t="str">
         <v/>
       </c>
+      <c r="J93" t="str">
+        <v xml:space="preserve">G67 1JE   </v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -3140,6 +3419,9 @@
       <c r="I94" t="str">
         <v/>
       </c>
+      <c r="J94" t="str">
+        <v xml:space="preserve">G67 3NR   </v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -3169,6 +3451,9 @@
       <c r="I95" t="str">
         <v/>
       </c>
+      <c r="J95" t="str">
+        <v xml:space="preserve">G67 3NR   </v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -3198,6 +3483,9 @@
       <c r="I96" t="str">
         <v/>
       </c>
+      <c r="J96" t="str">
+        <v xml:space="preserve">G67 3NR   </v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -3227,6 +3515,9 @@
       <c r="I97" t="str">
         <v/>
       </c>
+      <c r="J97" t="str">
+        <v xml:space="preserve">G33 2AF   </v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -3256,6 +3547,9 @@
       <c r="I98" t="str">
         <v/>
       </c>
+      <c r="J98" t="str">
+        <v xml:space="preserve">G33 2AF   </v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -3285,6 +3579,9 @@
       <c r="I99" t="str">
         <v>Lori has agreed to extend her availability via email on 02/04/2025 - MT</v>
       </c>
+      <c r="J99" t="str">
+        <v xml:space="preserve">G68 9GH   </v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -3314,6 +3611,9 @@
       <c r="I100" t="str">
         <v/>
       </c>
+      <c r="J100" t="str">
+        <v xml:space="preserve">G68 9GH   </v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -3343,6 +3643,9 @@
       <c r="I101" t="str">
         <v/>
       </c>
+      <c r="J101" t="str">
+        <v xml:space="preserve">G68 9GH   </v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -3372,6 +3675,9 @@
       <c r="I102" t="str">
         <v/>
       </c>
+      <c r="J102" t="str">
+        <v xml:space="preserve">G68 9GH   </v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -3401,10 +3707,13 @@
       <c r="I103" t="str">
         <v/>
       </c>
+      <c r="J103" t="str">
+        <v xml:space="preserve">G68 9GH   </v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I103"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J103"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update capacity dashboard with latest service location data
Modified capacity_dashboard.xlsx to include new service location entries and associated metadata.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -12672,7 +12672,7 @@
         <v>3</v>
       </c>
       <c r="G17" t="str">
-        <v>Specialised Care Client</v>
+        <v>Office Hours Client</v>
       </c>
       <c r="H17">
         <v>10</v>
@@ -12681,7 +12681,7 @@
         <v>60</v>
       </c>
       <c r="J17" t="str">
-        <v>Specialised Care Client</v>
+        <v>Care and Companionship Client</v>
       </c>
       <c r="K17">
         <v>10</v>
@@ -12690,7 +12690,7 @@
         <v>60</v>
       </c>
       <c r="M17" t="str">
-        <v>Office Hours Client</v>
+        <v>Care and Companionship Client</v>
       </c>
       <c r="N17">
         <v>10</v>
@@ -14362,7 +14362,7 @@
         <v>4.75</v>
       </c>
       <c r="G43" t="str">
-        <v>Specialised Care Client</v>
+        <v>Care and Companionship Client</v>
       </c>
       <c r="H43">
         <v>10</v>
@@ -20246,25 +20246,25 @@
         <v>Employee \ Client</v>
       </c>
       <c r="B1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+        <v>Office Hours Client 09:00-12:00 (60m)</v>
       </c>
       <c r="C1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+        <v>Office Hours Client 14:00-17:00 (60m)</v>
       </c>
       <c r="D1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="E1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="F1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="G1" t="str">
-        <v>Office Hours Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="H1" t="str">
-        <v>Office Hours Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="I1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20273,7 +20273,7 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="K1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="L1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20285,10 +20285,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="O1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="P1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="Q1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20300,40 +20300,40 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="T1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
       <c r="U1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="V1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 09:00-12:00 (420m)</v>
       </c>
       <c r="W1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 14:00-17:00 (420m)</v>
       </c>
       <c r="X1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
       <c r="Y1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="Z1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AA1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AA1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (420m)</v>
-      </c>
       <c r="AB1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (420m)</v>
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
       <c r="AC1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="AD1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AD1" t="str">
+      <c r="AE1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="AE1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
       <c r="AF1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (180m)</v>
@@ -20604,11 +20604,11 @@
       <c r="U2">
         <v>0.09</v>
       </c>
-      <c r="V2">
-        <v>0.09</v>
-      </c>
-      <c r="W2">
-        <v>0.09</v>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
       </c>
       <c r="X2">
         <v>0.09</v>
@@ -20619,11 +20619,11 @@
       <c r="Z2">
         <v>0.09</v>
       </c>
-      <c r="AA2" t="str">
-        <v/>
-      </c>
-      <c r="AB2" t="str">
-        <v/>
+      <c r="AA2">
+        <v>0.09</v>
+      </c>
+      <c r="AB2">
+        <v>0.09</v>
       </c>
       <c r="AC2">
         <v>0.09</v>
@@ -20903,11 +20903,11 @@
       <c r="U3">
         <v>0</v>
       </c>
-      <c r="V3">
-        <v>0</v>
-      </c>
-      <c r="W3">
-        <v>0</v>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
       </c>
       <c r="X3">
         <v>0</v>
@@ -20918,11 +20918,11 @@
       <c r="Z3">
         <v>0</v>
       </c>
-      <c r="AA3" t="str">
-        <v/>
-      </c>
-      <c r="AB3" t="str">
-        <v/>
+      <c r="AA3">
+        <v>0</v>
+      </c>
+      <c r="AB3">
+        <v>0</v>
       </c>
       <c r="AC3">
         <v>0</v>
@@ -21142,26 +21142,26 @@
       <c r="A4" t="str">
         <v>Asokhia (NL), Deborah</v>
       </c>
-      <c r="B4" t="str">
-        <v/>
-      </c>
-      <c r="C4">
+      <c r="B4">
         <v>0.78</v>
       </c>
-      <c r="D4" t="str">
-        <v/>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4">
+        <v>0.78</v>
       </c>
       <c r="E4">
         <v>0.78</v>
       </c>
-      <c r="F4" t="str">
-        <v/>
+      <c r="F4">
+        <v>0.78</v>
       </c>
       <c r="G4">
         <v>0.78</v>
       </c>
-      <c r="H4" t="str">
-        <v/>
+      <c r="H4">
+        <v>0.78</v>
       </c>
       <c r="I4">
         <v>0.78</v>
@@ -21169,8 +21169,8 @@
       <c r="J4">
         <v>0.78</v>
       </c>
-      <c r="K4">
-        <v>0.78</v>
+      <c r="K4" t="str">
+        <v/>
       </c>
       <c r="L4">
         <v>0.78</v>
@@ -21181,8 +21181,8 @@
       <c r="N4">
         <v>0.78</v>
       </c>
-      <c r="O4">
-        <v>0.78</v>
+      <c r="O4" t="str">
+        <v/>
       </c>
       <c r="P4" t="str">
         <v/>
@@ -21196,41 +21196,41 @@
       <c r="S4">
         <v>0.78</v>
       </c>
-      <c r="T4" t="str">
-        <v/>
+      <c r="T4">
+        <v>0.78</v>
       </c>
       <c r="U4" t="str">
         <v/>
       </c>
-      <c r="V4">
-        <v>0.78</v>
-      </c>
-      <c r="W4">
-        <v>0.78</v>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
       </c>
       <c r="X4">
         <v>0.78</v>
       </c>
-      <c r="Y4">
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4">
         <v>0.78</v>
       </c>
-      <c r="Z4" t="str">
-        <v/>
-      </c>
       <c r="AA4" t="str">
         <v/>
       </c>
-      <c r="AB4" t="str">
-        <v/>
-      </c>
-      <c r="AC4">
+      <c r="AB4">
         <v>0.78</v>
       </c>
-      <c r="AD4" t="str">
-        <v/>
-      </c>
-      <c r="AE4">
+      <c r="AC4" t="str">
+        <v/>
+      </c>
+      <c r="AD4">
         <v>0.78</v>
+      </c>
+      <c r="AE4" t="str">
+        <v/>
       </c>
       <c r="AF4" t="str">
         <v/>
@@ -21441,26 +21441,26 @@
       <c r="A5" t="str">
         <v>Brooke O'Brien (NL) (GH)</v>
       </c>
-      <c r="B5" t="str">
-        <v/>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5" t="str">
-        <v/>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5">
+        <v>0</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5" t="str">
-        <v/>
+      <c r="F5">
+        <v>0</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
-      <c r="H5" t="str">
-        <v/>
+      <c r="H5">
+        <v>0</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -21468,8 +21468,8 @@
       <c r="J5">
         <v>0</v>
       </c>
-      <c r="K5">
-        <v>0</v>
+      <c r="K5" t="str">
+        <v/>
       </c>
       <c r="L5">
         <v>0</v>
@@ -21483,8 +21483,8 @@
       <c r="O5">
         <v>0</v>
       </c>
-      <c r="P5" t="str">
-        <v/>
+      <c r="P5">
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -21498,38 +21498,38 @@
       <c r="T5">
         <v>0</v>
       </c>
-      <c r="U5">
-        <v>0</v>
-      </c>
-      <c r="V5">
-        <v>0</v>
-      </c>
-      <c r="W5">
-        <v>0</v>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v/>
       </c>
       <c r="X5">
         <v>0</v>
       </c>
-      <c r="Y5">
-        <v>0</v>
-      </c>
-      <c r="Z5" t="str">
-        <v/>
+      <c r="Y5" t="str">
+        <v/>
+      </c>
+      <c r="Z5">
+        <v>0</v>
       </c>
       <c r="AA5" t="str">
         <v/>
       </c>
-      <c r="AB5" t="str">
-        <v/>
-      </c>
-      <c r="AC5">
-        <v>0</v>
-      </c>
-      <c r="AD5" t="str">
-        <v/>
-      </c>
-      <c r="AE5">
-        <v>0</v>
+      <c r="AB5">
+        <v>0</v>
+      </c>
+      <c r="AC5" t="str">
+        <v/>
+      </c>
+      <c r="AD5">
+        <v>0</v>
+      </c>
+      <c r="AE5" t="str">
+        <v/>
       </c>
       <c r="AF5">
         <v>0</v>
@@ -22039,26 +22039,26 @@
       <c r="A7" t="str">
         <v>Donna Gabillard (NL)</v>
       </c>
-      <c r="B7" t="str">
-        <v/>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7" t="str">
-        <v/>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7">
+        <v>0</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
-      <c r="F7" t="str">
-        <v/>
+      <c r="F7">
+        <v>0</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
-      <c r="H7" t="str">
-        <v/>
+      <c r="H7">
+        <v>0</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -22096,38 +22096,38 @@
       <c r="T7">
         <v>0</v>
       </c>
-      <c r="U7">
-        <v>0</v>
-      </c>
-      <c r="V7">
-        <v>0</v>
-      </c>
-      <c r="W7">
-        <v>0</v>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v/>
       </c>
       <c r="X7">
         <v>0</v>
       </c>
-      <c r="Y7">
-        <v>0</v>
-      </c>
-      <c r="Z7" t="str">
-        <v/>
+      <c r="Y7" t="str">
+        <v/>
+      </c>
+      <c r="Z7">
+        <v>0</v>
       </c>
       <c r="AA7" t="str">
         <v/>
       </c>
-      <c r="AB7" t="str">
-        <v/>
-      </c>
-      <c r="AC7">
-        <v>0</v>
-      </c>
-      <c r="AD7" t="str">
-        <v/>
-      </c>
-      <c r="AE7">
-        <v>0</v>
+      <c r="AB7">
+        <v>0</v>
+      </c>
+      <c r="AC7" t="str">
+        <v/>
+      </c>
+      <c r="AD7">
+        <v>0</v>
+      </c>
+      <c r="AE7" t="str">
+        <v/>
       </c>
       <c r="AF7">
         <v>0</v>
@@ -22398,11 +22398,11 @@
       <c r="U8">
         <v>0</v>
       </c>
-      <c r="V8">
-        <v>0</v>
-      </c>
-      <c r="W8">
-        <v>0</v>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
       </c>
       <c r="X8">
         <v>0</v>
@@ -22413,11 +22413,11 @@
       <c r="Z8">
         <v>0</v>
       </c>
-      <c r="AA8" t="str">
-        <v/>
-      </c>
-      <c r="AB8" t="str">
-        <v/>
+      <c r="AA8">
+        <v>0</v>
+      </c>
+      <c r="AB8">
+        <v>0</v>
       </c>
       <c r="AC8">
         <v>0</v>
@@ -22637,26 +22637,26 @@
       <c r="A9" t="str">
         <v>Lynsey (GH) Mooney (NL)</v>
       </c>
-      <c r="B9" t="str">
-        <v/>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9" t="str">
-        <v/>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9">
+        <v>0</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
-      <c r="F9" t="str">
-        <v/>
+      <c r="F9">
+        <v>0</v>
       </c>
       <c r="G9">
         <v>0</v>
       </c>
-      <c r="H9" t="str">
-        <v/>
+      <c r="H9">
+        <v>0</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -22694,38 +22694,38 @@
       <c r="T9">
         <v>0</v>
       </c>
-      <c r="U9">
-        <v>0</v>
-      </c>
-      <c r="V9">
-        <v>0</v>
-      </c>
-      <c r="W9">
-        <v>0</v>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
       </c>
       <c r="X9">
         <v>0</v>
       </c>
-      <c r="Y9">
-        <v>0</v>
-      </c>
-      <c r="Z9" t="str">
-        <v/>
+      <c r="Y9" t="str">
+        <v/>
+      </c>
+      <c r="Z9">
+        <v>0</v>
       </c>
       <c r="AA9" t="str">
         <v/>
       </c>
-      <c r="AB9" t="str">
-        <v/>
-      </c>
-      <c r="AC9">
-        <v>0</v>
-      </c>
-      <c r="AD9" t="str">
-        <v/>
-      </c>
-      <c r="AE9">
-        <v>0</v>
+      <c r="AB9">
+        <v>0</v>
+      </c>
+      <c r="AC9" t="str">
+        <v/>
+      </c>
+      <c r="AD9">
+        <v>0</v>
+      </c>
+      <c r="AE9" t="str">
+        <v/>
       </c>
       <c r="AF9">
         <v>0</v>
@@ -22996,11 +22996,11 @@
       <c r="U10">
         <v>0</v>
       </c>
-      <c r="V10">
-        <v>0</v>
-      </c>
-      <c r="W10">
-        <v>0</v>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v/>
       </c>
       <c r="X10">
         <v>0</v>
@@ -23011,11 +23011,11 @@
       <c r="Z10">
         <v>0</v>
       </c>
-      <c r="AA10" t="str">
-        <v/>
-      </c>
-      <c r="AB10" t="str">
-        <v/>
+      <c r="AA10">
+        <v>0</v>
+      </c>
+      <c r="AB10">
+        <v>0</v>
       </c>
       <c r="AC10">
         <v>0</v>
@@ -23295,11 +23295,11 @@
       <c r="U11">
         <v>0</v>
       </c>
-      <c r="V11">
-        <v>0</v>
-      </c>
-      <c r="W11">
-        <v>0</v>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
       </c>
       <c r="X11">
         <v>0</v>
@@ -23310,11 +23310,11 @@
       <c r="Z11">
         <v>0</v>
       </c>
-      <c r="AA11" t="str">
-        <v/>
-      </c>
-      <c r="AB11" t="str">
-        <v/>
+      <c r="AA11">
+        <v>0</v>
+      </c>
+      <c r="AB11">
+        <v>0</v>
       </c>
       <c r="AC11">
         <v>0</v>
@@ -23594,11 +23594,11 @@
       <c r="U12">
         <v>0</v>
       </c>
-      <c r="V12">
-        <v>0</v>
-      </c>
-      <c r="W12">
-        <v>0</v>
+      <c r="V12" t="str">
+        <v/>
+      </c>
+      <c r="W12" t="str">
+        <v/>
       </c>
       <c r="X12">
         <v>0</v>
@@ -23609,11 +23609,11 @@
       <c r="Z12">
         <v>0</v>
       </c>
-      <c r="AA12" t="str">
-        <v/>
-      </c>
-      <c r="AB12" t="str">
-        <v/>
+      <c r="AA12">
+        <v>0</v>
+      </c>
+      <c r="AB12">
+        <v>0</v>
       </c>
       <c r="AC12">
         <v>0</v>
@@ -23860,8 +23860,8 @@
       <c r="J13">
         <v>0</v>
       </c>
-      <c r="K13">
-        <v>0</v>
+      <c r="K13" t="str">
+        <v/>
       </c>
       <c r="L13">
         <v>0</v>
@@ -23875,8 +23875,8 @@
       <c r="O13">
         <v>0</v>
       </c>
-      <c r="P13" t="str">
-        <v/>
+      <c r="P13">
+        <v>0</v>
       </c>
       <c r="Q13">
         <v>0</v>
@@ -23893,11 +23893,11 @@
       <c r="U13">
         <v>0</v>
       </c>
-      <c r="V13">
-        <v>0</v>
-      </c>
-      <c r="W13">
-        <v>0</v>
+      <c r="V13" t="str">
+        <v/>
+      </c>
+      <c r="W13" t="str">
+        <v/>
       </c>
       <c r="X13">
         <v>0</v>
@@ -23908,11 +23908,11 @@
       <c r="Z13">
         <v>0</v>
       </c>
-      <c r="AA13" t="str">
-        <v/>
-      </c>
-      <c r="AB13" t="str">
-        <v/>
+      <c r="AA13">
+        <v>0</v>
+      </c>
+      <c r="AB13">
+        <v>0</v>
       </c>
       <c r="AC13">
         <v>0</v>
@@ -24132,23 +24132,23 @@
       <c r="A14" t="str">
         <v>Sophie Lamont (NL) (GH)</v>
       </c>
-      <c r="B14">
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14">
         <v>0.16</v>
-      </c>
-      <c r="C14" t="str">
-        <v/>
       </c>
       <c r="D14">
         <v>0.16</v>
       </c>
-      <c r="E14" t="str">
-        <v/>
+      <c r="E14">
+        <v>0.16</v>
       </c>
       <c r="F14">
         <v>0.16</v>
       </c>
-      <c r="G14" t="str">
-        <v/>
+      <c r="G14">
+        <v>0.16</v>
       </c>
       <c r="H14">
         <v>0.16</v>
@@ -24159,8 +24159,8 @@
       <c r="J14">
         <v>0.16</v>
       </c>
-      <c r="K14">
-        <v>0.16</v>
+      <c r="K14" t="str">
+        <v/>
       </c>
       <c r="L14">
         <v>0.16</v>
@@ -24171,8 +24171,8 @@
       <c r="N14">
         <v>0.16</v>
       </c>
-      <c r="O14">
-        <v>0.16</v>
+      <c r="O14" t="str">
+        <v/>
       </c>
       <c r="P14" t="str">
         <v/>
@@ -24189,38 +24189,38 @@
       <c r="T14" t="str">
         <v/>
       </c>
-      <c r="U14" t="str">
-        <v/>
-      </c>
-      <c r="V14">
+      <c r="U14">
         <v>0.16</v>
       </c>
-      <c r="W14">
+      <c r="V14" t="str">
+        <v/>
+      </c>
+      <c r="W14" t="str">
+        <v/>
+      </c>
+      <c r="X14" t="str">
+        <v/>
+      </c>
+      <c r="Y14">
         <v>0.16</v>
       </c>
-      <c r="X14">
+      <c r="Z14" t="str">
+        <v/>
+      </c>
+      <c r="AA14">
         <v>0.16</v>
       </c>
-      <c r="Y14" t="str">
-        <v/>
-      </c>
-      <c r="Z14">
+      <c r="AB14" t="str">
+        <v/>
+      </c>
+      <c r="AC14">
         <v>0.16</v>
       </c>
-      <c r="AA14" t="str">
-        <v/>
-      </c>
-      <c r="AB14" t="str">
-        <v/>
-      </c>
-      <c r="AC14" t="str">
-        <v/>
-      </c>
-      <c r="AD14">
+      <c r="AD14" t="str">
+        <v/>
+      </c>
+      <c r="AE14">
         <v>0.16</v>
-      </c>
-      <c r="AE14" t="str">
-        <v/>
       </c>
       <c r="AF14" t="str">
         <v/>
@@ -24443,46 +24443,46 @@
         <v>Employee \ Client</v>
       </c>
       <c r="B1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+        <v>Office Hours Client 09:00-12:00 (60m)</v>
       </c>
       <c r="C1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+        <v>Office Hours Client 14:00-17:00 (60m)</v>
       </c>
       <c r="D1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (420m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="E1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (420m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="F1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="G1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="H1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="I1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="J1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="K1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="L1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="M1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="N1" t="str">
-        <v>Office Hours Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="O1" t="str">
-        <v>Office Hours Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="P1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
@@ -24497,40 +24497,40 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="T1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
       <c r="U1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="V1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 09:00-12:00 (420m)</v>
       </c>
       <c r="W1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+        <v>Specialised Care Client 14:00-17:00 (420m)</v>
       </c>
       <c r="X1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
       <c r="Y1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="Z1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
       <c r="AA1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="AB1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
       <c r="AC1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="AD1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
       <c r="AE1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="AF1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -24726,11 +24726,11 @@
       <c r="C2">
         <v>0.16</v>
       </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v/>
+      <c r="D2">
+        <v>0.16</v>
+      </c>
+      <c r="E2">
+        <v>0.16</v>
       </c>
       <c r="F2">
         <v>0.16</v>
@@ -24780,11 +24780,11 @@
       <c r="U2">
         <v>0.16</v>
       </c>
-      <c r="V2">
-        <v>0.16</v>
-      </c>
-      <c r="W2">
-        <v>0.16</v>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
       </c>
       <c r="X2">
         <v>0.16</v>
@@ -25004,11 +25004,11 @@
       <c r="C3">
         <v>0</v>
       </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v/>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -25058,11 +25058,11 @@
       <c r="U3">
         <v>0</v>
       </c>
-      <c r="V3">
-        <v>0</v>
-      </c>
-      <c r="W3">
-        <v>0</v>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
       </c>
       <c r="X3">
         <v>0</v>
@@ -25282,11 +25282,11 @@
       <c r="C4">
         <v>0</v>
       </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v/>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -25336,11 +25336,11 @@
       <c r="U4">
         <v>0</v>
       </c>
-      <c r="V4">
-        <v>0</v>
-      </c>
-      <c r="W4">
-        <v>0</v>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
       </c>
       <c r="X4">
         <v>0</v>
@@ -25560,23 +25560,23 @@
       <c r="C5" t="str">
         <v/>
       </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v/>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
-      <c r="G5" t="str">
-        <v/>
+      <c r="G5">
+        <v>0</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
-      <c r="I5" t="str">
-        <v/>
+      <c r="I5">
+        <v>0</v>
       </c>
       <c r="J5">
         <v>0</v>
@@ -25587,14 +25587,14 @@
       <c r="L5">
         <v>0</v>
       </c>
-      <c r="M5" t="str">
-        <v/>
+      <c r="M5">
+        <v>0</v>
       </c>
       <c r="N5">
         <v>0</v>
       </c>
-      <c r="O5" t="str">
-        <v/>
+      <c r="O5">
+        <v>0</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -25611,11 +25611,11 @@
       <c r="T5">
         <v>0</v>
       </c>
-      <c r="U5">
-        <v>0</v>
-      </c>
-      <c r="V5">
-        <v>0</v>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
       </c>
       <c r="W5" t="str">
         <v/>
@@ -25623,26 +25623,26 @@
       <c r="X5">
         <v>0</v>
       </c>
-      <c r="Y5">
-        <v>0</v>
+      <c r="Y5" t="str">
+        <v/>
       </c>
       <c r="Z5">
         <v>0</v>
       </c>
-      <c r="AA5">
-        <v>0</v>
+      <c r="AA5" t="str">
+        <v/>
       </c>
       <c r="AB5">
         <v>0</v>
       </c>
-      <c r="AC5">
-        <v>0</v>
+      <c r="AC5" t="str">
+        <v/>
       </c>
       <c r="AD5">
         <v>0</v>
       </c>
-      <c r="AE5">
-        <v>0</v>
+      <c r="AE5" t="str">
+        <v/>
       </c>
       <c r="AF5">
         <v>0</v>
@@ -26116,23 +26116,23 @@
       <c r="C7" t="str">
         <v/>
       </c>
-      <c r="D7" t="str">
-        <v/>
-      </c>
-      <c r="E7" t="str">
-        <v/>
+      <c r="D7">
+        <v>0.05</v>
+      </c>
+      <c r="E7">
+        <v>0.05</v>
       </c>
       <c r="F7">
         <v>0.05</v>
       </c>
-      <c r="G7" t="str">
-        <v/>
+      <c r="G7">
+        <v>0.05</v>
       </c>
       <c r="H7">
         <v>0.05</v>
       </c>
-      <c r="I7" t="str">
-        <v/>
+      <c r="I7">
+        <v>0.05</v>
       </c>
       <c r="J7">
         <v>0.05</v>
@@ -26143,14 +26143,14 @@
       <c r="L7">
         <v>0.05</v>
       </c>
-      <c r="M7" t="str">
-        <v/>
+      <c r="M7">
+        <v>0.05</v>
       </c>
       <c r="N7">
         <v>0.05</v>
       </c>
-      <c r="O7" t="str">
-        <v/>
+      <c r="O7">
+        <v>0.05</v>
       </c>
       <c r="P7">
         <v>0.05</v>
@@ -26167,11 +26167,11 @@
       <c r="T7">
         <v>0.05</v>
       </c>
-      <c r="U7">
-        <v>0.05</v>
-      </c>
-      <c r="V7">
-        <v>0.05</v>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
       </c>
       <c r="W7" t="str">
         <v/>
@@ -26179,26 +26179,26 @@
       <c r="X7">
         <v>0.05</v>
       </c>
-      <c r="Y7">
-        <v>0.05</v>
+      <c r="Y7" t="str">
+        <v/>
       </c>
       <c r="Z7">
         <v>0.05</v>
       </c>
-      <c r="AA7">
-        <v>0.05</v>
+      <c r="AA7" t="str">
+        <v/>
       </c>
       <c r="AB7">
         <v>0.05</v>
       </c>
-      <c r="AC7">
-        <v>0.05</v>
+      <c r="AC7" t="str">
+        <v/>
       </c>
       <c r="AD7">
         <v>0.05</v>
       </c>
-      <c r="AE7">
-        <v>0.05</v>
+      <c r="AE7" t="str">
+        <v/>
       </c>
       <c r="AF7">
         <v>0.05</v>
@@ -26394,23 +26394,23 @@
       <c r="C8" t="str">
         <v/>
       </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8" t="str">
-        <v/>
+      <c r="D8">
+        <v>0.08</v>
+      </c>
+      <c r="E8">
+        <v>0.08</v>
       </c>
       <c r="F8">
         <v>0.08</v>
       </c>
-      <c r="G8" t="str">
-        <v/>
+      <c r="G8">
+        <v>0.08</v>
       </c>
       <c r="H8">
         <v>0.08</v>
       </c>
-      <c r="I8" t="str">
-        <v/>
+      <c r="I8">
+        <v>0.08</v>
       </c>
       <c r="J8">
         <v>0.08</v>
@@ -26421,14 +26421,14 @@
       <c r="L8">
         <v>0.08</v>
       </c>
-      <c r="M8" t="str">
-        <v/>
+      <c r="M8">
+        <v>0.08</v>
       </c>
       <c r="N8">
         <v>0.08</v>
       </c>
-      <c r="O8" t="str">
-        <v/>
+      <c r="O8">
+        <v>0.08</v>
       </c>
       <c r="P8">
         <v>0.08</v>
@@ -26445,11 +26445,11 @@
       <c r="T8">
         <v>0.08</v>
       </c>
-      <c r="U8">
-        <v>0.08</v>
-      </c>
-      <c r="V8">
-        <v>0.08</v>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
       </c>
       <c r="W8" t="str">
         <v/>
@@ -26457,26 +26457,26 @@
       <c r="X8">
         <v>0.08</v>
       </c>
-      <c r="Y8">
-        <v>0.08</v>
+      <c r="Y8" t="str">
+        <v/>
       </c>
       <c r="Z8">
         <v>0.08</v>
       </c>
-      <c r="AA8">
-        <v>0.08</v>
+      <c r="AA8" t="str">
+        <v/>
       </c>
       <c r="AB8">
         <v>0.08</v>
       </c>
-      <c r="AC8">
-        <v>0.08</v>
+      <c r="AC8" t="str">
+        <v/>
       </c>
       <c r="AD8">
         <v>0.08</v>
       </c>
-      <c r="AE8">
-        <v>0.08</v>
+      <c r="AE8" t="str">
+        <v/>
       </c>
       <c r="AF8">
         <v>0.08</v>
@@ -26672,41 +26672,41 @@
       <c r="C9" t="str">
         <v/>
       </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
-      <c r="E9" t="str">
-        <v/>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
-      <c r="G9" t="str">
-        <v/>
+      <c r="G9">
+        <v>0</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
-      <c r="I9" t="str">
-        <v/>
+      <c r="I9">
+        <v>0</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
-      <c r="K9" t="str">
-        <v/>
+      <c r="K9">
+        <v>0</v>
       </c>
       <c r="L9">
         <v>0</v>
       </c>
-      <c r="M9" t="str">
-        <v/>
+      <c r="M9">
+        <v>0</v>
       </c>
       <c r="N9">
         <v>0</v>
       </c>
-      <c r="O9" t="str">
-        <v/>
+      <c r="O9">
+        <v>0</v>
       </c>
       <c r="P9">
         <v>0</v>
@@ -26723,38 +26723,38 @@
       <c r="T9">
         <v>0</v>
       </c>
-      <c r="U9">
-        <v>0</v>
-      </c>
-      <c r="V9">
-        <v>0</v>
-      </c>
-      <c r="W9">
-        <v>0</v>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
       </c>
       <c r="X9">
         <v>0</v>
       </c>
-      <c r="Y9">
-        <v>0</v>
+      <c r="Y9" t="str">
+        <v/>
       </c>
       <c r="Z9">
         <v>0</v>
       </c>
-      <c r="AA9">
-        <v>0</v>
+      <c r="AA9" t="str">
+        <v/>
       </c>
       <c r="AB9">
         <v>0</v>
       </c>
-      <c r="AC9">
-        <v>0</v>
+      <c r="AC9" t="str">
+        <v/>
       </c>
       <c r="AD9">
         <v>0</v>
       </c>
-      <c r="AE9">
-        <v>0</v>
+      <c r="AE9" t="str">
+        <v/>
       </c>
       <c r="AF9">
         <v>0</v>
@@ -26950,11 +26950,11 @@
       <c r="C10">
         <v>0.1</v>
       </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
-      <c r="E10" t="str">
-        <v/>
+      <c r="D10">
+        <v>0.1</v>
+      </c>
+      <c r="E10">
+        <v>0.1</v>
       </c>
       <c r="F10">
         <v>0.1</v>
@@ -27004,11 +27004,11 @@
       <c r="U10">
         <v>0.1</v>
       </c>
-      <c r="V10">
-        <v>0.1</v>
-      </c>
-      <c r="W10">
-        <v>0.1</v>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v/>
       </c>
       <c r="X10">
         <v>0.1</v>
@@ -27228,11 +27228,11 @@
       <c r="C11">
         <v>0.01</v>
       </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
-      <c r="E11" t="str">
-        <v/>
+      <c r="D11">
+        <v>0.01</v>
+      </c>
+      <c r="E11">
+        <v>0.01</v>
       </c>
       <c r="F11">
         <v>0.01</v>
@@ -27282,11 +27282,11 @@
       <c r="U11">
         <v>0.01</v>
       </c>
-      <c r="V11">
-        <v>0.01</v>
-      </c>
-      <c r="W11">
-        <v>0.01</v>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
       </c>
       <c r="X11">
         <v>0.01</v>
@@ -27506,11 +27506,11 @@
       <c r="C12">
         <v>0</v>
       </c>
-      <c r="D12" t="str">
-        <v/>
-      </c>
-      <c r="E12" t="str">
-        <v/>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -27560,11 +27560,11 @@
       <c r="U12">
         <v>0</v>
       </c>
-      <c r="V12">
-        <v>0</v>
-      </c>
-      <c r="W12">
-        <v>0</v>
+      <c r="V12" t="str">
+        <v/>
+      </c>
+      <c r="W12" t="str">
+        <v/>
       </c>
       <c r="X12">
         <v>0</v>
@@ -27784,11 +27784,11 @@
       <c r="C13">
         <v>0</v>
       </c>
-      <c r="D13" t="str">
-        <v/>
-      </c>
-      <c r="E13" t="str">
-        <v/>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -27838,11 +27838,11 @@
       <c r="U13">
         <v>0</v>
       </c>
-      <c r="V13">
-        <v>0</v>
-      </c>
-      <c r="W13">
-        <v>0</v>
+      <c r="V13" t="str">
+        <v/>
+      </c>
+      <c r="W13" t="str">
+        <v/>
       </c>
       <c r="X13">
         <v>0</v>
@@ -28068,13 +28068,13 @@
         <v>Employee \ Client</v>
       </c>
       <c r="B1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="C1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="D1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (360m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="E1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -28083,7 +28083,7 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="G1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="H1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -28101,28 +28101,28 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="M1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="N1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="O1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="P1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="Q1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="R1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
       <c r="S1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="T1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 09:00-12:00 (360m)</v>
       </c>
       <c r="U1" t="str">
         <v>Specialised Care Client 14:00-17:00 (360m)</v>
@@ -28324,8 +28324,8 @@
       <c r="C2">
         <v>0.25</v>
       </c>
-      <c r="D2" t="str">
-        <v/>
+      <c r="D2">
+        <v>0.25</v>
       </c>
       <c r="E2">
         <v>0.25</v>
@@ -28372,8 +28372,8 @@
       <c r="S2">
         <v>0.25</v>
       </c>
-      <c r="T2">
-        <v>0.25</v>
+      <c r="T2" t="str">
+        <v/>
       </c>
       <c r="U2" t="str">
         <v/>
@@ -28572,8 +28572,8 @@
       <c r="B3">
         <v>0.07</v>
       </c>
-      <c r="C3" t="str">
-        <v/>
+      <c r="C3">
+        <v>0.07</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -28584,8 +28584,8 @@
       <c r="F3">
         <v>0.07</v>
       </c>
-      <c r="G3" t="str">
-        <v/>
+      <c r="G3">
+        <v>0.07</v>
       </c>
       <c r="H3">
         <v>0.07</v>
@@ -28620,11 +28620,11 @@
       <c r="R3">
         <v>0.07</v>
       </c>
-      <c r="S3">
-        <v>0.07</v>
-      </c>
-      <c r="T3">
-        <v>0.07</v>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
       </c>
       <c r="U3" t="str">
         <v/>
@@ -28823,8 +28823,8 @@
       <c r="B4">
         <v>0.13</v>
       </c>
-      <c r="C4" t="str">
-        <v/>
+      <c r="C4">
+        <v>0.13</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -28835,8 +28835,8 @@
       <c r="F4">
         <v>0.13</v>
       </c>
-      <c r="G4" t="str">
-        <v/>
+      <c r="G4">
+        <v>0.13</v>
       </c>
       <c r="H4">
         <v>0.13</v>
@@ -28871,11 +28871,11 @@
       <c r="R4">
         <v>0.13</v>
       </c>
-      <c r="S4">
-        <v>0.13</v>
-      </c>
-      <c r="T4">
-        <v>0.13</v>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
       </c>
       <c r="U4" t="str">
         <v/>
@@ -29074,8 +29074,8 @@
       <c r="B5">
         <v>0.78</v>
       </c>
-      <c r="C5" t="str">
-        <v/>
+      <c r="C5">
+        <v>0.78</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -29086,8 +29086,8 @@
       <c r="F5">
         <v>0.78</v>
       </c>
-      <c r="G5" t="str">
-        <v/>
+      <c r="G5">
+        <v>0.78</v>
       </c>
       <c r="H5">
         <v>0.78</v>
@@ -29122,11 +29122,11 @@
       <c r="R5">
         <v>0.78</v>
       </c>
-      <c r="S5">
-        <v>0.78</v>
-      </c>
-      <c r="T5">
-        <v>0.78</v>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
       </c>
       <c r="U5" t="str">
         <v/>
@@ -29830,8 +29830,8 @@
       <c r="C8">
         <v>0.25</v>
       </c>
-      <c r="D8" t="str">
-        <v/>
+      <c r="D8">
+        <v>0.25</v>
       </c>
       <c r="E8">
         <v>0.25</v>
@@ -29878,8 +29878,8 @@
       <c r="S8">
         <v>0.25</v>
       </c>
-      <c r="T8">
-        <v>0.25</v>
+      <c r="T8" t="str">
+        <v/>
       </c>
       <c r="U8" t="str">
         <v/>
@@ -30078,8 +30078,8 @@
       <c r="B9">
         <v>0.08</v>
       </c>
-      <c r="C9" t="str">
-        <v/>
+      <c r="C9">
+        <v>0.08</v>
       </c>
       <c r="D9" t="str">
         <v/>
@@ -30090,8 +30090,8 @@
       <c r="F9">
         <v>0.08</v>
       </c>
-      <c r="G9" t="str">
-        <v/>
+      <c r="G9">
+        <v>0.08</v>
       </c>
       <c r="H9">
         <v>0.08</v>
@@ -30126,11 +30126,11 @@
       <c r="R9">
         <v>0.08</v>
       </c>
-      <c r="S9">
-        <v>0.08</v>
-      </c>
-      <c r="T9">
-        <v>0.08</v>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
       </c>
       <c r="U9" t="str">
         <v/>
@@ -30329,11 +30329,11 @@
       <c r="B10">
         <v>0</v>
       </c>
-      <c r="C10" t="str">
-        <v/>
-      </c>
-      <c r="D10" t="str">
-        <v/>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -30377,11 +30377,11 @@
       <c r="R10">
         <v>0</v>
       </c>
-      <c r="S10">
-        <v>0</v>
-      </c>
-      <c r="T10">
-        <v>0</v>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
       </c>
       <c r="U10" t="str">
         <v/>
@@ -30583,8 +30583,8 @@
       <c r="C11">
         <v>0.1</v>
       </c>
-      <c r="D11" t="str">
-        <v/>
+      <c r="D11">
+        <v>0.1</v>
       </c>
       <c r="E11">
         <v>0.1</v>
@@ -30631,8 +30631,8 @@
       <c r="S11">
         <v>0.1</v>
       </c>
-      <c r="T11">
-        <v>0.1</v>
+      <c r="T11" t="str">
+        <v/>
       </c>
       <c r="U11" t="str">
         <v/>
@@ -30834,8 +30834,8 @@
       <c r="C12">
         <v>0</v>
       </c>
-      <c r="D12" t="str">
-        <v/>
+      <c r="D12">
+        <v>0</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -30882,8 +30882,8 @@
       <c r="S12">
         <v>0</v>
       </c>
-      <c r="T12">
-        <v>0</v>
+      <c r="T12" t="str">
+        <v/>
       </c>
       <c r="U12" t="str">
         <v/>
@@ -31085,8 +31085,8 @@
       <c r="C13">
         <v>0.14</v>
       </c>
-      <c r="D13" t="str">
-        <v/>
+      <c r="D13">
+        <v>0.14</v>
       </c>
       <c r="E13">
         <v>0.14</v>
@@ -31133,8 +31133,8 @@
       <c r="S13">
         <v>0.14</v>
       </c>
-      <c r="T13">
-        <v>0.14</v>
+      <c r="T13" t="str">
+        <v/>
       </c>
       <c r="U13" t="str">
         <v/>
@@ -31336,8 +31336,8 @@
       <c r="C14">
         <v>0</v>
       </c>
-      <c r="D14" t="str">
-        <v/>
+      <c r="D14">
+        <v>0</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -31384,8 +31384,8 @@
       <c r="S14">
         <v>0</v>
       </c>
-      <c r="T14">
-        <v>0</v>
+      <c r="T14" t="str">
+        <v/>
       </c>
       <c r="U14" t="str">
         <v/>
@@ -31596,8 +31596,8 @@
       <c r="F15">
         <v>0</v>
       </c>
-      <c r="G15" t="str">
-        <v/>
+      <c r="G15">
+        <v>0</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -31635,8 +31635,8 @@
       <c r="S15">
         <v>0</v>
       </c>
-      <c r="T15">
-        <v>0</v>
+      <c r="T15" t="str">
+        <v/>
       </c>
       <c r="U15" t="str">
         <v/>
@@ -31838,8 +31838,8 @@
       <c r="C16">
         <v>0.09</v>
       </c>
-      <c r="D16" t="str">
-        <v/>
+      <c r="D16">
+        <v>0.09</v>
       </c>
       <c r="E16">
         <v>0.09</v>
@@ -31886,8 +31886,8 @@
       <c r="S16">
         <v>0.09</v>
       </c>
-      <c r="T16">
-        <v>0.09</v>
+      <c r="T16" t="str">
+        <v/>
       </c>
       <c r="U16" t="str">
         <v/>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update capacity dashboard to include new planning factors
Added new columns to capacity_dashboard.xlsx for client distance, time windows, and visit times.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3690,19 +3690,19 @@
         <v>Brown, Christine 33333-.6875 (60m)</v>
       </c>
       <c r="AD1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AE1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="AE1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AF1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AG1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AH1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (165m)</v>
-      </c>
-      <c r="AH1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AI1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -3723,13 +3723,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AO1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AP1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AQ1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AR1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -3738,67 +3738,67 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AT1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AU1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AU1" t="str">
+      <c r="AV1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AV1" t="str">
+      <c r="AW1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AW1" t="str">
+      <c r="AX1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AX1" t="str">
+      <c r="AY1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AY1" t="str">
+      <c r="AZ1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BA1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BA1" t="str">
+      <c r="BB1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BB1" t="str">
+      <c r="BC1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BC1" t="str">
+      <c r="BD1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BD1" t="str">
+      <c r="BE1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BF1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BG1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BH1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BI1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BJ1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BK1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BK1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BM1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BN1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BO1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -3810,10 +3810,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BR1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BS1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BS1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -6569,10 +6569,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AC1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AD1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (240m)</v>
-      </c>
-      <c r="AD1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AE1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -6593,13 +6593,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AK1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AM1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -6608,58 +6608,58 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AP1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AQ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AQ1" t="str">
+      <c r="AR1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AR1" t="str">
+      <c r="AS1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AS1" t="str">
+      <c r="AT1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AT1" t="str">
+      <c r="AU1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AU1" t="str">
+      <c r="AV1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AV1" t="str">
+      <c r="AW1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AW1" t="str">
+      <c r="AX1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AX1" t="str">
+      <c r="AY1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AY1" t="str">
+      <c r="AZ1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BA1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BA1" t="str">
+      <c r="BB1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BB1" t="str">
+      <c r="BC1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BC1" t="str">
+      <c r="BD1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BD1" t="str">
+      <c r="BE1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BF1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BG1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BG1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BH1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -6668,16 +6668,16 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BJ1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BK1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
-      <c r="BK1" t="str">
+      <c r="BL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BL1" t="str">
+      <c r="BM1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (180m)</v>
-      </c>
-      <c r="BM1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -7022,56 +7022,56 @@
       <c r="AP3">
         <v>0</v>
       </c>
-      <c r="AQ3" t="str">
-        <v/>
-      </c>
-      <c r="AR3">
-        <v>0</v>
-      </c>
-      <c r="AS3" t="str">
-        <v/>
-      </c>
-      <c r="AT3">
-        <v>0</v>
-      </c>
-      <c r="AU3" t="str">
-        <v/>
-      </c>
-      <c r="AV3">
-        <v>0</v>
-      </c>
-      <c r="AW3" t="str">
-        <v/>
-      </c>
-      <c r="AX3">
-        <v>0</v>
-      </c>
-      <c r="AY3" t="str">
-        <v/>
-      </c>
-      <c r="AZ3">
-        <v>0</v>
-      </c>
-      <c r="BA3" t="str">
-        <v/>
-      </c>
-      <c r="BB3">
-        <v>0</v>
-      </c>
-      <c r="BC3" t="str">
-        <v/>
-      </c>
-      <c r="BD3">
-        <v>0</v>
+      <c r="AQ3">
+        <v>0</v>
+      </c>
+      <c r="AR3" t="str">
+        <v/>
+      </c>
+      <c r="AS3">
+        <v>0</v>
+      </c>
+      <c r="AT3" t="str">
+        <v/>
+      </c>
+      <c r="AU3">
+        <v>0</v>
+      </c>
+      <c r="AV3" t="str">
+        <v/>
+      </c>
+      <c r="AW3">
+        <v>0</v>
+      </c>
+      <c r="AX3" t="str">
+        <v/>
+      </c>
+      <c r="AY3">
+        <v>0</v>
+      </c>
+      <c r="AZ3" t="str">
+        <v/>
+      </c>
+      <c r="BA3">
+        <v>0</v>
+      </c>
+      <c r="BB3" t="str">
+        <v/>
+      </c>
+      <c r="BC3">
+        <v>0</v>
+      </c>
+      <c r="BD3" t="str">
+        <v/>
       </c>
       <c r="BE3">
         <v>0</v>
       </c>
-      <c r="BF3" t="str">
-        <v/>
-      </c>
-      <c r="BG3">
-        <v>0</v>
+      <c r="BF3">
+        <v>0</v>
+      </c>
+      <c r="BG3" t="str">
+        <v/>
       </c>
       <c r="BH3">
         <v>0</v>
@@ -8010,11 +8010,11 @@
       <c r="AB8">
         <v>0.78</v>
       </c>
-      <c r="AC8" t="str">
-        <v/>
-      </c>
-      <c r="AD8">
+      <c r="AC8">
         <v>0.78</v>
+      </c>
+      <c r="AD8" t="str">
+        <v/>
       </c>
       <c r="AE8">
         <v>0.78</v>
@@ -8052,56 +8052,56 @@
       <c r="AP8">
         <v>0.78</v>
       </c>
-      <c r="AQ8" t="str">
-        <v/>
-      </c>
-      <c r="AR8">
+      <c r="AQ8">
         <v>0.78</v>
       </c>
-      <c r="AS8" t="str">
-        <v/>
-      </c>
-      <c r="AT8">
+      <c r="AR8" t="str">
+        <v/>
+      </c>
+      <c r="AS8">
         <v>0.78</v>
       </c>
-      <c r="AU8" t="str">
-        <v/>
-      </c>
-      <c r="AV8">
+      <c r="AT8" t="str">
+        <v/>
+      </c>
+      <c r="AU8">
         <v>0.78</v>
       </c>
-      <c r="AW8" t="str">
-        <v/>
-      </c>
-      <c r="AX8">
+      <c r="AV8" t="str">
+        <v/>
+      </c>
+      <c r="AW8">
         <v>0.78</v>
       </c>
-      <c r="AY8" t="str">
-        <v/>
-      </c>
-      <c r="AZ8">
+      <c r="AX8" t="str">
+        <v/>
+      </c>
+      <c r="AY8">
         <v>0.78</v>
       </c>
-      <c r="BA8" t="str">
-        <v/>
-      </c>
-      <c r="BB8">
+      <c r="AZ8" t="str">
+        <v/>
+      </c>
+      <c r="BA8">
         <v>0.78</v>
       </c>
-      <c r="BC8" t="str">
-        <v/>
-      </c>
-      <c r="BD8">
+      <c r="BB8" t="str">
+        <v/>
+      </c>
+      <c r="BC8">
         <v>0.78</v>
+      </c>
+      <c r="BD8" t="str">
+        <v/>
       </c>
       <c r="BE8">
         <v>0.78</v>
       </c>
-      <c r="BF8" t="str">
-        <v/>
-      </c>
-      <c r="BG8">
+      <c r="BF8">
         <v>0.78</v>
+      </c>
+      <c r="BG8" t="str">
+        <v/>
       </c>
       <c r="BH8">
         <v>0.78</v>
@@ -16853,16 +16853,16 @@
         <v>Armstrong (NL), Hugh .4375-66667 (60m)</v>
       </c>
       <c r="AF1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AH1" t="str">
         <v>Companionship Client 09:00-17:00 (120m)</v>
       </c>
-      <c r="AG1" t="str">
+      <c r="AI1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="AH1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="AI1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AJ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -16877,49 +16877,49 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AN1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AO1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AP1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="AQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AR1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AS1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
-      <c r="AS1" t="str">
+      <c r="AU1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="AT1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="AU1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AW1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AX1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AY1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AX1" t="str">
+      <c r="AZ1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AY1" t="str">
+      <c r="BA1" t="str">
         <v>Specialised Care Client 09:00-12:00 (420m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BB1" t="str">
         <v>Specialised Care Client 14:00-17:00 (420m)</v>
-      </c>
-      <c r="BA1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BB1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BC1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
@@ -16934,22 +16934,22 @@
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BG1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BH1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BI1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BJ1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BK1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BL1" t="str">
         <v>Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BK1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BL1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BM1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
@@ -16958,22 +16958,22 @@
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BO1" t="str">
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BP1" t="str">
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BP1" t="str">
+      <c r="BR1" t="str">
         <v>Office Hours Client 09:00-12:00 (510m)</v>
       </c>
-      <c r="BQ1" t="str">
+      <c r="BS1" t="str">
         <v>Office Hours Client 14:00-17:00 (510m)</v>
       </c>
-      <c r="BR1" t="str">
+      <c r="BT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BS1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BT1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BU1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
@@ -16982,10 +16982,10 @@
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BW1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BX1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BY1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -17157,17 +17157,17 @@
       <c r="AX2">
         <v>0.25</v>
       </c>
-      <c r="AY2" t="str">
-        <v/>
-      </c>
-      <c r="AZ2" t="str">
-        <v/>
-      </c>
-      <c r="BA2">
+      <c r="AY2">
         <v>0.25</v>
       </c>
-      <c r="BB2">
+      <c r="AZ2">
         <v>0.25</v>
+      </c>
+      <c r="BA2" t="str">
+        <v/>
+      </c>
+      <c r="BB2" t="str">
+        <v/>
       </c>
       <c r="BC2">
         <v>0.25</v>
@@ -17208,17 +17208,17 @@
       <c r="BO2">
         <v>0.25</v>
       </c>
-      <c r="BP2" t="str">
-        <v/>
-      </c>
-      <c r="BQ2" t="str">
-        <v/>
-      </c>
-      <c r="BR2">
+      <c r="BP2">
         <v>0.25</v>
       </c>
-      <c r="BS2">
+      <c r="BQ2">
         <v>0.25</v>
+      </c>
+      <c r="BR2" t="str">
+        <v/>
+      </c>
+      <c r="BS2" t="str">
+        <v/>
       </c>
       <c r="BT2">
         <v>0.25</v>
@@ -17405,17 +17405,17 @@
       <c r="AX3">
         <v>0.01</v>
       </c>
-      <c r="AY3" t="str">
-        <v/>
-      </c>
-      <c r="AZ3" t="str">
-        <v/>
-      </c>
-      <c r="BA3">
+      <c r="AY3">
         <v>0.01</v>
       </c>
-      <c r="BB3">
+      <c r="AZ3">
         <v>0.01</v>
+      </c>
+      <c r="BA3" t="str">
+        <v/>
+      </c>
+      <c r="BB3" t="str">
+        <v/>
       </c>
       <c r="BC3">
         <v>0.01</v>
@@ -17456,17 +17456,17 @@
       <c r="BO3">
         <v>0.01</v>
       </c>
-      <c r="BP3" t="str">
-        <v/>
-      </c>
-      <c r="BQ3" t="str">
-        <v/>
-      </c>
-      <c r="BR3">
+      <c r="BP3">
         <v>0.01</v>
       </c>
-      <c r="BS3">
+      <c r="BQ3">
         <v>0.01</v>
+      </c>
+      <c r="BR3" t="str">
+        <v/>
+      </c>
+      <c r="BS3" t="str">
+        <v/>
       </c>
       <c r="BT3">
         <v>0.01</v>
@@ -17620,14 +17620,14 @@
       <c r="AM4">
         <v>0</v>
       </c>
-      <c r="AN4" t="str">
-        <v/>
+      <c r="AN4">
+        <v>0</v>
       </c>
       <c r="AO4">
         <v>0</v>
       </c>
-      <c r="AP4">
-        <v>0</v>
+      <c r="AP4" t="str">
+        <v/>
       </c>
       <c r="AQ4">
         <v>0</v>
@@ -17650,17 +17650,17 @@
       <c r="AW4">
         <v>0</v>
       </c>
-      <c r="AX4" t="str">
-        <v/>
-      </c>
-      <c r="AY4" t="str">
-        <v/>
+      <c r="AX4">
+        <v>0</v>
+      </c>
+      <c r="AY4">
+        <v>0</v>
       </c>
       <c r="AZ4" t="str">
         <v/>
       </c>
-      <c r="BA4">
-        <v>0</v>
+      <c r="BA4" t="str">
+        <v/>
       </c>
       <c r="BB4" t="str">
         <v/>
@@ -17686,14 +17686,14 @@
       <c r="BI4">
         <v>0</v>
       </c>
-      <c r="BJ4">
-        <v>0</v>
+      <c r="BJ4" t="str">
+        <v/>
       </c>
       <c r="BK4">
         <v>0</v>
       </c>
-      <c r="BL4" t="str">
-        <v/>
+      <c r="BL4">
+        <v>0</v>
       </c>
       <c r="BM4">
         <v>0</v>
@@ -17707,14 +17707,14 @@
       <c r="BP4" t="str">
         <v/>
       </c>
-      <c r="BQ4" t="str">
-        <v/>
-      </c>
-      <c r="BR4">
-        <v>0</v>
-      </c>
-      <c r="BS4">
-        <v>0</v>
+      <c r="BQ4">
+        <v>0</v>
+      </c>
+      <c r="BR4" t="str">
+        <v/>
+      </c>
+      <c r="BS4" t="str">
+        <v/>
       </c>
       <c r="BT4">
         <v>0</v>
@@ -18116,14 +18116,14 @@
       <c r="AM6">
         <v>0.05</v>
       </c>
-      <c r="AN6" t="str">
-        <v/>
+      <c r="AN6">
+        <v>0.05</v>
       </c>
       <c r="AO6">
         <v>0.05</v>
       </c>
-      <c r="AP6">
-        <v>0.05</v>
+      <c r="AP6" t="str">
+        <v/>
       </c>
       <c r="AQ6">
         <v>0.05</v>
@@ -18146,17 +18146,17 @@
       <c r="AW6">
         <v>0.05</v>
       </c>
-      <c r="AX6" t="str">
-        <v/>
-      </c>
-      <c r="AY6" t="str">
-        <v/>
+      <c r="AX6">
+        <v>0.05</v>
+      </c>
+      <c r="AY6">
+        <v>0.05</v>
       </c>
       <c r="AZ6" t="str">
         <v/>
       </c>
-      <c r="BA6">
-        <v>0.05</v>
+      <c r="BA6" t="str">
+        <v/>
       </c>
       <c r="BB6" t="str">
         <v/>
@@ -18182,14 +18182,14 @@
       <c r="BI6">
         <v>0.05</v>
       </c>
-      <c r="BJ6">
-        <v>0.05</v>
+      <c r="BJ6" t="str">
+        <v/>
       </c>
       <c r="BK6">
         <v>0.05</v>
       </c>
-      <c r="BL6" t="str">
-        <v/>
+      <c r="BL6">
+        <v>0.05</v>
       </c>
       <c r="BM6">
         <v>0.05</v>
@@ -18203,14 +18203,14 @@
       <c r="BP6" t="str">
         <v/>
       </c>
-      <c r="BQ6" t="str">
-        <v/>
-      </c>
-      <c r="BR6">
+      <c r="BQ6">
         <v>0.05</v>
       </c>
-      <c r="BS6">
-        <v>0.05</v>
+      <c r="BR6" t="str">
+        <v/>
+      </c>
+      <c r="BS6" t="str">
+        <v/>
       </c>
       <c r="BT6">
         <v>0.05</v>
@@ -18397,17 +18397,17 @@
       <c r="AX7">
         <v>0</v>
       </c>
-      <c r="AY7" t="str">
-        <v/>
-      </c>
-      <c r="AZ7" t="str">
-        <v/>
-      </c>
-      <c r="BA7">
-        <v>0</v>
-      </c>
-      <c r="BB7">
-        <v>0</v>
+      <c r="AY7">
+        <v>0</v>
+      </c>
+      <c r="AZ7">
+        <v>0</v>
+      </c>
+      <c r="BA7" t="str">
+        <v/>
+      </c>
+      <c r="BB7" t="str">
+        <v/>
       </c>
       <c r="BC7">
         <v>0</v>
@@ -18448,17 +18448,17 @@
       <c r="BO7">
         <v>0</v>
       </c>
-      <c r="BP7" t="str">
-        <v/>
-      </c>
-      <c r="BQ7" t="str">
-        <v/>
-      </c>
-      <c r="BR7">
-        <v>0</v>
-      </c>
-      <c r="BS7">
-        <v>0</v>
+      <c r="BP7">
+        <v>0</v>
+      </c>
+      <c r="BQ7">
+        <v>0</v>
+      </c>
+      <c r="BR7" t="str">
+        <v/>
+      </c>
+      <c r="BS7" t="str">
+        <v/>
       </c>
       <c r="BT7">
         <v>0</v>
@@ -18645,17 +18645,17 @@
       <c r="AX8">
         <v>0.08</v>
       </c>
-      <c r="AY8" t="str">
-        <v/>
-      </c>
-      <c r="AZ8" t="str">
-        <v/>
-      </c>
-      <c r="BA8">
+      <c r="AY8">
         <v>0.08</v>
       </c>
-      <c r="BB8">
+      <c r="AZ8">
         <v>0.08</v>
+      </c>
+      <c r="BA8" t="str">
+        <v/>
+      </c>
+      <c r="BB8" t="str">
+        <v/>
       </c>
       <c r="BC8">
         <v>0.08</v>
@@ -18696,17 +18696,17 @@
       <c r="BO8">
         <v>0.08</v>
       </c>
-      <c r="BP8" t="str">
-        <v/>
-      </c>
-      <c r="BQ8" t="str">
-        <v/>
-      </c>
-      <c r="BR8">
+      <c r="BP8">
         <v>0.08</v>
       </c>
-      <c r="BS8">
+      <c r="BQ8">
         <v>0.08</v>
+      </c>
+      <c r="BR8" t="str">
+        <v/>
+      </c>
+      <c r="BS8" t="str">
+        <v/>
       </c>
       <c r="BT8">
         <v>0.08</v>
@@ -18890,17 +18890,17 @@
       <c r="AW9">
         <v>0</v>
       </c>
-      <c r="AX9" t="str">
-        <v/>
-      </c>
-      <c r="AY9" t="str">
-        <v/>
+      <c r="AX9">
+        <v>0</v>
+      </c>
+      <c r="AY9">
+        <v>0</v>
       </c>
       <c r="AZ9" t="str">
         <v/>
       </c>
-      <c r="BA9">
-        <v>0</v>
+      <c r="BA9" t="str">
+        <v/>
       </c>
       <c r="BB9" t="str">
         <v/>
@@ -18926,14 +18926,14 @@
       <c r="BI9">
         <v>0</v>
       </c>
-      <c r="BJ9">
-        <v>0</v>
+      <c r="BJ9" t="str">
+        <v/>
       </c>
       <c r="BK9">
         <v>0</v>
       </c>
-      <c r="BL9" t="str">
-        <v/>
+      <c r="BL9">
+        <v>0</v>
       </c>
       <c r="BM9">
         <v>0</v>
@@ -18947,14 +18947,14 @@
       <c r="BP9" t="str">
         <v/>
       </c>
-      <c r="BQ9" t="str">
-        <v/>
-      </c>
-      <c r="BR9">
-        <v>0</v>
-      </c>
-      <c r="BS9">
-        <v>0</v>
+      <c r="BQ9">
+        <v>0</v>
+      </c>
+      <c r="BR9" t="str">
+        <v/>
+      </c>
+      <c r="BS9" t="str">
+        <v/>
       </c>
       <c r="BT9">
         <v>0</v>
@@ -19141,17 +19141,17 @@
       <c r="AX10">
         <v>0</v>
       </c>
-      <c r="AY10" t="str">
-        <v/>
-      </c>
-      <c r="AZ10" t="str">
-        <v/>
-      </c>
-      <c r="BA10">
-        <v>0</v>
-      </c>
-      <c r="BB10">
-        <v>0</v>
+      <c r="AY10">
+        <v>0</v>
+      </c>
+      <c r="AZ10">
+        <v>0</v>
+      </c>
+      <c r="BA10" t="str">
+        <v/>
+      </c>
+      <c r="BB10" t="str">
+        <v/>
       </c>
       <c r="BC10">
         <v>0</v>
@@ -19192,17 +19192,17 @@
       <c r="BO10">
         <v>0</v>
       </c>
-      <c r="BP10" t="str">
-        <v/>
-      </c>
-      <c r="BQ10" t="str">
-        <v/>
-      </c>
-      <c r="BR10">
-        <v>0</v>
-      </c>
-      <c r="BS10">
-        <v>0</v>
+      <c r="BP10">
+        <v>0</v>
+      </c>
+      <c r="BQ10">
+        <v>0</v>
+      </c>
+      <c r="BR10" t="str">
+        <v/>
+      </c>
+      <c r="BS10" t="str">
+        <v/>
       </c>
       <c r="BT10">
         <v>0</v>
@@ -19332,17 +19332,17 @@
       <c r="AE11">
         <v>0.88</v>
       </c>
-      <c r="AF11" t="str">
-        <v/>
-      </c>
-      <c r="AG11" t="str">
-        <v/>
-      </c>
-      <c r="AH11">
+      <c r="AF11">
         <v>0.78</v>
       </c>
-      <c r="AI11">
+      <c r="AG11">
         <v>0.78</v>
+      </c>
+      <c r="AH11" t="str">
+        <v/>
+      </c>
+      <c r="AI11" t="str">
+        <v/>
       </c>
       <c r="AJ11">
         <v>0.78</v>
@@ -19356,38 +19356,38 @@
       <c r="AM11">
         <v>0.78</v>
       </c>
-      <c r="AN11" t="str">
-        <v/>
+      <c r="AN11">
+        <v>0.78</v>
       </c>
       <c r="AO11">
         <v>0.78</v>
       </c>
-      <c r="AP11">
-        <v>0.78</v>
+      <c r="AP11" t="str">
+        <v/>
       </c>
       <c r="AQ11">
         <v>0.78</v>
       </c>
-      <c r="AR11" t="str">
-        <v/>
-      </c>
-      <c r="AS11" t="str">
-        <v/>
-      </c>
-      <c r="AT11">
+      <c r="AR11">
         <v>0.78</v>
       </c>
-      <c r="AU11">
+      <c r="AS11">
         <v>0.78</v>
+      </c>
+      <c r="AT11" t="str">
+        <v/>
+      </c>
+      <c r="AU11" t="str">
+        <v/>
       </c>
       <c r="AV11">
         <v>0.78</v>
       </c>
-      <c r="AW11" t="str">
-        <v/>
-      </c>
-      <c r="AX11" t="str">
-        <v/>
+      <c r="AW11">
+        <v>0.78</v>
+      </c>
+      <c r="AX11">
+        <v>0.78</v>
       </c>
       <c r="AY11" t="str">
         <v/>
@@ -19419,53 +19419,53 @@
       <c r="BH11" t="str">
         <v/>
       </c>
-      <c r="BI11">
+      <c r="BI11" t="str">
+        <v/>
+      </c>
+      <c r="BJ11" t="str">
+        <v/>
+      </c>
+      <c r="BK11">
         <v>0.78</v>
       </c>
-      <c r="BJ11">
+      <c r="BL11">
         <v>0.78</v>
       </c>
-      <c r="BK11" t="str">
-        <v/>
-      </c>
-      <c r="BL11" t="str">
-        <v/>
-      </c>
       <c r="BM11" t="str">
         <v/>
       </c>
       <c r="BN11" t="str">
         <v/>
       </c>
-      <c r="BO11">
+      <c r="BO11" t="str">
+        <v/>
+      </c>
+      <c r="BP11" t="str">
+        <v/>
+      </c>
+      <c r="BQ11">
         <v>0.78</v>
       </c>
-      <c r="BP11" t="str">
-        <v/>
-      </c>
-      <c r="BQ11" t="str">
-        <v/>
-      </c>
-      <c r="BR11">
+      <c r="BR11" t="str">
+        <v/>
+      </c>
+      <c r="BS11" t="str">
+        <v/>
+      </c>
+      <c r="BT11">
         <v>0.78</v>
       </c>
-      <c r="BS11" t="str">
-        <v/>
-      </c>
-      <c r="BT11" t="str">
-        <v/>
-      </c>
       <c r="BU11" t="str">
         <v/>
       </c>
       <c r="BV11" t="str">
         <v/>
       </c>
-      <c r="BW11">
-        <v>0.78</v>
-      </c>
-      <c r="BX11">
-        <v>0.78</v>
+      <c r="BW11" t="str">
+        <v/>
+      </c>
+      <c r="BX11" t="str">
+        <v/>
       </c>
       <c r="BY11">
         <v>0.78</v>
@@ -19637,17 +19637,17 @@
       <c r="AX12">
         <v>0</v>
       </c>
-      <c r="AY12" t="str">
-        <v/>
-      </c>
-      <c r="AZ12" t="str">
-        <v/>
-      </c>
-      <c r="BA12">
-        <v>0</v>
-      </c>
-      <c r="BB12">
-        <v>0</v>
+      <c r="AY12">
+        <v>0</v>
+      </c>
+      <c r="AZ12">
+        <v>0</v>
+      </c>
+      <c r="BA12" t="str">
+        <v/>
+      </c>
+      <c r="BB12" t="str">
+        <v/>
       </c>
       <c r="BC12">
         <v>0</v>
@@ -19688,17 +19688,17 @@
       <c r="BO12">
         <v>0</v>
       </c>
-      <c r="BP12" t="str">
-        <v/>
-      </c>
-      <c r="BQ12" t="str">
-        <v/>
-      </c>
-      <c r="BR12">
-        <v>0</v>
-      </c>
-      <c r="BS12">
-        <v>0</v>
+      <c r="BP12">
+        <v>0</v>
+      </c>
+      <c r="BQ12">
+        <v>0</v>
+      </c>
+      <c r="BR12" t="str">
+        <v/>
+      </c>
+      <c r="BS12" t="str">
+        <v/>
       </c>
       <c r="BT12">
         <v>0</v>
@@ -19852,14 +19852,14 @@
       <c r="AM13">
         <v>0.17</v>
       </c>
-      <c r="AN13" t="str">
-        <v/>
+      <c r="AN13">
+        <v>0.17</v>
       </c>
       <c r="AO13">
         <v>0.17</v>
       </c>
-      <c r="AP13">
-        <v>0.17</v>
+      <c r="AP13" t="str">
+        <v/>
       </c>
       <c r="AQ13">
         <v>0.17</v>
@@ -19885,17 +19885,17 @@
       <c r="AX13">
         <v>0.17</v>
       </c>
-      <c r="AY13" t="str">
-        <v/>
-      </c>
-      <c r="AZ13" t="str">
-        <v/>
-      </c>
-      <c r="BA13">
+      <c r="AY13">
         <v>0.17</v>
       </c>
-      <c r="BB13">
+      <c r="AZ13">
         <v>0.17</v>
+      </c>
+      <c r="BA13" t="str">
+        <v/>
+      </c>
+      <c r="BB13" t="str">
+        <v/>
       </c>
       <c r="BC13">
         <v>0.17</v>
@@ -19936,17 +19936,17 @@
       <c r="BO13">
         <v>0.17</v>
       </c>
-      <c r="BP13" t="str">
-        <v/>
-      </c>
-      <c r="BQ13" t="str">
-        <v/>
-      </c>
-      <c r="BR13">
+      <c r="BP13">
         <v>0.17</v>
       </c>
-      <c r="BS13">
+      <c r="BQ13">
         <v>0.17</v>
+      </c>
+      <c r="BR13" t="str">
+        <v/>
+      </c>
+      <c r="BS13" t="str">
+        <v/>
       </c>
       <c r="BT13">
         <v>0.17</v>
@@ -20360,13 +20360,13 @@
         <v>Anderson, Margaret 33333-1.375 (60m)</v>
       </c>
       <c r="AN1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AO1" t="str">
         <v>Office Hours Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AO1" t="str">
+      <c r="AP1" t="str">
         <v>Office Hours Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="AP1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20387,10 +20387,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AW1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (285m)</v>
-      </c>
-      <c r="AX1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AY1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20399,13 +20399,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BA1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BB1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BC1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BD1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20414,58 +20414,58 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BF1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BG1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BH1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BI1" t="str">
         <v>Specialised Care Client 09:00-12:00 (420m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BJ1" t="str">
         <v>Specialised Care Client 14:00-17:00 (420m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BK1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BK1" t="str">
+      <c r="BL1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BL1" t="str">
+      <c r="BM1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BM1" t="str">
+      <c r="BN1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BN1" t="str">
+      <c r="BO1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BO1" t="str">
+      <c r="BP1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BP1" t="str">
+      <c r="BQ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BQ1" t="str">
+      <c r="BR1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BR1" t="str">
+      <c r="BS1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (180m)</v>
       </c>
-      <c r="BS1" t="str">
+      <c r="BT1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BT1" t="str">
+      <c r="BU1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BU1" t="str">
+      <c r="BV1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BV1" t="str">
+      <c r="BW1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BW1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
@@ -20474,58 +20474,58 @@
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BZ1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="CA1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CA1" t="str">
+      <c r="CB1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="CB1" t="str">
+      <c r="CC1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="CC1" t="str">
+      <c r="CD1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="CD1" t="str">
+      <c r="CE1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="CE1" t="str">
+      <c r="CF1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CF1" t="str">
+      <c r="CG1" t="str">
         <v>Office Hours Client 09:00-12:00 (330m)</v>
       </c>
-      <c r="CG1" t="str">
+      <c r="CH1" t="str">
         <v>Office Hours Client 14:00-17:00 (330m)</v>
       </c>
-      <c r="CH1" t="str">
+      <c r="CI1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CI1" t="str">
+      <c r="CJ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
-      <c r="CJ1" t="str">
+      <c r="CK1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (150m)</v>
-      </c>
-      <c r="CK1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CM1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="CO1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="CP1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CP1" t="str">
+      <c r="CQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="CQ1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CR1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20718,14 +20718,14 @@
       <c r="BG2">
         <v>0.09</v>
       </c>
-      <c r="BH2" t="str">
-        <v/>
+      <c r="BH2">
+        <v>0.09</v>
       </c>
       <c r="BI2" t="str">
         <v/>
       </c>
-      <c r="BJ2">
-        <v>0.09</v>
+      <c r="BJ2" t="str">
+        <v/>
       </c>
       <c r="BK2">
         <v>0.09</v>
@@ -20790,14 +20790,14 @@
       <c r="CE2">
         <v>0.09</v>
       </c>
-      <c r="CF2" t="str">
-        <v/>
+      <c r="CF2">
+        <v>0.09</v>
       </c>
       <c r="CG2" t="str">
         <v/>
       </c>
-      <c r="CH2">
-        <v>0.09</v>
+      <c r="CH2" t="str">
+        <v/>
       </c>
       <c r="CI2">
         <v>0.09</v>
@@ -21017,14 +21017,14 @@
       <c r="BG3">
         <v>0</v>
       </c>
-      <c r="BH3" t="str">
-        <v/>
+      <c r="BH3">
+        <v>0</v>
       </c>
       <c r="BI3" t="str">
         <v/>
       </c>
-      <c r="BJ3">
-        <v>0</v>
+      <c r="BJ3" t="str">
+        <v/>
       </c>
       <c r="BK3">
         <v>0</v>
@@ -21089,14 +21089,14 @@
       <c r="CE3">
         <v>0</v>
       </c>
-      <c r="CF3" t="str">
-        <v/>
+      <c r="CF3">
+        <v>0</v>
       </c>
       <c r="CG3" t="str">
         <v/>
       </c>
-      <c r="CH3">
-        <v>0</v>
+      <c r="CH3" t="str">
+        <v/>
       </c>
       <c r="CI3">
         <v>0</v>
@@ -21259,11 +21259,11 @@
       <c r="AN4">
         <v>0.78</v>
       </c>
-      <c r="AO4" t="str">
-        <v/>
-      </c>
-      <c r="AP4">
+      <c r="AO4">
         <v>0.78</v>
+      </c>
+      <c r="AP4" t="str">
+        <v/>
       </c>
       <c r="AQ4">
         <v>0.78</v>
@@ -21283,11 +21283,11 @@
       <c r="AV4">
         <v>0.78</v>
       </c>
-      <c r="AW4" t="str">
-        <v/>
-      </c>
-      <c r="AX4">
+      <c r="AW4">
         <v>0.78</v>
+      </c>
+      <c r="AX4" t="str">
+        <v/>
       </c>
       <c r="AY4">
         <v>0.78</v>
@@ -21295,14 +21295,14 @@
       <c r="AZ4">
         <v>0.78</v>
       </c>
-      <c r="BA4" t="str">
-        <v/>
+      <c r="BA4">
+        <v>0.78</v>
       </c>
       <c r="BB4" t="str">
         <v/>
       </c>
-      <c r="BC4">
-        <v>0.78</v>
+      <c r="BC4" t="str">
+        <v/>
       </c>
       <c r="BD4">
         <v>0.78</v>
@@ -21313,8 +21313,8 @@
       <c r="BF4">
         <v>0.78</v>
       </c>
-      <c r="BG4" t="str">
-        <v/>
+      <c r="BG4">
+        <v>0.78</v>
       </c>
       <c r="BH4" t="str">
         <v/>
@@ -21322,45 +21322,45 @@
       <c r="BI4" t="str">
         <v/>
       </c>
-      <c r="BJ4">
+      <c r="BJ4" t="str">
+        <v/>
+      </c>
+      <c r="BK4">
         <v>0.78</v>
       </c>
-      <c r="BK4" t="str">
-        <v/>
-      </c>
-      <c r="BL4">
+      <c r="BL4" t="str">
+        <v/>
+      </c>
+      <c r="BM4">
         <v>0.78</v>
       </c>
-      <c r="BM4" t="str">
-        <v/>
-      </c>
-      <c r="BN4">
+      <c r="BN4" t="str">
+        <v/>
+      </c>
+      <c r="BO4">
         <v>0.78</v>
       </c>
-      <c r="BO4" t="str">
-        <v/>
-      </c>
-      <c r="BP4">
+      <c r="BP4" t="str">
+        <v/>
+      </c>
+      <c r="BQ4">
         <v>0.78</v>
       </c>
-      <c r="BQ4" t="str">
-        <v/>
-      </c>
       <c r="BR4" t="str">
         <v/>
       </c>
-      <c r="BS4">
+      <c r="BS4" t="str">
+        <v/>
+      </c>
+      <c r="BT4">
         <v>0.78</v>
       </c>
-      <c r="BT4" t="str">
-        <v/>
-      </c>
-      <c r="BU4">
+      <c r="BU4" t="str">
+        <v/>
+      </c>
+      <c r="BV4">
         <v>0.78</v>
       </c>
-      <c r="BV4" t="str">
-        <v/>
-      </c>
       <c r="BW4" t="str">
         <v/>
       </c>
@@ -21370,59 +21370,59 @@
       <c r="BY4" t="str">
         <v/>
       </c>
-      <c r="BZ4">
-        <v>0.78</v>
+      <c r="BZ4" t="str">
+        <v/>
       </c>
       <c r="CA4">
         <v>0.78</v>
       </c>
-      <c r="CB4" t="str">
-        <v/>
-      </c>
-      <c r="CC4">
+      <c r="CB4">
         <v>0.78</v>
       </c>
-      <c r="CD4" t="str">
-        <v/>
-      </c>
-      <c r="CE4">
+      <c r="CC4" t="str">
+        <v/>
+      </c>
+      <c r="CD4">
         <v>0.78</v>
       </c>
-      <c r="CF4" t="str">
-        <v/>
+      <c r="CE4" t="str">
+        <v/>
+      </c>
+      <c r="CF4">
+        <v>0.78</v>
       </c>
       <c r="CG4" t="str">
         <v/>
       </c>
-      <c r="CH4">
+      <c r="CH4" t="str">
+        <v/>
+      </c>
+      <c r="CI4">
         <v>0.78</v>
       </c>
-      <c r="CI4" t="str">
-        <v/>
-      </c>
       <c r="CJ4" t="str">
         <v/>
       </c>
-      <c r="CK4">
-        <v>0.78</v>
+      <c r="CK4" t="str">
+        <v/>
       </c>
       <c r="CL4">
         <v>0.78</v>
       </c>
-      <c r="CM4" t="str">
-        <v/>
+      <c r="CM4">
+        <v>0.78</v>
       </c>
       <c r="CN4" t="str">
         <v/>
       </c>
-      <c r="CO4">
+      <c r="CO4" t="str">
+        <v/>
+      </c>
+      <c r="CP4">
         <v>0.78</v>
       </c>
-      <c r="CP4" t="str">
-        <v/>
-      </c>
-      <c r="CQ4">
-        <v>0.78</v>
+      <c r="CQ4" t="str">
+        <v/>
       </c>
       <c r="CR4">
         <v>0.78</v>
@@ -21558,11 +21558,11 @@
       <c r="AN5">
         <v>0</v>
       </c>
-      <c r="AO5" t="str">
-        <v/>
-      </c>
-      <c r="AP5">
-        <v>0</v>
+      <c r="AO5">
+        <v>0</v>
+      </c>
+      <c r="AP5" t="str">
+        <v/>
       </c>
       <c r="AQ5">
         <v>0</v>
@@ -21582,11 +21582,11 @@
       <c r="AV5">
         <v>0</v>
       </c>
-      <c r="AW5" t="str">
-        <v/>
-      </c>
-      <c r="AX5">
-        <v>0</v>
+      <c r="AW5">
+        <v>0</v>
+      </c>
+      <c r="AX5" t="str">
+        <v/>
       </c>
       <c r="AY5">
         <v>0</v>
@@ -21612,8 +21612,8 @@
       <c r="BF5">
         <v>0</v>
       </c>
-      <c r="BG5" t="str">
-        <v/>
+      <c r="BG5">
+        <v>0</v>
       </c>
       <c r="BH5" t="str">
         <v/>
@@ -21621,47 +21621,47 @@
       <c r="BI5" t="str">
         <v/>
       </c>
-      <c r="BJ5">
-        <v>0</v>
-      </c>
-      <c r="BK5" t="str">
-        <v/>
-      </c>
-      <c r="BL5">
-        <v>0</v>
-      </c>
-      <c r="BM5" t="str">
-        <v/>
-      </c>
-      <c r="BN5">
-        <v>0</v>
-      </c>
-      <c r="BO5" t="str">
-        <v/>
-      </c>
-      <c r="BP5">
-        <v>0</v>
-      </c>
-      <c r="BQ5" t="str">
-        <v/>
-      </c>
-      <c r="BR5">
-        <v>0</v>
+      <c r="BJ5" t="str">
+        <v/>
+      </c>
+      <c r="BK5">
+        <v>0</v>
+      </c>
+      <c r="BL5" t="str">
+        <v/>
+      </c>
+      <c r="BM5">
+        <v>0</v>
+      </c>
+      <c r="BN5" t="str">
+        <v/>
+      </c>
+      <c r="BO5">
+        <v>0</v>
+      </c>
+      <c r="BP5" t="str">
+        <v/>
+      </c>
+      <c r="BQ5">
+        <v>0</v>
+      </c>
+      <c r="BR5" t="str">
+        <v/>
       </c>
       <c r="BS5">
         <v>0</v>
       </c>
-      <c r="BT5" t="str">
-        <v/>
-      </c>
-      <c r="BU5">
-        <v>0</v>
-      </c>
-      <c r="BV5" t="str">
-        <v/>
-      </c>
-      <c r="BW5">
-        <v>0</v>
+      <c r="BT5">
+        <v>0</v>
+      </c>
+      <c r="BU5" t="str">
+        <v/>
+      </c>
+      <c r="BV5">
+        <v>0</v>
+      </c>
+      <c r="BW5" t="str">
+        <v/>
       </c>
       <c r="BX5">
         <v>0</v>
@@ -21675,32 +21675,32 @@
       <c r="CA5">
         <v>0</v>
       </c>
-      <c r="CB5" t="str">
-        <v/>
-      </c>
-      <c r="CC5">
-        <v>0</v>
-      </c>
-      <c r="CD5" t="str">
-        <v/>
-      </c>
-      <c r="CE5">
-        <v>0</v>
-      </c>
-      <c r="CF5" t="str">
-        <v/>
+      <c r="CB5">
+        <v>0</v>
+      </c>
+      <c r="CC5" t="str">
+        <v/>
+      </c>
+      <c r="CD5">
+        <v>0</v>
+      </c>
+      <c r="CE5" t="str">
+        <v/>
+      </c>
+      <c r="CF5">
+        <v>0</v>
       </c>
       <c r="CG5" t="str">
         <v/>
       </c>
-      <c r="CH5">
-        <v>0</v>
-      </c>
-      <c r="CI5" t="str">
-        <v/>
-      </c>
-      <c r="CJ5">
-        <v>0</v>
+      <c r="CH5" t="str">
+        <v/>
+      </c>
+      <c r="CI5">
+        <v>0</v>
+      </c>
+      <c r="CJ5" t="str">
+        <v/>
       </c>
       <c r="CK5">
         <v>0</v>
@@ -22156,11 +22156,11 @@
       <c r="AN7">
         <v>0</v>
       </c>
-      <c r="AO7" t="str">
-        <v/>
-      </c>
-      <c r="AP7">
-        <v>0</v>
+      <c r="AO7">
+        <v>0</v>
+      </c>
+      <c r="AP7" t="str">
+        <v/>
       </c>
       <c r="AQ7">
         <v>0</v>
@@ -22210,8 +22210,8 @@
       <c r="BF7">
         <v>0</v>
       </c>
-      <c r="BG7" t="str">
-        <v/>
+      <c r="BG7">
+        <v>0</v>
       </c>
       <c r="BH7" t="str">
         <v/>
@@ -22219,47 +22219,47 @@
       <c r="BI7" t="str">
         <v/>
       </c>
-      <c r="BJ7">
-        <v>0</v>
-      </c>
-      <c r="BK7" t="str">
-        <v/>
-      </c>
-      <c r="BL7">
-        <v>0</v>
-      </c>
-      <c r="BM7" t="str">
-        <v/>
-      </c>
-      <c r="BN7">
-        <v>0</v>
-      </c>
-      <c r="BO7" t="str">
-        <v/>
-      </c>
-      <c r="BP7">
-        <v>0</v>
-      </c>
-      <c r="BQ7" t="str">
-        <v/>
-      </c>
-      <c r="BR7">
-        <v>0</v>
+      <c r="BJ7" t="str">
+        <v/>
+      </c>
+      <c r="BK7">
+        <v>0</v>
+      </c>
+      <c r="BL7" t="str">
+        <v/>
+      </c>
+      <c r="BM7">
+        <v>0</v>
+      </c>
+      <c r="BN7" t="str">
+        <v/>
+      </c>
+      <c r="BO7">
+        <v>0</v>
+      </c>
+      <c r="BP7" t="str">
+        <v/>
+      </c>
+      <c r="BQ7">
+        <v>0</v>
+      </c>
+      <c r="BR7" t="str">
+        <v/>
       </c>
       <c r="BS7">
         <v>0</v>
       </c>
-      <c r="BT7" t="str">
-        <v/>
-      </c>
-      <c r="BU7">
-        <v>0</v>
-      </c>
-      <c r="BV7" t="str">
-        <v/>
-      </c>
-      <c r="BW7">
-        <v>0</v>
+      <c r="BT7">
+        <v>0</v>
+      </c>
+      <c r="BU7" t="str">
+        <v/>
+      </c>
+      <c r="BV7">
+        <v>0</v>
+      </c>
+      <c r="BW7" t="str">
+        <v/>
       </c>
       <c r="BX7">
         <v>0</v>
@@ -22273,26 +22273,26 @@
       <c r="CA7">
         <v>0</v>
       </c>
-      <c r="CB7" t="str">
-        <v/>
-      </c>
-      <c r="CC7">
-        <v>0</v>
-      </c>
-      <c r="CD7" t="str">
-        <v/>
-      </c>
-      <c r="CE7">
-        <v>0</v>
-      </c>
-      <c r="CF7" t="str">
-        <v/>
+      <c r="CB7">
+        <v>0</v>
+      </c>
+      <c r="CC7" t="str">
+        <v/>
+      </c>
+      <c r="CD7">
+        <v>0</v>
+      </c>
+      <c r="CE7" t="str">
+        <v/>
+      </c>
+      <c r="CF7">
+        <v>0</v>
       </c>
       <c r="CG7" t="str">
         <v/>
       </c>
-      <c r="CH7">
-        <v>0</v>
+      <c r="CH7" t="str">
+        <v/>
       </c>
       <c r="CI7">
         <v>0</v>
@@ -22512,14 +22512,14 @@
       <c r="BG8">
         <v>0</v>
       </c>
-      <c r="BH8" t="str">
-        <v/>
+      <c r="BH8">
+        <v>0</v>
       </c>
       <c r="BI8" t="str">
         <v/>
       </c>
-      <c r="BJ8">
-        <v>0</v>
+      <c r="BJ8" t="str">
+        <v/>
       </c>
       <c r="BK8">
         <v>0</v>
@@ -22584,14 +22584,14 @@
       <c r="CE8">
         <v>0</v>
       </c>
-      <c r="CF8" t="str">
-        <v/>
+      <c r="CF8">
+        <v>0</v>
       </c>
       <c r="CG8" t="str">
         <v/>
       </c>
-      <c r="CH8">
-        <v>0</v>
+      <c r="CH8" t="str">
+        <v/>
       </c>
       <c r="CI8">
         <v>0</v>
@@ -22754,11 +22754,11 @@
       <c r="AN9">
         <v>0</v>
       </c>
-      <c r="AO9" t="str">
-        <v/>
-      </c>
-      <c r="AP9">
-        <v>0</v>
+      <c r="AO9">
+        <v>0</v>
+      </c>
+      <c r="AP9" t="str">
+        <v/>
       </c>
       <c r="AQ9">
         <v>0</v>
@@ -22808,8 +22808,8 @@
       <c r="BF9">
         <v>0</v>
       </c>
-      <c r="BG9" t="str">
-        <v/>
+      <c r="BG9">
+        <v>0</v>
       </c>
       <c r="BH9" t="str">
         <v/>
@@ -22817,47 +22817,47 @@
       <c r="BI9" t="str">
         <v/>
       </c>
-      <c r="BJ9">
-        <v>0</v>
-      </c>
-      <c r="BK9" t="str">
-        <v/>
-      </c>
-      <c r="BL9">
-        <v>0</v>
-      </c>
-      <c r="BM9" t="str">
-        <v/>
-      </c>
-      <c r="BN9">
-        <v>0</v>
-      </c>
-      <c r="BO9" t="str">
-        <v/>
-      </c>
-      <c r="BP9">
-        <v>0</v>
-      </c>
-      <c r="BQ9" t="str">
-        <v/>
-      </c>
-      <c r="BR9">
-        <v>0</v>
+      <c r="BJ9" t="str">
+        <v/>
+      </c>
+      <c r="BK9">
+        <v>0</v>
+      </c>
+      <c r="BL9" t="str">
+        <v/>
+      </c>
+      <c r="BM9">
+        <v>0</v>
+      </c>
+      <c r="BN9" t="str">
+        <v/>
+      </c>
+      <c r="BO9">
+        <v>0</v>
+      </c>
+      <c r="BP9" t="str">
+        <v/>
+      </c>
+      <c r="BQ9">
+        <v>0</v>
+      </c>
+      <c r="BR9" t="str">
+        <v/>
       </c>
       <c r="BS9">
         <v>0</v>
       </c>
-      <c r="BT9" t="str">
-        <v/>
-      </c>
-      <c r="BU9">
-        <v>0</v>
-      </c>
-      <c r="BV9" t="str">
-        <v/>
-      </c>
-      <c r="BW9">
-        <v>0</v>
+      <c r="BT9">
+        <v>0</v>
+      </c>
+      <c r="BU9" t="str">
+        <v/>
+      </c>
+      <c r="BV9">
+        <v>0</v>
+      </c>
+      <c r="BW9" t="str">
+        <v/>
       </c>
       <c r="BX9">
         <v>0</v>
@@ -22871,26 +22871,26 @@
       <c r="CA9">
         <v>0</v>
       </c>
-      <c r="CB9" t="str">
-        <v/>
-      </c>
-      <c r="CC9">
-        <v>0</v>
-      </c>
-      <c r="CD9" t="str">
-        <v/>
-      </c>
-      <c r="CE9">
-        <v>0</v>
-      </c>
-      <c r="CF9" t="str">
-        <v/>
+      <c r="CB9">
+        <v>0</v>
+      </c>
+      <c r="CC9" t="str">
+        <v/>
+      </c>
+      <c r="CD9">
+        <v>0</v>
+      </c>
+      <c r="CE9" t="str">
+        <v/>
+      </c>
+      <c r="CF9">
+        <v>0</v>
       </c>
       <c r="CG9" t="str">
         <v/>
       </c>
-      <c r="CH9">
-        <v>0</v>
+      <c r="CH9" t="str">
+        <v/>
       </c>
       <c r="CI9">
         <v>0</v>
@@ -23110,14 +23110,14 @@
       <c r="BG10">
         <v>0</v>
       </c>
-      <c r="BH10" t="str">
-        <v/>
+      <c r="BH10">
+        <v>0</v>
       </c>
       <c r="BI10" t="str">
         <v/>
       </c>
-      <c r="BJ10">
-        <v>0</v>
+      <c r="BJ10" t="str">
+        <v/>
       </c>
       <c r="BK10">
         <v>0</v>
@@ -23182,14 +23182,14 @@
       <c r="CE10">
         <v>0</v>
       </c>
-      <c r="CF10" t="str">
-        <v/>
+      <c r="CF10">
+        <v>0</v>
       </c>
       <c r="CG10" t="str">
         <v/>
       </c>
-      <c r="CH10">
-        <v>0</v>
+      <c r="CH10" t="str">
+        <v/>
       </c>
       <c r="CI10">
         <v>0</v>
@@ -23409,14 +23409,14 @@
       <c r="BG11">
         <v>0</v>
       </c>
-      <c r="BH11" t="str">
-        <v/>
+      <c r="BH11">
+        <v>0</v>
       </c>
       <c r="BI11" t="str">
         <v/>
       </c>
-      <c r="BJ11">
-        <v>0</v>
+      <c r="BJ11" t="str">
+        <v/>
       </c>
       <c r="BK11">
         <v>0</v>
@@ -23481,14 +23481,14 @@
       <c r="CE11">
         <v>0</v>
       </c>
-      <c r="CF11" t="str">
-        <v/>
+      <c r="CF11">
+        <v>0</v>
       </c>
       <c r="CG11" t="str">
         <v/>
       </c>
-      <c r="CH11">
-        <v>0</v>
+      <c r="CH11" t="str">
+        <v/>
       </c>
       <c r="CI11">
         <v>0</v>
@@ -23708,14 +23708,14 @@
       <c r="BG12">
         <v>0</v>
       </c>
-      <c r="BH12" t="str">
-        <v/>
+      <c r="BH12">
+        <v>0</v>
       </c>
       <c r="BI12" t="str">
         <v/>
       </c>
-      <c r="BJ12">
-        <v>0</v>
+      <c r="BJ12" t="str">
+        <v/>
       </c>
       <c r="BK12">
         <v>0</v>
@@ -23780,14 +23780,14 @@
       <c r="CE12">
         <v>0</v>
       </c>
-      <c r="CF12" t="str">
-        <v/>
+      <c r="CF12">
+        <v>0</v>
       </c>
       <c r="CG12" t="str">
         <v/>
       </c>
-      <c r="CH12">
-        <v>0</v>
+      <c r="CH12" t="str">
+        <v/>
       </c>
       <c r="CI12">
         <v>0</v>
@@ -23974,11 +23974,11 @@
       <c r="AV13">
         <v>0</v>
       </c>
-      <c r="AW13" t="str">
-        <v/>
-      </c>
-      <c r="AX13">
-        <v>0</v>
+      <c r="AW13">
+        <v>0</v>
+      </c>
+      <c r="AX13" t="str">
+        <v/>
       </c>
       <c r="AY13">
         <v>0</v>
@@ -24007,14 +24007,14 @@
       <c r="BG13">
         <v>0</v>
       </c>
-      <c r="BH13" t="str">
-        <v/>
+      <c r="BH13">
+        <v>0</v>
       </c>
       <c r="BI13" t="str">
         <v/>
       </c>
-      <c r="BJ13">
-        <v>0</v>
+      <c r="BJ13" t="str">
+        <v/>
       </c>
       <c r="BK13">
         <v>0</v>
@@ -24079,20 +24079,20 @@
       <c r="CE13">
         <v>0</v>
       </c>
-      <c r="CF13" t="str">
-        <v/>
+      <c r="CF13">
+        <v>0</v>
       </c>
       <c r="CG13" t="str">
         <v/>
       </c>
-      <c r="CH13">
-        <v>0</v>
-      </c>
-      <c r="CI13" t="str">
-        <v/>
-      </c>
-      <c r="CJ13">
-        <v>0</v>
+      <c r="CH13" t="str">
+        <v/>
+      </c>
+      <c r="CI13">
+        <v>0</v>
+      </c>
+      <c r="CJ13" t="str">
+        <v/>
       </c>
       <c r="CK13">
         <v>0</v>
@@ -24246,11 +24246,11 @@
       <c r="AM14">
         <v>0.81</v>
       </c>
-      <c r="AN14" t="str">
-        <v/>
-      </c>
-      <c r="AO14">
+      <c r="AN14">
         <v>0.16</v>
+      </c>
+      <c r="AO14" t="str">
+        <v/>
       </c>
       <c r="AP14">
         <v>0.16</v>
@@ -24273,11 +24273,11 @@
       <c r="AV14">
         <v>0.16</v>
       </c>
-      <c r="AW14" t="str">
-        <v/>
-      </c>
-      <c r="AX14">
+      <c r="AW14">
         <v>0.16</v>
+      </c>
+      <c r="AX14" t="str">
+        <v/>
       </c>
       <c r="AY14">
         <v>0.16</v>
@@ -24285,14 +24285,14 @@
       <c r="AZ14">
         <v>0.16</v>
       </c>
-      <c r="BA14" t="str">
-        <v/>
+      <c r="BA14">
+        <v>0.16</v>
       </c>
       <c r="BB14" t="str">
         <v/>
       </c>
-      <c r="BC14">
-        <v>0.16</v>
+      <c r="BC14" t="str">
+        <v/>
       </c>
       <c r="BD14">
         <v>0.16</v>
@@ -24300,14 +24300,14 @@
       <c r="BE14">
         <v>0.16</v>
       </c>
-      <c r="BF14" t="str">
-        <v/>
-      </c>
-      <c r="BG14">
+      <c r="BF14">
         <v>0.16</v>
       </c>
-      <c r="BH14" t="str">
-        <v/>
+      <c r="BG14" t="str">
+        <v/>
+      </c>
+      <c r="BH14">
+        <v>0.16</v>
       </c>
       <c r="BI14" t="str">
         <v/>
@@ -24315,104 +24315,104 @@
       <c r="BJ14" t="str">
         <v/>
       </c>
-      <c r="BK14">
+      <c r="BK14" t="str">
+        <v/>
+      </c>
+      <c r="BL14">
         <v>0.16</v>
       </c>
-      <c r="BL14" t="str">
-        <v/>
-      </c>
-      <c r="BM14">
+      <c r="BM14" t="str">
+        <v/>
+      </c>
+      <c r="BN14">
         <v>0.16</v>
       </c>
-      <c r="BN14" t="str">
-        <v/>
-      </c>
-      <c r="BO14">
+      <c r="BO14" t="str">
+        <v/>
+      </c>
+      <c r="BP14">
         <v>0.16</v>
       </c>
-      <c r="BP14" t="str">
-        <v/>
-      </c>
-      <c r="BQ14">
+      <c r="BQ14" t="str">
+        <v/>
+      </c>
+      <c r="BR14">
         <v>0.16</v>
       </c>
-      <c r="BR14" t="str">
-        <v/>
-      </c>
       <c r="BS14" t="str">
         <v/>
       </c>
-      <c r="BT14">
+      <c r="BT14" t="str">
+        <v/>
+      </c>
+      <c r="BU14">
         <v>0.16</v>
       </c>
-      <c r="BU14" t="str">
-        <v/>
-      </c>
-      <c r="BV14">
+      <c r="BV14" t="str">
+        <v/>
+      </c>
+      <c r="BW14">
         <v>0.16</v>
       </c>
-      <c r="BW14" t="str">
-        <v/>
-      </c>
       <c r="BX14" t="str">
         <v/>
       </c>
       <c r="BY14" t="str">
         <v/>
       </c>
-      <c r="BZ14">
+      <c r="BZ14" t="str">
+        <v/>
+      </c>
+      <c r="CA14">
         <v>0.16</v>
       </c>
-      <c r="CA14" t="str">
-        <v/>
-      </c>
-      <c r="CB14">
+      <c r="CB14" t="str">
+        <v/>
+      </c>
+      <c r="CC14">
         <v>0.16</v>
       </c>
-      <c r="CC14" t="str">
-        <v/>
-      </c>
-      <c r="CD14">
-        <v>0.16</v>
+      <c r="CD14" t="str">
+        <v/>
       </c>
       <c r="CE14">
         <v>0.16</v>
       </c>
-      <c r="CF14" t="str">
-        <v/>
+      <c r="CF14">
+        <v>0.16</v>
       </c>
       <c r="CG14" t="str">
         <v/>
       </c>
-      <c r="CH14">
+      <c r="CH14" t="str">
+        <v/>
+      </c>
+      <c r="CI14">
         <v>0.16</v>
       </c>
-      <c r="CI14" t="str">
-        <v/>
-      </c>
       <c r="CJ14" t="str">
         <v/>
       </c>
-      <c r="CK14">
-        <v>0.16</v>
+      <c r="CK14" t="str">
+        <v/>
       </c>
       <c r="CL14">
         <v>0.16</v>
       </c>
-      <c r="CM14" t="str">
-        <v/>
+      <c r="CM14">
+        <v>0.16</v>
       </c>
       <c r="CN14" t="str">
         <v/>
       </c>
-      <c r="CO14">
+      <c r="CO14" t="str">
+        <v/>
+      </c>
+      <c r="CP14">
         <v>0.16</v>
       </c>
-      <c r="CP14" t="str">
-        <v/>
-      </c>
-      <c r="CQ14">
-        <v>0.16</v>
+      <c r="CQ14" t="str">
+        <v/>
       </c>
       <c r="CR14">
         <v>0.16</v>
@@ -24551,19 +24551,19 @@
         <v>Brown, Christine 59375-66667 (60m)</v>
       </c>
       <c r="AL1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AM1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AN1" t="str">
         <v>Office Hours Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AM1" t="str">
+      <c r="AO1" t="str">
         <v>Office Hours Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AN1" t="str">
+      <c r="AP1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="AO1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="AP1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -24578,49 +24578,49 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AU1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AW1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="AX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AY1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AZ1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BA1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BB1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BA1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BB1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BC1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BD1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BE1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BF1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BG1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BH1" t="str">
         <v>Specialised Care Client 09:00-12:00 (420m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BI1" t="str">
         <v>Specialised Care Client 14:00-17:00 (420m)</v>
-      </c>
-      <c r="BH1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BI1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BJ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
@@ -24641,31 +24641,31 @@
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BP1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BQ1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BR1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BQ1" t="str">
+      <c r="BS1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BR1" t="str">
+      <c r="BT1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BS1" t="str">
+      <c r="BU1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (180m)</v>
-      </c>
-      <c r="BT1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BU1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BW1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BX1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BY1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
@@ -24674,19 +24674,19 @@
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
       <c r="CA1" t="str">
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="CB1" t="str">
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="CC1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="CB1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="CC1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="CD1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CE1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="CF1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -24698,7 +24698,7 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CI1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="CJ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -24888,17 +24888,17 @@
       <c r="BE2">
         <v>0.16</v>
       </c>
-      <c r="BF2" t="str">
-        <v/>
-      </c>
-      <c r="BG2" t="str">
-        <v/>
-      </c>
-      <c r="BH2">
+      <c r="BF2">
         <v>0.16</v>
       </c>
-      <c r="BI2">
+      <c r="BG2">
         <v>0.16</v>
+      </c>
+      <c r="BH2" t="str">
+        <v/>
+      </c>
+      <c r="BI2" t="str">
+        <v/>
       </c>
       <c r="BJ2">
         <v>0.16</v>
@@ -25166,17 +25166,17 @@
       <c r="BE3">
         <v>0</v>
       </c>
-      <c r="BF3" t="str">
-        <v/>
-      </c>
-      <c r="BG3" t="str">
-        <v/>
-      </c>
-      <c r="BH3">
-        <v>0</v>
-      </c>
-      <c r="BI3">
-        <v>0</v>
+      <c r="BF3">
+        <v>0</v>
+      </c>
+      <c r="BG3">
+        <v>0</v>
+      </c>
+      <c r="BH3" t="str">
+        <v/>
+      </c>
+      <c r="BI3" t="str">
+        <v/>
       </c>
       <c r="BJ3">
         <v>0</v>
@@ -25444,17 +25444,17 @@
       <c r="BE4">
         <v>0</v>
       </c>
-      <c r="BF4" t="str">
-        <v/>
-      </c>
-      <c r="BG4" t="str">
-        <v/>
-      </c>
-      <c r="BH4">
-        <v>0</v>
-      </c>
-      <c r="BI4">
-        <v>0</v>
+      <c r="BF4">
+        <v>0</v>
+      </c>
+      <c r="BG4">
+        <v>0</v>
+      </c>
+      <c r="BH4" t="str">
+        <v/>
+      </c>
+      <c r="BI4" t="str">
+        <v/>
       </c>
       <c r="BJ4">
         <v>0</v>
@@ -25665,14 +25665,14 @@
       <c r="AL5">
         <v>0</v>
       </c>
-      <c r="AM5" t="str">
-        <v/>
+      <c r="AM5">
+        <v>0</v>
       </c>
       <c r="AN5">
         <v>0</v>
       </c>
-      <c r="AO5">
-        <v>0</v>
+      <c r="AO5" t="str">
+        <v/>
       </c>
       <c r="AP5">
         <v>0</v>
@@ -25689,14 +25689,14 @@
       <c r="AT5">
         <v>0</v>
       </c>
-      <c r="AU5" t="str">
-        <v/>
+      <c r="AU5">
+        <v>0</v>
       </c>
       <c r="AV5">
         <v>0</v>
       </c>
-      <c r="AW5">
-        <v>0</v>
+      <c r="AW5" t="str">
+        <v/>
       </c>
       <c r="AX5">
         <v>0</v>
@@ -25719,17 +25719,17 @@
       <c r="BD5">
         <v>0</v>
       </c>
-      <c r="BE5" t="str">
-        <v/>
-      </c>
-      <c r="BF5" t="str">
-        <v/>
+      <c r="BE5">
+        <v>0</v>
+      </c>
+      <c r="BF5">
+        <v>0</v>
       </c>
       <c r="BG5" t="str">
         <v/>
       </c>
-      <c r="BH5">
-        <v>0</v>
+      <c r="BH5" t="str">
+        <v/>
       </c>
       <c r="BI5" t="str">
         <v/>
@@ -25755,17 +25755,17 @@
       <c r="BP5">
         <v>0</v>
       </c>
-      <c r="BQ5">
-        <v>0</v>
-      </c>
-      <c r="BR5" t="str">
-        <v/>
+      <c r="BQ5" t="str">
+        <v/>
+      </c>
+      <c r="BR5">
+        <v>0</v>
       </c>
       <c r="BS5">
         <v>0</v>
       </c>
-      <c r="BT5">
-        <v>0</v>
+      <c r="BT5" t="str">
+        <v/>
       </c>
       <c r="BU5">
         <v>0</v>
@@ -25776,8 +25776,8 @@
       <c r="BW5">
         <v>0</v>
       </c>
-      <c r="BX5" t="str">
-        <v/>
+      <c r="BX5">
+        <v>0</v>
       </c>
       <c r="BY5">
         <v>0</v>
@@ -25788,17 +25788,17 @@
       <c r="CA5">
         <v>0</v>
       </c>
-      <c r="CB5">
-        <v>0</v>
-      </c>
-      <c r="CC5" t="str">
-        <v/>
+      <c r="CB5" t="str">
+        <v/>
+      </c>
+      <c r="CC5">
+        <v>0</v>
       </c>
       <c r="CD5">
         <v>0</v>
       </c>
-      <c r="CE5">
-        <v>0</v>
+      <c r="CE5" t="str">
+        <v/>
       </c>
       <c r="CF5">
         <v>0</v>
@@ -26221,14 +26221,14 @@
       <c r="AL7">
         <v>0.05</v>
       </c>
-      <c r="AM7" t="str">
-        <v/>
+      <c r="AM7">
+        <v>0.05</v>
       </c>
       <c r="AN7">
         <v>0.05</v>
       </c>
-      <c r="AO7">
-        <v>0.05</v>
+      <c r="AO7" t="str">
+        <v/>
       </c>
       <c r="AP7">
         <v>0.05</v>
@@ -26245,14 +26245,14 @@
       <c r="AT7">
         <v>0.05</v>
       </c>
-      <c r="AU7" t="str">
-        <v/>
+      <c r="AU7">
+        <v>0.05</v>
       </c>
       <c r="AV7">
         <v>0.05</v>
       </c>
-      <c r="AW7">
-        <v>0.05</v>
+      <c r="AW7" t="str">
+        <v/>
       </c>
       <c r="AX7">
         <v>0.05</v>
@@ -26275,17 +26275,17 @@
       <c r="BD7">
         <v>0.05</v>
       </c>
-      <c r="BE7" t="str">
-        <v/>
-      </c>
-      <c r="BF7" t="str">
-        <v/>
+      <c r="BE7">
+        <v>0.05</v>
+      </c>
+      <c r="BF7">
+        <v>0.05</v>
       </c>
       <c r="BG7" t="str">
         <v/>
       </c>
-      <c r="BH7">
-        <v>0.05</v>
+      <c r="BH7" t="str">
+        <v/>
       </c>
       <c r="BI7" t="str">
         <v/>
@@ -26311,20 +26311,20 @@
       <c r="BP7">
         <v>0.05</v>
       </c>
-      <c r="BQ7">
+      <c r="BQ7" t="str">
+        <v/>
+      </c>
+      <c r="BR7">
         <v>0.05</v>
       </c>
-      <c r="BR7" t="str">
-        <v/>
-      </c>
-      <c r="BS7" t="str">
-        <v/>
-      </c>
-      <c r="BT7">
+      <c r="BS7">
         <v>0.05</v>
       </c>
-      <c r="BU7">
-        <v>0.05</v>
+      <c r="BT7" t="str">
+        <v/>
+      </c>
+      <c r="BU7" t="str">
+        <v/>
       </c>
       <c r="BV7">
         <v>0.05</v>
@@ -26332,8 +26332,8 @@
       <c r="BW7">
         <v>0.05</v>
       </c>
-      <c r="BX7" t="str">
-        <v/>
+      <c r="BX7">
+        <v>0.05</v>
       </c>
       <c r="BY7">
         <v>0.05</v>
@@ -26344,17 +26344,17 @@
       <c r="CA7">
         <v>0.05</v>
       </c>
-      <c r="CB7">
+      <c r="CB7" t="str">
+        <v/>
+      </c>
+      <c r="CC7">
         <v>0.05</v>
-      </c>
-      <c r="CC7" t="str">
-        <v/>
       </c>
       <c r="CD7">
         <v>0.05</v>
       </c>
-      <c r="CE7">
-        <v>0.05</v>
+      <c r="CE7" t="str">
+        <v/>
       </c>
       <c r="CF7">
         <v>0.05</v>
@@ -26499,14 +26499,14 @@
       <c r="AL8">
         <v>0.08</v>
       </c>
-      <c r="AM8" t="str">
-        <v/>
+      <c r="AM8">
+        <v>0.08</v>
       </c>
       <c r="AN8">
         <v>0.08</v>
       </c>
-      <c r="AO8">
-        <v>0.08</v>
+      <c r="AO8" t="str">
+        <v/>
       </c>
       <c r="AP8">
         <v>0.08</v>
@@ -26523,14 +26523,14 @@
       <c r="AT8">
         <v>0.08</v>
       </c>
-      <c r="AU8" t="str">
-        <v/>
+      <c r="AU8">
+        <v>0.08</v>
       </c>
       <c r="AV8">
         <v>0.08</v>
       </c>
-      <c r="AW8">
-        <v>0.08</v>
+      <c r="AW8" t="str">
+        <v/>
       </c>
       <c r="AX8">
         <v>0.08</v>
@@ -26553,17 +26553,17 @@
       <c r="BD8">
         <v>0.08</v>
       </c>
-      <c r="BE8" t="str">
-        <v/>
-      </c>
-      <c r="BF8" t="str">
-        <v/>
+      <c r="BE8">
+        <v>0.08</v>
+      </c>
+      <c r="BF8">
+        <v>0.08</v>
       </c>
       <c r="BG8" t="str">
         <v/>
       </c>
-      <c r="BH8">
-        <v>0.08</v>
+      <c r="BH8" t="str">
+        <v/>
       </c>
       <c r="BI8" t="str">
         <v/>
@@ -26589,17 +26589,17 @@
       <c r="BP8">
         <v>0.08</v>
       </c>
-      <c r="BQ8">
+      <c r="BQ8" t="str">
+        <v/>
+      </c>
+      <c r="BR8">
         <v>0.08</v>
-      </c>
-      <c r="BR8" t="str">
-        <v/>
       </c>
       <c r="BS8">
         <v>0.08</v>
       </c>
-      <c r="BT8">
-        <v>0.08</v>
+      <c r="BT8" t="str">
+        <v/>
       </c>
       <c r="BU8">
         <v>0.08</v>
@@ -26610,8 +26610,8 @@
       <c r="BW8">
         <v>0.08</v>
       </c>
-      <c r="BX8" t="str">
-        <v/>
+      <c r="BX8">
+        <v>0.08</v>
       </c>
       <c r="BY8">
         <v>0.08</v>
@@ -26622,17 +26622,17 @@
       <c r="CA8">
         <v>0.08</v>
       </c>
-      <c r="CB8">
+      <c r="CB8" t="str">
+        <v/>
+      </c>
+      <c r="CC8">
         <v>0.08</v>
-      </c>
-      <c r="CC8" t="str">
-        <v/>
       </c>
       <c r="CD8">
         <v>0.08</v>
       </c>
-      <c r="CE8">
-        <v>0.08</v>
+      <c r="CE8" t="str">
+        <v/>
       </c>
       <c r="CF8">
         <v>0.08</v>
@@ -26777,14 +26777,14 @@
       <c r="AL9">
         <v>0</v>
       </c>
-      <c r="AM9" t="str">
-        <v/>
+      <c r="AM9">
+        <v>0</v>
       </c>
       <c r="AN9">
         <v>0</v>
       </c>
-      <c r="AO9">
-        <v>0</v>
+      <c r="AO9" t="str">
+        <v/>
       </c>
       <c r="AP9">
         <v>0</v>
@@ -26831,17 +26831,17 @@
       <c r="BD9">
         <v>0</v>
       </c>
-      <c r="BE9" t="str">
-        <v/>
-      </c>
-      <c r="BF9" t="str">
-        <v/>
+      <c r="BE9">
+        <v>0</v>
+      </c>
+      <c r="BF9">
+        <v>0</v>
       </c>
       <c r="BG9" t="str">
         <v/>
       </c>
-      <c r="BH9">
-        <v>0</v>
+      <c r="BH9" t="str">
+        <v/>
       </c>
       <c r="BI9" t="str">
         <v/>
@@ -26867,17 +26867,17 @@
       <c r="BP9">
         <v>0</v>
       </c>
-      <c r="BQ9">
-        <v>0</v>
-      </c>
-      <c r="BR9" t="str">
-        <v/>
+      <c r="BQ9" t="str">
+        <v/>
+      </c>
+      <c r="BR9">
+        <v>0</v>
       </c>
       <c r="BS9">
         <v>0</v>
       </c>
-      <c r="BT9">
-        <v>0</v>
+      <c r="BT9" t="str">
+        <v/>
       </c>
       <c r="BU9">
         <v>0</v>
@@ -26888,8 +26888,8 @@
       <c r="BW9">
         <v>0</v>
       </c>
-      <c r="BX9" t="str">
-        <v/>
+      <c r="BX9">
+        <v>0</v>
       </c>
       <c r="BY9">
         <v>0</v>
@@ -26900,8 +26900,8 @@
       <c r="CA9">
         <v>0</v>
       </c>
-      <c r="CB9">
-        <v>0</v>
+      <c r="CB9" t="str">
+        <v/>
       </c>
       <c r="CC9">
         <v>0</v>
@@ -27112,17 +27112,17 @@
       <c r="BE10">
         <v>0.1</v>
       </c>
-      <c r="BF10" t="str">
-        <v/>
-      </c>
-      <c r="BG10" t="str">
-        <v/>
-      </c>
-      <c r="BH10">
+      <c r="BF10">
         <v>0.1</v>
       </c>
-      <c r="BI10">
+      <c r="BG10">
         <v>0.1</v>
+      </c>
+      <c r="BH10" t="str">
+        <v/>
+      </c>
+      <c r="BI10" t="str">
+        <v/>
       </c>
       <c r="BJ10">
         <v>0.1</v>
@@ -27390,17 +27390,17 @@
       <c r="BE11">
         <v>0.01</v>
       </c>
-      <c r="BF11" t="str">
-        <v/>
-      </c>
-      <c r="BG11" t="str">
-        <v/>
-      </c>
-      <c r="BH11">
+      <c r="BF11">
         <v>0.01</v>
       </c>
-      <c r="BI11">
+      <c r="BG11">
         <v>0.01</v>
+      </c>
+      <c r="BH11" t="str">
+        <v/>
+      </c>
+      <c r="BI11" t="str">
+        <v/>
       </c>
       <c r="BJ11">
         <v>0.01</v>
@@ -27668,17 +27668,17 @@
       <c r="BE12">
         <v>0</v>
       </c>
-      <c r="BF12" t="str">
-        <v/>
-      </c>
-      <c r="BG12" t="str">
-        <v/>
-      </c>
-      <c r="BH12">
-        <v>0</v>
-      </c>
-      <c r="BI12">
-        <v>0</v>
+      <c r="BF12">
+        <v>0</v>
+      </c>
+      <c r="BG12">
+        <v>0</v>
+      </c>
+      <c r="BH12" t="str">
+        <v/>
+      </c>
+      <c r="BI12" t="str">
+        <v/>
       </c>
       <c r="BJ12">
         <v>0</v>
@@ -27946,17 +27946,17 @@
       <c r="BE13">
         <v>0</v>
       </c>
-      <c r="BF13" t="str">
-        <v/>
-      </c>
-      <c r="BG13" t="str">
-        <v/>
-      </c>
-      <c r="BH13">
-        <v>0</v>
-      </c>
-      <c r="BI13">
-        <v>0</v>
+      <c r="BF13">
+        <v>0</v>
+      </c>
+      <c r="BG13">
+        <v>0</v>
+      </c>
+      <c r="BH13" t="str">
+        <v/>
+      </c>
+      <c r="BI13" t="str">
+        <v/>
       </c>
       <c r="BJ13">
         <v>0</v>
@@ -28173,10 +28173,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AK1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (285m)</v>
-      </c>
-      <c r="AL1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AM1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -28200,13 +28200,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AT1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AU1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AV1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AW1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -28215,82 +28215,82 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AY1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AZ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BA1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BA1" t="str">
+      <c r="BB1" t="str">
         <v>Specialised Care Client 09:00-12:00 (360m)</v>
       </c>
-      <c r="BB1" t="str">
+      <c r="BC1" t="str">
         <v>Specialised Care Client 14:00-17:00 (360m)</v>
       </c>
-      <c r="BC1" t="str">
+      <c r="BD1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BD1" t="str">
+      <c r="BE1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BF1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BG1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BH1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BI1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BJ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (240m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BK1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BK1" t="str">
+      <c r="BL1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BL1" t="str">
+      <c r="BM1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BM1" t="str">
+      <c r="BN1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BN1" t="str">
+      <c r="BO1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BO1" t="str">
+      <c r="BP1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BP1" t="str">
+      <c r="BQ1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BQ1" t="str">
+      <c r="BR1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BR1" t="str">
+      <c r="BS1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BS1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BU1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (180m)</v>
       </c>
-      <c r="BV1" t="str">
+      <c r="BW1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
-      <c r="BW1" t="str">
+      <c r="BX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BX1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BY1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -28471,14 +28471,14 @@
       <c r="AZ2">
         <v>0.25</v>
       </c>
-      <c r="BA2" t="str">
-        <v/>
+      <c r="BA2">
+        <v>0.25</v>
       </c>
       <c r="BB2" t="str">
         <v/>
       </c>
-      <c r="BC2">
-        <v>0.25</v>
+      <c r="BC2" t="str">
+        <v/>
       </c>
       <c r="BD2">
         <v>0.25</v>
@@ -28674,11 +28674,11 @@
       <c r="AJ3">
         <v>0.07</v>
       </c>
-      <c r="AK3" t="str">
-        <v/>
-      </c>
-      <c r="AL3">
+      <c r="AK3">
         <v>0.07</v>
+      </c>
+      <c r="AL3" t="str">
+        <v/>
       </c>
       <c r="AM3">
         <v>0.07</v>
@@ -28719,8 +28719,8 @@
       <c r="AY3">
         <v>0.07</v>
       </c>
-      <c r="AZ3" t="str">
-        <v/>
+      <c r="AZ3">
+        <v>0.07</v>
       </c>
       <c r="BA3" t="str">
         <v/>
@@ -28728,56 +28728,56 @@
       <c r="BB3" t="str">
         <v/>
       </c>
-      <c r="BC3">
+      <c r="BC3" t="str">
+        <v/>
+      </c>
+      <c r="BD3">
         <v>0.07</v>
       </c>
-      <c r="BD3" t="str">
-        <v/>
-      </c>
-      <c r="BE3">
+      <c r="BE3" t="str">
+        <v/>
+      </c>
+      <c r="BF3">
         <v>0.07</v>
       </c>
-      <c r="BF3" t="str">
-        <v/>
-      </c>
-      <c r="BG3">
+      <c r="BG3" t="str">
+        <v/>
+      </c>
+      <c r="BH3">
         <v>0.07</v>
       </c>
-      <c r="BH3" t="str">
-        <v/>
-      </c>
       <c r="BI3" t="str">
         <v/>
       </c>
-      <c r="BJ3">
+      <c r="BJ3" t="str">
+        <v/>
+      </c>
+      <c r="BK3">
         <v>0.07</v>
       </c>
-      <c r="BK3" t="str">
-        <v/>
-      </c>
-      <c r="BL3">
+      <c r="BL3" t="str">
+        <v/>
+      </c>
+      <c r="BM3">
         <v>0.07</v>
       </c>
-      <c r="BM3" t="str">
-        <v/>
-      </c>
-      <c r="BN3">
-        <v>0.07</v>
+      <c r="BN3" t="str">
+        <v/>
       </c>
       <c r="BO3">
         <v>0.07</v>
       </c>
-      <c r="BP3" t="str">
-        <v/>
-      </c>
-      <c r="BQ3">
+      <c r="BP3">
         <v>0.07</v>
       </c>
-      <c r="BR3" t="str">
-        <v/>
-      </c>
-      <c r="BS3">
+      <c r="BQ3" t="str">
+        <v/>
+      </c>
+      <c r="BR3">
         <v>0.07</v>
+      </c>
+      <c r="BS3" t="str">
+        <v/>
       </c>
       <c r="BT3">
         <v>0.07</v>
@@ -28785,11 +28785,11 @@
       <c r="BU3">
         <v>0.07</v>
       </c>
-      <c r="BV3" t="str">
-        <v/>
-      </c>
-      <c r="BW3">
+      <c r="BV3">
         <v>0.07</v>
+      </c>
+      <c r="BW3" t="str">
+        <v/>
       </c>
       <c r="BX3">
         <v>0.07</v>
@@ -28925,11 +28925,11 @@
       <c r="AJ4">
         <v>0.13</v>
       </c>
-      <c r="AK4" t="str">
-        <v/>
-      </c>
-      <c r="AL4">
+      <c r="AK4">
         <v>0.13</v>
+      </c>
+      <c r="AL4" t="str">
+        <v/>
       </c>
       <c r="AM4">
         <v>0.13</v>
@@ -28970,8 +28970,8 @@
       <c r="AY4">
         <v>0.13</v>
       </c>
-      <c r="AZ4" t="str">
-        <v/>
+      <c r="AZ4">
+        <v>0.13</v>
       </c>
       <c r="BA4" t="str">
         <v/>
@@ -28979,56 +28979,56 @@
       <c r="BB4" t="str">
         <v/>
       </c>
-      <c r="BC4">
+      <c r="BC4" t="str">
+        <v/>
+      </c>
+      <c r="BD4">
         <v>0.13</v>
       </c>
-      <c r="BD4" t="str">
-        <v/>
-      </c>
-      <c r="BE4">
+      <c r="BE4" t="str">
+        <v/>
+      </c>
+      <c r="BF4">
         <v>0.13</v>
       </c>
-      <c r="BF4" t="str">
-        <v/>
-      </c>
-      <c r="BG4">
+      <c r="BG4" t="str">
+        <v/>
+      </c>
+      <c r="BH4">
         <v>0.13</v>
       </c>
-      <c r="BH4" t="str">
-        <v/>
-      </c>
       <c r="BI4" t="str">
         <v/>
       </c>
-      <c r="BJ4">
+      <c r="BJ4" t="str">
+        <v/>
+      </c>
+      <c r="BK4">
         <v>0.13</v>
       </c>
-      <c r="BK4" t="str">
-        <v/>
-      </c>
-      <c r="BL4">
+      <c r="BL4" t="str">
+        <v/>
+      </c>
+      <c r="BM4">
         <v>0.13</v>
       </c>
-      <c r="BM4" t="str">
-        <v/>
-      </c>
-      <c r="BN4">
-        <v>0.13</v>
+      <c r="BN4" t="str">
+        <v/>
       </c>
       <c r="BO4">
         <v>0.13</v>
       </c>
-      <c r="BP4" t="str">
-        <v/>
-      </c>
-      <c r="BQ4">
+      <c r="BP4">
         <v>0.13</v>
       </c>
-      <c r="BR4" t="str">
-        <v/>
-      </c>
-      <c r="BS4">
+      <c r="BQ4" t="str">
+        <v/>
+      </c>
+      <c r="BR4">
         <v>0.13</v>
+      </c>
+      <c r="BS4" t="str">
+        <v/>
       </c>
       <c r="BT4">
         <v>0.13</v>
@@ -29036,11 +29036,11 @@
       <c r="BU4">
         <v>0.13</v>
       </c>
-      <c r="BV4" t="str">
-        <v/>
-      </c>
-      <c r="BW4">
+      <c r="BV4">
         <v>0.13</v>
+      </c>
+      <c r="BW4" t="str">
+        <v/>
       </c>
       <c r="BX4">
         <v>0.13</v>
@@ -29176,11 +29176,11 @@
       <c r="AJ5">
         <v>0.78</v>
       </c>
-      <c r="AK5" t="str">
-        <v/>
-      </c>
-      <c r="AL5">
+      <c r="AK5">
         <v>0.78</v>
+      </c>
+      <c r="AL5" t="str">
+        <v/>
       </c>
       <c r="AM5">
         <v>0.78</v>
@@ -29221,8 +29221,8 @@
       <c r="AY5">
         <v>0.78</v>
       </c>
-      <c r="AZ5" t="str">
-        <v/>
+      <c r="AZ5">
+        <v>0.78</v>
       </c>
       <c r="BA5" t="str">
         <v/>
@@ -29230,56 +29230,56 @@
       <c r="BB5" t="str">
         <v/>
       </c>
-      <c r="BC5">
+      <c r="BC5" t="str">
+        <v/>
+      </c>
+      <c r="BD5">
         <v>0.78</v>
       </c>
-      <c r="BD5" t="str">
-        <v/>
-      </c>
-      <c r="BE5">
+      <c r="BE5" t="str">
+        <v/>
+      </c>
+      <c r="BF5">
         <v>0.78</v>
       </c>
-      <c r="BF5" t="str">
-        <v/>
-      </c>
-      <c r="BG5">
+      <c r="BG5" t="str">
+        <v/>
+      </c>
+      <c r="BH5">
         <v>0.78</v>
       </c>
-      <c r="BH5" t="str">
-        <v/>
-      </c>
-      <c r="BI5">
-        <v>0.78</v>
+      <c r="BI5" t="str">
+        <v/>
       </c>
       <c r="BJ5">
         <v>0.78</v>
       </c>
-      <c r="BK5" t="str">
-        <v/>
-      </c>
-      <c r="BL5">
+      <c r="BK5">
         <v>0.78</v>
       </c>
-      <c r="BM5" t="str">
-        <v/>
-      </c>
-      <c r="BN5">
+      <c r="BL5" t="str">
+        <v/>
+      </c>
+      <c r="BM5">
         <v>0.78</v>
+      </c>
+      <c r="BN5" t="str">
+        <v/>
       </c>
       <c r="BO5">
         <v>0.78</v>
       </c>
-      <c r="BP5" t="str">
-        <v/>
-      </c>
-      <c r="BQ5">
+      <c r="BP5">
         <v>0.78</v>
       </c>
-      <c r="BR5" t="str">
-        <v/>
-      </c>
-      <c r="BS5">
+      <c r="BQ5" t="str">
+        <v/>
+      </c>
+      <c r="BR5">
         <v>0.78</v>
+      </c>
+      <c r="BS5" t="str">
+        <v/>
       </c>
       <c r="BT5">
         <v>0.78</v>
@@ -29287,11 +29287,11 @@
       <c r="BU5">
         <v>0.78</v>
       </c>
-      <c r="BV5" t="str">
-        <v/>
-      </c>
-      <c r="BW5">
+      <c r="BV5">
         <v>0.78</v>
+      </c>
+      <c r="BW5" t="str">
+        <v/>
       </c>
       <c r="BX5">
         <v>0.78</v>
@@ -29977,14 +29977,14 @@
       <c r="AZ8">
         <v>0.25</v>
       </c>
-      <c r="BA8" t="str">
-        <v/>
+      <c r="BA8">
+        <v>0.25</v>
       </c>
       <c r="BB8" t="str">
         <v/>
       </c>
-      <c r="BC8">
-        <v>0.25</v>
+      <c r="BC8" t="str">
+        <v/>
       </c>
       <c r="BD8">
         <v>0.25</v>
@@ -30180,11 +30180,11 @@
       <c r="AJ9">
         <v>0.08</v>
       </c>
-      <c r="AK9" t="str">
-        <v/>
-      </c>
-      <c r="AL9">
+      <c r="AK9">
         <v>0.08</v>
+      </c>
+      <c r="AL9" t="str">
+        <v/>
       </c>
       <c r="AM9">
         <v>0.08</v>
@@ -30225,8 +30225,8 @@
       <c r="AY9">
         <v>0.08</v>
       </c>
-      <c r="AZ9" t="str">
-        <v/>
+      <c r="AZ9">
+        <v>0.08</v>
       </c>
       <c r="BA9" t="str">
         <v/>
@@ -30234,56 +30234,56 @@
       <c r="BB9" t="str">
         <v/>
       </c>
-      <c r="BC9">
+      <c r="BC9" t="str">
+        <v/>
+      </c>
+      <c r="BD9">
         <v>0.08</v>
       </c>
-      <c r="BD9" t="str">
-        <v/>
-      </c>
-      <c r="BE9">
+      <c r="BE9" t="str">
+        <v/>
+      </c>
+      <c r="BF9">
         <v>0.08</v>
       </c>
-      <c r="BF9" t="str">
-        <v/>
-      </c>
-      <c r="BG9">
+      <c r="BG9" t="str">
+        <v/>
+      </c>
+      <c r="BH9">
         <v>0.08</v>
       </c>
-      <c r="BH9" t="str">
-        <v/>
-      </c>
-      <c r="BI9">
-        <v>0.08</v>
+      <c r="BI9" t="str">
+        <v/>
       </c>
       <c r="BJ9">
         <v>0.08</v>
       </c>
-      <c r="BK9" t="str">
-        <v/>
-      </c>
-      <c r="BL9">
+      <c r="BK9">
         <v>0.08</v>
       </c>
-      <c r="BM9" t="str">
-        <v/>
-      </c>
-      <c r="BN9">
+      <c r="BL9" t="str">
+        <v/>
+      </c>
+      <c r="BM9">
         <v>0.08</v>
+      </c>
+      <c r="BN9" t="str">
+        <v/>
       </c>
       <c r="BO9">
         <v>0.08</v>
       </c>
-      <c r="BP9" t="str">
-        <v/>
-      </c>
-      <c r="BQ9">
+      <c r="BP9">
         <v>0.08</v>
       </c>
-      <c r="BR9" t="str">
-        <v/>
-      </c>
-      <c r="BS9">
+      <c r="BQ9" t="str">
+        <v/>
+      </c>
+      <c r="BR9">
         <v>0.08</v>
+      </c>
+      <c r="BS9" t="str">
+        <v/>
       </c>
       <c r="BT9">
         <v>0.08</v>
@@ -30291,11 +30291,11 @@
       <c r="BU9">
         <v>0.08</v>
       </c>
-      <c r="BV9" t="str">
-        <v/>
-      </c>
-      <c r="BW9">
+      <c r="BV9">
         <v>0.08</v>
+      </c>
+      <c r="BW9" t="str">
+        <v/>
       </c>
       <c r="BX9">
         <v>0.08</v>
@@ -30476,8 +30476,8 @@
       <c r="AY10">
         <v>0</v>
       </c>
-      <c r="AZ10" t="str">
-        <v/>
+      <c r="AZ10">
+        <v>0</v>
       </c>
       <c r="BA10" t="str">
         <v/>
@@ -30485,56 +30485,56 @@
       <c r="BB10" t="str">
         <v/>
       </c>
-      <c r="BC10">
-        <v>0</v>
-      </c>
-      <c r="BD10" t="str">
-        <v/>
-      </c>
-      <c r="BE10">
-        <v>0</v>
-      </c>
-      <c r="BF10" t="str">
-        <v/>
-      </c>
-      <c r="BG10">
-        <v>0</v>
-      </c>
-      <c r="BH10" t="str">
-        <v/>
-      </c>
-      <c r="BI10">
-        <v>0</v>
+      <c r="BC10" t="str">
+        <v/>
+      </c>
+      <c r="BD10">
+        <v>0</v>
+      </c>
+      <c r="BE10" t="str">
+        <v/>
+      </c>
+      <c r="BF10">
+        <v>0</v>
+      </c>
+      <c r="BG10" t="str">
+        <v/>
+      </c>
+      <c r="BH10">
+        <v>0</v>
+      </c>
+      <c r="BI10" t="str">
+        <v/>
       </c>
       <c r="BJ10">
         <v>0</v>
       </c>
-      <c r="BK10" t="str">
-        <v/>
-      </c>
-      <c r="BL10">
-        <v>0</v>
-      </c>
-      <c r="BM10" t="str">
-        <v/>
-      </c>
-      <c r="BN10">
-        <v>0</v>
+      <c r="BK10">
+        <v>0</v>
+      </c>
+      <c r="BL10" t="str">
+        <v/>
+      </c>
+      <c r="BM10">
+        <v>0</v>
+      </c>
+      <c r="BN10" t="str">
+        <v/>
       </c>
       <c r="BO10">
         <v>0</v>
       </c>
-      <c r="BP10" t="str">
-        <v/>
-      </c>
-      <c r="BQ10">
-        <v>0</v>
-      </c>
-      <c r="BR10" t="str">
-        <v/>
-      </c>
-      <c r="BS10">
-        <v>0</v>
+      <c r="BP10">
+        <v>0</v>
+      </c>
+      <c r="BQ10" t="str">
+        <v/>
+      </c>
+      <c r="BR10">
+        <v>0</v>
+      </c>
+      <c r="BS10" t="str">
+        <v/>
       </c>
       <c r="BT10">
         <v>0</v>
@@ -30730,14 +30730,14 @@
       <c r="AZ11">
         <v>0.1</v>
       </c>
-      <c r="BA11" t="str">
-        <v/>
+      <c r="BA11">
+        <v>0.1</v>
       </c>
       <c r="BB11" t="str">
         <v/>
       </c>
-      <c r="BC11">
-        <v>0.1</v>
+      <c r="BC11" t="str">
+        <v/>
       </c>
       <c r="BD11">
         <v>0.1</v>
@@ -30981,14 +30981,14 @@
       <c r="AZ12">
         <v>0</v>
       </c>
-      <c r="BA12" t="str">
-        <v/>
+      <c r="BA12">
+        <v>0</v>
       </c>
       <c r="BB12" t="str">
         <v/>
       </c>
-      <c r="BC12">
-        <v>0</v>
+      <c r="BC12" t="str">
+        <v/>
       </c>
       <c r="BD12">
         <v>0</v>
@@ -31232,14 +31232,14 @@
       <c r="AZ13">
         <v>0.14</v>
       </c>
-      <c r="BA13" t="str">
-        <v/>
+      <c r="BA13">
+        <v>0.14</v>
       </c>
       <c r="BB13" t="str">
         <v/>
       </c>
-      <c r="BC13">
-        <v>0.14</v>
+      <c r="BC13" t="str">
+        <v/>
       </c>
       <c r="BD13">
         <v>0.14</v>
@@ -31483,14 +31483,14 @@
       <c r="AZ14">
         <v>0</v>
       </c>
-      <c r="BA14" t="str">
-        <v/>
+      <c r="BA14">
+        <v>0</v>
       </c>
       <c r="BB14" t="str">
         <v/>
       </c>
-      <c r="BC14">
-        <v>0</v>
+      <c r="BC14" t="str">
+        <v/>
       </c>
       <c r="BD14">
         <v>0</v>
@@ -31686,11 +31686,11 @@
       <c r="AJ15">
         <v>0</v>
       </c>
-      <c r="AK15" t="str">
-        <v/>
-      </c>
-      <c r="AL15">
-        <v>0</v>
+      <c r="AK15">
+        <v>0</v>
+      </c>
+      <c r="AL15" t="str">
+        <v/>
       </c>
       <c r="AM15">
         <v>0</v>
@@ -31734,14 +31734,14 @@
       <c r="AZ15">
         <v>0</v>
       </c>
-      <c r="BA15" t="str">
-        <v/>
+      <c r="BA15">
+        <v>0</v>
       </c>
       <c r="BB15" t="str">
         <v/>
       </c>
-      <c r="BC15">
-        <v>0</v>
+      <c r="BC15" t="str">
+        <v/>
       </c>
       <c r="BD15">
         <v>0</v>
@@ -31797,11 +31797,11 @@
       <c r="BU15">
         <v>0</v>
       </c>
-      <c r="BV15" t="str">
-        <v/>
-      </c>
-      <c r="BW15">
-        <v>0</v>
+      <c r="BV15">
+        <v>0</v>
+      </c>
+      <c r="BW15" t="str">
+        <v/>
       </c>
       <c r="BX15">
         <v>0</v>
@@ -31985,14 +31985,14 @@
       <c r="AZ16">
         <v>0.09</v>
       </c>
-      <c r="BA16" t="str">
-        <v/>
+      <c r="BA16">
+        <v>0.09</v>
       </c>
       <c r="BB16" t="str">
         <v/>
       </c>
-      <c r="BC16">
-        <v>0.09</v>
+      <c r="BC16" t="str">
+        <v/>
       </c>
       <c r="BD16">
         <v>0.09</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update schedule to assign visits directly from Excel file
Replace database scheduling with direct assignment from the Excel file.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3693,16 +3693,16 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AE1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="AF1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="AF1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
       <c r="AG1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AH1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (165m)</v>
       </c>
       <c r="AI1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -3711,7 +3711,7 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AK1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -3720,16 +3720,16 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AN1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (165m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AO1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AP1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AQ1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AR1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -3738,67 +3738,67 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AT1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AU1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AU1" t="str">
+      <c r="AV1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AV1" t="str">
+      <c r="AW1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AW1" t="str">
+      <c r="AX1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AX1" t="str">
+      <c r="AY1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AY1" t="str">
+      <c r="AZ1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BA1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BA1" t="str">
+      <c r="BB1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BB1" t="str">
+      <c r="BC1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BC1" t="str">
+      <c r="BD1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BD1" t="str">
+      <c r="BE1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BF1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BG1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BH1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BI1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BJ1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BK1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BK1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BM1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BN1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BO1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -3810,10 +3810,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BR1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BS1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BS1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -6566,13 +6566,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AB1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AC1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AD1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (240m)</v>
       </c>
       <c r="AE1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -6590,16 +6590,16 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AJ1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (240m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AK1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AL1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AM1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -6608,58 +6608,58 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AP1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AQ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AQ1" t="str">
+      <c r="AR1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AR1" t="str">
+      <c r="AS1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AS1" t="str">
+      <c r="AT1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AT1" t="str">
+      <c r="AU1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AU1" t="str">
+      <c r="AV1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AV1" t="str">
+      <c r="AW1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AW1" t="str">
+      <c r="AX1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AX1" t="str">
+      <c r="AY1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AY1" t="str">
+      <c r="AZ1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BA1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BA1" t="str">
+      <c r="BB1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BB1" t="str">
+      <c r="BC1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BC1" t="str">
+      <c r="BD1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BD1" t="str">
+      <c r="BE1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BF1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BG1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BG1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BH1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -6668,16 +6668,16 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BJ1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BK1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
-      <c r="BK1" t="str">
+      <c r="BL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BL1" t="str">
+      <c r="BM1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (180m)</v>
-      </c>
-      <c r="BM1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -7022,56 +7022,56 @@
       <c r="AP3">
         <v>0</v>
       </c>
-      <c r="AQ3" t="str">
-        <v/>
-      </c>
-      <c r="AR3">
-        <v>0</v>
-      </c>
-      <c r="AS3" t="str">
-        <v/>
-      </c>
-      <c r="AT3">
-        <v>0</v>
-      </c>
-      <c r="AU3" t="str">
-        <v/>
-      </c>
-      <c r="AV3">
-        <v>0</v>
-      </c>
-      <c r="AW3" t="str">
-        <v/>
-      </c>
-      <c r="AX3">
-        <v>0</v>
-      </c>
-      <c r="AY3" t="str">
-        <v/>
-      </c>
-      <c r="AZ3">
-        <v>0</v>
-      </c>
-      <c r="BA3" t="str">
-        <v/>
-      </c>
-      <c r="BB3">
-        <v>0</v>
-      </c>
-      <c r="BC3" t="str">
-        <v/>
-      </c>
-      <c r="BD3">
-        <v>0</v>
+      <c r="AQ3">
+        <v>0</v>
+      </c>
+      <c r="AR3" t="str">
+        <v/>
+      </c>
+      <c r="AS3">
+        <v>0</v>
+      </c>
+      <c r="AT3" t="str">
+        <v/>
+      </c>
+      <c r="AU3">
+        <v>0</v>
+      </c>
+      <c r="AV3" t="str">
+        <v/>
+      </c>
+      <c r="AW3">
+        <v>0</v>
+      </c>
+      <c r="AX3" t="str">
+        <v/>
+      </c>
+      <c r="AY3">
+        <v>0</v>
+      </c>
+      <c r="AZ3" t="str">
+        <v/>
+      </c>
+      <c r="BA3">
+        <v>0</v>
+      </c>
+      <c r="BB3" t="str">
+        <v/>
+      </c>
+      <c r="BC3">
+        <v>0</v>
+      </c>
+      <c r="BD3" t="str">
+        <v/>
       </c>
       <c r="BE3">
         <v>0</v>
       </c>
-      <c r="BF3" t="str">
-        <v/>
-      </c>
-      <c r="BG3">
-        <v>0</v>
+      <c r="BF3">
+        <v>0</v>
+      </c>
+      <c r="BG3" t="str">
+        <v/>
       </c>
       <c r="BH3">
         <v>0</v>
@@ -8013,8 +8013,8 @@
       <c r="AC8">
         <v>0.78</v>
       </c>
-      <c r="AD8">
-        <v>0.78</v>
+      <c r="AD8" t="str">
+        <v/>
       </c>
       <c r="AE8">
         <v>0.78</v>
@@ -8031,8 +8031,8 @@
       <c r="AI8">
         <v>0.78</v>
       </c>
-      <c r="AJ8" t="str">
-        <v/>
+      <c r="AJ8">
+        <v>0.78</v>
       </c>
       <c r="AK8">
         <v>0.78</v>
@@ -8052,56 +8052,56 @@
       <c r="AP8">
         <v>0.78</v>
       </c>
-      <c r="AQ8" t="str">
-        <v/>
-      </c>
-      <c r="AR8">
+      <c r="AQ8">
         <v>0.78</v>
       </c>
-      <c r="AS8" t="str">
-        <v/>
-      </c>
-      <c r="AT8">
+      <c r="AR8" t="str">
+        <v/>
+      </c>
+      <c r="AS8">
         <v>0.78</v>
       </c>
-      <c r="AU8" t="str">
-        <v/>
-      </c>
-      <c r="AV8">
+      <c r="AT8" t="str">
+        <v/>
+      </c>
+      <c r="AU8">
         <v>0.78</v>
       </c>
-      <c r="AW8" t="str">
-        <v/>
-      </c>
-      <c r="AX8">
+      <c r="AV8" t="str">
+        <v/>
+      </c>
+      <c r="AW8">
         <v>0.78</v>
       </c>
-      <c r="AY8" t="str">
-        <v/>
-      </c>
-      <c r="AZ8">
+      <c r="AX8" t="str">
+        <v/>
+      </c>
+      <c r="AY8">
         <v>0.78</v>
       </c>
-      <c r="BA8" t="str">
-        <v/>
-      </c>
-      <c r="BB8">
+      <c r="AZ8" t="str">
+        <v/>
+      </c>
+      <c r="BA8">
         <v>0.78</v>
       </c>
-      <c r="BC8" t="str">
-        <v/>
-      </c>
-      <c r="BD8">
+      <c r="BB8" t="str">
+        <v/>
+      </c>
+      <c r="BC8">
         <v>0.78</v>
+      </c>
+      <c r="BD8" t="str">
+        <v/>
       </c>
       <c r="BE8">
         <v>0.78</v>
       </c>
-      <c r="BF8" t="str">
-        <v/>
-      </c>
-      <c r="BG8">
+      <c r="BF8">
         <v>0.78</v>
+      </c>
+      <c r="BG8" t="str">
+        <v/>
       </c>
       <c r="BH8">
         <v>0.78</v>
@@ -16859,10 +16859,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AH1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AI1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AJ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -16874,52 +16874,52 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AM1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AN1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AO1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AP1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="AQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AR1" t="str">
-        <v>Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AS1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
-      <c r="AT1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
       <c r="AU1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AW1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AX1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AY1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AX1" t="str">
+      <c r="AZ1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AY1" t="str">
+      <c r="BA1" t="str">
         <v>Specialised Care Client 09:00-12:00 (420m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BB1" t="str">
         <v>Specialised Care Client 14:00-17:00 (420m)</v>
-      </c>
-      <c r="BA1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BB1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BC1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
@@ -16934,22 +16934,22 @@
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BG1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BH1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BI1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BJ1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BK1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BL1" t="str">
         <v>Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BK1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BL1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BM1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
@@ -16958,22 +16958,22 @@
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BO1" t="str">
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BP1" t="str">
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BP1" t="str">
+      <c r="BR1" t="str">
         <v>Office Hours Client 09:00-12:00 (510m)</v>
       </c>
-      <c r="BQ1" t="str">
+      <c r="BS1" t="str">
         <v>Office Hours Client 14:00-17:00 (510m)</v>
       </c>
-      <c r="BR1" t="str">
+      <c r="BT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BS1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BT1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BU1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
@@ -16982,10 +16982,10 @@
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BW1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BX1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BY1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -17157,17 +17157,17 @@
       <c r="AX2">
         <v>0.25</v>
       </c>
-      <c r="AY2" t="str">
-        <v/>
-      </c>
-      <c r="AZ2" t="str">
-        <v/>
-      </c>
-      <c r="BA2">
+      <c r="AY2">
         <v>0.25</v>
       </c>
-      <c r="BB2">
+      <c r="AZ2">
         <v>0.25</v>
+      </c>
+      <c r="BA2" t="str">
+        <v/>
+      </c>
+      <c r="BB2" t="str">
+        <v/>
       </c>
       <c r="BC2">
         <v>0.25</v>
@@ -17208,17 +17208,17 @@
       <c r="BO2">
         <v>0.25</v>
       </c>
-      <c r="BP2" t="str">
-        <v/>
-      </c>
-      <c r="BQ2" t="str">
-        <v/>
-      </c>
-      <c r="BR2">
+      <c r="BP2">
         <v>0.25</v>
       </c>
-      <c r="BS2">
+      <c r="BQ2">
         <v>0.25</v>
+      </c>
+      <c r="BR2" t="str">
+        <v/>
+      </c>
+      <c r="BS2" t="str">
+        <v/>
       </c>
       <c r="BT2">
         <v>0.25</v>
@@ -17405,17 +17405,17 @@
       <c r="AX3">
         <v>0.01</v>
       </c>
-      <c r="AY3" t="str">
-        <v/>
-      </c>
-      <c r="AZ3" t="str">
-        <v/>
-      </c>
-      <c r="BA3">
+      <c r="AY3">
         <v>0.01</v>
       </c>
-      <c r="BB3">
+      <c r="AZ3">
         <v>0.01</v>
+      </c>
+      <c r="BA3" t="str">
+        <v/>
+      </c>
+      <c r="BB3" t="str">
+        <v/>
       </c>
       <c r="BC3">
         <v>0.01</v>
@@ -17456,17 +17456,17 @@
       <c r="BO3">
         <v>0.01</v>
       </c>
-      <c r="BP3" t="str">
-        <v/>
-      </c>
-      <c r="BQ3" t="str">
-        <v/>
-      </c>
-      <c r="BR3">
+      <c r="BP3">
         <v>0.01</v>
       </c>
-      <c r="BS3">
+      <c r="BQ3">
         <v>0.01</v>
+      </c>
+      <c r="BR3" t="str">
+        <v/>
+      </c>
+      <c r="BS3" t="str">
+        <v/>
       </c>
       <c r="BT3">
         <v>0.01</v>
@@ -17605,8 +17605,8 @@
       <c r="AH4">
         <v>0</v>
       </c>
-      <c r="AI4" t="str">
-        <v/>
+      <c r="AI4">
+        <v>0</v>
       </c>
       <c r="AJ4">
         <v>0</v>
@@ -17626,8 +17626,8 @@
       <c r="AO4">
         <v>0</v>
       </c>
-      <c r="AP4">
-        <v>0</v>
+      <c r="AP4" t="str">
+        <v/>
       </c>
       <c r="AQ4">
         <v>0</v>
@@ -17650,17 +17650,17 @@
       <c r="AW4">
         <v>0</v>
       </c>
-      <c r="AX4" t="str">
-        <v/>
-      </c>
-      <c r="AY4" t="str">
-        <v/>
+      <c r="AX4">
+        <v>0</v>
+      </c>
+      <c r="AY4">
+        <v>0</v>
       </c>
       <c r="AZ4" t="str">
         <v/>
       </c>
-      <c r="BA4">
-        <v>0</v>
+      <c r="BA4" t="str">
+        <v/>
       </c>
       <c r="BB4" t="str">
         <v/>
@@ -17686,14 +17686,14 @@
       <c r="BI4">
         <v>0</v>
       </c>
-      <c r="BJ4">
-        <v>0</v>
+      <c r="BJ4" t="str">
+        <v/>
       </c>
       <c r="BK4">
         <v>0</v>
       </c>
-      <c r="BL4" t="str">
-        <v/>
+      <c r="BL4">
+        <v>0</v>
       </c>
       <c r="BM4">
         <v>0</v>
@@ -17707,14 +17707,14 @@
       <c r="BP4" t="str">
         <v/>
       </c>
-      <c r="BQ4" t="str">
-        <v/>
-      </c>
-      <c r="BR4">
-        <v>0</v>
-      </c>
-      <c r="BS4">
-        <v>0</v>
+      <c r="BQ4">
+        <v>0</v>
+      </c>
+      <c r="BR4" t="str">
+        <v/>
+      </c>
+      <c r="BS4" t="str">
+        <v/>
       </c>
       <c r="BT4">
         <v>0</v>
@@ -18101,8 +18101,8 @@
       <c r="AH6">
         <v>0.05</v>
       </c>
-      <c r="AI6" t="str">
-        <v/>
+      <c r="AI6">
+        <v>0.05</v>
       </c>
       <c r="AJ6">
         <v>0.05</v>
@@ -18122,8 +18122,8 @@
       <c r="AO6">
         <v>0.05</v>
       </c>
-      <c r="AP6">
-        <v>0.05</v>
+      <c r="AP6" t="str">
+        <v/>
       </c>
       <c r="AQ6">
         <v>0.05</v>
@@ -18146,17 +18146,17 @@
       <c r="AW6">
         <v>0.05</v>
       </c>
-      <c r="AX6" t="str">
-        <v/>
-      </c>
-      <c r="AY6" t="str">
-        <v/>
+      <c r="AX6">
+        <v>0.05</v>
+      </c>
+      <c r="AY6">
+        <v>0.05</v>
       </c>
       <c r="AZ6" t="str">
         <v/>
       </c>
-      <c r="BA6">
-        <v>0.05</v>
+      <c r="BA6" t="str">
+        <v/>
       </c>
       <c r="BB6" t="str">
         <v/>
@@ -18182,14 +18182,14 @@
       <c r="BI6">
         <v>0.05</v>
       </c>
-      <c r="BJ6">
-        <v>0.05</v>
+      <c r="BJ6" t="str">
+        <v/>
       </c>
       <c r="BK6">
         <v>0.05</v>
       </c>
-      <c r="BL6" t="str">
-        <v/>
+      <c r="BL6">
+        <v>0.05</v>
       </c>
       <c r="BM6">
         <v>0.05</v>
@@ -18203,14 +18203,14 @@
       <c r="BP6" t="str">
         <v/>
       </c>
-      <c r="BQ6" t="str">
-        <v/>
-      </c>
-      <c r="BR6">
+      <c r="BQ6">
         <v>0.05</v>
       </c>
-      <c r="BS6">
-        <v>0.05</v>
+      <c r="BR6" t="str">
+        <v/>
+      </c>
+      <c r="BS6" t="str">
+        <v/>
       </c>
       <c r="BT6">
         <v>0.05</v>
@@ -18397,17 +18397,17 @@
       <c r="AX7">
         <v>0</v>
       </c>
-      <c r="AY7" t="str">
-        <v/>
-      </c>
-      <c r="AZ7" t="str">
-        <v/>
-      </c>
-      <c r="BA7">
-        <v>0</v>
-      </c>
-      <c r="BB7">
-        <v>0</v>
+      <c r="AY7">
+        <v>0</v>
+      </c>
+      <c r="AZ7">
+        <v>0</v>
+      </c>
+      <c r="BA7" t="str">
+        <v/>
+      </c>
+      <c r="BB7" t="str">
+        <v/>
       </c>
       <c r="BC7">
         <v>0</v>
@@ -18448,17 +18448,17 @@
       <c r="BO7">
         <v>0</v>
       </c>
-      <c r="BP7" t="str">
-        <v/>
-      </c>
-      <c r="BQ7" t="str">
-        <v/>
-      </c>
-      <c r="BR7">
-        <v>0</v>
-      </c>
-      <c r="BS7">
-        <v>0</v>
+      <c r="BP7">
+        <v>0</v>
+      </c>
+      <c r="BQ7">
+        <v>0</v>
+      </c>
+      <c r="BR7" t="str">
+        <v/>
+      </c>
+      <c r="BS7" t="str">
+        <v/>
       </c>
       <c r="BT7">
         <v>0</v>
@@ -18645,17 +18645,17 @@
       <c r="AX8">
         <v>0.08</v>
       </c>
-      <c r="AY8" t="str">
-        <v/>
-      </c>
-      <c r="AZ8" t="str">
-        <v/>
-      </c>
-      <c r="BA8">
+      <c r="AY8">
         <v>0.08</v>
       </c>
-      <c r="BB8">
+      <c r="AZ8">
         <v>0.08</v>
+      </c>
+      <c r="BA8" t="str">
+        <v/>
+      </c>
+      <c r="BB8" t="str">
+        <v/>
       </c>
       <c r="BC8">
         <v>0.08</v>
@@ -18696,17 +18696,17 @@
       <c r="BO8">
         <v>0.08</v>
       </c>
-      <c r="BP8" t="str">
-        <v/>
-      </c>
-      <c r="BQ8" t="str">
-        <v/>
-      </c>
-      <c r="BR8">
+      <c r="BP8">
         <v>0.08</v>
       </c>
-      <c r="BS8">
+      <c r="BQ8">
         <v>0.08</v>
+      </c>
+      <c r="BR8" t="str">
+        <v/>
+      </c>
+      <c r="BS8" t="str">
+        <v/>
       </c>
       <c r="BT8">
         <v>0.08</v>
@@ -18890,17 +18890,17 @@
       <c r="AW9">
         <v>0</v>
       </c>
-      <c r="AX9" t="str">
-        <v/>
-      </c>
-      <c r="AY9" t="str">
-        <v/>
+      <c r="AX9">
+        <v>0</v>
+      </c>
+      <c r="AY9">
+        <v>0</v>
       </c>
       <c r="AZ9" t="str">
         <v/>
       </c>
-      <c r="BA9">
-        <v>0</v>
+      <c r="BA9" t="str">
+        <v/>
       </c>
       <c r="BB9" t="str">
         <v/>
@@ -18926,14 +18926,14 @@
       <c r="BI9">
         <v>0</v>
       </c>
-      <c r="BJ9">
-        <v>0</v>
+      <c r="BJ9" t="str">
+        <v/>
       </c>
       <c r="BK9">
         <v>0</v>
       </c>
-      <c r="BL9" t="str">
-        <v/>
+      <c r="BL9">
+        <v>0</v>
       </c>
       <c r="BM9">
         <v>0</v>
@@ -18947,14 +18947,14 @@
       <c r="BP9" t="str">
         <v/>
       </c>
-      <c r="BQ9" t="str">
-        <v/>
-      </c>
-      <c r="BR9">
-        <v>0</v>
-      </c>
-      <c r="BS9">
-        <v>0</v>
+      <c r="BQ9">
+        <v>0</v>
+      </c>
+      <c r="BR9" t="str">
+        <v/>
+      </c>
+      <c r="BS9" t="str">
+        <v/>
       </c>
       <c r="BT9">
         <v>0</v>
@@ -19141,17 +19141,17 @@
       <c r="AX10">
         <v>0</v>
       </c>
-      <c r="AY10" t="str">
-        <v/>
-      </c>
-      <c r="AZ10" t="str">
-        <v/>
-      </c>
-      <c r="BA10">
-        <v>0</v>
-      </c>
-      <c r="BB10">
-        <v>0</v>
+      <c r="AY10">
+        <v>0</v>
+      </c>
+      <c r="AZ10">
+        <v>0</v>
+      </c>
+      <c r="BA10" t="str">
+        <v/>
+      </c>
+      <c r="BB10" t="str">
+        <v/>
       </c>
       <c r="BC10">
         <v>0</v>
@@ -19192,17 +19192,17 @@
       <c r="BO10">
         <v>0</v>
       </c>
-      <c r="BP10" t="str">
-        <v/>
-      </c>
-      <c r="BQ10" t="str">
-        <v/>
-      </c>
-      <c r="BR10">
-        <v>0</v>
-      </c>
-      <c r="BS10">
-        <v>0</v>
+      <c r="BP10">
+        <v>0</v>
+      </c>
+      <c r="BQ10">
+        <v>0</v>
+      </c>
+      <c r="BR10" t="str">
+        <v/>
+      </c>
+      <c r="BS10" t="str">
+        <v/>
       </c>
       <c r="BT10">
         <v>0</v>
@@ -19338,8 +19338,8 @@
       <c r="AG11">
         <v>0.78</v>
       </c>
-      <c r="AH11">
-        <v>0.78</v>
+      <c r="AH11" t="str">
+        <v/>
       </c>
       <c r="AI11" t="str">
         <v/>
@@ -19353,41 +19353,41 @@
       <c r="AL11">
         <v>0.78</v>
       </c>
-      <c r="AM11" t="str">
-        <v/>
-      </c>
-      <c r="AN11" t="str">
-        <v/>
+      <c r="AM11">
+        <v>0.78</v>
+      </c>
+      <c r="AN11">
+        <v>0.78</v>
       </c>
       <c r="AO11">
         <v>0.78</v>
       </c>
-      <c r="AP11">
-        <v>0.78</v>
+      <c r="AP11" t="str">
+        <v/>
       </c>
       <c r="AQ11">
         <v>0.78</v>
       </c>
-      <c r="AR11" t="str">
-        <v/>
-      </c>
-      <c r="AS11" t="str">
-        <v/>
-      </c>
-      <c r="AT11">
+      <c r="AR11">
         <v>0.78</v>
       </c>
-      <c r="AU11">
+      <c r="AS11">
         <v>0.78</v>
+      </c>
+      <c r="AT11" t="str">
+        <v/>
+      </c>
+      <c r="AU11" t="str">
+        <v/>
       </c>
       <c r="AV11">
         <v>0.78</v>
       </c>
-      <c r="AW11" t="str">
-        <v/>
-      </c>
-      <c r="AX11" t="str">
-        <v/>
+      <c r="AW11">
+        <v>0.78</v>
+      </c>
+      <c r="AX11">
+        <v>0.78</v>
       </c>
       <c r="AY11" t="str">
         <v/>
@@ -19419,53 +19419,53 @@
       <c r="BH11" t="str">
         <v/>
       </c>
-      <c r="BI11">
+      <c r="BI11" t="str">
+        <v/>
+      </c>
+      <c r="BJ11" t="str">
+        <v/>
+      </c>
+      <c r="BK11">
         <v>0.78</v>
       </c>
-      <c r="BJ11">
+      <c r="BL11">
         <v>0.78</v>
       </c>
-      <c r="BK11" t="str">
-        <v/>
-      </c>
-      <c r="BL11" t="str">
-        <v/>
-      </c>
       <c r="BM11" t="str">
         <v/>
       </c>
       <c r="BN11" t="str">
         <v/>
       </c>
-      <c r="BO11">
+      <c r="BO11" t="str">
+        <v/>
+      </c>
+      <c r="BP11" t="str">
+        <v/>
+      </c>
+      <c r="BQ11">
         <v>0.78</v>
       </c>
-      <c r="BP11" t="str">
-        <v/>
-      </c>
-      <c r="BQ11" t="str">
-        <v/>
-      </c>
-      <c r="BR11">
+      <c r="BR11" t="str">
+        <v/>
+      </c>
+      <c r="BS11" t="str">
+        <v/>
+      </c>
+      <c r="BT11">
         <v>0.78</v>
       </c>
-      <c r="BS11" t="str">
-        <v/>
-      </c>
-      <c r="BT11" t="str">
-        <v/>
-      </c>
       <c r="BU11" t="str">
         <v/>
       </c>
       <c r="BV11" t="str">
         <v/>
       </c>
-      <c r="BW11">
-        <v>0.78</v>
-      </c>
-      <c r="BX11">
-        <v>0.78</v>
+      <c r="BW11" t="str">
+        <v/>
+      </c>
+      <c r="BX11" t="str">
+        <v/>
       </c>
       <c r="BY11">
         <v>0.78</v>
@@ -19637,17 +19637,17 @@
       <c r="AX12">
         <v>0</v>
       </c>
-      <c r="AY12" t="str">
-        <v/>
-      </c>
-      <c r="AZ12" t="str">
-        <v/>
-      </c>
-      <c r="BA12">
-        <v>0</v>
-      </c>
-      <c r="BB12">
-        <v>0</v>
+      <c r="AY12">
+        <v>0</v>
+      </c>
+      <c r="AZ12">
+        <v>0</v>
+      </c>
+      <c r="BA12" t="str">
+        <v/>
+      </c>
+      <c r="BB12" t="str">
+        <v/>
       </c>
       <c r="BC12">
         <v>0</v>
@@ -19688,17 +19688,17 @@
       <c r="BO12">
         <v>0</v>
       </c>
-      <c r="BP12" t="str">
-        <v/>
-      </c>
-      <c r="BQ12" t="str">
-        <v/>
-      </c>
-      <c r="BR12">
-        <v>0</v>
-      </c>
-      <c r="BS12">
-        <v>0</v>
+      <c r="BP12">
+        <v>0</v>
+      </c>
+      <c r="BQ12">
+        <v>0</v>
+      </c>
+      <c r="BR12" t="str">
+        <v/>
+      </c>
+      <c r="BS12" t="str">
+        <v/>
       </c>
       <c r="BT12">
         <v>0</v>
@@ -19837,8 +19837,8 @@
       <c r="AH13">
         <v>0.17</v>
       </c>
-      <c r="AI13" t="str">
-        <v/>
+      <c r="AI13">
+        <v>0.17</v>
       </c>
       <c r="AJ13">
         <v>0.17</v>
@@ -19858,8 +19858,8 @@
       <c r="AO13">
         <v>0.17</v>
       </c>
-      <c r="AP13">
-        <v>0.17</v>
+      <c r="AP13" t="str">
+        <v/>
       </c>
       <c r="AQ13">
         <v>0.17</v>
@@ -19885,17 +19885,17 @@
       <c r="AX13">
         <v>0.17</v>
       </c>
-      <c r="AY13" t="str">
-        <v/>
-      </c>
-      <c r="AZ13" t="str">
-        <v/>
-      </c>
-      <c r="BA13">
+      <c r="AY13">
         <v>0.17</v>
       </c>
-      <c r="BB13">
+      <c r="AZ13">
         <v>0.17</v>
+      </c>
+      <c r="BA13" t="str">
+        <v/>
+      </c>
+      <c r="BB13" t="str">
+        <v/>
       </c>
       <c r="BC13">
         <v>0.17</v>
@@ -19936,17 +19936,17 @@
       <c r="BO13">
         <v>0.17</v>
       </c>
-      <c r="BP13" t="str">
-        <v/>
-      </c>
-      <c r="BQ13" t="str">
-        <v/>
-      </c>
-      <c r="BR13">
+      <c r="BP13">
         <v>0.17</v>
       </c>
-      <c r="BS13">
+      <c r="BQ13">
         <v>0.17</v>
+      </c>
+      <c r="BR13" t="str">
+        <v/>
+      </c>
+      <c r="BS13" t="str">
+        <v/>
       </c>
       <c r="BT13">
         <v>0.17</v>
@@ -20363,13 +20363,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AO1" t="str">
+        <v>Office Hours Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="AP1" t="str">
+        <v>Office Hours Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="AQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="AP1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="AQ1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AR1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20381,16 +20381,16 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AU1" t="str">
-        <v>Office Hours Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AV1" t="str">
-        <v>Office Hours Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AW1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AX1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="AY1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20402,70 +20402,70 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BB1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="BC1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="BD1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BC1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BD1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="BE1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BF1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BG1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BH1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BI1" t="str">
         <v>Specialised Care Client 09:00-12:00 (420m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BJ1" t="str">
         <v>Specialised Care Client 14:00-17:00 (420m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BK1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BK1" t="str">
+      <c r="BL1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BL1" t="str">
+      <c r="BM1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BM1" t="str">
+      <c r="BN1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BN1" t="str">
+      <c r="BO1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BO1" t="str">
+      <c r="BP1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BP1" t="str">
+      <c r="BQ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BQ1" t="str">
+      <c r="BR1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BR1" t="str">
+      <c r="BS1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (180m)</v>
       </c>
-      <c r="BS1" t="str">
+      <c r="BT1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BT1" t="str">
+      <c r="BU1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BU1" t="str">
+      <c r="BV1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BV1" t="str">
+      <c r="BW1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BW1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
@@ -20474,58 +20474,58 @@
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BZ1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="CA1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CA1" t="str">
+      <c r="CB1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="CB1" t="str">
+      <c r="CC1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="CC1" t="str">
+      <c r="CD1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="CD1" t="str">
+      <c r="CE1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="CE1" t="str">
+      <c r="CF1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CF1" t="str">
+      <c r="CG1" t="str">
         <v>Office Hours Client 09:00-12:00 (330m)</v>
       </c>
-      <c r="CG1" t="str">
+      <c r="CH1" t="str">
         <v>Office Hours Client 14:00-17:00 (330m)</v>
       </c>
-      <c r="CH1" t="str">
+      <c r="CI1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CI1" t="str">
+      <c r="CJ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
-      <c r="CJ1" t="str">
+      <c r="CK1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (150m)</v>
-      </c>
-      <c r="CK1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CM1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="CO1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="CP1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CP1" t="str">
+      <c r="CQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="CQ1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CR1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20718,14 +20718,14 @@
       <c r="BG2">
         <v>0.09</v>
       </c>
-      <c r="BH2" t="str">
-        <v/>
+      <c r="BH2">
+        <v>0.09</v>
       </c>
       <c r="BI2" t="str">
         <v/>
       </c>
-      <c r="BJ2">
-        <v>0.09</v>
+      <c r="BJ2" t="str">
+        <v/>
       </c>
       <c r="BK2">
         <v>0.09</v>
@@ -20790,14 +20790,14 @@
       <c r="CE2">
         <v>0.09</v>
       </c>
-      <c r="CF2" t="str">
-        <v/>
+      <c r="CF2">
+        <v>0.09</v>
       </c>
       <c r="CG2" t="str">
         <v/>
       </c>
-      <c r="CH2">
-        <v>0.09</v>
+      <c r="CH2" t="str">
+        <v/>
       </c>
       <c r="CI2">
         <v>0.09</v>
@@ -21017,14 +21017,14 @@
       <c r="BG3">
         <v>0</v>
       </c>
-      <c r="BH3" t="str">
-        <v/>
+      <c r="BH3">
+        <v>0</v>
       </c>
       <c r="BI3" t="str">
         <v/>
       </c>
-      <c r="BJ3">
-        <v>0</v>
+      <c r="BJ3" t="str">
+        <v/>
       </c>
       <c r="BK3">
         <v>0</v>
@@ -21089,14 +21089,14 @@
       <c r="CE3">
         <v>0</v>
       </c>
-      <c r="CF3" t="str">
-        <v/>
+      <c r="CF3">
+        <v>0</v>
       </c>
       <c r="CG3" t="str">
         <v/>
       </c>
-      <c r="CH3">
-        <v>0</v>
+      <c r="CH3" t="str">
+        <v/>
       </c>
       <c r="CI3">
         <v>0</v>
@@ -21265,8 +21265,8 @@
       <c r="AP4" t="str">
         <v/>
       </c>
-      <c r="AQ4" t="str">
-        <v/>
+      <c r="AQ4">
+        <v>0.78</v>
       </c>
       <c r="AR4">
         <v>0.78</v>
@@ -21280,14 +21280,14 @@
       <c r="AU4">
         <v>0.78</v>
       </c>
-      <c r="AV4" t="str">
-        <v/>
+      <c r="AV4">
+        <v>0.78</v>
       </c>
       <c r="AW4">
         <v>0.78</v>
       </c>
-      <c r="AX4">
-        <v>0.78</v>
+      <c r="AX4" t="str">
+        <v/>
       </c>
       <c r="AY4">
         <v>0.78</v>
@@ -21298,14 +21298,14 @@
       <c r="BA4">
         <v>0.78</v>
       </c>
-      <c r="BB4">
+      <c r="BB4" t="str">
+        <v/>
+      </c>
+      <c r="BC4" t="str">
+        <v/>
+      </c>
+      <c r="BD4">
         <v>0.78</v>
-      </c>
-      <c r="BC4">
-        <v>0.78</v>
-      </c>
-      <c r="BD4" t="str">
-        <v/>
       </c>
       <c r="BE4">
         <v>0.78</v>
@@ -21313,8 +21313,8 @@
       <c r="BF4">
         <v>0.78</v>
       </c>
-      <c r="BG4" t="str">
-        <v/>
+      <c r="BG4">
+        <v>0.78</v>
       </c>
       <c r="BH4" t="str">
         <v/>
@@ -21322,45 +21322,45 @@
       <c r="BI4" t="str">
         <v/>
       </c>
-      <c r="BJ4">
+      <c r="BJ4" t="str">
+        <v/>
+      </c>
+      <c r="BK4">
         <v>0.78</v>
       </c>
-      <c r="BK4" t="str">
-        <v/>
-      </c>
-      <c r="BL4">
+      <c r="BL4" t="str">
+        <v/>
+      </c>
+      <c r="BM4">
         <v>0.78</v>
       </c>
-      <c r="BM4" t="str">
-        <v/>
-      </c>
-      <c r="BN4">
+      <c r="BN4" t="str">
+        <v/>
+      </c>
+      <c r="BO4">
         <v>0.78</v>
       </c>
-      <c r="BO4" t="str">
-        <v/>
-      </c>
-      <c r="BP4">
+      <c r="BP4" t="str">
+        <v/>
+      </c>
+      <c r="BQ4">
         <v>0.78</v>
       </c>
-      <c r="BQ4" t="str">
-        <v/>
-      </c>
       <c r="BR4" t="str">
         <v/>
       </c>
-      <c r="BS4">
+      <c r="BS4" t="str">
+        <v/>
+      </c>
+      <c r="BT4">
         <v>0.78</v>
       </c>
-      <c r="BT4" t="str">
-        <v/>
-      </c>
-      <c r="BU4">
+      <c r="BU4" t="str">
+        <v/>
+      </c>
+      <c r="BV4">
         <v>0.78</v>
       </c>
-      <c r="BV4" t="str">
-        <v/>
-      </c>
       <c r="BW4" t="str">
         <v/>
       </c>
@@ -21370,59 +21370,59 @@
       <c r="BY4" t="str">
         <v/>
       </c>
-      <c r="BZ4">
-        <v>0.78</v>
+      <c r="BZ4" t="str">
+        <v/>
       </c>
       <c r="CA4">
         <v>0.78</v>
       </c>
-      <c r="CB4" t="str">
-        <v/>
-      </c>
-      <c r="CC4">
+      <c r="CB4">
         <v>0.78</v>
       </c>
-      <c r="CD4" t="str">
-        <v/>
-      </c>
-      <c r="CE4">
+      <c r="CC4" t="str">
+        <v/>
+      </c>
+      <c r="CD4">
         <v>0.78</v>
       </c>
-      <c r="CF4" t="str">
-        <v/>
+      <c r="CE4" t="str">
+        <v/>
+      </c>
+      <c r="CF4">
+        <v>0.78</v>
       </c>
       <c r="CG4" t="str">
         <v/>
       </c>
-      <c r="CH4">
+      <c r="CH4" t="str">
+        <v/>
+      </c>
+      <c r="CI4">
         <v>0.78</v>
       </c>
-      <c r="CI4" t="str">
-        <v/>
-      </c>
       <c r="CJ4" t="str">
         <v/>
       </c>
-      <c r="CK4">
-        <v>0.78</v>
+      <c r="CK4" t="str">
+        <v/>
       </c>
       <c r="CL4">
         <v>0.78</v>
       </c>
-      <c r="CM4" t="str">
-        <v/>
+      <c r="CM4">
+        <v>0.78</v>
       </c>
       <c r="CN4" t="str">
         <v/>
       </c>
-      <c r="CO4">
+      <c r="CO4" t="str">
+        <v/>
+      </c>
+      <c r="CP4">
         <v>0.78</v>
       </c>
-      <c r="CP4" t="str">
-        <v/>
-      </c>
-      <c r="CQ4">
-        <v>0.78</v>
+      <c r="CQ4" t="str">
+        <v/>
       </c>
       <c r="CR4">
         <v>0.78</v>
@@ -21561,8 +21561,8 @@
       <c r="AO5">
         <v>0</v>
       </c>
-      <c r="AP5">
-        <v>0</v>
+      <c r="AP5" t="str">
+        <v/>
       </c>
       <c r="AQ5">
         <v>0</v>
@@ -21579,14 +21579,14 @@
       <c r="AU5">
         <v>0</v>
       </c>
-      <c r="AV5" t="str">
-        <v/>
+      <c r="AV5">
+        <v>0</v>
       </c>
       <c r="AW5">
         <v>0</v>
       </c>
-      <c r="AX5">
-        <v>0</v>
+      <c r="AX5" t="str">
+        <v/>
       </c>
       <c r="AY5">
         <v>0</v>
@@ -21603,8 +21603,8 @@
       <c r="BC5">
         <v>0</v>
       </c>
-      <c r="BD5" t="str">
-        <v/>
+      <c r="BD5">
+        <v>0</v>
       </c>
       <c r="BE5">
         <v>0</v>
@@ -21612,8 +21612,8 @@
       <c r="BF5">
         <v>0</v>
       </c>
-      <c r="BG5" t="str">
-        <v/>
+      <c r="BG5">
+        <v>0</v>
       </c>
       <c r="BH5" t="str">
         <v/>
@@ -21621,47 +21621,47 @@
       <c r="BI5" t="str">
         <v/>
       </c>
-      <c r="BJ5">
-        <v>0</v>
-      </c>
-      <c r="BK5" t="str">
-        <v/>
-      </c>
-      <c r="BL5">
-        <v>0</v>
-      </c>
-      <c r="BM5" t="str">
-        <v/>
-      </c>
-      <c r="BN5">
-        <v>0</v>
-      </c>
-      <c r="BO5" t="str">
-        <v/>
-      </c>
-      <c r="BP5">
-        <v>0</v>
-      </c>
-      <c r="BQ5" t="str">
-        <v/>
-      </c>
-      <c r="BR5">
-        <v>0</v>
+      <c r="BJ5" t="str">
+        <v/>
+      </c>
+      <c r="BK5">
+        <v>0</v>
+      </c>
+      <c r="BL5" t="str">
+        <v/>
+      </c>
+      <c r="BM5">
+        <v>0</v>
+      </c>
+      <c r="BN5" t="str">
+        <v/>
+      </c>
+      <c r="BO5">
+        <v>0</v>
+      </c>
+      <c r="BP5" t="str">
+        <v/>
+      </c>
+      <c r="BQ5">
+        <v>0</v>
+      </c>
+      <c r="BR5" t="str">
+        <v/>
       </c>
       <c r="BS5">
         <v>0</v>
       </c>
-      <c r="BT5" t="str">
-        <v/>
-      </c>
-      <c r="BU5">
-        <v>0</v>
-      </c>
-      <c r="BV5" t="str">
-        <v/>
-      </c>
-      <c r="BW5">
-        <v>0</v>
+      <c r="BT5">
+        <v>0</v>
+      </c>
+      <c r="BU5" t="str">
+        <v/>
+      </c>
+      <c r="BV5">
+        <v>0</v>
+      </c>
+      <c r="BW5" t="str">
+        <v/>
       </c>
       <c r="BX5">
         <v>0</v>
@@ -21675,32 +21675,32 @@
       <c r="CA5">
         <v>0</v>
       </c>
-      <c r="CB5" t="str">
-        <v/>
-      </c>
-      <c r="CC5">
-        <v>0</v>
-      </c>
-      <c r="CD5" t="str">
-        <v/>
-      </c>
-      <c r="CE5">
-        <v>0</v>
-      </c>
-      <c r="CF5" t="str">
-        <v/>
+      <c r="CB5">
+        <v>0</v>
+      </c>
+      <c r="CC5" t="str">
+        <v/>
+      </c>
+      <c r="CD5">
+        <v>0</v>
+      </c>
+      <c r="CE5" t="str">
+        <v/>
+      </c>
+      <c r="CF5">
+        <v>0</v>
       </c>
       <c r="CG5" t="str">
         <v/>
       </c>
-      <c r="CH5">
-        <v>0</v>
-      </c>
-      <c r="CI5" t="str">
-        <v/>
-      </c>
-      <c r="CJ5">
-        <v>0</v>
+      <c r="CH5" t="str">
+        <v/>
+      </c>
+      <c r="CI5">
+        <v>0</v>
+      </c>
+      <c r="CJ5" t="str">
+        <v/>
       </c>
       <c r="CK5">
         <v>0</v>
@@ -22159,8 +22159,8 @@
       <c r="AO7">
         <v>0</v>
       </c>
-      <c r="AP7">
-        <v>0</v>
+      <c r="AP7" t="str">
+        <v/>
       </c>
       <c r="AQ7">
         <v>0</v>
@@ -22177,8 +22177,8 @@
       <c r="AU7">
         <v>0</v>
       </c>
-      <c r="AV7" t="str">
-        <v/>
+      <c r="AV7">
+        <v>0</v>
       </c>
       <c r="AW7">
         <v>0</v>
@@ -22210,8 +22210,8 @@
       <c r="BF7">
         <v>0</v>
       </c>
-      <c r="BG7" t="str">
-        <v/>
+      <c r="BG7">
+        <v>0</v>
       </c>
       <c r="BH7" t="str">
         <v/>
@@ -22219,47 +22219,47 @@
       <c r="BI7" t="str">
         <v/>
       </c>
-      <c r="BJ7">
-        <v>0</v>
-      </c>
-      <c r="BK7" t="str">
-        <v/>
-      </c>
-      <c r="BL7">
-        <v>0</v>
-      </c>
-      <c r="BM7" t="str">
-        <v/>
-      </c>
-      <c r="BN7">
-        <v>0</v>
-      </c>
-      <c r="BO7" t="str">
-        <v/>
-      </c>
-      <c r="BP7">
-        <v>0</v>
-      </c>
-      <c r="BQ7" t="str">
-        <v/>
-      </c>
-      <c r="BR7">
-        <v>0</v>
+      <c r="BJ7" t="str">
+        <v/>
+      </c>
+      <c r="BK7">
+        <v>0</v>
+      </c>
+      <c r="BL7" t="str">
+        <v/>
+      </c>
+      <c r="BM7">
+        <v>0</v>
+      </c>
+      <c r="BN7" t="str">
+        <v/>
+      </c>
+      <c r="BO7">
+        <v>0</v>
+      </c>
+      <c r="BP7" t="str">
+        <v/>
+      </c>
+      <c r="BQ7">
+        <v>0</v>
+      </c>
+      <c r="BR7" t="str">
+        <v/>
       </c>
       <c r="BS7">
         <v>0</v>
       </c>
-      <c r="BT7" t="str">
-        <v/>
-      </c>
-      <c r="BU7">
-        <v>0</v>
-      </c>
-      <c r="BV7" t="str">
-        <v/>
-      </c>
-      <c r="BW7">
-        <v>0</v>
+      <c r="BT7">
+        <v>0</v>
+      </c>
+      <c r="BU7" t="str">
+        <v/>
+      </c>
+      <c r="BV7">
+        <v>0</v>
+      </c>
+      <c r="BW7" t="str">
+        <v/>
       </c>
       <c r="BX7">
         <v>0</v>
@@ -22273,26 +22273,26 @@
       <c r="CA7">
         <v>0</v>
       </c>
-      <c r="CB7" t="str">
-        <v/>
-      </c>
-      <c r="CC7">
-        <v>0</v>
-      </c>
-      <c r="CD7" t="str">
-        <v/>
-      </c>
-      <c r="CE7">
-        <v>0</v>
-      </c>
-      <c r="CF7" t="str">
-        <v/>
+      <c r="CB7">
+        <v>0</v>
+      </c>
+      <c r="CC7" t="str">
+        <v/>
+      </c>
+      <c r="CD7">
+        <v>0</v>
+      </c>
+      <c r="CE7" t="str">
+        <v/>
+      </c>
+      <c r="CF7">
+        <v>0</v>
       </c>
       <c r="CG7" t="str">
         <v/>
       </c>
-      <c r="CH7">
-        <v>0</v>
+      <c r="CH7" t="str">
+        <v/>
       </c>
       <c r="CI7">
         <v>0</v>
@@ -22512,14 +22512,14 @@
       <c r="BG8">
         <v>0</v>
       </c>
-      <c r="BH8" t="str">
-        <v/>
+      <c r="BH8">
+        <v>0</v>
       </c>
       <c r="BI8" t="str">
         <v/>
       </c>
-      <c r="BJ8">
-        <v>0</v>
+      <c r="BJ8" t="str">
+        <v/>
       </c>
       <c r="BK8">
         <v>0</v>
@@ -22584,14 +22584,14 @@
       <c r="CE8">
         <v>0</v>
       </c>
-      <c r="CF8" t="str">
-        <v/>
+      <c r="CF8">
+        <v>0</v>
       </c>
       <c r="CG8" t="str">
         <v/>
       </c>
-      <c r="CH8">
-        <v>0</v>
+      <c r="CH8" t="str">
+        <v/>
       </c>
       <c r="CI8">
         <v>0</v>
@@ -22757,8 +22757,8 @@
       <c r="AO9">
         <v>0</v>
       </c>
-      <c r="AP9">
-        <v>0</v>
+      <c r="AP9" t="str">
+        <v/>
       </c>
       <c r="AQ9">
         <v>0</v>
@@ -22775,8 +22775,8 @@
       <c r="AU9">
         <v>0</v>
       </c>
-      <c r="AV9" t="str">
-        <v/>
+      <c r="AV9">
+        <v>0</v>
       </c>
       <c r="AW9">
         <v>0</v>
@@ -22808,8 +22808,8 @@
       <c r="BF9">
         <v>0</v>
       </c>
-      <c r="BG9" t="str">
-        <v/>
+      <c r="BG9">
+        <v>0</v>
       </c>
       <c r="BH9" t="str">
         <v/>
@@ -22817,47 +22817,47 @@
       <c r="BI9" t="str">
         <v/>
       </c>
-      <c r="BJ9">
-        <v>0</v>
-      </c>
-      <c r="BK9" t="str">
-        <v/>
-      </c>
-      <c r="BL9">
-        <v>0</v>
-      </c>
-      <c r="BM9" t="str">
-        <v/>
-      </c>
-      <c r="BN9">
-        <v>0</v>
-      </c>
-      <c r="BO9" t="str">
-        <v/>
-      </c>
-      <c r="BP9">
-        <v>0</v>
-      </c>
-      <c r="BQ9" t="str">
-        <v/>
-      </c>
-      <c r="BR9">
-        <v>0</v>
+      <c r="BJ9" t="str">
+        <v/>
+      </c>
+      <c r="BK9">
+        <v>0</v>
+      </c>
+      <c r="BL9" t="str">
+        <v/>
+      </c>
+      <c r="BM9">
+        <v>0</v>
+      </c>
+      <c r="BN9" t="str">
+        <v/>
+      </c>
+      <c r="BO9">
+        <v>0</v>
+      </c>
+      <c r="BP9" t="str">
+        <v/>
+      </c>
+      <c r="BQ9">
+        <v>0</v>
+      </c>
+      <c r="BR9" t="str">
+        <v/>
       </c>
       <c r="BS9">
         <v>0</v>
       </c>
-      <c r="BT9" t="str">
-        <v/>
-      </c>
-      <c r="BU9">
-        <v>0</v>
-      </c>
-      <c r="BV9" t="str">
-        <v/>
-      </c>
-      <c r="BW9">
-        <v>0</v>
+      <c r="BT9">
+        <v>0</v>
+      </c>
+      <c r="BU9" t="str">
+        <v/>
+      </c>
+      <c r="BV9">
+        <v>0</v>
+      </c>
+      <c r="BW9" t="str">
+        <v/>
       </c>
       <c r="BX9">
         <v>0</v>
@@ -22871,26 +22871,26 @@
       <c r="CA9">
         <v>0</v>
       </c>
-      <c r="CB9" t="str">
-        <v/>
-      </c>
-      <c r="CC9">
-        <v>0</v>
-      </c>
-      <c r="CD9" t="str">
-        <v/>
-      </c>
-      <c r="CE9">
-        <v>0</v>
-      </c>
-      <c r="CF9" t="str">
-        <v/>
+      <c r="CB9">
+        <v>0</v>
+      </c>
+      <c r="CC9" t="str">
+        <v/>
+      </c>
+      <c r="CD9">
+        <v>0</v>
+      </c>
+      <c r="CE9" t="str">
+        <v/>
+      </c>
+      <c r="CF9">
+        <v>0</v>
       </c>
       <c r="CG9" t="str">
         <v/>
       </c>
-      <c r="CH9">
-        <v>0</v>
+      <c r="CH9" t="str">
+        <v/>
       </c>
       <c r="CI9">
         <v>0</v>
@@ -23110,14 +23110,14 @@
       <c r="BG10">
         <v>0</v>
       </c>
-      <c r="BH10" t="str">
-        <v/>
+      <c r="BH10">
+        <v>0</v>
       </c>
       <c r="BI10" t="str">
         <v/>
       </c>
-      <c r="BJ10">
-        <v>0</v>
+      <c r="BJ10" t="str">
+        <v/>
       </c>
       <c r="BK10">
         <v>0</v>
@@ -23182,14 +23182,14 @@
       <c r="CE10">
         <v>0</v>
       </c>
-      <c r="CF10" t="str">
-        <v/>
+      <c r="CF10">
+        <v>0</v>
       </c>
       <c r="CG10" t="str">
         <v/>
       </c>
-      <c r="CH10">
-        <v>0</v>
+      <c r="CH10" t="str">
+        <v/>
       </c>
       <c r="CI10">
         <v>0</v>
@@ -23409,14 +23409,14 @@
       <c r="BG11">
         <v>0</v>
       </c>
-      <c r="BH11" t="str">
-        <v/>
+      <c r="BH11">
+        <v>0</v>
       </c>
       <c r="BI11" t="str">
         <v/>
       </c>
-      <c r="BJ11">
-        <v>0</v>
+      <c r="BJ11" t="str">
+        <v/>
       </c>
       <c r="BK11">
         <v>0</v>
@@ -23481,14 +23481,14 @@
       <c r="CE11">
         <v>0</v>
       </c>
-      <c r="CF11" t="str">
-        <v/>
+      <c r="CF11">
+        <v>0</v>
       </c>
       <c r="CG11" t="str">
         <v/>
       </c>
-      <c r="CH11">
-        <v>0</v>
+      <c r="CH11" t="str">
+        <v/>
       </c>
       <c r="CI11">
         <v>0</v>
@@ -23708,14 +23708,14 @@
       <c r="BG12">
         <v>0</v>
       </c>
-      <c r="BH12" t="str">
-        <v/>
+      <c r="BH12">
+        <v>0</v>
       </c>
       <c r="BI12" t="str">
         <v/>
       </c>
-      <c r="BJ12">
-        <v>0</v>
+      <c r="BJ12" t="str">
+        <v/>
       </c>
       <c r="BK12">
         <v>0</v>
@@ -23780,14 +23780,14 @@
       <c r="CE12">
         <v>0</v>
       </c>
-      <c r="CF12" t="str">
-        <v/>
+      <c r="CF12">
+        <v>0</v>
       </c>
       <c r="CG12" t="str">
         <v/>
       </c>
-      <c r="CH12">
-        <v>0</v>
+      <c r="CH12" t="str">
+        <v/>
       </c>
       <c r="CI12">
         <v>0</v>
@@ -23977,8 +23977,8 @@
       <c r="AW13">
         <v>0</v>
       </c>
-      <c r="AX13">
-        <v>0</v>
+      <c r="AX13" t="str">
+        <v/>
       </c>
       <c r="AY13">
         <v>0</v>
@@ -23995,8 +23995,8 @@
       <c r="BC13">
         <v>0</v>
       </c>
-      <c r="BD13" t="str">
-        <v/>
+      <c r="BD13">
+        <v>0</v>
       </c>
       <c r="BE13">
         <v>0</v>
@@ -24007,14 +24007,14 @@
       <c r="BG13">
         <v>0</v>
       </c>
-      <c r="BH13" t="str">
-        <v/>
+      <c r="BH13">
+        <v>0</v>
       </c>
       <c r="BI13" t="str">
         <v/>
       </c>
-      <c r="BJ13">
-        <v>0</v>
+      <c r="BJ13" t="str">
+        <v/>
       </c>
       <c r="BK13">
         <v>0</v>
@@ -24079,20 +24079,20 @@
       <c r="CE13">
         <v>0</v>
       </c>
-      <c r="CF13" t="str">
-        <v/>
+      <c r="CF13">
+        <v>0</v>
       </c>
       <c r="CG13" t="str">
         <v/>
       </c>
-      <c r="CH13">
-        <v>0</v>
-      </c>
-      <c r="CI13" t="str">
-        <v/>
-      </c>
-      <c r="CJ13">
-        <v>0</v>
+      <c r="CH13" t="str">
+        <v/>
+      </c>
+      <c r="CI13">
+        <v>0</v>
+      </c>
+      <c r="CJ13" t="str">
+        <v/>
       </c>
       <c r="CK13">
         <v>0</v>
@@ -24249,14 +24249,14 @@
       <c r="AN14">
         <v>0.16</v>
       </c>
-      <c r="AO14">
+      <c r="AO14" t="str">
+        <v/>
+      </c>
+      <c r="AP14">
         <v>0.16</v>
       </c>
-      <c r="AP14" t="str">
-        <v/>
-      </c>
-      <c r="AQ14" t="str">
-        <v/>
+      <c r="AQ14">
+        <v>0.16</v>
       </c>
       <c r="AR14">
         <v>0.16</v>
@@ -24267,8 +24267,8 @@
       <c r="AT14">
         <v>0.16</v>
       </c>
-      <c r="AU14" t="str">
-        <v/>
+      <c r="AU14">
+        <v>0.16</v>
       </c>
       <c r="AV14">
         <v>0.16</v>
@@ -24276,8 +24276,8 @@
       <c r="AW14">
         <v>0.16</v>
       </c>
-      <c r="AX14">
-        <v>0.16</v>
+      <c r="AX14" t="str">
+        <v/>
       </c>
       <c r="AY14">
         <v>0.16</v>
@@ -24288,26 +24288,26 @@
       <c r="BA14">
         <v>0.16</v>
       </c>
-      <c r="BB14">
+      <c r="BB14" t="str">
+        <v/>
+      </c>
+      <c r="BC14" t="str">
+        <v/>
+      </c>
+      <c r="BD14">
         <v>0.16</v>
-      </c>
-      <c r="BC14">
-        <v>0.16</v>
-      </c>
-      <c r="BD14" t="str">
-        <v/>
       </c>
       <c r="BE14">
         <v>0.16</v>
       </c>
-      <c r="BF14" t="str">
-        <v/>
-      </c>
-      <c r="BG14">
+      <c r="BF14">
         <v>0.16</v>
       </c>
-      <c r="BH14" t="str">
-        <v/>
+      <c r="BG14" t="str">
+        <v/>
+      </c>
+      <c r="BH14">
+        <v>0.16</v>
       </c>
       <c r="BI14" t="str">
         <v/>
@@ -24315,104 +24315,104 @@
       <c r="BJ14" t="str">
         <v/>
       </c>
-      <c r="BK14">
+      <c r="BK14" t="str">
+        <v/>
+      </c>
+      <c r="BL14">
         <v>0.16</v>
       </c>
-      <c r="BL14" t="str">
-        <v/>
-      </c>
-      <c r="BM14">
+      <c r="BM14" t="str">
+        <v/>
+      </c>
+      <c r="BN14">
         <v>0.16</v>
       </c>
-      <c r="BN14" t="str">
-        <v/>
-      </c>
-      <c r="BO14">
+      <c r="BO14" t="str">
+        <v/>
+      </c>
+      <c r="BP14">
         <v>0.16</v>
       </c>
-      <c r="BP14" t="str">
-        <v/>
-      </c>
-      <c r="BQ14">
+      <c r="BQ14" t="str">
+        <v/>
+      </c>
+      <c r="BR14">
         <v>0.16</v>
       </c>
-      <c r="BR14" t="str">
-        <v/>
-      </c>
       <c r="BS14" t="str">
         <v/>
       </c>
-      <c r="BT14">
+      <c r="BT14" t="str">
+        <v/>
+      </c>
+      <c r="BU14">
         <v>0.16</v>
       </c>
-      <c r="BU14" t="str">
-        <v/>
-      </c>
-      <c r="BV14">
+      <c r="BV14" t="str">
+        <v/>
+      </c>
+      <c r="BW14">
         <v>0.16</v>
       </c>
-      <c r="BW14" t="str">
-        <v/>
-      </c>
       <c r="BX14" t="str">
         <v/>
       </c>
       <c r="BY14" t="str">
         <v/>
       </c>
-      <c r="BZ14">
+      <c r="BZ14" t="str">
+        <v/>
+      </c>
+      <c r="CA14">
         <v>0.16</v>
       </c>
-      <c r="CA14" t="str">
-        <v/>
-      </c>
-      <c r="CB14">
+      <c r="CB14" t="str">
+        <v/>
+      </c>
+      <c r="CC14">
         <v>0.16</v>
       </c>
-      <c r="CC14" t="str">
-        <v/>
-      </c>
-      <c r="CD14">
-        <v>0.16</v>
+      <c r="CD14" t="str">
+        <v/>
       </c>
       <c r="CE14">
         <v>0.16</v>
       </c>
-      <c r="CF14" t="str">
-        <v/>
+      <c r="CF14">
+        <v>0.16</v>
       </c>
       <c r="CG14" t="str">
         <v/>
       </c>
-      <c r="CH14">
+      <c r="CH14" t="str">
+        <v/>
+      </c>
+      <c r="CI14">
         <v>0.16</v>
       </c>
-      <c r="CI14" t="str">
-        <v/>
-      </c>
       <c r="CJ14" t="str">
         <v/>
       </c>
-      <c r="CK14">
-        <v>0.16</v>
+      <c r="CK14" t="str">
+        <v/>
       </c>
       <c r="CL14">
         <v>0.16</v>
       </c>
-      <c r="CM14" t="str">
-        <v/>
+      <c r="CM14">
+        <v>0.16</v>
       </c>
       <c r="CN14" t="str">
         <v/>
       </c>
-      <c r="CO14">
+      <c r="CO14" t="str">
+        <v/>
+      </c>
+      <c r="CP14">
         <v>0.16</v>
       </c>
-      <c r="CP14" t="str">
-        <v/>
-      </c>
-      <c r="CQ14">
-        <v>0.16</v>
+      <c r="CQ14" t="str">
+        <v/>
       </c>
       <c r="CR14">
         <v>0.16</v>
@@ -24557,13 +24557,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AN1" t="str">
+        <v>Office Hours Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="AO1" t="str">
+        <v>Office Hours Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="AP1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="AO1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="AP1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -24572,19 +24572,19 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AS1" t="str">
-        <v>Office Hours Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AT1" t="str">
-        <v>Office Hours Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AU1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AW1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="AX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -24596,31 +24596,31 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BA1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BB1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BC1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BD1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BE1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BF1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BG1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BH1" t="str">
         <v>Specialised Care Client 09:00-12:00 (420m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BI1" t="str">
         <v>Specialised Care Client 14:00-17:00 (420m)</v>
-      </c>
-      <c r="BH1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BI1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BJ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
@@ -24641,31 +24641,31 @@
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BP1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BQ1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BR1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BQ1" t="str">
+      <c r="BS1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BR1" t="str">
+      <c r="BT1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BS1" t="str">
+      <c r="BU1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (180m)</v>
-      </c>
-      <c r="BT1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BU1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BW1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BX1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BY1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
@@ -24674,19 +24674,19 @@
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
       <c r="CA1" t="str">
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="CB1" t="str">
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="CC1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="CB1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="CC1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="CD1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CE1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="CF1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -24698,7 +24698,7 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CI1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="CJ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -24888,17 +24888,17 @@
       <c r="BE2">
         <v>0.16</v>
       </c>
-      <c r="BF2" t="str">
-        <v/>
-      </c>
-      <c r="BG2" t="str">
-        <v/>
-      </c>
-      <c r="BH2">
+      <c r="BF2">
         <v>0.16</v>
       </c>
-      <c r="BI2">
+      <c r="BG2">
         <v>0.16</v>
+      </c>
+      <c r="BH2" t="str">
+        <v/>
+      </c>
+      <c r="BI2" t="str">
+        <v/>
       </c>
       <c r="BJ2">
         <v>0.16</v>
@@ -25166,17 +25166,17 @@
       <c r="BE3">
         <v>0</v>
       </c>
-      <c r="BF3" t="str">
-        <v/>
-      </c>
-      <c r="BG3" t="str">
-        <v/>
-      </c>
-      <c r="BH3">
-        <v>0</v>
-      </c>
-      <c r="BI3">
-        <v>0</v>
+      <c r="BF3">
+        <v>0</v>
+      </c>
+      <c r="BG3">
+        <v>0</v>
+      </c>
+      <c r="BH3" t="str">
+        <v/>
+      </c>
+      <c r="BI3" t="str">
+        <v/>
       </c>
       <c r="BJ3">
         <v>0</v>
@@ -25444,17 +25444,17 @@
       <c r="BE4">
         <v>0</v>
       </c>
-      <c r="BF4" t="str">
-        <v/>
-      </c>
-      <c r="BG4" t="str">
-        <v/>
-      </c>
-      <c r="BH4">
-        <v>0</v>
-      </c>
-      <c r="BI4">
-        <v>0</v>
+      <c r="BF4">
+        <v>0</v>
+      </c>
+      <c r="BG4">
+        <v>0</v>
+      </c>
+      <c r="BH4" t="str">
+        <v/>
+      </c>
+      <c r="BI4" t="str">
+        <v/>
       </c>
       <c r="BJ4">
         <v>0</v>
@@ -25671,8 +25671,8 @@
       <c r="AN5">
         <v>0</v>
       </c>
-      <c r="AO5">
-        <v>0</v>
+      <c r="AO5" t="str">
+        <v/>
       </c>
       <c r="AP5">
         <v>0</v>
@@ -25686,8 +25686,8 @@
       <c r="AS5">
         <v>0</v>
       </c>
-      <c r="AT5" t="str">
-        <v/>
+      <c r="AT5">
+        <v>0</v>
       </c>
       <c r="AU5">
         <v>0</v>
@@ -25695,8 +25695,8 @@
       <c r="AV5">
         <v>0</v>
       </c>
-      <c r="AW5">
-        <v>0</v>
+      <c r="AW5" t="str">
+        <v/>
       </c>
       <c r="AX5">
         <v>0</v>
@@ -25710,8 +25710,8 @@
       <c r="BA5">
         <v>0</v>
       </c>
-      <c r="BB5" t="str">
-        <v/>
+      <c r="BB5">
+        <v>0</v>
       </c>
       <c r="BC5">
         <v>0</v>
@@ -25719,17 +25719,17 @@
       <c r="BD5">
         <v>0</v>
       </c>
-      <c r="BE5" t="str">
-        <v/>
-      </c>
-      <c r="BF5" t="str">
-        <v/>
+      <c r="BE5">
+        <v>0</v>
+      </c>
+      <c r="BF5">
+        <v>0</v>
       </c>
       <c r="BG5" t="str">
         <v/>
       </c>
-      <c r="BH5">
-        <v>0</v>
+      <c r="BH5" t="str">
+        <v/>
       </c>
       <c r="BI5" t="str">
         <v/>
@@ -25755,17 +25755,17 @@
       <c r="BP5">
         <v>0</v>
       </c>
-      <c r="BQ5">
-        <v>0</v>
-      </c>
-      <c r="BR5" t="str">
-        <v/>
+      <c r="BQ5" t="str">
+        <v/>
+      </c>
+      <c r="BR5">
+        <v>0</v>
       </c>
       <c r="BS5">
         <v>0</v>
       </c>
-      <c r="BT5">
-        <v>0</v>
+      <c r="BT5" t="str">
+        <v/>
       </c>
       <c r="BU5">
         <v>0</v>
@@ -25776,8 +25776,8 @@
       <c r="BW5">
         <v>0</v>
       </c>
-      <c r="BX5" t="str">
-        <v/>
+      <c r="BX5">
+        <v>0</v>
       </c>
       <c r="BY5">
         <v>0</v>
@@ -25788,17 +25788,17 @@
       <c r="CA5">
         <v>0</v>
       </c>
-      <c r="CB5">
-        <v>0</v>
-      </c>
-      <c r="CC5" t="str">
-        <v/>
+      <c r="CB5" t="str">
+        <v/>
+      </c>
+      <c r="CC5">
+        <v>0</v>
       </c>
       <c r="CD5">
         <v>0</v>
       </c>
-      <c r="CE5">
-        <v>0</v>
+      <c r="CE5" t="str">
+        <v/>
       </c>
       <c r="CF5">
         <v>0</v>
@@ -26227,8 +26227,8 @@
       <c r="AN7">
         <v>0.05</v>
       </c>
-      <c r="AO7">
-        <v>0.05</v>
+      <c r="AO7" t="str">
+        <v/>
       </c>
       <c r="AP7">
         <v>0.05</v>
@@ -26242,8 +26242,8 @@
       <c r="AS7">
         <v>0.05</v>
       </c>
-      <c r="AT7" t="str">
-        <v/>
+      <c r="AT7">
+        <v>0.05</v>
       </c>
       <c r="AU7">
         <v>0.05</v>
@@ -26251,8 +26251,8 @@
       <c r="AV7">
         <v>0.05</v>
       </c>
-      <c r="AW7">
-        <v>0.05</v>
+      <c r="AW7" t="str">
+        <v/>
       </c>
       <c r="AX7">
         <v>0.05</v>
@@ -26266,8 +26266,8 @@
       <c r="BA7">
         <v>0.05</v>
       </c>
-      <c r="BB7" t="str">
-        <v/>
+      <c r="BB7">
+        <v>0.05</v>
       </c>
       <c r="BC7">
         <v>0.05</v>
@@ -26275,17 +26275,17 @@
       <c r="BD7">
         <v>0.05</v>
       </c>
-      <c r="BE7" t="str">
-        <v/>
-      </c>
-      <c r="BF7" t="str">
-        <v/>
+      <c r="BE7">
+        <v>0.05</v>
+      </c>
+      <c r="BF7">
+        <v>0.05</v>
       </c>
       <c r="BG7" t="str">
         <v/>
       </c>
-      <c r="BH7">
-        <v>0.05</v>
+      <c r="BH7" t="str">
+        <v/>
       </c>
       <c r="BI7" t="str">
         <v/>
@@ -26311,20 +26311,20 @@
       <c r="BP7">
         <v>0.05</v>
       </c>
-      <c r="BQ7">
+      <c r="BQ7" t="str">
+        <v/>
+      </c>
+      <c r="BR7">
         <v>0.05</v>
       </c>
-      <c r="BR7" t="str">
-        <v/>
-      </c>
-      <c r="BS7" t="str">
-        <v/>
-      </c>
-      <c r="BT7">
+      <c r="BS7">
         <v>0.05</v>
       </c>
-      <c r="BU7">
-        <v>0.05</v>
+      <c r="BT7" t="str">
+        <v/>
+      </c>
+      <c r="BU7" t="str">
+        <v/>
       </c>
       <c r="BV7">
         <v>0.05</v>
@@ -26332,8 +26332,8 @@
       <c r="BW7">
         <v>0.05</v>
       </c>
-      <c r="BX7" t="str">
-        <v/>
+      <c r="BX7">
+        <v>0.05</v>
       </c>
       <c r="BY7">
         <v>0.05</v>
@@ -26344,17 +26344,17 @@
       <c r="CA7">
         <v>0.05</v>
       </c>
-      <c r="CB7">
+      <c r="CB7" t="str">
+        <v/>
+      </c>
+      <c r="CC7">
         <v>0.05</v>
-      </c>
-      <c r="CC7" t="str">
-        <v/>
       </c>
       <c r="CD7">
         <v>0.05</v>
       </c>
-      <c r="CE7">
-        <v>0.05</v>
+      <c r="CE7" t="str">
+        <v/>
       </c>
       <c r="CF7">
         <v>0.05</v>
@@ -26505,8 +26505,8 @@
       <c r="AN8">
         <v>0.08</v>
       </c>
-      <c r="AO8">
-        <v>0.08</v>
+      <c r="AO8" t="str">
+        <v/>
       </c>
       <c r="AP8">
         <v>0.08</v>
@@ -26520,8 +26520,8 @@
       <c r="AS8">
         <v>0.08</v>
       </c>
-      <c r="AT8" t="str">
-        <v/>
+      <c r="AT8">
+        <v>0.08</v>
       </c>
       <c r="AU8">
         <v>0.08</v>
@@ -26529,8 +26529,8 @@
       <c r="AV8">
         <v>0.08</v>
       </c>
-      <c r="AW8">
-        <v>0.08</v>
+      <c r="AW8" t="str">
+        <v/>
       </c>
       <c r="AX8">
         <v>0.08</v>
@@ -26544,8 +26544,8 @@
       <c r="BA8">
         <v>0.08</v>
       </c>
-      <c r="BB8" t="str">
-        <v/>
+      <c r="BB8">
+        <v>0.08</v>
       </c>
       <c r="BC8">
         <v>0.08</v>
@@ -26553,17 +26553,17 @@
       <c r="BD8">
         <v>0.08</v>
       </c>
-      <c r="BE8" t="str">
-        <v/>
-      </c>
-      <c r="BF8" t="str">
-        <v/>
+      <c r="BE8">
+        <v>0.08</v>
+      </c>
+      <c r="BF8">
+        <v>0.08</v>
       </c>
       <c r="BG8" t="str">
         <v/>
       </c>
-      <c r="BH8">
-        <v>0.08</v>
+      <c r="BH8" t="str">
+        <v/>
       </c>
       <c r="BI8" t="str">
         <v/>
@@ -26589,17 +26589,17 @@
       <c r="BP8">
         <v>0.08</v>
       </c>
-      <c r="BQ8">
+      <c r="BQ8" t="str">
+        <v/>
+      </c>
+      <c r="BR8">
         <v>0.08</v>
-      </c>
-      <c r="BR8" t="str">
-        <v/>
       </c>
       <c r="BS8">
         <v>0.08</v>
       </c>
-      <c r="BT8">
-        <v>0.08</v>
+      <c r="BT8" t="str">
+        <v/>
       </c>
       <c r="BU8">
         <v>0.08</v>
@@ -26610,8 +26610,8 @@
       <c r="BW8">
         <v>0.08</v>
       </c>
-      <c r="BX8" t="str">
-        <v/>
+      <c r="BX8">
+        <v>0.08</v>
       </c>
       <c r="BY8">
         <v>0.08</v>
@@ -26622,17 +26622,17 @@
       <c r="CA8">
         <v>0.08</v>
       </c>
-      <c r="CB8">
+      <c r="CB8" t="str">
+        <v/>
+      </c>
+      <c r="CC8">
         <v>0.08</v>
-      </c>
-      <c r="CC8" t="str">
-        <v/>
       </c>
       <c r="CD8">
         <v>0.08</v>
       </c>
-      <c r="CE8">
-        <v>0.08</v>
+      <c r="CE8" t="str">
+        <v/>
       </c>
       <c r="CF8">
         <v>0.08</v>
@@ -26783,8 +26783,8 @@
       <c r="AN9">
         <v>0</v>
       </c>
-      <c r="AO9">
-        <v>0</v>
+      <c r="AO9" t="str">
+        <v/>
       </c>
       <c r="AP9">
         <v>0</v>
@@ -26798,8 +26798,8 @@
       <c r="AS9">
         <v>0</v>
       </c>
-      <c r="AT9" t="str">
-        <v/>
+      <c r="AT9">
+        <v>0</v>
       </c>
       <c r="AU9">
         <v>0</v>
@@ -26831,17 +26831,17 @@
       <c r="BD9">
         <v>0</v>
       </c>
-      <c r="BE9" t="str">
-        <v/>
-      </c>
-      <c r="BF9" t="str">
-        <v/>
+      <c r="BE9">
+        <v>0</v>
+      </c>
+      <c r="BF9">
+        <v>0</v>
       </c>
       <c r="BG9" t="str">
         <v/>
       </c>
-      <c r="BH9">
-        <v>0</v>
+      <c r="BH9" t="str">
+        <v/>
       </c>
       <c r="BI9" t="str">
         <v/>
@@ -26867,17 +26867,17 @@
       <c r="BP9">
         <v>0</v>
       </c>
-      <c r="BQ9">
-        <v>0</v>
-      </c>
-      <c r="BR9" t="str">
-        <v/>
+      <c r="BQ9" t="str">
+        <v/>
+      </c>
+      <c r="BR9">
+        <v>0</v>
       </c>
       <c r="BS9">
         <v>0</v>
       </c>
-      <c r="BT9">
-        <v>0</v>
+      <c r="BT9" t="str">
+        <v/>
       </c>
       <c r="BU9">
         <v>0</v>
@@ -26888,8 +26888,8 @@
       <c r="BW9">
         <v>0</v>
       </c>
-      <c r="BX9" t="str">
-        <v/>
+      <c r="BX9">
+        <v>0</v>
       </c>
       <c r="BY9">
         <v>0</v>
@@ -26900,8 +26900,8 @@
       <c r="CA9">
         <v>0</v>
       </c>
-      <c r="CB9">
-        <v>0</v>
+      <c r="CB9" t="str">
+        <v/>
       </c>
       <c r="CC9">
         <v>0</v>
@@ -27112,17 +27112,17 @@
       <c r="BE10">
         <v>0.1</v>
       </c>
-      <c r="BF10" t="str">
-        <v/>
-      </c>
-      <c r="BG10" t="str">
-        <v/>
-      </c>
-      <c r="BH10">
+      <c r="BF10">
         <v>0.1</v>
       </c>
-      <c r="BI10">
+      <c r="BG10">
         <v>0.1</v>
+      </c>
+      <c r="BH10" t="str">
+        <v/>
+      </c>
+      <c r="BI10" t="str">
+        <v/>
       </c>
       <c r="BJ10">
         <v>0.1</v>
@@ -27390,17 +27390,17 @@
       <c r="BE11">
         <v>0.01</v>
       </c>
-      <c r="BF11" t="str">
-        <v/>
-      </c>
-      <c r="BG11" t="str">
-        <v/>
-      </c>
-      <c r="BH11">
+      <c r="BF11">
         <v>0.01</v>
       </c>
-      <c r="BI11">
+      <c r="BG11">
         <v>0.01</v>
+      </c>
+      <c r="BH11" t="str">
+        <v/>
+      </c>
+      <c r="BI11" t="str">
+        <v/>
       </c>
       <c r="BJ11">
         <v>0.01</v>
@@ -27668,17 +27668,17 @@
       <c r="BE12">
         <v>0</v>
       </c>
-      <c r="BF12" t="str">
-        <v/>
-      </c>
-      <c r="BG12" t="str">
-        <v/>
-      </c>
-      <c r="BH12">
-        <v>0</v>
-      </c>
-      <c r="BI12">
-        <v>0</v>
+      <c r="BF12">
+        <v>0</v>
+      </c>
+      <c r="BG12">
+        <v>0</v>
+      </c>
+      <c r="BH12" t="str">
+        <v/>
+      </c>
+      <c r="BI12" t="str">
+        <v/>
       </c>
       <c r="BJ12">
         <v>0</v>
@@ -27946,17 +27946,17 @@
       <c r="BE13">
         <v>0</v>
       </c>
-      <c r="BF13" t="str">
-        <v/>
-      </c>
-      <c r="BG13" t="str">
-        <v/>
-      </c>
-      <c r="BH13">
-        <v>0</v>
-      </c>
-      <c r="BI13">
-        <v>0</v>
+      <c r="BF13">
+        <v>0</v>
+      </c>
+      <c r="BG13">
+        <v>0</v>
+      </c>
+      <c r="BH13" t="str">
+        <v/>
+      </c>
+      <c r="BI13" t="str">
+        <v/>
       </c>
       <c r="BJ13">
         <v>0</v>
@@ -28173,10 +28173,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AK1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AL1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="AM1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -28194,7 +28194,7 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AR1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AS1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -28203,10 +28203,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AU1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AV1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AW1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -28215,82 +28215,82 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AY1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AZ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BA1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BA1" t="str">
+      <c r="BB1" t="str">
         <v>Specialised Care Client 09:00-12:00 (360m)</v>
       </c>
-      <c r="BB1" t="str">
+      <c r="BC1" t="str">
         <v>Specialised Care Client 14:00-17:00 (360m)</v>
       </c>
-      <c r="BC1" t="str">
+      <c r="BD1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BD1" t="str">
+      <c r="BE1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BF1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BG1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BH1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BI1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BJ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (240m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BK1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BK1" t="str">
+      <c r="BL1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BL1" t="str">
+      <c r="BM1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BM1" t="str">
+      <c r="BN1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BN1" t="str">
+      <c r="BO1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BO1" t="str">
+      <c r="BP1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BP1" t="str">
+      <c r="BQ1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BQ1" t="str">
+      <c r="BR1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BR1" t="str">
+      <c r="BS1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BS1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BU1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (180m)</v>
       </c>
-      <c r="BV1" t="str">
+      <c r="BW1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
-      <c r="BW1" t="str">
+      <c r="BX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BX1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BY1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -28471,14 +28471,14 @@
       <c r="AZ2">
         <v>0.25</v>
       </c>
-      <c r="BA2" t="str">
-        <v/>
+      <c r="BA2">
+        <v>0.25</v>
       </c>
       <c r="BB2" t="str">
         <v/>
       </c>
-      <c r="BC2">
-        <v>0.25</v>
+      <c r="BC2" t="str">
+        <v/>
       </c>
       <c r="BD2">
         <v>0.25</v>
@@ -28677,8 +28677,8 @@
       <c r="AK3">
         <v>0.07</v>
       </c>
-      <c r="AL3">
-        <v>0.07</v>
+      <c r="AL3" t="str">
+        <v/>
       </c>
       <c r="AM3">
         <v>0.07</v>
@@ -28695,8 +28695,8 @@
       <c r="AQ3">
         <v>0.07</v>
       </c>
-      <c r="AR3" t="str">
-        <v/>
+      <c r="AR3">
+        <v>0.07</v>
       </c>
       <c r="AS3">
         <v>0.07</v>
@@ -28719,8 +28719,8 @@
       <c r="AY3">
         <v>0.07</v>
       </c>
-      <c r="AZ3" t="str">
-        <v/>
+      <c r="AZ3">
+        <v>0.07</v>
       </c>
       <c r="BA3" t="str">
         <v/>
@@ -28728,56 +28728,56 @@
       <c r="BB3" t="str">
         <v/>
       </c>
-      <c r="BC3">
+      <c r="BC3" t="str">
+        <v/>
+      </c>
+      <c r="BD3">
         <v>0.07</v>
       </c>
-      <c r="BD3" t="str">
-        <v/>
-      </c>
-      <c r="BE3">
+      <c r="BE3" t="str">
+        <v/>
+      </c>
+      <c r="BF3">
         <v>0.07</v>
       </c>
-      <c r="BF3" t="str">
-        <v/>
-      </c>
-      <c r="BG3">
+      <c r="BG3" t="str">
+        <v/>
+      </c>
+      <c r="BH3">
         <v>0.07</v>
       </c>
-      <c r="BH3" t="str">
-        <v/>
-      </c>
       <c r="BI3" t="str">
         <v/>
       </c>
-      <c r="BJ3">
+      <c r="BJ3" t="str">
+        <v/>
+      </c>
+      <c r="BK3">
         <v>0.07</v>
       </c>
-      <c r="BK3" t="str">
-        <v/>
-      </c>
-      <c r="BL3">
+      <c r="BL3" t="str">
+        <v/>
+      </c>
+      <c r="BM3">
         <v>0.07</v>
       </c>
-      <c r="BM3" t="str">
-        <v/>
-      </c>
-      <c r="BN3">
-        <v>0.07</v>
+      <c r="BN3" t="str">
+        <v/>
       </c>
       <c r="BO3">
         <v>0.07</v>
       </c>
-      <c r="BP3" t="str">
-        <v/>
-      </c>
-      <c r="BQ3">
+      <c r="BP3">
         <v>0.07</v>
       </c>
-      <c r="BR3" t="str">
-        <v/>
-      </c>
-      <c r="BS3">
+      <c r="BQ3" t="str">
+        <v/>
+      </c>
+      <c r="BR3">
         <v>0.07</v>
+      </c>
+      <c r="BS3" t="str">
+        <v/>
       </c>
       <c r="BT3">
         <v>0.07</v>
@@ -28785,11 +28785,11 @@
       <c r="BU3">
         <v>0.07</v>
       </c>
-      <c r="BV3" t="str">
-        <v/>
-      </c>
-      <c r="BW3">
+      <c r="BV3">
         <v>0.07</v>
+      </c>
+      <c r="BW3" t="str">
+        <v/>
       </c>
       <c r="BX3">
         <v>0.07</v>
@@ -28928,8 +28928,8 @@
       <c r="AK4">
         <v>0.13</v>
       </c>
-      <c r="AL4">
-        <v>0.13</v>
+      <c r="AL4" t="str">
+        <v/>
       </c>
       <c r="AM4">
         <v>0.13</v>
@@ -28946,8 +28946,8 @@
       <c r="AQ4">
         <v>0.13</v>
       </c>
-      <c r="AR4" t="str">
-        <v/>
+      <c r="AR4">
+        <v>0.13</v>
       </c>
       <c r="AS4">
         <v>0.13</v>
@@ -28970,8 +28970,8 @@
       <c r="AY4">
         <v>0.13</v>
       </c>
-      <c r="AZ4" t="str">
-        <v/>
+      <c r="AZ4">
+        <v>0.13</v>
       </c>
       <c r="BA4" t="str">
         <v/>
@@ -28979,56 +28979,56 @@
       <c r="BB4" t="str">
         <v/>
       </c>
-      <c r="BC4">
+      <c r="BC4" t="str">
+        <v/>
+      </c>
+      <c r="BD4">
         <v>0.13</v>
       </c>
-      <c r="BD4" t="str">
-        <v/>
-      </c>
-      <c r="BE4">
+      <c r="BE4" t="str">
+        <v/>
+      </c>
+      <c r="BF4">
         <v>0.13</v>
       </c>
-      <c r="BF4" t="str">
-        <v/>
-      </c>
-      <c r="BG4">
+      <c r="BG4" t="str">
+        <v/>
+      </c>
+      <c r="BH4">
         <v>0.13</v>
       </c>
-      <c r="BH4" t="str">
-        <v/>
-      </c>
       <c r="BI4" t="str">
         <v/>
       </c>
-      <c r="BJ4">
+      <c r="BJ4" t="str">
+        <v/>
+      </c>
+      <c r="BK4">
         <v>0.13</v>
       </c>
-      <c r="BK4" t="str">
-        <v/>
-      </c>
-      <c r="BL4">
+      <c r="BL4" t="str">
+        <v/>
+      </c>
+      <c r="BM4">
         <v>0.13</v>
       </c>
-      <c r="BM4" t="str">
-        <v/>
-      </c>
-      <c r="BN4">
-        <v>0.13</v>
+      <c r="BN4" t="str">
+        <v/>
       </c>
       <c r="BO4">
         <v>0.13</v>
       </c>
-      <c r="BP4" t="str">
-        <v/>
-      </c>
-      <c r="BQ4">
+      <c r="BP4">
         <v>0.13</v>
       </c>
-      <c r="BR4" t="str">
-        <v/>
-      </c>
-      <c r="BS4">
+      <c r="BQ4" t="str">
+        <v/>
+      </c>
+      <c r="BR4">
         <v>0.13</v>
+      </c>
+      <c r="BS4" t="str">
+        <v/>
       </c>
       <c r="BT4">
         <v>0.13</v>
@@ -29036,11 +29036,11 @@
       <c r="BU4">
         <v>0.13</v>
       </c>
-      <c r="BV4" t="str">
-        <v/>
-      </c>
-      <c r="BW4">
+      <c r="BV4">
         <v>0.13</v>
+      </c>
+      <c r="BW4" t="str">
+        <v/>
       </c>
       <c r="BX4">
         <v>0.13</v>
@@ -29179,8 +29179,8 @@
       <c r="AK5">
         <v>0.78</v>
       </c>
-      <c r="AL5">
-        <v>0.78</v>
+      <c r="AL5" t="str">
+        <v/>
       </c>
       <c r="AM5">
         <v>0.78</v>
@@ -29197,8 +29197,8 @@
       <c r="AQ5">
         <v>0.78</v>
       </c>
-      <c r="AR5" t="str">
-        <v/>
+      <c r="AR5">
+        <v>0.78</v>
       </c>
       <c r="AS5">
         <v>0.78</v>
@@ -29221,8 +29221,8 @@
       <c r="AY5">
         <v>0.78</v>
       </c>
-      <c r="AZ5" t="str">
-        <v/>
+      <c r="AZ5">
+        <v>0.78</v>
       </c>
       <c r="BA5" t="str">
         <v/>
@@ -29230,56 +29230,56 @@
       <c r="BB5" t="str">
         <v/>
       </c>
-      <c r="BC5">
+      <c r="BC5" t="str">
+        <v/>
+      </c>
+      <c r="BD5">
         <v>0.78</v>
       </c>
-      <c r="BD5" t="str">
-        <v/>
-      </c>
-      <c r="BE5">
+      <c r="BE5" t="str">
+        <v/>
+      </c>
+      <c r="BF5">
         <v>0.78</v>
       </c>
-      <c r="BF5" t="str">
-        <v/>
-      </c>
-      <c r="BG5">
+      <c r="BG5" t="str">
+        <v/>
+      </c>
+      <c r="BH5">
         <v>0.78</v>
       </c>
-      <c r="BH5" t="str">
-        <v/>
-      </c>
-      <c r="BI5">
-        <v>0.78</v>
+      <c r="BI5" t="str">
+        <v/>
       </c>
       <c r="BJ5">
         <v>0.78</v>
       </c>
-      <c r="BK5" t="str">
-        <v/>
-      </c>
-      <c r="BL5">
+      <c r="BK5">
         <v>0.78</v>
       </c>
-      <c r="BM5" t="str">
-        <v/>
-      </c>
-      <c r="BN5">
+      <c r="BL5" t="str">
+        <v/>
+      </c>
+      <c r="BM5">
         <v>0.78</v>
+      </c>
+      <c r="BN5" t="str">
+        <v/>
       </c>
       <c r="BO5">
         <v>0.78</v>
       </c>
-      <c r="BP5" t="str">
-        <v/>
-      </c>
-      <c r="BQ5">
+      <c r="BP5">
         <v>0.78</v>
       </c>
-      <c r="BR5" t="str">
-        <v/>
-      </c>
-      <c r="BS5">
+      <c r="BQ5" t="str">
+        <v/>
+      </c>
+      <c r="BR5">
         <v>0.78</v>
+      </c>
+      <c r="BS5" t="str">
+        <v/>
       </c>
       <c r="BT5">
         <v>0.78</v>
@@ -29287,11 +29287,11 @@
       <c r="BU5">
         <v>0.78</v>
       </c>
-      <c r="BV5" t="str">
-        <v/>
-      </c>
-      <c r="BW5">
+      <c r="BV5">
         <v>0.78</v>
+      </c>
+      <c r="BW5" t="str">
+        <v/>
       </c>
       <c r="BX5">
         <v>0.78</v>
@@ -29977,14 +29977,14 @@
       <c r="AZ8">
         <v>0.25</v>
       </c>
-      <c r="BA8" t="str">
-        <v/>
+      <c r="BA8">
+        <v>0.25</v>
       </c>
       <c r="BB8" t="str">
         <v/>
       </c>
-      <c r="BC8">
-        <v>0.25</v>
+      <c r="BC8" t="str">
+        <v/>
       </c>
       <c r="BD8">
         <v>0.25</v>
@@ -30183,8 +30183,8 @@
       <c r="AK9">
         <v>0.08</v>
       </c>
-      <c r="AL9">
-        <v>0.08</v>
+      <c r="AL9" t="str">
+        <v/>
       </c>
       <c r="AM9">
         <v>0.08</v>
@@ -30201,8 +30201,8 @@
       <c r="AQ9">
         <v>0.08</v>
       </c>
-      <c r="AR9" t="str">
-        <v/>
+      <c r="AR9">
+        <v>0.08</v>
       </c>
       <c r="AS9">
         <v>0.08</v>
@@ -30225,8 +30225,8 @@
       <c r="AY9">
         <v>0.08</v>
       </c>
-      <c r="AZ9" t="str">
-        <v/>
+      <c r="AZ9">
+        <v>0.08</v>
       </c>
       <c r="BA9" t="str">
         <v/>
@@ -30234,56 +30234,56 @@
       <c r="BB9" t="str">
         <v/>
       </c>
-      <c r="BC9">
+      <c r="BC9" t="str">
+        <v/>
+      </c>
+      <c r="BD9">
         <v>0.08</v>
       </c>
-      <c r="BD9" t="str">
-        <v/>
-      </c>
-      <c r="BE9">
+      <c r="BE9" t="str">
+        <v/>
+      </c>
+      <c r="BF9">
         <v>0.08</v>
       </c>
-      <c r="BF9" t="str">
-        <v/>
-      </c>
-      <c r="BG9">
+      <c r="BG9" t="str">
+        <v/>
+      </c>
+      <c r="BH9">
         <v>0.08</v>
       </c>
-      <c r="BH9" t="str">
-        <v/>
-      </c>
-      <c r="BI9">
-        <v>0.08</v>
+      <c r="BI9" t="str">
+        <v/>
       </c>
       <c r="BJ9">
         <v>0.08</v>
       </c>
-      <c r="BK9" t="str">
-        <v/>
-      </c>
-      <c r="BL9">
+      <c r="BK9">
         <v>0.08</v>
       </c>
-      <c r="BM9" t="str">
-        <v/>
-      </c>
-      <c r="BN9">
+      <c r="BL9" t="str">
+        <v/>
+      </c>
+      <c r="BM9">
         <v>0.08</v>
+      </c>
+      <c r="BN9" t="str">
+        <v/>
       </c>
       <c r="BO9">
         <v>0.08</v>
       </c>
-      <c r="BP9" t="str">
-        <v/>
-      </c>
-      <c r="BQ9">
+      <c r="BP9">
         <v>0.08</v>
       </c>
-      <c r="BR9" t="str">
-        <v/>
-      </c>
-      <c r="BS9">
+      <c r="BQ9" t="str">
+        <v/>
+      </c>
+      <c r="BR9">
         <v>0.08</v>
+      </c>
+      <c r="BS9" t="str">
+        <v/>
       </c>
       <c r="BT9">
         <v>0.08</v>
@@ -30291,11 +30291,11 @@
       <c r="BU9">
         <v>0.08</v>
       </c>
-      <c r="BV9" t="str">
-        <v/>
-      </c>
-      <c r="BW9">
+      <c r="BV9">
         <v>0.08</v>
+      </c>
+      <c r="BW9" t="str">
+        <v/>
       </c>
       <c r="BX9">
         <v>0.08</v>
@@ -30476,8 +30476,8 @@
       <c r="AY10">
         <v>0</v>
       </c>
-      <c r="AZ10" t="str">
-        <v/>
+      <c r="AZ10">
+        <v>0</v>
       </c>
       <c r="BA10" t="str">
         <v/>
@@ -30485,56 +30485,56 @@
       <c r="BB10" t="str">
         <v/>
       </c>
-      <c r="BC10">
-        <v>0</v>
-      </c>
-      <c r="BD10" t="str">
-        <v/>
-      </c>
-      <c r="BE10">
-        <v>0</v>
-      </c>
-      <c r="BF10" t="str">
-        <v/>
-      </c>
-      <c r="BG10">
-        <v>0</v>
-      </c>
-      <c r="BH10" t="str">
-        <v/>
-      </c>
-      <c r="BI10">
-        <v>0</v>
+      <c r="BC10" t="str">
+        <v/>
+      </c>
+      <c r="BD10">
+        <v>0</v>
+      </c>
+      <c r="BE10" t="str">
+        <v/>
+      </c>
+      <c r="BF10">
+        <v>0</v>
+      </c>
+      <c r="BG10" t="str">
+        <v/>
+      </c>
+      <c r="BH10">
+        <v>0</v>
+      </c>
+      <c r="BI10" t="str">
+        <v/>
       </c>
       <c r="BJ10">
         <v>0</v>
       </c>
-      <c r="BK10" t="str">
-        <v/>
-      </c>
-      <c r="BL10">
-        <v>0</v>
-      </c>
-      <c r="BM10" t="str">
-        <v/>
-      </c>
-      <c r="BN10">
-        <v>0</v>
+      <c r="BK10">
+        <v>0</v>
+      </c>
+      <c r="BL10" t="str">
+        <v/>
+      </c>
+      <c r="BM10">
+        <v>0</v>
+      </c>
+      <c r="BN10" t="str">
+        <v/>
       </c>
       <c r="BO10">
         <v>0</v>
       </c>
-      <c r="BP10" t="str">
-        <v/>
-      </c>
-      <c r="BQ10">
-        <v>0</v>
-      </c>
-      <c r="BR10" t="str">
-        <v/>
-      </c>
-      <c r="BS10">
-        <v>0</v>
+      <c r="BP10">
+        <v>0</v>
+      </c>
+      <c r="BQ10" t="str">
+        <v/>
+      </c>
+      <c r="BR10">
+        <v>0</v>
+      </c>
+      <c r="BS10" t="str">
+        <v/>
       </c>
       <c r="BT10">
         <v>0</v>
@@ -30730,14 +30730,14 @@
       <c r="AZ11">
         <v>0.1</v>
       </c>
-      <c r="BA11" t="str">
-        <v/>
+      <c r="BA11">
+        <v>0.1</v>
       </c>
       <c r="BB11" t="str">
         <v/>
       </c>
-      <c r="BC11">
-        <v>0.1</v>
+      <c r="BC11" t="str">
+        <v/>
       </c>
       <c r="BD11">
         <v>0.1</v>
@@ -30981,14 +30981,14 @@
       <c r="AZ12">
         <v>0</v>
       </c>
-      <c r="BA12" t="str">
-        <v/>
+      <c r="BA12">
+        <v>0</v>
       </c>
       <c r="BB12" t="str">
         <v/>
       </c>
-      <c r="BC12">
-        <v>0</v>
+      <c r="BC12" t="str">
+        <v/>
       </c>
       <c r="BD12">
         <v>0</v>
@@ -31232,14 +31232,14 @@
       <c r="AZ13">
         <v>0.14</v>
       </c>
-      <c r="BA13" t="str">
-        <v/>
+      <c r="BA13">
+        <v>0.14</v>
       </c>
       <c r="BB13" t="str">
         <v/>
       </c>
-      <c r="BC13">
-        <v>0.14</v>
+      <c r="BC13" t="str">
+        <v/>
       </c>
       <c r="BD13">
         <v>0.14</v>
@@ -31483,14 +31483,14 @@
       <c r="AZ14">
         <v>0</v>
       </c>
-      <c r="BA14" t="str">
-        <v/>
+      <c r="BA14">
+        <v>0</v>
       </c>
       <c r="BB14" t="str">
         <v/>
       </c>
-      <c r="BC14">
-        <v>0</v>
+      <c r="BC14" t="str">
+        <v/>
       </c>
       <c r="BD14">
         <v>0</v>
@@ -31689,8 +31689,8 @@
       <c r="AK15">
         <v>0</v>
       </c>
-      <c r="AL15">
-        <v>0</v>
+      <c r="AL15" t="str">
+        <v/>
       </c>
       <c r="AM15">
         <v>0</v>
@@ -31707,8 +31707,8 @@
       <c r="AQ15">
         <v>0</v>
       </c>
-      <c r="AR15" t="str">
-        <v/>
+      <c r="AR15">
+        <v>0</v>
       </c>
       <c r="AS15">
         <v>0</v>
@@ -31734,14 +31734,14 @@
       <c r="AZ15">
         <v>0</v>
       </c>
-      <c r="BA15" t="str">
-        <v/>
+      <c r="BA15">
+        <v>0</v>
       </c>
       <c r="BB15" t="str">
         <v/>
       </c>
-      <c r="BC15">
-        <v>0</v>
+      <c r="BC15" t="str">
+        <v/>
       </c>
       <c r="BD15">
         <v>0</v>
@@ -31797,11 +31797,11 @@
       <c r="BU15">
         <v>0</v>
       </c>
-      <c r="BV15" t="str">
-        <v/>
-      </c>
-      <c r="BW15">
-        <v>0</v>
+      <c r="BV15">
+        <v>0</v>
+      </c>
+      <c r="BW15" t="str">
+        <v/>
       </c>
       <c r="BX15">
         <v>0</v>
@@ -31985,14 +31985,14 @@
       <c r="AZ16">
         <v>0.09</v>
       </c>
-      <c r="BA16" t="str">
-        <v/>
+      <c r="BA16">
+        <v>0.09</v>
       </c>
       <c r="BB16" t="str">
         <v/>
       </c>
-      <c r="BC16">
-        <v>0.09</v>
+      <c r="BC16" t="str">
+        <v/>
       </c>
       <c r="BD16">
         <v>0.09</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Improve dashboard rendering by adjusting component hierarchy
Adds stack trace information to the 'attached_assets/Pasted--at-WeeklySchedulingTab-https-f111f999-5923-4927-b1a6-82fa47fe9a5b-00-31gtcnbbujc90.picard.replit.dev/src/components/weekly-scheduling-tab.tsx.txt' file, likely for debugging or performance analysis of the dashboard component and its nested elements like `WeeklySchedulingTab` and `Presence`.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3690,19 +3690,19 @@
         <v>Brown, Christine 33333-.6875 (60m)</v>
       </c>
       <c r="AD1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="AE1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="AE1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AF1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AG1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (165m)</v>
+      </c>
+      <c r="AH1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="AH1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (165m)</v>
       </c>
       <c r="AI1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -3723,13 +3723,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AO1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AP1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AQ1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AR1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -3738,67 +3738,67 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AT1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="AU1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="AV1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="AW1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="AX1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="AY1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="AZ1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BA1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BB1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BC1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BD1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BE1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BF1" t="str">
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BG1" t="str">
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BH1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="AU1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="AV1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="AW1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="AX1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="AY1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="AZ1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BA1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BB1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BC1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BD1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BE1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BF1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BG1" t="str">
+      <c r="BI1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BJ1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BK1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BJ1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BK1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BM1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="BN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BN1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BO1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -3810,10 +3810,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BR1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="BS1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BS1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -16853,16 +16853,16 @@
         <v>Armstrong (NL), Hugh .4375-66667 (60m)</v>
       </c>
       <c r="AF1" t="str">
+        <v>Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="AH1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="AG1" t="str">
+      <c r="AI1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="AH1" t="str">
-        <v>Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="AI1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AJ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -16877,49 +16877,49 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AN1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="AO1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AP1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AR1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="AS1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="AT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="AS1" t="str">
+      <c r="AU1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="AT1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="AU1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AW1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
       <c r="AX1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="AY1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (420m)</v>
+      </c>
+      <c r="AZ1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (420m)</v>
+      </c>
+      <c r="BA1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BB1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BA1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (420m)</v>
-      </c>
-      <c r="BB1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (420m)</v>
       </c>
       <c r="BC1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
@@ -16934,22 +16934,22 @@
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BG1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
       <c r="BH1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BI1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BJ1" t="str">
+        <v>Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BK1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BL1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BK1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BL1" t="str">
-        <v>Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BM1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
@@ -16958,22 +16958,22 @@
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BO1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BP1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+        <v>Office Hours Client 09:00-12:00 (510m)</v>
       </c>
       <c r="BQ1" t="str">
+        <v>Office Hours Client 14:00-17:00 (510m)</v>
+      </c>
+      <c r="BR1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BR1" t="str">
-        <v>Office Hours Client 09:00-12:00 (510m)</v>
-      </c>
       <c r="BS1" t="str">
-        <v>Office Hours Client 14:00-17:00 (510m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BT1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BU1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
@@ -16982,10 +16982,10 @@
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BW1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BX1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BY1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -17157,17 +17157,17 @@
       <c r="AX2">
         <v>0.25</v>
       </c>
-      <c r="AY2">
+      <c r="AY2" t="str">
+        <v/>
+      </c>
+      <c r="AZ2" t="str">
+        <v/>
+      </c>
+      <c r="BA2">
         <v>0.25</v>
       </c>
-      <c r="AZ2">
+      <c r="BB2">
         <v>0.25</v>
-      </c>
-      <c r="BA2" t="str">
-        <v/>
-      </c>
-      <c r="BB2" t="str">
-        <v/>
       </c>
       <c r="BC2">
         <v>0.25</v>
@@ -17208,17 +17208,17 @@
       <c r="BO2">
         <v>0.25</v>
       </c>
-      <c r="BP2">
+      <c r="BP2" t="str">
+        <v/>
+      </c>
+      <c r="BQ2" t="str">
+        <v/>
+      </c>
+      <c r="BR2">
         <v>0.25</v>
       </c>
-      <c r="BQ2">
+      <c r="BS2">
         <v>0.25</v>
-      </c>
-      <c r="BR2" t="str">
-        <v/>
-      </c>
-      <c r="BS2" t="str">
-        <v/>
       </c>
       <c r="BT2">
         <v>0.25</v>
@@ -17405,17 +17405,17 @@
       <c r="AX3">
         <v>0.01</v>
       </c>
-      <c r="AY3">
+      <c r="AY3" t="str">
+        <v/>
+      </c>
+      <c r="AZ3" t="str">
+        <v/>
+      </c>
+      <c r="BA3">
         <v>0.01</v>
       </c>
-      <c r="AZ3">
+      <c r="BB3">
         <v>0.01</v>
-      </c>
-      <c r="BA3" t="str">
-        <v/>
-      </c>
-      <c r="BB3" t="str">
-        <v/>
       </c>
       <c r="BC3">
         <v>0.01</v>
@@ -17456,17 +17456,17 @@
       <c r="BO3">
         <v>0.01</v>
       </c>
-      <c r="BP3">
+      <c r="BP3" t="str">
+        <v/>
+      </c>
+      <c r="BQ3" t="str">
+        <v/>
+      </c>
+      <c r="BR3">
         <v>0.01</v>
       </c>
-      <c r="BQ3">
+      <c r="BS3">
         <v>0.01</v>
-      </c>
-      <c r="BR3" t="str">
-        <v/>
-      </c>
-      <c r="BS3" t="str">
-        <v/>
       </c>
       <c r="BT3">
         <v>0.01</v>
@@ -17620,14 +17620,14 @@
       <c r="AM4">
         <v>0</v>
       </c>
-      <c r="AN4">
-        <v>0</v>
+      <c r="AN4" t="str">
+        <v/>
       </c>
       <c r="AO4">
         <v>0</v>
       </c>
-      <c r="AP4" t="str">
-        <v/>
+      <c r="AP4">
+        <v>0</v>
       </c>
       <c r="AQ4">
         <v>0</v>
@@ -17650,17 +17650,17 @@
       <c r="AW4">
         <v>0</v>
       </c>
-      <c r="AX4">
-        <v>0</v>
-      </c>
-      <c r="AY4">
-        <v>0</v>
+      <c r="AX4" t="str">
+        <v/>
+      </c>
+      <c r="AY4" t="str">
+        <v/>
       </c>
       <c r="AZ4" t="str">
         <v/>
       </c>
-      <c r="BA4" t="str">
-        <v/>
+      <c r="BA4">
+        <v>0</v>
       </c>
       <c r="BB4" t="str">
         <v/>
@@ -17686,14 +17686,14 @@
       <c r="BI4">
         <v>0</v>
       </c>
-      <c r="BJ4" t="str">
-        <v/>
+      <c r="BJ4">
+        <v>0</v>
       </c>
       <c r="BK4">
         <v>0</v>
       </c>
-      <c r="BL4">
-        <v>0</v>
+      <c r="BL4" t="str">
+        <v/>
       </c>
       <c r="BM4">
         <v>0</v>
@@ -17707,14 +17707,14 @@
       <c r="BP4" t="str">
         <v/>
       </c>
-      <c r="BQ4">
-        <v>0</v>
-      </c>
-      <c r="BR4" t="str">
-        <v/>
-      </c>
-      <c r="BS4" t="str">
-        <v/>
+      <c r="BQ4" t="str">
+        <v/>
+      </c>
+      <c r="BR4">
+        <v>0</v>
+      </c>
+      <c r="BS4">
+        <v>0</v>
       </c>
       <c r="BT4">
         <v>0</v>
@@ -18116,14 +18116,14 @@
       <c r="AM6">
         <v>0.05</v>
       </c>
-      <c r="AN6">
-        <v>0.05</v>
+      <c r="AN6" t="str">
+        <v/>
       </c>
       <c r="AO6">
         <v>0.05</v>
       </c>
-      <c r="AP6" t="str">
-        <v/>
+      <c r="AP6">
+        <v>0.05</v>
       </c>
       <c r="AQ6">
         <v>0.05</v>
@@ -18146,17 +18146,17 @@
       <c r="AW6">
         <v>0.05</v>
       </c>
-      <c r="AX6">
+      <c r="AX6" t="str">
+        <v/>
+      </c>
+      <c r="AY6" t="str">
+        <v/>
+      </c>
+      <c r="AZ6" t="str">
+        <v/>
+      </c>
+      <c r="BA6">
         <v>0.05</v>
-      </c>
-      <c r="AY6">
-        <v>0.05</v>
-      </c>
-      <c r="AZ6" t="str">
-        <v/>
-      </c>
-      <c r="BA6" t="str">
-        <v/>
       </c>
       <c r="BB6" t="str">
         <v/>
@@ -18182,14 +18182,14 @@
       <c r="BI6">
         <v>0.05</v>
       </c>
-      <c r="BJ6" t="str">
-        <v/>
+      <c r="BJ6">
+        <v>0.05</v>
       </c>
       <c r="BK6">
         <v>0.05</v>
       </c>
-      <c r="BL6">
-        <v>0.05</v>
+      <c r="BL6" t="str">
+        <v/>
       </c>
       <c r="BM6">
         <v>0.05</v>
@@ -18203,14 +18203,14 @@
       <c r="BP6" t="str">
         <v/>
       </c>
-      <c r="BQ6">
+      <c r="BQ6" t="str">
+        <v/>
+      </c>
+      <c r="BR6">
         <v>0.05</v>
       </c>
-      <c r="BR6" t="str">
-        <v/>
-      </c>
-      <c r="BS6" t="str">
-        <v/>
+      <c r="BS6">
+        <v>0.05</v>
       </c>
       <c r="BT6">
         <v>0.05</v>
@@ -18397,17 +18397,17 @@
       <c r="AX7">
         <v>0</v>
       </c>
-      <c r="AY7">
-        <v>0</v>
-      </c>
-      <c r="AZ7">
-        <v>0</v>
-      </c>
-      <c r="BA7" t="str">
-        <v/>
-      </c>
-      <c r="BB7" t="str">
-        <v/>
+      <c r="AY7" t="str">
+        <v/>
+      </c>
+      <c r="AZ7" t="str">
+        <v/>
+      </c>
+      <c r="BA7">
+        <v>0</v>
+      </c>
+      <c r="BB7">
+        <v>0</v>
       </c>
       <c r="BC7">
         <v>0</v>
@@ -18448,17 +18448,17 @@
       <c r="BO7">
         <v>0</v>
       </c>
-      <c r="BP7">
-        <v>0</v>
-      </c>
-      <c r="BQ7">
-        <v>0</v>
-      </c>
-      <c r="BR7" t="str">
-        <v/>
-      </c>
-      <c r="BS7" t="str">
-        <v/>
+      <c r="BP7" t="str">
+        <v/>
+      </c>
+      <c r="BQ7" t="str">
+        <v/>
+      </c>
+      <c r="BR7">
+        <v>0</v>
+      </c>
+      <c r="BS7">
+        <v>0</v>
       </c>
       <c r="BT7">
         <v>0</v>
@@ -18645,17 +18645,17 @@
       <c r="AX8">
         <v>0.08</v>
       </c>
-      <c r="AY8">
+      <c r="AY8" t="str">
+        <v/>
+      </c>
+      <c r="AZ8" t="str">
+        <v/>
+      </c>
+      <c r="BA8">
         <v>0.08</v>
       </c>
-      <c r="AZ8">
+      <c r="BB8">
         <v>0.08</v>
-      </c>
-      <c r="BA8" t="str">
-        <v/>
-      </c>
-      <c r="BB8" t="str">
-        <v/>
       </c>
       <c r="BC8">
         <v>0.08</v>
@@ -18696,17 +18696,17 @@
       <c r="BO8">
         <v>0.08</v>
       </c>
-      <c r="BP8">
+      <c r="BP8" t="str">
+        <v/>
+      </c>
+      <c r="BQ8" t="str">
+        <v/>
+      </c>
+      <c r="BR8">
         <v>0.08</v>
       </c>
-      <c r="BQ8">
+      <c r="BS8">
         <v>0.08</v>
-      </c>
-      <c r="BR8" t="str">
-        <v/>
-      </c>
-      <c r="BS8" t="str">
-        <v/>
       </c>
       <c r="BT8">
         <v>0.08</v>
@@ -18890,17 +18890,17 @@
       <c r="AW9">
         <v>0</v>
       </c>
-      <c r="AX9">
-        <v>0</v>
-      </c>
-      <c r="AY9">
-        <v>0</v>
+      <c r="AX9" t="str">
+        <v/>
+      </c>
+      <c r="AY9" t="str">
+        <v/>
       </c>
       <c r="AZ9" t="str">
         <v/>
       </c>
-      <c r="BA9" t="str">
-        <v/>
+      <c r="BA9">
+        <v>0</v>
       </c>
       <c r="BB9" t="str">
         <v/>
@@ -18926,14 +18926,14 @@
       <c r="BI9">
         <v>0</v>
       </c>
-      <c r="BJ9" t="str">
-        <v/>
+      <c r="BJ9">
+        <v>0</v>
       </c>
       <c r="BK9">
         <v>0</v>
       </c>
-      <c r="BL9">
-        <v>0</v>
+      <c r="BL9" t="str">
+        <v/>
       </c>
       <c r="BM9">
         <v>0</v>
@@ -18947,14 +18947,14 @@
       <c r="BP9" t="str">
         <v/>
       </c>
-      <c r="BQ9">
-        <v>0</v>
-      </c>
-      <c r="BR9" t="str">
-        <v/>
-      </c>
-      <c r="BS9" t="str">
-        <v/>
+      <c r="BQ9" t="str">
+        <v/>
+      </c>
+      <c r="BR9">
+        <v>0</v>
+      </c>
+      <c r="BS9">
+        <v>0</v>
       </c>
       <c r="BT9">
         <v>0</v>
@@ -19141,17 +19141,17 @@
       <c r="AX10">
         <v>0</v>
       </c>
-      <c r="AY10">
-        <v>0</v>
-      </c>
-      <c r="AZ10">
-        <v>0</v>
-      </c>
-      <c r="BA10" t="str">
-        <v/>
-      </c>
-      <c r="BB10" t="str">
-        <v/>
+      <c r="AY10" t="str">
+        <v/>
+      </c>
+      <c r="AZ10" t="str">
+        <v/>
+      </c>
+      <c r="BA10">
+        <v>0</v>
+      </c>
+      <c r="BB10">
+        <v>0</v>
       </c>
       <c r="BC10">
         <v>0</v>
@@ -19192,17 +19192,17 @@
       <c r="BO10">
         <v>0</v>
       </c>
-      <c r="BP10">
-        <v>0</v>
-      </c>
-      <c r="BQ10">
-        <v>0</v>
-      </c>
-      <c r="BR10" t="str">
-        <v/>
-      </c>
-      <c r="BS10" t="str">
-        <v/>
+      <c r="BP10" t="str">
+        <v/>
+      </c>
+      <c r="BQ10" t="str">
+        <v/>
+      </c>
+      <c r="BR10">
+        <v>0</v>
+      </c>
+      <c r="BS10">
+        <v>0</v>
       </c>
       <c r="BT10">
         <v>0</v>
@@ -19332,17 +19332,17 @@
       <c r="AE11">
         <v>0.88</v>
       </c>
-      <c r="AF11">
+      <c r="AF11" t="str">
+        <v/>
+      </c>
+      <c r="AG11" t="str">
+        <v/>
+      </c>
+      <c r="AH11">
         <v>0.78</v>
       </c>
-      <c r="AG11">
+      <c r="AI11">
         <v>0.78</v>
-      </c>
-      <c r="AH11" t="str">
-        <v/>
-      </c>
-      <c r="AI11" t="str">
-        <v/>
       </c>
       <c r="AJ11">
         <v>0.78</v>
@@ -19356,116 +19356,116 @@
       <c r="AM11">
         <v>0.78</v>
       </c>
-      <c r="AN11">
-        <v>0.78</v>
+      <c r="AN11" t="str">
+        <v/>
       </c>
       <c r="AO11">
         <v>0.78</v>
       </c>
-      <c r="AP11" t="str">
-        <v/>
+      <c r="AP11">
+        <v>0.78</v>
       </c>
       <c r="AQ11">
         <v>0.78</v>
       </c>
-      <c r="AR11">
+      <c r="AR11" t="str">
+        <v/>
+      </c>
+      <c r="AS11" t="str">
+        <v/>
+      </c>
+      <c r="AT11">
         <v>0.78</v>
       </c>
-      <c r="AS11">
+      <c r="AU11">
         <v>0.78</v>
-      </c>
-      <c r="AT11" t="str">
-        <v/>
-      </c>
-      <c r="AU11" t="str">
-        <v/>
       </c>
       <c r="AV11">
         <v>0.78</v>
       </c>
-      <c r="AW11">
+      <c r="AW11" t="str">
+        <v/>
+      </c>
+      <c r="AX11" t="str">
+        <v/>
+      </c>
+      <c r="AY11" t="str">
+        <v/>
+      </c>
+      <c r="AZ11" t="str">
+        <v/>
+      </c>
+      <c r="BA11" t="str">
+        <v/>
+      </c>
+      <c r="BB11" t="str">
+        <v/>
+      </c>
+      <c r="BC11" t="str">
+        <v/>
+      </c>
+      <c r="BD11" t="str">
+        <v/>
+      </c>
+      <c r="BE11" t="str">
+        <v/>
+      </c>
+      <c r="BF11" t="str">
+        <v/>
+      </c>
+      <c r="BG11" t="str">
+        <v/>
+      </c>
+      <c r="BH11" t="str">
+        <v/>
+      </c>
+      <c r="BI11">
         <v>0.78</v>
       </c>
-      <c r="AX11">
+      <c r="BJ11">
         <v>0.78</v>
       </c>
-      <c r="AY11" t="str">
-        <v/>
-      </c>
-      <c r="AZ11" t="str">
-        <v/>
-      </c>
-      <c r="BA11" t="str">
-        <v/>
-      </c>
-      <c r="BB11" t="str">
-        <v/>
-      </c>
-      <c r="BC11" t="str">
-        <v/>
-      </c>
-      <c r="BD11" t="str">
-        <v/>
-      </c>
-      <c r="BE11" t="str">
-        <v/>
-      </c>
-      <c r="BF11" t="str">
-        <v/>
-      </c>
-      <c r="BG11" t="str">
-        <v/>
-      </c>
-      <c r="BH11" t="str">
-        <v/>
-      </c>
-      <c r="BI11" t="str">
-        <v/>
-      </c>
-      <c r="BJ11" t="str">
-        <v/>
-      </c>
-      <c r="BK11">
+      <c r="BK11" t="str">
+        <v/>
+      </c>
+      <c r="BL11" t="str">
+        <v/>
+      </c>
+      <c r="BM11" t="str">
+        <v/>
+      </c>
+      <c r="BN11" t="str">
+        <v/>
+      </c>
+      <c r="BO11">
         <v>0.78</v>
       </c>
-      <c r="BL11">
+      <c r="BP11" t="str">
+        <v/>
+      </c>
+      <c r="BQ11" t="str">
+        <v/>
+      </c>
+      <c r="BR11">
         <v>0.78</v>
       </c>
-      <c r="BM11" t="str">
-        <v/>
-      </c>
-      <c r="BN11" t="str">
-        <v/>
-      </c>
-      <c r="BO11" t="str">
-        <v/>
-      </c>
-      <c r="BP11" t="str">
-        <v/>
-      </c>
-      <c r="BQ11">
+      <c r="BS11" t="str">
+        <v/>
+      </c>
+      <c r="BT11" t="str">
+        <v/>
+      </c>
+      <c r="BU11" t="str">
+        <v/>
+      </c>
+      <c r="BV11" t="str">
+        <v/>
+      </c>
+      <c r="BW11">
         <v>0.78</v>
       </c>
-      <c r="BR11" t="str">
-        <v/>
-      </c>
-      <c r="BS11" t="str">
-        <v/>
-      </c>
-      <c r="BT11">
+      <c r="BX11">
         <v>0.78</v>
-      </c>
-      <c r="BU11" t="str">
-        <v/>
-      </c>
-      <c r="BV11" t="str">
-        <v/>
-      </c>
-      <c r="BW11" t="str">
-        <v/>
-      </c>
-      <c r="BX11" t="str">
-        <v/>
       </c>
       <c r="BY11">
         <v>0.78</v>
@@ -19637,17 +19637,17 @@
       <c r="AX12">
         <v>0</v>
       </c>
-      <c r="AY12">
-        <v>0</v>
-      </c>
-      <c r="AZ12">
-        <v>0</v>
-      </c>
-      <c r="BA12" t="str">
-        <v/>
-      </c>
-      <c r="BB12" t="str">
-        <v/>
+      <c r="AY12" t="str">
+        <v/>
+      </c>
+      <c r="AZ12" t="str">
+        <v/>
+      </c>
+      <c r="BA12">
+        <v>0</v>
+      </c>
+      <c r="BB12">
+        <v>0</v>
       </c>
       <c r="BC12">
         <v>0</v>
@@ -19688,17 +19688,17 @@
       <c r="BO12">
         <v>0</v>
       </c>
-      <c r="BP12">
-        <v>0</v>
-      </c>
-      <c r="BQ12">
-        <v>0</v>
-      </c>
-      <c r="BR12" t="str">
-        <v/>
-      </c>
-      <c r="BS12" t="str">
-        <v/>
+      <c r="BP12" t="str">
+        <v/>
+      </c>
+      <c r="BQ12" t="str">
+        <v/>
+      </c>
+      <c r="BR12">
+        <v>0</v>
+      </c>
+      <c r="BS12">
+        <v>0</v>
       </c>
       <c r="BT12">
         <v>0</v>
@@ -19852,14 +19852,14 @@
       <c r="AM13">
         <v>0.17</v>
       </c>
-      <c r="AN13">
-        <v>0.17</v>
+      <c r="AN13" t="str">
+        <v/>
       </c>
       <c r="AO13">
         <v>0.17</v>
       </c>
-      <c r="AP13" t="str">
-        <v/>
+      <c r="AP13">
+        <v>0.17</v>
       </c>
       <c r="AQ13">
         <v>0.17</v>
@@ -19885,17 +19885,17 @@
       <c r="AX13">
         <v>0.17</v>
       </c>
-      <c r="AY13">
+      <c r="AY13" t="str">
+        <v/>
+      </c>
+      <c r="AZ13" t="str">
+        <v/>
+      </c>
+      <c r="BA13">
         <v>0.17</v>
       </c>
-      <c r="AZ13">
+      <c r="BB13">
         <v>0.17</v>
-      </c>
-      <c r="BA13" t="str">
-        <v/>
-      </c>
-      <c r="BB13" t="str">
-        <v/>
       </c>
       <c r="BC13">
         <v>0.17</v>
@@ -19936,17 +19936,17 @@
       <c r="BO13">
         <v>0.17</v>
       </c>
-      <c r="BP13">
+      <c r="BP13" t="str">
+        <v/>
+      </c>
+      <c r="BQ13" t="str">
+        <v/>
+      </c>
+      <c r="BR13">
         <v>0.17</v>
       </c>
-      <c r="BQ13">
+      <c r="BS13">
         <v>0.17</v>
-      </c>
-      <c r="BR13" t="str">
-        <v/>
-      </c>
-      <c r="BS13" t="str">
-        <v/>
       </c>
       <c r="BT13">
         <v>0.17</v>
@@ -20360,13 +20360,13 @@
         <v>Anderson, Margaret 33333-1.375 (60m)</v>
       </c>
       <c r="AN1" t="str">
+        <v>Office Hours Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="AO1" t="str">
+        <v>Office Hours Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="AP1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="AO1" t="str">
-        <v>Office Hours Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="AP1" t="str">
-        <v>Office Hours Client 14:00-17:00 (60m)</v>
       </c>
       <c r="AQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20387,10 +20387,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AW1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+      </c>
+      <c r="AX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="AX1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="AY1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20399,13 +20399,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BA1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BB1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BC1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BD1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20414,58 +20414,58 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BF1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
       <c r="BG1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BH1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (420m)</v>
+      </c>
+      <c r="BI1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (420m)</v>
+      </c>
+      <c r="BJ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BK1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BI1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (420m)</v>
-      </c>
-      <c r="BJ1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (420m)</v>
-      </c>
-      <c r="BK1" t="str">
+      <c r="BL1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BL1" t="str">
+      <c r="BM1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BM1" t="str">
+      <c r="BN1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BN1" t="str">
+      <c r="BO1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BO1" t="str">
+      <c r="BP1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BP1" t="str">
+      <c r="BQ1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BQ1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
       <c r="BR1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (180m)</v>
       </c>
       <c r="BS1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (180m)</v>
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
       <c r="BT1" t="str">
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BU1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BU1" t="str">
+      <c r="BV1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BV1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
-      </c>
       <c r="BW1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
@@ -20474,58 +20474,58 @@
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BZ1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CA1" t="str">
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="CB1" t="str">
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="CC1" t="str">
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="CD1" t="str">
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="CE1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CB1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="CC1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="CD1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="CE1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
       <c r="CF1" t="str">
+        <v>Office Hours Client 09:00-12:00 (330m)</v>
+      </c>
+      <c r="CG1" t="str">
+        <v>Office Hours Client 14:00-17:00 (330m)</v>
+      </c>
+      <c r="CH1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CG1" t="str">
-        <v>Office Hours Client 09:00-12:00 (330m)</v>
-      </c>
-      <c r="CH1" t="str">
-        <v>Office Hours Client 14:00-17:00 (330m)</v>
-      </c>
       <c r="CI1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+      </c>
+      <c r="CJ1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (150m)</v>
+      </c>
+      <c r="CK1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="CJ1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
-      </c>
-      <c r="CK1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (150m)</v>
       </c>
       <c r="CL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CM1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="CN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="CO1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="CP1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
-      <c r="CP1" t="str">
+      <c r="CQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="CQ1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="CR1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -20718,14 +20718,14 @@
       <c r="BG2">
         <v>0.09</v>
       </c>
-      <c r="BH2">
+      <c r="BH2" t="str">
+        <v/>
+      </c>
+      <c r="BI2" t="str">
+        <v/>
+      </c>
+      <c r="BJ2">
         <v>0.09</v>
-      </c>
-      <c r="BI2" t="str">
-        <v/>
-      </c>
-      <c r="BJ2" t="str">
-        <v/>
       </c>
       <c r="BK2">
         <v>0.09</v>
@@ -20790,14 +20790,14 @@
       <c r="CE2">
         <v>0.09</v>
       </c>
-      <c r="CF2">
+      <c r="CF2" t="str">
+        <v/>
+      </c>
+      <c r="CG2" t="str">
+        <v/>
+      </c>
+      <c r="CH2">
         <v>0.09</v>
-      </c>
-      <c r="CG2" t="str">
-        <v/>
-      </c>
-      <c r="CH2" t="str">
-        <v/>
       </c>
       <c r="CI2">
         <v>0.09</v>
@@ -21017,14 +21017,14 @@
       <c r="BG3">
         <v>0</v>
       </c>
-      <c r="BH3">
-        <v>0</v>
+      <c r="BH3" t="str">
+        <v/>
       </c>
       <c r="BI3" t="str">
         <v/>
       </c>
-      <c r="BJ3" t="str">
-        <v/>
+      <c r="BJ3">
+        <v>0</v>
       </c>
       <c r="BK3">
         <v>0</v>
@@ -21089,14 +21089,14 @@
       <c r="CE3">
         <v>0</v>
       </c>
-      <c r="CF3">
-        <v>0</v>
+      <c r="CF3" t="str">
+        <v/>
       </c>
       <c r="CG3" t="str">
         <v/>
       </c>
-      <c r="CH3" t="str">
-        <v/>
+      <c r="CH3">
+        <v>0</v>
       </c>
       <c r="CI3">
         <v>0</v>
@@ -21259,11 +21259,11 @@
       <c r="AN4">
         <v>0.78</v>
       </c>
-      <c r="AO4">
+      <c r="AO4" t="str">
+        <v/>
+      </c>
+      <c r="AP4">
         <v>0.78</v>
-      </c>
-      <c r="AP4" t="str">
-        <v/>
       </c>
       <c r="AQ4">
         <v>0.78</v>
@@ -21283,11 +21283,11 @@
       <c r="AV4">
         <v>0.78</v>
       </c>
-      <c r="AW4">
+      <c r="AW4" t="str">
+        <v/>
+      </c>
+      <c r="AX4">
         <v>0.78</v>
-      </c>
-      <c r="AX4" t="str">
-        <v/>
       </c>
       <c r="AY4">
         <v>0.78</v>
@@ -21295,14 +21295,14 @@
       <c r="AZ4">
         <v>0.78</v>
       </c>
-      <c r="BA4">
+      <c r="BA4" t="str">
+        <v/>
+      </c>
+      <c r="BB4" t="str">
+        <v/>
+      </c>
+      <c r="BC4">
         <v>0.78</v>
-      </c>
-      <c r="BB4" t="str">
-        <v/>
-      </c>
-      <c r="BC4" t="str">
-        <v/>
       </c>
       <c r="BD4">
         <v>0.78</v>
@@ -21313,116 +21313,116 @@
       <c r="BF4">
         <v>0.78</v>
       </c>
-      <c r="BG4">
+      <c r="BG4" t="str">
+        <v/>
+      </c>
+      <c r="BH4" t="str">
+        <v/>
+      </c>
+      <c r="BI4" t="str">
+        <v/>
+      </c>
+      <c r="BJ4">
         <v>0.78</v>
       </c>
-      <c r="BH4" t="str">
-        <v/>
-      </c>
-      <c r="BI4" t="str">
-        <v/>
-      </c>
-      <c r="BJ4" t="str">
-        <v/>
-      </c>
-      <c r="BK4">
+      <c r="BK4" t="str">
+        <v/>
+      </c>
+      <c r="BL4">
         <v>0.78</v>
       </c>
-      <c r="BL4" t="str">
-        <v/>
-      </c>
-      <c r="BM4">
+      <c r="BM4" t="str">
+        <v/>
+      </c>
+      <c r="BN4">
         <v>0.78</v>
       </c>
-      <c r="BN4" t="str">
-        <v/>
-      </c>
-      <c r="BO4">
+      <c r="BO4" t="str">
+        <v/>
+      </c>
+      <c r="BP4">
         <v>0.78</v>
       </c>
-      <c r="BP4" t="str">
-        <v/>
-      </c>
-      <c r="BQ4">
+      <c r="BQ4" t="str">
+        <v/>
+      </c>
+      <c r="BR4" t="str">
+        <v/>
+      </c>
+      <c r="BS4">
         <v>0.78</v>
       </c>
-      <c r="BR4" t="str">
-        <v/>
-      </c>
-      <c r="BS4" t="str">
-        <v/>
-      </c>
-      <c r="BT4">
+      <c r="BT4" t="str">
+        <v/>
+      </c>
+      <c r="BU4">
         <v>0.78</v>
       </c>
-      <c r="BU4" t="str">
-        <v/>
-      </c>
-      <c r="BV4">
+      <c r="BV4" t="str">
+        <v/>
+      </c>
+      <c r="BW4" t="str">
+        <v/>
+      </c>
+      <c r="BX4" t="str">
+        <v/>
+      </c>
+      <c r="BY4" t="str">
+        <v/>
+      </c>
+      <c r="BZ4">
         <v>0.78</v>
-      </c>
-      <c r="BW4" t="str">
-        <v/>
-      </c>
-      <c r="BX4" t="str">
-        <v/>
-      </c>
-      <c r="BY4" t="str">
-        <v/>
-      </c>
-      <c r="BZ4" t="str">
-        <v/>
       </c>
       <c r="CA4">
         <v>0.78</v>
       </c>
-      <c r="CB4">
+      <c r="CB4" t="str">
+        <v/>
+      </c>
+      <c r="CC4">
         <v>0.78</v>
       </c>
-      <c r="CC4" t="str">
-        <v/>
-      </c>
-      <c r="CD4">
+      <c r="CD4" t="str">
+        <v/>
+      </c>
+      <c r="CE4">
         <v>0.78</v>
       </c>
-      <c r="CE4" t="str">
-        <v/>
-      </c>
-      <c r="CF4">
+      <c r="CF4" t="str">
+        <v/>
+      </c>
+      <c r="CG4" t="str">
+        <v/>
+      </c>
+      <c r="CH4">
         <v>0.78</v>
       </c>
-      <c r="CG4" t="str">
-        <v/>
-      </c>
-      <c r="CH4" t="str">
-        <v/>
-      </c>
-      <c r="CI4">
+      <c r="CI4" t="str">
+        <v/>
+      </c>
+      <c r="CJ4" t="str">
+        <v/>
+      </c>
+      <c r="CK4">
         <v>0.78</v>
-      </c>
-      <c r="CJ4" t="str">
-        <v/>
-      </c>
-      <c r="CK4" t="str">
-        <v/>
       </c>
       <c r="CL4">
         <v>0.78</v>
       </c>
-      <c r="CM4">
+      <c r="CM4" t="str">
+        <v/>
+      </c>
+      <c r="CN4" t="str">
+        <v/>
+      </c>
+      <c r="CO4">
         <v>0.78</v>
       </c>
-      <c r="CN4" t="str">
-        <v/>
-      </c>
-      <c r="CO4" t="str">
-        <v/>
-      </c>
-      <c r="CP4">
+      <c r="CP4" t="str">
+        <v/>
+      </c>
+      <c r="CQ4">
         <v>0.78</v>
-      </c>
-      <c r="CQ4" t="str">
-        <v/>
       </c>
       <c r="CR4">
         <v>0.78</v>
@@ -21558,11 +21558,11 @@
       <c r="AN5">
         <v>0</v>
       </c>
-      <c r="AO5">
-        <v>0</v>
-      </c>
-      <c r="AP5" t="str">
-        <v/>
+      <c r="AO5" t="str">
+        <v/>
+      </c>
+      <c r="AP5">
+        <v>0</v>
       </c>
       <c r="AQ5">
         <v>0</v>
@@ -21582,11 +21582,11 @@
       <c r="AV5">
         <v>0</v>
       </c>
-      <c r="AW5">
-        <v>0</v>
-      </c>
-      <c r="AX5" t="str">
-        <v/>
+      <c r="AW5" t="str">
+        <v/>
+      </c>
+      <c r="AX5">
+        <v>0</v>
       </c>
       <c r="AY5">
         <v>0</v>
@@ -21612,8 +21612,8 @@
       <c r="BF5">
         <v>0</v>
       </c>
-      <c r="BG5">
-        <v>0</v>
+      <c r="BG5" t="str">
+        <v/>
       </c>
       <c r="BH5" t="str">
         <v/>
@@ -21621,47 +21621,47 @@
       <c r="BI5" t="str">
         <v/>
       </c>
-      <c r="BJ5" t="str">
-        <v/>
-      </c>
-      <c r="BK5">
-        <v>0</v>
-      </c>
-      <c r="BL5" t="str">
-        <v/>
-      </c>
-      <c r="BM5">
-        <v>0</v>
-      </c>
-      <c r="BN5" t="str">
-        <v/>
-      </c>
-      <c r="BO5">
-        <v>0</v>
-      </c>
-      <c r="BP5" t="str">
-        <v/>
-      </c>
-      <c r="BQ5">
-        <v>0</v>
-      </c>
-      <c r="BR5" t="str">
-        <v/>
+      <c r="BJ5">
+        <v>0</v>
+      </c>
+      <c r="BK5" t="str">
+        <v/>
+      </c>
+      <c r="BL5">
+        <v>0</v>
+      </c>
+      <c r="BM5" t="str">
+        <v/>
+      </c>
+      <c r="BN5">
+        <v>0</v>
+      </c>
+      <c r="BO5" t="str">
+        <v/>
+      </c>
+      <c r="BP5">
+        <v>0</v>
+      </c>
+      <c r="BQ5" t="str">
+        <v/>
+      </c>
+      <c r="BR5">
+        <v>0</v>
       </c>
       <c r="BS5">
         <v>0</v>
       </c>
-      <c r="BT5">
-        <v>0</v>
-      </c>
-      <c r="BU5" t="str">
-        <v/>
-      </c>
-      <c r="BV5">
-        <v>0</v>
-      </c>
-      <c r="BW5" t="str">
-        <v/>
+      <c r="BT5" t="str">
+        <v/>
+      </c>
+      <c r="BU5">
+        <v>0</v>
+      </c>
+      <c r="BV5" t="str">
+        <v/>
+      </c>
+      <c r="BW5">
+        <v>0</v>
       </c>
       <c r="BX5">
         <v>0</v>
@@ -21675,32 +21675,32 @@
       <c r="CA5">
         <v>0</v>
       </c>
-      <c r="CB5">
-        <v>0</v>
-      </c>
-      <c r="CC5" t="str">
-        <v/>
-      </c>
-      <c r="CD5">
-        <v>0</v>
-      </c>
-      <c r="CE5" t="str">
-        <v/>
-      </c>
-      <c r="CF5">
-        <v>0</v>
+      <c r="CB5" t="str">
+        <v/>
+      </c>
+      <c r="CC5">
+        <v>0</v>
+      </c>
+      <c r="CD5" t="str">
+        <v/>
+      </c>
+      <c r="CE5">
+        <v>0</v>
+      </c>
+      <c r="CF5" t="str">
+        <v/>
       </c>
       <c r="CG5" t="str">
         <v/>
       </c>
-      <c r="CH5" t="str">
-        <v/>
-      </c>
-      <c r="CI5">
-        <v>0</v>
-      </c>
-      <c r="CJ5" t="str">
-        <v/>
+      <c r="CH5">
+        <v>0</v>
+      </c>
+      <c r="CI5" t="str">
+        <v/>
+      </c>
+      <c r="CJ5">
+        <v>0</v>
       </c>
       <c r="CK5">
         <v>0</v>
@@ -22156,11 +22156,11 @@
       <c r="AN7">
         <v>0</v>
       </c>
-      <c r="AO7">
-        <v>0</v>
-      </c>
-      <c r="AP7" t="str">
-        <v/>
+      <c r="AO7" t="str">
+        <v/>
+      </c>
+      <c r="AP7">
+        <v>0</v>
       </c>
       <c r="AQ7">
         <v>0</v>
@@ -22210,8 +22210,8 @@
       <c r="BF7">
         <v>0</v>
       </c>
-      <c r="BG7">
-        <v>0</v>
+      <c r="BG7" t="str">
+        <v/>
       </c>
       <c r="BH7" t="str">
         <v/>
@@ -22219,47 +22219,47 @@
       <c r="BI7" t="str">
         <v/>
       </c>
-      <c r="BJ7" t="str">
-        <v/>
-      </c>
-      <c r="BK7">
-        <v>0</v>
-      </c>
-      <c r="BL7" t="str">
-        <v/>
-      </c>
-      <c r="BM7">
-        <v>0</v>
-      </c>
-      <c r="BN7" t="str">
-        <v/>
-      </c>
-      <c r="BO7">
-        <v>0</v>
-      </c>
-      <c r="BP7" t="str">
-        <v/>
-      </c>
-      <c r="BQ7">
-        <v>0</v>
-      </c>
-      <c r="BR7" t="str">
-        <v/>
+      <c r="BJ7">
+        <v>0</v>
+      </c>
+      <c r="BK7" t="str">
+        <v/>
+      </c>
+      <c r="BL7">
+        <v>0</v>
+      </c>
+      <c r="BM7" t="str">
+        <v/>
+      </c>
+      <c r="BN7">
+        <v>0</v>
+      </c>
+      <c r="BO7" t="str">
+        <v/>
+      </c>
+      <c r="BP7">
+        <v>0</v>
+      </c>
+      <c r="BQ7" t="str">
+        <v/>
+      </c>
+      <c r="BR7">
+        <v>0</v>
       </c>
       <c r="BS7">
         <v>0</v>
       </c>
-      <c r="BT7">
-        <v>0</v>
-      </c>
-      <c r="BU7" t="str">
-        <v/>
-      </c>
-      <c r="BV7">
-        <v>0</v>
-      </c>
-      <c r="BW7" t="str">
-        <v/>
+      <c r="BT7" t="str">
+        <v/>
+      </c>
+      <c r="BU7">
+        <v>0</v>
+      </c>
+      <c r="BV7" t="str">
+        <v/>
+      </c>
+      <c r="BW7">
+        <v>0</v>
       </c>
       <c r="BX7">
         <v>0</v>
@@ -22273,26 +22273,26 @@
       <c r="CA7">
         <v>0</v>
       </c>
-      <c r="CB7">
-        <v>0</v>
-      </c>
-      <c r="CC7" t="str">
-        <v/>
-      </c>
-      <c r="CD7">
-        <v>0</v>
-      </c>
-      <c r="CE7" t="str">
-        <v/>
-      </c>
-      <c r="CF7">
-        <v>0</v>
+      <c r="CB7" t="str">
+        <v/>
+      </c>
+      <c r="CC7">
+        <v>0</v>
+      </c>
+      <c r="CD7" t="str">
+        <v/>
+      </c>
+      <c r="CE7">
+        <v>0</v>
+      </c>
+      <c r="CF7" t="str">
+        <v/>
       </c>
       <c r="CG7" t="str">
         <v/>
       </c>
-      <c r="CH7" t="str">
-        <v/>
+      <c r="CH7">
+        <v>0</v>
       </c>
       <c r="CI7">
         <v>0</v>
@@ -22512,14 +22512,14 @@
       <c r="BG8">
         <v>0</v>
       </c>
-      <c r="BH8">
-        <v>0</v>
+      <c r="BH8" t="str">
+        <v/>
       </c>
       <c r="BI8" t="str">
         <v/>
       </c>
-      <c r="BJ8" t="str">
-        <v/>
+      <c r="BJ8">
+        <v>0</v>
       </c>
       <c r="BK8">
         <v>0</v>
@@ -22584,14 +22584,14 @@
       <c r="CE8">
         <v>0</v>
       </c>
-      <c r="CF8">
-        <v>0</v>
+      <c r="CF8" t="str">
+        <v/>
       </c>
       <c r="CG8" t="str">
         <v/>
       </c>
-      <c r="CH8" t="str">
-        <v/>
+      <c r="CH8">
+        <v>0</v>
       </c>
       <c r="CI8">
         <v>0</v>
@@ -22754,11 +22754,11 @@
       <c r="AN9">
         <v>0</v>
       </c>
-      <c r="AO9">
-        <v>0</v>
-      </c>
-      <c r="AP9" t="str">
-        <v/>
+      <c r="AO9" t="str">
+        <v/>
+      </c>
+      <c r="AP9">
+        <v>0</v>
       </c>
       <c r="AQ9">
         <v>0</v>
@@ -22808,8 +22808,8 @@
       <c r="BF9">
         <v>0</v>
       </c>
-      <c r="BG9">
-        <v>0</v>
+      <c r="BG9" t="str">
+        <v/>
       </c>
       <c r="BH9" t="str">
         <v/>
@@ -22817,47 +22817,47 @@
       <c r="BI9" t="str">
         <v/>
       </c>
-      <c r="BJ9" t="str">
-        <v/>
-      </c>
-      <c r="BK9">
-        <v>0</v>
-      </c>
-      <c r="BL9" t="str">
-        <v/>
-      </c>
-      <c r="BM9">
-        <v>0</v>
-      </c>
-      <c r="BN9" t="str">
-        <v/>
-      </c>
-      <c r="BO9">
-        <v>0</v>
-      </c>
-      <c r="BP9" t="str">
-        <v/>
-      </c>
-      <c r="BQ9">
-        <v>0</v>
-      </c>
-      <c r="BR9" t="str">
-        <v/>
+      <c r="BJ9">
+        <v>0</v>
+      </c>
+      <c r="BK9" t="str">
+        <v/>
+      </c>
+      <c r="BL9">
+        <v>0</v>
+      </c>
+      <c r="BM9" t="str">
+        <v/>
+      </c>
+      <c r="BN9">
+        <v>0</v>
+      </c>
+      <c r="BO9" t="str">
+        <v/>
+      </c>
+      <c r="BP9">
+        <v>0</v>
+      </c>
+      <c r="BQ9" t="str">
+        <v/>
+      </c>
+      <c r="BR9">
+        <v>0</v>
       </c>
       <c r="BS9">
         <v>0</v>
       </c>
-      <c r="BT9">
-        <v>0</v>
-      </c>
-      <c r="BU9" t="str">
-        <v/>
-      </c>
-      <c r="BV9">
-        <v>0</v>
-      </c>
-      <c r="BW9" t="str">
-        <v/>
+      <c r="BT9" t="str">
+        <v/>
+      </c>
+      <c r="BU9">
+        <v>0</v>
+      </c>
+      <c r="BV9" t="str">
+        <v/>
+      </c>
+      <c r="BW9">
+        <v>0</v>
       </c>
       <c r="BX9">
         <v>0</v>
@@ -22871,26 +22871,26 @@
       <c r="CA9">
         <v>0</v>
       </c>
-      <c r="CB9">
-        <v>0</v>
-      </c>
-      <c r="CC9" t="str">
-        <v/>
-      </c>
-      <c r="CD9">
-        <v>0</v>
-      </c>
-      <c r="CE9" t="str">
-        <v/>
-      </c>
-      <c r="CF9">
-        <v>0</v>
+      <c r="CB9" t="str">
+        <v/>
+      </c>
+      <c r="CC9">
+        <v>0</v>
+      </c>
+      <c r="CD9" t="str">
+        <v/>
+      </c>
+      <c r="CE9">
+        <v>0</v>
+      </c>
+      <c r="CF9" t="str">
+        <v/>
       </c>
       <c r="CG9" t="str">
         <v/>
       </c>
-      <c r="CH9" t="str">
-        <v/>
+      <c r="CH9">
+        <v>0</v>
       </c>
       <c r="CI9">
         <v>0</v>
@@ -23110,14 +23110,14 @@
       <c r="BG10">
         <v>0</v>
       </c>
-      <c r="BH10">
-        <v>0</v>
+      <c r="BH10" t="str">
+        <v/>
       </c>
       <c r="BI10" t="str">
         <v/>
       </c>
-      <c r="BJ10" t="str">
-        <v/>
+      <c r="BJ10">
+        <v>0</v>
       </c>
       <c r="BK10">
         <v>0</v>
@@ -23182,14 +23182,14 @@
       <c r="CE10">
         <v>0</v>
       </c>
-      <c r="CF10">
-        <v>0</v>
+      <c r="CF10" t="str">
+        <v/>
       </c>
       <c r="CG10" t="str">
         <v/>
       </c>
-      <c r="CH10" t="str">
-        <v/>
+      <c r="CH10">
+        <v>0</v>
       </c>
       <c r="CI10">
         <v>0</v>
@@ -23409,14 +23409,14 @@
       <c r="BG11">
         <v>0</v>
       </c>
-      <c r="BH11">
-        <v>0</v>
+      <c r="BH11" t="str">
+        <v/>
       </c>
       <c r="BI11" t="str">
         <v/>
       </c>
-      <c r="BJ11" t="str">
-        <v/>
+      <c r="BJ11">
+        <v>0</v>
       </c>
       <c r="BK11">
         <v>0</v>
@@ -23481,14 +23481,14 @@
       <c r="CE11">
         <v>0</v>
       </c>
-      <c r="CF11">
-        <v>0</v>
+      <c r="CF11" t="str">
+        <v/>
       </c>
       <c r="CG11" t="str">
         <v/>
       </c>
-      <c r="CH11" t="str">
-        <v/>
+      <c r="CH11">
+        <v>0</v>
       </c>
       <c r="CI11">
         <v>0</v>
@@ -23708,14 +23708,14 @@
       <c r="BG12">
         <v>0</v>
       </c>
-      <c r="BH12">
-        <v>0</v>
+      <c r="BH12" t="str">
+        <v/>
       </c>
       <c r="BI12" t="str">
         <v/>
       </c>
-      <c r="BJ12" t="str">
-        <v/>
+      <c r="BJ12">
+        <v>0</v>
       </c>
       <c r="BK12">
         <v>0</v>
@@ -23780,14 +23780,14 @@
       <c r="CE12">
         <v>0</v>
       </c>
-      <c r="CF12">
-        <v>0</v>
+      <c r="CF12" t="str">
+        <v/>
       </c>
       <c r="CG12" t="str">
         <v/>
       </c>
-      <c r="CH12" t="str">
-        <v/>
+      <c r="CH12">
+        <v>0</v>
       </c>
       <c r="CI12">
         <v>0</v>
@@ -23974,11 +23974,11 @@
       <c r="AV13">
         <v>0</v>
       </c>
-      <c r="AW13">
-        <v>0</v>
-      </c>
-      <c r="AX13" t="str">
-        <v/>
+      <c r="AW13" t="str">
+        <v/>
+      </c>
+      <c r="AX13">
+        <v>0</v>
       </c>
       <c r="AY13">
         <v>0</v>
@@ -24007,14 +24007,14 @@
       <c r="BG13">
         <v>0</v>
       </c>
-      <c r="BH13">
-        <v>0</v>
+      <c r="BH13" t="str">
+        <v/>
       </c>
       <c r="BI13" t="str">
         <v/>
       </c>
-      <c r="BJ13" t="str">
-        <v/>
+      <c r="BJ13">
+        <v>0</v>
       </c>
       <c r="BK13">
         <v>0</v>
@@ -24079,20 +24079,20 @@
       <c r="CE13">
         <v>0</v>
       </c>
-      <c r="CF13">
-        <v>0</v>
+      <c r="CF13" t="str">
+        <v/>
       </c>
       <c r="CG13" t="str">
         <v/>
       </c>
-      <c r="CH13" t="str">
-        <v/>
-      </c>
-      <c r="CI13">
-        <v>0</v>
-      </c>
-      <c r="CJ13" t="str">
-        <v/>
+      <c r="CH13">
+        <v>0</v>
+      </c>
+      <c r="CI13" t="str">
+        <v/>
+      </c>
+      <c r="CJ13">
+        <v>0</v>
       </c>
       <c r="CK13">
         <v>0</v>
@@ -24246,11 +24246,11 @@
       <c r="AM14">
         <v>0.81</v>
       </c>
-      <c r="AN14">
+      <c r="AN14" t="str">
+        <v/>
+      </c>
+      <c r="AO14">
         <v>0.16</v>
-      </c>
-      <c r="AO14" t="str">
-        <v/>
       </c>
       <c r="AP14">
         <v>0.16</v>
@@ -24273,11 +24273,11 @@
       <c r="AV14">
         <v>0.16</v>
       </c>
-      <c r="AW14">
+      <c r="AW14" t="str">
+        <v/>
+      </c>
+      <c r="AX14">
         <v>0.16</v>
-      </c>
-      <c r="AX14" t="str">
-        <v/>
       </c>
       <c r="AY14">
         <v>0.16</v>
@@ -24285,14 +24285,14 @@
       <c r="AZ14">
         <v>0.16</v>
       </c>
-      <c r="BA14">
+      <c r="BA14" t="str">
+        <v/>
+      </c>
+      <c r="BB14" t="str">
+        <v/>
+      </c>
+      <c r="BC14">
         <v>0.16</v>
-      </c>
-      <c r="BB14" t="str">
-        <v/>
-      </c>
-      <c r="BC14" t="str">
-        <v/>
       </c>
       <c r="BD14">
         <v>0.16</v>
@@ -24300,119 +24300,119 @@
       <c r="BE14">
         <v>0.16</v>
       </c>
-      <c r="BF14">
+      <c r="BF14" t="str">
+        <v/>
+      </c>
+      <c r="BG14">
         <v>0.16</v>
       </c>
-      <c r="BG14" t="str">
-        <v/>
-      </c>
-      <c r="BH14">
+      <c r="BH14" t="str">
+        <v/>
+      </c>
+      <c r="BI14" t="str">
+        <v/>
+      </c>
+      <c r="BJ14" t="str">
+        <v/>
+      </c>
+      <c r="BK14">
         <v>0.16</v>
       </c>
-      <c r="BI14" t="str">
-        <v/>
-      </c>
-      <c r="BJ14" t="str">
-        <v/>
-      </c>
-      <c r="BK14" t="str">
-        <v/>
-      </c>
-      <c r="BL14">
+      <c r="BL14" t="str">
+        <v/>
+      </c>
+      <c r="BM14">
         <v>0.16</v>
       </c>
-      <c r="BM14" t="str">
-        <v/>
-      </c>
-      <c r="BN14">
+      <c r="BN14" t="str">
+        <v/>
+      </c>
+      <c r="BO14">
         <v>0.16</v>
       </c>
-      <c r="BO14" t="str">
-        <v/>
-      </c>
-      <c r="BP14">
+      <c r="BP14" t="str">
+        <v/>
+      </c>
+      <c r="BQ14">
         <v>0.16</v>
       </c>
-      <c r="BQ14" t="str">
-        <v/>
-      </c>
-      <c r="BR14">
+      <c r="BR14" t="str">
+        <v/>
+      </c>
+      <c r="BS14" t="str">
+        <v/>
+      </c>
+      <c r="BT14">
         <v>0.16</v>
       </c>
-      <c r="BS14" t="str">
-        <v/>
-      </c>
-      <c r="BT14" t="str">
-        <v/>
-      </c>
-      <c r="BU14">
+      <c r="BU14" t="str">
+        <v/>
+      </c>
+      <c r="BV14">
         <v>0.16</v>
       </c>
-      <c r="BV14" t="str">
-        <v/>
-      </c>
-      <c r="BW14">
+      <c r="BW14" t="str">
+        <v/>
+      </c>
+      <c r="BX14" t="str">
+        <v/>
+      </c>
+      <c r="BY14" t="str">
+        <v/>
+      </c>
+      <c r="BZ14">
         <v>0.16</v>
       </c>
-      <c r="BX14" t="str">
-        <v/>
-      </c>
-      <c r="BY14" t="str">
-        <v/>
-      </c>
-      <c r="BZ14" t="str">
-        <v/>
-      </c>
-      <c r="CA14">
+      <c r="CA14" t="str">
+        <v/>
+      </c>
+      <c r="CB14">
         <v>0.16</v>
       </c>
-      <c r="CB14" t="str">
-        <v/>
-      </c>
-      <c r="CC14">
+      <c r="CC14" t="str">
+        <v/>
+      </c>
+      <c r="CD14">
         <v>0.16</v>
-      </c>
-      <c r="CD14" t="str">
-        <v/>
       </c>
       <c r="CE14">
         <v>0.16</v>
       </c>
-      <c r="CF14">
+      <c r="CF14" t="str">
+        <v/>
+      </c>
+      <c r="CG14" t="str">
+        <v/>
+      </c>
+      <c r="CH14">
         <v>0.16</v>
       </c>
-      <c r="CG14" t="str">
-        <v/>
-      </c>
-      <c r="CH14" t="str">
-        <v/>
-      </c>
-      <c r="CI14">
+      <c r="CI14" t="str">
+        <v/>
+      </c>
+      <c r="CJ14" t="str">
+        <v/>
+      </c>
+      <c r="CK14">
         <v>0.16</v>
-      </c>
-      <c r="CJ14" t="str">
-        <v/>
-      </c>
-      <c r="CK14" t="str">
-        <v/>
       </c>
       <c r="CL14">
         <v>0.16</v>
       </c>
-      <c r="CM14">
+      <c r="CM14" t="str">
+        <v/>
+      </c>
+      <c r="CN14" t="str">
+        <v/>
+      </c>
+      <c r="CO14">
         <v>0.16</v>
       </c>
-      <c r="CN14" t="str">
-        <v/>
-      </c>
-      <c r="CO14" t="str">
-        <v/>
-      </c>
-      <c r="CP14">
+      <c r="CP14" t="str">
+        <v/>
+      </c>
+      <c r="CQ14">
         <v>0.16</v>
-      </c>
-      <c r="CQ14" t="str">
-        <v/>
       </c>
       <c r="CR14">
         <v>0.16</v>
@@ -24551,19 +24551,19 @@
         <v>Brown, Christine 59375-66667 (60m)</v>
       </c>
       <c r="AL1" t="str">
+        <v>Office Hours Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="AM1" t="str">
+        <v>Office Hours Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="AN1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="AO1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="AM1" t="str">
+      <c r="AP1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="AN1" t="str">
-        <v>Office Hours Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="AO1" t="str">
-        <v>Office Hours Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="AP1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -24578,49 +24578,49 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AU1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="AV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AW1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AY1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="AZ1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="BA1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BB1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BA1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BB1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BC1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BD1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
       <c r="BE1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BF1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (420m)</v>
+      </c>
+      <c r="BG1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (420m)</v>
+      </c>
+      <c r="BH1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BI1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BH1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (420m)</v>
-      </c>
-      <c r="BI1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (420m)</v>
       </c>
       <c r="BJ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
@@ -24641,31 +24641,31 @@
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BP1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BQ1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
       <c r="BR1" t="str">
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BS1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (180m)</v>
+      </c>
+      <c r="BT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BS1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BT1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
       <c r="BU1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (180m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BW1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
       <c r="BX1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BY1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
@@ -24674,19 +24674,19 @@
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
       <c r="CA1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CB1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CC1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="CD1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CE1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="CF1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -24698,7 +24698,7 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CI1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CJ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -24888,17 +24888,17 @@
       <c r="BE2">
         <v>0.16</v>
       </c>
-      <c r="BF2">
+      <c r="BF2" t="str">
+        <v/>
+      </c>
+      <c r="BG2" t="str">
+        <v/>
+      </c>
+      <c r="BH2">
         <v>0.16</v>
       </c>
-      <c r="BG2">
+      <c r="BI2">
         <v>0.16</v>
-      </c>
-      <c r="BH2" t="str">
-        <v/>
-      </c>
-      <c r="BI2" t="str">
-        <v/>
       </c>
       <c r="BJ2">
         <v>0.16</v>
@@ -25166,17 +25166,17 @@
       <c r="BE3">
         <v>0</v>
       </c>
-      <c r="BF3">
-        <v>0</v>
-      </c>
-      <c r="BG3">
-        <v>0</v>
-      </c>
-      <c r="BH3" t="str">
-        <v/>
-      </c>
-      <c r="BI3" t="str">
-        <v/>
+      <c r="BF3" t="str">
+        <v/>
+      </c>
+      <c r="BG3" t="str">
+        <v/>
+      </c>
+      <c r="BH3">
+        <v>0</v>
+      </c>
+      <c r="BI3">
+        <v>0</v>
       </c>
       <c r="BJ3">
         <v>0</v>
@@ -25444,17 +25444,17 @@
       <c r="BE4">
         <v>0</v>
       </c>
-      <c r="BF4">
-        <v>0</v>
-      </c>
-      <c r="BG4">
-        <v>0</v>
-      </c>
-      <c r="BH4" t="str">
-        <v/>
-      </c>
-      <c r="BI4" t="str">
-        <v/>
+      <c r="BF4" t="str">
+        <v/>
+      </c>
+      <c r="BG4" t="str">
+        <v/>
+      </c>
+      <c r="BH4">
+        <v>0</v>
+      </c>
+      <c r="BI4">
+        <v>0</v>
       </c>
       <c r="BJ4">
         <v>0</v>
@@ -25665,14 +25665,14 @@
       <c r="AL5">
         <v>0</v>
       </c>
-      <c r="AM5">
-        <v>0</v>
+      <c r="AM5" t="str">
+        <v/>
       </c>
       <c r="AN5">
         <v>0</v>
       </c>
-      <c r="AO5" t="str">
-        <v/>
+      <c r="AO5">
+        <v>0</v>
       </c>
       <c r="AP5">
         <v>0</v>
@@ -25689,14 +25689,14 @@
       <c r="AT5">
         <v>0</v>
       </c>
-      <c r="AU5">
-        <v>0</v>
+      <c r="AU5" t="str">
+        <v/>
       </c>
       <c r="AV5">
         <v>0</v>
       </c>
-      <c r="AW5" t="str">
-        <v/>
+      <c r="AW5">
+        <v>0</v>
       </c>
       <c r="AX5">
         <v>0</v>
@@ -25719,17 +25719,17 @@
       <c r="BD5">
         <v>0</v>
       </c>
-      <c r="BE5">
-        <v>0</v>
-      </c>
-      <c r="BF5">
-        <v>0</v>
+      <c r="BE5" t="str">
+        <v/>
+      </c>
+      <c r="BF5" t="str">
+        <v/>
       </c>
       <c r="BG5" t="str">
         <v/>
       </c>
-      <c r="BH5" t="str">
-        <v/>
+      <c r="BH5">
+        <v>0</v>
       </c>
       <c r="BI5" t="str">
         <v/>
@@ -25755,17 +25755,17 @@
       <c r="BP5">
         <v>0</v>
       </c>
-      <c r="BQ5" t="str">
-        <v/>
-      </c>
-      <c r="BR5">
-        <v>0</v>
+      <c r="BQ5">
+        <v>0</v>
+      </c>
+      <c r="BR5" t="str">
+        <v/>
       </c>
       <c r="BS5">
         <v>0</v>
       </c>
-      <c r="BT5" t="str">
-        <v/>
+      <c r="BT5">
+        <v>0</v>
       </c>
       <c r="BU5">
         <v>0</v>
@@ -25776,8 +25776,8 @@
       <c r="BW5">
         <v>0</v>
       </c>
-      <c r="BX5">
-        <v>0</v>
+      <c r="BX5" t="str">
+        <v/>
       </c>
       <c r="BY5">
         <v>0</v>
@@ -25788,17 +25788,17 @@
       <c r="CA5">
         <v>0</v>
       </c>
-      <c r="CB5" t="str">
-        <v/>
-      </c>
-      <c r="CC5">
-        <v>0</v>
+      <c r="CB5">
+        <v>0</v>
+      </c>
+      <c r="CC5" t="str">
+        <v/>
       </c>
       <c r="CD5">
         <v>0</v>
       </c>
-      <c r="CE5" t="str">
-        <v/>
+      <c r="CE5">
+        <v>0</v>
       </c>
       <c r="CF5">
         <v>0</v>
@@ -26221,14 +26221,14 @@
       <c r="AL7">
         <v>0.05</v>
       </c>
-      <c r="AM7">
-        <v>0.05</v>
+      <c r="AM7" t="str">
+        <v/>
       </c>
       <c r="AN7">
         <v>0.05</v>
       </c>
-      <c r="AO7" t="str">
-        <v/>
+      <c r="AO7">
+        <v>0.05</v>
       </c>
       <c r="AP7">
         <v>0.05</v>
@@ -26245,14 +26245,14 @@
       <c r="AT7">
         <v>0.05</v>
       </c>
-      <c r="AU7">
-        <v>0.05</v>
+      <c r="AU7" t="str">
+        <v/>
       </c>
       <c r="AV7">
         <v>0.05</v>
       </c>
-      <c r="AW7" t="str">
-        <v/>
+      <c r="AW7">
+        <v>0.05</v>
       </c>
       <c r="AX7">
         <v>0.05</v>
@@ -26275,17 +26275,17 @@
       <c r="BD7">
         <v>0.05</v>
       </c>
-      <c r="BE7">
+      <c r="BE7" t="str">
+        <v/>
+      </c>
+      <c r="BF7" t="str">
+        <v/>
+      </c>
+      <c r="BG7" t="str">
+        <v/>
+      </c>
+      <c r="BH7">
         <v>0.05</v>
-      </c>
-      <c r="BF7">
-        <v>0.05</v>
-      </c>
-      <c r="BG7" t="str">
-        <v/>
-      </c>
-      <c r="BH7" t="str">
-        <v/>
       </c>
       <c r="BI7" t="str">
         <v/>
@@ -26311,20 +26311,20 @@
       <c r="BP7">
         <v>0.05</v>
       </c>
-      <c r="BQ7" t="str">
-        <v/>
-      </c>
-      <c r="BR7">
+      <c r="BQ7">
         <v>0.05</v>
       </c>
-      <c r="BS7">
+      <c r="BR7" t="str">
+        <v/>
+      </c>
+      <c r="BS7" t="str">
+        <v/>
+      </c>
+      <c r="BT7">
         <v>0.05</v>
       </c>
-      <c r="BT7" t="str">
-        <v/>
-      </c>
-      <c r="BU7" t="str">
-        <v/>
+      <c r="BU7">
+        <v>0.05</v>
       </c>
       <c r="BV7">
         <v>0.05</v>
@@ -26332,8 +26332,8 @@
       <c r="BW7">
         <v>0.05</v>
       </c>
-      <c r="BX7">
-        <v>0.05</v>
+      <c r="BX7" t="str">
+        <v/>
       </c>
       <c r="BY7">
         <v>0.05</v>
@@ -26344,17 +26344,17 @@
       <c r="CA7">
         <v>0.05</v>
       </c>
-      <c r="CB7" t="str">
-        <v/>
-      </c>
-      <c r="CC7">
+      <c r="CB7">
         <v>0.05</v>
+      </c>
+      <c r="CC7" t="str">
+        <v/>
       </c>
       <c r="CD7">
         <v>0.05</v>
       </c>
-      <c r="CE7" t="str">
-        <v/>
+      <c r="CE7">
+        <v>0.05</v>
       </c>
       <c r="CF7">
         <v>0.05</v>
@@ -26499,14 +26499,14 @@
       <c r="AL8">
         <v>0.08</v>
       </c>
-      <c r="AM8">
-        <v>0.08</v>
+      <c r="AM8" t="str">
+        <v/>
       </c>
       <c r="AN8">
         <v>0.08</v>
       </c>
-      <c r="AO8" t="str">
-        <v/>
+      <c r="AO8">
+        <v>0.08</v>
       </c>
       <c r="AP8">
         <v>0.08</v>
@@ -26523,14 +26523,14 @@
       <c r="AT8">
         <v>0.08</v>
       </c>
-      <c r="AU8">
-        <v>0.08</v>
+      <c r="AU8" t="str">
+        <v/>
       </c>
       <c r="AV8">
         <v>0.08</v>
       </c>
-      <c r="AW8" t="str">
-        <v/>
+      <c r="AW8">
+        <v>0.08</v>
       </c>
       <c r="AX8">
         <v>0.08</v>
@@ -26553,17 +26553,17 @@
       <c r="BD8">
         <v>0.08</v>
       </c>
-      <c r="BE8">
+      <c r="BE8" t="str">
+        <v/>
+      </c>
+      <c r="BF8" t="str">
+        <v/>
+      </c>
+      <c r="BG8" t="str">
+        <v/>
+      </c>
+      <c r="BH8">
         <v>0.08</v>
-      </c>
-      <c r="BF8">
-        <v>0.08</v>
-      </c>
-      <c r="BG8" t="str">
-        <v/>
-      </c>
-      <c r="BH8" t="str">
-        <v/>
       </c>
       <c r="BI8" t="str">
         <v/>
@@ -26589,17 +26589,17 @@
       <c r="BP8">
         <v>0.08</v>
       </c>
-      <c r="BQ8" t="str">
-        <v/>
-      </c>
-      <c r="BR8">
+      <c r="BQ8">
         <v>0.08</v>
+      </c>
+      <c r="BR8" t="str">
+        <v/>
       </c>
       <c r="BS8">
         <v>0.08</v>
       </c>
-      <c r="BT8" t="str">
-        <v/>
+      <c r="BT8">
+        <v>0.08</v>
       </c>
       <c r="BU8">
         <v>0.08</v>
@@ -26610,8 +26610,8 @@
       <c r="BW8">
         <v>0.08</v>
       </c>
-      <c r="BX8">
-        <v>0.08</v>
+      <c r="BX8" t="str">
+        <v/>
       </c>
       <c r="BY8">
         <v>0.08</v>
@@ -26622,17 +26622,17 @@
       <c r="CA8">
         <v>0.08</v>
       </c>
-      <c r="CB8" t="str">
-        <v/>
-      </c>
-      <c r="CC8">
+      <c r="CB8">
         <v>0.08</v>
+      </c>
+      <c r="CC8" t="str">
+        <v/>
       </c>
       <c r="CD8">
         <v>0.08</v>
       </c>
-      <c r="CE8" t="str">
-        <v/>
+      <c r="CE8">
+        <v>0.08</v>
       </c>
       <c r="CF8">
         <v>0.08</v>
@@ -26777,14 +26777,14 @@
       <c r="AL9">
         <v>0</v>
       </c>
-      <c r="AM9">
-        <v>0</v>
+      <c r="AM9" t="str">
+        <v/>
       </c>
       <c r="AN9">
         <v>0</v>
       </c>
-      <c r="AO9" t="str">
-        <v/>
+      <c r="AO9">
+        <v>0</v>
       </c>
       <c r="AP9">
         <v>0</v>
@@ -26831,17 +26831,17 @@
       <c r="BD9">
         <v>0</v>
       </c>
-      <c r="BE9">
-        <v>0</v>
-      </c>
-      <c r="BF9">
-        <v>0</v>
+      <c r="BE9" t="str">
+        <v/>
+      </c>
+      <c r="BF9" t="str">
+        <v/>
       </c>
       <c r="BG9" t="str">
         <v/>
       </c>
-      <c r="BH9" t="str">
-        <v/>
+      <c r="BH9">
+        <v>0</v>
       </c>
       <c r="BI9" t="str">
         <v/>
@@ -26867,17 +26867,17 @@
       <c r="BP9">
         <v>0</v>
       </c>
-      <c r="BQ9" t="str">
-        <v/>
-      </c>
-      <c r="BR9">
-        <v>0</v>
+      <c r="BQ9">
+        <v>0</v>
+      </c>
+      <c r="BR9" t="str">
+        <v/>
       </c>
       <c r="BS9">
         <v>0</v>
       </c>
-      <c r="BT9" t="str">
-        <v/>
+      <c r="BT9">
+        <v>0</v>
       </c>
       <c r="BU9">
         <v>0</v>
@@ -26888,8 +26888,8 @@
       <c r="BW9">
         <v>0</v>
       </c>
-      <c r="BX9">
-        <v>0</v>
+      <c r="BX9" t="str">
+        <v/>
       </c>
       <c r="BY9">
         <v>0</v>
@@ -26900,8 +26900,8 @@
       <c r="CA9">
         <v>0</v>
       </c>
-      <c r="CB9" t="str">
-        <v/>
+      <c r="CB9">
+        <v>0</v>
       </c>
       <c r="CC9">
         <v>0</v>
@@ -27112,17 +27112,17 @@
       <c r="BE10">
         <v>0.1</v>
       </c>
-      <c r="BF10">
+      <c r="BF10" t="str">
+        <v/>
+      </c>
+      <c r="BG10" t="str">
+        <v/>
+      </c>
+      <c r="BH10">
         <v>0.1</v>
       </c>
-      <c r="BG10">
+      <c r="BI10">
         <v>0.1</v>
-      </c>
-      <c r="BH10" t="str">
-        <v/>
-      </c>
-      <c r="BI10" t="str">
-        <v/>
       </c>
       <c r="BJ10">
         <v>0.1</v>
@@ -27390,17 +27390,17 @@
       <c r="BE11">
         <v>0.01</v>
       </c>
-      <c r="BF11">
+      <c r="BF11" t="str">
+        <v/>
+      </c>
+      <c r="BG11" t="str">
+        <v/>
+      </c>
+      <c r="BH11">
         <v>0.01</v>
       </c>
-      <c r="BG11">
+      <c r="BI11">
         <v>0.01</v>
-      </c>
-      <c r="BH11" t="str">
-        <v/>
-      </c>
-      <c r="BI11" t="str">
-        <v/>
       </c>
       <c r="BJ11">
         <v>0.01</v>
@@ -27668,17 +27668,17 @@
       <c r="BE12">
         <v>0</v>
       </c>
-      <c r="BF12">
-        <v>0</v>
-      </c>
-      <c r="BG12">
-        <v>0</v>
-      </c>
-      <c r="BH12" t="str">
-        <v/>
-      </c>
-      <c r="BI12" t="str">
-        <v/>
+      <c r="BF12" t="str">
+        <v/>
+      </c>
+      <c r="BG12" t="str">
+        <v/>
+      </c>
+      <c r="BH12">
+        <v>0</v>
+      </c>
+      <c r="BI12">
+        <v>0</v>
       </c>
       <c r="BJ12">
         <v>0</v>
@@ -27946,17 +27946,17 @@
       <c r="BE13">
         <v>0</v>
       </c>
-      <c r="BF13">
-        <v>0</v>
-      </c>
-      <c r="BG13">
-        <v>0</v>
-      </c>
-      <c r="BH13" t="str">
-        <v/>
-      </c>
-      <c r="BI13" t="str">
-        <v/>
+      <c r="BF13" t="str">
+        <v/>
+      </c>
+      <c r="BG13" t="str">
+        <v/>
+      </c>
+      <c r="BH13">
+        <v>0</v>
+      </c>
+      <c r="BI13">
+        <v>0</v>
       </c>
       <c r="BJ13">
         <v>0</v>
@@ -28173,10 +28173,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AK1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+      </c>
+      <c r="AL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="AL1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="AM1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -28200,13 +28200,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AT1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AU1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AV1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AW1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -28215,82 +28215,82 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AY1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="AZ1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BA1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (360m)</v>
+      </c>
+      <c r="BB1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (360m)</v>
+      </c>
+      <c r="BC1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BD1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BE1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BF1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BG1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BH1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BI1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (240m)</v>
+      </c>
+      <c r="BJ1" t="str">
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BK1" t="str">
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BL1" t="str">
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BM1" t="str">
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="AZ1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BA1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BB1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (360m)</v>
-      </c>
-      <c r="BC1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (360m)</v>
-      </c>
-      <c r="BD1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BE1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BF1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BG1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BH1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BI1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BJ1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (240m)</v>
-      </c>
-      <c r="BK1" t="str">
+      <c r="BO1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BL1" t="str">
+      <c r="BP1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BM1" t="str">
+      <c r="BQ1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BN1" t="str">
+      <c r="BR1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BO1" t="str">
+      <c r="BS1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BP1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BQ1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BR1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BS1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BU1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (180m)</v>
+      </c>
+      <c r="BV1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+      </c>
+      <c r="BW1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="BX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BV1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (180m)</v>
-      </c>
-      <c r="BW1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
-      </c>
-      <c r="BX1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BY1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -28471,14 +28471,14 @@
       <c r="AZ2">
         <v>0.25</v>
       </c>
-      <c r="BA2">
+      <c r="BA2" t="str">
+        <v/>
+      </c>
+      <c r="BB2" t="str">
+        <v/>
+      </c>
+      <c r="BC2">
         <v>0.25</v>
-      </c>
-      <c r="BB2" t="str">
-        <v/>
-      </c>
-      <c r="BC2" t="str">
-        <v/>
       </c>
       <c r="BD2">
         <v>0.25</v>
@@ -28674,11 +28674,11 @@
       <c r="AJ3">
         <v>0.07</v>
       </c>
-      <c r="AK3">
+      <c r="AK3" t="str">
+        <v/>
+      </c>
+      <c r="AL3">
         <v>0.07</v>
-      </c>
-      <c r="AL3" t="str">
-        <v/>
       </c>
       <c r="AM3">
         <v>0.07</v>
@@ -28719,65 +28719,65 @@
       <c r="AY3">
         <v>0.07</v>
       </c>
-      <c r="AZ3">
+      <c r="AZ3" t="str">
+        <v/>
+      </c>
+      <c r="BA3" t="str">
+        <v/>
+      </c>
+      <c r="BB3" t="str">
+        <v/>
+      </c>
+      <c r="BC3">
         <v>0.07</v>
       </c>
-      <c r="BA3" t="str">
-        <v/>
-      </c>
-      <c r="BB3" t="str">
-        <v/>
-      </c>
-      <c r="BC3" t="str">
-        <v/>
-      </c>
-      <c r="BD3">
+      <c r="BD3" t="str">
+        <v/>
+      </c>
+      <c r="BE3">
         <v>0.07</v>
       </c>
-      <c r="BE3" t="str">
-        <v/>
-      </c>
-      <c r="BF3">
+      <c r="BF3" t="str">
+        <v/>
+      </c>
+      <c r="BG3">
         <v>0.07</v>
       </c>
-      <c r="BG3" t="str">
-        <v/>
-      </c>
-      <c r="BH3">
+      <c r="BH3" t="str">
+        <v/>
+      </c>
+      <c r="BI3" t="str">
+        <v/>
+      </c>
+      <c r="BJ3">
         <v>0.07</v>
       </c>
-      <c r="BI3" t="str">
-        <v/>
-      </c>
-      <c r="BJ3" t="str">
-        <v/>
-      </c>
-      <c r="BK3">
+      <c r="BK3" t="str">
+        <v/>
+      </c>
+      <c r="BL3">
         <v>0.07</v>
       </c>
-      <c r="BL3" t="str">
-        <v/>
-      </c>
-      <c r="BM3">
+      <c r="BM3" t="str">
+        <v/>
+      </c>
+      <c r="BN3">
         <v>0.07</v>
-      </c>
-      <c r="BN3" t="str">
-        <v/>
       </c>
       <c r="BO3">
         <v>0.07</v>
       </c>
-      <c r="BP3">
+      <c r="BP3" t="str">
+        <v/>
+      </c>
+      <c r="BQ3">
         <v>0.07</v>
       </c>
-      <c r="BQ3" t="str">
-        <v/>
-      </c>
-      <c r="BR3">
+      <c r="BR3" t="str">
+        <v/>
+      </c>
+      <c r="BS3">
         <v>0.07</v>
-      </c>
-      <c r="BS3" t="str">
-        <v/>
       </c>
       <c r="BT3">
         <v>0.07</v>
@@ -28785,11 +28785,11 @@
       <c r="BU3">
         <v>0.07</v>
       </c>
-      <c r="BV3">
+      <c r="BV3" t="str">
+        <v/>
+      </c>
+      <c r="BW3">
         <v>0.07</v>
-      </c>
-      <c r="BW3" t="str">
-        <v/>
       </c>
       <c r="BX3">
         <v>0.07</v>
@@ -28925,11 +28925,11 @@
       <c r="AJ4">
         <v>0.13</v>
       </c>
-      <c r="AK4">
+      <c r="AK4" t="str">
+        <v/>
+      </c>
+      <c r="AL4">
         <v>0.13</v>
-      </c>
-      <c r="AL4" t="str">
-        <v/>
       </c>
       <c r="AM4">
         <v>0.13</v>
@@ -28970,65 +28970,65 @@
       <c r="AY4">
         <v>0.13</v>
       </c>
-      <c r="AZ4">
+      <c r="AZ4" t="str">
+        <v/>
+      </c>
+      <c r="BA4" t="str">
+        <v/>
+      </c>
+      <c r="BB4" t="str">
+        <v/>
+      </c>
+      <c r="BC4">
         <v>0.13</v>
       </c>
-      <c r="BA4" t="str">
-        <v/>
-      </c>
-      <c r="BB4" t="str">
-        <v/>
-      </c>
-      <c r="BC4" t="str">
-        <v/>
-      </c>
-      <c r="BD4">
+      <c r="BD4" t="str">
+        <v/>
+      </c>
+      <c r="BE4">
         <v>0.13</v>
       </c>
-      <c r="BE4" t="str">
-        <v/>
-      </c>
-      <c r="BF4">
+      <c r="BF4" t="str">
+        <v/>
+      </c>
+      <c r="BG4">
         <v>0.13</v>
       </c>
-      <c r="BG4" t="str">
-        <v/>
-      </c>
-      <c r="BH4">
+      <c r="BH4" t="str">
+        <v/>
+      </c>
+      <c r="BI4" t="str">
+        <v/>
+      </c>
+      <c r="BJ4">
         <v>0.13</v>
       </c>
-      <c r="BI4" t="str">
-        <v/>
-      </c>
-      <c r="BJ4" t="str">
-        <v/>
-      </c>
-      <c r="BK4">
+      <c r="BK4" t="str">
+        <v/>
+      </c>
+      <c r="BL4">
         <v>0.13</v>
       </c>
-      <c r="BL4" t="str">
-        <v/>
-      </c>
-      <c r="BM4">
+      <c r="BM4" t="str">
+        <v/>
+      </c>
+      <c r="BN4">
         <v>0.13</v>
-      </c>
-      <c r="BN4" t="str">
-        <v/>
       </c>
       <c r="BO4">
         <v>0.13</v>
       </c>
-      <c r="BP4">
+      <c r="BP4" t="str">
+        <v/>
+      </c>
+      <c r="BQ4">
         <v>0.13</v>
       </c>
-      <c r="BQ4" t="str">
-        <v/>
-      </c>
-      <c r="BR4">
+      <c r="BR4" t="str">
+        <v/>
+      </c>
+      <c r="BS4">
         <v>0.13</v>
-      </c>
-      <c r="BS4" t="str">
-        <v/>
       </c>
       <c r="BT4">
         <v>0.13</v>
@@ -29036,11 +29036,11 @@
       <c r="BU4">
         <v>0.13</v>
       </c>
-      <c r="BV4">
+      <c r="BV4" t="str">
+        <v/>
+      </c>
+      <c r="BW4">
         <v>0.13</v>
-      </c>
-      <c r="BW4" t="str">
-        <v/>
       </c>
       <c r="BX4">
         <v>0.13</v>
@@ -29176,11 +29176,11 @@
       <c r="AJ5">
         <v>0.78</v>
       </c>
-      <c r="AK5">
+      <c r="AK5" t="str">
+        <v/>
+      </c>
+      <c r="AL5">
         <v>0.78</v>
-      </c>
-      <c r="AL5" t="str">
-        <v/>
       </c>
       <c r="AM5">
         <v>0.78</v>
@@ -29221,65 +29221,65 @@
       <c r="AY5">
         <v>0.78</v>
       </c>
-      <c r="AZ5">
+      <c r="AZ5" t="str">
+        <v/>
+      </c>
+      <c r="BA5" t="str">
+        <v/>
+      </c>
+      <c r="BB5" t="str">
+        <v/>
+      </c>
+      <c r="BC5">
         <v>0.78</v>
       </c>
-      <c r="BA5" t="str">
-        <v/>
-      </c>
-      <c r="BB5" t="str">
-        <v/>
-      </c>
-      <c r="BC5" t="str">
-        <v/>
-      </c>
-      <c r="BD5">
+      <c r="BD5" t="str">
+        <v/>
+      </c>
+      <c r="BE5">
         <v>0.78</v>
       </c>
-      <c r="BE5" t="str">
-        <v/>
-      </c>
-      <c r="BF5">
+      <c r="BF5" t="str">
+        <v/>
+      </c>
+      <c r="BG5">
         <v>0.78</v>
       </c>
-      <c r="BG5" t="str">
-        <v/>
-      </c>
-      <c r="BH5">
+      <c r="BH5" t="str">
+        <v/>
+      </c>
+      <c r="BI5">
         <v>0.78</v>
-      </c>
-      <c r="BI5" t="str">
-        <v/>
       </c>
       <c r="BJ5">
         <v>0.78</v>
       </c>
-      <c r="BK5">
+      <c r="BK5" t="str">
+        <v/>
+      </c>
+      <c r="BL5">
         <v>0.78</v>
       </c>
-      <c r="BL5" t="str">
-        <v/>
-      </c>
-      <c r="BM5">
+      <c r="BM5" t="str">
+        <v/>
+      </c>
+      <c r="BN5">
         <v>0.78</v>
-      </c>
-      <c r="BN5" t="str">
-        <v/>
       </c>
       <c r="BO5">
         <v>0.78</v>
       </c>
-      <c r="BP5">
+      <c r="BP5" t="str">
+        <v/>
+      </c>
+      <c r="BQ5">
         <v>0.78</v>
       </c>
-      <c r="BQ5" t="str">
-        <v/>
-      </c>
-      <c r="BR5">
+      <c r="BR5" t="str">
+        <v/>
+      </c>
+      <c r="BS5">
         <v>0.78</v>
-      </c>
-      <c r="BS5" t="str">
-        <v/>
       </c>
       <c r="BT5">
         <v>0.78</v>
@@ -29287,11 +29287,11 @@
       <c r="BU5">
         <v>0.78</v>
       </c>
-      <c r="BV5">
+      <c r="BV5" t="str">
+        <v/>
+      </c>
+      <c r="BW5">
         <v>0.78</v>
-      </c>
-      <c r="BW5" t="str">
-        <v/>
       </c>
       <c r="BX5">
         <v>0.78</v>
@@ -29977,14 +29977,14 @@
       <c r="AZ8">
         <v>0.25</v>
       </c>
-      <c r="BA8">
+      <c r="BA8" t="str">
+        <v/>
+      </c>
+      <c r="BB8" t="str">
+        <v/>
+      </c>
+      <c r="BC8">
         <v>0.25</v>
-      </c>
-      <c r="BB8" t="str">
-        <v/>
-      </c>
-      <c r="BC8" t="str">
-        <v/>
       </c>
       <c r="BD8">
         <v>0.25</v>
@@ -30180,11 +30180,11 @@
       <c r="AJ9">
         <v>0.08</v>
       </c>
-      <c r="AK9">
+      <c r="AK9" t="str">
+        <v/>
+      </c>
+      <c r="AL9">
         <v>0.08</v>
-      </c>
-      <c r="AL9" t="str">
-        <v/>
       </c>
       <c r="AM9">
         <v>0.08</v>
@@ -30225,65 +30225,65 @@
       <c r="AY9">
         <v>0.08</v>
       </c>
-      <c r="AZ9">
+      <c r="AZ9" t="str">
+        <v/>
+      </c>
+      <c r="BA9" t="str">
+        <v/>
+      </c>
+      <c r="BB9" t="str">
+        <v/>
+      </c>
+      <c r="BC9">
         <v>0.08</v>
       </c>
-      <c r="BA9" t="str">
-        <v/>
-      </c>
-      <c r="BB9" t="str">
-        <v/>
-      </c>
-      <c r="BC9" t="str">
-        <v/>
-      </c>
-      <c r="BD9">
+      <c r="BD9" t="str">
+        <v/>
+      </c>
+      <c r="BE9">
         <v>0.08</v>
       </c>
-      <c r="BE9" t="str">
-        <v/>
-      </c>
-      <c r="BF9">
+      <c r="BF9" t="str">
+        <v/>
+      </c>
+      <c r="BG9">
         <v>0.08</v>
       </c>
-      <c r="BG9" t="str">
-        <v/>
-      </c>
-      <c r="BH9">
+      <c r="BH9" t="str">
+        <v/>
+      </c>
+      <c r="BI9">
         <v>0.08</v>
-      </c>
-      <c r="BI9" t="str">
-        <v/>
       </c>
       <c r="BJ9">
         <v>0.08</v>
       </c>
-      <c r="BK9">
+      <c r="BK9" t="str">
+        <v/>
+      </c>
+      <c r="BL9">
         <v>0.08</v>
       </c>
-      <c r="BL9" t="str">
-        <v/>
-      </c>
-      <c r="BM9">
+      <c r="BM9" t="str">
+        <v/>
+      </c>
+      <c r="BN9">
         <v>0.08</v>
-      </c>
-      <c r="BN9" t="str">
-        <v/>
       </c>
       <c r="BO9">
         <v>0.08</v>
       </c>
-      <c r="BP9">
+      <c r="BP9" t="str">
+        <v/>
+      </c>
+      <c r="BQ9">
         <v>0.08</v>
       </c>
-      <c r="BQ9" t="str">
-        <v/>
-      </c>
-      <c r="BR9">
+      <c r="BR9" t="str">
+        <v/>
+      </c>
+      <c r="BS9">
         <v>0.08</v>
-      </c>
-      <c r="BS9" t="str">
-        <v/>
       </c>
       <c r="BT9">
         <v>0.08</v>
@@ -30291,11 +30291,11 @@
       <c r="BU9">
         <v>0.08</v>
       </c>
-      <c r="BV9">
+      <c r="BV9" t="str">
+        <v/>
+      </c>
+      <c r="BW9">
         <v>0.08</v>
-      </c>
-      <c r="BW9" t="str">
-        <v/>
       </c>
       <c r="BX9">
         <v>0.08</v>
@@ -30476,8 +30476,8 @@
       <c r="AY10">
         <v>0</v>
       </c>
-      <c r="AZ10">
-        <v>0</v>
+      <c r="AZ10" t="str">
+        <v/>
       </c>
       <c r="BA10" t="str">
         <v/>
@@ -30485,56 +30485,56 @@
       <c r="BB10" t="str">
         <v/>
       </c>
-      <c r="BC10" t="str">
-        <v/>
-      </c>
-      <c r="BD10">
-        <v>0</v>
-      </c>
-      <c r="BE10" t="str">
-        <v/>
-      </c>
-      <c r="BF10">
-        <v>0</v>
-      </c>
-      <c r="BG10" t="str">
-        <v/>
-      </c>
-      <c r="BH10">
-        <v>0</v>
-      </c>
-      <c r="BI10" t="str">
-        <v/>
+      <c r="BC10">
+        <v>0</v>
+      </c>
+      <c r="BD10" t="str">
+        <v/>
+      </c>
+      <c r="BE10">
+        <v>0</v>
+      </c>
+      <c r="BF10" t="str">
+        <v/>
+      </c>
+      <c r="BG10">
+        <v>0</v>
+      </c>
+      <c r="BH10" t="str">
+        <v/>
+      </c>
+      <c r="BI10">
+        <v>0</v>
       </c>
       <c r="BJ10">
         <v>0</v>
       </c>
-      <c r="BK10">
-        <v>0</v>
-      </c>
-      <c r="BL10" t="str">
-        <v/>
-      </c>
-      <c r="BM10">
-        <v>0</v>
-      </c>
-      <c r="BN10" t="str">
-        <v/>
+      <c r="BK10" t="str">
+        <v/>
+      </c>
+      <c r="BL10">
+        <v>0</v>
+      </c>
+      <c r="BM10" t="str">
+        <v/>
+      </c>
+      <c r="BN10">
+        <v>0</v>
       </c>
       <c r="BO10">
         <v>0</v>
       </c>
-      <c r="BP10">
-        <v>0</v>
-      </c>
-      <c r="BQ10" t="str">
-        <v/>
-      </c>
-      <c r="BR10">
-        <v>0</v>
-      </c>
-      <c r="BS10" t="str">
-        <v/>
+      <c r="BP10" t="str">
+        <v/>
+      </c>
+      <c r="BQ10">
+        <v>0</v>
+      </c>
+      <c r="BR10" t="str">
+        <v/>
+      </c>
+      <c r="BS10">
+        <v>0</v>
       </c>
       <c r="BT10">
         <v>0</v>
@@ -30730,14 +30730,14 @@
       <c r="AZ11">
         <v>0.1</v>
       </c>
-      <c r="BA11">
+      <c r="BA11" t="str">
+        <v/>
+      </c>
+      <c r="BB11" t="str">
+        <v/>
+      </c>
+      <c r="BC11">
         <v>0.1</v>
-      </c>
-      <c r="BB11" t="str">
-        <v/>
-      </c>
-      <c r="BC11" t="str">
-        <v/>
       </c>
       <c r="BD11">
         <v>0.1</v>
@@ -30981,14 +30981,14 @@
       <c r="AZ12">
         <v>0</v>
       </c>
-      <c r="BA12">
-        <v>0</v>
+      <c r="BA12" t="str">
+        <v/>
       </c>
       <c r="BB12" t="str">
         <v/>
       </c>
-      <c r="BC12" t="str">
-        <v/>
+      <c r="BC12">
+        <v>0</v>
       </c>
       <c r="BD12">
         <v>0</v>
@@ -31232,14 +31232,14 @@
       <c r="AZ13">
         <v>0.14</v>
       </c>
-      <c r="BA13">
+      <c r="BA13" t="str">
+        <v/>
+      </c>
+      <c r="BB13" t="str">
+        <v/>
+      </c>
+      <c r="BC13">
         <v>0.14</v>
-      </c>
-      <c r="BB13" t="str">
-        <v/>
-      </c>
-      <c r="BC13" t="str">
-        <v/>
       </c>
       <c r="BD13">
         <v>0.14</v>
@@ -31483,14 +31483,14 @@
       <c r="AZ14">
         <v>0</v>
       </c>
-      <c r="BA14">
-        <v>0</v>
+      <c r="BA14" t="str">
+        <v/>
       </c>
       <c r="BB14" t="str">
         <v/>
       </c>
-      <c r="BC14" t="str">
-        <v/>
+      <c r="BC14">
+        <v>0</v>
       </c>
       <c r="BD14">
         <v>0</v>
@@ -31686,11 +31686,11 @@
       <c r="AJ15">
         <v>0</v>
       </c>
-      <c r="AK15">
-        <v>0</v>
-      </c>
-      <c r="AL15" t="str">
-        <v/>
+      <c r="AK15" t="str">
+        <v/>
+      </c>
+      <c r="AL15">
+        <v>0</v>
       </c>
       <c r="AM15">
         <v>0</v>
@@ -31734,14 +31734,14 @@
       <c r="AZ15">
         <v>0</v>
       </c>
-      <c r="BA15">
-        <v>0</v>
+      <c r="BA15" t="str">
+        <v/>
       </c>
       <c r="BB15" t="str">
         <v/>
       </c>
-      <c r="BC15" t="str">
-        <v/>
+      <c r="BC15">
+        <v>0</v>
       </c>
       <c r="BD15">
         <v>0</v>
@@ -31797,11 +31797,11 @@
       <c r="BU15">
         <v>0</v>
       </c>
-      <c r="BV15">
-        <v>0</v>
-      </c>
-      <c r="BW15" t="str">
-        <v/>
+      <c r="BV15" t="str">
+        <v/>
+      </c>
+      <c r="BW15">
+        <v>0</v>
       </c>
       <c r="BX15">
         <v>0</v>
@@ -31985,14 +31985,14 @@
       <c r="AZ16">
         <v>0.09</v>
       </c>
-      <c r="BA16">
+      <c r="BA16" t="str">
+        <v/>
+      </c>
+      <c r="BB16" t="str">
+        <v/>
+      </c>
+      <c r="BC16">
         <v>0.09</v>
-      </c>
-      <c r="BB16" t="str">
-        <v/>
-      </c>
-      <c r="BC16" t="str">
-        <v/>
       </c>
       <c r="BD16">
         <v>0.09</v>

</xml_diff>

<commit_message>
Improve weekly plan view to show employee availability and visits
Refactor weekly plan tab to display vertical days with available employee time slots, enhance employee search to only show assigned employees, and display visit counts per employee.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: bffc5ac4-3baf-45b9-b032-d481ce008e0d
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f111f999-5923-4927-b1a6-82fa47fe9a5b/bffc5ac4-3baf-45b9-b032-d481ce008e0d/6X6nk7m
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3690,19 +3690,19 @@
         <v>Brown, Christine 33333-.6875 (60m)</v>
       </c>
       <c r="AD1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AE1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="AE1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AF1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AG1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AH1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (165m)</v>
-      </c>
-      <c r="AH1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AI1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -3723,13 +3723,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AO1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AP1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AQ1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AR1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -3738,67 +3738,67 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AT1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AU1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AU1" t="str">
+      <c r="AV1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AV1" t="str">
+      <c r="AW1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AW1" t="str">
+      <c r="AX1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AX1" t="str">
+      <c r="AY1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AY1" t="str">
+      <c r="AZ1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BA1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BA1" t="str">
+      <c r="BB1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BB1" t="str">
+      <c r="BC1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BC1" t="str">
+      <c r="BD1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BD1" t="str">
+      <c r="BE1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BF1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BG1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BH1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BI1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BJ1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BK1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BK1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BM1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BN1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BO1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -3810,10 +3810,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BR1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BS1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BS1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -6569,10 +6569,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AC1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AD1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (240m)</v>
-      </c>
-      <c r="AD1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AE1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -6593,13 +6593,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AK1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AM1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -6608,58 +6608,58 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AP1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AQ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AQ1" t="str">
+      <c r="AR1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AR1" t="str">
+      <c r="AS1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AS1" t="str">
+      <c r="AT1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AT1" t="str">
+      <c r="AU1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AU1" t="str">
+      <c r="AV1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AV1" t="str">
+      <c r="AW1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AW1" t="str">
+      <c r="AX1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AX1" t="str">
+      <c r="AY1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AY1" t="str">
+      <c r="AZ1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BA1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BA1" t="str">
+      <c r="BB1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BB1" t="str">
+      <c r="BC1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BC1" t="str">
+      <c r="BD1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BD1" t="str">
+      <c r="BE1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BF1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BG1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BG1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BH1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -6668,16 +6668,16 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BJ1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BK1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
-      <c r="BK1" t="str">
+      <c r="BL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BL1" t="str">
+      <c r="BM1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (180m)</v>
-      </c>
-      <c r="BM1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -7022,56 +7022,56 @@
       <c r="AP3">
         <v>0</v>
       </c>
-      <c r="AQ3" t="str">
-        <v/>
-      </c>
-      <c r="AR3">
-        <v>0</v>
-      </c>
-      <c r="AS3" t="str">
-        <v/>
-      </c>
-      <c r="AT3">
-        <v>0</v>
-      </c>
-      <c r="AU3" t="str">
-        <v/>
-      </c>
-      <c r="AV3">
-        <v>0</v>
-      </c>
-      <c r="AW3" t="str">
-        <v/>
-      </c>
-      <c r="AX3">
-        <v>0</v>
-      </c>
-      <c r="AY3" t="str">
-        <v/>
-      </c>
-      <c r="AZ3">
-        <v>0</v>
-      </c>
-      <c r="BA3" t="str">
-        <v/>
-      </c>
-      <c r="BB3">
-        <v>0</v>
-      </c>
-      <c r="BC3" t="str">
-        <v/>
-      </c>
-      <c r="BD3">
-        <v>0</v>
+      <c r="AQ3">
+        <v>0</v>
+      </c>
+      <c r="AR3" t="str">
+        <v/>
+      </c>
+      <c r="AS3">
+        <v>0</v>
+      </c>
+      <c r="AT3" t="str">
+        <v/>
+      </c>
+      <c r="AU3">
+        <v>0</v>
+      </c>
+      <c r="AV3" t="str">
+        <v/>
+      </c>
+      <c r="AW3">
+        <v>0</v>
+      </c>
+      <c r="AX3" t="str">
+        <v/>
+      </c>
+      <c r="AY3">
+        <v>0</v>
+      </c>
+      <c r="AZ3" t="str">
+        <v/>
+      </c>
+      <c r="BA3">
+        <v>0</v>
+      </c>
+      <c r="BB3" t="str">
+        <v/>
+      </c>
+      <c r="BC3">
+        <v>0</v>
+      </c>
+      <c r="BD3" t="str">
+        <v/>
       </c>
       <c r="BE3">
         <v>0</v>
       </c>
-      <c r="BF3" t="str">
-        <v/>
-      </c>
-      <c r="BG3">
-        <v>0</v>
+      <c r="BF3">
+        <v>0</v>
+      </c>
+      <c r="BG3" t="str">
+        <v/>
       </c>
       <c r="BH3">
         <v>0</v>
@@ -8010,11 +8010,11 @@
       <c r="AB8">
         <v>0.78</v>
       </c>
-      <c r="AC8" t="str">
-        <v/>
-      </c>
-      <c r="AD8">
+      <c r="AC8">
         <v>0.78</v>
+      </c>
+      <c r="AD8" t="str">
+        <v/>
       </c>
       <c r="AE8">
         <v>0.78</v>
@@ -8052,56 +8052,56 @@
       <c r="AP8">
         <v>0.78</v>
       </c>
-      <c r="AQ8" t="str">
-        <v/>
-      </c>
-      <c r="AR8">
+      <c r="AQ8">
         <v>0.78</v>
       </c>
-      <c r="AS8" t="str">
-        <v/>
-      </c>
-      <c r="AT8">
+      <c r="AR8" t="str">
+        <v/>
+      </c>
+      <c r="AS8">
         <v>0.78</v>
       </c>
-      <c r="AU8" t="str">
-        <v/>
-      </c>
-      <c r="AV8">
+      <c r="AT8" t="str">
+        <v/>
+      </c>
+      <c r="AU8">
         <v>0.78</v>
       </c>
-      <c r="AW8" t="str">
-        <v/>
-      </c>
-      <c r="AX8">
+      <c r="AV8" t="str">
+        <v/>
+      </c>
+      <c r="AW8">
         <v>0.78</v>
       </c>
-      <c r="AY8" t="str">
-        <v/>
-      </c>
-      <c r="AZ8">
+      <c r="AX8" t="str">
+        <v/>
+      </c>
+      <c r="AY8">
         <v>0.78</v>
       </c>
-      <c r="BA8" t="str">
-        <v/>
-      </c>
-      <c r="BB8">
+      <c r="AZ8" t="str">
+        <v/>
+      </c>
+      <c r="BA8">
         <v>0.78</v>
       </c>
-      <c r="BC8" t="str">
-        <v/>
-      </c>
-      <c r="BD8">
+      <c r="BB8" t="str">
+        <v/>
+      </c>
+      <c r="BC8">
         <v>0.78</v>
+      </c>
+      <c r="BD8" t="str">
+        <v/>
       </c>
       <c r="BE8">
         <v>0.78</v>
       </c>
-      <c r="BF8" t="str">
-        <v/>
-      </c>
-      <c r="BG8">
+      <c r="BF8">
         <v>0.78</v>
+      </c>
+      <c r="BG8" t="str">
+        <v/>
       </c>
       <c r="BH8">
         <v>0.78</v>
@@ -22403,16 +22403,16 @@
         <v>Anderson, Margaret 33333-2.375 (60m)</v>
       </c>
       <c r="AJ1" t="str">
+        <v>Armstrong (NL), Hugh .4375-66667 (60m)</v>
+      </c>
+      <c r="AK1" t="str">
+        <v>Brown, Christine 59375-66667 (60m)</v>
+      </c>
+      <c r="AL1" t="str">
         <v>Office Hours Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AK1" t="str">
+      <c r="AM1" t="str">
         <v>Office Hours Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="AL1" t="str">
-        <v>Armstrong (NL), Hugh .4375-66667 (60m)</v>
-      </c>
-      <c r="AM1" t="str">
-        <v>Brown, Christine 59375-66667 (60m)</v>
       </c>
       <c r="AN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
@@ -22681,16 +22681,16 @@
         <v>1.01</v>
       </c>
       <c r="AJ2">
+        <v>0.68</v>
+      </c>
+      <c r="AK2">
+        <v>1.03</v>
+      </c>
+      <c r="AL2">
         <v>0.16</v>
       </c>
-      <c r="AK2">
+      <c r="AM2">
         <v>0.16</v>
-      </c>
-      <c r="AL2">
-        <v>0.68</v>
-      </c>
-      <c r="AM2">
-        <v>1.03</v>
       </c>
       <c r="AN2">
         <v>0.16</v>
@@ -22959,16 +22959,16 @@
         <v>0.9</v>
       </c>
       <c r="AJ3">
-        <v>0</v>
+        <v>0.86</v>
       </c>
       <c r="AK3">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="AL3">
-        <v>0.86</v>
+        <v>0</v>
       </c>
       <c r="AM3">
-        <v>0.77</v>
+        <v>0</v>
       </c>
       <c r="AN3">
         <v>0</v>
@@ -23237,16 +23237,16 @@
         <v>0.97</v>
       </c>
       <c r="AJ4">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="AK4">
-        <v>0</v>
+        <v>1.03</v>
       </c>
       <c r="AL4">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="AM4">
-        <v>1.03</v>
+        <v>0</v>
       </c>
       <c r="AN4">
         <v>0</v>
@@ -23515,16 +23515,16 @@
         <v>0.74</v>
       </c>
       <c r="AJ5">
-        <v>0</v>
-      </c>
-      <c r="AK5" t="str">
-        <v/>
+        <v>0.99</v>
+      </c>
+      <c r="AK5">
+        <v>0.77</v>
       </c>
       <c r="AL5">
-        <v>0.99</v>
-      </c>
-      <c r="AM5">
-        <v>0.77</v>
+        <v>0</v>
+      </c>
+      <c r="AM5" t="str">
+        <v/>
       </c>
       <c r="AN5">
         <v>0</v>
@@ -23792,17 +23792,17 @@
       <c r="AI6">
         <v>0.77</v>
       </c>
-      <c r="AJ6" t="str">
-        <v/>
-      </c>
-      <c r="AK6" t="str">
-        <v/>
-      </c>
-      <c r="AL6">
+      <c r="AJ6">
         <v>0.99</v>
       </c>
-      <c r="AM6">
+      <c r="AK6">
         <v>0.79</v>
+      </c>
+      <c r="AL6" t="str">
+        <v/>
+      </c>
+      <c r="AM6" t="str">
+        <v/>
       </c>
       <c r="AN6" t="str">
         <v/>
@@ -24071,16 +24071,16 @@
         <v>0.88</v>
       </c>
       <c r="AJ7">
+        <v>0.77</v>
+      </c>
+      <c r="AK7">
+        <v>1.04</v>
+      </c>
+      <c r="AL7">
         <v>0.05</v>
       </c>
-      <c r="AK7" t="str">
-        <v/>
-      </c>
-      <c r="AL7">
-        <v>0.77</v>
-      </c>
-      <c r="AM7">
-        <v>1.04</v>
+      <c r="AM7" t="str">
+        <v/>
       </c>
       <c r="AN7">
         <v>0.05</v>
@@ -24349,16 +24349,16 @@
         <v>0.89</v>
       </c>
       <c r="AJ8">
+        <v>1.07</v>
+      </c>
+      <c r="AK8">
+        <v>0.91</v>
+      </c>
+      <c r="AL8">
         <v>0.08</v>
       </c>
-      <c r="AK8" t="str">
-        <v/>
-      </c>
-      <c r="AL8">
-        <v>1.07</v>
-      </c>
-      <c r="AM8">
-        <v>0.91</v>
+      <c r="AM8" t="str">
+        <v/>
       </c>
       <c r="AN8">
         <v>0.08</v>
@@ -24627,16 +24627,16 @@
         <v>0.66</v>
       </c>
       <c r="AJ9">
-        <v>0</v>
-      </c>
-      <c r="AK9" t="str">
-        <v/>
+        <v>0.88</v>
+      </c>
+      <c r="AK9">
+        <v>0.72</v>
       </c>
       <c r="AL9">
-        <v>0.88</v>
-      </c>
-      <c r="AM9">
-        <v>0.72</v>
+        <v>0</v>
+      </c>
+      <c r="AM9" t="str">
+        <v/>
       </c>
       <c r="AN9">
         <v>0</v>
@@ -24905,16 +24905,16 @@
         <v>0.2</v>
       </c>
       <c r="AJ10">
+        <v>0.2</v>
+      </c>
+      <c r="AK10">
+        <v>0.2</v>
+      </c>
+      <c r="AL10">
         <v>0.1</v>
       </c>
-      <c r="AK10">
+      <c r="AM10">
         <v>0.1</v>
-      </c>
-      <c r="AL10">
-        <v>0.2</v>
-      </c>
-      <c r="AM10">
-        <v>0.2</v>
       </c>
       <c r="AN10">
         <v>0.1</v>
@@ -25183,16 +25183,16 @@
         <v>0.76</v>
       </c>
       <c r="AJ11">
+        <v>0.98</v>
+      </c>
+      <c r="AK11">
+        <v>0.8</v>
+      </c>
+      <c r="AL11">
         <v>0.01</v>
       </c>
-      <c r="AK11">
+      <c r="AM11">
         <v>0.01</v>
-      </c>
-      <c r="AL11">
-        <v>0.98</v>
-      </c>
-      <c r="AM11">
-        <v>0.8</v>
       </c>
       <c r="AN11">
         <v>0.01</v>
@@ -25461,16 +25461,16 @@
         <v>0.63</v>
       </c>
       <c r="AJ12">
-        <v>0</v>
+        <v>0.46</v>
       </c>
       <c r="AK12">
-        <v>0</v>
+        <v>0.46</v>
       </c>
       <c r="AL12">
-        <v>0.46</v>
+        <v>0</v>
       </c>
       <c r="AM12">
-        <v>0.46</v>
+        <v>0</v>
       </c>
       <c r="AN12">
         <v>0</v>
@@ -25739,16 +25739,16 @@
         <v>0.66</v>
       </c>
       <c r="AJ13">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="AK13">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="AL13">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="AM13">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="AN13">
         <v>0</v>
@@ -26031,10 +26031,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AK1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (285m)</v>
-      </c>
-      <c r="AL1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AM1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -26058,13 +26058,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AT1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AU1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AV1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="AW1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -26073,82 +26073,82 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AY1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AZ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BA1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BA1" t="str">
+      <c r="BB1" t="str">
         <v>Specialised Care Client 09:00-12:00 (360m)</v>
       </c>
-      <c r="BB1" t="str">
+      <c r="BC1" t="str">
         <v>Specialised Care Client 14:00-17:00 (360m)</v>
       </c>
-      <c r="BC1" t="str">
+      <c r="BD1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BD1" t="str">
+      <c r="BE1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BF1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BG1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BH1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BI1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BJ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (240m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BK1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BK1" t="str">
+      <c r="BL1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BL1" t="str">
+      <c r="BM1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BM1" t="str">
+      <c r="BN1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BN1" t="str">
+      <c r="BO1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BO1" t="str">
+      <c r="BP1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BP1" t="str">
+      <c r="BQ1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BQ1" t="str">
+      <c r="BR1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BR1" t="str">
+      <c r="BS1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BS1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BT1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BU1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (180m)</v>
       </c>
-      <c r="BV1" t="str">
+      <c r="BW1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
-      <c r="BW1" t="str">
+      <c r="BX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BX1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BY1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -26329,14 +26329,14 @@
       <c r="AZ2">
         <v>0.25</v>
       </c>
-      <c r="BA2" t="str">
-        <v/>
+      <c r="BA2">
+        <v>0.25</v>
       </c>
       <c r="BB2" t="str">
         <v/>
       </c>
-      <c r="BC2">
-        <v>0.25</v>
+      <c r="BC2" t="str">
+        <v/>
       </c>
       <c r="BD2">
         <v>0.25</v>
@@ -26532,11 +26532,11 @@
       <c r="AJ3">
         <v>0.07</v>
       </c>
-      <c r="AK3" t="str">
-        <v/>
-      </c>
-      <c r="AL3">
+      <c r="AK3">
         <v>0.07</v>
+      </c>
+      <c r="AL3" t="str">
+        <v/>
       </c>
       <c r="AM3">
         <v>0.07</v>
@@ -26577,8 +26577,8 @@
       <c r="AY3">
         <v>0.07</v>
       </c>
-      <c r="AZ3" t="str">
-        <v/>
+      <c r="AZ3">
+        <v>0.07</v>
       </c>
       <c r="BA3" t="str">
         <v/>
@@ -26586,56 +26586,56 @@
       <c r="BB3" t="str">
         <v/>
       </c>
-      <c r="BC3">
+      <c r="BC3" t="str">
+        <v/>
+      </c>
+      <c r="BD3">
         <v>0.07</v>
       </c>
-      <c r="BD3" t="str">
-        <v/>
-      </c>
-      <c r="BE3">
+      <c r="BE3" t="str">
+        <v/>
+      </c>
+      <c r="BF3">
         <v>0.07</v>
       </c>
-      <c r="BF3" t="str">
-        <v/>
-      </c>
-      <c r="BG3">
+      <c r="BG3" t="str">
+        <v/>
+      </c>
+      <c r="BH3">
         <v>0.07</v>
       </c>
-      <c r="BH3" t="str">
-        <v/>
-      </c>
       <c r="BI3" t="str">
         <v/>
       </c>
-      <c r="BJ3">
+      <c r="BJ3" t="str">
+        <v/>
+      </c>
+      <c r="BK3">
         <v>0.07</v>
       </c>
-      <c r="BK3" t="str">
-        <v/>
-      </c>
-      <c r="BL3">
+      <c r="BL3" t="str">
+        <v/>
+      </c>
+      <c r="BM3">
         <v>0.07</v>
       </c>
-      <c r="BM3" t="str">
-        <v/>
-      </c>
-      <c r="BN3">
-        <v>0.07</v>
+      <c r="BN3" t="str">
+        <v/>
       </c>
       <c r="BO3">
         <v>0.07</v>
       </c>
-      <c r="BP3" t="str">
-        <v/>
-      </c>
-      <c r="BQ3">
+      <c r="BP3">
         <v>0.07</v>
       </c>
-      <c r="BR3" t="str">
-        <v/>
-      </c>
-      <c r="BS3">
+      <c r="BQ3" t="str">
+        <v/>
+      </c>
+      <c r="BR3">
         <v>0.07</v>
+      </c>
+      <c r="BS3" t="str">
+        <v/>
       </c>
       <c r="BT3">
         <v>0.07</v>
@@ -26643,11 +26643,11 @@
       <c r="BU3">
         <v>0.07</v>
       </c>
-      <c r="BV3" t="str">
-        <v/>
-      </c>
-      <c r="BW3">
+      <c r="BV3">
         <v>0.07</v>
+      </c>
+      <c r="BW3" t="str">
+        <v/>
       </c>
       <c r="BX3">
         <v>0.07</v>
@@ -26783,11 +26783,11 @@
       <c r="AJ4">
         <v>0.13</v>
       </c>
-      <c r="AK4" t="str">
-        <v/>
-      </c>
-      <c r="AL4">
+      <c r="AK4">
         <v>0.13</v>
+      </c>
+      <c r="AL4" t="str">
+        <v/>
       </c>
       <c r="AM4">
         <v>0.13</v>
@@ -26828,8 +26828,8 @@
       <c r="AY4">
         <v>0.13</v>
       </c>
-      <c r="AZ4" t="str">
-        <v/>
+      <c r="AZ4">
+        <v>0.13</v>
       </c>
       <c r="BA4" t="str">
         <v/>
@@ -26837,56 +26837,56 @@
       <c r="BB4" t="str">
         <v/>
       </c>
-      <c r="BC4">
+      <c r="BC4" t="str">
+        <v/>
+      </c>
+      <c r="BD4">
         <v>0.13</v>
       </c>
-      <c r="BD4" t="str">
-        <v/>
-      </c>
-      <c r="BE4">
+      <c r="BE4" t="str">
+        <v/>
+      </c>
+      <c r="BF4">
         <v>0.13</v>
       </c>
-      <c r="BF4" t="str">
-        <v/>
-      </c>
-      <c r="BG4">
+      <c r="BG4" t="str">
+        <v/>
+      </c>
+      <c r="BH4">
         <v>0.13</v>
       </c>
-      <c r="BH4" t="str">
-        <v/>
-      </c>
       <c r="BI4" t="str">
         <v/>
       </c>
-      <c r="BJ4">
+      <c r="BJ4" t="str">
+        <v/>
+      </c>
+      <c r="BK4">
         <v>0.13</v>
       </c>
-      <c r="BK4" t="str">
-        <v/>
-      </c>
-      <c r="BL4">
+      <c r="BL4" t="str">
+        <v/>
+      </c>
+      <c r="BM4">
         <v>0.13</v>
       </c>
-      <c r="BM4" t="str">
-        <v/>
-      </c>
-      <c r="BN4">
-        <v>0.13</v>
+      <c r="BN4" t="str">
+        <v/>
       </c>
       <c r="BO4">
         <v>0.13</v>
       </c>
-      <c r="BP4" t="str">
-        <v/>
-      </c>
-      <c r="BQ4">
+      <c r="BP4">
         <v>0.13</v>
       </c>
-      <c r="BR4" t="str">
-        <v/>
-      </c>
-      <c r="BS4">
+      <c r="BQ4" t="str">
+        <v/>
+      </c>
+      <c r="BR4">
         <v>0.13</v>
+      </c>
+      <c r="BS4" t="str">
+        <v/>
       </c>
       <c r="BT4">
         <v>0.13</v>
@@ -26894,11 +26894,11 @@
       <c r="BU4">
         <v>0.13</v>
       </c>
-      <c r="BV4" t="str">
-        <v/>
-      </c>
-      <c r="BW4">
+      <c r="BV4">
         <v>0.13</v>
+      </c>
+      <c r="BW4" t="str">
+        <v/>
       </c>
       <c r="BX4">
         <v>0.13</v>
@@ -27034,11 +27034,11 @@
       <c r="AJ5">
         <v>0.78</v>
       </c>
-      <c r="AK5" t="str">
-        <v/>
-      </c>
-      <c r="AL5">
+      <c r="AK5">
         <v>0.78</v>
+      </c>
+      <c r="AL5" t="str">
+        <v/>
       </c>
       <c r="AM5">
         <v>0.78</v>
@@ -27079,8 +27079,8 @@
       <c r="AY5">
         <v>0.78</v>
       </c>
-      <c r="AZ5" t="str">
-        <v/>
+      <c r="AZ5">
+        <v>0.78</v>
       </c>
       <c r="BA5" t="str">
         <v/>
@@ -27088,56 +27088,56 @@
       <c r="BB5" t="str">
         <v/>
       </c>
-      <c r="BC5">
+      <c r="BC5" t="str">
+        <v/>
+      </c>
+      <c r="BD5">
         <v>0.78</v>
       </c>
-      <c r="BD5" t="str">
-        <v/>
-      </c>
-      <c r="BE5">
+      <c r="BE5" t="str">
+        <v/>
+      </c>
+      <c r="BF5">
         <v>0.78</v>
       </c>
-      <c r="BF5" t="str">
-        <v/>
-      </c>
-      <c r="BG5">
+      <c r="BG5" t="str">
+        <v/>
+      </c>
+      <c r="BH5">
         <v>0.78</v>
       </c>
-      <c r="BH5" t="str">
-        <v/>
-      </c>
-      <c r="BI5">
-        <v>0.78</v>
+      <c r="BI5" t="str">
+        <v/>
       </c>
       <c r="BJ5">
         <v>0.78</v>
       </c>
-      <c r="BK5" t="str">
-        <v/>
-      </c>
-      <c r="BL5">
+      <c r="BK5">
         <v>0.78</v>
       </c>
-      <c r="BM5" t="str">
-        <v/>
-      </c>
-      <c r="BN5">
+      <c r="BL5" t="str">
+        <v/>
+      </c>
+      <c r="BM5">
         <v>0.78</v>
+      </c>
+      <c r="BN5" t="str">
+        <v/>
       </c>
       <c r="BO5">
         <v>0.78</v>
       </c>
-      <c r="BP5" t="str">
-        <v/>
-      </c>
-      <c r="BQ5">
+      <c r="BP5">
         <v>0.78</v>
       </c>
-      <c r="BR5" t="str">
-        <v/>
-      </c>
-      <c r="BS5">
+      <c r="BQ5" t="str">
+        <v/>
+      </c>
+      <c r="BR5">
         <v>0.78</v>
+      </c>
+      <c r="BS5" t="str">
+        <v/>
       </c>
       <c r="BT5">
         <v>0.78</v>
@@ -27145,11 +27145,11 @@
       <c r="BU5">
         <v>0.78</v>
       </c>
-      <c r="BV5" t="str">
-        <v/>
-      </c>
-      <c r="BW5">
+      <c r="BV5">
         <v>0.78</v>
+      </c>
+      <c r="BW5" t="str">
+        <v/>
       </c>
       <c r="BX5">
         <v>0.78</v>
@@ -27835,14 +27835,14 @@
       <c r="AZ8">
         <v>0.25</v>
       </c>
-      <c r="BA8" t="str">
-        <v/>
+      <c r="BA8">
+        <v>0.25</v>
       </c>
       <c r="BB8" t="str">
         <v/>
       </c>
-      <c r="BC8">
-        <v>0.25</v>
+      <c r="BC8" t="str">
+        <v/>
       </c>
       <c r="BD8">
         <v>0.25</v>
@@ -28038,11 +28038,11 @@
       <c r="AJ9">
         <v>0.08</v>
       </c>
-      <c r="AK9" t="str">
-        <v/>
-      </c>
-      <c r="AL9">
+      <c r="AK9">
         <v>0.08</v>
+      </c>
+      <c r="AL9" t="str">
+        <v/>
       </c>
       <c r="AM9">
         <v>0.08</v>
@@ -28083,8 +28083,8 @@
       <c r="AY9">
         <v>0.08</v>
       </c>
-      <c r="AZ9" t="str">
-        <v/>
+      <c r="AZ9">
+        <v>0.08</v>
       </c>
       <c r="BA9" t="str">
         <v/>
@@ -28092,56 +28092,56 @@
       <c r="BB9" t="str">
         <v/>
       </c>
-      <c r="BC9">
+      <c r="BC9" t="str">
+        <v/>
+      </c>
+      <c r="BD9">
         <v>0.08</v>
       </c>
-      <c r="BD9" t="str">
-        <v/>
-      </c>
-      <c r="BE9">
+      <c r="BE9" t="str">
+        <v/>
+      </c>
+      <c r="BF9">
         <v>0.08</v>
       </c>
-      <c r="BF9" t="str">
-        <v/>
-      </c>
-      <c r="BG9">
+      <c r="BG9" t="str">
+        <v/>
+      </c>
+      <c r="BH9">
         <v>0.08</v>
       </c>
-      <c r="BH9" t="str">
-        <v/>
-      </c>
-      <c r="BI9">
-        <v>0.08</v>
+      <c r="BI9" t="str">
+        <v/>
       </c>
       <c r="BJ9">
         <v>0.08</v>
       </c>
-      <c r="BK9" t="str">
-        <v/>
-      </c>
-      <c r="BL9">
+      <c r="BK9">
         <v>0.08</v>
       </c>
-      <c r="BM9" t="str">
-        <v/>
-      </c>
-      <c r="BN9">
+      <c r="BL9" t="str">
+        <v/>
+      </c>
+      <c r="BM9">
         <v>0.08</v>
+      </c>
+      <c r="BN9" t="str">
+        <v/>
       </c>
       <c r="BO9">
         <v>0.08</v>
       </c>
-      <c r="BP9" t="str">
-        <v/>
-      </c>
-      <c r="BQ9">
+      <c r="BP9">
         <v>0.08</v>
       </c>
-      <c r="BR9" t="str">
-        <v/>
-      </c>
-      <c r="BS9">
+      <c r="BQ9" t="str">
+        <v/>
+      </c>
+      <c r="BR9">
         <v>0.08</v>
+      </c>
+      <c r="BS9" t="str">
+        <v/>
       </c>
       <c r="BT9">
         <v>0.08</v>
@@ -28149,11 +28149,11 @@
       <c r="BU9">
         <v>0.08</v>
       </c>
-      <c r="BV9" t="str">
-        <v/>
-      </c>
-      <c r="BW9">
+      <c r="BV9">
         <v>0.08</v>
+      </c>
+      <c r="BW9" t="str">
+        <v/>
       </c>
       <c r="BX9">
         <v>0.08</v>
@@ -28334,8 +28334,8 @@
       <c r="AY10">
         <v>0</v>
       </c>
-      <c r="AZ10" t="str">
-        <v/>
+      <c r="AZ10">
+        <v>0</v>
       </c>
       <c r="BA10" t="str">
         <v/>
@@ -28343,56 +28343,56 @@
       <c r="BB10" t="str">
         <v/>
       </c>
-      <c r="BC10">
-        <v>0</v>
-      </c>
-      <c r="BD10" t="str">
-        <v/>
-      </c>
-      <c r="BE10">
-        <v>0</v>
-      </c>
-      <c r="BF10" t="str">
-        <v/>
-      </c>
-      <c r="BG10">
-        <v>0</v>
-      </c>
-      <c r="BH10" t="str">
-        <v/>
-      </c>
-      <c r="BI10">
-        <v>0</v>
+      <c r="BC10" t="str">
+        <v/>
+      </c>
+      <c r="BD10">
+        <v>0</v>
+      </c>
+      <c r="BE10" t="str">
+        <v/>
+      </c>
+      <c r="BF10">
+        <v>0</v>
+      </c>
+      <c r="BG10" t="str">
+        <v/>
+      </c>
+      <c r="BH10">
+        <v>0</v>
+      </c>
+      <c r="BI10" t="str">
+        <v/>
       </c>
       <c r="BJ10">
         <v>0</v>
       </c>
-      <c r="BK10" t="str">
-        <v/>
-      </c>
-      <c r="BL10">
-        <v>0</v>
-      </c>
-      <c r="BM10" t="str">
-        <v/>
-      </c>
-      <c r="BN10">
-        <v>0</v>
+      <c r="BK10">
+        <v>0</v>
+      </c>
+      <c r="BL10" t="str">
+        <v/>
+      </c>
+      <c r="BM10">
+        <v>0</v>
+      </c>
+      <c r="BN10" t="str">
+        <v/>
       </c>
       <c r="BO10">
         <v>0</v>
       </c>
-      <c r="BP10" t="str">
-        <v/>
-      </c>
-      <c r="BQ10">
-        <v>0</v>
-      </c>
-      <c r="BR10" t="str">
-        <v/>
-      </c>
-      <c r="BS10">
-        <v>0</v>
+      <c r="BP10">
+        <v>0</v>
+      </c>
+      <c r="BQ10" t="str">
+        <v/>
+      </c>
+      <c r="BR10">
+        <v>0</v>
+      </c>
+      <c r="BS10" t="str">
+        <v/>
       </c>
       <c r="BT10">
         <v>0</v>
@@ -28588,14 +28588,14 @@
       <c r="AZ11">
         <v>0.1</v>
       </c>
-      <c r="BA11" t="str">
-        <v/>
+      <c r="BA11">
+        <v>0.1</v>
       </c>
       <c r="BB11" t="str">
         <v/>
       </c>
-      <c r="BC11">
-        <v>0.1</v>
+      <c r="BC11" t="str">
+        <v/>
       </c>
       <c r="BD11">
         <v>0.1</v>
@@ -28839,14 +28839,14 @@
       <c r="AZ12">
         <v>0</v>
       </c>
-      <c r="BA12" t="str">
-        <v/>
+      <c r="BA12">
+        <v>0</v>
       </c>
       <c r="BB12" t="str">
         <v/>
       </c>
-      <c r="BC12">
-        <v>0</v>
+      <c r="BC12" t="str">
+        <v/>
       </c>
       <c r="BD12">
         <v>0</v>
@@ -29090,14 +29090,14 @@
       <c r="AZ13">
         <v>0.14</v>
       </c>
-      <c r="BA13" t="str">
-        <v/>
+      <c r="BA13">
+        <v>0.14</v>
       </c>
       <c r="BB13" t="str">
         <v/>
       </c>
-      <c r="BC13">
-        <v>0.14</v>
+      <c r="BC13" t="str">
+        <v/>
       </c>
       <c r="BD13">
         <v>0.14</v>
@@ -29341,14 +29341,14 @@
       <c r="AZ14">
         <v>0</v>
       </c>
-      <c r="BA14" t="str">
-        <v/>
+      <c r="BA14">
+        <v>0</v>
       </c>
       <c r="BB14" t="str">
         <v/>
       </c>
-      <c r="BC14">
-        <v>0</v>
+      <c r="BC14" t="str">
+        <v/>
       </c>
       <c r="BD14">
         <v>0</v>
@@ -29544,11 +29544,11 @@
       <c r="AJ15">
         <v>0</v>
       </c>
-      <c r="AK15" t="str">
-        <v/>
-      </c>
-      <c r="AL15">
-        <v>0</v>
+      <c r="AK15">
+        <v>0</v>
+      </c>
+      <c r="AL15" t="str">
+        <v/>
       </c>
       <c r="AM15">
         <v>0</v>
@@ -29592,14 +29592,14 @@
       <c r="AZ15">
         <v>0</v>
       </c>
-      <c r="BA15" t="str">
-        <v/>
+      <c r="BA15">
+        <v>0</v>
       </c>
       <c r="BB15" t="str">
         <v/>
       </c>
-      <c r="BC15">
-        <v>0</v>
+      <c r="BC15" t="str">
+        <v/>
       </c>
       <c r="BD15">
         <v>0</v>
@@ -29655,11 +29655,11 @@
       <c r="BU15">
         <v>0</v>
       </c>
-      <c r="BV15" t="str">
-        <v/>
-      </c>
-      <c r="BW15">
-        <v>0</v>
+      <c r="BV15">
+        <v>0</v>
+      </c>
+      <c r="BW15" t="str">
+        <v/>
       </c>
       <c r="BX15">
         <v>0</v>
@@ -29843,14 +29843,14 @@
       <c r="AZ16">
         <v>0.09</v>
       </c>
-      <c r="BA16" t="str">
-        <v/>
+      <c r="BA16">
+        <v>0.09</v>
       </c>
       <c r="BB16" t="str">
         <v/>
       </c>
-      <c r="BC16">
-        <v>0.09</v>
+      <c r="BC16" t="str">
+        <v/>
       </c>
       <c r="BD16">
         <v>0.09</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update scheduling to better display daily employee visits and improve visit allocation flexibility
Adjusted the capacity dashboard to vertically display daily employee visits and enhanced the scheduling generator to accommodate visits with slightly earlier start times by rounding them to the nearest hour, improving overall allocation efficiency.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -18218,13 +18218,13 @@
         <v>Anderson, Margaret 33333-1.375 (60m)</v>
       </c>
       <c r="AN1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AO1" t="str">
         <v>Office Hours Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AO1" t="str">
+      <c r="AP1" t="str">
         <v>Office Hours Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="AP1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -18245,10 +18245,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AW1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (285m)</v>
-      </c>
-      <c r="AX1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AY1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -18257,13 +18257,13 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BA1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BB1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BC1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BD1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -18272,58 +18272,58 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BF1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BG1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BH1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BI1" t="str">
         <v>Specialised Care Client 09:00-12:00 (420m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BJ1" t="str">
         <v>Specialised Care Client 14:00-17:00 (420m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BK1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BK1" t="str">
+      <c r="BL1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BL1" t="str">
+      <c r="BM1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BM1" t="str">
+      <c r="BN1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BN1" t="str">
+      <c r="BO1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BO1" t="str">
+      <c r="BP1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BP1" t="str">
+      <c r="BQ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BQ1" t="str">
+      <c r="BR1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BR1" t="str">
+      <c r="BS1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (180m)</v>
       </c>
-      <c r="BS1" t="str">
+      <c r="BT1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BT1" t="str">
+      <c r="BU1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BU1" t="str">
+      <c r="BV1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BV1" t="str">
+      <c r="BW1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
-      </c>
-      <c r="BW1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
@@ -18332,58 +18332,58 @@
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="BZ1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="CA1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CA1" t="str">
+      <c r="CB1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="CB1" t="str">
+      <c r="CC1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="CC1" t="str">
+      <c r="CD1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="CD1" t="str">
+      <c r="CE1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="CE1" t="str">
+      <c r="CF1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CF1" t="str">
+      <c r="CG1" t="str">
         <v>Office Hours Client 09:00-12:00 (330m)</v>
       </c>
-      <c r="CG1" t="str">
+      <c r="CH1" t="str">
         <v>Office Hours Client 14:00-17:00 (330m)</v>
       </c>
-      <c r="CH1" t="str">
+      <c r="CI1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CI1" t="str">
+      <c r="CJ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
-      <c r="CJ1" t="str">
+      <c r="CK1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (150m)</v>
-      </c>
-      <c r="CK1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CL1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CM1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CN1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="CO1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+      </c>
+      <c r="CP1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="CP1" t="str">
+      <c r="CQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="CQ1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CR1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -18576,14 +18576,14 @@
       <c r="BG2">
         <v>0.09</v>
       </c>
-      <c r="BH2" t="str">
-        <v/>
+      <c r="BH2">
+        <v>0.09</v>
       </c>
       <c r="BI2" t="str">
         <v/>
       </c>
-      <c r="BJ2">
-        <v>0.09</v>
+      <c r="BJ2" t="str">
+        <v/>
       </c>
       <c r="BK2">
         <v>0.09</v>
@@ -18648,14 +18648,14 @@
       <c r="CE2">
         <v>0.09</v>
       </c>
-      <c r="CF2" t="str">
-        <v/>
+      <c r="CF2">
+        <v>0.09</v>
       </c>
       <c r="CG2" t="str">
         <v/>
       </c>
-      <c r="CH2">
-        <v>0.09</v>
+      <c r="CH2" t="str">
+        <v/>
       </c>
       <c r="CI2">
         <v>0.09</v>
@@ -18875,14 +18875,14 @@
       <c r="BG3">
         <v>0</v>
       </c>
-      <c r="BH3" t="str">
-        <v/>
+      <c r="BH3">
+        <v>0</v>
       </c>
       <c r="BI3" t="str">
         <v/>
       </c>
-      <c r="BJ3">
-        <v>0</v>
+      <c r="BJ3" t="str">
+        <v/>
       </c>
       <c r="BK3">
         <v>0</v>
@@ -18947,14 +18947,14 @@
       <c r="CE3">
         <v>0</v>
       </c>
-      <c r="CF3" t="str">
-        <v/>
+      <c r="CF3">
+        <v>0</v>
       </c>
       <c r="CG3" t="str">
         <v/>
       </c>
-      <c r="CH3">
-        <v>0</v>
+      <c r="CH3" t="str">
+        <v/>
       </c>
       <c r="CI3">
         <v>0</v>
@@ -19117,11 +19117,11 @@
       <c r="AN4">
         <v>0.78</v>
       </c>
-      <c r="AO4" t="str">
-        <v/>
-      </c>
-      <c r="AP4">
+      <c r="AO4">
         <v>0.78</v>
+      </c>
+      <c r="AP4" t="str">
+        <v/>
       </c>
       <c r="AQ4">
         <v>0.78</v>
@@ -19141,11 +19141,11 @@
       <c r="AV4">
         <v>0.78</v>
       </c>
-      <c r="AW4" t="str">
-        <v/>
-      </c>
-      <c r="AX4">
+      <c r="AW4">
         <v>0.78</v>
+      </c>
+      <c r="AX4" t="str">
+        <v/>
       </c>
       <c r="AY4">
         <v>0.78</v>
@@ -19153,14 +19153,14 @@
       <c r="AZ4">
         <v>0.78</v>
       </c>
-      <c r="BA4" t="str">
-        <v/>
+      <c r="BA4">
+        <v>0.78</v>
       </c>
       <c r="BB4" t="str">
         <v/>
       </c>
-      <c r="BC4">
-        <v>0.78</v>
+      <c r="BC4" t="str">
+        <v/>
       </c>
       <c r="BD4">
         <v>0.78</v>
@@ -19171,8 +19171,8 @@
       <c r="BF4">
         <v>0.78</v>
       </c>
-      <c r="BG4" t="str">
-        <v/>
+      <c r="BG4">
+        <v>0.78</v>
       </c>
       <c r="BH4" t="str">
         <v/>
@@ -19180,45 +19180,45 @@
       <c r="BI4" t="str">
         <v/>
       </c>
-      <c r="BJ4">
+      <c r="BJ4" t="str">
+        <v/>
+      </c>
+      <c r="BK4">
         <v>0.78</v>
       </c>
-      <c r="BK4" t="str">
-        <v/>
-      </c>
-      <c r="BL4">
+      <c r="BL4" t="str">
+        <v/>
+      </c>
+      <c r="BM4">
         <v>0.78</v>
       </c>
-      <c r="BM4" t="str">
-        <v/>
-      </c>
-      <c r="BN4">
+      <c r="BN4" t="str">
+        <v/>
+      </c>
+      <c r="BO4">
         <v>0.78</v>
       </c>
-      <c r="BO4" t="str">
-        <v/>
-      </c>
-      <c r="BP4">
+      <c r="BP4" t="str">
+        <v/>
+      </c>
+      <c r="BQ4">
         <v>0.78</v>
       </c>
-      <c r="BQ4" t="str">
-        <v/>
-      </c>
       <c r="BR4" t="str">
         <v/>
       </c>
-      <c r="BS4">
+      <c r="BS4" t="str">
+        <v/>
+      </c>
+      <c r="BT4">
         <v>0.78</v>
       </c>
-      <c r="BT4" t="str">
-        <v/>
-      </c>
-      <c r="BU4">
+      <c r="BU4" t="str">
+        <v/>
+      </c>
+      <c r="BV4">
         <v>0.78</v>
       </c>
-      <c r="BV4" t="str">
-        <v/>
-      </c>
       <c r="BW4" t="str">
         <v/>
       </c>
@@ -19228,59 +19228,59 @@
       <c r="BY4" t="str">
         <v/>
       </c>
-      <c r="BZ4">
-        <v>0.78</v>
+      <c r="BZ4" t="str">
+        <v/>
       </c>
       <c r="CA4">
         <v>0.78</v>
       </c>
-      <c r="CB4" t="str">
-        <v/>
-      </c>
-      <c r="CC4">
+      <c r="CB4">
         <v>0.78</v>
       </c>
-      <c r="CD4" t="str">
-        <v/>
-      </c>
-      <c r="CE4">
+      <c r="CC4" t="str">
+        <v/>
+      </c>
+      <c r="CD4">
         <v>0.78</v>
       </c>
-      <c r="CF4" t="str">
-        <v/>
+      <c r="CE4" t="str">
+        <v/>
+      </c>
+      <c r="CF4">
+        <v>0.78</v>
       </c>
       <c r="CG4" t="str">
         <v/>
       </c>
-      <c r="CH4">
+      <c r="CH4" t="str">
+        <v/>
+      </c>
+      <c r="CI4">
         <v>0.78</v>
       </c>
-      <c r="CI4" t="str">
-        <v/>
-      </c>
       <c r="CJ4" t="str">
         <v/>
       </c>
-      <c r="CK4">
-        <v>0.78</v>
+      <c r="CK4" t="str">
+        <v/>
       </c>
       <c r="CL4">
         <v>0.78</v>
       </c>
-      <c r="CM4" t="str">
-        <v/>
+      <c r="CM4">
+        <v>0.78</v>
       </c>
       <c r="CN4" t="str">
         <v/>
       </c>
-      <c r="CO4">
+      <c r="CO4" t="str">
+        <v/>
+      </c>
+      <c r="CP4">
         <v>0.78</v>
       </c>
-      <c r="CP4" t="str">
-        <v/>
-      </c>
-      <c r="CQ4">
-        <v>0.78</v>
+      <c r="CQ4" t="str">
+        <v/>
       </c>
       <c r="CR4">
         <v>0.78</v>
@@ -19416,11 +19416,11 @@
       <c r="AN5">
         <v>0</v>
       </c>
-      <c r="AO5" t="str">
-        <v/>
-      </c>
-      <c r="AP5">
-        <v>0</v>
+      <c r="AO5">
+        <v>0</v>
+      </c>
+      <c r="AP5" t="str">
+        <v/>
       </c>
       <c r="AQ5">
         <v>0</v>
@@ -19440,11 +19440,11 @@
       <c r="AV5">
         <v>0</v>
       </c>
-      <c r="AW5" t="str">
-        <v/>
-      </c>
-      <c r="AX5">
-        <v>0</v>
+      <c r="AW5">
+        <v>0</v>
+      </c>
+      <c r="AX5" t="str">
+        <v/>
       </c>
       <c r="AY5">
         <v>0</v>
@@ -19470,8 +19470,8 @@
       <c r="BF5">
         <v>0</v>
       </c>
-      <c r="BG5" t="str">
-        <v/>
+      <c r="BG5">
+        <v>0</v>
       </c>
       <c r="BH5" t="str">
         <v/>
@@ -19479,47 +19479,47 @@
       <c r="BI5" t="str">
         <v/>
       </c>
-      <c r="BJ5">
-        <v>0</v>
-      </c>
-      <c r="BK5" t="str">
-        <v/>
-      </c>
-      <c r="BL5">
-        <v>0</v>
-      </c>
-      <c r="BM5" t="str">
-        <v/>
-      </c>
-      <c r="BN5">
-        <v>0</v>
-      </c>
-      <c r="BO5" t="str">
-        <v/>
-      </c>
-      <c r="BP5">
-        <v>0</v>
-      </c>
-      <c r="BQ5" t="str">
-        <v/>
-      </c>
-      <c r="BR5">
-        <v>0</v>
+      <c r="BJ5" t="str">
+        <v/>
+      </c>
+      <c r="BK5">
+        <v>0</v>
+      </c>
+      <c r="BL5" t="str">
+        <v/>
+      </c>
+      <c r="BM5">
+        <v>0</v>
+      </c>
+      <c r="BN5" t="str">
+        <v/>
+      </c>
+      <c r="BO5">
+        <v>0</v>
+      </c>
+      <c r="BP5" t="str">
+        <v/>
+      </c>
+      <c r="BQ5">
+        <v>0</v>
+      </c>
+      <c r="BR5" t="str">
+        <v/>
       </c>
       <c r="BS5">
         <v>0</v>
       </c>
-      <c r="BT5" t="str">
-        <v/>
-      </c>
-      <c r="BU5">
-        <v>0</v>
-      </c>
-      <c r="BV5" t="str">
-        <v/>
-      </c>
-      <c r="BW5">
-        <v>0</v>
+      <c r="BT5">
+        <v>0</v>
+      </c>
+      <c r="BU5" t="str">
+        <v/>
+      </c>
+      <c r="BV5">
+        <v>0</v>
+      </c>
+      <c r="BW5" t="str">
+        <v/>
       </c>
       <c r="BX5">
         <v>0</v>
@@ -19533,32 +19533,32 @@
       <c r="CA5">
         <v>0</v>
       </c>
-      <c r="CB5" t="str">
-        <v/>
-      </c>
-      <c r="CC5">
-        <v>0</v>
-      </c>
-      <c r="CD5" t="str">
-        <v/>
-      </c>
-      <c r="CE5">
-        <v>0</v>
-      </c>
-      <c r="CF5" t="str">
-        <v/>
+      <c r="CB5">
+        <v>0</v>
+      </c>
+      <c r="CC5" t="str">
+        <v/>
+      </c>
+      <c r="CD5">
+        <v>0</v>
+      </c>
+      <c r="CE5" t="str">
+        <v/>
+      </c>
+      <c r="CF5">
+        <v>0</v>
       </c>
       <c r="CG5" t="str">
         <v/>
       </c>
-      <c r="CH5">
-        <v>0</v>
-      </c>
-      <c r="CI5" t="str">
-        <v/>
-      </c>
-      <c r="CJ5">
-        <v>0</v>
+      <c r="CH5" t="str">
+        <v/>
+      </c>
+      <c r="CI5">
+        <v>0</v>
+      </c>
+      <c r="CJ5" t="str">
+        <v/>
       </c>
       <c r="CK5">
         <v>0</v>
@@ -20014,11 +20014,11 @@
       <c r="AN7">
         <v>0</v>
       </c>
-      <c r="AO7" t="str">
-        <v/>
-      </c>
-      <c r="AP7">
-        <v>0</v>
+      <c r="AO7">
+        <v>0</v>
+      </c>
+      <c r="AP7" t="str">
+        <v/>
       </c>
       <c r="AQ7">
         <v>0</v>
@@ -20068,8 +20068,8 @@
       <c r="BF7">
         <v>0</v>
       </c>
-      <c r="BG7" t="str">
-        <v/>
+      <c r="BG7">
+        <v>0</v>
       </c>
       <c r="BH7" t="str">
         <v/>
@@ -20077,47 +20077,47 @@
       <c r="BI7" t="str">
         <v/>
       </c>
-      <c r="BJ7">
-        <v>0</v>
-      </c>
-      <c r="BK7" t="str">
-        <v/>
-      </c>
-      <c r="BL7">
-        <v>0</v>
-      </c>
-      <c r="BM7" t="str">
-        <v/>
-      </c>
-      <c r="BN7">
-        <v>0</v>
-      </c>
-      <c r="BO7" t="str">
-        <v/>
-      </c>
-      <c r="BP7">
-        <v>0</v>
-      </c>
-      <c r="BQ7" t="str">
-        <v/>
-      </c>
-      <c r="BR7">
-        <v>0</v>
+      <c r="BJ7" t="str">
+        <v/>
+      </c>
+      <c r="BK7">
+        <v>0</v>
+      </c>
+      <c r="BL7" t="str">
+        <v/>
+      </c>
+      <c r="BM7">
+        <v>0</v>
+      </c>
+      <c r="BN7" t="str">
+        <v/>
+      </c>
+      <c r="BO7">
+        <v>0</v>
+      </c>
+      <c r="BP7" t="str">
+        <v/>
+      </c>
+      <c r="BQ7">
+        <v>0</v>
+      </c>
+      <c r="BR7" t="str">
+        <v/>
       </c>
       <c r="BS7">
         <v>0</v>
       </c>
-      <c r="BT7" t="str">
-        <v/>
-      </c>
-      <c r="BU7">
-        <v>0</v>
-      </c>
-      <c r="BV7" t="str">
-        <v/>
-      </c>
-      <c r="BW7">
-        <v>0</v>
+      <c r="BT7">
+        <v>0</v>
+      </c>
+      <c r="BU7" t="str">
+        <v/>
+      </c>
+      <c r="BV7">
+        <v>0</v>
+      </c>
+      <c r="BW7" t="str">
+        <v/>
       </c>
       <c r="BX7">
         <v>0</v>
@@ -20131,26 +20131,26 @@
       <c r="CA7">
         <v>0</v>
       </c>
-      <c r="CB7" t="str">
-        <v/>
-      </c>
-      <c r="CC7">
-        <v>0</v>
-      </c>
-      <c r="CD7" t="str">
-        <v/>
-      </c>
-      <c r="CE7">
-        <v>0</v>
-      </c>
-      <c r="CF7" t="str">
-        <v/>
+      <c r="CB7">
+        <v>0</v>
+      </c>
+      <c r="CC7" t="str">
+        <v/>
+      </c>
+      <c r="CD7">
+        <v>0</v>
+      </c>
+      <c r="CE7" t="str">
+        <v/>
+      </c>
+      <c r="CF7">
+        <v>0</v>
       </c>
       <c r="CG7" t="str">
         <v/>
       </c>
-      <c r="CH7">
-        <v>0</v>
+      <c r="CH7" t="str">
+        <v/>
       </c>
       <c r="CI7">
         <v>0</v>
@@ -20370,14 +20370,14 @@
       <c r="BG8">
         <v>0</v>
       </c>
-      <c r="BH8" t="str">
-        <v/>
+      <c r="BH8">
+        <v>0</v>
       </c>
       <c r="BI8" t="str">
         <v/>
       </c>
-      <c r="BJ8">
-        <v>0</v>
+      <c r="BJ8" t="str">
+        <v/>
       </c>
       <c r="BK8">
         <v>0</v>
@@ -20442,14 +20442,14 @@
       <c r="CE8">
         <v>0</v>
       </c>
-      <c r="CF8" t="str">
-        <v/>
+      <c r="CF8">
+        <v>0</v>
       </c>
       <c r="CG8" t="str">
         <v/>
       </c>
-      <c r="CH8">
-        <v>0</v>
+      <c r="CH8" t="str">
+        <v/>
       </c>
       <c r="CI8">
         <v>0</v>
@@ -20612,11 +20612,11 @@
       <c r="AN9">
         <v>0</v>
       </c>
-      <c r="AO9" t="str">
-        <v/>
-      </c>
-      <c r="AP9">
-        <v>0</v>
+      <c r="AO9">
+        <v>0</v>
+      </c>
+      <c r="AP9" t="str">
+        <v/>
       </c>
       <c r="AQ9">
         <v>0</v>
@@ -20666,8 +20666,8 @@
       <c r="BF9">
         <v>0</v>
       </c>
-      <c r="BG9" t="str">
-        <v/>
+      <c r="BG9">
+        <v>0</v>
       </c>
       <c r="BH9" t="str">
         <v/>
@@ -20675,47 +20675,47 @@
       <c r="BI9" t="str">
         <v/>
       </c>
-      <c r="BJ9">
-        <v>0</v>
-      </c>
-      <c r="BK9" t="str">
-        <v/>
-      </c>
-      <c r="BL9">
-        <v>0</v>
-      </c>
-      <c r="BM9" t="str">
-        <v/>
-      </c>
-      <c r="BN9">
-        <v>0</v>
-      </c>
-      <c r="BO9" t="str">
-        <v/>
-      </c>
-      <c r="BP9">
-        <v>0</v>
-      </c>
-      <c r="BQ9" t="str">
-        <v/>
-      </c>
-      <c r="BR9">
-        <v>0</v>
+      <c r="BJ9" t="str">
+        <v/>
+      </c>
+      <c r="BK9">
+        <v>0</v>
+      </c>
+      <c r="BL9" t="str">
+        <v/>
+      </c>
+      <c r="BM9">
+        <v>0</v>
+      </c>
+      <c r="BN9" t="str">
+        <v/>
+      </c>
+      <c r="BO9">
+        <v>0</v>
+      </c>
+      <c r="BP9" t="str">
+        <v/>
+      </c>
+      <c r="BQ9">
+        <v>0</v>
+      </c>
+      <c r="BR9" t="str">
+        <v/>
       </c>
       <c r="BS9">
         <v>0</v>
       </c>
-      <c r="BT9" t="str">
-        <v/>
-      </c>
-      <c r="BU9">
-        <v>0</v>
-      </c>
-      <c r="BV9" t="str">
-        <v/>
-      </c>
-      <c r="BW9">
-        <v>0</v>
+      <c r="BT9">
+        <v>0</v>
+      </c>
+      <c r="BU9" t="str">
+        <v/>
+      </c>
+      <c r="BV9">
+        <v>0</v>
+      </c>
+      <c r="BW9" t="str">
+        <v/>
       </c>
       <c r="BX9">
         <v>0</v>
@@ -20729,26 +20729,26 @@
       <c r="CA9">
         <v>0</v>
       </c>
-      <c r="CB9" t="str">
-        <v/>
-      </c>
-      <c r="CC9">
-        <v>0</v>
-      </c>
-      <c r="CD9" t="str">
-        <v/>
-      </c>
-      <c r="CE9">
-        <v>0</v>
-      </c>
-      <c r="CF9" t="str">
-        <v/>
+      <c r="CB9">
+        <v>0</v>
+      </c>
+      <c r="CC9" t="str">
+        <v/>
+      </c>
+      <c r="CD9">
+        <v>0</v>
+      </c>
+      <c r="CE9" t="str">
+        <v/>
+      </c>
+      <c r="CF9">
+        <v>0</v>
       </c>
       <c r="CG9" t="str">
         <v/>
       </c>
-      <c r="CH9">
-        <v>0</v>
+      <c r="CH9" t="str">
+        <v/>
       </c>
       <c r="CI9">
         <v>0</v>
@@ -20968,14 +20968,14 @@
       <c r="BG10">
         <v>0</v>
       </c>
-      <c r="BH10" t="str">
-        <v/>
+      <c r="BH10">
+        <v>0</v>
       </c>
       <c r="BI10" t="str">
         <v/>
       </c>
-      <c r="BJ10">
-        <v>0</v>
+      <c r="BJ10" t="str">
+        <v/>
       </c>
       <c r="BK10">
         <v>0</v>
@@ -21040,14 +21040,14 @@
       <c r="CE10">
         <v>0</v>
       </c>
-      <c r="CF10" t="str">
-        <v/>
+      <c r="CF10">
+        <v>0</v>
       </c>
       <c r="CG10" t="str">
         <v/>
       </c>
-      <c r="CH10">
-        <v>0</v>
+      <c r="CH10" t="str">
+        <v/>
       </c>
       <c r="CI10">
         <v>0</v>
@@ -21267,14 +21267,14 @@
       <c r="BG11">
         <v>0</v>
       </c>
-      <c r="BH11" t="str">
-        <v/>
+      <c r="BH11">
+        <v>0</v>
       </c>
       <c r="BI11" t="str">
         <v/>
       </c>
-      <c r="BJ11">
-        <v>0</v>
+      <c r="BJ11" t="str">
+        <v/>
       </c>
       <c r="BK11">
         <v>0</v>
@@ -21339,14 +21339,14 @@
       <c r="CE11">
         <v>0</v>
       </c>
-      <c r="CF11" t="str">
-        <v/>
+      <c r="CF11">
+        <v>0</v>
       </c>
       <c r="CG11" t="str">
         <v/>
       </c>
-      <c r="CH11">
-        <v>0</v>
+      <c r="CH11" t="str">
+        <v/>
       </c>
       <c r="CI11">
         <v>0</v>
@@ -21566,14 +21566,14 @@
       <c r="BG12">
         <v>0</v>
       </c>
-      <c r="BH12" t="str">
-        <v/>
+      <c r="BH12">
+        <v>0</v>
       </c>
       <c r="BI12" t="str">
         <v/>
       </c>
-      <c r="BJ12">
-        <v>0</v>
+      <c r="BJ12" t="str">
+        <v/>
       </c>
       <c r="BK12">
         <v>0</v>
@@ -21638,14 +21638,14 @@
       <c r="CE12">
         <v>0</v>
       </c>
-      <c r="CF12" t="str">
-        <v/>
+      <c r="CF12">
+        <v>0</v>
       </c>
       <c r="CG12" t="str">
         <v/>
       </c>
-      <c r="CH12">
-        <v>0</v>
+      <c r="CH12" t="str">
+        <v/>
       </c>
       <c r="CI12">
         <v>0</v>
@@ -21832,11 +21832,11 @@
       <c r="AV13">
         <v>0</v>
       </c>
-      <c r="AW13" t="str">
-        <v/>
-      </c>
-      <c r="AX13">
-        <v>0</v>
+      <c r="AW13">
+        <v>0</v>
+      </c>
+      <c r="AX13" t="str">
+        <v/>
       </c>
       <c r="AY13">
         <v>0</v>
@@ -21865,14 +21865,14 @@
       <c r="BG13">
         <v>0</v>
       </c>
-      <c r="BH13" t="str">
-        <v/>
+      <c r="BH13">
+        <v>0</v>
       </c>
       <c r="BI13" t="str">
         <v/>
       </c>
-      <c r="BJ13">
-        <v>0</v>
+      <c r="BJ13" t="str">
+        <v/>
       </c>
       <c r="BK13">
         <v>0</v>
@@ -21937,20 +21937,20 @@
       <c r="CE13">
         <v>0</v>
       </c>
-      <c r="CF13" t="str">
-        <v/>
+      <c r="CF13">
+        <v>0</v>
       </c>
       <c r="CG13" t="str">
         <v/>
       </c>
-      <c r="CH13">
-        <v>0</v>
-      </c>
-      <c r="CI13" t="str">
-        <v/>
-      </c>
-      <c r="CJ13">
-        <v>0</v>
+      <c r="CH13" t="str">
+        <v/>
+      </c>
+      <c r="CI13">
+        <v>0</v>
+      </c>
+      <c r="CJ13" t="str">
+        <v/>
       </c>
       <c r="CK13">
         <v>0</v>
@@ -22104,11 +22104,11 @@
       <c r="AM14">
         <v>0.81</v>
       </c>
-      <c r="AN14" t="str">
-        <v/>
-      </c>
-      <c r="AO14">
+      <c r="AN14">
         <v>0.16</v>
+      </c>
+      <c r="AO14" t="str">
+        <v/>
       </c>
       <c r="AP14">
         <v>0.16</v>
@@ -22131,11 +22131,11 @@
       <c r="AV14">
         <v>0.16</v>
       </c>
-      <c r="AW14" t="str">
-        <v/>
-      </c>
-      <c r="AX14">
+      <c r="AW14">
         <v>0.16</v>
+      </c>
+      <c r="AX14" t="str">
+        <v/>
       </c>
       <c r="AY14">
         <v>0.16</v>
@@ -22143,14 +22143,14 @@
       <c r="AZ14">
         <v>0.16</v>
       </c>
-      <c r="BA14" t="str">
-        <v/>
+      <c r="BA14">
+        <v>0.16</v>
       </c>
       <c r="BB14" t="str">
         <v/>
       </c>
-      <c r="BC14">
-        <v>0.16</v>
+      <c r="BC14" t="str">
+        <v/>
       </c>
       <c r="BD14">
         <v>0.16</v>
@@ -22158,14 +22158,14 @@
       <c r="BE14">
         <v>0.16</v>
       </c>
-      <c r="BF14" t="str">
-        <v/>
-      </c>
-      <c r="BG14">
+      <c r="BF14">
         <v>0.16</v>
       </c>
-      <c r="BH14" t="str">
-        <v/>
+      <c r="BG14" t="str">
+        <v/>
+      </c>
+      <c r="BH14">
+        <v>0.16</v>
       </c>
       <c r="BI14" t="str">
         <v/>
@@ -22173,104 +22173,104 @@
       <c r="BJ14" t="str">
         <v/>
       </c>
-      <c r="BK14">
+      <c r="BK14" t="str">
+        <v/>
+      </c>
+      <c r="BL14">
         <v>0.16</v>
       </c>
-      <c r="BL14" t="str">
-        <v/>
-      </c>
-      <c r="BM14">
+      <c r="BM14" t="str">
+        <v/>
+      </c>
+      <c r="BN14">
         <v>0.16</v>
       </c>
-      <c r="BN14" t="str">
-        <v/>
-      </c>
-      <c r="BO14">
+      <c r="BO14" t="str">
+        <v/>
+      </c>
+      <c r="BP14">
         <v>0.16</v>
       </c>
-      <c r="BP14" t="str">
-        <v/>
-      </c>
-      <c r="BQ14">
+      <c r="BQ14" t="str">
+        <v/>
+      </c>
+      <c r="BR14">
         <v>0.16</v>
       </c>
-      <c r="BR14" t="str">
-        <v/>
-      </c>
       <c r="BS14" t="str">
         <v/>
       </c>
-      <c r="BT14">
+      <c r="BT14" t="str">
+        <v/>
+      </c>
+      <c r="BU14">
         <v>0.16</v>
       </c>
-      <c r="BU14" t="str">
-        <v/>
-      </c>
-      <c r="BV14">
+      <c r="BV14" t="str">
+        <v/>
+      </c>
+      <c r="BW14">
         <v>0.16</v>
       </c>
-      <c r="BW14" t="str">
-        <v/>
-      </c>
       <c r="BX14" t="str">
         <v/>
       </c>
       <c r="BY14" t="str">
         <v/>
       </c>
-      <c r="BZ14">
+      <c r="BZ14" t="str">
+        <v/>
+      </c>
+      <c r="CA14">
         <v>0.16</v>
       </c>
-      <c r="CA14" t="str">
-        <v/>
-      </c>
-      <c r="CB14">
+      <c r="CB14" t="str">
+        <v/>
+      </c>
+      <c r="CC14">
         <v>0.16</v>
       </c>
-      <c r="CC14" t="str">
-        <v/>
-      </c>
-      <c r="CD14">
-        <v>0.16</v>
+      <c r="CD14" t="str">
+        <v/>
       </c>
       <c r="CE14">
         <v>0.16</v>
       </c>
-      <c r="CF14" t="str">
-        <v/>
+      <c r="CF14">
+        <v>0.16</v>
       </c>
       <c r="CG14" t="str">
         <v/>
       </c>
-      <c r="CH14">
+      <c r="CH14" t="str">
+        <v/>
+      </c>
+      <c r="CI14">
         <v>0.16</v>
       </c>
-      <c r="CI14" t="str">
-        <v/>
-      </c>
       <c r="CJ14" t="str">
         <v/>
       </c>
-      <c r="CK14">
-        <v>0.16</v>
+      <c r="CK14" t="str">
+        <v/>
       </c>
       <c r="CL14">
         <v>0.16</v>
       </c>
-      <c r="CM14" t="str">
-        <v/>
+      <c r="CM14">
+        <v>0.16</v>
       </c>
       <c r="CN14" t="str">
         <v/>
       </c>
-      <c r="CO14">
+      <c r="CO14" t="str">
+        <v/>
+      </c>
+      <c r="CP14">
         <v>0.16</v>
       </c>
-      <c r="CP14" t="str">
-        <v/>
-      </c>
-      <c r="CQ14">
-        <v>0.16</v>
+      <c r="CQ14" t="str">
+        <v/>
       </c>
       <c r="CR14">
         <v>0.16</v>
@@ -22409,19 +22409,19 @@
         <v>Brown, Christine 59375-66667 (60m)</v>
       </c>
       <c r="AL1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AM1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AN1" t="str">
         <v>Office Hours Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="AM1" t="str">
+      <c r="AO1" t="str">
         <v>Office Hours Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="AN1" t="str">
+      <c r="AP1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="AO1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="AP1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AQ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -22436,49 +22436,49 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AU1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AW1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="AX1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AY1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="AZ1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BA1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BB1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
-      </c>
-      <c r="BA1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BB1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BC1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BD1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BE1" t="str">
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+      </c>
+      <c r="BF1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BG1" t="str">
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BH1" t="str">
         <v>Specialised Care Client 09:00-12:00 (420m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BI1" t="str">
         <v>Specialised Care Client 14:00-17:00 (420m)</v>
-      </c>
-      <c r="BH1" t="str">
-        <v>Specialised Care Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="BI1" t="str">
-        <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BJ1" t="str">
         <v>Specialised Care Client 09:00-12:00 (60m)</v>
@@ -22499,31 +22499,31 @@
         <v>Specialised Care Client 14:00-17:00 (60m)</v>
       </c>
       <c r="BP1" t="str">
+        <v>Specialised Care Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="BQ1" t="str">
+        <v>Specialised Care Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="BR1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
-      <c r="BQ1" t="str">
+      <c r="BS1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
       </c>
-      <c r="BR1" t="str">
+      <c r="BT1" t="str">
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
-      <c r="BS1" t="str">
+      <c r="BU1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (180m)</v>
-      </c>
-      <c r="BT1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="BU1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BV1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BW1" t="str">
-        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BX1" t="str">
-        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="BY1" t="str">
         <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
@@ -22532,19 +22532,19 @@
         <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
       </c>
       <c r="CA1" t="str">
+        <v>Multiple Care (Primary) Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="CB1" t="str">
+        <v>Multiple Care (Primary) Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="CC1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="CB1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="CC1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="CD1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CE1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (285m)</v>
       </c>
       <c r="CF1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -22556,7 +22556,7 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="CI1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
       <c r="CJ1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -22746,17 +22746,17 @@
       <c r="BE2">
         <v>0.16</v>
       </c>
-      <c r="BF2" t="str">
-        <v/>
-      </c>
-      <c r="BG2" t="str">
-        <v/>
-      </c>
-      <c r="BH2">
+      <c r="BF2">
         <v>0.16</v>
       </c>
-      <c r="BI2">
+      <c r="BG2">
         <v>0.16</v>
+      </c>
+      <c r="BH2" t="str">
+        <v/>
+      </c>
+      <c r="BI2" t="str">
+        <v/>
       </c>
       <c r="BJ2">
         <v>0.16</v>
@@ -23024,17 +23024,17 @@
       <c r="BE3">
         <v>0</v>
       </c>
-      <c r="BF3" t="str">
-        <v/>
-      </c>
-      <c r="BG3" t="str">
-        <v/>
-      </c>
-      <c r="BH3">
-        <v>0</v>
-      </c>
-      <c r="BI3">
-        <v>0</v>
+      <c r="BF3">
+        <v>0</v>
+      </c>
+      <c r="BG3">
+        <v>0</v>
+      </c>
+      <c r="BH3" t="str">
+        <v/>
+      </c>
+      <c r="BI3" t="str">
+        <v/>
       </c>
       <c r="BJ3">
         <v>0</v>
@@ -23302,17 +23302,17 @@
       <c r="BE4">
         <v>0</v>
       </c>
-      <c r="BF4" t="str">
-        <v/>
-      </c>
-      <c r="BG4" t="str">
-        <v/>
-      </c>
-      <c r="BH4">
-        <v>0</v>
-      </c>
-      <c r="BI4">
-        <v>0</v>
+      <c r="BF4">
+        <v>0</v>
+      </c>
+      <c r="BG4">
+        <v>0</v>
+      </c>
+      <c r="BH4" t="str">
+        <v/>
+      </c>
+      <c r="BI4" t="str">
+        <v/>
       </c>
       <c r="BJ4">
         <v>0</v>
@@ -23523,14 +23523,14 @@
       <c r="AL5">
         <v>0</v>
       </c>
-      <c r="AM5" t="str">
-        <v/>
+      <c r="AM5">
+        <v>0</v>
       </c>
       <c r="AN5">
         <v>0</v>
       </c>
-      <c r="AO5">
-        <v>0</v>
+      <c r="AO5" t="str">
+        <v/>
       </c>
       <c r="AP5">
         <v>0</v>
@@ -23547,14 +23547,14 @@
       <c r="AT5">
         <v>0</v>
       </c>
-      <c r="AU5" t="str">
-        <v/>
+      <c r="AU5">
+        <v>0</v>
       </c>
       <c r="AV5">
         <v>0</v>
       </c>
-      <c r="AW5">
-        <v>0</v>
+      <c r="AW5" t="str">
+        <v/>
       </c>
       <c r="AX5">
         <v>0</v>
@@ -23577,17 +23577,17 @@
       <c r="BD5">
         <v>0</v>
       </c>
-      <c r="BE5" t="str">
-        <v/>
-      </c>
-      <c r="BF5" t="str">
-        <v/>
+      <c r="BE5">
+        <v>0</v>
+      </c>
+      <c r="BF5">
+        <v>0</v>
       </c>
       <c r="BG5" t="str">
         <v/>
       </c>
-      <c r="BH5">
-        <v>0</v>
+      <c r="BH5" t="str">
+        <v/>
       </c>
       <c r="BI5" t="str">
         <v/>
@@ -23613,17 +23613,17 @@
       <c r="BP5">
         <v>0</v>
       </c>
-      <c r="BQ5">
-        <v>0</v>
-      </c>
-      <c r="BR5" t="str">
-        <v/>
+      <c r="BQ5" t="str">
+        <v/>
+      </c>
+      <c r="BR5">
+        <v>0</v>
       </c>
       <c r="BS5">
         <v>0</v>
       </c>
-      <c r="BT5">
-        <v>0</v>
+      <c r="BT5" t="str">
+        <v/>
       </c>
       <c r="BU5">
         <v>0</v>
@@ -23634,8 +23634,8 @@
       <c r="BW5">
         <v>0</v>
       </c>
-      <c r="BX5" t="str">
-        <v/>
+      <c r="BX5">
+        <v>0</v>
       </c>
       <c r="BY5">
         <v>0</v>
@@ -23646,17 +23646,17 @@
       <c r="CA5">
         <v>0</v>
       </c>
-      <c r="CB5">
-        <v>0</v>
-      </c>
-      <c r="CC5" t="str">
-        <v/>
+      <c r="CB5" t="str">
+        <v/>
+      </c>
+      <c r="CC5">
+        <v>0</v>
       </c>
       <c r="CD5">
         <v>0</v>
       </c>
-      <c r="CE5">
-        <v>0</v>
+      <c r="CE5" t="str">
+        <v/>
       </c>
       <c r="CF5">
         <v>0</v>
@@ -24079,14 +24079,14 @@
       <c r="AL7">
         <v>0.05</v>
       </c>
-      <c r="AM7" t="str">
-        <v/>
+      <c r="AM7">
+        <v>0.05</v>
       </c>
       <c r="AN7">
         <v>0.05</v>
       </c>
-      <c r="AO7">
-        <v>0.05</v>
+      <c r="AO7" t="str">
+        <v/>
       </c>
       <c r="AP7">
         <v>0.05</v>
@@ -24103,14 +24103,14 @@
       <c r="AT7">
         <v>0.05</v>
       </c>
-      <c r="AU7" t="str">
-        <v/>
+      <c r="AU7">
+        <v>0.05</v>
       </c>
       <c r="AV7">
         <v>0.05</v>
       </c>
-      <c r="AW7">
-        <v>0.05</v>
+      <c r="AW7" t="str">
+        <v/>
       </c>
       <c r="AX7">
         <v>0.05</v>
@@ -24133,17 +24133,17 @@
       <c r="BD7">
         <v>0.05</v>
       </c>
-      <c r="BE7" t="str">
-        <v/>
-      </c>
-      <c r="BF7" t="str">
-        <v/>
+      <c r="BE7">
+        <v>0.05</v>
+      </c>
+      <c r="BF7">
+        <v>0.05</v>
       </c>
       <c r="BG7" t="str">
         <v/>
       </c>
-      <c r="BH7">
-        <v>0.05</v>
+      <c r="BH7" t="str">
+        <v/>
       </c>
       <c r="BI7" t="str">
         <v/>
@@ -24169,20 +24169,20 @@
       <c r="BP7">
         <v>0.05</v>
       </c>
-      <c r="BQ7">
+      <c r="BQ7" t="str">
+        <v/>
+      </c>
+      <c r="BR7">
         <v>0.05</v>
       </c>
-      <c r="BR7" t="str">
-        <v/>
-      </c>
-      <c r="BS7" t="str">
-        <v/>
-      </c>
-      <c r="BT7">
+      <c r="BS7">
         <v>0.05</v>
       </c>
-      <c r="BU7">
-        <v>0.05</v>
+      <c r="BT7" t="str">
+        <v/>
+      </c>
+      <c r="BU7" t="str">
+        <v/>
       </c>
       <c r="BV7">
         <v>0.05</v>
@@ -24190,8 +24190,8 @@
       <c r="BW7">
         <v>0.05</v>
       </c>
-      <c r="BX7" t="str">
-        <v/>
+      <c r="BX7">
+        <v>0.05</v>
       </c>
       <c r="BY7">
         <v>0.05</v>
@@ -24202,17 +24202,17 @@
       <c r="CA7">
         <v>0.05</v>
       </c>
-      <c r="CB7">
+      <c r="CB7" t="str">
+        <v/>
+      </c>
+      <c r="CC7">
         <v>0.05</v>
-      </c>
-      <c r="CC7" t="str">
-        <v/>
       </c>
       <c r="CD7">
         <v>0.05</v>
       </c>
-      <c r="CE7">
-        <v>0.05</v>
+      <c r="CE7" t="str">
+        <v/>
       </c>
       <c r="CF7">
         <v>0.05</v>
@@ -24357,14 +24357,14 @@
       <c r="AL8">
         <v>0.08</v>
       </c>
-      <c r="AM8" t="str">
-        <v/>
+      <c r="AM8">
+        <v>0.08</v>
       </c>
       <c r="AN8">
         <v>0.08</v>
       </c>
-      <c r="AO8">
-        <v>0.08</v>
+      <c r="AO8" t="str">
+        <v/>
       </c>
       <c r="AP8">
         <v>0.08</v>
@@ -24381,14 +24381,14 @@
       <c r="AT8">
         <v>0.08</v>
       </c>
-      <c r="AU8" t="str">
-        <v/>
+      <c r="AU8">
+        <v>0.08</v>
       </c>
       <c r="AV8">
         <v>0.08</v>
       </c>
-      <c r="AW8">
-        <v>0.08</v>
+      <c r="AW8" t="str">
+        <v/>
       </c>
       <c r="AX8">
         <v>0.08</v>
@@ -24411,17 +24411,17 @@
       <c r="BD8">
         <v>0.08</v>
       </c>
-      <c r="BE8" t="str">
-        <v/>
-      </c>
-      <c r="BF8" t="str">
-        <v/>
+      <c r="BE8">
+        <v>0.08</v>
+      </c>
+      <c r="BF8">
+        <v>0.08</v>
       </c>
       <c r="BG8" t="str">
         <v/>
       </c>
-      <c r="BH8">
-        <v>0.08</v>
+      <c r="BH8" t="str">
+        <v/>
       </c>
       <c r="BI8" t="str">
         <v/>
@@ -24447,17 +24447,17 @@
       <c r="BP8">
         <v>0.08</v>
       </c>
-      <c r="BQ8">
+      <c r="BQ8" t="str">
+        <v/>
+      </c>
+      <c r="BR8">
         <v>0.08</v>
-      </c>
-      <c r="BR8" t="str">
-        <v/>
       </c>
       <c r="BS8">
         <v>0.08</v>
       </c>
-      <c r="BT8">
-        <v>0.08</v>
+      <c r="BT8" t="str">
+        <v/>
       </c>
       <c r="BU8">
         <v>0.08</v>
@@ -24468,8 +24468,8 @@
       <c r="BW8">
         <v>0.08</v>
       </c>
-      <c r="BX8" t="str">
-        <v/>
+      <c r="BX8">
+        <v>0.08</v>
       </c>
       <c r="BY8">
         <v>0.08</v>
@@ -24480,17 +24480,17 @@
       <c r="CA8">
         <v>0.08</v>
       </c>
-      <c r="CB8">
+      <c r="CB8" t="str">
+        <v/>
+      </c>
+      <c r="CC8">
         <v>0.08</v>
-      </c>
-      <c r="CC8" t="str">
-        <v/>
       </c>
       <c r="CD8">
         <v>0.08</v>
       </c>
-      <c r="CE8">
-        <v>0.08</v>
+      <c r="CE8" t="str">
+        <v/>
       </c>
       <c r="CF8">
         <v>0.08</v>
@@ -24635,14 +24635,14 @@
       <c r="AL9">
         <v>0</v>
       </c>
-      <c r="AM9" t="str">
-        <v/>
+      <c r="AM9">
+        <v>0</v>
       </c>
       <c r="AN9">
         <v>0</v>
       </c>
-      <c r="AO9">
-        <v>0</v>
+      <c r="AO9" t="str">
+        <v/>
       </c>
       <c r="AP9">
         <v>0</v>
@@ -24689,17 +24689,17 @@
       <c r="BD9">
         <v>0</v>
       </c>
-      <c r="BE9" t="str">
-        <v/>
-      </c>
-      <c r="BF9" t="str">
-        <v/>
+      <c r="BE9">
+        <v>0</v>
+      </c>
+      <c r="BF9">
+        <v>0</v>
       </c>
       <c r="BG9" t="str">
         <v/>
       </c>
-      <c r="BH9">
-        <v>0</v>
+      <c r="BH9" t="str">
+        <v/>
       </c>
       <c r="BI9" t="str">
         <v/>
@@ -24725,17 +24725,17 @@
       <c r="BP9">
         <v>0</v>
       </c>
-      <c r="BQ9">
-        <v>0</v>
-      </c>
-      <c r="BR9" t="str">
-        <v/>
+      <c r="BQ9" t="str">
+        <v/>
+      </c>
+      <c r="BR9">
+        <v>0</v>
       </c>
       <c r="BS9">
         <v>0</v>
       </c>
-      <c r="BT9">
-        <v>0</v>
+      <c r="BT9" t="str">
+        <v/>
       </c>
       <c r="BU9">
         <v>0</v>
@@ -24746,8 +24746,8 @@
       <c r="BW9">
         <v>0</v>
       </c>
-      <c r="BX9" t="str">
-        <v/>
+      <c r="BX9">
+        <v>0</v>
       </c>
       <c r="BY9">
         <v>0</v>
@@ -24758,8 +24758,8 @@
       <c r="CA9">
         <v>0</v>
       </c>
-      <c r="CB9">
-        <v>0</v>
+      <c r="CB9" t="str">
+        <v/>
       </c>
       <c r="CC9">
         <v>0</v>
@@ -24970,17 +24970,17 @@
       <c r="BE10">
         <v>0.1</v>
       </c>
-      <c r="BF10" t="str">
-        <v/>
-      </c>
-      <c r="BG10" t="str">
-        <v/>
-      </c>
-      <c r="BH10">
+      <c r="BF10">
         <v>0.1</v>
       </c>
-      <c r="BI10">
+      <c r="BG10">
         <v>0.1</v>
+      </c>
+      <c r="BH10" t="str">
+        <v/>
+      </c>
+      <c r="BI10" t="str">
+        <v/>
       </c>
       <c r="BJ10">
         <v>0.1</v>
@@ -25248,17 +25248,17 @@
       <c r="BE11">
         <v>0.01</v>
       </c>
-      <c r="BF11" t="str">
-        <v/>
-      </c>
-      <c r="BG11" t="str">
-        <v/>
-      </c>
-      <c r="BH11">
+      <c r="BF11">
         <v>0.01</v>
       </c>
-      <c r="BI11">
+      <c r="BG11">
         <v>0.01</v>
+      </c>
+      <c r="BH11" t="str">
+        <v/>
+      </c>
+      <c r="BI11" t="str">
+        <v/>
       </c>
       <c r="BJ11">
         <v>0.01</v>
@@ -25526,17 +25526,17 @@
       <c r="BE12">
         <v>0</v>
       </c>
-      <c r="BF12" t="str">
-        <v/>
-      </c>
-      <c r="BG12" t="str">
-        <v/>
-      </c>
-      <c r="BH12">
-        <v>0</v>
-      </c>
-      <c r="BI12">
-        <v>0</v>
+      <c r="BF12">
+        <v>0</v>
+      </c>
+      <c r="BG12">
+        <v>0</v>
+      </c>
+      <c r="BH12" t="str">
+        <v/>
+      </c>
+      <c r="BI12" t="str">
+        <v/>
       </c>
       <c r="BJ12">
         <v>0</v>
@@ -25804,17 +25804,17 @@
       <c r="BE13">
         <v>0</v>
       </c>
-      <c r="BF13" t="str">
-        <v/>
-      </c>
-      <c r="BG13" t="str">
-        <v/>
-      </c>
-      <c r="BH13">
-        <v>0</v>
-      </c>
-      <c r="BI13">
-        <v>0</v>
+      <c r="BF13">
+        <v>0</v>
+      </c>
+      <c r="BG13">
+        <v>0</v>
+      </c>
+      <c r="BH13" t="str">
+        <v/>
+      </c>
+      <c r="BI13" t="str">
+        <v/>
       </c>
       <c r="BJ13">
         <v>0</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Organize the weekly plan to show employees and visits more efficiently
Update the UI layout for the weekly plan to display employees on the side and unallocated visits horizontally at the bottom, improving scannability and reducing vertical scrolling.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -3744,7 +3744,7 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AV1" t="str">
-        <v>Lynch (NL), Roselyn 66667-33333 (60m)</v>
+        <v>Brown, Christine 33333-.6875 (60m)</v>
       </c>
       <c r="AW1" t="str">
         <v>Lynch (NL), Roselyn 66667-33333 (60m)</v>
@@ -3753,79 +3753,79 @@
         <v>Lynch (NL), Roselyn 66667-33333 (60m)</v>
       </c>
       <c r="AY1" t="str">
+        <v>Lynch (NL), Roselyn 66667-33333 (60m)</v>
+      </c>
+      <c r="AZ1" t="str">
         <v>Murray (NL), James 34.75-66667 (60m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BA1" t="str">
         <v>Campbell, Neil 33333-84375 (60m)</v>
       </c>
-      <c r="BA1" t="str">
+      <c r="BB1" t="str">
         <v>Campbell, Neil 66667-4.625 (120m)</v>
       </c>
-      <c r="BB1" t="str">
+      <c r="BC1" t="str">
         <v>O'Brien (NL), Josephine 66667-33333 (60m)</v>
       </c>
-      <c r="BC1" t="str">
+      <c r="BD1" t="str">
         <v>O'Brien (NL), Josephine 34.75-66667 (60m)</v>
       </c>
-      <c r="BD1" t="str">
+      <c r="BE1" t="str">
         <v>O'Brien (NL), Josephine .4375-66667 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BF1" t="str">
         <v>Barrons (NL/HCAH), Shirley 33333-4.375 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BG1" t="str">
         <v>Barrons (NL/HCAH), Shirley 66667-33333 (60m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BH1" t="str">
         <v>Barrons (NL/HCAH), Shirley 33333-84375 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BI1" t="str">
         <v>Munro (NL), Alistair 66667-33333 (60m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BJ1" t="str">
         <v>Docherty (NL), Elizabeth .4375-66667 (60m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BK1" t="str">
         <v>Mullen (NL), Eileen 59375-66667 (60m)</v>
       </c>
-      <c r="BK1" t="str">
+      <c r="BL1" t="str">
         <v>Mullen (NL), Eileen 34.75-66667 (60m)</v>
       </c>
-      <c r="BL1" t="str">
+      <c r="BM1" t="str">
         <v>McIntyre (NL), Donald 66667-33333 (60m)</v>
       </c>
-      <c r="BM1" t="str">
+      <c r="BN1" t="str">
         <v>Robertson (NL), Doreen 66667-78125 (120m)</v>
       </c>
-      <c r="BN1" t="str">
+      <c r="BO1" t="str">
         <v>Kennedy (NL), Roberta 33333-53125 (60m)</v>
       </c>
-      <c r="BO1" t="str">
+      <c r="BP1" t="str">
         <v>Morris, Jack 66667-33333 (60m)</v>
       </c>
-      <c r="BP1" t="str">
+      <c r="BQ1" t="str">
         <v>Collie, Mattie 59375-66667 (60m)</v>
       </c>
-      <c r="BQ1" t="str">
+      <c r="BR1" t="str">
         <v>Goldsmith, Astrid 34.75-66667 (60m)</v>
       </c>
-      <c r="BR1" t="str">
+      <c r="BS1" t="str">
         <v>Pedrick, Michael 33333-66667 (120m)</v>
       </c>
-      <c r="BS1" t="str">
+      <c r="BT1" t="str">
         <v>Whyte, Jean 66667-33333 (60m)</v>
       </c>
-      <c r="BT1" t="str">
+      <c r="BU1" t="str">
         <v>Anderson, Margaret 33333-84375 (60m)</v>
       </c>
-      <c r="BU1" t="str">
+      <c r="BV1" t="str">
         <v>Anderson, Margaret 33333-.6875 (60m)</v>
       </c>
-      <c r="BV1" t="str">
+      <c r="BW1" t="str">
         <v>Anderson, Margaret 33333-4.375 (60m)</v>
-      </c>
-      <c r="BW1" t="str">
-        <v>Brown, Christine 33333-.6875 (60m)</v>
       </c>
     </row>
     <row r="2">
@@ -3971,7 +3971,7 @@
         <v>0</v>
       </c>
       <c r="AV2">
-        <v>0.81</v>
+        <v>0.77</v>
       </c>
       <c r="AW2">
         <v>0.81</v>
@@ -3980,16 +3980,16 @@
         <v>0.81</v>
       </c>
       <c r="AY2">
+        <v>0.81</v>
+      </c>
+      <c r="AZ2">
         <v>0.7</v>
-      </c>
-      <c r="AZ2">
-        <v>0.79</v>
       </c>
       <c r="BA2">
         <v>0.79</v>
       </c>
       <c r="BB2">
-        <v>0.68</v>
+        <v>0.79</v>
       </c>
       <c r="BC2">
         <v>0.68</v>
@@ -3998,7 +3998,7 @@
         <v>0.68</v>
       </c>
       <c r="BE2">
-        <v>0.72</v>
+        <v>0.68</v>
       </c>
       <c r="BF2">
         <v>0.72</v>
@@ -4007,43 +4007,43 @@
         <v>0.72</v>
       </c>
       <c r="BH2">
+        <v>0.72</v>
+      </c>
+      <c r="BI2">
         <v>0.68</v>
       </c>
-      <c r="BI2">
+      <c r="BJ2">
         <v>0.81</v>
-      </c>
-      <c r="BJ2">
-        <v>0.99</v>
       </c>
       <c r="BK2">
         <v>0.99</v>
       </c>
       <c r="BL2">
+        <v>0.99</v>
+      </c>
+      <c r="BM2">
         <v>0.68</v>
       </c>
-      <c r="BM2">
+      <c r="BN2">
         <v>0.74</v>
       </c>
-      <c r="BN2">
+      <c r="BO2">
         <v>0.92</v>
       </c>
-      <c r="BO2">
+      <c r="BP2">
         <v>0.7</v>
       </c>
-      <c r="BP2">
+      <c r="BQ2">
         <v>1.08</v>
       </c>
-      <c r="BQ2">
+      <c r="BR2">
         <v>0.83</v>
       </c>
-      <c r="BR2">
+      <c r="BS2">
         <v>0.88</v>
       </c>
-      <c r="BS2">
+      <c r="BT2">
         <v>1.01</v>
-      </c>
-      <c r="BT2">
-        <v>0.74</v>
       </c>
       <c r="BU2">
         <v>0.74</v>
@@ -4052,7 +4052,7 @@
         <v>0.74</v>
       </c>
       <c r="BW2">
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="3">
@@ -4198,7 +4198,7 @@
         <v>0.14</v>
       </c>
       <c r="AV3">
-        <v>0.24</v>
+        <v>0.64</v>
       </c>
       <c r="AW3">
         <v>0.24</v>
@@ -4210,13 +4210,13 @@
         <v>0.24</v>
       </c>
       <c r="AZ3">
-        <v>1.04</v>
+        <v>0.24</v>
       </c>
       <c r="BA3">
         <v>1.04</v>
       </c>
       <c r="BB3">
-        <v>0.24</v>
+        <v>1.04</v>
       </c>
       <c r="BC3">
         <v>0.24</v>
@@ -4237,10 +4237,10 @@
         <v>0.24</v>
       </c>
       <c r="BI3">
+        <v>0.24</v>
+      </c>
+      <c r="BJ3">
         <v>0.89</v>
-      </c>
-      <c r="BJ3">
-        <v>0.24</v>
       </c>
       <c r="BK3">
         <v>0.24</v>
@@ -4249,10 +4249,10 @@
         <v>0.24</v>
       </c>
       <c r="BM3">
+        <v>0.24</v>
+      </c>
+      <c r="BN3">
         <v>0.75</v>
-      </c>
-      <c r="BN3">
-        <v>0.24</v>
       </c>
       <c r="BO3">
         <v>0.24</v>
@@ -4270,7 +4270,7 @@
         <v>0.24</v>
       </c>
       <c r="BT3">
-        <v>0.26</v>
+        <v>0.24</v>
       </c>
       <c r="BU3">
         <v>0.26</v>
@@ -4279,7 +4279,7 @@
         <v>0.26</v>
       </c>
       <c r="BW3">
-        <v>0.64</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="4">
@@ -4425,7 +4425,7 @@
         <v>0.03</v>
       </c>
       <c r="AV4">
-        <v>0.84</v>
+        <v>0.8</v>
       </c>
       <c r="AW4">
         <v>0.84</v>
@@ -4434,16 +4434,16 @@
         <v>0.84</v>
       </c>
       <c r="AY4">
+        <v>0.84</v>
+      </c>
+      <c r="AZ4">
         <v>0.73</v>
-      </c>
-      <c r="AZ4">
-        <v>0.82</v>
       </c>
       <c r="BA4">
         <v>0.82</v>
       </c>
       <c r="BB4">
-        <v>0.66</v>
+        <v>0.82</v>
       </c>
       <c r="BC4">
         <v>0.66</v>
@@ -4452,7 +4452,7 @@
         <v>0.66</v>
       </c>
       <c r="BE4">
-        <v>0.71</v>
+        <v>0.66</v>
       </c>
       <c r="BF4">
         <v>0.71</v>
@@ -4461,43 +4461,43 @@
         <v>0.71</v>
       </c>
       <c r="BH4">
+        <v>0.71</v>
+      </c>
+      <c r="BI4">
         <v>0.66</v>
       </c>
-      <c r="BI4">
+      <c r="BJ4">
         <v>0.82</v>
-      </c>
-      <c r="BJ4">
-        <v>1.04</v>
       </c>
       <c r="BK4">
         <v>1.04</v>
       </c>
       <c r="BL4">
+        <v>1.04</v>
+      </c>
+      <c r="BM4">
         <v>0.66</v>
       </c>
-      <c r="BM4">
+      <c r="BN4">
         <v>0.75</v>
       </c>
-      <c r="BN4">
+      <c r="BO4">
         <v>0.93</v>
       </c>
-      <c r="BO4">
+      <c r="BP4">
         <v>0.71</v>
       </c>
-      <c r="BP4">
+      <c r="BQ4">
         <v>1.11</v>
       </c>
-      <c r="BQ4">
+      <c r="BR4">
         <v>0.82</v>
       </c>
-      <c r="BR4">
+      <c r="BS4">
         <v>0.93</v>
       </c>
-      <c r="BS4">
+      <c r="BT4">
         <v>1.09</v>
-      </c>
-      <c r="BT4">
-        <v>0.75</v>
       </c>
       <c r="BU4">
         <v>0.75</v>
@@ -4506,7 +4506,7 @@
         <v>0.75</v>
       </c>
       <c r="BW4">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="5">
@@ -4652,7 +4652,7 @@
         <v>0</v>
       </c>
       <c r="AV5">
-        <v>0.32</v>
+        <v>0.39</v>
       </c>
       <c r="AW5">
         <v>0.32</v>
@@ -4661,16 +4661,16 @@
         <v>0.32</v>
       </c>
       <c r="AY5">
+        <v>0.32</v>
+      </c>
+      <c r="AZ5">
         <v>0.37</v>
-      </c>
-      <c r="AZ5">
-        <v>0.43</v>
       </c>
       <c r="BA5">
         <v>0.43</v>
       </c>
       <c r="BB5">
-        <v>0.79</v>
+        <v>0.43</v>
       </c>
       <c r="BC5">
         <v>0.79</v>
@@ -4679,7 +4679,7 @@
         <v>0.79</v>
       </c>
       <c r="BE5">
-        <v>0.74</v>
+        <v>0.79</v>
       </c>
       <c r="BF5">
         <v>0.74</v>
@@ -4688,43 +4688,43 @@
         <v>0.74</v>
       </c>
       <c r="BH5">
+        <v>0.74</v>
+      </c>
+      <c r="BI5">
         <v>0.77</v>
       </c>
-      <c r="BI5">
+      <c r="BJ5">
         <v>0.41</v>
-      </c>
-      <c r="BJ5">
-        <v>0.23</v>
       </c>
       <c r="BK5">
         <v>0.23</v>
       </c>
       <c r="BL5">
+        <v>0.23</v>
+      </c>
+      <c r="BM5">
         <v>0.77</v>
       </c>
-      <c r="BM5">
+      <c r="BN5">
         <v>0.43</v>
       </c>
-      <c r="BN5">
+      <c r="BO5">
         <v>0.39</v>
-      </c>
-      <c r="BO5">
-        <v>0.34</v>
       </c>
       <c r="BP5">
         <v>0.34</v>
       </c>
       <c r="BQ5">
+        <v>0.34</v>
+      </c>
+      <c r="BR5">
         <v>0.63</v>
       </c>
-      <c r="BR5">
+      <c r="BS5">
         <v>0.14</v>
       </c>
-      <c r="BS5">
+      <c r="BT5">
         <v>0.28</v>
-      </c>
-      <c r="BT5">
-        <v>0.57</v>
       </c>
       <c r="BU5">
         <v>0.57</v>
@@ -4733,7 +4733,7 @@
         <v>0.57</v>
       </c>
       <c r="BW5">
-        <v>0.39</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="6">
@@ -4879,7 +4879,7 @@
         <v>0</v>
       </c>
       <c r="AV6">
-        <v>0.39</v>
+        <v>0.46</v>
       </c>
       <c r="AW6">
         <v>0.39</v>
@@ -4888,16 +4888,16 @@
         <v>0.39</v>
       </c>
       <c r="AY6">
+        <v>0.39</v>
+      </c>
+      <c r="AZ6">
         <v>0.43</v>
-      </c>
-      <c r="AZ6">
-        <v>0.5</v>
       </c>
       <c r="BA6">
         <v>0.5</v>
       </c>
       <c r="BB6">
-        <v>0.81</v>
+        <v>0.5</v>
       </c>
       <c r="BC6">
         <v>0.81</v>
@@ -4906,7 +4906,7 @@
         <v>0.81</v>
       </c>
       <c r="BE6">
-        <v>0.77</v>
+        <v>0.81</v>
       </c>
       <c r="BF6">
         <v>0.77</v>
@@ -4915,43 +4915,43 @@
         <v>0.77</v>
       </c>
       <c r="BH6">
+        <v>0.77</v>
+      </c>
+      <c r="BI6">
         <v>0.81</v>
       </c>
-      <c r="BI6">
+      <c r="BJ6">
         <v>0.48</v>
-      </c>
-      <c r="BJ6">
-        <v>0.28</v>
       </c>
       <c r="BK6">
         <v>0.28</v>
       </c>
       <c r="BL6">
+        <v>0.28</v>
+      </c>
+      <c r="BM6">
         <v>0.81</v>
       </c>
-      <c r="BM6">
+      <c r="BN6">
         <v>0.52</v>
       </c>
-      <c r="BN6">
+      <c r="BO6">
         <v>0.41</v>
       </c>
-      <c r="BO6">
+      <c r="BP6">
         <v>0.43</v>
       </c>
-      <c r="BP6">
+      <c r="BQ6">
         <v>0.37</v>
       </c>
-      <c r="BQ6">
+      <c r="BR6">
         <v>0.68</v>
       </c>
-      <c r="BR6">
+      <c r="BS6">
         <v>0.17</v>
       </c>
-      <c r="BS6">
+      <c r="BT6">
         <v>0.3</v>
-      </c>
-      <c r="BT6">
-        <v>0.63</v>
       </c>
       <c r="BU6">
         <v>0.63</v>
@@ -4960,7 +4960,7 @@
         <v>0.63</v>
       </c>
       <c r="BW6">
-        <v>0.46</v>
+        <v>0.63</v>
       </c>
     </row>
   </sheetData>
@@ -6617,10 +6617,10 @@
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="AS1" t="str">
+        <v>Brown, Christine 33333-.6875 (60m)</v>
+      </c>
+      <c r="AT1" t="str">
         <v>Clements (NL), Jessie 33333-53125 (60m)</v>
-      </c>
-      <c r="AT1" t="str">
-        <v>Lynch (NL), Roselyn 66667-33333 (60m)</v>
       </c>
       <c r="AU1" t="str">
         <v>Lynch (NL), Roselyn 66667-33333 (60m)</v>
@@ -6629,64 +6629,64 @@
         <v>Lynch (NL), Roselyn 66667-33333 (60m)</v>
       </c>
       <c r="AW1" t="str">
+        <v>Lynch (NL), Roselyn 66667-33333 (60m)</v>
+      </c>
+      <c r="AX1" t="str">
         <v>Murray (NL), James .4375-66667 (60m)</v>
       </c>
-      <c r="AX1" t="str">
+      <c r="AY1" t="str">
         <v>Campbell, Neil 33333-84375 (60m)</v>
       </c>
-      <c r="AY1" t="str">
+      <c r="AZ1" t="str">
         <v>Campbell, Neil 66667-5.625 (120m)</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BA1" t="str">
         <v>O'Brien (NL), Josephine 66667-33333 (60m)</v>
       </c>
-      <c r="BA1" t="str">
+      <c r="BB1" t="str">
         <v>O'Brien (NL), Josephine .4375-66667 (60m)</v>
       </c>
-      <c r="BB1" t="str">
+      <c r="BC1" t="str">
         <v>Barrons (NL/HCAH), Shirley 33333-5.375 (60m)</v>
       </c>
-      <c r="BC1" t="str">
+      <c r="BD1" t="str">
         <v>Barrons (NL/HCAH), Shirley 66667-33333 (60m)</v>
       </c>
-      <c r="BD1" t="str">
+      <c r="BE1" t="str">
         <v>Barrons (NL/HCAH), Shirley 33333-84375 (60m)</v>
       </c>
-      <c r="BE1" t="str">
+      <c r="BF1" t="str">
         <v>Munro (NL), Alistair 66667-33333 (60m)</v>
       </c>
-      <c r="BF1" t="str">
+      <c r="BG1" t="str">
         <v>Docherty (NL), Elizabeth .4375-66667 (60m)</v>
       </c>
-      <c r="BG1" t="str">
+      <c r="BH1" t="str">
         <v>Mullen (NL), Eileen 66667-33333 (60m)</v>
       </c>
-      <c r="BH1" t="str">
+      <c r="BI1" t="str">
         <v>Mullen (NL), Eileen 35.75-66667 (60m)</v>
       </c>
-      <c r="BI1" t="str">
+      <c r="BJ1" t="str">
         <v>McIntyre (NL), Donald 66667-33333 (60m)</v>
       </c>
-      <c r="BJ1" t="str">
+      <c r="BK1" t="str">
         <v>Morris, Jack 66667-33333 (60m)</v>
       </c>
-      <c r="BK1" t="str">
+      <c r="BL1" t="str">
         <v>Collie, Mattie 59375-33333 (120m)</v>
       </c>
-      <c r="BL1" t="str">
+      <c r="BM1" t="str">
         <v>Goldsmith, Astrid 35.75-66667 (60m)</v>
       </c>
-      <c r="BM1" t="str">
+      <c r="BN1" t="str">
         <v>Hannah, Marion 33333-33333 (180m)</v>
       </c>
-      <c r="BN1" t="str">
+      <c r="BO1" t="str">
         <v>Anderson, Margaret 33333-.6875 (60m)</v>
       </c>
-      <c r="BO1" t="str">
+      <c r="BP1" t="str">
         <v>Anderson, Margaret 33333-5.375 (60m)</v>
-      </c>
-      <c r="BP1" t="str">
-        <v>Brown, Christine 33333-.6875 (60m)</v>
       </c>
     </row>
     <row r="2">
@@ -6823,10 +6823,10 @@
         <v>0</v>
       </c>
       <c r="AS2">
+        <v>1.03</v>
+      </c>
+      <c r="AT2">
         <v>0.77</v>
-      </c>
-      <c r="AT2">
-        <v>0.94</v>
       </c>
       <c r="AU2">
         <v>0.94</v>
@@ -6835,22 +6835,22 @@
         <v>0.94</v>
       </c>
       <c r="AW2">
+        <v>0.94</v>
+      </c>
+      <c r="AX2">
         <v>1.01</v>
-      </c>
-      <c r="AX2">
-        <v>1.03</v>
       </c>
       <c r="AY2">
         <v>1.03</v>
       </c>
       <c r="AZ2">
-        <v>0.72</v>
+        <v>1.03</v>
       </c>
       <c r="BA2">
         <v>0.72</v>
       </c>
       <c r="BB2">
-        <v>0.77</v>
+        <v>0.72</v>
       </c>
       <c r="BC2">
         <v>0.77</v>
@@ -6859,40 +6859,40 @@
         <v>0.77</v>
       </c>
       <c r="BE2">
+        <v>0.77</v>
+      </c>
+      <c r="BF2">
         <v>0.72</v>
       </c>
-      <c r="BF2">
+      <c r="BG2">
         <v>1.03</v>
-      </c>
-      <c r="BG2">
-        <v>0.66</v>
       </c>
       <c r="BH2">
         <v>0.66</v>
       </c>
       <c r="BI2">
+        <v>0.66</v>
+      </c>
+      <c r="BJ2">
         <v>0.72</v>
       </c>
-      <c r="BJ2">
+      <c r="BK2">
         <v>0.99</v>
       </c>
-      <c r="BK2">
+      <c r="BL2">
         <v>0.72</v>
       </c>
-      <c r="BL2">
+      <c r="BM2">
         <v>0.79</v>
       </c>
-      <c r="BM2">
+      <c r="BN2">
         <v>0.68</v>
-      </c>
-      <c r="BN2">
-        <v>0.97</v>
       </c>
       <c r="BO2">
         <v>0.97</v>
       </c>
       <c r="BP2">
-        <v>1.03</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="3">
@@ -7029,10 +7029,10 @@
         <v>0</v>
       </c>
       <c r="AS3">
+        <v>0.77</v>
+      </c>
+      <c r="AT3">
         <v>1.08</v>
-      </c>
-      <c r="AT3">
-        <v>0.81</v>
       </c>
       <c r="AU3">
         <v>0.81</v>
@@ -7041,22 +7041,22 @@
         <v>0.81</v>
       </c>
       <c r="AW3">
+        <v>0.81</v>
+      </c>
+      <c r="AX3">
         <v>0.7</v>
-      </c>
-      <c r="AX3">
-        <v>0.79</v>
       </c>
       <c r="AY3">
         <v>0.79</v>
       </c>
       <c r="AZ3">
-        <v>0.68</v>
+        <v>0.79</v>
       </c>
       <c r="BA3">
         <v>0.68</v>
       </c>
       <c r="BB3">
-        <v>0.72</v>
+        <v>0.68</v>
       </c>
       <c r="BC3">
         <v>0.72</v>
@@ -7065,40 +7065,40 @@
         <v>0.72</v>
       </c>
       <c r="BE3">
+        <v>0.72</v>
+      </c>
+      <c r="BF3">
         <v>0.68</v>
       </c>
-      <c r="BF3">
+      <c r="BG3">
         <v>0.81</v>
-      </c>
-      <c r="BG3">
-        <v>0.99</v>
       </c>
       <c r="BH3">
         <v>0.99</v>
       </c>
       <c r="BI3">
+        <v>0.99</v>
+      </c>
+      <c r="BJ3">
         <v>0.68</v>
       </c>
-      <c r="BJ3">
+      <c r="BK3">
         <v>0.7</v>
       </c>
-      <c r="BK3">
+      <c r="BL3">
         <v>1.08</v>
       </c>
-      <c r="BL3">
+      <c r="BM3">
         <v>0.83</v>
       </c>
-      <c r="BM3">
+      <c r="BN3">
         <v>0.48</v>
-      </c>
-      <c r="BN3">
-        <v>0.74</v>
       </c>
       <c r="BO3">
         <v>0.74</v>
       </c>
       <c r="BP3">
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="4">
@@ -7235,7 +7235,7 @@
         <v>0.25</v>
       </c>
       <c r="AS4">
-        <v>0.35</v>
+        <v>0.75</v>
       </c>
       <c r="AT4">
         <v>0.35</v>
@@ -7250,13 +7250,13 @@
         <v>0.35</v>
       </c>
       <c r="AX4">
-        <v>1.15</v>
+        <v>0.35</v>
       </c>
       <c r="AY4">
         <v>1.15</v>
       </c>
       <c r="AZ4">
-        <v>0.35</v>
+        <v>1.15</v>
       </c>
       <c r="BA4">
         <v>0.35</v>
@@ -7274,10 +7274,10 @@
         <v>0.35</v>
       </c>
       <c r="BF4">
+        <v>0.35</v>
+      </c>
+      <c r="BG4">
         <v>0.99</v>
-      </c>
-      <c r="BG4">
-        <v>0.35</v>
       </c>
       <c r="BH4">
         <v>0.35</v>
@@ -7298,13 +7298,13 @@
         <v>0.35</v>
       </c>
       <c r="BN4">
-        <v>0.37</v>
+        <v>0.35</v>
       </c>
       <c r="BO4">
         <v>0.37</v>
       </c>
       <c r="BP4">
-        <v>0.75</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="5">
@@ -7441,10 +7441,10 @@
         <v>0</v>
       </c>
       <c r="AS5">
+        <v>0.77</v>
+      </c>
+      <c r="AT5">
         <v>1.06</v>
-      </c>
-      <c r="AT5">
-        <v>0.81</v>
       </c>
       <c r="AU5">
         <v>0.81</v>
@@ -7453,22 +7453,22 @@
         <v>0.81</v>
       </c>
       <c r="AW5">
+        <v>0.81</v>
+      </c>
+      <c r="AX5">
         <v>0.7</v>
-      </c>
-      <c r="AX5">
-        <v>0.79</v>
       </c>
       <c r="AY5">
         <v>0.79</v>
       </c>
       <c r="AZ5">
-        <v>0.63</v>
+        <v>0.79</v>
       </c>
       <c r="BA5">
         <v>0.63</v>
       </c>
       <c r="BB5">
-        <v>0.68</v>
+        <v>0.63</v>
       </c>
       <c r="BC5">
         <v>0.68</v>
@@ -7477,40 +7477,40 @@
         <v>0.68</v>
       </c>
       <c r="BE5">
+        <v>0.68</v>
+      </c>
+      <c r="BF5">
         <v>0.63</v>
       </c>
-      <c r="BF5">
+      <c r="BG5">
         <v>0.79</v>
-      </c>
-      <c r="BG5">
-        <v>1.01</v>
       </c>
       <c r="BH5">
         <v>1.01</v>
       </c>
       <c r="BI5">
+        <v>1.01</v>
+      </c>
+      <c r="BJ5">
         <v>0.63</v>
       </c>
-      <c r="BJ5">
+      <c r="BK5">
         <v>0.68</v>
       </c>
-      <c r="BK5">
+      <c r="BL5">
         <v>1.08</v>
       </c>
-      <c r="BL5">
+      <c r="BM5">
         <v>0.79</v>
       </c>
-      <c r="BM5">
+      <c r="BN5">
         <v>0.5</v>
-      </c>
-      <c r="BN5">
-        <v>0.72</v>
       </c>
       <c r="BO5">
         <v>0.72</v>
       </c>
       <c r="BP5">
-        <v>0.77</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="6">
@@ -7647,10 +7647,10 @@
         <v>0.25</v>
       </c>
       <c r="AS6">
+        <v>0.35</v>
+      </c>
+      <c r="AT6">
         <v>0.82</v>
-      </c>
-      <c r="AT6">
-        <v>0.35</v>
       </c>
       <c r="AU6">
         <v>0.35</v>
@@ -7689,22 +7689,22 @@
         <v>0.35</v>
       </c>
       <c r="BG6">
-        <v>0.73</v>
+        <v>0.35</v>
       </c>
       <c r="BH6">
         <v>0.73</v>
       </c>
       <c r="BI6">
-        <v>0.35</v>
+        <v>0.73</v>
       </c>
       <c r="BJ6">
         <v>0.35</v>
       </c>
       <c r="BK6">
+        <v>0.35</v>
+      </c>
+      <c r="BL6">
         <v>1.11</v>
-      </c>
-      <c r="BL6">
-        <v>0.35</v>
       </c>
       <c r="BM6">
         <v>0.35</v>
@@ -7853,10 +7853,10 @@
         <v>0</v>
       </c>
       <c r="AS7">
+        <v>0.92</v>
+      </c>
+      <c r="AT7">
         <v>0.81</v>
-      </c>
-      <c r="AT7">
-        <v>1.01</v>
       </c>
       <c r="AU7">
         <v>1.01</v>
@@ -7865,7 +7865,7 @@
         <v>1.01</v>
       </c>
       <c r="AW7">
-        <v>0.9</v>
+        <v>1.01</v>
       </c>
       <c r="AX7">
         <v>0.9</v>
@@ -7874,13 +7874,13 @@
         <v>0.9</v>
       </c>
       <c r="AZ7">
-        <v>0.54</v>
+        <v>0.9</v>
       </c>
       <c r="BA7">
         <v>0.54</v>
       </c>
       <c r="BB7">
-        <v>0.59</v>
+        <v>0.54</v>
       </c>
       <c r="BC7">
         <v>0.59</v>
@@ -7889,40 +7889,40 @@
         <v>0.59</v>
       </c>
       <c r="BE7">
+        <v>0.59</v>
+      </c>
+      <c r="BF7">
         <v>0.54</v>
       </c>
-      <c r="BF7">
+      <c r="BG7">
         <v>0.92</v>
-      </c>
-      <c r="BG7">
-        <v>0.77</v>
       </c>
       <c r="BH7">
         <v>0.77</v>
       </c>
       <c r="BI7">
+        <v>0.77</v>
+      </c>
+      <c r="BJ7">
         <v>0.54</v>
       </c>
-      <c r="BJ7">
+      <c r="BK7">
         <v>0.9</v>
       </c>
-      <c r="BK7">
+      <c r="BL7">
         <v>0.79</v>
       </c>
-      <c r="BL7">
+      <c r="BM7">
         <v>0.66</v>
       </c>
-      <c r="BM7">
+      <c r="BN7">
         <v>0.79</v>
-      </c>
-      <c r="BN7">
-        <v>0.77</v>
       </c>
       <c r="BO7">
         <v>0.77</v>
       </c>
       <c r="BP7">
-        <v>0.92</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="8">
@@ -12672,7 +12672,7 @@
         <v>3</v>
       </c>
       <c r="G17" t="str">
-        <v>Care and Companionship Client</v>
+        <v>Office Hours Client</v>
       </c>
       <c r="H17">
         <v>10</v>
@@ -12699,7 +12699,7 @@
         <v>60</v>
       </c>
       <c r="P17" t="str">
-        <v>Office Hours Client</v>
+        <v>Care and Companionship Client</v>
       </c>
       <c r="Q17">
         <v>10</v>
@@ -16312,7 +16312,7 @@
         <v>8</v>
       </c>
       <c r="G73" t="str">
-        <v>Campbell, Neil</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="H73">
         <v>3</v>
@@ -16327,19 +16327,19 @@
         <v>3</v>
       </c>
       <c r="L73">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M73" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="N73">
         <v>3</v>
       </c>
       <c r="O73">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P73" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="Q73">
         <v>3</v>
@@ -16664,7 +16664,7 @@
         <v>60</v>
       </c>
       <c r="P78" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="Q78">
         <v>8</v>
@@ -16673,7 +16673,7 @@
         <v>60</v>
       </c>
       <c r="S78" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="T78">
         <v>8</v>
@@ -18104,19 +18104,19 @@
         <v>Employee \ Client</v>
       </c>
       <c r="B1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Office Hours Client 09:00-12:00 (60m)</v>
       </c>
       <c r="C1" t="str">
-        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
+        <v>Office Hours Client 14:00-17:00 (60m)</v>
       </c>
       <c r="D1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="E1" t="str">
-        <v>Office Hours Client 09:00-12:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="F1" t="str">
-        <v>Office Hours Client 14:00-17:00 (60m)</v>
+        <v>Care and Companionship Client 09:00-17:00 (60m)</v>
       </c>
       <c r="G1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -19003,8 +19003,8 @@
       <c r="B4">
         <v>0.78</v>
       </c>
-      <c r="C4">
-        <v>0.78</v>
+      <c r="C4" t="str">
+        <v/>
       </c>
       <c r="D4">
         <v>0.78</v>
@@ -19012,8 +19012,8 @@
       <c r="E4">
         <v>0.78</v>
       </c>
-      <c r="F4" t="str">
-        <v/>
+      <c r="F4">
+        <v>0.78</v>
       </c>
       <c r="G4">
         <v>0.78</v>
@@ -19302,8 +19302,8 @@
       <c r="B5">
         <v>0</v>
       </c>
-      <c r="C5">
-        <v>0</v>
+      <c r="C5" t="str">
+        <v/>
       </c>
       <c r="D5">
         <v>0</v>
@@ -19311,8 +19311,8 @@
       <c r="E5">
         <v>0</v>
       </c>
-      <c r="F5" t="str">
-        <v/>
+      <c r="F5">
+        <v>0</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -19900,8 +19900,8 @@
       <c r="B7">
         <v>0</v>
       </c>
-      <c r="C7">
-        <v>0</v>
+      <c r="C7" t="str">
+        <v/>
       </c>
       <c r="D7">
         <v>0</v>
@@ -19909,8 +19909,8 @@
       <c r="E7">
         <v>0</v>
       </c>
-      <c r="F7" t="str">
-        <v/>
+      <c r="F7">
+        <v>0</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -20498,8 +20498,8 @@
       <c r="B9">
         <v>0</v>
       </c>
-      <c r="C9">
-        <v>0</v>
+      <c r="C9" t="str">
+        <v/>
       </c>
       <c r="D9">
         <v>0</v>
@@ -20507,8 +20507,8 @@
       <c r="E9">
         <v>0</v>
       </c>
-      <c r="F9" t="str">
-        <v/>
+      <c r="F9">
+        <v>0</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -21990,8 +21990,8 @@
       <c r="A14" t="str">
         <v>Sophie Lamont (NL) (GH)</v>
       </c>
-      <c r="B14">
-        <v>0.16</v>
+      <c r="B14" t="str">
+        <v/>
       </c>
       <c r="C14">
         <v>0.16</v>
@@ -21999,8 +21999,8 @@
       <c r="D14">
         <v>0.16</v>
       </c>
-      <c r="E14" t="str">
-        <v/>
+      <c r="E14">
+        <v>0.16</v>
       </c>
       <c r="F14">
         <v>0.16</v>
@@ -22301,16 +22301,16 @@
         <v>Employee \ Client</v>
       </c>
       <c r="B1" t="str">
+        <v>Office Hours Client 09:00-12:00 (60m)</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Office Hours Client 14:00-17:00 (60m)</v>
+      </c>
+      <c r="D1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (120m)</v>
       </c>
-      <c r="C1" t="str">
+      <c r="E1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Office Hours Client 09:00-12:00 (60m)</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Office Hours Client 14:00-17:00 (60m)</v>
       </c>
       <c r="F1" t="str">
         <v>Care and Companionship Client 09:00-17:00 (60m)</v>
@@ -23415,14 +23415,14 @@
       <c r="B5">
         <v>0</v>
       </c>
-      <c r="C5">
-        <v>0</v>
+      <c r="C5" t="str">
+        <v/>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
-      <c r="E5" t="str">
-        <v/>
+      <c r="E5">
+        <v>0</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -23971,14 +23971,14 @@
       <c r="B7">
         <v>0.05</v>
       </c>
-      <c r="C7">
-        <v>0.05</v>
+      <c r="C7" t="str">
+        <v/>
       </c>
       <c r="D7">
         <v>0.05</v>
       </c>
-      <c r="E7" t="str">
-        <v/>
+      <c r="E7">
+        <v>0.05</v>
       </c>
       <c r="F7">
         <v>0.05</v>
@@ -24249,14 +24249,14 @@
       <c r="B8">
         <v>0.08</v>
       </c>
-      <c r="C8">
-        <v>0.08</v>
+      <c r="C8" t="str">
+        <v/>
       </c>
       <c r="D8">
         <v>0.08</v>
       </c>
-      <c r="E8" t="str">
-        <v/>
+      <c r="E8">
+        <v>0.08</v>
       </c>
       <c r="F8">
         <v>0.08</v>
@@ -24527,14 +24527,14 @@
       <c r="B9">
         <v>0</v>
       </c>
-      <c r="C9">
-        <v>0</v>
+      <c r="C9" t="str">
+        <v/>
       </c>
       <c r="D9">
         <v>0</v>
       </c>
-      <c r="E9" t="str">
-        <v/>
+      <c r="E9">
+        <v>0</v>
       </c>
       <c r="F9">
         <v>0</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Improve weekly run display by adding travel time and home location indicators
Updates capacity dashboard to include travel time and home location markers.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -7361,13 +7361,13 @@
         <v>60</v>
       </c>
       <c r="S2" t="str">
-        <v>Bryce (NL), Angela</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="T2">
         <v>11</v>
       </c>
       <c r="U2">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
@@ -7464,7 +7464,7 @@
         <v>120</v>
       </c>
       <c r="J4" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>Kennedy (NL), Isabelle</v>
       </c>
       <c r="K4">
         <v>1</v>
@@ -7473,13 +7473,13 @@
         <v>120</v>
       </c>
       <c r="M4" t="str">
-        <v>Kennedy (NL), Isabelle</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N4">
         <v>1</v>
       </c>
       <c r="O4">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P4" t="str">
         <v>East NL, Glasgow</v>
@@ -7491,13 +7491,13 @@
         <v>60</v>
       </c>
       <c r="S4" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="T4">
         <v>1</v>
       </c>
       <c r="U4">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5">
@@ -7529,13 +7529,13 @@
         <v>120</v>
       </c>
       <c r="J5" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K5">
         <v>2</v>
       </c>
       <c r="L5">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M5" t="str">
         <v>East NL, Glasgow</v>
@@ -7547,13 +7547,13 @@
         <v>60</v>
       </c>
       <c r="P5" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="Q5">
         <v>2</v>
       </c>
       <c r="R5">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S5" t="str">
         <v>Mullen (NL), Eileen</v>
@@ -7612,13 +7612,13 @@
         <v>120</v>
       </c>
       <c r="P6" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q6">
         <v>2</v>
       </c>
       <c r="R6">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S6" t="str">
         <v>East NL, Glasgow</v>
@@ -7650,13 +7650,13 @@
         <v>2</v>
       </c>
       <c r="G7" t="str">
-        <v>Reid, Robert</v>
+        <v>Lynch (NL), Roselyn</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="I7">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J7" t="str">
         <v>Lynch (NL), Roselyn</v>
@@ -7668,13 +7668,13 @@
         <v>60</v>
       </c>
       <c r="M7" t="str">
-        <v>Lynch (NL), Roselyn</v>
+        <v>Reid, Robert</v>
       </c>
       <c r="N7">
         <v>1</v>
       </c>
       <c r="O7">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P7" t="str">
         <v>Bryce (NL), Angela</v>
@@ -7686,7 +7686,7 @@
         <v>120</v>
       </c>
       <c r="S7" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="T7">
         <v>5</v>
@@ -7724,13 +7724,13 @@
         <v>120</v>
       </c>
       <c r="J8" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M8" t="str">
         <v>East NL, Glasgow</v>
@@ -7742,13 +7742,13 @@
         <v>60</v>
       </c>
       <c r="P8" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="Q8">
         <v>1</v>
       </c>
       <c r="R8">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S8" t="str">
         <v>Kennedy (NL), Isabelle</v>
@@ -7816,13 +7816,13 @@
         <v>120</v>
       </c>
       <c r="S9" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T9">
         <v>5</v>
       </c>
       <c r="U9">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10">
@@ -7946,7 +7946,7 @@
         <v>60</v>
       </c>
       <c r="S11" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="T11">
         <v>15</v>
@@ -7984,7 +7984,7 @@
         <v>120</v>
       </c>
       <c r="J12" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>Kennedy (NL), Isabelle</v>
       </c>
       <c r="K12">
         <v>1</v>
@@ -7993,13 +7993,13 @@
         <v>120</v>
       </c>
       <c r="M12" t="str">
-        <v>Kennedy (NL), Isabelle</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N12">
         <v>1</v>
       </c>
       <c r="O12">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P12" t="str">
         <v>East NL, Glasgow</v>
@@ -8011,13 +8011,13 @@
         <v>60</v>
       </c>
       <c r="S12" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="T12">
         <v>1</v>
       </c>
       <c r="U12">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="13">
@@ -8058,7 +8058,7 @@
         <v>120</v>
       </c>
       <c r="M13" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="N13">
         <v>13</v>
@@ -8067,7 +8067,7 @@
         <v>60</v>
       </c>
       <c r="P13" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="Q13">
         <v>13</v>
@@ -8105,7 +8105,7 @@
         <v>3</v>
       </c>
       <c r="G14" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="H14">
         <v>4</v>
@@ -8114,16 +8114,16 @@
         <v>60</v>
       </c>
       <c r="J14" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Gray (NL), Mary</v>
       </c>
       <c r="K14">
         <v>4</v>
       </c>
       <c r="L14">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M14" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="N14">
         <v>4</v>
@@ -8141,7 +8141,7 @@
         <v>60</v>
       </c>
       <c r="S14" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="T14">
         <v>4</v>
@@ -8206,7 +8206,7 @@
         <v>120</v>
       </c>
       <c r="S15" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>Kennedy (NL), Isabelle</v>
       </c>
       <c r="T15">
         <v>5</v>
@@ -8235,13 +8235,13 @@
         <v>6</v>
       </c>
       <c r="G16" t="str">
-        <v>Reid, Robert</v>
+        <v>Lynch (NL), Roselyn</v>
       </c>
       <c r="H16">
         <v>4</v>
       </c>
       <c r="I16">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J16" t="str">
         <v>Lynch (NL), Roselyn</v>
@@ -8259,16 +8259,16 @@
         <v>4</v>
       </c>
       <c r="O16">
-        <v>60</v>
+        <v>285</v>
       </c>
       <c r="P16" t="str">
-        <v>Lynch (NL), Roselyn</v>
+        <v>Reid, Robert</v>
       </c>
       <c r="Q16">
         <v>4</v>
       </c>
       <c r="R16">
-        <v>285</v>
+        <v>120</v>
       </c>
       <c r="S16" t="str">
         <v>Bryce (NL), Angela</v>
@@ -8327,16 +8327,16 @@
         <v>60</v>
       </c>
       <c r="P17" t="str">
-        <v>Anderson, Margaret</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="Q17">
         <v>11</v>
       </c>
       <c r="R17">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S17" t="str">
-        <v>Anderson, Margaret</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T17">
         <v>11</v>
@@ -8365,22 +8365,22 @@
         <v>5.75</v>
       </c>
       <c r="G18" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott (NL), Edith</v>
       </c>
       <c r="H18">
         <v>1</v>
       </c>
       <c r="I18">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J18" t="str">
-        <v>Scott (NL), Edith</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="K18">
         <v>1</v>
       </c>
       <c r="L18">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M18" t="str">
         <v>Barrons (NL/HCAH), Shirley</v>
@@ -8430,7 +8430,7 @@
         <v>2</v>
       </c>
       <c r="G19" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="H19">
         <v>10</v>
@@ -8439,7 +8439,7 @@
         <v>60</v>
       </c>
       <c r="J19" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Barrons (NL/HCAH), Shirley</v>
       </c>
       <c r="K19">
         <v>10</v>
@@ -8448,7 +8448,7 @@
         <v>60</v>
       </c>
       <c r="M19" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Barrons (NL/HCAH), Shirley</v>
       </c>
       <c r="N19">
         <v>10</v>
@@ -8457,7 +8457,7 @@
         <v>60</v>
       </c>
       <c r="P19" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Barrons (NL/HCAH), Shirley</v>
       </c>
       <c r="Q19">
         <v>10</v>
@@ -8466,7 +8466,7 @@
         <v>60</v>
       </c>
       <c r="S19" t="str">
-        <v>Duncan, George</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="T19">
         <v>10</v>
@@ -8652,16 +8652,16 @@
         <v>285</v>
       </c>
       <c r="P22" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="Q22">
         <v>5</v>
       </c>
       <c r="R22">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S22" t="str">
-        <v>Lindsay, Martha</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="T22">
         <v>5</v>
@@ -8782,7 +8782,7 @@
         <v>60</v>
       </c>
       <c r="P24" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q24">
         <v>15</v>
@@ -8894,7 +8894,7 @@
         <v>360</v>
       </c>
       <c r="J26" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="K26">
         <v>13</v>
@@ -8903,7 +8903,7 @@
         <v>60</v>
       </c>
       <c r="M26" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="N26">
         <v>13</v>
@@ -8912,7 +8912,7 @@
         <v>60</v>
       </c>
       <c r="P26" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q26">
         <v>13</v>
@@ -8921,7 +8921,7 @@
         <v>60</v>
       </c>
       <c r="S26" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="T26">
         <v>13</v>
@@ -8950,7 +8950,7 @@
         <v>5</v>
       </c>
       <c r="G27" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="H27">
         <v>4</v>
@@ -8959,7 +8959,7 @@
         <v>60</v>
       </c>
       <c r="J27" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="K27">
         <v>4</v>
@@ -8968,7 +8968,7 @@
         <v>60</v>
       </c>
       <c r="M27" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="N27">
         <v>4</v>
@@ -8977,7 +8977,7 @@
         <v>60</v>
       </c>
       <c r="P27" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="Q27">
         <v>4</v>
@@ -8986,7 +8986,7 @@
         <v>60</v>
       </c>
       <c r="S27" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="T27">
         <v>4</v>
@@ -9107,16 +9107,16 @@
         <v>285</v>
       </c>
       <c r="P29" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="Q29">
         <v>8</v>
       </c>
       <c r="R29">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S29" t="str">
-        <v>Lindsay, Martha</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="T29">
         <v>8</v>
@@ -9181,7 +9181,7 @@
         <v>60</v>
       </c>
       <c r="S30" t="str">
-        <v>Anderson, Margaret</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="T30">
         <v>11</v>
@@ -9210,22 +9210,22 @@
         <v>4</v>
       </c>
       <c r="G31" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott (NL), Edith</v>
       </c>
       <c r="H31">
         <v>1</v>
       </c>
       <c r="I31">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="J31" t="str">
-        <v>Scott (NL), Edith</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="K31">
         <v>1</v>
       </c>
       <c r="L31">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="M31" t="str">
         <v>Grant (NL), Helen</v>
@@ -9293,16 +9293,16 @@
         <v>60</v>
       </c>
       <c r="M32" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="N32">
         <v>3</v>
       </c>
       <c r="O32">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P32" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="Q32">
         <v>3</v>
@@ -9405,13 +9405,13 @@
         <v>2</v>
       </c>
       <c r="G34" t="str">
-        <v>Reid, Robert</v>
+        <v>Lynch (NL), Roselyn</v>
       </c>
       <c r="H34">
         <v>1</v>
       </c>
       <c r="I34">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J34" t="str">
         <v>Lynch (NL), Roselyn</v>
@@ -9423,16 +9423,16 @@
         <v>60</v>
       </c>
       <c r="M34" t="str">
-        <v>Lynch (NL), Roselyn</v>
+        <v>Reid, Robert</v>
       </c>
       <c r="N34">
         <v>1</v>
       </c>
       <c r="O34">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P34" t="str">
-        <v>Gibb (NL), Irene</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="Q34">
         <v>5</v>
@@ -9441,7 +9441,7 @@
         <v>60</v>
       </c>
       <c r="S34" t="str">
-        <v>Brown, Christine</v>
+        <v>Gibb (NL), Irene</v>
       </c>
       <c r="T34">
         <v>5</v>
@@ -9701,13 +9701,13 @@
         <v>60</v>
       </c>
       <c r="S38" t="str">
-        <v>Russell (NL), Julia</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="T38">
         <v>4</v>
       </c>
       <c r="U38">
-        <v>285</v>
+        <v>60</v>
       </c>
     </row>
     <row r="39">
@@ -9730,7 +9730,7 @@
         <v>9</v>
       </c>
       <c r="G39" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="H39">
         <v>13</v>
@@ -9757,7 +9757,7 @@
         <v>60</v>
       </c>
       <c r="P39" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q39">
         <v>13</v>
@@ -9766,7 +9766,7 @@
         <v>60</v>
       </c>
       <c r="S39" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="T39">
         <v>13</v>
@@ -9795,7 +9795,7 @@
         <v>5</v>
       </c>
       <c r="G40" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="H40">
         <v>4</v>
@@ -9822,7 +9822,7 @@
         <v>60</v>
       </c>
       <c r="P40" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q40">
         <v>4</v>
@@ -9831,7 +9831,7 @@
         <v>60</v>
       </c>
       <c r="S40" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="T40">
         <v>4</v>
@@ -9860,13 +9860,13 @@
         <v>7</v>
       </c>
       <c r="G41" t="str">
-        <v>Reid, Robert</v>
+        <v>Lynch (NL), Roselyn</v>
       </c>
       <c r="H41">
         <v>4</v>
       </c>
       <c r="I41">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J41" t="str">
         <v>Lynch (NL), Roselyn</v>
@@ -9884,19 +9884,19 @@
         <v>4</v>
       </c>
       <c r="O41">
-        <v>60</v>
+        <v>285</v>
       </c>
       <c r="P41" t="str">
-        <v>Lynch (NL), Roselyn</v>
+        <v>Reid, Robert</v>
       </c>
       <c r="Q41">
         <v>4</v>
       </c>
       <c r="R41">
-        <v>285</v>
+        <v>120</v>
       </c>
       <c r="S41" t="str">
-        <v>Gibb (NL), Irene</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="T41">
         <v>8</v>
@@ -9961,13 +9961,13 @@
         <v>60</v>
       </c>
       <c r="S42" t="str">
-        <v>Bryce (NL), Angela</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="T42">
         <v>11</v>
       </c>
       <c r="U42">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="43">
@@ -10026,7 +10026,7 @@
         <v>60</v>
       </c>
       <c r="S43" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="T43">
         <v>6</v>
@@ -10055,7 +10055,7 @@
         <v>4.75</v>
       </c>
       <c r="G44" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="H44">
         <v>10</v>
@@ -10064,7 +10064,7 @@
         <v>60</v>
       </c>
       <c r="J44" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="K44">
         <v>10</v>
@@ -10073,25 +10073,25 @@
         <v>60</v>
       </c>
       <c r="M44" t="str">
-        <v>O'Hara (NL), Rose</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="N44">
         <v>10</v>
       </c>
       <c r="O44">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="P44" t="str">
-        <v>Bryce (NL), Angela</v>
+        <v>Law (NL), Angela</v>
       </c>
       <c r="Q44">
         <v>10</v>
       </c>
       <c r="R44">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="S44" t="str">
-        <v>Duncan, George</v>
+        <v>Barrons (NL/HCAH), Shirley</v>
       </c>
       <c r="T44">
         <v>10</v>
@@ -10351,13 +10351,13 @@
         <v>60</v>
       </c>
       <c r="S48" t="str">
-        <v>Mclachlan, William</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="T48">
         <v>8</v>
       </c>
       <c r="U48">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="49">
@@ -10537,7 +10537,7 @@
         <v>60</v>
       </c>
       <c r="P51" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q51">
         <v>15</v>
@@ -10611,13 +10611,13 @@
         <v>60</v>
       </c>
       <c r="S52" t="str">
-        <v>Russell (NL), Julia</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="T52">
         <v>4</v>
       </c>
       <c r="U52">
-        <v>285</v>
+        <v>60</v>
       </c>
     </row>
     <row r="53">
@@ -10640,7 +10640,7 @@
         <v>8</v>
       </c>
       <c r="G53" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="H53">
         <v>13</v>
@@ -10667,7 +10667,7 @@
         <v>60</v>
       </c>
       <c r="P53" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q53">
         <v>13</v>
@@ -10705,7 +10705,7 @@
         <v>6</v>
       </c>
       <c r="G54" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="H54">
         <v>4</v>
@@ -10732,7 +10732,7 @@
         <v>60</v>
       </c>
       <c r="P54" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q54">
         <v>4</v>
@@ -10779,7 +10779,7 @@
         <v>60</v>
       </c>
       <c r="J55" t="str">
-        <v>Whyte, Jean</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="K55">
         <v>1</v>
@@ -10797,7 +10797,7 @@
         <v>60</v>
       </c>
       <c r="P55" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Whyte, Jean</v>
       </c>
       <c r="Q55">
         <v>1</v>
@@ -11095,22 +11095,22 @@
         <v>5.75</v>
       </c>
       <c r="G60" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott (NL), Edith</v>
       </c>
       <c r="H60">
         <v>1</v>
       </c>
       <c r="I60">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J60" t="str">
-        <v>Scott (NL), Edith</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="K60">
         <v>1</v>
       </c>
       <c r="L60">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M60" t="str">
         <v>Barrons (NL/HCAH), Shirley</v>
@@ -11317,7 +11317,7 @@
         <v>60</v>
       </c>
       <c r="P63" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="Q63">
         <v>5</v>
@@ -11326,7 +11326,7 @@
         <v>60</v>
       </c>
       <c r="S63" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="T63">
         <v>5</v>
@@ -11716,7 +11716,7 @@
         <v>60</v>
       </c>
       <c r="S69" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="T69">
         <v>15</v>
@@ -11754,7 +11754,7 @@
         <v>60</v>
       </c>
       <c r="J70" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="K70">
         <v>1</v>
@@ -11772,7 +11772,7 @@
         <v>60</v>
       </c>
       <c r="P70" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="Q70">
         <v>1</v>
@@ -11902,7 +11902,7 @@
         <v>60</v>
       </c>
       <c r="P72" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="Q72">
         <v>8</v>
@@ -11911,7 +11911,7 @@
         <v>60</v>
       </c>
       <c r="S72" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="T72">
         <v>8</v>
@@ -11958,7 +11958,7 @@
         <v>60</v>
       </c>
       <c r="M73" t="str">
-        <v>Campbell, Neil</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="N73">
         <v>11</v>
@@ -11982,7 +11982,7 @@
         <v>11</v>
       </c>
       <c r="U73">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="74">

</xml_diff>

<commit_message>
Checkpoint before assistant change: Limit the maximum number of employee travel to twenty
Adjusted the maximum travel allowance for employees to 20, enforcing stricter limits.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -7325,22 +7325,22 @@
         <v>6</v>
       </c>
       <c r="G2" t="str">
-        <v>Robertson (NL), Doreen</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="H2">
         <v>8</v>
       </c>
       <c r="I2">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J2" t="str">
-        <v>Murray (NL), James</v>
+        <v>Robertson (NL), Doreen</v>
       </c>
       <c r="K2">
         <v>8</v>
       </c>
       <c r="L2">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M2" t="str">
         <v>Brown, Christine</v>
@@ -7361,7 +7361,7 @@
         <v>60</v>
       </c>
       <c r="S2" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T2">
         <v>11</v>
@@ -7455,7 +7455,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="str">
-        <v>Collie, Mattie</v>
+        <v>Kennedy (NL), Isabelle</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -7464,13 +7464,13 @@
         <v>120</v>
       </c>
       <c r="J4" t="str">
-        <v>Kennedy (NL), Isabelle</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K4">
         <v>1</v>
       </c>
       <c r="L4">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M4" t="str">
         <v>East NL, Glasgow</v>
@@ -7482,16 +7482,16 @@
         <v>60</v>
       </c>
       <c r="P4" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q4">
         <v>1</v>
       </c>
       <c r="R4">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S4" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="T4">
         <v>1</v>
@@ -7520,13 +7520,13 @@
         <v>4</v>
       </c>
       <c r="G5" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H5">
         <v>2</v>
       </c>
       <c r="I5">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J5" t="str">
         <v>East NL, Glasgow</v>
@@ -7538,13 +7538,13 @@
         <v>60</v>
       </c>
       <c r="M5" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="N5">
         <v>2</v>
       </c>
       <c r="O5">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P5" t="str">
         <v>Duffy, Sarah Anne (goes by Anne)</v>
@@ -7556,13 +7556,13 @@
         <v>120</v>
       </c>
       <c r="S5" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Kennedy (NL), Isabelle</v>
       </c>
       <c r="T5">
         <v>3</v>
       </c>
       <c r="U5">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6">
@@ -7603,13 +7603,13 @@
         <v>120</v>
       </c>
       <c r="M6" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N6">
         <v>2</v>
       </c>
       <c r="O6">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P6" t="str">
         <v>East NL, Glasgow</v>
@@ -7621,13 +7621,13 @@
         <v>60</v>
       </c>
       <c r="S6" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="T6">
         <v>2</v>
       </c>
       <c r="U6">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7">
@@ -7715,13 +7715,13 @@
         <v>10</v>
       </c>
       <c r="G8" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H8">
         <v>1</v>
       </c>
       <c r="I8">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J8" t="str">
         <v>East NL, Glasgow</v>
@@ -7733,13 +7733,13 @@
         <v>60</v>
       </c>
       <c r="M8" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="N8">
         <v>1</v>
       </c>
       <c r="O8">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P8" t="str">
         <v>Duffy, Sarah Anne (goes by Anne)</v>
@@ -7807,13 +7807,13 @@
         <v>60</v>
       </c>
       <c r="P9" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q9">
         <v>5</v>
       </c>
       <c r="R9">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S9" t="str">
         <v>East NL, Glasgow</v>
@@ -7872,13 +7872,13 @@
         <v>60</v>
       </c>
       <c r="P10" t="str">
-        <v>Robertson (NL), Doreen</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q10">
         <v>7</v>
       </c>
       <c r="R10">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S10" t="str">
         <v>Campbell, Neil</v>
@@ -7975,7 +7975,7 @@
         <v>3</v>
       </c>
       <c r="G12" t="str">
-        <v>Collie, Mattie</v>
+        <v>Kennedy (NL), Isabelle</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -7984,13 +7984,13 @@
         <v>120</v>
       </c>
       <c r="J12" t="str">
-        <v>Kennedy (NL), Isabelle</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K12">
         <v>1</v>
       </c>
       <c r="L12">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M12" t="str">
         <v>East NL, Glasgow</v>
@@ -8002,16 +8002,16 @@
         <v>60</v>
       </c>
       <c r="P12" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q12">
         <v>1</v>
       </c>
       <c r="R12">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S12" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="T12">
         <v>1</v>
@@ -8058,7 +8058,7 @@
         <v>120</v>
       </c>
       <c r="M13" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="N13">
         <v>13</v>
@@ -8067,7 +8067,7 @@
         <v>60</v>
       </c>
       <c r="P13" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="Q13">
         <v>13</v>
@@ -8105,7 +8105,7 @@
         <v>3</v>
       </c>
       <c r="G14" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="H14">
         <v>4</v>
@@ -8114,16 +8114,16 @@
         <v>60</v>
       </c>
       <c r="J14" t="str">
-        <v>Gray (NL), Mary</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="K14">
         <v>4</v>
       </c>
       <c r="L14">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M14" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="N14">
         <v>4</v>
@@ -8132,7 +8132,7 @@
         <v>60</v>
       </c>
       <c r="P14" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q14">
         <v>4</v>
@@ -8141,13 +8141,13 @@
         <v>60</v>
       </c>
       <c r="S14" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Gray (NL), Mary</v>
       </c>
       <c r="T14">
         <v>4</v>
       </c>
       <c r="U14">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15">
@@ -8327,13 +8327,13 @@
         <v>60</v>
       </c>
       <c r="P17" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q17">
         <v>11</v>
       </c>
       <c r="R17">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S17" t="str">
         <v>Campbell, Neil</v>
@@ -8430,7 +8430,7 @@
         <v>2</v>
       </c>
       <c r="G19" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="H19">
         <v>10</v>
@@ -8439,7 +8439,7 @@
         <v>60</v>
       </c>
       <c r="J19" t="str">
-        <v>Barrons (NL/HCAH), Shirley</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="K19">
         <v>10</v>
@@ -8448,7 +8448,7 @@
         <v>60</v>
       </c>
       <c r="M19" t="str">
-        <v>Barrons (NL/HCAH), Shirley</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="N19">
         <v>10</v>
@@ -8457,7 +8457,7 @@
         <v>60</v>
       </c>
       <c r="P19" t="str">
-        <v>Barrons (NL/HCAH), Shirley</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="Q19">
         <v>10</v>
@@ -8466,7 +8466,7 @@
         <v>60</v>
       </c>
       <c r="S19" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>Lynch (NL), Roselyn</v>
       </c>
       <c r="T19">
         <v>10</v>
@@ -8513,7 +8513,7 @@
         <v>60</v>
       </c>
       <c r="M20" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="N20">
         <v>3</v>
@@ -8522,7 +8522,7 @@
         <v>60</v>
       </c>
       <c r="P20" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q20">
         <v>3</v>
@@ -8820,7 +8820,7 @@
         <v>3</v>
       </c>
       <c r="G25" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="H25">
         <v>1</v>
@@ -8838,7 +8838,7 @@
         <v>60</v>
       </c>
       <c r="M25" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="N25">
         <v>1</v>
@@ -8903,7 +8903,7 @@
         <v>60</v>
       </c>
       <c r="M26" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="N26">
         <v>13</v>
@@ -8921,7 +8921,7 @@
         <v>60</v>
       </c>
       <c r="S26" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="T26">
         <v>13</v>
@@ -8959,7 +8959,7 @@
         <v>60</v>
       </c>
       <c r="J27" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="K27">
         <v>4</v>
@@ -8977,7 +8977,7 @@
         <v>60</v>
       </c>
       <c r="P27" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q27">
         <v>4</v>
@@ -8986,7 +8986,7 @@
         <v>60</v>
       </c>
       <c r="S27" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="T27">
         <v>4</v>
@@ -9145,7 +9145,7 @@
         <v>6</v>
       </c>
       <c r="G30" t="str">
-        <v>Morris, Jack</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="H30">
         <v>8</v>
@@ -9154,7 +9154,7 @@
         <v>60</v>
       </c>
       <c r="J30" t="str">
-        <v>Murray (NL), James</v>
+        <v>Morris, Jack</v>
       </c>
       <c r="K30">
         <v>8</v>
@@ -9181,7 +9181,7 @@
         <v>60</v>
       </c>
       <c r="S30" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T30">
         <v>11</v>
@@ -9275,34 +9275,34 @@
         <v>6.75</v>
       </c>
       <c r="G32" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H32">
         <v>2</v>
       </c>
       <c r="I32">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J32" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="K32">
         <v>2</v>
       </c>
       <c r="L32">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M32" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="N32">
         <v>3</v>
       </c>
       <c r="O32">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P32" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q32">
         <v>3</v>
@@ -9358,22 +9358,22 @@
         <v>60</v>
       </c>
       <c r="M33" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N33">
         <v>2</v>
       </c>
       <c r="O33">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P33" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="Q33">
         <v>2</v>
       </c>
       <c r="R33">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S33" t="str">
         <v>McInnes (NL), James</v>
@@ -9497,22 +9497,22 @@
         <v>60</v>
       </c>
       <c r="P35" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q35">
         <v>4</v>
       </c>
       <c r="R35">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S35" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="T35">
         <v>4</v>
       </c>
       <c r="U35">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="36">
@@ -9562,22 +9562,22 @@
         <v>60</v>
       </c>
       <c r="P36" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q36">
         <v>5</v>
       </c>
       <c r="R36">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S36" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="T36">
         <v>5</v>
       </c>
       <c r="U36">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="37">
@@ -9665,22 +9665,22 @@
         <v>4</v>
       </c>
       <c r="G38" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H38">
         <v>1</v>
       </c>
       <c r="I38">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J38" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="K38">
         <v>1</v>
       </c>
       <c r="L38">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M38" t="str">
         <v>Clements (NL), Jessie</v>
@@ -9689,16 +9689,16 @@
         <v>1</v>
       </c>
       <c r="O38">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P38" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="Q38">
         <v>1</v>
       </c>
       <c r="R38">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S38" t="str">
         <v>Mullen (NL), Eileen</v>
@@ -9925,7 +9925,7 @@
         <v>5</v>
       </c>
       <c r="G42" t="str">
-        <v>Morris, Jack</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="H42">
         <v>8</v>
@@ -9934,7 +9934,7 @@
         <v>60</v>
       </c>
       <c r="J42" t="str">
-        <v>Murray (NL), James</v>
+        <v>Morris, Jack</v>
       </c>
       <c r="K42">
         <v>8</v>
@@ -9961,7 +9961,7 @@
         <v>60</v>
       </c>
       <c r="S42" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T42">
         <v>11</v>
@@ -10055,7 +10055,7 @@
         <v>4.75</v>
       </c>
       <c r="G44" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="H44">
         <v>10</v>
@@ -10064,7 +10064,7 @@
         <v>60</v>
       </c>
       <c r="J44" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="K44">
         <v>10</v>
@@ -10073,7 +10073,7 @@
         <v>60</v>
       </c>
       <c r="M44" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Lynch (NL), Roselyn</v>
       </c>
       <c r="N44">
         <v>10</v>
@@ -10082,16 +10082,16 @@
         <v>60</v>
       </c>
       <c r="P44" t="str">
-        <v>Law (NL), Angela</v>
+        <v>Lynch (NL), Roselyn</v>
       </c>
       <c r="Q44">
         <v>10</v>
       </c>
       <c r="R44">
-        <v>240</v>
+        <v>60</v>
       </c>
       <c r="S44" t="str">
-        <v>Barrons (NL/HCAH), Shirley</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T44">
         <v>10</v>
@@ -10277,7 +10277,7 @@
         <v>60</v>
       </c>
       <c r="P47" t="str">
-        <v>Morris, Jack</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="Q47">
         <v>18</v>
@@ -10286,7 +10286,7 @@
         <v>60</v>
       </c>
       <c r="S47" t="str">
-        <v>Murray (NL), James</v>
+        <v>Morris, Jack</v>
       </c>
       <c r="T47">
         <v>18</v>
@@ -10575,7 +10575,7 @@
         <v>3</v>
       </c>
       <c r="G52" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="H52">
         <v>1</v>
@@ -10584,7 +10584,7 @@
         <v>60</v>
       </c>
       <c r="J52" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="K52">
         <v>1</v>
@@ -11178,7 +11178,7 @@
         <v>60</v>
       </c>
       <c r="M61" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="N61">
         <v>3</v>
@@ -11187,7 +11187,7 @@
         <v>60</v>
       </c>
       <c r="P61" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q61">
         <v>3</v>
@@ -11642,13 +11642,13 @@
         <v>60</v>
       </c>
       <c r="P68" t="str">
-        <v>Hood, Catherine</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q68">
         <v>7</v>
       </c>
       <c r="R68">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S68" t="str">
         <v>Campbell, Neil</v>
@@ -11745,7 +11745,7 @@
         <v>5</v>
       </c>
       <c r="G70" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="H70">
         <v>1</v>
@@ -11763,7 +11763,7 @@
         <v>60</v>
       </c>
       <c r="M70" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="N70">
         <v>1</v>
@@ -11940,7 +11940,7 @@
         <v>5</v>
       </c>
       <c r="G73" t="str">
-        <v>Morris, Jack</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="H73">
         <v>8</v>
@@ -11949,7 +11949,7 @@
         <v>60</v>
       </c>
       <c r="J73" t="str">
-        <v>Murray (NL), James</v>
+        <v>Morris, Jack</v>
       </c>
       <c r="K73">
         <v>8</v>
@@ -11958,7 +11958,7 @@
         <v>60</v>
       </c>
       <c r="M73" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="N73">
         <v>11</v>
@@ -11982,7 +11982,7 @@
         <v>11</v>
       </c>
       <c r="U73">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="74">
@@ -12005,22 +12005,22 @@
         <v>4</v>
       </c>
       <c r="G74" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="H74">
         <v>1</v>
       </c>
       <c r="I74">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J74" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="K74">
         <v>1</v>
       </c>
       <c r="L74">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M74" t="str">
         <v>Mullen (NL), Eileen</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update capacity dashboard with new metrics
Added new columns and calculations to the capacity dashboard spreadsheet.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -7325,22 +7325,22 @@
         <v>6</v>
       </c>
       <c r="G2" t="str">
-        <v>Murray (NL), James</v>
+        <v>Robertson (NL), Doreen</v>
       </c>
       <c r="H2">
         <v>8</v>
       </c>
       <c r="I2">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J2" t="str">
-        <v>Robertson (NL), Doreen</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="K2">
         <v>8</v>
       </c>
       <c r="L2">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M2" t="str">
         <v>Brown, Christine</v>
@@ -7455,7 +7455,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="str">
-        <v>Kennedy (NL), Isabelle</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -7464,40 +7464,40 @@
         <v>120</v>
       </c>
       <c r="J4" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="K4">
         <v>1</v>
       </c>
       <c r="L4">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M4" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Kennedy (NL), Isabelle</v>
       </c>
       <c r="N4">
         <v>1</v>
       </c>
       <c r="O4">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P4" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q4">
         <v>1</v>
       </c>
       <c r="R4">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S4" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T4">
         <v>1</v>
       </c>
       <c r="U4">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5">
@@ -7520,49 +7520,49 @@
         <v>4</v>
       </c>
       <c r="G5" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H5">
         <v>2</v>
       </c>
       <c r="I5">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J5" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="K5">
         <v>2</v>
       </c>
       <c r="L5">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M5" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N5">
         <v>2</v>
       </c>
       <c r="O5">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P5" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q5">
         <v>2</v>
       </c>
       <c r="R5">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S5" t="str">
-        <v>Kennedy (NL), Isabelle</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="T5">
         <v>3</v>
       </c>
       <c r="U5">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -7603,31 +7603,31 @@
         <v>120</v>
       </c>
       <c r="M6" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="N6">
         <v>2</v>
       </c>
       <c r="O6">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P6" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="Q6">
         <v>2</v>
       </c>
       <c r="R6">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S6" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T6">
         <v>2</v>
       </c>
       <c r="U6">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7">
@@ -7715,40 +7715,40 @@
         <v>10</v>
       </c>
       <c r="G8" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H8">
         <v>1</v>
       </c>
       <c r="I8">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J8" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M8" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N8">
         <v>1</v>
       </c>
       <c r="O8">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P8" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q8">
         <v>1</v>
       </c>
       <c r="R8">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S8" t="str">
         <v>Kennedy (NL), Isabelle</v>
@@ -7807,22 +7807,22 @@
         <v>60</v>
       </c>
       <c r="P9" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="Q9">
         <v>5</v>
       </c>
       <c r="R9">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S9" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="T9">
         <v>5</v>
       </c>
       <c r="U9">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10">
@@ -7975,7 +7975,7 @@
         <v>3</v>
       </c>
       <c r="G12" t="str">
-        <v>Kennedy (NL), Isabelle</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -7984,40 +7984,40 @@
         <v>120</v>
       </c>
       <c r="J12" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="K12">
         <v>1</v>
       </c>
       <c r="L12">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M12" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Kennedy (NL), Isabelle</v>
       </c>
       <c r="N12">
         <v>1</v>
       </c>
       <c r="O12">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P12" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q12">
         <v>1</v>
       </c>
       <c r="R12">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S12" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T12">
         <v>1</v>
       </c>
       <c r="U12">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">
@@ -8206,7 +8206,7 @@
         <v>120</v>
       </c>
       <c r="S15" t="str">
-        <v>Kennedy (NL), Isabelle</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="T15">
         <v>5</v>
@@ -8430,7 +8430,7 @@
         <v>2</v>
       </c>
       <c r="G19" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="H19">
         <v>10</v>
@@ -8439,7 +8439,7 @@
         <v>60</v>
       </c>
       <c r="J19" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Lynch (NL), Roselyn</v>
       </c>
       <c r="K19">
         <v>10</v>
@@ -8448,7 +8448,7 @@
         <v>60</v>
       </c>
       <c r="M19" t="str">
-        <v>Murray (NL), James</v>
+        <v>Lynch (NL), Roselyn</v>
       </c>
       <c r="N19">
         <v>10</v>
@@ -8457,7 +8457,7 @@
         <v>60</v>
       </c>
       <c r="P19" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q19">
         <v>10</v>
@@ -8466,7 +8466,7 @@
         <v>60</v>
       </c>
       <c r="S19" t="str">
-        <v>Lynch (NL), Roselyn</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T19">
         <v>10</v>
@@ -8513,7 +8513,7 @@
         <v>60</v>
       </c>
       <c r="M20" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="N20">
         <v>3</v>
@@ -8522,7 +8522,7 @@
         <v>60</v>
       </c>
       <c r="P20" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="Q20">
         <v>3</v>
@@ -8820,7 +8820,7 @@
         <v>3</v>
       </c>
       <c r="G25" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H25">
         <v>1</v>
@@ -8838,7 +8838,7 @@
         <v>60</v>
       </c>
       <c r="M25" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="N25">
         <v>1</v>
@@ -9145,7 +9145,7 @@
         <v>6</v>
       </c>
       <c r="G30" t="str">
-        <v>Murray (NL), James</v>
+        <v>Morris, Jack</v>
       </c>
       <c r="H30">
         <v>8</v>
@@ -9154,7 +9154,7 @@
         <v>60</v>
       </c>
       <c r="J30" t="str">
-        <v>Morris, Jack</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="K30">
         <v>8</v>
@@ -9275,34 +9275,34 @@
         <v>6.75</v>
       </c>
       <c r="G32" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H32">
         <v>2</v>
       </c>
       <c r="I32">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J32" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K32">
         <v>2</v>
       </c>
       <c r="L32">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M32" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="N32">
         <v>3</v>
       </c>
       <c r="O32">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P32" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="Q32">
         <v>3</v>
@@ -9358,22 +9358,22 @@
         <v>60</v>
       </c>
       <c r="M33" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="N33">
         <v>2</v>
       </c>
       <c r="O33">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P33" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q33">
         <v>2</v>
       </c>
       <c r="R33">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S33" t="str">
         <v>McInnes (NL), James</v>
@@ -9497,22 +9497,22 @@
         <v>60</v>
       </c>
       <c r="P35" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="Q35">
         <v>4</v>
       </c>
       <c r="R35">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S35" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T35">
         <v>4</v>
       </c>
       <c r="U35">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="36">
@@ -9562,22 +9562,22 @@
         <v>60</v>
       </c>
       <c r="P36" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="Q36">
         <v>5</v>
       </c>
       <c r="R36">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S36" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T36">
         <v>5</v>
       </c>
       <c r="U36">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37">
@@ -9665,22 +9665,22 @@
         <v>4</v>
       </c>
       <c r="G38" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H38">
         <v>1</v>
       </c>
       <c r="I38">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J38" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K38">
         <v>1</v>
       </c>
       <c r="L38">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M38" t="str">
         <v>Clements (NL), Jessie</v>
@@ -9689,16 +9689,16 @@
         <v>1</v>
       </c>
       <c r="O38">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P38" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q38">
         <v>1</v>
       </c>
       <c r="R38">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S38" t="str">
         <v>Mullen (NL), Eileen</v>
@@ -9925,7 +9925,7 @@
         <v>5</v>
       </c>
       <c r="G42" t="str">
-        <v>Murray (NL), James</v>
+        <v>Morris, Jack</v>
       </c>
       <c r="H42">
         <v>8</v>
@@ -9934,7 +9934,7 @@
         <v>60</v>
       </c>
       <c r="J42" t="str">
-        <v>Morris, Jack</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="K42">
         <v>8</v>
@@ -10055,7 +10055,7 @@
         <v>4.75</v>
       </c>
       <c r="G44" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Lynch (NL), Roselyn</v>
       </c>
       <c r="H44">
         <v>10</v>
@@ -10064,7 +10064,7 @@
         <v>60</v>
       </c>
       <c r="J44" t="str">
-        <v>Murray (NL), James</v>
+        <v>Lynch (NL), Roselyn</v>
       </c>
       <c r="K44">
         <v>10</v>
@@ -10073,7 +10073,7 @@
         <v>60</v>
       </c>
       <c r="M44" t="str">
-        <v>Lynch (NL), Roselyn</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="N44">
         <v>10</v>
@@ -10082,7 +10082,7 @@
         <v>60</v>
       </c>
       <c r="P44" t="str">
-        <v>Lynch (NL), Roselyn</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q44">
         <v>10</v>
@@ -10097,7 +10097,7 @@
         <v>10</v>
       </c>
       <c r="U44">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="45">
@@ -10277,7 +10277,7 @@
         <v>60</v>
       </c>
       <c r="P47" t="str">
-        <v>Murray (NL), James</v>
+        <v>Morris, Jack</v>
       </c>
       <c r="Q47">
         <v>18</v>
@@ -10286,7 +10286,7 @@
         <v>60</v>
       </c>
       <c r="S47" t="str">
-        <v>Morris, Jack</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="T47">
         <v>18</v>
@@ -10575,7 +10575,7 @@
         <v>3</v>
       </c>
       <c r="G52" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H52">
         <v>1</v>
@@ -10584,7 +10584,7 @@
         <v>60</v>
       </c>
       <c r="J52" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="K52">
         <v>1</v>
@@ -11178,7 +11178,7 @@
         <v>60</v>
       </c>
       <c r="M61" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="N61">
         <v>3</v>
@@ -11187,7 +11187,7 @@
         <v>60</v>
       </c>
       <c r="P61" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="Q61">
         <v>3</v>
@@ -11745,7 +11745,7 @@
         <v>5</v>
       </c>
       <c r="G70" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H70">
         <v>1</v>
@@ -11754,7 +11754,7 @@
         <v>60</v>
       </c>
       <c r="J70" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="K70">
         <v>1</v>
@@ -11763,7 +11763,7 @@
         <v>60</v>
       </c>
       <c r="M70" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="N70">
         <v>1</v>
@@ -11772,7 +11772,7 @@
         <v>60</v>
       </c>
       <c r="P70" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q70">
         <v>1</v>
@@ -11940,7 +11940,7 @@
         <v>5</v>
       </c>
       <c r="G73" t="str">
-        <v>Murray (NL), James</v>
+        <v>Morris, Jack</v>
       </c>
       <c r="H73">
         <v>8</v>
@@ -11949,7 +11949,7 @@
         <v>60</v>
       </c>
       <c r="J73" t="str">
-        <v>Morris, Jack</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="K73">
         <v>8</v>
@@ -12005,22 +12005,22 @@
         <v>4</v>
       </c>
       <c r="G74" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H74">
         <v>1</v>
       </c>
       <c r="I74">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J74" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="K74">
         <v>1</v>
       </c>
       <c r="L74">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M74" t="str">
         <v>Mullen (NL), Eileen</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update capacity dashboard to show employee availability
Updated capacity_dashboard.xlsx to reflect employee availability changes.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -7159,22 +7159,22 @@
         <v>6</v>
       </c>
       <c r="G2" t="str">
-        <v>Murray (NL), James</v>
+        <v>Robertson (NL), Doreen</v>
       </c>
       <c r="H2">
         <v>8</v>
       </c>
       <c r="I2">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J2" t="str">
-        <v>Robertson (NL), Doreen</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="K2">
         <v>8</v>
       </c>
       <c r="L2">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M2" t="str">
         <v>Brown, Christine</v>
@@ -7195,13 +7195,13 @@
         <v>60</v>
       </c>
       <c r="S2" t="str">
-        <v>Campbell, Neil</v>
+        <v>Bryce (NL), Angela</v>
       </c>
       <c r="T2">
         <v>11</v>
       </c>
       <c r="U2">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3">
@@ -7289,7 +7289,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -7298,16 +7298,16 @@
         <v>120</v>
       </c>
       <c r="J4" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="K4">
         <v>1</v>
       </c>
       <c r="L4">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M4" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="N4">
         <v>1</v>
@@ -7316,13 +7316,13 @@
         <v>120</v>
       </c>
       <c r="P4" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q4">
         <v>1</v>
       </c>
       <c r="R4">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S4" t="str">
         <v>Whyte, Jean</v>
@@ -7437,7 +7437,7 @@
         <v>120</v>
       </c>
       <c r="M6" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="N6">
         <v>5</v>
@@ -7446,7 +7446,7 @@
         <v>60</v>
       </c>
       <c r="P6" t="str">
-        <v>Brown, Christine</v>
+        <v>Lindsay (NL), Martha</v>
       </c>
       <c r="Q6">
         <v>5</v>
@@ -7455,7 +7455,7 @@
         <v>60</v>
       </c>
       <c r="S6" t="str">
-        <v>Lindsay (NL), Martha</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="T6">
         <v>5</v>
@@ -7502,13 +7502,13 @@
         <v>120</v>
       </c>
       <c r="M7" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Whyte, Jean</v>
       </c>
       <c r="N7">
         <v>2</v>
       </c>
       <c r="O7">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P7" t="str">
         <v>Clements (NL), Jessie</v>
@@ -7517,10 +7517,10 @@
         <v>2</v>
       </c>
       <c r="R7">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S7" t="str">
-        <v>Whyte, Jean</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="T7">
         <v>2</v>
@@ -7641,13 +7641,13 @@
         <v>60</v>
       </c>
       <c r="P9" t="str">
-        <v>Campbell, Neil</v>
+        <v>Robertson (NL), Doreen</v>
       </c>
       <c r="Q9">
         <v>7</v>
       </c>
       <c r="R9">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S9" t="str">
         <v>Campbell, Neil</v>
@@ -7715,7 +7715,7 @@
         <v>60</v>
       </c>
       <c r="S10" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="T10">
         <v>15</v>
@@ -7744,7 +7744,7 @@
         <v>3</v>
       </c>
       <c r="G11" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -7753,16 +7753,16 @@
         <v>120</v>
       </c>
       <c r="J11" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="K11">
         <v>1</v>
       </c>
       <c r="L11">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M11" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="N11">
         <v>1</v>
@@ -7771,13 +7771,13 @@
         <v>120</v>
       </c>
       <c r="P11" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q11">
         <v>1</v>
       </c>
       <c r="R11">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S11" t="str">
         <v>Whyte, Jean</v>
@@ -7818,7 +7818,7 @@
         <v>510</v>
       </c>
       <c r="J12" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="K12">
         <v>13</v>
@@ -7845,7 +7845,7 @@
         <v>60</v>
       </c>
       <c r="S12" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="T12">
         <v>13</v>
@@ -7874,7 +7874,7 @@
         <v>3</v>
       </c>
       <c r="G13" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="H13">
         <v>4</v>
@@ -7901,7 +7901,7 @@
         <v>60</v>
       </c>
       <c r="P13" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="Q13">
         <v>4</v>
@@ -7910,7 +7910,7 @@
         <v>60</v>
       </c>
       <c r="S13" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="T13">
         <v>4</v>
@@ -8004,7 +8004,7 @@
         <v>4.75</v>
       </c>
       <c r="G15" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -8013,7 +8013,7 @@
         <v>60</v>
       </c>
       <c r="J15" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K15">
         <v>1</v>
@@ -8031,7 +8031,7 @@
         <v>60</v>
       </c>
       <c r="P15" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q15">
         <v>1</v>
@@ -8069,7 +8069,7 @@
         <v>6</v>
       </c>
       <c r="G16" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H16">
         <v>2</v>
@@ -8078,7 +8078,7 @@
         <v>60</v>
       </c>
       <c r="J16" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K16">
         <v>2</v>
@@ -8152,7 +8152,7 @@
         <v>60</v>
       </c>
       <c r="M17" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="N17">
         <v>2</v>
@@ -8161,7 +8161,7 @@
         <v>60</v>
       </c>
       <c r="P17" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q17">
         <v>2</v>
@@ -8199,22 +8199,22 @@
         <v>4.5</v>
       </c>
       <c r="G18" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="H18">
         <v>5</v>
       </c>
       <c r="I18">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J18" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="K18">
         <v>5</v>
       </c>
       <c r="L18">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M18" t="str">
         <v>Campbell, Neil</v>
@@ -8264,7 +8264,7 @@
         <v>8</v>
       </c>
       <c r="G19" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H19">
         <v>1</v>
@@ -8273,7 +8273,7 @@
         <v>60</v>
       </c>
       <c r="J19" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K19">
         <v>1</v>
@@ -8356,7 +8356,7 @@
         <v>120</v>
       </c>
       <c r="P20" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="Q20">
         <v>4</v>
@@ -8365,7 +8365,7 @@
         <v>60</v>
       </c>
       <c r="S20" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T20">
         <v>4</v>
@@ -8394,7 +8394,7 @@
         <v>4</v>
       </c>
       <c r="G21" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H21">
         <v>1</v>
@@ -8403,7 +8403,7 @@
         <v>60</v>
       </c>
       <c r="J21" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K21">
         <v>1</v>
@@ -8486,7 +8486,7 @@
         <v>60</v>
       </c>
       <c r="P22" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="Q22">
         <v>15</v>
@@ -8524,7 +8524,7 @@
         <v>5</v>
       </c>
       <c r="G23" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H23">
         <v>1</v>
@@ -8533,7 +8533,7 @@
         <v>60</v>
       </c>
       <c r="J23" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K23">
         <v>1</v>
@@ -8551,7 +8551,7 @@
         <v>60</v>
       </c>
       <c r="P23" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q23">
         <v>1</v>
@@ -8560,13 +8560,13 @@
         <v>60</v>
       </c>
       <c r="S23" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Russell (NL), Julia</v>
       </c>
       <c r="T23">
         <v>4</v>
       </c>
       <c r="U23">
-        <v>60</v>
+        <v>285</v>
       </c>
     </row>
     <row r="24">
@@ -8607,7 +8607,7 @@
         <v>120</v>
       </c>
       <c r="M24" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="N24">
         <v>13</v>
@@ -8625,7 +8625,7 @@
         <v>60</v>
       </c>
       <c r="S24" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="T24">
         <v>13</v>
@@ -8654,7 +8654,7 @@
         <v>5</v>
       </c>
       <c r="G25" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="H25">
         <v>4</v>
@@ -8672,7 +8672,7 @@
         <v>60</v>
       </c>
       <c r="M25" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="N25">
         <v>4</v>
@@ -8690,13 +8690,13 @@
         <v>60</v>
       </c>
       <c r="S25" t="str">
-        <v>Gray (NL), Mary</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="T25">
         <v>4</v>
       </c>
       <c r="U25">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26">
@@ -8719,22 +8719,22 @@
         <v>4</v>
       </c>
       <c r="G26" t="str">
-        <v>Scott (NL), Edith</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="H26">
         <v>1</v>
       </c>
       <c r="I26">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="J26" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott (NL), Edith</v>
       </c>
       <c r="K26">
         <v>1</v>
       </c>
       <c r="L26">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="M26" t="str">
         <v>Grant (NL), Helen</v>
@@ -8784,7 +8784,7 @@
         <v>3</v>
       </c>
       <c r="G27" t="str">
-        <v>Campbell, Neil</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="H27">
         <v>3</v>
@@ -8793,7 +8793,7 @@
         <v>60</v>
       </c>
       <c r="J27" t="str">
-        <v>Campbell, Neil</v>
+        <v>Lindsay (NL), Martha</v>
       </c>
       <c r="K27">
         <v>3</v>
@@ -8808,10 +8808,10 @@
         <v>3</v>
       </c>
       <c r="O27">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P27" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q27">
         <v>3</v>
@@ -8820,13 +8820,13 @@
         <v>60</v>
       </c>
       <c r="S27" t="str">
-        <v>Brown, Christine</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T27">
         <v>3</v>
       </c>
       <c r="U27">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="28">
@@ -8849,22 +8849,22 @@
         <v>4.75</v>
       </c>
       <c r="G28" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H28">
         <v>1</v>
       </c>
       <c r="I28">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J28" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K28">
         <v>1</v>
       </c>
       <c r="L28">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M28" t="str">
         <v>Clements (NL), Jessie</v>
@@ -8873,16 +8873,16 @@
         <v>1</v>
       </c>
       <c r="O28">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P28" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q28">
         <v>1</v>
       </c>
       <c r="R28">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S28" t="str">
         <v>McInnes (NL), James</v>
@@ -8914,22 +8914,22 @@
         <v>6</v>
       </c>
       <c r="G29" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H29">
         <v>2</v>
       </c>
       <c r="I29">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J29" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K29">
         <v>2</v>
       </c>
       <c r="L29">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M29" t="str">
         <v>Clements (NL), Jessie</v>
@@ -8997,22 +8997,22 @@
         <v>60</v>
       </c>
       <c r="M30" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="N30">
         <v>2</v>
       </c>
       <c r="O30">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P30" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q30">
         <v>2</v>
       </c>
       <c r="R30">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S30" t="str">
         <v>McInnes (NL), James</v>
@@ -9053,7 +9053,7 @@
         <v>120</v>
       </c>
       <c r="J31" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Gibb (NL), Irene</v>
       </c>
       <c r="K31">
         <v>5</v>
@@ -9062,7 +9062,7 @@
         <v>60</v>
       </c>
       <c r="M31" t="str">
-        <v>Gibb (NL), Irene</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="N31">
         <v>5</v>
@@ -9071,7 +9071,7 @@
         <v>60</v>
       </c>
       <c r="P31" t="str">
-        <v>Brown, Christine</v>
+        <v>Lindsay (NL), Martha</v>
       </c>
       <c r="Q31">
         <v>5</v>
@@ -9080,7 +9080,7 @@
         <v>60</v>
       </c>
       <c r="S31" t="str">
-        <v>Lindsay (NL), Martha</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="T31">
         <v>5</v>
@@ -9109,22 +9109,22 @@
         <v>6</v>
       </c>
       <c r="G32" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H32">
         <v>1</v>
       </c>
       <c r="I32">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J32" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K32">
         <v>1</v>
       </c>
       <c r="L32">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M32" t="str">
         <v>Clements (NL), Jessie</v>
@@ -9201,22 +9201,22 @@
         <v>60</v>
       </c>
       <c r="P33" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="Q33">
         <v>4</v>
       </c>
       <c r="R33">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S33" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T33">
         <v>4</v>
       </c>
       <c r="U33">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34">
@@ -9239,22 +9239,22 @@
         <v>9</v>
       </c>
       <c r="G34" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H34">
         <v>1</v>
       </c>
       <c r="I34">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J34" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K34">
         <v>1</v>
       </c>
       <c r="L34">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M34" t="str">
         <v>Clements (NL), Jessie</v>
@@ -9304,22 +9304,22 @@
         <v>4</v>
       </c>
       <c r="G35" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H35">
         <v>1</v>
       </c>
       <c r="I35">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J35" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K35">
         <v>1</v>
       </c>
       <c r="L35">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M35" t="str">
         <v>Clements (NL), Jessie</v>
@@ -9328,25 +9328,25 @@
         <v>1</v>
       </c>
       <c r="O35">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P35" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q35">
         <v>1</v>
       </c>
       <c r="R35">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S35" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Russell (NL), Julia</v>
       </c>
       <c r="T35">
         <v>4</v>
       </c>
       <c r="U35">
-        <v>60</v>
+        <v>285</v>
       </c>
     </row>
     <row r="36">
@@ -9369,7 +9369,7 @@
         <v>8</v>
       </c>
       <c r="G36" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="H36">
         <v>13</v>
@@ -9396,7 +9396,7 @@
         <v>60</v>
       </c>
       <c r="P36" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="Q36">
         <v>13</v>
@@ -9405,7 +9405,7 @@
         <v>60</v>
       </c>
       <c r="S36" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="T36">
         <v>13</v>
@@ -9434,7 +9434,7 @@
         <v>2</v>
       </c>
       <c r="G37" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="H37">
         <v>4</v>
@@ -9461,7 +9461,7 @@
         <v>60</v>
       </c>
       <c r="P37" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="Q37">
         <v>4</v>
@@ -9470,7 +9470,7 @@
         <v>60</v>
       </c>
       <c r="S37" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="T37">
         <v>4</v>
@@ -9535,7 +9535,7 @@
         <v>60</v>
       </c>
       <c r="S38" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="T38">
         <v>6</v>
@@ -9564,7 +9564,7 @@
         <v>3</v>
       </c>
       <c r="G39" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H39">
         <v>1</v>
@@ -9573,7 +9573,7 @@
         <v>60</v>
       </c>
       <c r="J39" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K39">
         <v>1</v>
@@ -9591,7 +9591,7 @@
         <v>60</v>
       </c>
       <c r="P39" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q39">
         <v>1</v>
@@ -9629,7 +9629,7 @@
         <v>7.75</v>
       </c>
       <c r="G40" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H40">
         <v>2</v>
@@ -9638,7 +9638,7 @@
         <v>60</v>
       </c>
       <c r="J40" t="str">
-        <v>Collie, Mattie</v>
+        <v>Whyte, Jean</v>
       </c>
       <c r="K40">
         <v>2</v>
@@ -9647,7 +9647,7 @@
         <v>60</v>
       </c>
       <c r="M40" t="str">
-        <v>Whyte, Jean</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N40">
         <v>2</v>
@@ -9712,7 +9712,7 @@
         <v>60</v>
       </c>
       <c r="M41" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="N41">
         <v>2</v>
@@ -9721,7 +9721,7 @@
         <v>60</v>
       </c>
       <c r="P41" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q41">
         <v>2</v>
@@ -9851,7 +9851,7 @@
         <v>60</v>
       </c>
       <c r="P43" t="str">
-        <v>Murray (NL), James</v>
+        <v>Morris, Jack</v>
       </c>
       <c r="Q43">
         <v>18</v>
@@ -9860,7 +9860,7 @@
         <v>60</v>
       </c>
       <c r="S43" t="str">
-        <v>Morris, Jack</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="T43">
         <v>18</v>
@@ -9889,7 +9889,7 @@
         <v>10</v>
       </c>
       <c r="G44" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H44">
         <v>1</v>
@@ -9898,7 +9898,7 @@
         <v>60</v>
       </c>
       <c r="J44" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K44">
         <v>1</v>
@@ -9907,7 +9907,7 @@
         <v>60</v>
       </c>
       <c r="M44" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Whyte, Jean</v>
       </c>
       <c r="N44">
         <v>2</v>
@@ -9925,7 +9925,7 @@
         <v>60</v>
       </c>
       <c r="S44" t="str">
-        <v>Whyte, Jean</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="T44">
         <v>2</v>
@@ -9972,7 +9972,7 @@
         <v>60</v>
       </c>
       <c r="M45" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="N45">
         <v>4</v>
@@ -9981,7 +9981,7 @@
         <v>60</v>
       </c>
       <c r="P45" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q45">
         <v>4</v>
@@ -10046,7 +10046,7 @@
         <v>60</v>
       </c>
       <c r="P46" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="Q46">
         <v>15</v>
@@ -10084,7 +10084,7 @@
         <v>3</v>
       </c>
       <c r="G47" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H47">
         <v>1</v>
@@ -10093,7 +10093,7 @@
         <v>60</v>
       </c>
       <c r="J47" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K47">
         <v>1</v>
@@ -10111,7 +10111,7 @@
         <v>60</v>
       </c>
       <c r="P47" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q47">
         <v>1</v>
@@ -10149,7 +10149,7 @@
         <v>5</v>
       </c>
       <c r="G48" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="H48">
         <v>13</v>
@@ -10176,7 +10176,7 @@
         <v>60</v>
       </c>
       <c r="P48" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="Q48">
         <v>13</v>
@@ -10214,7 +10214,7 @@
         <v>6</v>
       </c>
       <c r="G49" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="H49">
         <v>4</v>
@@ -10241,7 +10241,7 @@
         <v>60</v>
       </c>
       <c r="P49" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="Q49">
         <v>4</v>
@@ -10279,25 +10279,25 @@
         <v>8</v>
       </c>
       <c r="G50" t="str">
-        <v>Murray (NL), James</v>
+        <v>Robertson (NL), Doreen</v>
       </c>
       <c r="H50">
         <v>8</v>
       </c>
       <c r="I50">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J50" t="str">
-        <v>Robertson (NL), Doreen</v>
+        <v>Morris, Jack</v>
       </c>
       <c r="K50">
         <v>8</v>
       </c>
       <c r="L50">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M50" t="str">
-        <v>Morris, Jack</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="N50">
         <v>8</v>
@@ -10315,7 +10315,7 @@
         <v>60</v>
       </c>
       <c r="S50" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret</v>
       </c>
       <c r="T50">
         <v>11</v>
@@ -10344,7 +10344,7 @@
         <v>9</v>
       </c>
       <c r="G51" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H51">
         <v>1</v>
@@ -10353,7 +10353,7 @@
         <v>60</v>
       </c>
       <c r="J51" t="str">
-        <v>Collie, Mattie</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="K51">
         <v>1</v>
@@ -10362,7 +10362,7 @@
         <v>60</v>
       </c>
       <c r="M51" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="N51">
         <v>1</v>
@@ -10492,7 +10492,7 @@
         <v>60</v>
       </c>
       <c r="M53" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="N53">
         <v>15</v>
@@ -10501,7 +10501,7 @@
         <v>60</v>
       </c>
       <c r="P53" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q53">
         <v>15</v>
@@ -10539,7 +10539,7 @@
         <v>9</v>
       </c>
       <c r="G54" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Whyte, Jean</v>
       </c>
       <c r="H54">
         <v>1</v>
@@ -10548,7 +10548,7 @@
         <v>60</v>
       </c>
       <c r="J54" t="str">
-        <v>Whyte, Jean</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="K54">
         <v>1</v>
@@ -10575,13 +10575,13 @@
         <v>60</v>
       </c>
       <c r="S54" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Pedrick, Michael</v>
       </c>
       <c r="T54">
         <v>6</v>
       </c>
       <c r="U54">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="55">
@@ -10622,7 +10622,7 @@
         <v>60</v>
       </c>
       <c r="M55" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret</v>
       </c>
       <c r="N55">
         <v>11</v>
@@ -10631,16 +10631,16 @@
         <v>60</v>
       </c>
       <c r="P55" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret</v>
       </c>
       <c r="Q55">
         <v>11</v>
       </c>
       <c r="R55">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S55" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T55">
         <v>11</v>
@@ -10669,22 +10669,22 @@
         <v>5.75</v>
       </c>
       <c r="G56" t="str">
-        <v>Scott (NL), Edith</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="H56">
         <v>1</v>
       </c>
       <c r="I56">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J56" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott (NL), Edith</v>
       </c>
       <c r="K56">
         <v>1</v>
       </c>
       <c r="L56">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M56" t="str">
         <v>Barrons (NL/HCAH), Shirley</v>
@@ -10705,7 +10705,7 @@
         <v>60</v>
       </c>
       <c r="S56" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="T56">
         <v>6</v>
@@ -10752,7 +10752,7 @@
         <v>60</v>
       </c>
       <c r="M57" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="N57">
         <v>2</v>
@@ -10767,16 +10767,16 @@
         <v>2</v>
       </c>
       <c r="R57">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="S57" t="str">
-        <v>Collie, Mattie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T57">
         <v>2</v>
       </c>
       <c r="U57">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="58">
@@ -10817,7 +10817,7 @@
         <v>285</v>
       </c>
       <c r="M58" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="N58">
         <v>5</v>
@@ -10826,7 +10826,7 @@
         <v>60</v>
       </c>
       <c r="P58" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="Q58">
         <v>5</v>
@@ -10864,7 +10864,7 @@
         <v>6.75</v>
       </c>
       <c r="G59" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="H59">
         <v>10</v>
@@ -10873,16 +10873,16 @@
         <v>60</v>
       </c>
       <c r="J59" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="K59">
         <v>10</v>
       </c>
       <c r="L59">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="M59" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="N59">
         <v>10</v>
@@ -10891,7 +10891,7 @@
         <v>60</v>
       </c>
       <c r="P59" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="Q59">
         <v>10</v>
@@ -10900,7 +10900,7 @@
         <v>60</v>
       </c>
       <c r="S59" t="str">
-        <v>Murray (NL), James</v>
+        <v>Kennedy (NL), Roberta</v>
       </c>
       <c r="T59">
         <v>10</v>
@@ -10956,7 +10956,7 @@
         <v>60</v>
       </c>
       <c r="P60" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="Q60">
         <v>4</v>
@@ -10971,7 +10971,7 @@
         <v>4</v>
       </c>
       <c r="U60">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="61">
@@ -11068,7 +11068,7 @@
         <v>480</v>
       </c>
       <c r="J62" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="K62">
         <v>15</v>
@@ -11086,7 +11086,7 @@
         <v>60</v>
       </c>
       <c r="P62" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q62">
         <v>15</v>
@@ -11124,7 +11124,7 @@
         <v>3</v>
       </c>
       <c r="G63" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie</v>
       </c>
       <c r="H63">
         <v>1</v>
@@ -11139,16 +11139,16 @@
         <v>1</v>
       </c>
       <c r="L63">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="M63" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N63">
         <v>1</v>
       </c>
       <c r="O63">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="P63" t="str">
         <v>Clements (NL), Jessie</v>
@@ -11160,7 +11160,7 @@
         <v>60</v>
       </c>
       <c r="S63" t="str">
-        <v>Collie, Mattie</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="T63">
         <v>1</v>
@@ -11254,7 +11254,7 @@
         <v>7</v>
       </c>
       <c r="G65" t="str">
-        <v>Murray (NL), James</v>
+        <v>Morris, Jack</v>
       </c>
       <c r="H65">
         <v>8</v>
@@ -11263,7 +11263,7 @@
         <v>60</v>
       </c>
       <c r="J65" t="str">
-        <v>Morris, Jack</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="K65">
         <v>8</v>
@@ -11281,7 +11281,7 @@
         <v>60</v>
       </c>
       <c r="P65" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret</v>
       </c>
       <c r="Q65">
         <v>11</v>
@@ -11290,7 +11290,7 @@
         <v>60</v>
       </c>
       <c r="S65" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret</v>
       </c>
       <c r="T65">
         <v>11</v>
@@ -11393,7 +11393,7 @@
         <v>120</v>
       </c>
       <c r="J67" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="K67">
         <v>3</v>
@@ -11402,7 +11402,7 @@
         <v>60</v>
       </c>
       <c r="M67" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="N67">
         <v>3</v>
@@ -11411,7 +11411,7 @@
         <v>60</v>
       </c>
       <c r="P67" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="Q67">
         <v>3</v>
@@ -11420,7 +11420,7 @@
         <v>60</v>
       </c>
       <c r="S67" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="T67">
         <v>3</v>
@@ -11514,7 +11514,7 @@
         <v>6</v>
       </c>
       <c r="G69" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="H69">
         <v>8</v>
@@ -11523,7 +11523,7 @@
         <v>60</v>
       </c>
       <c r="J69" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="K69">
         <v>8</v>
@@ -11532,7 +11532,7 @@
         <v>60</v>
       </c>
       <c r="M69" t="str">
-        <v>Murray (NL), James</v>
+        <v>Morris, Jack</v>
       </c>
       <c r="N69">
         <v>9</v>
@@ -11541,7 +11541,7 @@
         <v>60</v>
       </c>
       <c r="P69" t="str">
-        <v>Campbell, Neil</v>
+        <v>Murray (NL), James</v>
       </c>
       <c r="Q69">
         <v>9</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update capacity dashboard with latest scheduling information
Update capacity_dashboard.xlsx with new data relevant to employee scheduling and visit feasibility.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -7195,13 +7195,13 @@
         <v>60</v>
       </c>
       <c r="S2" t="str">
-        <v>Bryce (NL), Angela</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="T2">
         <v>11</v>
       </c>
       <c r="U2">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
@@ -7298,7 +7298,7 @@
         <v>120</v>
       </c>
       <c r="J4" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="K4">
         <v>1</v>
@@ -7313,16 +7313,16 @@
         <v>1</v>
       </c>
       <c r="O4">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P4" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="Q4">
         <v>1</v>
       </c>
       <c r="R4">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S4" t="str">
         <v>Whyte, Jean</v>
@@ -7437,7 +7437,7 @@
         <v>120</v>
       </c>
       <c r="M6" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="N6">
         <v>5</v>
@@ -7446,7 +7446,7 @@
         <v>60</v>
       </c>
       <c r="P6" t="str">
-        <v>Lindsay (NL), Martha</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="Q6">
         <v>5</v>
@@ -7455,7 +7455,7 @@
         <v>60</v>
       </c>
       <c r="S6" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Lindsay (NL), Martha</v>
       </c>
       <c r="T6">
         <v>5</v>
@@ -7715,7 +7715,7 @@
         <v>60</v>
       </c>
       <c r="S10" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="T10">
         <v>15</v>
@@ -7753,7 +7753,7 @@
         <v>120</v>
       </c>
       <c r="J11" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="K11">
         <v>1</v>
@@ -7768,16 +7768,16 @@
         <v>1</v>
       </c>
       <c r="O11">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P11" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="Q11">
         <v>1</v>
       </c>
       <c r="R11">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S11" t="str">
         <v>Whyte, Jean</v>
@@ -7818,7 +7818,7 @@
         <v>510</v>
       </c>
       <c r="J12" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="K12">
         <v>13</v>
@@ -7827,7 +7827,7 @@
         <v>60</v>
       </c>
       <c r="M12" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="N12">
         <v>13</v>
@@ -7874,7 +7874,7 @@
         <v>3</v>
       </c>
       <c r="G13" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="H13">
         <v>4</v>
@@ -7883,7 +7883,7 @@
         <v>60</v>
       </c>
       <c r="J13" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="K13">
         <v>4</v>
@@ -7910,7 +7910,7 @@
         <v>60</v>
       </c>
       <c r="S13" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="T13">
         <v>4</v>
@@ -8087,7 +8087,7 @@
         <v>60</v>
       </c>
       <c r="M16" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="N16">
         <v>3</v>
@@ -8096,7 +8096,7 @@
         <v>60</v>
       </c>
       <c r="P16" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="Q16">
         <v>3</v>
@@ -8199,22 +8199,22 @@
         <v>4.5</v>
       </c>
       <c r="G18" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="H18">
         <v>5</v>
       </c>
       <c r="I18">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J18" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="K18">
         <v>5</v>
       </c>
       <c r="L18">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M18" t="str">
         <v>Campbell, Neil</v>
@@ -8412,7 +8412,7 @@
         <v>60</v>
       </c>
       <c r="M21" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="N21">
         <v>3</v>
@@ -8421,7 +8421,7 @@
         <v>60</v>
       </c>
       <c r="P21" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="Q21">
         <v>3</v>
@@ -8486,7 +8486,7 @@
         <v>60</v>
       </c>
       <c r="P22" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q22">
         <v>15</v>
@@ -8560,13 +8560,13 @@
         <v>60</v>
       </c>
       <c r="S23" t="str">
-        <v>Russell (NL), Julia</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="T23">
         <v>4</v>
       </c>
       <c r="U23">
-        <v>285</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24">
@@ -8607,7 +8607,7 @@
         <v>120</v>
       </c>
       <c r="M24" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="N24">
         <v>13</v>
@@ -8616,7 +8616,7 @@
         <v>60</v>
       </c>
       <c r="P24" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q24">
         <v>13</v>
@@ -8625,7 +8625,7 @@
         <v>60</v>
       </c>
       <c r="S24" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="T24">
         <v>13</v>
@@ -8654,7 +8654,7 @@
         <v>5</v>
       </c>
       <c r="G25" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="H25">
         <v>4</v>
@@ -8663,7 +8663,7 @@
         <v>60</v>
       </c>
       <c r="J25" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="K25">
         <v>4</v>
@@ -8672,16 +8672,16 @@
         <v>60</v>
       </c>
       <c r="M25" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Gray (NL), Mary</v>
       </c>
       <c r="N25">
         <v>4</v>
       </c>
       <c r="O25">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P25" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="Q25">
         <v>4</v>
@@ -8690,7 +8690,7 @@
         <v>60</v>
       </c>
       <c r="S25" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="T25">
         <v>4</v>
@@ -8719,22 +8719,22 @@
         <v>4</v>
       </c>
       <c r="G26" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott (NL), Edith</v>
       </c>
       <c r="H26">
         <v>1</v>
       </c>
       <c r="I26">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="J26" t="str">
-        <v>Scott (NL), Edith</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="K26">
         <v>1</v>
       </c>
       <c r="L26">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="M26" t="str">
         <v>Grant (NL), Helen</v>
@@ -8784,7 +8784,7 @@
         <v>3</v>
       </c>
       <c r="G27" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="H27">
         <v>3</v>
@@ -8793,7 +8793,7 @@
         <v>60</v>
       </c>
       <c r="J27" t="str">
-        <v>Lindsay (NL), Martha</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="K27">
         <v>3</v>
@@ -8817,16 +8817,16 @@
         <v>3</v>
       </c>
       <c r="R27">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S27" t="str">
-        <v>Campbell, Neil</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="T27">
         <v>3</v>
       </c>
       <c r="U27">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28">
@@ -8932,16 +8932,16 @@
         <v>60</v>
       </c>
       <c r="M29" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="N29">
         <v>3</v>
       </c>
       <c r="O29">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P29" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="Q29">
         <v>3</v>
@@ -8950,13 +8950,13 @@
         <v>60</v>
       </c>
       <c r="S29" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="T29">
         <v>3</v>
       </c>
       <c r="U29">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30">
@@ -9053,7 +9053,7 @@
         <v>120</v>
       </c>
       <c r="J31" t="str">
-        <v>Gibb (NL), Irene</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="K31">
         <v>5</v>
@@ -9062,7 +9062,7 @@
         <v>60</v>
       </c>
       <c r="M31" t="str">
-        <v>Brown, Christine</v>
+        <v>Gibb (NL), Irene</v>
       </c>
       <c r="N31">
         <v>5</v>
@@ -9071,7 +9071,7 @@
         <v>60</v>
       </c>
       <c r="P31" t="str">
-        <v>Lindsay (NL), Martha</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="Q31">
         <v>5</v>
@@ -9080,7 +9080,7 @@
         <v>60</v>
       </c>
       <c r="S31" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Lindsay (NL), Martha</v>
       </c>
       <c r="T31">
         <v>5</v>
@@ -9257,16 +9257,16 @@
         <v>60</v>
       </c>
       <c r="M34" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="N34">
         <v>3</v>
       </c>
       <c r="O34">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P34" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="Q34">
         <v>3</v>
@@ -9275,13 +9275,13 @@
         <v>60</v>
       </c>
       <c r="S34" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="T34">
         <v>3</v>
       </c>
       <c r="U34">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="35">
@@ -9340,13 +9340,13 @@
         <v>60</v>
       </c>
       <c r="S35" t="str">
-        <v>Russell (NL), Julia</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="T35">
         <v>4</v>
       </c>
       <c r="U35">
-        <v>285</v>
+        <v>60</v>
       </c>
     </row>
     <row r="36">
@@ -9369,7 +9369,7 @@
         <v>8</v>
       </c>
       <c r="G36" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="H36">
         <v>13</v>
@@ -9396,7 +9396,7 @@
         <v>60</v>
       </c>
       <c r="P36" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q36">
         <v>13</v>
@@ -9405,7 +9405,7 @@
         <v>60</v>
       </c>
       <c r="S36" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="T36">
         <v>13</v>
@@ -9434,7 +9434,7 @@
         <v>2</v>
       </c>
       <c r="G37" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="H37">
         <v>4</v>
@@ -9461,7 +9461,7 @@
         <v>60</v>
       </c>
       <c r="P37" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q37">
         <v>4</v>
@@ -9470,7 +9470,7 @@
         <v>60</v>
       </c>
       <c r="S37" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="T37">
         <v>4</v>
@@ -9535,7 +9535,7 @@
         <v>60</v>
       </c>
       <c r="S38" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="T38">
         <v>6</v>
@@ -9656,7 +9656,7 @@
         <v>60</v>
       </c>
       <c r="P40" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="Q40">
         <v>3</v>
@@ -9665,7 +9665,7 @@
         <v>60</v>
       </c>
       <c r="S40" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="T40">
         <v>3</v>
@@ -10046,7 +10046,7 @@
         <v>60</v>
       </c>
       <c r="P46" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q46">
         <v>15</v>
@@ -10149,7 +10149,7 @@
         <v>5</v>
       </c>
       <c r="G48" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="H48">
         <v>13</v>
@@ -10158,7 +10158,7 @@
         <v>60</v>
       </c>
       <c r="J48" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="K48">
         <v>13</v>
@@ -10167,7 +10167,7 @@
         <v>60</v>
       </c>
       <c r="M48" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="N48">
         <v>13</v>
@@ -10176,7 +10176,7 @@
         <v>60</v>
       </c>
       <c r="P48" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="Q48">
         <v>13</v>
@@ -10185,7 +10185,7 @@
         <v>60</v>
       </c>
       <c r="S48" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="T48">
         <v>13</v>
@@ -10214,7 +10214,7 @@
         <v>6</v>
       </c>
       <c r="G49" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="H49">
         <v>4</v>
@@ -10223,7 +10223,7 @@
         <v>60</v>
       </c>
       <c r="J49" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="K49">
         <v>4</v>
@@ -10232,7 +10232,7 @@
         <v>60</v>
       </c>
       <c r="M49" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="N49">
         <v>4</v>
@@ -10241,7 +10241,7 @@
         <v>60</v>
       </c>
       <c r="P49" t="str">
-        <v>O'Brien (NL), Josephine</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="Q49">
         <v>4</v>
@@ -10250,7 +10250,7 @@
         <v>60</v>
       </c>
       <c r="S49" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>O'Brien (NL), Josephine</v>
       </c>
       <c r="T49">
         <v>4</v>
@@ -10315,7 +10315,7 @@
         <v>60</v>
       </c>
       <c r="S50" t="str">
-        <v>Anderson, Margaret</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="T50">
         <v>11</v>
@@ -10353,7 +10353,7 @@
         <v>60</v>
       </c>
       <c r="J51" t="str">
-        <v>Duffy, Sarah Anne (goes by Anne)</v>
+        <v>Clements (NL), Jessie</v>
       </c>
       <c r="K51">
         <v>1</v>
@@ -10362,7 +10362,7 @@
         <v>60</v>
       </c>
       <c r="M51" t="str">
-        <v>Clements (NL), Jessie</v>
+        <v>Duffy, Sarah Anne (goes by Anne)</v>
       </c>
       <c r="N51">
         <v>1</v>
@@ -10492,7 +10492,7 @@
         <v>60</v>
       </c>
       <c r="M53" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="N53">
         <v>15</v>
@@ -10501,7 +10501,7 @@
         <v>60</v>
       </c>
       <c r="P53" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="Q53">
         <v>15</v>
@@ -10539,7 +10539,7 @@
         <v>9</v>
       </c>
       <c r="G54" t="str">
-        <v>Whyte, Jean</v>
+        <v>Mullen (NL), Eileen</v>
       </c>
       <c r="H54">
         <v>1</v>
@@ -10548,7 +10548,7 @@
         <v>60</v>
       </c>
       <c r="J54" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Whyte, Jean</v>
       </c>
       <c r="K54">
         <v>1</v>
@@ -10622,7 +10622,7 @@
         <v>60</v>
       </c>
       <c r="M55" t="str">
-        <v>Anderson, Margaret</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="N55">
         <v>11</v>
@@ -10631,7 +10631,7 @@
         <v>60</v>
       </c>
       <c r="P55" t="str">
-        <v>Anderson, Margaret</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q55">
         <v>11</v>
@@ -10646,7 +10646,7 @@
         <v>11</v>
       </c>
       <c r="U55">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="56">
@@ -10669,22 +10669,22 @@
         <v>5.75</v>
       </c>
       <c r="G56" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott (NL), Edith</v>
       </c>
       <c r="H56">
         <v>1</v>
       </c>
       <c r="I56">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J56" t="str">
-        <v>Scott (NL), Edith</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="K56">
         <v>1</v>
       </c>
       <c r="L56">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M56" t="str">
         <v>Barrons (NL/HCAH), Shirley</v>
@@ -10705,7 +10705,7 @@
         <v>60</v>
       </c>
       <c r="S56" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="T56">
         <v>6</v>
@@ -10817,7 +10817,7 @@
         <v>285</v>
       </c>
       <c r="M58" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="N58">
         <v>5</v>
@@ -10826,7 +10826,7 @@
         <v>60</v>
       </c>
       <c r="P58" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="Q58">
         <v>5</v>
@@ -10864,7 +10864,7 @@
         <v>6.75</v>
       </c>
       <c r="G59" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Barrons (NL/HCAH), Shirley</v>
       </c>
       <c r="H59">
         <v>10</v>
@@ -10873,7 +10873,7 @@
         <v>60</v>
       </c>
       <c r="J59" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Barrons (NL/HCAH), Shirley</v>
       </c>
       <c r="K59">
         <v>10</v>
@@ -10882,7 +10882,7 @@
         <v>60</v>
       </c>
       <c r="M59" t="str">
-        <v>Mullen (NL), Eileen</v>
+        <v>Lynch (NL), Roselyn</v>
       </c>
       <c r="N59">
         <v>10</v>
@@ -10891,7 +10891,7 @@
         <v>60</v>
       </c>
       <c r="P59" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="Q59">
         <v>10</v>
@@ -10900,7 +10900,7 @@
         <v>60</v>
       </c>
       <c r="S59" t="str">
-        <v>Kennedy (NL), Roberta</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="T59">
         <v>10</v>
@@ -11068,7 +11068,7 @@
         <v>480</v>
       </c>
       <c r="J62" t="str">
-        <v>McIntyre (NL), Donald</v>
+        <v>Munro (NL), Alistair</v>
       </c>
       <c r="K62">
         <v>15</v>
@@ -11086,7 +11086,7 @@
         <v>60</v>
       </c>
       <c r="P62" t="str">
-        <v>Munro (NL), Alistair</v>
+        <v>McIntyre (NL), Donald</v>
       </c>
       <c r="Q62">
         <v>15</v>
@@ -11281,7 +11281,7 @@
         <v>60</v>
       </c>
       <c r="P65" t="str">
-        <v>Anderson, Margaret</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="Q65">
         <v>11</v>
@@ -11290,7 +11290,7 @@
         <v>60</v>
       </c>
       <c r="S65" t="str">
-        <v>Anderson, Margaret</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T65">
         <v>11</v>
@@ -11514,7 +11514,7 @@
         <v>6</v>
       </c>
       <c r="G69" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty (NL), Elizabeth</v>
       </c>
       <c r="H69">
         <v>8</v>
@@ -11523,7 +11523,7 @@
         <v>60</v>
       </c>
       <c r="J69" t="str">
-        <v>Docherty (NL), Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="K69">
         <v>8</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update dashboard data to reflect current capacity
Update capacity dashboard data in the Excel file.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -7163,22 +7163,22 @@
         <v>6</v>
       </c>
       <c r="G2" t="str">
-        <v>Murray, James</v>
+        <v>Robertson, Doreen (F)</v>
       </c>
       <c r="H2">
         <v>8</v>
       </c>
       <c r="I2">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J2" t="str">
-        <v>Robertson, Doreen (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="K2">
         <v>8</v>
       </c>
       <c r="L2">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M2" t="str">
         <v>Brown, Christine</v>
@@ -7199,7 +7199,7 @@
         <v>60</v>
       </c>
       <c r="S2" t="str">
-        <v>Campbell, Neil</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="T2">
         <v>11</v>
@@ -7293,7 +7293,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -7302,16 +7302,16 @@
         <v>120</v>
       </c>
       <c r="J4" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Duffy, Sarah Anne (F)</v>
       </c>
       <c r="K4">
         <v>1</v>
       </c>
       <c r="L4">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M4" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N4">
         <v>1</v>
@@ -7320,13 +7320,13 @@
         <v>120</v>
       </c>
       <c r="P4" t="str">
-        <v>Duffy, Sarah Anne (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q4">
         <v>1</v>
       </c>
       <c r="R4">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S4" t="str">
         <v>Whyte, Jean (F)</v>
@@ -7506,13 +7506,13 @@
         <v>120</v>
       </c>
       <c r="M7" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="N7">
         <v>2</v>
       </c>
       <c r="O7">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P7" t="str">
         <v>Clements, Jessie (F)</v>
@@ -7521,10 +7521,10 @@
         <v>2</v>
       </c>
       <c r="R7">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S7" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T7">
         <v>2</v>
@@ -7645,13 +7645,13 @@
         <v>60</v>
       </c>
       <c r="P9" t="str">
-        <v>Campbell, Neil</v>
+        <v>Robertson, Doreen (F)</v>
       </c>
       <c r="Q9">
         <v>7</v>
       </c>
       <c r="R9">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S9" t="str">
         <v>Campbell, Neil</v>
@@ -7748,7 +7748,7 @@
         <v>3</v>
       </c>
       <c r="G11" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -7757,16 +7757,16 @@
         <v>120</v>
       </c>
       <c r="J11" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Duffy, Sarah Anne (F)</v>
       </c>
       <c r="K11">
         <v>1</v>
       </c>
       <c r="L11">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M11" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N11">
         <v>1</v>
@@ -7775,13 +7775,13 @@
         <v>120</v>
       </c>
       <c r="P11" t="str">
-        <v>Duffy, Sarah Anne (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q11">
         <v>1</v>
       </c>
       <c r="R11">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S11" t="str">
         <v>Whyte, Jean (F)</v>
@@ -7822,7 +7822,7 @@
         <v>510</v>
       </c>
       <c r="J12" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="K12">
         <v>13</v>
@@ -7831,7 +7831,7 @@
         <v>60</v>
       </c>
       <c r="M12" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="N12">
         <v>13</v>
@@ -7840,7 +7840,7 @@
         <v>60</v>
       </c>
       <c r="P12" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="Q12">
         <v>13</v>
@@ -7878,7 +7878,7 @@
         <v>3</v>
       </c>
       <c r="G13" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="H13">
         <v>4</v>
@@ -7887,7 +7887,7 @@
         <v>60</v>
       </c>
       <c r="J13" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="K13">
         <v>4</v>
@@ -7896,7 +7896,7 @@
         <v>60</v>
       </c>
       <c r="M13" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="N13">
         <v>4</v>
@@ -7943,7 +7943,7 @@
         <v>4.75</v>
       </c>
       <c r="G14" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -7952,7 +7952,7 @@
         <v>60</v>
       </c>
       <c r="J14" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K14">
         <v>1</v>
@@ -7970,7 +7970,7 @@
         <v>60</v>
       </c>
       <c r="P14" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q14">
         <v>1</v>
@@ -8008,7 +8008,7 @@
         <v>6</v>
       </c>
       <c r="G15" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H15">
         <v>2</v>
@@ -8017,7 +8017,7 @@
         <v>60</v>
       </c>
       <c r="J15" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K15">
         <v>2</v>
@@ -8026,7 +8026,7 @@
         <v>60</v>
       </c>
       <c r="M15" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="N15">
         <v>3</v>
@@ -8035,7 +8035,7 @@
         <v>60</v>
       </c>
       <c r="P15" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="Q15">
         <v>3</v>
@@ -8091,7 +8091,7 @@
         <v>60</v>
       </c>
       <c r="M16" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N16">
         <v>2</v>
@@ -8100,7 +8100,7 @@
         <v>60</v>
       </c>
       <c r="P16" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q16">
         <v>2</v>
@@ -8203,7 +8203,7 @@
         <v>8</v>
       </c>
       <c r="G18" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H18">
         <v>1</v>
@@ -8212,7 +8212,7 @@
         <v>60</v>
       </c>
       <c r="J18" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K18">
         <v>1</v>
@@ -8295,7 +8295,7 @@
         <v>120</v>
       </c>
       <c r="P19" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q19">
         <v>4</v>
@@ -8304,7 +8304,7 @@
         <v>60</v>
       </c>
       <c r="S19" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T19">
         <v>4</v>
@@ -8333,7 +8333,7 @@
         <v>4</v>
       </c>
       <c r="G20" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -8342,7 +8342,7 @@
         <v>60</v>
       </c>
       <c r="J20" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K20">
         <v>1</v>
@@ -8351,7 +8351,7 @@
         <v>60</v>
       </c>
       <c r="M20" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="N20">
         <v>3</v>
@@ -8360,7 +8360,7 @@
         <v>60</v>
       </c>
       <c r="P20" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="Q20">
         <v>3</v>
@@ -8463,7 +8463,7 @@
         <v>5</v>
       </c>
       <c r="G22" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H22">
         <v>1</v>
@@ -8472,7 +8472,7 @@
         <v>60</v>
       </c>
       <c r="J22" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K22">
         <v>1</v>
@@ -8490,7 +8490,7 @@
         <v>60</v>
       </c>
       <c r="P22" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q22">
         <v>1</v>
@@ -8537,7 +8537,7 @@
         <v>180</v>
       </c>
       <c r="J23" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="K23">
         <v>13</v>
@@ -8546,7 +8546,7 @@
         <v>60</v>
       </c>
       <c r="M23" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="N23">
         <v>13</v>
@@ -8555,7 +8555,7 @@
         <v>60</v>
       </c>
       <c r="P23" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="Q23">
         <v>13</v>
@@ -8564,7 +8564,7 @@
         <v>60</v>
       </c>
       <c r="S23" t="str">
-        <v>Munro, Alistair</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="T23">
         <v>13</v>
@@ -8593,7 +8593,7 @@
         <v>5</v>
       </c>
       <c r="G24" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="H24">
         <v>4</v>
@@ -8602,7 +8602,7 @@
         <v>60</v>
       </c>
       <c r="J24" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="K24">
         <v>4</v>
@@ -8611,7 +8611,7 @@
         <v>60</v>
       </c>
       <c r="M24" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="N24">
         <v>4</v>
@@ -8620,7 +8620,7 @@
         <v>60</v>
       </c>
       <c r="P24" t="str">
-        <v>Munro, Alistair</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="Q24">
         <v>4</v>
@@ -8629,7 +8629,7 @@
         <v>60</v>
       </c>
       <c r="S24" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="T24">
         <v>4</v>
@@ -8723,7 +8723,7 @@
         <v>3</v>
       </c>
       <c r="G26" t="str">
-        <v>Campbell, Neil</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="H26">
         <v>3</v>
@@ -8732,7 +8732,7 @@
         <v>60</v>
       </c>
       <c r="J26" t="str">
-        <v>Campbell, Neil</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="K26">
         <v>3</v>
@@ -8741,16 +8741,16 @@
         <v>60</v>
       </c>
       <c r="M26" t="str">
-        <v>Campbell, Neil</v>
+        <v>Lindsay, Martha (F)</v>
       </c>
       <c r="N26">
         <v>3</v>
       </c>
       <c r="O26">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P26" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q26">
         <v>3</v>
@@ -8759,7 +8759,7 @@
         <v>60</v>
       </c>
       <c r="S26" t="str">
-        <v>Brown, Christine</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T26">
         <v>3</v>
@@ -8788,13 +8788,13 @@
         <v>4.75</v>
       </c>
       <c r="G27" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H27">
         <v>1</v>
       </c>
       <c r="I27">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J27" t="str">
         <v>East NL, Glasgow</v>
@@ -8806,13 +8806,13 @@
         <v>60</v>
       </c>
       <c r="M27" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N27">
         <v>1</v>
       </c>
       <c r="O27">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P27" t="str">
         <v>Clements, Jessie (F)</v>
@@ -8821,16 +8821,16 @@
         <v>1</v>
       </c>
       <c r="R27">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S27" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T27">
         <v>1</v>
       </c>
       <c r="U27">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28">
@@ -8853,13 +8853,13 @@
         <v>6</v>
       </c>
       <c r="G28" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H28">
         <v>2</v>
       </c>
       <c r="I28">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J28" t="str">
         <v>East NL, Glasgow</v>
@@ -8871,25 +8871,25 @@
         <v>60</v>
       </c>
       <c r="M28" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N28">
         <v>2</v>
       </c>
       <c r="O28">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P28" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="Q28">
         <v>3</v>
       </c>
       <c r="R28">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S28" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="T28">
         <v>3</v>
@@ -8936,13 +8936,13 @@
         <v>60</v>
       </c>
       <c r="M29" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N29">
         <v>2</v>
       </c>
       <c r="O29">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P29" t="str">
         <v>East NL, Glasgow</v>
@@ -8954,13 +8954,13 @@
         <v>60</v>
       </c>
       <c r="S29" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T29">
         <v>2</v>
       </c>
       <c r="U29">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30">
@@ -9048,13 +9048,13 @@
         <v>6</v>
       </c>
       <c r="G31" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H31">
         <v>1</v>
       </c>
       <c r="I31">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J31" t="str">
         <v>East NL, Glasgow</v>
@@ -9066,13 +9066,13 @@
         <v>60</v>
       </c>
       <c r="M31" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N31">
         <v>1</v>
       </c>
       <c r="O31">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P31" t="str">
         <v>Clements, Jessie (F)</v>
@@ -9140,13 +9140,13 @@
         <v>60</v>
       </c>
       <c r="P32" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q32">
         <v>4</v>
       </c>
       <c r="R32">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S32" t="str">
         <v>East NL, Glasgow</v>
@@ -9178,13 +9178,13 @@
         <v>9</v>
       </c>
       <c r="G33" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H33">
         <v>1</v>
       </c>
       <c r="I33">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J33" t="str">
         <v>East NL, Glasgow</v>
@@ -9196,25 +9196,25 @@
         <v>60</v>
       </c>
       <c r="M33" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N33">
         <v>1</v>
       </c>
       <c r="O33">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P33" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="Q33">
         <v>3</v>
       </c>
       <c r="R33">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S33" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="T33">
         <v>3</v>
@@ -9243,13 +9243,13 @@
         <v>4</v>
       </c>
       <c r="G34" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H34">
         <v>1</v>
       </c>
       <c r="I34">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J34" t="str">
         <v>East NL, Glasgow</v>
@@ -9261,13 +9261,13 @@
         <v>60</v>
       </c>
       <c r="M34" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N34">
         <v>1</v>
       </c>
       <c r="O34">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P34" t="str">
         <v>Clements, Jessie (F)</v>
@@ -9276,16 +9276,16 @@
         <v>1</v>
       </c>
       <c r="R34">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S34" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T34">
         <v>1</v>
       </c>
       <c r="U34">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35">
@@ -9308,7 +9308,7 @@
         <v>8</v>
       </c>
       <c r="G35" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="H35">
         <v>13</v>
@@ -9317,7 +9317,7 @@
         <v>60</v>
       </c>
       <c r="J35" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="K35">
         <v>13</v>
@@ -9326,7 +9326,7 @@
         <v>60</v>
       </c>
       <c r="M35" t="str">
-        <v>Munro, Alistair</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="N35">
         <v>13</v>
@@ -9335,7 +9335,7 @@
         <v>60</v>
       </c>
       <c r="P35" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="Q35">
         <v>13</v>
@@ -9373,7 +9373,7 @@
         <v>2</v>
       </c>
       <c r="G36" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="H36">
         <v>4</v>
@@ -9382,7 +9382,7 @@
         <v>60</v>
       </c>
       <c r="J36" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="K36">
         <v>4</v>
@@ -9391,7 +9391,7 @@
         <v>60</v>
       </c>
       <c r="M36" t="str">
-        <v>Munro, Alistair</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="N36">
         <v>4</v>
@@ -9400,7 +9400,7 @@
         <v>60</v>
       </c>
       <c r="P36" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="Q36">
         <v>4</v>
@@ -9503,7 +9503,7 @@
         <v>3</v>
       </c>
       <c r="G38" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H38">
         <v>1</v>
@@ -9512,7 +9512,7 @@
         <v>60</v>
       </c>
       <c r="J38" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K38">
         <v>1</v>
@@ -9530,7 +9530,7 @@
         <v>60</v>
       </c>
       <c r="P38" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q38">
         <v>1</v>
@@ -9568,7 +9568,7 @@
         <v>7.75</v>
       </c>
       <c r="G39" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H39">
         <v>2</v>
@@ -9577,7 +9577,7 @@
         <v>60</v>
       </c>
       <c r="J39" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="K39">
         <v>2</v>
@@ -9586,7 +9586,7 @@
         <v>60</v>
       </c>
       <c r="M39" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N39">
         <v>2</v>
@@ -9595,7 +9595,7 @@
         <v>60</v>
       </c>
       <c r="P39" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="Q39">
         <v>3</v>
@@ -9604,7 +9604,7 @@
         <v>60</v>
       </c>
       <c r="S39" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="T39">
         <v>3</v>
@@ -9651,7 +9651,7 @@
         <v>60</v>
       </c>
       <c r="M40" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N40">
         <v>2</v>
@@ -9660,7 +9660,7 @@
         <v>60</v>
       </c>
       <c r="P40" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q40">
         <v>2</v>
@@ -9790,7 +9790,7 @@
         <v>60</v>
       </c>
       <c r="P42" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="Q42">
         <v>18</v>
@@ -9799,7 +9799,7 @@
         <v>60</v>
       </c>
       <c r="S42" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="T42">
         <v>18</v>
@@ -9828,7 +9828,7 @@
         <v>10</v>
       </c>
       <c r="G43" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H43">
         <v>1</v>
@@ -9837,7 +9837,7 @@
         <v>60</v>
       </c>
       <c r="J43" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K43">
         <v>1</v>
@@ -9846,7 +9846,7 @@
         <v>60</v>
       </c>
       <c r="M43" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="N43">
         <v>2</v>
@@ -9864,7 +9864,7 @@
         <v>60</v>
       </c>
       <c r="S43" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T43">
         <v>2</v>
@@ -9911,7 +9911,7 @@
         <v>60</v>
       </c>
       <c r="M44" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N44">
         <v>4</v>
@@ -9920,7 +9920,7 @@
         <v>60</v>
       </c>
       <c r="P44" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q44">
         <v>4</v>
@@ -10023,7 +10023,7 @@
         <v>3</v>
       </c>
       <c r="G46" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H46">
         <v>1</v>
@@ -10032,7 +10032,7 @@
         <v>60</v>
       </c>
       <c r="J46" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K46">
         <v>1</v>
@@ -10050,7 +10050,7 @@
         <v>60</v>
       </c>
       <c r="P46" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q46">
         <v>1</v>
@@ -10088,7 +10088,7 @@
         <v>5</v>
       </c>
       <c r="G47" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="H47">
         <v>13</v>
@@ -10097,7 +10097,7 @@
         <v>60</v>
       </c>
       <c r="J47" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="K47">
         <v>13</v>
@@ -10106,7 +10106,7 @@
         <v>60</v>
       </c>
       <c r="M47" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="N47">
         <v>13</v>
@@ -10115,7 +10115,7 @@
         <v>60</v>
       </c>
       <c r="P47" t="str">
-        <v>Munro, Alistair</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="Q47">
         <v>13</v>
@@ -10124,7 +10124,7 @@
         <v>60</v>
       </c>
       <c r="S47" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="T47">
         <v>13</v>
@@ -10153,7 +10153,7 @@
         <v>6</v>
       </c>
       <c r="G48" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="H48">
         <v>4</v>
@@ -10162,7 +10162,7 @@
         <v>60</v>
       </c>
       <c r="J48" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="K48">
         <v>4</v>
@@ -10171,7 +10171,7 @@
         <v>60</v>
       </c>
       <c r="M48" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="N48">
         <v>4</v>
@@ -10180,7 +10180,7 @@
         <v>60</v>
       </c>
       <c r="P48" t="str">
-        <v>Munro, Alistair</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="Q48">
         <v>4</v>
@@ -10189,7 +10189,7 @@
         <v>60</v>
       </c>
       <c r="S48" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="T48">
         <v>4</v>
@@ -10218,7 +10218,7 @@
         <v>8</v>
       </c>
       <c r="G49" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="H49">
         <v>8</v>
@@ -10227,7 +10227,7 @@
         <v>60</v>
       </c>
       <c r="J49" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="K49">
         <v>8</v>
@@ -10245,7 +10245,7 @@
         <v>60</v>
       </c>
       <c r="P49" t="str">
-        <v>Campbell, Neil</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="Q49">
         <v>11</v>
@@ -10254,7 +10254,7 @@
         <v>60</v>
       </c>
       <c r="S49" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="T49">
         <v>11</v>
@@ -10283,7 +10283,7 @@
         <v>9</v>
       </c>
       <c r="G50" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H50">
         <v>1</v>
@@ -10292,7 +10292,7 @@
         <v>60</v>
       </c>
       <c r="J50" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Duffy, Sarah Anne (F)</v>
       </c>
       <c r="K50">
         <v>1</v>
@@ -10301,7 +10301,7 @@
         <v>60</v>
       </c>
       <c r="M50" t="str">
-        <v>Duffy, Sarah Anne (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N50">
         <v>1</v>
@@ -10496,7 +10496,7 @@
         <v>60</v>
       </c>
       <c r="M53" t="str">
-        <v>Campbell, Neil</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="N53">
         <v>11</v>
@@ -10505,7 +10505,7 @@
         <v>60</v>
       </c>
       <c r="P53" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="Q53">
         <v>11</v>
@@ -10514,13 +10514,13 @@
         <v>60</v>
       </c>
       <c r="S53" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="T53">
         <v>11</v>
       </c>
       <c r="U53">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="54">
@@ -10626,7 +10626,7 @@
         <v>60</v>
       </c>
       <c r="M55" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N55">
         <v>2</v>
@@ -10635,7 +10635,7 @@
         <v>60</v>
       </c>
       <c r="P55" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q55">
         <v>2</v>
@@ -10738,7 +10738,7 @@
         <v>6.75</v>
       </c>
       <c r="G57" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Barrons, Shirley</v>
       </c>
       <c r="H57">
         <v>10</v>
@@ -10747,7 +10747,7 @@
         <v>60</v>
       </c>
       <c r="J57" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Barrons, Shirley</v>
       </c>
       <c r="K57">
         <v>10</v>
@@ -10756,7 +10756,7 @@
         <v>60</v>
       </c>
       <c r="M57" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Lynch, Roselyn (F)</v>
       </c>
       <c r="N57">
         <v>10</v>
@@ -10765,16 +10765,16 @@
         <v>60</v>
       </c>
       <c r="P57" t="str">
-        <v>Murray, James</v>
+        <v>Lynch, Roselyn (F)</v>
       </c>
       <c r="Q57">
         <v>10</v>
       </c>
       <c r="R57">
-        <v>60</v>
+        <v>285</v>
       </c>
       <c r="S57" t="str">
-        <v>Campbell, Neil</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="T57">
         <v>10</v>
@@ -10830,7 +10830,7 @@
         <v>60</v>
       </c>
       <c r="P58" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q58">
         <v>4</v>
@@ -10839,7 +10839,7 @@
         <v>60</v>
       </c>
       <c r="S58" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T58">
         <v>4</v>
@@ -10998,7 +10998,7 @@
         <v>3</v>
       </c>
       <c r="G61" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H61">
         <v>1</v>
@@ -11007,7 +11007,7 @@
         <v>60</v>
       </c>
       <c r="J61" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K61">
         <v>1</v>
@@ -11025,7 +11025,7 @@
         <v>60</v>
       </c>
       <c r="P61" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q61">
         <v>1</v>
@@ -11128,7 +11128,7 @@
         <v>7</v>
       </c>
       <c r="G63" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="H63">
         <v>8</v>
@@ -11137,7 +11137,7 @@
         <v>60</v>
       </c>
       <c r="J63" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="K63">
         <v>8</v>
@@ -11155,7 +11155,7 @@
         <v>60</v>
       </c>
       <c r="P63" t="str">
-        <v>Campbell, Neil</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="Q63">
         <v>11</v>
@@ -11164,7 +11164,7 @@
         <v>60</v>
       </c>
       <c r="S63" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="T63">
         <v>11</v>
@@ -11202,7 +11202,7 @@
         <v>120</v>
       </c>
       <c r="J64" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="K64">
         <v>3</v>
@@ -11220,7 +11220,7 @@
         <v>60</v>
       </c>
       <c r="P64" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q64">
         <v>3</v>
@@ -11294,7 +11294,7 @@
         <v>60</v>
       </c>
       <c r="S65" t="str">
-        <v>Campbell, Neil</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="T65">
         <v>17</v>
@@ -11341,7 +11341,7 @@
         <v>60</v>
       </c>
       <c r="M66" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="N66">
         <v>9</v>
@@ -11350,7 +11350,7 @@
         <v>60</v>
       </c>
       <c r="P66" t="str">
-        <v>Campbell, Neil</v>
+        <v>Murray, James</v>
       </c>
       <c r="Q66">
         <v>9</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update employee gender data for the dashboard
Update the capacity_dashboard.xlsx file with corrected employee gender data.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -7199,13 +7199,13 @@
         <v>60</v>
       </c>
       <c r="S2" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Bryce, Angela (F)</v>
       </c>
       <c r="T2">
         <v>11</v>
       </c>
       <c r="U2">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3">
@@ -7441,7 +7441,7 @@
         <v>120</v>
       </c>
       <c r="M6" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="N6">
         <v>5</v>
@@ -7450,7 +7450,7 @@
         <v>60</v>
       </c>
       <c r="P6" t="str">
-        <v>Brown, Christine</v>
+        <v>Lindsay, Martha (F)</v>
       </c>
       <c r="Q6">
         <v>5</v>
@@ -7459,7 +7459,7 @@
         <v>60</v>
       </c>
       <c r="S6" t="str">
-        <v>Lindsay, Martha (F)</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="T6">
         <v>5</v>
@@ -7701,7 +7701,7 @@
         <v>60</v>
       </c>
       <c r="M10" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="N10">
         <v>15</v>
@@ -7710,7 +7710,7 @@
         <v>60</v>
       </c>
       <c r="P10" t="str">
-        <v>McIntyre, Donald</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="Q10">
         <v>15</v>
@@ -7822,7 +7822,7 @@
         <v>510</v>
       </c>
       <c r="J12" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="K12">
         <v>13</v>
@@ -7831,7 +7831,7 @@
         <v>60</v>
       </c>
       <c r="M12" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="N12">
         <v>13</v>
@@ -7840,7 +7840,7 @@
         <v>60</v>
       </c>
       <c r="P12" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="Q12">
         <v>13</v>
@@ -7878,7 +7878,7 @@
         <v>3</v>
       </c>
       <c r="G13" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="H13">
         <v>4</v>
@@ -7887,7 +7887,7 @@
         <v>60</v>
       </c>
       <c r="J13" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="K13">
         <v>4</v>
@@ -7896,7 +7896,7 @@
         <v>60</v>
       </c>
       <c r="M13" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="N13">
         <v>4</v>
@@ -8026,7 +8026,7 @@
         <v>60</v>
       </c>
       <c r="M15" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N15">
         <v>3</v>
@@ -8035,7 +8035,7 @@
         <v>60</v>
       </c>
       <c r="P15" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q15">
         <v>3</v>
@@ -8138,22 +8138,22 @@
         <v>4.5</v>
       </c>
       <c r="G17" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="H17">
         <v>5</v>
       </c>
       <c r="I17">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J17" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="K17">
         <v>5</v>
       </c>
       <c r="L17">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M17" t="str">
         <v>Campbell, Neil</v>
@@ -8351,7 +8351,7 @@
         <v>60</v>
       </c>
       <c r="M20" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N20">
         <v>3</v>
@@ -8360,7 +8360,7 @@
         <v>60</v>
       </c>
       <c r="P20" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q20">
         <v>3</v>
@@ -8425,7 +8425,7 @@
         <v>60</v>
       </c>
       <c r="P21" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="Q21">
         <v>15</v>
@@ -8499,13 +8499,13 @@
         <v>60</v>
       </c>
       <c r="S22" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Russell, Julia (F)</v>
       </c>
       <c r="T22">
         <v>4</v>
       </c>
       <c r="U22">
-        <v>60</v>
+        <v>285</v>
       </c>
     </row>
     <row r="23">
@@ -8537,7 +8537,7 @@
         <v>180</v>
       </c>
       <c r="J23" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="K23">
         <v>13</v>
@@ -8546,7 +8546,7 @@
         <v>60</v>
       </c>
       <c r="M23" t="str">
-        <v>Munro, Alistair</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="N23">
         <v>13</v>
@@ -8555,7 +8555,7 @@
         <v>60</v>
       </c>
       <c r="P23" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="Q23">
         <v>13</v>
@@ -8564,7 +8564,7 @@
         <v>60</v>
       </c>
       <c r="S23" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="T23">
         <v>13</v>
@@ -8593,7 +8593,7 @@
         <v>5</v>
       </c>
       <c r="G24" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="H24">
         <v>4</v>
@@ -8602,7 +8602,7 @@
         <v>60</v>
       </c>
       <c r="J24" t="str">
-        <v>Munro, Alistair</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="K24">
         <v>4</v>
@@ -8611,7 +8611,7 @@
         <v>60</v>
       </c>
       <c r="M24" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="N24">
         <v>4</v>
@@ -8620,7 +8620,7 @@
         <v>60</v>
       </c>
       <c r="P24" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="Q24">
         <v>4</v>
@@ -8629,7 +8629,7 @@
         <v>60</v>
       </c>
       <c r="S24" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="T24">
         <v>4</v>
@@ -8658,22 +8658,22 @@
         <v>4</v>
       </c>
       <c r="G25" t="str">
-        <v>Scott, Edith (F)</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="H25">
         <v>1</v>
       </c>
       <c r="I25">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="J25" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott, Edith (F)</v>
       </c>
       <c r="K25">
         <v>1</v>
       </c>
       <c r="L25">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="M25" t="str">
         <v>Grant, Helen (F)</v>
@@ -8723,7 +8723,7 @@
         <v>3</v>
       </c>
       <c r="G26" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="H26">
         <v>3</v>
@@ -8732,7 +8732,7 @@
         <v>60</v>
       </c>
       <c r="J26" t="str">
-        <v>Brown, Christine</v>
+        <v>Lindsay, Martha (F)</v>
       </c>
       <c r="K26">
         <v>3</v>
@@ -8741,7 +8741,7 @@
         <v>60</v>
       </c>
       <c r="M26" t="str">
-        <v>Lindsay, Martha (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="N26">
         <v>3</v>
@@ -8765,7 +8765,7 @@
         <v>3</v>
       </c>
       <c r="U26">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="27">
@@ -8880,16 +8880,16 @@
         <v>60</v>
       </c>
       <c r="P28" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q28">
         <v>3</v>
       </c>
       <c r="R28">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S28" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T28">
         <v>3</v>
@@ -8992,7 +8992,7 @@
         <v>120</v>
       </c>
       <c r="J30" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Gibb, Irene (F)</v>
       </c>
       <c r="K30">
         <v>5</v>
@@ -9001,7 +9001,7 @@
         <v>60</v>
       </c>
       <c r="M30" t="str">
-        <v>Gibb, Irene (F)</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="N30">
         <v>5</v>
@@ -9010,7 +9010,7 @@
         <v>60</v>
       </c>
       <c r="P30" t="str">
-        <v>Brown, Christine</v>
+        <v>Lindsay, Martha (F)</v>
       </c>
       <c r="Q30">
         <v>5</v>
@@ -9019,7 +9019,7 @@
         <v>60</v>
       </c>
       <c r="S30" t="str">
-        <v>Lindsay, Martha (F)</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="T30">
         <v>5</v>
@@ -9205,16 +9205,16 @@
         <v>60</v>
       </c>
       <c r="P33" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q33">
         <v>3</v>
       </c>
       <c r="R33">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S33" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T33">
         <v>3</v>
@@ -9308,7 +9308,7 @@
         <v>8</v>
       </c>
       <c r="G35" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="H35">
         <v>13</v>
@@ -9317,7 +9317,7 @@
         <v>60</v>
       </c>
       <c r="J35" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="K35">
         <v>13</v>
@@ -9335,7 +9335,7 @@
         <v>60</v>
       </c>
       <c r="P35" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="Q35">
         <v>13</v>
@@ -9373,7 +9373,7 @@
         <v>2</v>
       </c>
       <c r="G36" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="H36">
         <v>4</v>
@@ -9382,7 +9382,7 @@
         <v>60</v>
       </c>
       <c r="J36" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="K36">
         <v>4</v>
@@ -9400,7 +9400,7 @@
         <v>60</v>
       </c>
       <c r="P36" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="Q36">
         <v>4</v>
@@ -9474,7 +9474,7 @@
         <v>60</v>
       </c>
       <c r="S37" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="T37">
         <v>6</v>
@@ -9595,7 +9595,7 @@
         <v>60</v>
       </c>
       <c r="P39" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q39">
         <v>3</v>
@@ -9604,7 +9604,7 @@
         <v>60</v>
       </c>
       <c r="S39" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T39">
         <v>3</v>
@@ -9976,7 +9976,7 @@
         <v>60</v>
       </c>
       <c r="M45" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="N45">
         <v>15</v>
@@ -9994,7 +9994,7 @@
         <v>60</v>
       </c>
       <c r="S45" t="str">
-        <v>McIntyre, Donald</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="T45">
         <v>15</v>
@@ -10088,7 +10088,7 @@
         <v>5</v>
       </c>
       <c r="G47" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="H47">
         <v>13</v>
@@ -10097,7 +10097,7 @@
         <v>60</v>
       </c>
       <c r="J47" t="str">
-        <v>Munro, Alistair</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="K47">
         <v>13</v>
@@ -10106,7 +10106,7 @@
         <v>60</v>
       </c>
       <c r="M47" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="N47">
         <v>13</v>
@@ -10115,7 +10115,7 @@
         <v>60</v>
       </c>
       <c r="P47" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="Q47">
         <v>13</v>
@@ -10124,7 +10124,7 @@
         <v>60</v>
       </c>
       <c r="S47" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="T47">
         <v>13</v>
@@ -10153,7 +10153,7 @@
         <v>6</v>
       </c>
       <c r="G48" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="H48">
         <v>4</v>
@@ -10162,7 +10162,7 @@
         <v>60</v>
       </c>
       <c r="J48" t="str">
-        <v>Munro, Alistair</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="K48">
         <v>4</v>
@@ -10171,7 +10171,7 @@
         <v>60</v>
       </c>
       <c r="M48" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="N48">
         <v>4</v>
@@ -10180,7 +10180,7 @@
         <v>60</v>
       </c>
       <c r="P48" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="Q48">
         <v>4</v>
@@ -10189,7 +10189,7 @@
         <v>60</v>
       </c>
       <c r="S48" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="T48">
         <v>4</v>
@@ -10245,7 +10245,7 @@
         <v>60</v>
       </c>
       <c r="P49" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="Q49">
         <v>11</v>
@@ -10366,7 +10366,7 @@
         <v>60</v>
       </c>
       <c r="M51" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="N51">
         <v>15</v>
@@ -10375,7 +10375,7 @@
         <v>60</v>
       </c>
       <c r="P51" t="str">
-        <v>McIntyre, Donald</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="Q51">
         <v>15</v>
@@ -10496,7 +10496,7 @@
         <v>60</v>
       </c>
       <c r="M53" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="N53">
         <v>11</v>
@@ -10543,22 +10543,22 @@
         <v>6.75</v>
       </c>
       <c r="G54" t="str">
-        <v>Scott, Edith (F)</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="H54">
         <v>1</v>
       </c>
       <c r="I54">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J54" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott, Edith (F)</v>
       </c>
       <c r="K54">
         <v>1</v>
       </c>
       <c r="L54">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M54" t="str">
         <v>Barrons, Shirley</v>
@@ -10579,7 +10579,7 @@
         <v>60</v>
       </c>
       <c r="S54" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="T54">
         <v>6</v>
@@ -10691,7 +10691,7 @@
         <v>285</v>
       </c>
       <c r="M56" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="N56">
         <v>5</v>
@@ -10700,7 +10700,7 @@
         <v>60</v>
       </c>
       <c r="P56" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="Q56">
         <v>5</v>
@@ -10738,7 +10738,7 @@
         <v>6.75</v>
       </c>
       <c r="G57" t="str">
-        <v>Barrons, Shirley</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="H57">
         <v>10</v>
@@ -10747,7 +10747,7 @@
         <v>60</v>
       </c>
       <c r="J57" t="str">
-        <v>Barrons, Shirley</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="K57">
         <v>10</v>
@@ -10756,7 +10756,7 @@
         <v>60</v>
       </c>
       <c r="M57" t="str">
-        <v>Lynch, Roselyn (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="N57">
         <v>10</v>
@@ -10765,22 +10765,22 @@
         <v>60</v>
       </c>
       <c r="P57" t="str">
-        <v>Lynch, Roselyn (F)</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="Q57">
         <v>10</v>
       </c>
       <c r="R57">
-        <v>285</v>
+        <v>60</v>
       </c>
       <c r="S57" t="str">
-        <v>Munro, Alistair</v>
+        <v>Russell, Julia (F)</v>
       </c>
       <c r="T57">
         <v>10</v>
       </c>
       <c r="U57">
-        <v>60</v>
+        <v>285</v>
       </c>
     </row>
     <row r="58">
@@ -10942,7 +10942,7 @@
         <v>480</v>
       </c>
       <c r="J60" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="K60">
         <v>15</v>
@@ -10960,7 +10960,7 @@
         <v>60</v>
       </c>
       <c r="P60" t="str">
-        <v>McIntyre, Donald</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="Q60">
         <v>15</v>
@@ -11155,7 +11155,7 @@
         <v>60</v>
       </c>
       <c r="P63" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="Q63">
         <v>11</v>
@@ -11229,7 +11229,7 @@
         <v>60</v>
       </c>
       <c r="S64" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="T64">
         <v>14</v>
@@ -11294,7 +11294,7 @@
         <v>60</v>
       </c>
       <c r="S65" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T65">
         <v>17</v>
@@ -11323,7 +11323,7 @@
         <v>6</v>
       </c>
       <c r="G66" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="H66">
         <v>8</v>
@@ -11332,7 +11332,7 @@
         <v>60</v>
       </c>
       <c r="J66" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="K66">
         <v>8</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update capacity dashboard with the latest data
No changes made to capacity_dashboard.xlsx.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -7163,22 +7163,22 @@
         <v>6</v>
       </c>
       <c r="G2" t="str">
-        <v>Robertson, Doreen (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="H2">
         <v>8</v>
       </c>
       <c r="I2">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J2" t="str">
-        <v>Murray, James</v>
+        <v>Robertson, Doreen (F)</v>
       </c>
       <c r="K2">
         <v>8</v>
       </c>
       <c r="L2">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M2" t="str">
         <v>Brown, Christine</v>
@@ -7199,13 +7199,13 @@
         <v>60</v>
       </c>
       <c r="S2" t="str">
-        <v>Bryce, Angela (F)</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="T2">
         <v>11</v>
       </c>
       <c r="U2">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
@@ -7246,7 +7246,7 @@
         <v>120</v>
       </c>
       <c r="M3" t="str">
-        <v>Barrons, Shirley</v>
+        <v>Ramsay, Jean (F)</v>
       </c>
       <c r="N3">
         <v>5</v>
@@ -7264,7 +7264,7 @@
         <v>60</v>
       </c>
       <c r="S3" t="str">
-        <v>Ramsay, Jean (F)</v>
+        <v>Barrons, Shirley</v>
       </c>
       <c r="T3">
         <v>5</v>
@@ -7293,7 +7293,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -7302,16 +7302,16 @@
         <v>120</v>
       </c>
       <c r="J4" t="str">
-        <v>Duffy, Sarah Anne (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K4">
         <v>1</v>
       </c>
       <c r="L4">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M4" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N4">
         <v>1</v>
@@ -7320,13 +7320,13 @@
         <v>120</v>
       </c>
       <c r="P4" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Duffy, Sarah Anne (F)</v>
       </c>
       <c r="Q4">
         <v>1</v>
       </c>
       <c r="R4">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S4" t="str">
         <v>Whyte, Jean (F)</v>
@@ -7441,7 +7441,7 @@
         <v>120</v>
       </c>
       <c r="M6" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="N6">
         <v>5</v>
@@ -7450,7 +7450,7 @@
         <v>60</v>
       </c>
       <c r="P6" t="str">
-        <v>Lindsay, Martha (F)</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="Q6">
         <v>5</v>
@@ -7459,7 +7459,7 @@
         <v>60</v>
       </c>
       <c r="S6" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Lindsay, Martha (F)</v>
       </c>
       <c r="T6">
         <v>5</v>
@@ -7506,13 +7506,13 @@
         <v>120</v>
       </c>
       <c r="M7" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N7">
         <v>2</v>
       </c>
       <c r="O7">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P7" t="str">
         <v>Clements, Jessie (F)</v>
@@ -7521,10 +7521,10 @@
         <v>2</v>
       </c>
       <c r="R7">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S7" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="T7">
         <v>2</v>
@@ -7645,13 +7645,13 @@
         <v>60</v>
       </c>
       <c r="P9" t="str">
-        <v>Robertson, Doreen (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q9">
         <v>7</v>
       </c>
       <c r="R9">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S9" t="str">
         <v>Campbell, Neil</v>
@@ -7701,7 +7701,7 @@
         <v>60</v>
       </c>
       <c r="M10" t="str">
-        <v>McIntyre, Donald</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="N10">
         <v>15</v>
@@ -7710,7 +7710,7 @@
         <v>60</v>
       </c>
       <c r="P10" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="Q10">
         <v>15</v>
@@ -7748,7 +7748,7 @@
         <v>3</v>
       </c>
       <c r="G11" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -7757,16 +7757,16 @@
         <v>120</v>
       </c>
       <c r="J11" t="str">
-        <v>Duffy, Sarah Anne (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K11">
         <v>1</v>
       </c>
       <c r="L11">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M11" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N11">
         <v>1</v>
@@ -7775,13 +7775,13 @@
         <v>120</v>
       </c>
       <c r="P11" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Duffy, Sarah Anne (F)</v>
       </c>
       <c r="Q11">
         <v>1</v>
       </c>
       <c r="R11">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S11" t="str">
         <v>Whyte, Jean (F)</v>
@@ -7822,7 +7822,7 @@
         <v>510</v>
       </c>
       <c r="J12" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="K12">
         <v>13</v>
@@ -7831,7 +7831,7 @@
         <v>60</v>
       </c>
       <c r="M12" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="N12">
         <v>13</v>
@@ -7840,7 +7840,7 @@
         <v>60</v>
       </c>
       <c r="P12" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="Q12">
         <v>13</v>
@@ -7878,7 +7878,7 @@
         <v>3</v>
       </c>
       <c r="G13" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="H13">
         <v>4</v>
@@ -7887,7 +7887,7 @@
         <v>60</v>
       </c>
       <c r="J13" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="K13">
         <v>4</v>
@@ -7896,7 +7896,7 @@
         <v>60</v>
       </c>
       <c r="M13" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="N13">
         <v>4</v>
@@ -7943,7 +7943,7 @@
         <v>4.75</v>
       </c>
       <c r="G14" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -7952,7 +7952,7 @@
         <v>60</v>
       </c>
       <c r="J14" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K14">
         <v>1</v>
@@ -7970,7 +7970,7 @@
         <v>60</v>
       </c>
       <c r="P14" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q14">
         <v>1</v>
@@ -8008,7 +8008,7 @@
         <v>6</v>
       </c>
       <c r="G15" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H15">
         <v>2</v>
@@ -8017,7 +8017,7 @@
         <v>60</v>
       </c>
       <c r="J15" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="K15">
         <v>2</v>
@@ -8026,7 +8026,7 @@
         <v>60</v>
       </c>
       <c r="M15" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="N15">
         <v>3</v>
@@ -8035,7 +8035,7 @@
         <v>60</v>
       </c>
       <c r="P15" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="Q15">
         <v>3</v>
@@ -8091,7 +8091,7 @@
         <v>60</v>
       </c>
       <c r="M16" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N16">
         <v>2</v>
@@ -8100,7 +8100,7 @@
         <v>60</v>
       </c>
       <c r="P16" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q16">
         <v>2</v>
@@ -8138,22 +8138,22 @@
         <v>4.5</v>
       </c>
       <c r="G17" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="H17">
         <v>5</v>
       </c>
       <c r="I17">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J17" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="K17">
         <v>5</v>
       </c>
       <c r="L17">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M17" t="str">
         <v>Campbell, Neil</v>
@@ -8203,7 +8203,7 @@
         <v>8</v>
       </c>
       <c r="G18" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H18">
         <v>1</v>
@@ -8212,7 +8212,7 @@
         <v>60</v>
       </c>
       <c r="J18" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="K18">
         <v>1</v>
@@ -8295,7 +8295,7 @@
         <v>120</v>
       </c>
       <c r="P19" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q19">
         <v>4</v>
@@ -8304,7 +8304,7 @@
         <v>60</v>
       </c>
       <c r="S19" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="T19">
         <v>4</v>
@@ -8333,7 +8333,7 @@
         <v>4</v>
       </c>
       <c r="G20" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -8342,7 +8342,7 @@
         <v>60</v>
       </c>
       <c r="J20" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="K20">
         <v>1</v>
@@ -8351,7 +8351,7 @@
         <v>60</v>
       </c>
       <c r="M20" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="N20">
         <v>3</v>
@@ -8360,7 +8360,7 @@
         <v>60</v>
       </c>
       <c r="P20" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="Q20">
         <v>3</v>
@@ -8425,7 +8425,7 @@
         <v>60</v>
       </c>
       <c r="P21" t="str">
-        <v>McIntyre, Donald</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="Q21">
         <v>15</v>
@@ -8463,7 +8463,7 @@
         <v>5</v>
       </c>
       <c r="G22" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H22">
         <v>1</v>
@@ -8472,7 +8472,7 @@
         <v>60</v>
       </c>
       <c r="J22" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K22">
         <v>1</v>
@@ -8490,7 +8490,7 @@
         <v>60</v>
       </c>
       <c r="P22" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q22">
         <v>1</v>
@@ -8499,13 +8499,13 @@
         <v>60</v>
       </c>
       <c r="S22" t="str">
-        <v>Russell, Julia (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="T22">
         <v>4</v>
       </c>
       <c r="U22">
-        <v>285</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23">
@@ -8537,7 +8537,7 @@
         <v>180</v>
       </c>
       <c r="J23" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="K23">
         <v>13</v>
@@ -8555,7 +8555,7 @@
         <v>60</v>
       </c>
       <c r="P23" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="Q23">
         <v>13</v>
@@ -8593,7 +8593,7 @@
         <v>5</v>
       </c>
       <c r="G24" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="H24">
         <v>4</v>
@@ -8611,7 +8611,7 @@
         <v>60</v>
       </c>
       <c r="M24" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="N24">
         <v>4</v>
@@ -8629,7 +8629,7 @@
         <v>60</v>
       </c>
       <c r="S24" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="T24">
         <v>4</v>
@@ -8658,22 +8658,22 @@
         <v>4</v>
       </c>
       <c r="G25" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott, Edith (F)</v>
       </c>
       <c r="H25">
         <v>1</v>
       </c>
       <c r="I25">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="J25" t="str">
-        <v>Scott, Edith (F)</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="K25">
         <v>1</v>
       </c>
       <c r="L25">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="M25" t="str">
         <v>Grant, Helen (F)</v>
@@ -8685,7 +8685,7 @@
         <v>120</v>
       </c>
       <c r="P25" t="str">
-        <v>Barrons, Shirley</v>
+        <v>Ramsay, Jean (F)</v>
       </c>
       <c r="Q25">
         <v>5</v>
@@ -8723,7 +8723,7 @@
         <v>3</v>
       </c>
       <c r="G26" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="H26">
         <v>3</v>
@@ -8732,7 +8732,7 @@
         <v>60</v>
       </c>
       <c r="J26" t="str">
-        <v>Lindsay, Martha (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="K26">
         <v>3</v>
@@ -8756,16 +8756,16 @@
         <v>3</v>
       </c>
       <c r="R26">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S26" t="str">
-        <v>Campbell, Neil</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="T26">
         <v>3</v>
       </c>
       <c r="U26">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27">
@@ -8788,13 +8788,13 @@
         <v>4.75</v>
       </c>
       <c r="G27" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H27">
         <v>1</v>
       </c>
       <c r="I27">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J27" t="str">
         <v>East NL, Glasgow</v>
@@ -8806,13 +8806,13 @@
         <v>60</v>
       </c>
       <c r="M27" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N27">
         <v>1</v>
       </c>
       <c r="O27">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P27" t="str">
         <v>Clements, Jessie (F)</v>
@@ -8821,16 +8821,16 @@
         <v>1</v>
       </c>
       <c r="R27">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S27" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="T27">
         <v>1</v>
       </c>
       <c r="U27">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="28">
@@ -8853,13 +8853,13 @@
         <v>6</v>
       </c>
       <c r="G28" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H28">
         <v>2</v>
       </c>
       <c r="I28">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J28" t="str">
         <v>East NL, Glasgow</v>
@@ -8871,25 +8871,25 @@
         <v>60</v>
       </c>
       <c r="M28" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N28">
         <v>2</v>
       </c>
       <c r="O28">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P28" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="Q28">
         <v>3</v>
       </c>
       <c r="R28">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S28" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="T28">
         <v>3</v>
@@ -8936,13 +8936,13 @@
         <v>60</v>
       </c>
       <c r="M29" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N29">
         <v>2</v>
       </c>
       <c r="O29">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P29" t="str">
         <v>East NL, Glasgow</v>
@@ -8954,13 +8954,13 @@
         <v>60</v>
       </c>
       <c r="S29" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="T29">
         <v>2</v>
       </c>
       <c r="U29">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30">
@@ -8992,7 +8992,7 @@
         <v>120</v>
       </c>
       <c r="J30" t="str">
-        <v>Gibb, Irene (F)</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="K30">
         <v>5</v>
@@ -9001,7 +9001,7 @@
         <v>60</v>
       </c>
       <c r="M30" t="str">
-        <v>Brown, Christine</v>
+        <v>Gibb, Irene (F)</v>
       </c>
       <c r="N30">
         <v>5</v>
@@ -9010,7 +9010,7 @@
         <v>60</v>
       </c>
       <c r="P30" t="str">
-        <v>Lindsay, Martha (F)</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="Q30">
         <v>5</v>
@@ -9019,7 +9019,7 @@
         <v>60</v>
       </c>
       <c r="S30" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Lindsay, Martha (F)</v>
       </c>
       <c r="T30">
         <v>5</v>
@@ -9048,13 +9048,13 @@
         <v>6</v>
       </c>
       <c r="G31" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H31">
         <v>1</v>
       </c>
       <c r="I31">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J31" t="str">
         <v>East NL, Glasgow</v>
@@ -9066,13 +9066,13 @@
         <v>60</v>
       </c>
       <c r="M31" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N31">
         <v>1</v>
       </c>
       <c r="O31">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P31" t="str">
         <v>Clements, Jessie (F)</v>
@@ -9140,13 +9140,13 @@
         <v>60</v>
       </c>
       <c r="P32" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q32">
         <v>4</v>
       </c>
       <c r="R32">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S32" t="str">
         <v>East NL, Glasgow</v>
@@ -9178,13 +9178,13 @@
         <v>9</v>
       </c>
       <c r="G33" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H33">
         <v>1</v>
       </c>
       <c r="I33">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J33" t="str">
         <v>East NL, Glasgow</v>
@@ -9196,25 +9196,25 @@
         <v>60</v>
       </c>
       <c r="M33" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N33">
         <v>1</v>
       </c>
       <c r="O33">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P33" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="Q33">
         <v>3</v>
       </c>
       <c r="R33">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S33" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="T33">
         <v>3</v>
@@ -9243,13 +9243,13 @@
         <v>4</v>
       </c>
       <c r="G34" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H34">
         <v>1</v>
       </c>
       <c r="I34">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J34" t="str">
         <v>East NL, Glasgow</v>
@@ -9261,13 +9261,13 @@
         <v>60</v>
       </c>
       <c r="M34" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N34">
         <v>1</v>
       </c>
       <c r="O34">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P34" t="str">
         <v>Clements, Jessie (F)</v>
@@ -9276,16 +9276,16 @@
         <v>1</v>
       </c>
       <c r="R34">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S34" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="T34">
         <v>1</v>
       </c>
       <c r="U34">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="35">
@@ -9308,7 +9308,7 @@
         <v>8</v>
       </c>
       <c r="G35" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="H35">
         <v>13</v>
@@ -9326,7 +9326,7 @@
         <v>60</v>
       </c>
       <c r="M35" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="N35">
         <v>13</v>
@@ -9335,7 +9335,7 @@
         <v>60</v>
       </c>
       <c r="P35" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="Q35">
         <v>13</v>
@@ -9373,7 +9373,7 @@
         <v>2</v>
       </c>
       <c r="G36" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="H36">
         <v>4</v>
@@ -9391,7 +9391,7 @@
         <v>60</v>
       </c>
       <c r="M36" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="N36">
         <v>4</v>
@@ -9400,7 +9400,7 @@
         <v>60</v>
       </c>
       <c r="P36" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="Q36">
         <v>4</v>
@@ -9474,7 +9474,7 @@
         <v>60</v>
       </c>
       <c r="S37" t="str">
-        <v>McIntyre, Donald</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="T37">
         <v>6</v>
@@ -9503,7 +9503,7 @@
         <v>3</v>
       </c>
       <c r="G38" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H38">
         <v>1</v>
@@ -9512,7 +9512,7 @@
         <v>60</v>
       </c>
       <c r="J38" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K38">
         <v>1</v>
@@ -9530,7 +9530,7 @@
         <v>60</v>
       </c>
       <c r="P38" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q38">
         <v>1</v>
@@ -9568,7 +9568,7 @@
         <v>7.75</v>
       </c>
       <c r="G39" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H39">
         <v>2</v>
@@ -9577,7 +9577,7 @@
         <v>60</v>
       </c>
       <c r="J39" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="K39">
         <v>2</v>
@@ -9586,7 +9586,7 @@
         <v>60</v>
       </c>
       <c r="M39" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="N39">
         <v>2</v>
@@ -9595,7 +9595,7 @@
         <v>60</v>
       </c>
       <c r="P39" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="Q39">
         <v>3</v>
@@ -9604,7 +9604,7 @@
         <v>60</v>
       </c>
       <c r="S39" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="T39">
         <v>3</v>
@@ -9651,7 +9651,7 @@
         <v>60</v>
       </c>
       <c r="M40" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N40">
         <v>2</v>
@@ -9660,7 +9660,7 @@
         <v>60</v>
       </c>
       <c r="P40" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q40">
         <v>2</v>
@@ -9790,7 +9790,7 @@
         <v>60</v>
       </c>
       <c r="P42" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="Q42">
         <v>18</v>
@@ -9799,7 +9799,7 @@
         <v>60</v>
       </c>
       <c r="S42" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="T42">
         <v>18</v>
@@ -9828,7 +9828,7 @@
         <v>10</v>
       </c>
       <c r="G43" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H43">
         <v>1</v>
@@ -9837,7 +9837,7 @@
         <v>60</v>
       </c>
       <c r="J43" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="K43">
         <v>1</v>
@@ -9846,7 +9846,7 @@
         <v>60</v>
       </c>
       <c r="M43" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N43">
         <v>2</v>
@@ -9864,7 +9864,7 @@
         <v>60</v>
       </c>
       <c r="S43" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="T43">
         <v>2</v>
@@ -9911,7 +9911,7 @@
         <v>60</v>
       </c>
       <c r="M44" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N44">
         <v>4</v>
@@ -9920,7 +9920,7 @@
         <v>60</v>
       </c>
       <c r="P44" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q44">
         <v>4</v>
@@ -9976,7 +9976,7 @@
         <v>60</v>
       </c>
       <c r="M45" t="str">
-        <v>McIntyre, Donald</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="N45">
         <v>15</v>
@@ -9994,7 +9994,7 @@
         <v>60</v>
       </c>
       <c r="S45" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="T45">
         <v>15</v>
@@ -10023,7 +10023,7 @@
         <v>3</v>
       </c>
       <c r="G46" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H46">
         <v>1</v>
@@ -10032,7 +10032,7 @@
         <v>60</v>
       </c>
       <c r="J46" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K46">
         <v>1</v>
@@ -10050,7 +10050,7 @@
         <v>60</v>
       </c>
       <c r="P46" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q46">
         <v>1</v>
@@ -10088,7 +10088,7 @@
         <v>5</v>
       </c>
       <c r="G47" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="H47">
         <v>13</v>
@@ -10106,7 +10106,7 @@
         <v>60</v>
       </c>
       <c r="M47" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="N47">
         <v>13</v>
@@ -10124,7 +10124,7 @@
         <v>60</v>
       </c>
       <c r="S47" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="T47">
         <v>13</v>
@@ -10153,7 +10153,7 @@
         <v>6</v>
       </c>
       <c r="G48" t="str">
-        <v>McIntyre, Donald</v>
+        <v>O'Brien, Josephine (F)</v>
       </c>
       <c r="H48">
         <v>4</v>
@@ -10171,7 +10171,7 @@
         <v>60</v>
       </c>
       <c r="M48" t="str">
-        <v>O'Brien, Josephine (F)</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="N48">
         <v>4</v>
@@ -10189,7 +10189,7 @@
         <v>60</v>
       </c>
       <c r="S48" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="T48">
         <v>4</v>
@@ -10218,7 +10218,7 @@
         <v>8</v>
       </c>
       <c r="G49" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="H49">
         <v>8</v>
@@ -10227,7 +10227,7 @@
         <v>60</v>
       </c>
       <c r="J49" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="K49">
         <v>8</v>
@@ -10245,7 +10245,7 @@
         <v>60</v>
       </c>
       <c r="P49" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="Q49">
         <v>11</v>
@@ -10254,7 +10254,7 @@
         <v>60</v>
       </c>
       <c r="S49" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T49">
         <v>11</v>
@@ -10283,7 +10283,7 @@
         <v>9</v>
       </c>
       <c r="G50" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="H50">
         <v>1</v>
@@ -10292,7 +10292,7 @@
         <v>60</v>
       </c>
       <c r="J50" t="str">
-        <v>Duffy, Sarah Anne (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="K50">
         <v>1</v>
@@ -10301,7 +10301,7 @@
         <v>60</v>
       </c>
       <c r="M50" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Duffy, Sarah Anne (F)</v>
       </c>
       <c r="N50">
         <v>1</v>
@@ -10366,7 +10366,7 @@
         <v>60</v>
       </c>
       <c r="M51" t="str">
-        <v>McIntyre, Donald</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="N51">
         <v>15</v>
@@ -10375,7 +10375,7 @@
         <v>60</v>
       </c>
       <c r="P51" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="Q51">
         <v>15</v>
@@ -10496,7 +10496,7 @@
         <v>60</v>
       </c>
       <c r="M53" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="N53">
         <v>11</v>
@@ -10505,7 +10505,7 @@
         <v>60</v>
       </c>
       <c r="P53" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q53">
         <v>11</v>
@@ -10514,7 +10514,7 @@
         <v>60</v>
       </c>
       <c r="S53" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T53">
         <v>11</v>
@@ -10543,22 +10543,22 @@
         <v>6.75</v>
       </c>
       <c r="G54" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott, Edith (F)</v>
       </c>
       <c r="H54">
         <v>1</v>
       </c>
       <c r="I54">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J54" t="str">
-        <v>Scott, Edith (F)</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="K54">
         <v>1</v>
       </c>
       <c r="L54">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M54" t="str">
         <v>Barrons, Shirley</v>
@@ -10579,7 +10579,7 @@
         <v>60</v>
       </c>
       <c r="S54" t="str">
-        <v>McIntyre, Donald</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="T54">
         <v>6</v>
@@ -10626,7 +10626,7 @@
         <v>60</v>
       </c>
       <c r="M55" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N55">
         <v>2</v>
@@ -10635,7 +10635,7 @@
         <v>60</v>
       </c>
       <c r="P55" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q55">
         <v>2</v>
@@ -10691,7 +10691,7 @@
         <v>285</v>
       </c>
       <c r="M56" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="N56">
         <v>5</v>
@@ -10700,7 +10700,7 @@
         <v>60</v>
       </c>
       <c r="P56" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="Q56">
         <v>5</v>
@@ -10738,7 +10738,7 @@
         <v>6.75</v>
       </c>
       <c r="G57" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="H57">
         <v>10</v>
@@ -10747,7 +10747,7 @@
         <v>60</v>
       </c>
       <c r="J57" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>McInnes, James</v>
       </c>
       <c r="K57">
         <v>10</v>
@@ -10756,7 +10756,7 @@
         <v>60</v>
       </c>
       <c r="M57" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N57">
         <v>10</v>
@@ -10765,7 +10765,7 @@
         <v>60</v>
       </c>
       <c r="P57" t="str">
-        <v>McIntyre, Donald</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q57">
         <v>10</v>
@@ -10774,13 +10774,13 @@
         <v>60</v>
       </c>
       <c r="S57" t="str">
-        <v>Russell, Julia (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T57">
         <v>10</v>
       </c>
       <c r="U57">
-        <v>285</v>
+        <v>60</v>
       </c>
     </row>
     <row r="58">
@@ -10830,7 +10830,7 @@
         <v>60</v>
       </c>
       <c r="P58" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q58">
         <v>4</v>
@@ -10839,7 +10839,7 @@
         <v>60</v>
       </c>
       <c r="S58" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="T58">
         <v>4</v>
@@ -10942,7 +10942,7 @@
         <v>480</v>
       </c>
       <c r="J60" t="str">
-        <v>McIntyre, Donald</v>
+        <v>Munro, Alistair</v>
       </c>
       <c r="K60">
         <v>15</v>
@@ -10960,7 +10960,7 @@
         <v>60</v>
       </c>
       <c r="P60" t="str">
-        <v>Munro, Alistair</v>
+        <v>McIntyre, Donald</v>
       </c>
       <c r="Q60">
         <v>15</v>
@@ -10998,7 +10998,7 @@
         <v>3</v>
       </c>
       <c r="G61" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H61">
         <v>1</v>
@@ -11007,7 +11007,7 @@
         <v>60</v>
       </c>
       <c r="J61" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K61">
         <v>1</v>
@@ -11025,7 +11025,7 @@
         <v>60</v>
       </c>
       <c r="P61" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q61">
         <v>1</v>
@@ -11128,7 +11128,7 @@
         <v>7</v>
       </c>
       <c r="G63" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="H63">
         <v>8</v>
@@ -11137,7 +11137,7 @@
         <v>60</v>
       </c>
       <c r="J63" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="K63">
         <v>8</v>
@@ -11155,7 +11155,7 @@
         <v>60</v>
       </c>
       <c r="P63" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="Q63">
         <v>11</v>
@@ -11164,7 +11164,7 @@
         <v>60</v>
       </c>
       <c r="S63" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T63">
         <v>11</v>
@@ -11229,7 +11229,7 @@
         <v>60</v>
       </c>
       <c r="S64" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="T64">
         <v>14</v>
@@ -11294,7 +11294,7 @@
         <v>60</v>
       </c>
       <c r="S65" t="str">
-        <v>Campbell, Neil</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="T65">
         <v>17</v>
@@ -11323,7 +11323,7 @@
         <v>6</v>
       </c>
       <c r="G66" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="H66">
         <v>8</v>
@@ -11332,7 +11332,7 @@
         <v>60</v>
       </c>
       <c r="J66" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="K66">
         <v>8</v>
@@ -11341,7 +11341,7 @@
         <v>60</v>
       </c>
       <c r="M66" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="N66">
         <v>9</v>
@@ -11350,7 +11350,7 @@
         <v>60</v>
       </c>
       <c r="P66" t="str">
-        <v>Murray, James</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q66">
         <v>9</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update capacity dashboard with latest data
Updated capacity_dashboard.xlsx file.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -7199,7 +7199,7 @@
         <v>60</v>
       </c>
       <c r="S2" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T2">
         <v>11</v>
@@ -7246,7 +7246,7 @@
         <v>120</v>
       </c>
       <c r="M3" t="str">
-        <v>Ramsay, Jean (F)</v>
+        <v>Barrons, Shirley</v>
       </c>
       <c r="N3">
         <v>5</v>
@@ -7264,7 +7264,7 @@
         <v>60</v>
       </c>
       <c r="S3" t="str">
-        <v>Barrons, Shirley</v>
+        <v>Ramsay, Jean (F)</v>
       </c>
       <c r="T3">
         <v>5</v>
@@ -8026,7 +8026,7 @@
         <v>60</v>
       </c>
       <c r="M15" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N15">
         <v>3</v>
@@ -8035,7 +8035,7 @@
         <v>60</v>
       </c>
       <c r="P15" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q15">
         <v>3</v>
@@ -8351,7 +8351,7 @@
         <v>60</v>
       </c>
       <c r="M20" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N20">
         <v>3</v>
@@ -8360,7 +8360,7 @@
         <v>60</v>
       </c>
       <c r="P20" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q20">
         <v>3</v>
@@ -8685,7 +8685,7 @@
         <v>120</v>
       </c>
       <c r="P25" t="str">
-        <v>Ramsay, Jean (F)</v>
+        <v>Barrons, Shirley</v>
       </c>
       <c r="Q25">
         <v>5</v>
@@ -8723,7 +8723,7 @@
         <v>3</v>
       </c>
       <c r="G26" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="H26">
         <v>3</v>
@@ -8747,16 +8747,16 @@
         <v>3</v>
       </c>
       <c r="O26">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P26" t="str">
-        <v>Campbell, Neil</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="Q26">
         <v>3</v>
       </c>
       <c r="R26">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S26" t="str">
         <v>Brown, Christine</v>
@@ -8880,16 +8880,16 @@
         <v>120</v>
       </c>
       <c r="P28" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q28">
         <v>3</v>
       </c>
       <c r="R28">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S28" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T28">
         <v>3</v>
@@ -9205,16 +9205,16 @@
         <v>120</v>
       </c>
       <c r="P33" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q33">
         <v>3</v>
       </c>
       <c r="R33">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S33" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T33">
         <v>3</v>
@@ -9595,7 +9595,7 @@
         <v>60</v>
       </c>
       <c r="P39" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q39">
         <v>3</v>
@@ -9604,7 +9604,7 @@
         <v>60</v>
       </c>
       <c r="S39" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T39">
         <v>3</v>
@@ -10245,7 +10245,7 @@
         <v>60</v>
       </c>
       <c r="P49" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q49">
         <v>11</v>
@@ -10496,7 +10496,7 @@
         <v>60</v>
       </c>
       <c r="M53" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="N53">
         <v>11</v>
@@ -10520,7 +10520,7 @@
         <v>11</v>
       </c>
       <c r="U53">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="54">
@@ -10738,7 +10738,7 @@
         <v>6.75</v>
       </c>
       <c r="G57" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H57">
         <v>10</v>
@@ -10747,7 +10747,7 @@
         <v>60</v>
       </c>
       <c r="J57" t="str">
-        <v>McInnes, James</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K57">
         <v>10</v>
@@ -10756,7 +10756,7 @@
         <v>60</v>
       </c>
       <c r="M57" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N57">
         <v>10</v>
@@ -10765,7 +10765,7 @@
         <v>60</v>
       </c>
       <c r="P57" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="Q57">
         <v>10</v>
@@ -10774,7 +10774,7 @@
         <v>60</v>
       </c>
       <c r="S57" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T57">
         <v>10</v>
@@ -11155,7 +11155,7 @@
         <v>60</v>
       </c>
       <c r="P63" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q63">
         <v>11</v>
@@ -11202,7 +11202,7 @@
         <v>120</v>
       </c>
       <c r="J64" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K64">
         <v>3</v>
@@ -11220,7 +11220,7 @@
         <v>60</v>
       </c>
       <c r="P64" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="Q64">
         <v>3</v>
@@ -11294,7 +11294,7 @@
         <v>60</v>
       </c>
       <c r="S65" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T65">
         <v>17</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Improve capacity dashboard calculations for visit assignments
Update the `capacity_dashboard.xlsx` file to refine visit assignment logic, addressing issues where large gaps were preventing visits from being assigned.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -7199,13 +7199,13 @@
         <v>60</v>
       </c>
       <c r="S2" t="str">
-        <v>Campbell, Neil</v>
+        <v>Bryce, Angela (F)</v>
       </c>
       <c r="T2">
         <v>11</v>
       </c>
       <c r="U2">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3">
@@ -7293,7 +7293,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -7302,16 +7302,16 @@
         <v>120</v>
       </c>
       <c r="J4" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Duffy, Sarah Anne (F)</v>
       </c>
       <c r="K4">
         <v>1</v>
       </c>
       <c r="L4">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M4" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N4">
         <v>1</v>
@@ -7320,13 +7320,13 @@
         <v>120</v>
       </c>
       <c r="P4" t="str">
-        <v>Duffy, Sarah Anne (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q4">
         <v>1</v>
       </c>
       <c r="R4">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S4" t="str">
         <v>Whyte, Jean (F)</v>
@@ -7441,7 +7441,7 @@
         <v>120</v>
       </c>
       <c r="M6" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="N6">
         <v>5</v>
@@ -7450,7 +7450,7 @@
         <v>60</v>
       </c>
       <c r="P6" t="str">
-        <v>Brown, Christine</v>
+        <v>Lindsay, Martha (F)</v>
       </c>
       <c r="Q6">
         <v>5</v>
@@ -7459,7 +7459,7 @@
         <v>60</v>
       </c>
       <c r="S6" t="str">
-        <v>Lindsay, Martha (F)</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="T6">
         <v>5</v>
@@ -7506,13 +7506,13 @@
         <v>120</v>
       </c>
       <c r="M7" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="N7">
         <v>2</v>
       </c>
       <c r="O7">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P7" t="str">
         <v>Clements, Jessie (F)</v>
@@ -7521,10 +7521,10 @@
         <v>2</v>
       </c>
       <c r="R7">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S7" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T7">
         <v>2</v>
@@ -7748,7 +7748,7 @@
         <v>3</v>
       </c>
       <c r="G11" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -7757,16 +7757,16 @@
         <v>120</v>
       </c>
       <c r="J11" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Duffy, Sarah Anne (F)</v>
       </c>
       <c r="K11">
         <v>1</v>
       </c>
       <c r="L11">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M11" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N11">
         <v>1</v>
@@ -7775,13 +7775,13 @@
         <v>120</v>
       </c>
       <c r="P11" t="str">
-        <v>Duffy, Sarah Anne (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q11">
         <v>1</v>
       </c>
       <c r="R11">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S11" t="str">
         <v>Whyte, Jean (F)</v>
@@ -7943,7 +7943,7 @@
         <v>4.75</v>
       </c>
       <c r="G14" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -7952,7 +7952,7 @@
         <v>60</v>
       </c>
       <c r="J14" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K14">
         <v>1</v>
@@ -7970,7 +7970,7 @@
         <v>60</v>
       </c>
       <c r="P14" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q14">
         <v>1</v>
@@ -8008,7 +8008,7 @@
         <v>6</v>
       </c>
       <c r="G15" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H15">
         <v>2</v>
@@ -8017,7 +8017,7 @@
         <v>60</v>
       </c>
       <c r="J15" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K15">
         <v>2</v>
@@ -8091,7 +8091,7 @@
         <v>60</v>
       </c>
       <c r="M16" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N16">
         <v>2</v>
@@ -8100,7 +8100,7 @@
         <v>60</v>
       </c>
       <c r="P16" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q16">
         <v>2</v>
@@ -8138,22 +8138,22 @@
         <v>4.5</v>
       </c>
       <c r="G17" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="H17">
         <v>5</v>
       </c>
       <c r="I17">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J17" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="K17">
         <v>5</v>
       </c>
       <c r="L17">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M17" t="str">
         <v>Campbell, Neil</v>
@@ -8203,7 +8203,7 @@
         <v>8</v>
       </c>
       <c r="G18" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H18">
         <v>1</v>
@@ -8212,7 +8212,7 @@
         <v>60</v>
       </c>
       <c r="J18" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K18">
         <v>1</v>
@@ -8295,7 +8295,7 @@
         <v>120</v>
       </c>
       <c r="P19" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q19">
         <v>4</v>
@@ -8304,7 +8304,7 @@
         <v>60</v>
       </c>
       <c r="S19" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T19">
         <v>4</v>
@@ -8333,7 +8333,7 @@
         <v>4</v>
       </c>
       <c r="G20" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -8342,7 +8342,7 @@
         <v>60</v>
       </c>
       <c r="J20" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K20">
         <v>1</v>
@@ -8463,7 +8463,7 @@
         <v>5</v>
       </c>
       <c r="G22" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H22">
         <v>1</v>
@@ -8472,7 +8472,7 @@
         <v>60</v>
       </c>
       <c r="J22" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K22">
         <v>1</v>
@@ -8490,7 +8490,7 @@
         <v>60</v>
       </c>
       <c r="P22" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q22">
         <v>1</v>
@@ -8658,22 +8658,22 @@
         <v>4</v>
       </c>
       <c r="G25" t="str">
-        <v>Scott, Edith (F)</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="H25">
         <v>1</v>
       </c>
       <c r="I25">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="J25" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott, Edith (F)</v>
       </c>
       <c r="K25">
         <v>1</v>
       </c>
       <c r="L25">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="M25" t="str">
         <v>Grant, Helen (F)</v>
@@ -8723,7 +8723,7 @@
         <v>3</v>
       </c>
       <c r="G26" t="str">
-        <v>Campbell, Neil</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="H26">
         <v>3</v>
@@ -8732,7 +8732,7 @@
         <v>60</v>
       </c>
       <c r="J26" t="str">
-        <v>Campbell, Neil</v>
+        <v>Lindsay, Martha (F)</v>
       </c>
       <c r="K26">
         <v>3</v>
@@ -8747,10 +8747,10 @@
         <v>3</v>
       </c>
       <c r="O26">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P26" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q26">
         <v>3</v>
@@ -8759,13 +8759,13 @@
         <v>60</v>
       </c>
       <c r="S26" t="str">
-        <v>Brown, Christine</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T26">
         <v>3</v>
       </c>
       <c r="U26">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="27">
@@ -8788,13 +8788,13 @@
         <v>4.75</v>
       </c>
       <c r="G27" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H27">
         <v>1</v>
       </c>
       <c r="I27">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J27" t="str">
         <v>East NL, Glasgow</v>
@@ -8806,13 +8806,13 @@
         <v>60</v>
       </c>
       <c r="M27" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N27">
         <v>1</v>
       </c>
       <c r="O27">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P27" t="str">
         <v>Clements, Jessie (F)</v>
@@ -8821,16 +8821,16 @@
         <v>1</v>
       </c>
       <c r="R27">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S27" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T27">
         <v>1</v>
       </c>
       <c r="U27">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28">
@@ -8853,13 +8853,13 @@
         <v>6</v>
       </c>
       <c r="G28" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H28">
         <v>2</v>
       </c>
       <c r="I28">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J28" t="str">
         <v>East NL, Glasgow</v>
@@ -8871,13 +8871,13 @@
         <v>60</v>
       </c>
       <c r="M28" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N28">
         <v>2</v>
       </c>
       <c r="O28">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P28" t="str">
         <v>Clements, Jessie (F)</v>
@@ -8936,13 +8936,13 @@
         <v>60</v>
       </c>
       <c r="M29" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N29">
         <v>2</v>
       </c>
       <c r="O29">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P29" t="str">
         <v>East NL, Glasgow</v>
@@ -8954,13 +8954,13 @@
         <v>60</v>
       </c>
       <c r="S29" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T29">
         <v>2</v>
       </c>
       <c r="U29">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30">
@@ -8992,7 +8992,7 @@
         <v>120</v>
       </c>
       <c r="J30" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Gibb, Irene (F)</v>
       </c>
       <c r="K30">
         <v>5</v>
@@ -9001,7 +9001,7 @@
         <v>60</v>
       </c>
       <c r="M30" t="str">
-        <v>Gibb, Irene (F)</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="N30">
         <v>5</v>
@@ -9010,7 +9010,7 @@
         <v>60</v>
       </c>
       <c r="P30" t="str">
-        <v>Brown, Christine</v>
+        <v>Lindsay, Martha (F)</v>
       </c>
       <c r="Q30">
         <v>5</v>
@@ -9019,7 +9019,7 @@
         <v>60</v>
       </c>
       <c r="S30" t="str">
-        <v>Lindsay, Martha (F)</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="T30">
         <v>5</v>
@@ -9048,13 +9048,13 @@
         <v>6</v>
       </c>
       <c r="G31" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H31">
         <v>1</v>
       </c>
       <c r="I31">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J31" t="str">
         <v>East NL, Glasgow</v>
@@ -9066,13 +9066,13 @@
         <v>60</v>
       </c>
       <c r="M31" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N31">
         <v>1</v>
       </c>
       <c r="O31">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P31" t="str">
         <v>Clements, Jessie (F)</v>
@@ -9140,13 +9140,13 @@
         <v>60</v>
       </c>
       <c r="P32" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q32">
         <v>4</v>
       </c>
       <c r="R32">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S32" t="str">
         <v>East NL, Glasgow</v>
@@ -9178,13 +9178,13 @@
         <v>9</v>
       </c>
       <c r="G33" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H33">
         <v>1</v>
       </c>
       <c r="I33">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J33" t="str">
         <v>East NL, Glasgow</v>
@@ -9196,13 +9196,13 @@
         <v>60</v>
       </c>
       <c r="M33" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N33">
         <v>1</v>
       </c>
       <c r="O33">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P33" t="str">
         <v>Clements, Jessie (F)</v>
@@ -9243,13 +9243,13 @@
         <v>4</v>
       </c>
       <c r="G34" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H34">
         <v>1</v>
       </c>
       <c r="I34">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J34" t="str">
         <v>East NL, Glasgow</v>
@@ -9261,13 +9261,13 @@
         <v>60</v>
       </c>
       <c r="M34" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N34">
         <v>1</v>
       </c>
       <c r="O34">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P34" t="str">
         <v>Clements, Jessie (F)</v>
@@ -9276,16 +9276,16 @@
         <v>1</v>
       </c>
       <c r="R34">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S34" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T34">
         <v>1</v>
       </c>
       <c r="U34">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35">
@@ -9503,7 +9503,7 @@
         <v>3</v>
       </c>
       <c r="G38" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H38">
         <v>1</v>
@@ -9512,7 +9512,7 @@
         <v>60</v>
       </c>
       <c r="J38" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K38">
         <v>1</v>
@@ -9530,7 +9530,7 @@
         <v>60</v>
       </c>
       <c r="P38" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q38">
         <v>1</v>
@@ -9568,7 +9568,7 @@
         <v>7.75</v>
       </c>
       <c r="G39" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H39">
         <v>2</v>
@@ -9577,7 +9577,7 @@
         <v>60</v>
       </c>
       <c r="J39" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="K39">
         <v>2</v>
@@ -9586,7 +9586,7 @@
         <v>60</v>
       </c>
       <c r="M39" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N39">
         <v>2</v>
@@ -9651,7 +9651,7 @@
         <v>60</v>
       </c>
       <c r="M40" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N40">
         <v>2</v>
@@ -9660,7 +9660,7 @@
         <v>60</v>
       </c>
       <c r="P40" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q40">
         <v>2</v>
@@ -9790,7 +9790,7 @@
         <v>60</v>
       </c>
       <c r="P42" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="Q42">
         <v>18</v>
@@ -9799,7 +9799,7 @@
         <v>60</v>
       </c>
       <c r="S42" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="T42">
         <v>18</v>
@@ -9828,7 +9828,7 @@
         <v>10</v>
       </c>
       <c r="G43" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H43">
         <v>1</v>
@@ -9837,7 +9837,7 @@
         <v>60</v>
       </c>
       <c r="J43" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K43">
         <v>1</v>
@@ -9846,7 +9846,7 @@
         <v>60</v>
       </c>
       <c r="M43" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="N43">
         <v>2</v>
@@ -9864,7 +9864,7 @@
         <v>60</v>
       </c>
       <c r="S43" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T43">
         <v>2</v>
@@ -9911,7 +9911,7 @@
         <v>60</v>
       </c>
       <c r="M44" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N44">
         <v>4</v>
@@ -9920,7 +9920,7 @@
         <v>60</v>
       </c>
       <c r="P44" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q44">
         <v>4</v>
@@ -10023,7 +10023,7 @@
         <v>3</v>
       </c>
       <c r="G46" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H46">
         <v>1</v>
@@ -10032,7 +10032,7 @@
         <v>60</v>
       </c>
       <c r="J46" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K46">
         <v>1</v>
@@ -10050,7 +10050,7 @@
         <v>60</v>
       </c>
       <c r="P46" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q46">
         <v>1</v>
@@ -10218,7 +10218,7 @@
         <v>8</v>
       </c>
       <c r="G49" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="H49">
         <v>8</v>
@@ -10227,7 +10227,7 @@
         <v>60</v>
       </c>
       <c r="J49" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="K49">
         <v>8</v>
@@ -10245,7 +10245,7 @@
         <v>60</v>
       </c>
       <c r="P49" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="Q49">
         <v>11</v>
@@ -10254,7 +10254,7 @@
         <v>60</v>
       </c>
       <c r="S49" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="T49">
         <v>11</v>
@@ -10283,7 +10283,7 @@
         <v>9</v>
       </c>
       <c r="G50" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H50">
         <v>1</v>
@@ -10292,7 +10292,7 @@
         <v>60</v>
       </c>
       <c r="J50" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Duffy, Sarah Anne (F)</v>
       </c>
       <c r="K50">
         <v>1</v>
@@ -10301,7 +10301,7 @@
         <v>60</v>
       </c>
       <c r="M50" t="str">
-        <v>Duffy, Sarah Anne (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N50">
         <v>1</v>
@@ -10413,7 +10413,7 @@
         <v>9</v>
       </c>
       <c r="G52" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="H52">
         <v>1</v>
@@ -10431,7 +10431,7 @@
         <v>60</v>
       </c>
       <c r="M52" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="N52">
         <v>1</v>
@@ -10496,7 +10496,7 @@
         <v>60</v>
       </c>
       <c r="M53" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="N53">
         <v>11</v>
@@ -10505,7 +10505,7 @@
         <v>60</v>
       </c>
       <c r="P53" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="Q53">
         <v>11</v>
@@ -10514,13 +10514,13 @@
         <v>60</v>
       </c>
       <c r="S53" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="T53">
         <v>11</v>
       </c>
       <c r="U53">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="54">
@@ -10543,22 +10543,22 @@
         <v>6.75</v>
       </c>
       <c r="G54" t="str">
-        <v>Scott, Edith (F)</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="H54">
         <v>1</v>
       </c>
       <c r="I54">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J54" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott, Edith (F)</v>
       </c>
       <c r="K54">
         <v>1</v>
       </c>
       <c r="L54">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M54" t="str">
         <v>Barrons, Shirley</v>
@@ -10626,7 +10626,7 @@
         <v>60</v>
       </c>
       <c r="M55" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N55">
         <v>2</v>
@@ -10635,7 +10635,7 @@
         <v>60</v>
       </c>
       <c r="P55" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q55">
         <v>2</v>
@@ -10691,7 +10691,7 @@
         <v>285</v>
       </c>
       <c r="M56" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="N56">
         <v>5</v>
@@ -10700,7 +10700,7 @@
         <v>60</v>
       </c>
       <c r="P56" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="Q56">
         <v>5</v>
@@ -10738,7 +10738,7 @@
         <v>6.75</v>
       </c>
       <c r="G57" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Kennedy, Roberta</v>
       </c>
       <c r="H57">
         <v>10</v>
@@ -10747,16 +10747,16 @@
         <v>60</v>
       </c>
       <c r="J57" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>McConnell, Marion</v>
       </c>
       <c r="K57">
         <v>10</v>
       </c>
       <c r="L57">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="M57" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Duncan, George</v>
       </c>
       <c r="N57">
         <v>10</v>
@@ -10765,7 +10765,7 @@
         <v>60</v>
       </c>
       <c r="P57" t="str">
-        <v>Murray, James</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q57">
         <v>10</v>
@@ -10774,7 +10774,7 @@
         <v>60</v>
       </c>
       <c r="S57" t="str">
-        <v>Campbell, Neil</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="T57">
         <v>10</v>
@@ -10830,7 +10830,7 @@
         <v>60</v>
       </c>
       <c r="P58" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q58">
         <v>4</v>
@@ -10839,7 +10839,7 @@
         <v>60</v>
       </c>
       <c r="S58" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="T58">
         <v>4</v>
@@ -10998,7 +10998,7 @@
         <v>3</v>
       </c>
       <c r="G61" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="H61">
         <v>1</v>
@@ -11007,7 +11007,7 @@
         <v>60</v>
       </c>
       <c r="J61" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="K61">
         <v>1</v>
@@ -11025,7 +11025,7 @@
         <v>60</v>
       </c>
       <c r="P61" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="Q61">
         <v>1</v>
@@ -11128,7 +11128,7 @@
         <v>7</v>
       </c>
       <c r="G63" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="H63">
         <v>8</v>
@@ -11137,7 +11137,7 @@
         <v>60</v>
       </c>
       <c r="J63" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="K63">
         <v>8</v>
@@ -11155,7 +11155,7 @@
         <v>60</v>
       </c>
       <c r="P63" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="Q63">
         <v>11</v>
@@ -11164,7 +11164,7 @@
         <v>60</v>
       </c>
       <c r="S63" t="str">
-        <v>Campbell, Neil</v>
+        <v>Anderson, Margaret (F)</v>
       </c>
       <c r="T63">
         <v>11</v>
@@ -11229,7 +11229,7 @@
         <v>60</v>
       </c>
       <c r="S64" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="T64">
         <v>14</v>
@@ -11323,7 +11323,7 @@
         <v>6</v>
       </c>
       <c r="G66" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="H66">
         <v>8</v>
@@ -11332,7 +11332,7 @@
         <v>60</v>
       </c>
       <c r="J66" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="K66">
         <v>8</v>
@@ -11341,7 +11341,7 @@
         <v>60</v>
       </c>
       <c r="M66" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="N66">
         <v>9</v>
@@ -11350,7 +11350,7 @@
         <v>60</v>
       </c>
       <c r="P66" t="str">
-        <v>Campbell, Neil</v>
+        <v>Murray, James</v>
       </c>
       <c r="Q66">
         <v>9</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update dashboard with current capacity and allocation data
File: capacity_dashboard.xlsx
Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -7293,7 +7293,7 @@
         <v>4</v>
       </c>
       <c r="G4" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -7302,16 +7302,16 @@
         <v>120</v>
       </c>
       <c r="J4" t="str">
-        <v>Duffy, Sarah Anne (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K4">
         <v>1</v>
       </c>
       <c r="L4">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M4" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N4">
         <v>1</v>
@@ -7320,13 +7320,13 @@
         <v>120</v>
       </c>
       <c r="P4" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Duffy, Sarah Anne (F)</v>
       </c>
       <c r="Q4">
         <v>1</v>
       </c>
       <c r="R4">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S4" t="str">
         <v>Whyte, Jean (F)</v>
@@ -7441,7 +7441,7 @@
         <v>120</v>
       </c>
       <c r="M6" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="N6">
         <v>5</v>
@@ -7450,7 +7450,7 @@
         <v>60</v>
       </c>
       <c r="P6" t="str">
-        <v>Lindsay, Martha (F)</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="Q6">
         <v>5</v>
@@ -7459,7 +7459,7 @@
         <v>60</v>
       </c>
       <c r="S6" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Lindsay, Martha (F)</v>
       </c>
       <c r="T6">
         <v>5</v>
@@ -7506,13 +7506,13 @@
         <v>120</v>
       </c>
       <c r="M7" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N7">
         <v>2</v>
       </c>
       <c r="O7">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P7" t="str">
         <v>Clements, Jessie (F)</v>
@@ -7521,10 +7521,10 @@
         <v>2</v>
       </c>
       <c r="R7">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S7" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="T7">
         <v>2</v>
@@ -7748,7 +7748,7 @@
         <v>3</v>
       </c>
       <c r="G11" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -7757,16 +7757,16 @@
         <v>120</v>
       </c>
       <c r="J11" t="str">
-        <v>Duffy, Sarah Anne (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K11">
         <v>1</v>
       </c>
       <c r="L11">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M11" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N11">
         <v>1</v>
@@ -7775,13 +7775,13 @@
         <v>120</v>
       </c>
       <c r="P11" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Duffy, Sarah Anne (F)</v>
       </c>
       <c r="Q11">
         <v>1</v>
       </c>
       <c r="R11">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="S11" t="str">
         <v>Whyte, Jean (F)</v>
@@ -7943,7 +7943,7 @@
         <v>4.75</v>
       </c>
       <c r="G14" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -7952,7 +7952,7 @@
         <v>60</v>
       </c>
       <c r="J14" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K14">
         <v>1</v>
@@ -7970,7 +7970,7 @@
         <v>60</v>
       </c>
       <c r="P14" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q14">
         <v>1</v>
@@ -8008,7 +8008,7 @@
         <v>6</v>
       </c>
       <c r="G15" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H15">
         <v>2</v>
@@ -8017,7 +8017,7 @@
         <v>60</v>
       </c>
       <c r="J15" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="K15">
         <v>2</v>
@@ -8091,7 +8091,7 @@
         <v>60</v>
       </c>
       <c r="M16" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N16">
         <v>2</v>
@@ -8100,7 +8100,7 @@
         <v>60</v>
       </c>
       <c r="P16" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q16">
         <v>2</v>
@@ -8138,22 +8138,22 @@
         <v>4.5</v>
       </c>
       <c r="G17" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="H17">
         <v>5</v>
       </c>
       <c r="I17">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J17" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="K17">
         <v>5</v>
       </c>
       <c r="L17">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M17" t="str">
         <v>Campbell, Neil</v>
@@ -8203,7 +8203,7 @@
         <v>8</v>
       </c>
       <c r="G18" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H18">
         <v>1</v>
@@ -8212,7 +8212,7 @@
         <v>60</v>
       </c>
       <c r="J18" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="K18">
         <v>1</v>
@@ -8295,7 +8295,7 @@
         <v>120</v>
       </c>
       <c r="P19" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q19">
         <v>4</v>
@@ -8304,7 +8304,7 @@
         <v>60</v>
       </c>
       <c r="S19" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="T19">
         <v>4</v>
@@ -8333,7 +8333,7 @@
         <v>4</v>
       </c>
       <c r="G20" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -8342,7 +8342,7 @@
         <v>60</v>
       </c>
       <c r="J20" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="K20">
         <v>1</v>
@@ -8463,7 +8463,7 @@
         <v>5</v>
       </c>
       <c r="G22" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H22">
         <v>1</v>
@@ -8472,7 +8472,7 @@
         <v>60</v>
       </c>
       <c r="J22" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K22">
         <v>1</v>
@@ -8490,7 +8490,7 @@
         <v>60</v>
       </c>
       <c r="P22" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q22">
         <v>1</v>
@@ -8658,22 +8658,22 @@
         <v>4</v>
       </c>
       <c r="G25" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott, Edith (F)</v>
       </c>
       <c r="H25">
         <v>1</v>
       </c>
       <c r="I25">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="J25" t="str">
-        <v>Scott, Edith (F)</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="K25">
         <v>1</v>
       </c>
       <c r="L25">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="M25" t="str">
         <v>Grant, Helen (F)</v>
@@ -8723,7 +8723,7 @@
         <v>3</v>
       </c>
       <c r="G26" t="str">
-        <v>Brown, Christine</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="H26">
         <v>3</v>
@@ -8732,7 +8732,7 @@
         <v>60</v>
       </c>
       <c r="J26" t="str">
-        <v>Lindsay, Martha (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="K26">
         <v>3</v>
@@ -8747,10 +8747,10 @@
         <v>3</v>
       </c>
       <c r="O26">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P26" t="str">
-        <v>Campbell, Neil</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="Q26">
         <v>3</v>
@@ -8759,13 +8759,13 @@
         <v>60</v>
       </c>
       <c r="S26" t="str">
-        <v>Campbell, Neil</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="T26">
         <v>3</v>
       </c>
       <c r="U26">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27">
@@ -8788,13 +8788,13 @@
         <v>4.75</v>
       </c>
       <c r="G27" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H27">
         <v>1</v>
       </c>
       <c r="I27">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J27" t="str">
         <v>East NL, Glasgow</v>
@@ -8806,13 +8806,13 @@
         <v>60</v>
       </c>
       <c r="M27" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N27">
         <v>1</v>
       </c>
       <c r="O27">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P27" t="str">
         <v>Clements, Jessie (F)</v>
@@ -8821,16 +8821,16 @@
         <v>1</v>
       </c>
       <c r="R27">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S27" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="T27">
         <v>1</v>
       </c>
       <c r="U27">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="28">
@@ -8853,13 +8853,13 @@
         <v>6</v>
       </c>
       <c r="G28" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H28">
         <v>2</v>
       </c>
       <c r="I28">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J28" t="str">
         <v>East NL, Glasgow</v>
@@ -8871,13 +8871,13 @@
         <v>60</v>
       </c>
       <c r="M28" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N28">
         <v>2</v>
       </c>
       <c r="O28">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P28" t="str">
         <v>Clements, Jessie (F)</v>
@@ -8936,13 +8936,13 @@
         <v>60</v>
       </c>
       <c r="M29" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N29">
         <v>2</v>
       </c>
       <c r="O29">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="P29" t="str">
         <v>East NL, Glasgow</v>
@@ -8954,13 +8954,13 @@
         <v>60</v>
       </c>
       <c r="S29" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="T29">
         <v>2</v>
       </c>
       <c r="U29">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30">
@@ -8992,7 +8992,7 @@
         <v>120</v>
       </c>
       <c r="J30" t="str">
-        <v>Gibb, Irene (F)</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="K30">
         <v>5</v>
@@ -9001,7 +9001,7 @@
         <v>60</v>
       </c>
       <c r="M30" t="str">
-        <v>Brown, Christine</v>
+        <v>Gibb, Irene (F)</v>
       </c>
       <c r="N30">
         <v>5</v>
@@ -9010,7 +9010,7 @@
         <v>60</v>
       </c>
       <c r="P30" t="str">
-        <v>Lindsay, Martha (F)</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="Q30">
         <v>5</v>
@@ -9019,7 +9019,7 @@
         <v>60</v>
       </c>
       <c r="S30" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Lindsay, Martha (F)</v>
       </c>
       <c r="T30">
         <v>5</v>
@@ -9048,13 +9048,13 @@
         <v>6</v>
       </c>
       <c r="G31" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H31">
         <v>1</v>
       </c>
       <c r="I31">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J31" t="str">
         <v>East NL, Glasgow</v>
@@ -9066,13 +9066,13 @@
         <v>60</v>
       </c>
       <c r="M31" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N31">
         <v>1</v>
       </c>
       <c r="O31">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P31" t="str">
         <v>Clements, Jessie (F)</v>
@@ -9140,13 +9140,13 @@
         <v>60</v>
       </c>
       <c r="P32" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q32">
         <v>4</v>
       </c>
       <c r="R32">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S32" t="str">
         <v>East NL, Glasgow</v>
@@ -9178,13 +9178,13 @@
         <v>9</v>
       </c>
       <c r="G33" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H33">
         <v>1</v>
       </c>
       <c r="I33">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J33" t="str">
         <v>East NL, Glasgow</v>
@@ -9196,13 +9196,13 @@
         <v>60</v>
       </c>
       <c r="M33" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N33">
         <v>1</v>
       </c>
       <c r="O33">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P33" t="str">
         <v>Clements, Jessie (F)</v>
@@ -9243,13 +9243,13 @@
         <v>4</v>
       </c>
       <c r="G34" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H34">
         <v>1</v>
       </c>
       <c r="I34">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J34" t="str">
         <v>East NL, Glasgow</v>
@@ -9261,13 +9261,13 @@
         <v>60</v>
       </c>
       <c r="M34" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N34">
         <v>1</v>
       </c>
       <c r="O34">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="P34" t="str">
         <v>Clements, Jessie (F)</v>
@@ -9276,16 +9276,16 @@
         <v>1</v>
       </c>
       <c r="R34">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="S34" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="T34">
         <v>1</v>
       </c>
       <c r="U34">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="35">
@@ -9503,7 +9503,7 @@
         <v>3</v>
       </c>
       <c r="G38" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H38">
         <v>1</v>
@@ -9512,7 +9512,7 @@
         <v>60</v>
       </c>
       <c r="J38" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K38">
         <v>1</v>
@@ -9530,7 +9530,7 @@
         <v>60</v>
       </c>
       <c r="P38" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q38">
         <v>1</v>
@@ -9568,7 +9568,7 @@
         <v>7.75</v>
       </c>
       <c r="G39" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H39">
         <v>2</v>
@@ -9577,7 +9577,7 @@
         <v>60</v>
       </c>
       <c r="J39" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="K39">
         <v>2</v>
@@ -9586,7 +9586,7 @@
         <v>60</v>
       </c>
       <c r="M39" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="N39">
         <v>2</v>
@@ -9651,7 +9651,7 @@
         <v>60</v>
       </c>
       <c r="M40" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N40">
         <v>2</v>
@@ -9660,7 +9660,7 @@
         <v>60</v>
       </c>
       <c r="P40" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q40">
         <v>2</v>
@@ -9828,7 +9828,7 @@
         <v>10</v>
       </c>
       <c r="G43" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H43">
         <v>1</v>
@@ -9837,7 +9837,7 @@
         <v>60</v>
       </c>
       <c r="J43" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="K43">
         <v>1</v>
@@ -9846,7 +9846,7 @@
         <v>60</v>
       </c>
       <c r="M43" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N43">
         <v>2</v>
@@ -9864,7 +9864,7 @@
         <v>60</v>
       </c>
       <c r="S43" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="T43">
         <v>2</v>
@@ -9911,7 +9911,7 @@
         <v>60</v>
       </c>
       <c r="M44" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N44">
         <v>4</v>
@@ -9920,7 +9920,7 @@
         <v>60</v>
       </c>
       <c r="P44" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q44">
         <v>4</v>
@@ -10023,7 +10023,7 @@
         <v>3</v>
       </c>
       <c r="G46" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H46">
         <v>1</v>
@@ -10032,7 +10032,7 @@
         <v>60</v>
       </c>
       <c r="J46" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K46">
         <v>1</v>
@@ -10050,7 +10050,7 @@
         <v>60</v>
       </c>
       <c r="P46" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q46">
         <v>1</v>
@@ -10245,7 +10245,7 @@
         <v>60</v>
       </c>
       <c r="P49" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q49">
         <v>11</v>
@@ -10254,7 +10254,7 @@
         <v>60</v>
       </c>
       <c r="S49" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T49">
         <v>11</v>
@@ -10283,7 +10283,7 @@
         <v>9</v>
       </c>
       <c r="G50" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="H50">
         <v>1</v>
@@ -10292,7 +10292,7 @@
         <v>60</v>
       </c>
       <c r="J50" t="str">
-        <v>Duffy, Sarah Anne (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="K50">
         <v>1</v>
@@ -10301,7 +10301,7 @@
         <v>60</v>
       </c>
       <c r="M50" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Duffy, Sarah Anne (F)</v>
       </c>
       <c r="N50">
         <v>1</v>
@@ -10413,7 +10413,7 @@
         <v>9</v>
       </c>
       <c r="G52" t="str">
-        <v>Whyte, Jean (F)</v>
+        <v>Mullen, Eileen (F)</v>
       </c>
       <c r="H52">
         <v>1</v>
@@ -10431,7 +10431,7 @@
         <v>60</v>
       </c>
       <c r="M52" t="str">
-        <v>Mullen, Eileen (F)</v>
+        <v>Whyte, Jean (F)</v>
       </c>
       <c r="N52">
         <v>1</v>
@@ -10496,7 +10496,7 @@
         <v>60</v>
       </c>
       <c r="M53" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="N53">
         <v>11</v>
@@ -10505,7 +10505,7 @@
         <v>60</v>
       </c>
       <c r="P53" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q53">
         <v>11</v>
@@ -10514,13 +10514,13 @@
         <v>60</v>
       </c>
       <c r="S53" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T53">
         <v>11</v>
       </c>
       <c r="U53">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="54">
@@ -10543,22 +10543,22 @@
         <v>6.75</v>
       </c>
       <c r="G54" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Scott, Edith (F)</v>
       </c>
       <c r="H54">
         <v>1</v>
       </c>
       <c r="I54">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="J54" t="str">
-        <v>Scott, Edith (F)</v>
+        <v>Goldsmith, Astrid</v>
       </c>
       <c r="K54">
         <v>1</v>
       </c>
       <c r="L54">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="M54" t="str">
         <v>Barrons, Shirley</v>
@@ -10691,7 +10691,7 @@
         <v>285</v>
       </c>
       <c r="M56" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="N56">
         <v>5</v>
@@ -10700,7 +10700,7 @@
         <v>60</v>
       </c>
       <c r="P56" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="Q56">
         <v>5</v>
@@ -10738,25 +10738,25 @@
         <v>6.75</v>
       </c>
       <c r="G57" t="str">
-        <v>Kennedy, Roberta</v>
+        <v>McConnell, Marion</v>
       </c>
       <c r="H57">
         <v>10</v>
       </c>
       <c r="I57">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="J57" t="str">
-        <v>McConnell, Marion</v>
+        <v>Duncan, George</v>
       </c>
       <c r="K57">
         <v>10</v>
       </c>
       <c r="L57">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="M57" t="str">
-        <v>Duncan, George</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="N57">
         <v>10</v>
@@ -10765,7 +10765,7 @@
         <v>60</v>
       </c>
       <c r="P57" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q57">
         <v>10</v>
@@ -10774,7 +10774,7 @@
         <v>60</v>
       </c>
       <c r="S57" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="T57">
         <v>10</v>
@@ -11155,7 +11155,7 @@
         <v>60</v>
       </c>
       <c r="P63" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q63">
         <v>11</v>
@@ -11164,7 +11164,7 @@
         <v>60</v>
       </c>
       <c r="S63" t="str">
-        <v>Anderson, Margaret (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T63">
         <v>11</v>
@@ -11229,7 +11229,7 @@
         <v>60</v>
       </c>
       <c r="S64" t="str">
-        <v>Goldsmith, Astrid</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="T64">
         <v>14</v>
@@ -11323,7 +11323,7 @@
         <v>6</v>
       </c>
       <c r="G66" t="str">
-        <v>Brown, Christine</v>
+        <v>Docherty, Elizabeth</v>
       </c>
       <c r="H66">
         <v>8</v>
@@ -11332,7 +11332,7 @@
         <v>60</v>
       </c>
       <c r="J66" t="str">
-        <v>Docherty, Elizabeth</v>
+        <v>Brown, Christine</v>
       </c>
       <c r="K66">
         <v>8</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Improve visit time calculations to consider appointment priorities
Update logic to correctly handle visit time calculations, ensuring appointments are prioritized based on their assigned order.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -7199,13 +7199,13 @@
         <v>60</v>
       </c>
       <c r="S2" t="str">
-        <v>Bryce, Angela (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T2">
         <v>11</v>
       </c>
       <c r="U2">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
@@ -9790,7 +9790,7 @@
         <v>60</v>
       </c>
       <c r="P42" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="Q42">
         <v>18</v>
@@ -9799,7 +9799,7 @@
         <v>60</v>
       </c>
       <c r="S42" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="T42">
         <v>18</v>
@@ -10218,7 +10218,7 @@
         <v>8</v>
       </c>
       <c r="G49" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="H49">
         <v>8</v>
@@ -10227,7 +10227,7 @@
         <v>60</v>
       </c>
       <c r="J49" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="K49">
         <v>8</v>
@@ -10626,7 +10626,7 @@
         <v>60</v>
       </c>
       <c r="M55" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="N55">
         <v>2</v>
@@ -10635,7 +10635,7 @@
         <v>60</v>
       </c>
       <c r="P55" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q55">
         <v>2</v>
@@ -10738,16 +10738,16 @@
         <v>6.75</v>
       </c>
       <c r="G57" t="str">
-        <v>McConnell, Marion</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H57">
         <v>10</v>
       </c>
       <c r="I57">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="J57" t="str">
-        <v>Duncan, George</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K57">
         <v>10</v>
@@ -10756,7 +10756,7 @@
         <v>60</v>
       </c>
       <c r="M57" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="N57">
         <v>10</v>
@@ -10765,7 +10765,7 @@
         <v>60</v>
       </c>
       <c r="P57" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Murray, James</v>
       </c>
       <c r="Q57">
         <v>10</v>
@@ -10774,7 +10774,7 @@
         <v>60</v>
       </c>
       <c r="S57" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="T57">
         <v>10</v>
@@ -10830,7 +10830,7 @@
         <v>60</v>
       </c>
       <c r="P58" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="Q58">
         <v>4</v>
@@ -10839,7 +10839,7 @@
         <v>60</v>
       </c>
       <c r="S58" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="T58">
         <v>4</v>
@@ -10998,7 +10998,7 @@
         <v>3</v>
       </c>
       <c r="G61" t="str">
-        <v>Collie, Mattie (F)</v>
+        <v>East NL, Glasgow</v>
       </c>
       <c r="H61">
         <v>1</v>
@@ -11007,7 +11007,7 @@
         <v>60</v>
       </c>
       <c r="J61" t="str">
-        <v>East NL, Glasgow</v>
+        <v>Clements, Jessie (F)</v>
       </c>
       <c r="K61">
         <v>1</v>
@@ -11025,7 +11025,7 @@
         <v>60</v>
       </c>
       <c r="P61" t="str">
-        <v>Clements, Jessie (F)</v>
+        <v>Collie, Mattie (F)</v>
       </c>
       <c r="Q61">
         <v>1</v>
@@ -11128,7 +11128,7 @@
         <v>7</v>
       </c>
       <c r="G63" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="H63">
         <v>8</v>
@@ -11137,7 +11137,7 @@
         <v>60</v>
       </c>
       <c r="J63" t="str">
-        <v>Murray, James</v>
+        <v>Morris, Jack (F)</v>
       </c>
       <c r="K63">
         <v>8</v>
@@ -11341,7 +11341,7 @@
         <v>60</v>
       </c>
       <c r="M66" t="str">
-        <v>Morris, Jack (F)</v>
+        <v>Murray, James</v>
       </c>
       <c r="N66">
         <v>9</v>
@@ -11350,7 +11350,7 @@
         <v>60</v>
       </c>
       <c r="P66" t="str">
-        <v>Murray, James</v>
+        <v>Campbell, Neil</v>
       </c>
       <c r="Q66">
         <v>9</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update the capacity dashboard to reflect branch-specific data
Update capacity_dashboard.xlsx to implement branch-specific data loading.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J45"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,7 +442,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="B2" t="str">
         <v>30</v>
@@ -454,7 +454,7 @@
         <v>2025-11-03</v>
       </c>
       <c r="E2" t="str">
-        <v>Holiday</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -466,15 +466,15 @@
         <v>0</v>
       </c>
       <c r="I2" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v>Ola going on paternity leave (MU 21/10/2025) [availability ignored due to day-level leave]</v>
       </c>
       <c r="J2" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">AB11 8DQ  </v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="B3" t="str">
         <v>30</v>
@@ -501,12 +501,12 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J3" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">AB11 8DQ  </v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="B4" t="str">
         <v>30</v>
@@ -533,12 +533,12 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J4" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">AB11 8DQ  </v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="B5" t="str">
         <v>30</v>
@@ -565,12 +565,12 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J5" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">AB11 8DQ  </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="B6" t="str">
         <v>30</v>
@@ -597,12 +597,12 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J6" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">AB11 8DQ  </v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="B7" t="str">
         <v>30</v>
@@ -629,12 +629,12 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J7" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">AB11 8DQ  </v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="B8" t="str">
         <v>30</v>
@@ -661,18 +661,18 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J8" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">AB11 8DQ  </v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Eilish McNally</v>
+        <v>Kirstie Quirke (GH)</v>
       </c>
       <c r="B9" t="str">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C9" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D9" t="str">
         <v>2025-11-03</v>
@@ -681,510 +681,510 @@
         <v>Available</v>
       </c>
       <c r="F9" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G9" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H9" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I9" t="str">
         <v/>
       </c>
       <c r="J9" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">AB11 8LH  </v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Eilish McNally</v>
+        <v>Kirstie Quirke (GH)</v>
       </c>
       <c r="B10" t="str">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C10" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-06</v>
       </c>
       <c r="E10" t="str">
         <v>Available</v>
       </c>
       <c r="F10" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G10" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H10" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I10" t="str">
         <v/>
       </c>
       <c r="J10" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">AB11 8LH  </v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Eilish McNally</v>
+        <v>Kirstie Quirke (GH)</v>
       </c>
       <c r="B11" t="str">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C11" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D11" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-07</v>
       </c>
       <c r="E11" t="str">
         <v>Available</v>
       </c>
       <c r="F11" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>09:00-14:30</v>
       </c>
       <c r="G11" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H11" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I11" t="str">
         <v/>
       </c>
       <c r="J11" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">AB11 8LH  </v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Eilish McNally</v>
+        <v>Kirstie Quirke (GH)</v>
       </c>
       <c r="B12" t="str">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C12" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-09</v>
       </c>
       <c r="E12" t="str">
         <v>Available</v>
       </c>
       <c r="F12" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G12" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H12" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I12" t="str">
         <v/>
       </c>
       <c r="J12" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">AB11 8LH  </v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Marie Vettrino</v>
+        <v>Anish Kumar (GH)</v>
       </c>
       <c r="B13" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C13" t="str">
-        <v>3</v>
+        <v>5.33</v>
       </c>
       <c r="D13" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-07</v>
       </c>
       <c r="E13" t="str">
         <v>Available</v>
       </c>
       <c r="F13" t="str">
-        <v>09:30-10:30; 18:30-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G13" t="str">
-        <v>3</v>
+        <v>5.33</v>
       </c>
       <c r="H13" t="str">
-        <v>3</v>
+        <v>5.33</v>
       </c>
       <c r="I13" t="str">
         <v/>
       </c>
       <c r="J13" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">AB25 1GN  </v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Marie Vettrino</v>
+        <v>Anish Kumar (GH)</v>
       </c>
       <c r="B14" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C14" t="str">
-        <v>3</v>
+        <v>5.33</v>
       </c>
       <c r="D14" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-08</v>
       </c>
       <c r="E14" t="str">
         <v>Available</v>
       </c>
       <c r="F14" t="str">
-        <v>18:30-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G14" t="str">
-        <v>3</v>
+        <v>5.33</v>
       </c>
       <c r="H14" t="str">
-        <v>3</v>
+        <v>5.33</v>
       </c>
       <c r="I14" t="str">
         <v/>
       </c>
       <c r="J14" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">AB25 1GN  </v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Marie Vettrino</v>
+        <v>Anish Kumar (GH)</v>
       </c>
       <c r="B15" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C15" t="str">
-        <v>3</v>
+        <v>5.33</v>
       </c>
       <c r="D15" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-09</v>
       </c>
       <c r="E15" t="str">
         <v>Available</v>
       </c>
       <c r="F15" t="str">
-        <v>09:30-10:30; 18:30-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G15" t="str">
-        <v>3</v>
+        <v>5.33</v>
       </c>
       <c r="H15" t="str">
-        <v>3</v>
+        <v>5.33</v>
       </c>
       <c r="I15" t="str">
         <v/>
       </c>
       <c r="J15" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">AB25 1GN  </v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Marie Vettrino</v>
+        <v>Chance Devereaux-Colby (GH)</v>
       </c>
       <c r="B16" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C16" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="D16" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-04</v>
       </c>
       <c r="E16" t="str">
         <v>Available</v>
       </c>
       <c r="F16" t="str">
-        <v>10:30-11:30; 16:45-17:45</v>
+        <v>07:00-22:00</v>
       </c>
       <c r="G16" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H16" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="I16" t="str">
         <v/>
       </c>
       <c r="J16" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">AB24 2GG  </v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Marie Vettrino</v>
+        <v>Chance Devereaux-Colby (GH)</v>
       </c>
       <c r="B17" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C17" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="D17" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-05</v>
       </c>
       <c r="E17" t="str">
         <v>Available</v>
       </c>
       <c r="F17" t="str">
-        <v>10:30-11:30; 16:45-17:45</v>
+        <v>07:00-22:00</v>
       </c>
       <c r="G17" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H17" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="I17" t="str">
         <v/>
       </c>
       <c r="J17" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">AB24 2GG  </v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Chance Devereaux-Colby (GH)</v>
       </c>
       <c r="B18" t="str">
         <v>16</v>
       </c>
       <c r="C18" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="D18" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-06</v>
       </c>
       <c r="E18" t="str">
         <v>Available</v>
       </c>
       <c r="F18" t="str">
-        <v>09:30-15:00</v>
+        <v>07:00-22:00</v>
       </c>
       <c r="G18" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="H18" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="I18" t="str">
         <v/>
       </c>
       <c r="J18" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">AB24 2GG  </v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Chance Devereaux-Colby (GH)</v>
       </c>
       <c r="B19" t="str">
         <v>16</v>
       </c>
       <c r="C19" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="D19" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-08</v>
       </c>
       <c r="E19" t="str">
         <v>Available</v>
       </c>
       <c r="F19" t="str">
-        <v>09:30-15:00</v>
+        <v>07:00-22:00</v>
       </c>
       <c r="G19" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="H19" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="I19" t="str">
         <v/>
       </c>
       <c r="J19" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">AB24 2GG  </v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Chance Devereaux-Colby (GH)</v>
       </c>
       <c r="B20" t="str">
         <v>16</v>
       </c>
       <c r="C20" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="D20" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-09</v>
       </c>
       <c r="E20" t="str">
         <v>Available</v>
       </c>
       <c r="F20" t="str">
-        <v>09:30-15:00</v>
+        <v>07:00-22:00</v>
       </c>
       <c r="G20" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="H20" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="I20" t="str">
         <v/>
       </c>
       <c r="J20" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">AB24 2GG  </v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Sunny Addey (GH)</v>
       </c>
       <c r="B21" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C21" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="D21" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-04</v>
       </c>
       <c r="E21" t="str">
         <v>Available</v>
       </c>
       <c r="F21" t="str">
-        <v>09:30-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G21" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="H21" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="I21" t="str">
         <v/>
       </c>
       <c r="J21" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">AB24 1UW  </v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Sunny Addey (GH)</v>
       </c>
       <c r="B22" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C22" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="D22" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-05</v>
       </c>
       <c r="E22" t="str">
         <v>Available</v>
       </c>
       <c r="F22" t="str">
-        <v>09:30-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G22" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="H22" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="I22" t="str">
         <v/>
       </c>
       <c r="J22" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">AB24 1UW  </v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Sunny Addey (GH)</v>
       </c>
       <c r="B23" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C23" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="D23" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-06</v>
       </c>
       <c r="E23" t="str">
         <v>Available</v>
       </c>
       <c r="F23" t="str">
-        <v>09:30-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G23" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="H23" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="I23" t="str">
         <v/>
       </c>
       <c r="J23" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">AB24 1UW  </v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Sunny Addey (GH)</v>
       </c>
       <c r="B24" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C24" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="D24" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-07</v>
       </c>
       <c r="E24" t="str">
         <v>Available</v>
       </c>
       <c r="F24" t="str">
-        <v>09:30-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G24" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="H24" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="I24" t="str">
         <v/>
       </c>
       <c r="J24" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">AB24 1UW  </v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Romina Ferrara</v>
+        <v>Tobiloba Akinlosotu (GH)</v>
       </c>
       <c r="B25" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C25" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="D25" t="str">
         <v>2025-11-03</v>
@@ -1193,30 +1193,30 @@
         <v>Available</v>
       </c>
       <c r="F25" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G25" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="H25" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="I25" t="str">
         <v/>
       </c>
       <c r="J25" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">AB25 2RF  </v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Romina Ferrara</v>
+        <v>Tobiloba Akinlosotu (GH)</v>
       </c>
       <c r="B26" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C26" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="D26" t="str">
         <v>2025-11-04</v>
@@ -1225,129 +1225,129 @@
         <v>Available</v>
       </c>
       <c r="F26" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G26" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="H26" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="I26" t="str">
         <v/>
       </c>
       <c r="J26" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">AB25 2RF  </v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Romina Ferrara</v>
+        <v>Tobiloba Akinlosotu (GH)</v>
       </c>
       <c r="B27" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C27" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="D27" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-08</v>
       </c>
       <c r="E27" t="str">
         <v>Available</v>
       </c>
       <c r="F27" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G27" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="H27" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="I27" t="str">
         <v/>
       </c>
       <c r="J27" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">AB25 2RF  </v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Romina Ferrara</v>
+        <v>Tobiloba Akinlosotu (GH)</v>
       </c>
       <c r="B28" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C28" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="D28" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-09</v>
       </c>
       <c r="E28" t="str">
         <v>Available</v>
       </c>
       <c r="F28" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G28" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="H28" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="I28" t="str">
         <v/>
       </c>
       <c r="J28" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">AB25 2RF  </v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Romina Ferrara</v>
+        <v>Deborah Bright (W) (GH)</v>
       </c>
       <c r="B29" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C29" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="D29" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-03</v>
       </c>
       <c r="E29" t="str">
         <v>Available</v>
       </c>
       <c r="F29" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G29" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="H29" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="I29" t="str">
         <v/>
       </c>
       <c r="J29" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">AB24 3EX  </v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Deborah Bright (W) (GH)</v>
       </c>
       <c r="B30" t="str">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C30" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="D30" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-04</v>
       </c>
       <c r="E30" t="str">
         <v>Available</v>
@@ -1356,30 +1356,30 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G30" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H30" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="I30" t="str">
         <v/>
       </c>
       <c r="J30" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">AB24 3EX  </v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Deborah Bright (W) (GH)</v>
       </c>
       <c r="B31" t="str">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C31" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="D31" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-08</v>
       </c>
       <c r="E31" t="str">
         <v>Available</v>
@@ -1388,30 +1388,30 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G31" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H31" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="I31" t="str">
         <v/>
       </c>
       <c r="J31" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">AB24 3EX  </v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Deborah Bright (W) (GH)</v>
       </c>
       <c r="B32" t="str">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C32" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="D32" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-09</v>
       </c>
       <c r="E32" t="str">
         <v>Available</v>
@@ -1420,30 +1420,30 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G32" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H32" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="I32" t="str">
         <v/>
       </c>
       <c r="J32" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">AB24 3EX  </v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
       </c>
       <c r="B33" t="str">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C33" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="D33" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-04</v>
       </c>
       <c r="E33" t="str">
         <v>Available</v>
@@ -1452,30 +1452,30 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G33" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H33" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="I33" t="str">
         <v/>
       </c>
       <c r="J33" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">AB10 7BQ  </v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
       </c>
       <c r="B34" t="str">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C34" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="D34" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-05</v>
       </c>
       <c r="E34" t="str">
         <v>Available</v>
@@ -1484,30 +1484,30 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G34" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H34" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="I34" t="str">
         <v/>
       </c>
       <c r="J34" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">AB10 7BQ  </v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
       </c>
       <c r="B35" t="str">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C35" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="D35" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-06</v>
       </c>
       <c r="E35" t="str">
         <v>Available</v>
@@ -1516,30 +1516,30 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G35" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H35" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="I35" t="str">
         <v/>
       </c>
       <c r="J35" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">AB10 7BQ  </v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
       </c>
       <c r="B36" t="str">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C36" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="D36" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-07</v>
       </c>
       <c r="E36" t="str">
         <v>Available</v>
@@ -1548,725 +1548,309 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G36" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H36" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="I36" t="str">
         <v/>
       </c>
       <c r="J36" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">AB10 7BQ  </v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Anne Morrison</v>
+        <v>Jacqueline Clark</v>
       </c>
       <c r="B37" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C37" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="D37" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-04</v>
       </c>
       <c r="E37" t="str">
         <v>Available</v>
       </c>
       <c r="F37" t="str">
-        <v>12:00-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G37" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="H37" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="I37" t="str">
         <v/>
       </c>
       <c r="J37" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">AB11 8BP  </v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Anne Morrison</v>
+        <v>Jacqueline Clark</v>
       </c>
       <c r="B38" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C38" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="D38" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-05</v>
       </c>
       <c r="E38" t="str">
         <v>Available</v>
       </c>
       <c r="F38" t="str">
-        <v>12:00-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G38" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="H38" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="I38" t="str">
         <v/>
       </c>
       <c r="J38" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">AB11 8BP  </v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Anne Morrison</v>
+        <v>Jacqueline Clark</v>
       </c>
       <c r="B39" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C39" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="D39" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-06</v>
       </c>
       <c r="E39" t="str">
         <v>Available</v>
       </c>
       <c r="F39" t="str">
-        <v>09:15-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G39" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="H39" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="I39" t="str">
         <v/>
       </c>
       <c r="J39" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">AB11 8BP  </v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Anne Morrison</v>
+        <v>Jacqueline Clark</v>
       </c>
       <c r="B40" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C40" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="D40" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-07</v>
       </c>
       <c r="E40" t="str">
         <v>Available</v>
       </c>
       <c r="F40" t="str">
-        <v>09:15-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G40" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="H40" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="I40" t="str">
         <v/>
       </c>
       <c r="J40" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">AB11 8BP  </v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Anne Morrison</v>
+        <v>Sharon Jane Riley (W) (GH)</v>
       </c>
       <c r="B41" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C41" t="str">
-        <v>1.67</v>
+        <v>6</v>
       </c>
       <c r="D41" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-03</v>
       </c>
       <c r="E41" t="str">
         <v>Available</v>
       </c>
       <c r="F41" t="str">
-        <v>12:00-17:45</v>
+        <v>07:00-22:10</v>
       </c>
       <c r="G41" t="str">
-        <v>1.67</v>
+        <v>6</v>
       </c>
       <c r="H41" t="str">
-        <v>1.67</v>
+        <v>6</v>
       </c>
       <c r="I41" t="str">
         <v/>
       </c>
       <c r="J41" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">AB12 3WF  </v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Anne Morrison</v>
+        <v>Sharon Jane Riley (W) (GH)</v>
       </c>
       <c r="B42" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C42" t="str">
-        <v>1.67</v>
+        <v>6</v>
       </c>
       <c r="D42" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-04</v>
       </c>
       <c r="E42" t="str">
         <v>Available</v>
       </c>
       <c r="F42" t="str">
-        <v>21:00-22:00</v>
+        <v>07:00-22:10</v>
       </c>
       <c r="G42" t="str">
-        <v>1.67</v>
+        <v>6</v>
       </c>
       <c r="H42" t="str">
-        <v>1.67</v>
+        <v>6</v>
       </c>
       <c r="I42" t="str">
         <v/>
       </c>
       <c r="J42" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">AB12 3WF  </v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Sharon Jane Riley (W) (GH)</v>
       </c>
       <c r="B43" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C43" t="str">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="D43" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-05</v>
       </c>
       <c r="E43" t="str">
         <v>Available</v>
       </c>
       <c r="F43" t="str">
-        <v>08:00-18:00</v>
+        <v>07:00-22:10</v>
       </c>
       <c r="G43" t="str">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="H43" t="str">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="I43" t="str">
         <v/>
       </c>
       <c r="J43" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
+        <v xml:space="preserve">AB12 3WF  </v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Sharon Jane Riley (W) (GH)</v>
       </c>
       <c r="B44" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C44" t="str">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="D44" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-08</v>
       </c>
       <c r="E44" t="str">
         <v>Available</v>
       </c>
       <c r="F44" t="str">
-        <v>08:00-18:00</v>
+        <v>07:00-22:10</v>
       </c>
       <c r="G44" t="str">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="H44" t="str">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="I44" t="str">
         <v/>
       </c>
       <c r="J44" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
+        <v xml:space="preserve">AB12 3WF  </v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Sharon Jane Riley (W) (GH)</v>
       </c>
       <c r="B45" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C45" t="str">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="D45" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-09</v>
       </c>
       <c r="E45" t="str">
         <v>Available</v>
       </c>
       <c r="F45" t="str">
-        <v>08:00-18:00</v>
+        <v>07:00-22:10</v>
       </c>
       <c r="G45" t="str">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="H45" t="str">
-        <v>2.5</v>
+        <v>6</v>
       </c>
       <c r="I45" t="str">
         <v/>
       </c>
       <c r="J45" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v>Elizabeth Adams</v>
-      </c>
-      <c r="B46" t="str">
-        <v>10</v>
-      </c>
-      <c r="C46" t="str">
-        <v>2.5</v>
-      </c>
-      <c r="D46" t="str">
-        <v>2025-11-06</v>
-      </c>
-      <c r="E46" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F46" t="str">
-        <v>08:00-18:00</v>
-      </c>
-      <c r="G46" t="str">
-        <v>2.5</v>
-      </c>
-      <c r="H46" t="str">
-        <v>2.5</v>
-      </c>
-      <c r="I46" t="str">
-        <v/>
-      </c>
-      <c r="J46" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>Helen Morrison (GH)</v>
-      </c>
-      <c r="B47" t="str">
-        <v>15</v>
-      </c>
-      <c r="C47" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="D47" t="str">
-        <v>2025-11-03</v>
-      </c>
-      <c r="E47" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F47" t="str">
-        <v>08:00-16:30</v>
-      </c>
-      <c r="G47" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="H47" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="I47" t="str">
-        <v/>
-      </c>
-      <c r="J47" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>Helen Morrison (GH)</v>
-      </c>
-      <c r="B48" t="str">
-        <v>15</v>
-      </c>
-      <c r="C48" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="D48" t="str">
-        <v>2025-11-04</v>
-      </c>
-      <c r="E48" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F48" t="str">
-        <v>08:00-16:00</v>
-      </c>
-      <c r="G48" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="H48" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="I48" t="str">
-        <v/>
-      </c>
-      <c r="J48" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="str">
-        <v>Helen Morrison (GH)</v>
-      </c>
-      <c r="B49" t="str">
-        <v>15</v>
-      </c>
-      <c r="C49" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="D49" t="str">
-        <v>2025-11-08</v>
-      </c>
-      <c r="E49" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F49" t="str">
-        <v>08:00-16:30</v>
-      </c>
-      <c r="G49" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="H49" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="I49" t="str">
-        <v/>
-      </c>
-      <c r="J49" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="str">
-        <v>Helen Morrison (GH)</v>
-      </c>
-      <c r="B50" t="str">
-        <v>15</v>
-      </c>
-      <c r="C50" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="D50" t="str">
-        <v>2025-11-09</v>
-      </c>
-      <c r="E50" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F50" t="str">
-        <v>08:00-16:00</v>
-      </c>
-      <c r="G50" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="H50" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="I50" t="str">
-        <v/>
-      </c>
-      <c r="J50" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="str">
-        <v>Lorraine Parsons</v>
-      </c>
-      <c r="B51" t="str">
-        <v>10</v>
-      </c>
-      <c r="C51" t="str">
-        <v>3.33</v>
-      </c>
-      <c r="D51" t="str">
-        <v>2025-11-04</v>
-      </c>
-      <c r="E51" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F51" t="str">
-        <v>09:30-14:30</v>
-      </c>
-      <c r="G51" t="str">
-        <v>3.33</v>
-      </c>
-      <c r="H51" t="str">
-        <v>3.33</v>
-      </c>
-      <c r="I51" t="str">
-        <v/>
-      </c>
-      <c r="J51" t="str">
-        <v xml:space="preserve">EH22 4FP  </v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="str">
-        <v>Lorraine Parsons</v>
-      </c>
-      <c r="B52" t="str">
-        <v>10</v>
-      </c>
-      <c r="C52" t="str">
-        <v>3.33</v>
-      </c>
-      <c r="D52" t="str">
-        <v>2025-11-05</v>
-      </c>
-      <c r="E52" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F52" t="str">
-        <v>09:30-14:30</v>
-      </c>
-      <c r="G52" t="str">
-        <v>3.33</v>
-      </c>
-      <c r="H52" t="str">
-        <v>3.33</v>
-      </c>
-      <c r="I52" t="str">
-        <v/>
-      </c>
-      <c r="J52" t="str">
-        <v xml:space="preserve">EH22 4FP  </v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="str">
-        <v>Lorraine Parsons</v>
-      </c>
-      <c r="B53" t="str">
-        <v>10</v>
-      </c>
-      <c r="C53" t="str">
-        <v>3.33</v>
-      </c>
-      <c r="D53" t="str">
-        <v>2025-11-07</v>
-      </c>
-      <c r="E53" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F53" t="str">
-        <v>09:30-16:00</v>
-      </c>
-      <c r="G53" t="str">
-        <v>3.33</v>
-      </c>
-      <c r="H53" t="str">
-        <v>3.33</v>
-      </c>
-      <c r="I53" t="str">
-        <v/>
-      </c>
-      <c r="J53" t="str">
-        <v xml:space="preserve">EH22 4FP  </v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="B54" t="str">
-        <v>16</v>
-      </c>
-      <c r="C54" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D54" t="str">
-        <v>2025-11-03</v>
-      </c>
-      <c r="E54" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F54" t="str">
-        <v>08:00-15:30</v>
-      </c>
-      <c r="G54" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H54" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I54" t="str">
-        <v/>
-      </c>
-      <c r="J54" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="B55" t="str">
-        <v>16</v>
-      </c>
-      <c r="C55" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D55" t="str">
-        <v>2025-11-04</v>
-      </c>
-      <c r="E55" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F55" t="str">
-        <v>08:00-15:30</v>
-      </c>
-      <c r="G55" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H55" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I55" t="str">
-        <v/>
-      </c>
-      <c r="J55" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="B56" t="str">
-        <v>16</v>
-      </c>
-      <c r="C56" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D56" t="str">
-        <v>2025-11-05</v>
-      </c>
-      <c r="E56" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F56" t="str">
-        <v>08:00-15:30</v>
-      </c>
-      <c r="G56" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H56" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I56" t="str">
-        <v/>
-      </c>
-      <c r="J56" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="B57" t="str">
-        <v>16</v>
-      </c>
-      <c r="C57" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D57" t="str">
-        <v>2025-11-06</v>
-      </c>
-      <c r="E57" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F57" t="str">
-        <v>08:00-17:30</v>
-      </c>
-      <c r="G57" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H57" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I57" t="str">
-        <v/>
-      </c>
-      <c r="J57" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="B58" t="str">
-        <v>16</v>
-      </c>
-      <c r="C58" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D58" t="str">
-        <v>2025-11-07</v>
-      </c>
-      <c r="E58" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F58" t="str">
-        <v>08:00-15:30</v>
-      </c>
-      <c r="G58" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H58" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I58" t="str">
-        <v/>
-      </c>
-      <c r="J58" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
+        <v xml:space="preserve">AB12 3WF  </v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J45"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2306,22 +1890,22 @@
         <v>2025-11-03</v>
       </c>
       <c r="B2" t="str">
-        <v>20.27</v>
+        <v>25</v>
       </c>
       <c r="C2" t="str">
-        <v>20.27</v>
+        <v>25</v>
       </c>
       <c r="D2" t="str">
-        <v>0</v>
+        <v>4.29</v>
       </c>
       <c r="E2" t="str">
-        <v>4.29</v>
+        <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>34</v>
+        <v>38.5</v>
       </c>
       <c r="G2" t="str">
-        <v>-13.73</v>
+        <v>-13.5</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -2332,10 +1916,10 @@
         <v>2025-11-04</v>
       </c>
       <c r="B3" t="str">
-        <v>26.6</v>
+        <v>43.2</v>
       </c>
       <c r="C3" t="str">
-        <v>26.6</v>
+        <v>43.2</v>
       </c>
       <c r="D3" t="str">
         <v>0</v>
@@ -2344,13 +1928,13 @@
         <v>4.29</v>
       </c>
       <c r="F3" t="str">
-        <v>34</v>
+        <v>38.25</v>
       </c>
       <c r="G3" t="str">
-        <v>-7.4</v>
+        <v>4.95</v>
       </c>
       <c r="H3" t="str">
-        <v>Shortage</v>
+        <v>Sufficient</v>
       </c>
     </row>
     <row r="4">
@@ -2358,10 +1942,10 @@
         <v>2025-11-05</v>
       </c>
       <c r="B4" t="str">
-        <v>22.85</v>
+        <v>28.2</v>
       </c>
       <c r="C4" t="str">
-        <v>22.85</v>
+        <v>28.2</v>
       </c>
       <c r="D4" t="str">
         <v>0</v>
@@ -2370,10 +1954,10 @@
         <v>4.29</v>
       </c>
       <c r="F4" t="str">
-        <v>48.5</v>
+        <v>38.5</v>
       </c>
       <c r="G4" t="str">
-        <v>-25.65</v>
+        <v>-10.3</v>
       </c>
       <c r="H4" t="str">
         <v>Shortage</v>
@@ -2384,10 +1968,10 @@
         <v>2025-11-06</v>
       </c>
       <c r="B5" t="str">
-        <v>19.52</v>
+        <v>26.2</v>
       </c>
       <c r="C5" t="str">
-        <v>19.52</v>
+        <v>26.2</v>
       </c>
       <c r="D5" t="str">
         <v>0</v>
@@ -2396,10 +1980,10 @@
         <v>4.29</v>
       </c>
       <c r="F5" t="str">
-        <v>34</v>
+        <v>36.5</v>
       </c>
       <c r="G5" t="str">
-        <v>-14.48</v>
+        <v>-10.3</v>
       </c>
       <c r="H5" t="str">
         <v>Shortage</v>
@@ -2410,10 +1994,10 @@
         <v>2025-11-07</v>
       </c>
       <c r="B6" t="str">
-        <v>14.35</v>
+        <v>28.33</v>
       </c>
       <c r="C6" t="str">
-        <v>14.35</v>
+        <v>28.33</v>
       </c>
       <c r="D6" t="str">
         <v>0</v>
@@ -2422,10 +2006,10 @@
         <v>4.29</v>
       </c>
       <c r="F6" t="str">
-        <v>24.25</v>
+        <v>31.5</v>
       </c>
       <c r="G6" t="str">
-        <v>-9.9</v>
+        <v>-3.17</v>
       </c>
       <c r="H6" t="str">
         <v>Shortage</v>
@@ -2436,10 +2020,10 @@
         <v>2025-11-08</v>
       </c>
       <c r="B7" t="str">
-        <v>11.9</v>
+        <v>29.53</v>
       </c>
       <c r="C7" t="str">
-        <v>11.9</v>
+        <v>29.53</v>
       </c>
       <c r="D7" t="str">
         <v>0</v>
@@ -2448,10 +2032,10 @@
         <v>4.29</v>
       </c>
       <c r="F7" t="str">
-        <v>18.5</v>
+        <v>33.5</v>
       </c>
       <c r="G7" t="str">
-        <v>-6.6</v>
+        <v>-3.97</v>
       </c>
       <c r="H7" t="str">
         <v>Shortage</v>
@@ -2462,10 +2046,10 @@
         <v>2025-11-09</v>
       </c>
       <c r="B8" t="str">
-        <v>13.57</v>
+        <v>33.53</v>
       </c>
       <c r="C8" t="str">
-        <v>13.57</v>
+        <v>33.53</v>
       </c>
       <c r="D8" t="str">
         <v>0</v>
@@ -2474,10 +2058,10 @@
         <v>4.29</v>
       </c>
       <c r="F8" t="str">
-        <v>14.5</v>
+        <v>36</v>
       </c>
       <c r="G8" t="str">
-        <v>-0.93</v>
+        <v>-2.47</v>
       </c>
       <c r="H8" t="str">
         <v>Shortage</v>
@@ -2492,7 +2076,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H58"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2525,25 +2109,25 @@
         <v>2025-11-03</v>
       </c>
       <c r="B2" t="str">
-        <v>Anne Morrison</v>
+        <v>Addey (GH), Sunny</v>
       </c>
       <c r="C2" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D2" t="str">
-        <v>12:00-21:00</v>
+        <v>10:32-12:31</v>
       </c>
       <c r="E2" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="G2" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="3">
@@ -2551,7 +2135,7 @@
         <v>2025-11-03</v>
       </c>
       <c r="B3" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Deborah Bright (W) (GH)</v>
       </c>
       <c r="C3" t="str">
         <v>Available</v>
@@ -2560,13 +2144,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E3" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="F3" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="G3" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -2577,22 +2161,22 @@
         <v>2025-11-03</v>
       </c>
       <c r="B4" t="str">
-        <v>Eilish McNally</v>
+        <v>Kirstie Quirke (GH)</v>
       </c>
       <c r="C4" t="str">
         <v>Available</v>
       </c>
       <c r="D4" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E4" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H4" t="str">
         <v/>
@@ -2603,25 +2187,25 @@
         <v>2025-11-03</v>
       </c>
       <c r="B5" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Kumar (GH), Anish</v>
       </c>
       <c r="C5" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D5" t="str">
-        <v>08:00-18:00</v>
+        <v>14:01-16:02</v>
       </c>
       <c r="E5" t="str">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="F5" t="str">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="G5" t="str">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="6">
@@ -2629,13 +2213,13 @@
         <v>2025-11-03</v>
       </c>
       <c r="B6" t="str">
-        <v>Hartley-Oliver (GH), Ruby</v>
+        <v>Mackie (GH), Natalie</v>
       </c>
       <c r="C6" t="str">
         <v>Ad-hoc</v>
       </c>
       <c r="D6" t="str">
-        <v>10:00-12:00</v>
+        <v>09:29-10:30; 11:30-13:30; 16:05-17:05</v>
       </c>
       <c r="E6" t="str">
         <v>0</v>
@@ -2655,25 +2239,25 @@
         <v>2025-11-03</v>
       </c>
       <c r="B7" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="C7" t="str">
-        <v>Available</v>
+        <v>Maternity/Paternity</v>
       </c>
       <c r="D7" t="str">
-        <v>08:00-16:30</v>
+        <v/>
       </c>
       <c r="E7" t="str">
-        <v>3.75</v>
+        <v>4.29</v>
       </c>
       <c r="F7" t="str">
-        <v>3.75</v>
+        <v>4.29</v>
       </c>
       <c r="G7" t="str">
-        <v>3.75</v>
+        <v>0</v>
       </c>
       <c r="H7" t="str">
-        <v/>
+        <v>Ola going on paternity leave (MU 21/10/2025) [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="8">
@@ -2681,22 +2265,22 @@
         <v>2025-11-03</v>
       </c>
       <c r="B8" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Sharon Jane Riley (W) (GH)</v>
       </c>
       <c r="C8" t="str">
         <v>Available</v>
       </c>
       <c r="D8" t="str">
-        <v>09:30-15:00</v>
+        <v>07:00-22:10</v>
       </c>
       <c r="E8" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="F8" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="G8" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="H8" t="str">
         <v/>
@@ -2707,48 +2291,48 @@
         <v>2025-11-03</v>
       </c>
       <c r="B9" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Tobiloba Akinlosotu (GH)</v>
       </c>
       <c r="C9" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D9" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E9" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="F9" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="G9" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H9" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-04</v>
       </c>
       <c r="B10" t="str">
-        <v>Romina Ferrara</v>
+        <v>Chance Devereaux-Colby (GH)</v>
       </c>
       <c r="C10" t="str">
         <v>Available</v>
       </c>
       <c r="D10" t="str">
-        <v>09:15-10:15</v>
+        <v>07:00-22:00</v>
       </c>
       <c r="E10" t="str">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="F10" t="str">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="G10" t="str">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="H10" t="str">
         <v/>
@@ -2756,25 +2340,25 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-04</v>
       </c>
       <c r="B11" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Deborah Bright (W) (GH)</v>
       </c>
       <c r="C11" t="str">
         <v>Available</v>
       </c>
       <c r="D11" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E11" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F11" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G11" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -2785,22 +2369,22 @@
         <v>2025-11-04</v>
       </c>
       <c r="B12" t="str">
-        <v>Anne Morrison</v>
+        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
       </c>
       <c r="C12" t="str">
         <v>Available</v>
       </c>
       <c r="D12" t="str">
-        <v>12:00-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E12" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="F12" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="G12" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="H12" t="str">
         <v/>
@@ -2811,7 +2395,7 @@
         <v>2025-11-04</v>
       </c>
       <c r="B13" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Jacqueline Clark</v>
       </c>
       <c r="C13" t="str">
         <v>Available</v>
@@ -2820,13 +2404,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E13" t="str">
-        <v>2.86</v>
+        <v>4</v>
       </c>
       <c r="F13" t="str">
-        <v>2.86</v>
+        <v>4</v>
       </c>
       <c r="G13" t="str">
-        <v>2.86</v>
+        <v>4</v>
       </c>
       <c r="H13" t="str">
         <v/>
@@ -2837,25 +2421,25 @@
         <v>2025-11-04</v>
       </c>
       <c r="B14" t="str">
-        <v>Eilish McNally</v>
+        <v>Mackie (GH), Natalie</v>
       </c>
       <c r="C14" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D14" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>09:26-10:25; 12:53-13:52; 16:00-16:59</v>
       </c>
       <c r="E14" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F14" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G14" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="15">
@@ -2863,25 +2447,25 @@
         <v>2025-11-04</v>
       </c>
       <c r="B15" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="C15" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D15" t="str">
-        <v>08:00-18:00</v>
+        <v/>
       </c>
       <c r="E15" t="str">
-        <v>2.5</v>
+        <v>4.29</v>
       </c>
       <c r="F15" t="str">
-        <v>2.5</v>
+        <v>4.29</v>
       </c>
       <c r="G15" t="str">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="H15" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="16">
@@ -2889,25 +2473,25 @@
         <v>2025-11-04</v>
       </c>
       <c r="B16" t="str">
-        <v>Hartley-Oliver (GH), Ruby</v>
+        <v>Sharon Jane Riley (W) (GH)</v>
       </c>
       <c r="C16" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D16" t="str">
-        <v>13:59-16:59</v>
+        <v>07:00-22:10</v>
       </c>
       <c r="E16" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F16" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G16" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H16" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -2915,22 +2499,22 @@
         <v>2025-11-04</v>
       </c>
       <c r="B17" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Sunny Addey (GH)</v>
       </c>
       <c r="C17" t="str">
         <v>Available</v>
       </c>
       <c r="D17" t="str">
-        <v>08:00-16:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E17" t="str">
-        <v>3.75</v>
+        <v>7.5</v>
       </c>
       <c r="F17" t="str">
-        <v>3.75</v>
+        <v>7.5</v>
       </c>
       <c r="G17" t="str">
-        <v>3.75</v>
+        <v>7.5</v>
       </c>
       <c r="H17" t="str">
         <v/>
@@ -2941,22 +2525,22 @@
         <v>2025-11-04</v>
       </c>
       <c r="B18" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Tobiloba Akinlosotu (GH)</v>
       </c>
       <c r="C18" t="str">
         <v>Available</v>
       </c>
       <c r="D18" t="str">
-        <v>09:30-14:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E18" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="F18" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="G18" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="H18" t="str">
         <v/>
@@ -2964,51 +2548,51 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-05</v>
       </c>
       <c r="B19" t="str">
-        <v>Marie Vettrino</v>
+        <v>Bright (W) (GH), Deborah</v>
       </c>
       <c r="C19" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D19" t="str">
-        <v>09:30-10:30; 18:30-21:00</v>
+        <v>09:29-11:30</v>
       </c>
       <c r="E19" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F19" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G19" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H19" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-05</v>
       </c>
       <c r="B20" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Chance Devereaux-Colby (GH)</v>
       </c>
       <c r="C20" t="str">
         <v>Available</v>
       </c>
       <c r="D20" t="str">
-        <v>09:30-15:00</v>
+        <v>07:00-22:00</v>
       </c>
       <c r="E20" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="F20" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="G20" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -3016,51 +2600,51 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-05</v>
       </c>
       <c r="B21" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
       </c>
       <c r="C21" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D21" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E21" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="F21" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="G21" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H21" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-05</v>
       </c>
       <c r="B22" t="str">
-        <v>Romina Ferrara</v>
+        <v>Jacqueline Clark</v>
       </c>
       <c r="C22" t="str">
         <v>Available</v>
       </c>
       <c r="D22" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E22" t="str">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F22" t="str">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G22" t="str">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H22" t="str">
         <v/>
@@ -3068,28 +2652,28 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-05</v>
       </c>
       <c r="B23" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Mackie (GH), Natalie</v>
       </c>
       <c r="C23" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D23" t="str">
-        <v>08:00-15:30</v>
+        <v>07:59-09:00; 09:29-10:30; 10:59-12:00; 12:29-13:30; 16:00-16:59</v>
       </c>
       <c r="E23" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="F23" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="G23" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H23" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="24">
@@ -3097,25 +2681,25 @@
         <v>2025-11-05</v>
       </c>
       <c r="B24" t="str">
-        <v>Anne Morrison</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="C24" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D24" t="str">
-        <v>09:15-21:00</v>
+        <v/>
       </c>
       <c r="E24" t="str">
-        <v>1.67</v>
+        <v>4.29</v>
       </c>
       <c r="F24" t="str">
-        <v>1.67</v>
+        <v>4.29</v>
       </c>
       <c r="G24" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="H24" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="25">
@@ -3123,22 +2707,22 @@
         <v>2025-11-05</v>
       </c>
       <c r="B25" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Sharon Jane Riley (W) (GH)</v>
       </c>
       <c r="C25" t="str">
         <v>Available</v>
       </c>
       <c r="D25" t="str">
-        <v>08:00-21:30</v>
+        <v>07:00-22:10</v>
       </c>
       <c r="E25" t="str">
-        <v>2.86</v>
+        <v>6</v>
       </c>
       <c r="F25" t="str">
-        <v>2.86</v>
+        <v>6</v>
       </c>
       <c r="G25" t="str">
-        <v>2.86</v>
+        <v>6</v>
       </c>
       <c r="H25" t="str">
         <v/>
@@ -3149,22 +2733,22 @@
         <v>2025-11-05</v>
       </c>
       <c r="B26" t="str">
-        <v>Eilish McNally</v>
+        <v>Sunny Addey (GH)</v>
       </c>
       <c r="C26" t="str">
         <v>Available</v>
       </c>
       <c r="D26" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E26" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="F26" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="G26" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H26" t="str">
         <v/>
@@ -3172,25 +2756,25 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B27" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Chance Devereaux-Colby (GH)</v>
       </c>
       <c r="C27" t="str">
         <v>Available</v>
       </c>
       <c r="D27" t="str">
-        <v>08:00-18:00</v>
+        <v>07:00-22:00</v>
       </c>
       <c r="E27" t="str">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="F27" t="str">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="G27" t="str">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="H27" t="str">
         <v/>
@@ -3198,25 +2782,25 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B28" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
       </c>
       <c r="C28" t="str">
         <v>Available</v>
       </c>
       <c r="D28" t="str">
-        <v>09:30-14:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E28" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="F28" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="G28" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -3224,25 +2808,25 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B29" t="str">
-        <v>Marie Vettrino</v>
+        <v>Jacqueline Clark</v>
       </c>
       <c r="C29" t="str">
         <v>Available</v>
       </c>
       <c r="D29" t="str">
-        <v>18:30-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E29" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F29" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G29" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -3250,25 +2834,25 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B30" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Kirstie Quirke (GH)</v>
       </c>
       <c r="C30" t="str">
         <v>Available</v>
       </c>
       <c r="D30" t="str">
-        <v>09:30-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E30" t="str">
-        <v>2.29</v>
+        <v>4</v>
       </c>
       <c r="F30" t="str">
-        <v>2.29</v>
+        <v>4</v>
       </c>
       <c r="G30" t="str">
-        <v>2.29</v>
+        <v>4</v>
       </c>
       <c r="H30" t="str">
         <v/>
@@ -3276,16 +2860,16 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B31" t="str">
-        <v>Morrison (GH), Helen</v>
+        <v>Mackie (GH), Natalie</v>
       </c>
       <c r="C31" t="str">
         <v>Ad-hoc</v>
       </c>
       <c r="D31" t="str">
-        <v>07:59-09:00; 09:15-10:14</v>
+        <v>09:29-10:30; 11:30-13:30</v>
       </c>
       <c r="E31" t="str">
         <v>0</v>
@@ -3302,10 +2886,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B32" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="C32" t="str">
         <v>Holiday</v>
@@ -3328,51 +2912,51 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B33" t="str">
-        <v>Romina Ferrara</v>
+        <v>Riley (W) (GH), Sharon Jane</v>
       </c>
       <c r="C33" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D33" t="str">
-        <v>09:15-10:15</v>
+        <v>07:59-09:00; 11:44-12:45</v>
       </c>
       <c r="E33" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H33" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B34" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Sunny Addey (GH)</v>
       </c>
       <c r="C34" t="str">
         <v>Available</v>
       </c>
       <c r="D34" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E34" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F34" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G34" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H34" t="str">
         <v/>
@@ -3380,25 +2964,25 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B35" t="str">
-        <v>Anne Morrison</v>
+        <v>Anish Kumar (GH)</v>
       </c>
       <c r="C35" t="str">
         <v>Available</v>
       </c>
       <c r="D35" t="str">
-        <v>09:15-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E35" t="str">
-        <v>1.67</v>
+        <v>5.33</v>
       </c>
       <c r="F35" t="str">
-        <v>1.67</v>
+        <v>5.33</v>
       </c>
       <c r="G35" t="str">
-        <v>1.67</v>
+        <v>5.33</v>
       </c>
       <c r="H35" t="str">
         <v/>
@@ -3406,10 +2990,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B36" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
       </c>
       <c r="C36" t="str">
         <v>Available</v>
@@ -3418,13 +3002,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E36" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="F36" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="G36" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H36" t="str">
         <v/>
@@ -3432,25 +3016,25 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B37" t="str">
-        <v>Eilish McNally</v>
+        <v>Jacqueline Clark</v>
       </c>
       <c r="C37" t="str">
         <v>Available</v>
       </c>
       <c r="D37" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E37" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F37" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G37" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H37" t="str">
         <v/>
@@ -3458,25 +3042,25 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B38" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Kirstie Quirke (GH)</v>
       </c>
       <c r="C38" t="str">
         <v>Available</v>
       </c>
       <c r="D38" t="str">
-        <v>08:00-18:00</v>
+        <v>09:00-14:30</v>
       </c>
       <c r="E38" t="str">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="F38" t="str">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="G38" t="str">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="H38" t="str">
         <v/>
@@ -3484,16 +3068,16 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B39" t="str">
-        <v>Hartley-Oliver (GH), Ruby</v>
+        <v>Mackie (GH), Natalie</v>
       </c>
       <c r="C39" t="str">
         <v>Ad-hoc</v>
       </c>
       <c r="D39" t="str">
-        <v>13:59-16:59</v>
+        <v>09:29-10:30; 13:00-13:59; 14:15-15:00; 16:00-16:59</v>
       </c>
       <c r="E39" t="str">
         <v>0</v>
@@ -3510,103 +3094,103 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B40" t="str">
-        <v>Marie Vettrino</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="C40" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D40" t="str">
-        <v>09:30-10:30; 18:30-21:00</v>
+        <v/>
       </c>
       <c r="E40" t="str">
-        <v>3</v>
+        <v>4.29</v>
       </c>
       <c r="F40" t="str">
-        <v>3</v>
+        <v>4.29</v>
       </c>
       <c r="G40" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H40" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B41" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Riley (W) (GH), Sharon Jane</v>
       </c>
       <c r="C41" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D41" t="str">
-        <v>09:30-15:00</v>
+        <v>07:59-09:00</v>
       </c>
       <c r="E41" t="str">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="F41" t="str">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="G41" t="str">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="H41" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B42" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Sunny Addey (GH)</v>
       </c>
       <c r="C42" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D42" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E42" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="F42" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="G42" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H42" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-08</v>
       </c>
       <c r="B43" t="str">
-        <v>Romina Ferrara</v>
+        <v>Anish Kumar (GH)</v>
       </c>
       <c r="C43" t="str">
         <v>Available</v>
       </c>
       <c r="D43" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E43" t="str">
-        <v>1</v>
+        <v>5.33</v>
       </c>
       <c r="F43" t="str">
-        <v>1</v>
+        <v>5.33</v>
       </c>
       <c r="G43" t="str">
-        <v>1</v>
+        <v>5.33</v>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -3614,16 +3198,16 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-08</v>
       </c>
       <c r="B44" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Chance Devereaux-Colby (GH)</v>
       </c>
       <c r="C44" t="str">
         <v>Available</v>
       </c>
       <c r="D44" t="str">
-        <v>08:00-17:30</v>
+        <v>07:00-22:00</v>
       </c>
       <c r="E44" t="str">
         <v>3.2</v>
@@ -3640,36 +3224,36 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-08</v>
       </c>
       <c r="B45" t="str">
-        <v>Anne Morrison</v>
+        <v>Clark, Jacqueline</v>
       </c>
       <c r="C45" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D45" t="str">
-        <v>12:00-17:45</v>
+        <v>07:59-09:00; 09:29-10:30; 11:35-12:35; 16:00-16:59; 18:00-19:00</v>
       </c>
       <c r="E45" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="F45" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="G45" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="H45" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-08</v>
       </c>
       <c r="B46" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Deborah Bright (W) (GH)</v>
       </c>
       <c r="C46" t="str">
         <v>Available</v>
@@ -3678,13 +3262,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E46" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="F46" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="G46" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H46" t="str">
         <v/>
@@ -3692,103 +3276,103 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-08</v>
       </c>
       <c r="B47" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Lazar (GH), Nina</v>
       </c>
       <c r="C47" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D47" t="str">
-        <v>09:30-16:00</v>
+        <v>07:59-09:00; 10:00-10:59; 14:15-15:00; 16:30-17:30; 18:00-19:00</v>
       </c>
       <c r="E47" t="str">
-        <v>3.33</v>
+        <v>0</v>
       </c>
       <c r="F47" t="str">
-        <v>3.33</v>
+        <v>0</v>
       </c>
       <c r="G47" t="str">
-        <v>3.33</v>
+        <v>0</v>
       </c>
       <c r="H47" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-08</v>
       </c>
       <c r="B48" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="C48" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D48" t="str">
-        <v>09:30-15:00</v>
+        <v/>
       </c>
       <c r="E48" t="str">
-        <v>2.29</v>
+        <v>4.29</v>
       </c>
       <c r="F48" t="str">
-        <v>2.29</v>
+        <v>4.29</v>
       </c>
       <c r="G48" t="str">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="H48" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-08</v>
       </c>
       <c r="B49" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Sharon Jane Riley (W) (GH)</v>
       </c>
       <c r="C49" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D49" t="str">
-        <v/>
+        <v>07:00-22:10</v>
       </c>
       <c r="E49" t="str">
-        <v>4.29</v>
+        <v>6</v>
       </c>
       <c r="F49" t="str">
-        <v>4.29</v>
+        <v>6</v>
       </c>
       <c r="G49" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H49" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-08</v>
       </c>
       <c r="B50" t="str">
-        <v>Romina Ferrara</v>
+        <v>Tobiloba Akinlosotu (GH)</v>
       </c>
       <c r="C50" t="str">
         <v>Available</v>
       </c>
       <c r="D50" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E50" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="F50" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="G50" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -3796,42 +3380,42 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-09</v>
       </c>
       <c r="B51" t="str">
-        <v>Vettrino, Marie</v>
+        <v>Anish Kumar (GH)</v>
       </c>
       <c r="C51" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D51" t="str">
-        <v>19:00-21:29</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E51" t="str">
-        <v>0</v>
+        <v>5.33</v>
       </c>
       <c r="F51" t="str">
-        <v>0</v>
+        <v>5.33</v>
       </c>
       <c r="G51" t="str">
-        <v>0</v>
+        <v>5.33</v>
       </c>
       <c r="H51" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-09</v>
       </c>
       <c r="B52" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Chance Devereaux-Colby (GH)</v>
       </c>
       <c r="C52" t="str">
         <v>Available</v>
       </c>
       <c r="D52" t="str">
-        <v>08:00-15:30</v>
+        <v>07:00-22:00</v>
       </c>
       <c r="E52" t="str">
         <v>3.2</v>
@@ -3848,10 +3432,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-09</v>
       </c>
       <c r="B53" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Deborah Bright (W) (GH)</v>
       </c>
       <c r="C53" t="str">
         <v>Available</v>
@@ -3860,13 +3444,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E53" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="F53" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="G53" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H53" t="str">
         <v/>
@@ -3874,103 +3458,103 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-09</v>
       </c>
       <c r="B54" t="str">
-        <v>Hartley-Oliver (GH), Ruby</v>
+        <v>Kirstie Quirke (GH)</v>
       </c>
       <c r="C54" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D54" t="str">
-        <v>12:29-15:29</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E54" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F54" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G54" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H54" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-09</v>
       </c>
       <c r="B55" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Lazar (GH), Nina</v>
       </c>
       <c r="C55" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D55" t="str">
-        <v>08:00-16:30</v>
+        <v>07:59-09:00; 10:00-10:59; 14:15-15:00; 16:30-17:30; 18:00-19:00</v>
       </c>
       <c r="E55" t="str">
-        <v>3.75</v>
+        <v>0</v>
       </c>
       <c r="F55" t="str">
-        <v>3.75</v>
+        <v>0</v>
       </c>
       <c r="G55" t="str">
-        <v>3.75</v>
+        <v>0</v>
       </c>
       <c r="H55" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-09</v>
       </c>
       <c r="B56" t="str">
-        <v>Marie Vettrino</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="C56" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D56" t="str">
-        <v>10:30-11:30; 16:45-17:45</v>
+        <v/>
       </c>
       <c r="E56" t="str">
-        <v>3</v>
+        <v>4.29</v>
       </c>
       <c r="F56" t="str">
-        <v>3</v>
+        <v>4.29</v>
       </c>
       <c r="G56" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H56" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-09</v>
       </c>
       <c r="B57" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Sharon Jane Riley (W) (GH)</v>
       </c>
       <c r="C57" t="str">
         <v>Available</v>
       </c>
       <c r="D57" t="str">
-        <v>09:30-15:00</v>
+        <v>07:00-22:10</v>
       </c>
       <c r="E57" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="F57" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="G57" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="H57" t="str">
         <v/>
@@ -3978,196 +3562,40 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-09</v>
       </c>
       <c r="B58" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Tobiloba Akinlosotu (GH)</v>
       </c>
       <c r="C58" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D58" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E58" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="F58" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="G58" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H58" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <v>2025-11-09</v>
-      </c>
-      <c r="B59" t="str">
-        <v>Anne Morrison</v>
-      </c>
-      <c r="C59" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D59" t="str">
-        <v>21:00-22:00</v>
-      </c>
-      <c r="E59" t="str">
-        <v>1.67</v>
-      </c>
-      <c r="F59" t="str">
-        <v>1.67</v>
-      </c>
-      <c r="G59" t="str">
-        <v>1.67</v>
-      </c>
-      <c r="H59" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <v>2025-11-09</v>
-      </c>
-      <c r="B60" t="str">
-        <v>Dhaval Mithaiwala</v>
-      </c>
-      <c r="C60" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D60" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E60" t="str">
-        <v>2.86</v>
-      </c>
-      <c r="F60" t="str">
-        <v>2.86</v>
-      </c>
-      <c r="G60" t="str">
-        <v>2.86</v>
-      </c>
-      <c r="H60" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="str">
-        <v>2025-11-09</v>
-      </c>
-      <c r="B61" t="str">
-        <v>Helen Morrison (GH)</v>
-      </c>
-      <c r="C61" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D61" t="str">
-        <v>08:00-16:00</v>
-      </c>
-      <c r="E61" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="F61" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="G61" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="H61" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="str">
-        <v>2025-11-09</v>
-      </c>
-      <c r="B62" t="str">
-        <v>Marie Vettrino</v>
-      </c>
-      <c r="C62" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D62" t="str">
-        <v>10:30-11:30; 16:45-17:45</v>
-      </c>
-      <c r="E62" t="str">
-        <v>3</v>
-      </c>
-      <c r="F62" t="str">
-        <v>3</v>
-      </c>
-      <c r="G62" t="str">
-        <v>3</v>
-      </c>
-      <c r="H62" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="str">
-        <v>2025-11-09</v>
-      </c>
-      <c r="B63" t="str">
-        <v>Mikhaila (W) Calder</v>
-      </c>
-      <c r="C63" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D63" t="str">
-        <v>09:30-15:00</v>
-      </c>
-      <c r="E63" t="str">
-        <v>2.29</v>
-      </c>
-      <c r="F63" t="str">
-        <v>2.29</v>
-      </c>
-      <c r="G63" t="str">
-        <v>2.29</v>
-      </c>
-      <c r="H63" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="str">
-        <v>2025-11-09</v>
-      </c>
-      <c r="B64" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
-      </c>
-      <c r="C64" t="str">
-        <v>Holiday</v>
-      </c>
-      <c r="D64" t="str">
-        <v/>
-      </c>
-      <c r="E64" t="str">
-        <v>4.29</v>
-      </c>
-      <c r="F64" t="str">
-        <v>4.29</v>
-      </c>
-      <c r="G64" t="str">
-        <v>0</v>
-      </c>
-      <c r="H64" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H58"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4191,130 +3619,130 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Sunny Addey (GH)</v>
       </c>
       <c r="B2" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C2" t="str">
         <v>Driver</v>
       </c>
       <c r="D2" t="str">
-        <v>Mrs</v>
+        <v>Mr</v>
       </c>
       <c r="E2" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="F2" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
+        <v xml:space="preserve">AB24 1UW  </v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Tobiloba Akinlosotu (GH)</v>
       </c>
       <c r="B3" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C3" t="str">
         <v>Driver</v>
       </c>
       <c r="D3" t="str">
-        <v>Mrs</v>
+        <v>Mr</v>
       </c>
       <c r="E3" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="F3" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
+        <v xml:space="preserve">AB25 2RF  </v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Amy Brown</v>
+        <v>Deborah Bright (W) (GH)</v>
       </c>
       <c r="B4" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C4" t="str">
-        <v>Driver</v>
+        <v>Walker</v>
       </c>
       <c r="D4" t="str">
-        <v>Miss</v>
+        <v>Mrs</v>
       </c>
       <c r="E4" t="str">
         <v>female</v>
       </c>
       <c r="F4" t="str">
-        <v xml:space="preserve">EH21 6DQ  </v>
+        <v xml:space="preserve">AB24 3EX  </v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Jacqueline Clark</v>
       </c>
       <c r="B5" t="str">
         <v>16</v>
       </c>
       <c r="C5" t="str">
-        <v>Walker</v>
+        <v>Driver</v>
       </c>
       <c r="D5" t="str">
-        <v>Miss</v>
+        <v>Mrs</v>
       </c>
       <c r="E5" t="str">
         <v>female</v>
       </c>
       <c r="F5" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">AB11 8BP  </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Romina Ferrara</v>
+        <v>Chance Devereaux-Colby (GH)</v>
       </c>
       <c r="B6" t="str">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="C6" t="str">
         <v>Driver</v>
       </c>
       <c r="D6" t="str">
-        <v>Miss</v>
+        <v>Mr</v>
       </c>
       <c r="E6" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="F6" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">AB24 2GG  </v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Eilish McNally</v>
+        <v>Olakunle Folarin (GH)</v>
       </c>
       <c r="B7" t="str">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="C7" t="str">
         <v>Driver</v>
       </c>
       <c r="D7" t="str">
-        <v>Miss</v>
+        <v>Mr</v>
       </c>
       <c r="E7" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="F7" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">AB11 8DQ  </v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Anish Kumar (GH)</v>
       </c>
       <c r="B8" t="str">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C8" t="str">
         <v>Driver</v>
@@ -4326,38 +3754,38 @@
         <v>male</v>
       </c>
       <c r="F8" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">AB25 1GN  </v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Anne Morrison</v>
+        <v>Kirstie Quirke (GH)</v>
       </c>
       <c r="B9" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C9" t="str">
         <v>Driver</v>
       </c>
       <c r="D9" t="str">
-        <v>Mrs</v>
+        <v>Miss</v>
       </c>
       <c r="E9" t="str">
         <v>female</v>
       </c>
       <c r="F9" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">AB11 8LH  </v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Sharon Jane Riley (W) (GH)</v>
       </c>
       <c r="B10" t="str">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="C10" t="str">
-        <v>Driver</v>
+        <v>Walker</v>
       </c>
       <c r="D10" t="str">
         <v>Mrs</v>
@@ -4366,15 +3794,15 @@
         <v>female</v>
       </c>
       <c r="F10" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
+        <v xml:space="preserve">AB12 3WF  </v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
       </c>
       <c r="B11" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C11" t="str">
         <v>Driver</v>
@@ -4386,52 +3814,12 @@
         <v>female</v>
       </c>
       <c r="F11" t="str">
-        <v xml:space="preserve">EH22 4FP  </v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
-      </c>
-      <c r="B12" t="str">
-        <v>30</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Driver</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Mr</v>
-      </c>
-      <c r="E12" t="str">
-        <v>male</v>
-      </c>
-      <c r="F12" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Marie Vettrino</v>
-      </c>
-      <c r="B13" t="str">
-        <v>15</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Driver</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Miss</v>
-      </c>
-      <c r="E13" t="str">
-        <v>female</v>
-      </c>
-      <c r="F13" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">AB10 7BQ  </v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update the capacity dashboard spreadsheet with new data
Replaced the existing capacity_dashboard.xlsx file with an updated version.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J58"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,7 +442,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B2" t="str">
         <v>30</v>
@@ -454,7 +454,7 @@
         <v>2025-11-03</v>
       </c>
       <c r="E2" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Holiday</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -466,15 +466,15 @@
         <v>0</v>
       </c>
       <c r="I2" t="str">
-        <v>Ola going on paternity leave (MU 21/10/2025) [availability ignored due to day-level leave]</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J2" t="str">
-        <v xml:space="preserve">AB11 8DQ  </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B3" t="str">
         <v>30</v>
@@ -501,12 +501,12 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J3" t="str">
-        <v xml:space="preserve">AB11 8DQ  </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B4" t="str">
         <v>30</v>
@@ -533,12 +533,12 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J4" t="str">
-        <v xml:space="preserve">AB11 8DQ  </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B5" t="str">
         <v>30</v>
@@ -565,12 +565,12 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J5" t="str">
-        <v xml:space="preserve">AB11 8DQ  </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B6" t="str">
         <v>30</v>
@@ -597,12 +597,12 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J6" t="str">
-        <v xml:space="preserve">AB11 8DQ  </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B7" t="str">
         <v>30</v>
@@ -629,12 +629,12 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J7" t="str">
-        <v xml:space="preserve">AB11 8DQ  </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B8" t="str">
         <v>30</v>
@@ -661,18 +661,18 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J8" t="str">
-        <v xml:space="preserve">AB11 8DQ  </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Kirstie Quirke (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="B9" t="str">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C9" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D9" t="str">
         <v>2025-11-03</v>
@@ -681,510 +681,510 @@
         <v>Available</v>
       </c>
       <c r="F9" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="G9" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H9" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I9" t="str">
         <v/>
       </c>
       <c r="J9" t="str">
-        <v xml:space="preserve">AB11 8LH  </v>
+        <v xml:space="preserve">EH34 5HE  </v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Kirstie Quirke (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="B10" t="str">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C10" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-04</v>
       </c>
       <c r="E10" t="str">
         <v>Available</v>
       </c>
       <c r="F10" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="G10" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H10" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I10" t="str">
         <v/>
       </c>
       <c r="J10" t="str">
-        <v xml:space="preserve">AB11 8LH  </v>
+        <v xml:space="preserve">EH34 5HE  </v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Kirstie Quirke (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="B11" t="str">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C11" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-05</v>
       </c>
       <c r="E11" t="str">
         <v>Available</v>
       </c>
       <c r="F11" t="str">
-        <v>09:00-14:30</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="G11" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H11" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I11" t="str">
         <v/>
       </c>
       <c r="J11" t="str">
-        <v xml:space="preserve">AB11 8LH  </v>
+        <v xml:space="preserve">EH34 5HE  </v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Kirstie Quirke (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="B12" t="str">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C12" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D12" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-06</v>
       </c>
       <c r="E12" t="str">
         <v>Available</v>
       </c>
       <c r="F12" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="G12" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H12" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I12" t="str">
         <v/>
       </c>
       <c r="J12" t="str">
-        <v xml:space="preserve">AB11 8LH  </v>
+        <v xml:space="preserve">EH34 5HE  </v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Anish Kumar (GH)</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="B13" t="str">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C13" t="str">
-        <v>5.33</v>
+        <v>3</v>
       </c>
       <c r="D13" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-04</v>
       </c>
       <c r="E13" t="str">
         <v>Available</v>
       </c>
       <c r="F13" t="str">
-        <v>08:00-21:30</v>
+        <v>09:30-10:30; 18:30-21:00</v>
       </c>
       <c r="G13" t="str">
-        <v>5.33</v>
+        <v>3</v>
       </c>
       <c r="H13" t="str">
-        <v>5.33</v>
+        <v>3</v>
       </c>
       <c r="I13" t="str">
         <v/>
       </c>
       <c r="J13" t="str">
-        <v xml:space="preserve">AB25 1GN  </v>
+        <v xml:space="preserve">EH32 0DG  </v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Anish Kumar (GH)</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="B14" t="str">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C14" t="str">
-        <v>5.33</v>
+        <v>3</v>
       </c>
       <c r="D14" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-05</v>
       </c>
       <c r="E14" t="str">
         <v>Available</v>
       </c>
       <c r="F14" t="str">
-        <v>08:00-21:30</v>
+        <v>18:30-21:00</v>
       </c>
       <c r="G14" t="str">
-        <v>5.33</v>
+        <v>3</v>
       </c>
       <c r="H14" t="str">
-        <v>5.33</v>
+        <v>3</v>
       </c>
       <c r="I14" t="str">
         <v/>
       </c>
       <c r="J14" t="str">
-        <v xml:space="preserve">AB25 1GN  </v>
+        <v xml:space="preserve">EH32 0DG  </v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Anish Kumar (GH)</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="B15" t="str">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C15" t="str">
-        <v>5.33</v>
+        <v>3</v>
       </c>
       <c r="D15" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-06</v>
       </c>
       <c r="E15" t="str">
         <v>Available</v>
       </c>
       <c r="F15" t="str">
-        <v>08:00-21:30</v>
+        <v>09:30-10:30; 18:30-21:00</v>
       </c>
       <c r="G15" t="str">
-        <v>5.33</v>
+        <v>3</v>
       </c>
       <c r="H15" t="str">
-        <v>5.33</v>
+        <v>3</v>
       </c>
       <c r="I15" t="str">
         <v/>
       </c>
       <c r="J15" t="str">
-        <v xml:space="preserve">AB25 1GN  </v>
+        <v xml:space="preserve">EH32 0DG  </v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Chance Devereaux-Colby (GH)</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="B16" t="str">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C16" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="D16" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-08</v>
       </c>
       <c r="E16" t="str">
         <v>Available</v>
       </c>
       <c r="F16" t="str">
-        <v>07:00-22:00</v>
+        <v>10:30-11:30; 16:45-17:45</v>
       </c>
       <c r="G16" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="H16" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="I16" t="str">
         <v/>
       </c>
       <c r="J16" t="str">
-        <v xml:space="preserve">AB24 2GG  </v>
+        <v xml:space="preserve">EH32 0DG  </v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Chance Devereaux-Colby (GH)</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="B17" t="str">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C17" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="D17" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-09</v>
       </c>
       <c r="E17" t="str">
         <v>Available</v>
       </c>
       <c r="F17" t="str">
-        <v>07:00-22:00</v>
+        <v>10:30-11:30; 16:45-17:45</v>
       </c>
       <c r="G17" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="H17" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="I17" t="str">
         <v/>
       </c>
       <c r="J17" t="str">
-        <v xml:space="preserve">AB24 2GG  </v>
+        <v xml:space="preserve">EH32 0DG  </v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Chance Devereaux-Colby (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B18" t="str">
         <v>16</v>
       </c>
       <c r="C18" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="D18" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-03</v>
       </c>
       <c r="E18" t="str">
         <v>Available</v>
       </c>
       <c r="F18" t="str">
-        <v>07:00-22:00</v>
+        <v>09:30-15:00</v>
       </c>
       <c r="G18" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="H18" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="I18" t="str">
         <v/>
       </c>
       <c r="J18" t="str">
-        <v xml:space="preserve">AB24 2GG  </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Chance Devereaux-Colby (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B19" t="str">
         <v>16</v>
       </c>
       <c r="C19" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="D19" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-04</v>
       </c>
       <c r="E19" t="str">
         <v>Available</v>
       </c>
       <c r="F19" t="str">
-        <v>07:00-22:00</v>
+        <v>09:30-15:00</v>
       </c>
       <c r="G19" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="H19" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="I19" t="str">
         <v/>
       </c>
       <c r="J19" t="str">
-        <v xml:space="preserve">AB24 2GG  </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Chance Devereaux-Colby (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B20" t="str">
         <v>16</v>
       </c>
       <c r="C20" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="D20" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-05</v>
       </c>
       <c r="E20" t="str">
         <v>Available</v>
       </c>
       <c r="F20" t="str">
-        <v>07:00-22:00</v>
+        <v>09:30-15:00</v>
       </c>
       <c r="G20" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="H20" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="I20" t="str">
         <v/>
       </c>
       <c r="J20" t="str">
-        <v xml:space="preserve">AB24 2GG  </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Sunny Addey (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B21" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C21" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="D21" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-06</v>
       </c>
       <c r="E21" t="str">
         <v>Available</v>
       </c>
       <c r="F21" t="str">
-        <v>08:00-21:30</v>
+        <v>09:30-15:00</v>
       </c>
       <c r="G21" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="H21" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="I21" t="str">
         <v/>
       </c>
       <c r="J21" t="str">
-        <v xml:space="preserve">AB24 1UW  </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Sunny Addey (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B22" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C22" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="D22" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-07</v>
       </c>
       <c r="E22" t="str">
         <v>Available</v>
       </c>
       <c r="F22" t="str">
-        <v>08:00-21:30</v>
+        <v>09:30-15:00</v>
       </c>
       <c r="G22" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="H22" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="I22" t="str">
         <v/>
       </c>
       <c r="J22" t="str">
-        <v xml:space="preserve">AB24 1UW  </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Sunny Addey (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B23" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C23" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="D23" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-08</v>
       </c>
       <c r="E23" t="str">
         <v>Available</v>
       </c>
       <c r="F23" t="str">
-        <v>08:00-21:30</v>
+        <v>09:30-15:00</v>
       </c>
       <c r="G23" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="H23" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="I23" t="str">
         <v/>
       </c>
       <c r="J23" t="str">
-        <v xml:space="preserve">AB24 1UW  </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Sunny Addey (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B24" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C24" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="D24" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-09</v>
       </c>
       <c r="E24" t="str">
         <v>Available</v>
       </c>
       <c r="F24" t="str">
-        <v>08:00-21:30</v>
+        <v>09:30-15:00</v>
       </c>
       <c r="G24" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="H24" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="I24" t="str">
         <v/>
       </c>
       <c r="J24" t="str">
-        <v xml:space="preserve">AB24 1UW  </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Tobiloba Akinlosotu (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="B25" t="str">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="C25" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="D25" t="str">
         <v>2025-11-03</v>
@@ -1193,30 +1193,30 @@
         <v>Available</v>
       </c>
       <c r="F25" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G25" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="H25" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="I25" t="str">
         <v/>
       </c>
       <c r="J25" t="str">
-        <v xml:space="preserve">AB25 2RF  </v>
+        <v xml:space="preserve">EH32 9SS  </v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Tobiloba Akinlosotu (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="B26" t="str">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="C26" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="D26" t="str">
         <v>2025-11-04</v>
@@ -1225,129 +1225,129 @@
         <v>Available</v>
       </c>
       <c r="F26" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G26" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="H26" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="I26" t="str">
         <v/>
       </c>
       <c r="J26" t="str">
-        <v xml:space="preserve">AB25 2RF  </v>
+        <v xml:space="preserve">EH32 9SS  </v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Tobiloba Akinlosotu (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="B27" t="str">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="C27" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="D27" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-05</v>
       </c>
       <c r="E27" t="str">
         <v>Available</v>
       </c>
       <c r="F27" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G27" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="H27" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="I27" t="str">
         <v/>
       </c>
       <c r="J27" t="str">
-        <v xml:space="preserve">AB25 2RF  </v>
+        <v xml:space="preserve">EH32 9SS  </v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Tobiloba Akinlosotu (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="B28" t="str">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="C28" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="D28" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-06</v>
       </c>
       <c r="E28" t="str">
         <v>Available</v>
       </c>
       <c r="F28" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G28" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="H28" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="I28" t="str">
         <v/>
       </c>
       <c r="J28" t="str">
-        <v xml:space="preserve">AB25 2RF  </v>
+        <v xml:space="preserve">EH32 9SS  </v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Deborah Bright (W) (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="B29" t="str">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="C29" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="D29" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-07</v>
       </c>
       <c r="E29" t="str">
         <v>Available</v>
       </c>
       <c r="F29" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G29" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="H29" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="I29" t="str">
         <v/>
       </c>
       <c r="J29" t="str">
-        <v xml:space="preserve">AB24 3EX  </v>
+        <v xml:space="preserve">EH32 9SS  </v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Deborah Bright (W) (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B30" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C30" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="D30" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-03</v>
       </c>
       <c r="E30" t="str">
         <v>Available</v>
@@ -1356,30 +1356,30 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G30" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H30" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="I30" t="str">
         <v/>
       </c>
       <c r="J30" t="str">
-        <v xml:space="preserve">AB24 3EX  </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Deborah Bright (W) (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B31" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C31" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="D31" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-04</v>
       </c>
       <c r="E31" t="str">
         <v>Available</v>
@@ -1388,30 +1388,30 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G31" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H31" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="I31" t="str">
         <v/>
       </c>
       <c r="J31" t="str">
-        <v xml:space="preserve">AB24 3EX  </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Deborah Bright (W) (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B32" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C32" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="D32" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-05</v>
       </c>
       <c r="E32" t="str">
         <v>Available</v>
@@ -1420,30 +1420,30 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G32" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H32" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="I32" t="str">
         <v/>
       </c>
       <c r="J32" t="str">
-        <v xml:space="preserve">AB24 3EX  </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B33" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C33" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="D33" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-06</v>
       </c>
       <c r="E33" t="str">
         <v>Available</v>
@@ -1452,30 +1452,30 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G33" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H33" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="I33" t="str">
         <v/>
       </c>
       <c r="J33" t="str">
-        <v xml:space="preserve">AB10 7BQ  </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B34" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C34" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="D34" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-07</v>
       </c>
       <c r="E34" t="str">
         <v>Available</v>
@@ -1484,30 +1484,30 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G34" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H34" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="I34" t="str">
         <v/>
       </c>
       <c r="J34" t="str">
-        <v xml:space="preserve">AB10 7BQ  </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B35" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C35" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="D35" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-08</v>
       </c>
       <c r="E35" t="str">
         <v>Available</v>
@@ -1516,30 +1516,30 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G35" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H35" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="I35" t="str">
         <v/>
       </c>
       <c r="J35" t="str">
-        <v xml:space="preserve">AB10 7BQ  </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B36" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C36" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="D36" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-09</v>
       </c>
       <c r="E36" t="str">
         <v>Available</v>
@@ -1548,309 +1548,725 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G36" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H36" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="I36" t="str">
         <v/>
       </c>
       <c r="J36" t="str">
-        <v xml:space="preserve">AB10 7BQ  </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Jacqueline Clark</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B37" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C37" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="D37" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-03</v>
       </c>
       <c r="E37" t="str">
         <v>Available</v>
       </c>
       <c r="F37" t="str">
-        <v>08:00-21:30</v>
+        <v>12:00-21:00</v>
       </c>
       <c r="G37" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="H37" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="I37" t="str">
         <v/>
       </c>
       <c r="J37" t="str">
-        <v xml:space="preserve">AB11 8BP  </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Jacqueline Clark</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B38" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C38" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="D38" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-04</v>
       </c>
       <c r="E38" t="str">
         <v>Available</v>
       </c>
       <c r="F38" t="str">
-        <v>08:00-21:30</v>
+        <v>12:00-21:00</v>
       </c>
       <c r="G38" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="H38" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="I38" t="str">
         <v/>
       </c>
       <c r="J38" t="str">
-        <v xml:space="preserve">AB11 8BP  </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Jacqueline Clark</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B39" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C39" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="D39" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-05</v>
       </c>
       <c r="E39" t="str">
         <v>Available</v>
       </c>
       <c r="F39" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-21:00</v>
       </c>
       <c r="G39" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="H39" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="I39" t="str">
         <v/>
       </c>
       <c r="J39" t="str">
-        <v xml:space="preserve">AB11 8BP  </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Jacqueline Clark</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B40" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C40" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="D40" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-06</v>
       </c>
       <c r="E40" t="str">
         <v>Available</v>
       </c>
       <c r="F40" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-21:00</v>
       </c>
       <c r="G40" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="H40" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="I40" t="str">
         <v/>
       </c>
       <c r="J40" t="str">
-        <v xml:space="preserve">AB11 8BP  </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Sharon Jane Riley (W) (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B41" t="str">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C41" t="str">
-        <v>6</v>
+        <v>1.67</v>
       </c>
       <c r="D41" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-07</v>
       </c>
       <c r="E41" t="str">
         <v>Available</v>
       </c>
       <c r="F41" t="str">
-        <v>07:00-22:10</v>
+        <v>12:00-17:45</v>
       </c>
       <c r="G41" t="str">
-        <v>6</v>
+        <v>1.67</v>
       </c>
       <c r="H41" t="str">
-        <v>6</v>
+        <v>1.67</v>
       </c>
       <c r="I41" t="str">
         <v/>
       </c>
       <c r="J41" t="str">
-        <v xml:space="preserve">AB12 3WF  </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Sharon Jane Riley (W) (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B42" t="str">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C42" t="str">
-        <v>6</v>
+        <v>1.67</v>
       </c>
       <c r="D42" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-09</v>
       </c>
       <c r="E42" t="str">
         <v>Available</v>
       </c>
       <c r="F42" t="str">
-        <v>07:00-22:10</v>
+        <v>21:00-22:00</v>
       </c>
       <c r="G42" t="str">
-        <v>6</v>
+        <v>1.67</v>
       </c>
       <c r="H42" t="str">
-        <v>6</v>
+        <v>1.67</v>
       </c>
       <c r="I42" t="str">
         <v/>
       </c>
       <c r="J42" t="str">
-        <v xml:space="preserve">AB12 3WF  </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Sharon Jane Riley (W) (GH)</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="B43" t="str">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C43" t="str">
-        <v>6</v>
+        <v>2.5</v>
       </c>
       <c r="D43" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-03</v>
       </c>
       <c r="E43" t="str">
         <v>Available</v>
       </c>
       <c r="F43" t="str">
-        <v>07:00-22:10</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="G43" t="str">
-        <v>6</v>
+        <v>2.5</v>
       </c>
       <c r="H43" t="str">
-        <v>6</v>
+        <v>2.5</v>
       </c>
       <c r="I43" t="str">
         <v/>
       </c>
       <c r="J43" t="str">
-        <v xml:space="preserve">AB12 3WF  </v>
+        <v xml:space="preserve">EH21 6NQ  </v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Sharon Jane Riley (W) (GH)</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="B44" t="str">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C44" t="str">
-        <v>6</v>
+        <v>2.5</v>
       </c>
       <c r="D44" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-04</v>
       </c>
       <c r="E44" t="str">
         <v>Available</v>
       </c>
       <c r="F44" t="str">
-        <v>07:00-22:10</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="G44" t="str">
-        <v>6</v>
+        <v>2.5</v>
       </c>
       <c r="H44" t="str">
-        <v>6</v>
+        <v>2.5</v>
       </c>
       <c r="I44" t="str">
         <v/>
       </c>
       <c r="J44" t="str">
-        <v xml:space="preserve">AB12 3WF  </v>
+        <v xml:space="preserve">EH21 6NQ  </v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Sharon Jane Riley (W) (GH)</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="B45" t="str">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C45" t="str">
-        <v>6</v>
+        <v>2.5</v>
       </c>
       <c r="D45" t="str">
+        <v>2025-11-05</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F45" t="str">
+        <v>08:00-18:00</v>
+      </c>
+      <c r="G45" t="str">
+        <v>2.5</v>
+      </c>
+      <c r="H45" t="str">
+        <v>2.5</v>
+      </c>
+      <c r="I45" t="str">
+        <v/>
+      </c>
+      <c r="J45" t="str">
+        <v xml:space="preserve">EH21 6NQ  </v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Elizabeth Adams</v>
+      </c>
+      <c r="B46" t="str">
+        <v>10</v>
+      </c>
+      <c r="C46" t="str">
+        <v>2.5</v>
+      </c>
+      <c r="D46" t="str">
+        <v>2025-11-06</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F46" t="str">
+        <v>08:00-18:00</v>
+      </c>
+      <c r="G46" t="str">
+        <v>2.5</v>
+      </c>
+      <c r="H46" t="str">
+        <v>2.5</v>
+      </c>
+      <c r="I46" t="str">
+        <v/>
+      </c>
+      <c r="J46" t="str">
+        <v xml:space="preserve">EH21 6NQ  </v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Helen Morrison (GH)</v>
+      </c>
+      <c r="B47" t="str">
+        <v>15</v>
+      </c>
+      <c r="C47" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="D47" t="str">
+        <v>2025-11-03</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F47" t="str">
+        <v>08:00-16:30</v>
+      </c>
+      <c r="G47" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="H47" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47" t="str">
+        <v xml:space="preserve">EH21 6JY  </v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Helen Morrison (GH)</v>
+      </c>
+      <c r="B48" t="str">
+        <v>15</v>
+      </c>
+      <c r="C48" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="D48" t="str">
+        <v>2025-11-04</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F48" t="str">
+        <v>08:00-16:00</v>
+      </c>
+      <c r="G48" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="H48" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="I48" t="str">
+        <v/>
+      </c>
+      <c r="J48" t="str">
+        <v xml:space="preserve">EH21 6JY  </v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Helen Morrison (GH)</v>
+      </c>
+      <c r="B49" t="str">
+        <v>15</v>
+      </c>
+      <c r="C49" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="D49" t="str">
+        <v>2025-11-08</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F49" t="str">
+        <v>08:00-16:30</v>
+      </c>
+      <c r="G49" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="H49" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49" t="str">
+        <v xml:space="preserve">EH21 6JY  </v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Helen Morrison (GH)</v>
+      </c>
+      <c r="B50" t="str">
+        <v>15</v>
+      </c>
+      <c r="C50" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="D50" t="str">
         <v>2025-11-09</v>
       </c>
-      <c r="E45" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F45" t="str">
-        <v>07:00-22:10</v>
-      </c>
-      <c r="G45" t="str">
-        <v>6</v>
-      </c>
-      <c r="H45" t="str">
-        <v>6</v>
-      </c>
-      <c r="I45" t="str">
-        <v/>
-      </c>
-      <c r="J45" t="str">
-        <v xml:space="preserve">AB12 3WF  </v>
+      <c r="E50" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F50" t="str">
+        <v>08:00-16:00</v>
+      </c>
+      <c r="G50" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="H50" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
+        <v xml:space="preserve">EH21 6JY  </v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Lorraine Parsons</v>
+      </c>
+      <c r="B51" t="str">
+        <v>10</v>
+      </c>
+      <c r="C51" t="str">
+        <v>3.33</v>
+      </c>
+      <c r="D51" t="str">
+        <v>2025-11-04</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F51" t="str">
+        <v>09:30-14:30</v>
+      </c>
+      <c r="G51" t="str">
+        <v>3.33</v>
+      </c>
+      <c r="H51" t="str">
+        <v>3.33</v>
+      </c>
+      <c r="I51" t="str">
+        <v/>
+      </c>
+      <c r="J51" t="str">
+        <v xml:space="preserve">EH22 4FP  </v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Lorraine Parsons</v>
+      </c>
+      <c r="B52" t="str">
+        <v>10</v>
+      </c>
+      <c r="C52" t="str">
+        <v>3.33</v>
+      </c>
+      <c r="D52" t="str">
+        <v>2025-11-05</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F52" t="str">
+        <v>09:30-14:30</v>
+      </c>
+      <c r="G52" t="str">
+        <v>3.33</v>
+      </c>
+      <c r="H52" t="str">
+        <v>3.33</v>
+      </c>
+      <c r="I52" t="str">
+        <v/>
+      </c>
+      <c r="J52" t="str">
+        <v xml:space="preserve">EH22 4FP  </v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Lorraine Parsons</v>
+      </c>
+      <c r="B53" t="str">
+        <v>10</v>
+      </c>
+      <c r="C53" t="str">
+        <v>3.33</v>
+      </c>
+      <c r="D53" t="str">
+        <v>2025-11-07</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F53" t="str">
+        <v>09:30-16:00</v>
+      </c>
+      <c r="G53" t="str">
+        <v>3.33</v>
+      </c>
+      <c r="H53" t="str">
+        <v>3.33</v>
+      </c>
+      <c r="I53" t="str">
+        <v/>
+      </c>
+      <c r="J53" t="str">
+        <v xml:space="preserve">EH22 4FP  </v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Victoria Bateman (GH)</v>
+      </c>
+      <c r="B54" t="str">
+        <v>16</v>
+      </c>
+      <c r="C54" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="D54" t="str">
+        <v>2025-11-03</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F54" t="str">
+        <v>08:00-15:30</v>
+      </c>
+      <c r="G54" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H54" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="I54" t="str">
+        <v/>
+      </c>
+      <c r="J54" t="str">
+        <v xml:space="preserve">EH23 4NL  </v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Victoria Bateman (GH)</v>
+      </c>
+      <c r="B55" t="str">
+        <v>16</v>
+      </c>
+      <c r="C55" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="D55" t="str">
+        <v>2025-11-04</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F55" t="str">
+        <v>08:00-15:30</v>
+      </c>
+      <c r="G55" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H55" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55" t="str">
+        <v xml:space="preserve">EH23 4NL  </v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Victoria Bateman (GH)</v>
+      </c>
+      <c r="B56" t="str">
+        <v>16</v>
+      </c>
+      <c r="C56" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="D56" t="str">
+        <v>2025-11-05</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F56" t="str">
+        <v>08:00-15:30</v>
+      </c>
+      <c r="G56" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H56" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="I56" t="str">
+        <v/>
+      </c>
+      <c r="J56" t="str">
+        <v xml:space="preserve">EH23 4NL  </v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Victoria Bateman (GH)</v>
+      </c>
+      <c r="B57" t="str">
+        <v>16</v>
+      </c>
+      <c r="C57" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="D57" t="str">
+        <v>2025-11-06</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F57" t="str">
+        <v>08:00-17:30</v>
+      </c>
+      <c r="G57" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H57" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="I57" t="str">
+        <v/>
+      </c>
+      <c r="J57" t="str">
+        <v xml:space="preserve">EH23 4NL  </v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Victoria Bateman (GH)</v>
+      </c>
+      <c r="B58" t="str">
+        <v>16</v>
+      </c>
+      <c r="C58" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="D58" t="str">
+        <v>2025-11-07</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F58" t="str">
+        <v>08:00-15:30</v>
+      </c>
+      <c r="G58" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H58" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="I58" t="str">
+        <v/>
+      </c>
+      <c r="J58" t="str">
+        <v xml:space="preserve">EH23 4NL  </v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J58"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1890,22 +2306,22 @@
         <v>2025-11-03</v>
       </c>
       <c r="B2" t="str">
-        <v>25</v>
+        <v>20.27</v>
       </c>
       <c r="C2" t="str">
-        <v>25</v>
+        <v>20.27</v>
       </c>
       <c r="D2" t="str">
+        <v>0</v>
+      </c>
+      <c r="E2" t="str">
         <v>4.29</v>
       </c>
-      <c r="E2" t="str">
-        <v>0</v>
-      </c>
       <c r="F2" t="str">
-        <v>38.5</v>
+        <v>34</v>
       </c>
       <c r="G2" t="str">
-        <v>-13.5</v>
+        <v>-13.73</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -1916,10 +2332,10 @@
         <v>2025-11-04</v>
       </c>
       <c r="B3" t="str">
-        <v>43.2</v>
+        <v>26.6</v>
       </c>
       <c r="C3" t="str">
-        <v>43.2</v>
+        <v>26.6</v>
       </c>
       <c r="D3" t="str">
         <v>0</v>
@@ -1928,13 +2344,13 @@
         <v>4.29</v>
       </c>
       <c r="F3" t="str">
-        <v>38.25</v>
+        <v>34</v>
       </c>
       <c r="G3" t="str">
-        <v>4.95</v>
+        <v>-7.4</v>
       </c>
       <c r="H3" t="str">
-        <v>Sufficient</v>
+        <v>Shortage</v>
       </c>
     </row>
     <row r="4">
@@ -1942,10 +2358,10 @@
         <v>2025-11-05</v>
       </c>
       <c r="B4" t="str">
-        <v>28.2</v>
+        <v>22.85</v>
       </c>
       <c r="C4" t="str">
-        <v>28.2</v>
+        <v>22.85</v>
       </c>
       <c r="D4" t="str">
         <v>0</v>
@@ -1954,10 +2370,10 @@
         <v>4.29</v>
       </c>
       <c r="F4" t="str">
-        <v>38.5</v>
+        <v>48.5</v>
       </c>
       <c r="G4" t="str">
-        <v>-10.3</v>
+        <v>-25.65</v>
       </c>
       <c r="H4" t="str">
         <v>Shortage</v>
@@ -1968,10 +2384,10 @@
         <v>2025-11-06</v>
       </c>
       <c r="B5" t="str">
-        <v>26.2</v>
+        <v>19.52</v>
       </c>
       <c r="C5" t="str">
-        <v>26.2</v>
+        <v>19.52</v>
       </c>
       <c r="D5" t="str">
         <v>0</v>
@@ -1980,10 +2396,10 @@
         <v>4.29</v>
       </c>
       <c r="F5" t="str">
-        <v>36.5</v>
+        <v>34</v>
       </c>
       <c r="G5" t="str">
-        <v>-10.3</v>
+        <v>-14.48</v>
       </c>
       <c r="H5" t="str">
         <v>Shortage</v>
@@ -1994,10 +2410,10 @@
         <v>2025-11-07</v>
       </c>
       <c r="B6" t="str">
-        <v>28.33</v>
+        <v>14.35</v>
       </c>
       <c r="C6" t="str">
-        <v>28.33</v>
+        <v>14.35</v>
       </c>
       <c r="D6" t="str">
         <v>0</v>
@@ -2006,10 +2422,10 @@
         <v>4.29</v>
       </c>
       <c r="F6" t="str">
-        <v>31.5</v>
+        <v>24.25</v>
       </c>
       <c r="G6" t="str">
-        <v>-3.17</v>
+        <v>-9.9</v>
       </c>
       <c r="H6" t="str">
         <v>Shortage</v>
@@ -2020,10 +2436,10 @@
         <v>2025-11-08</v>
       </c>
       <c r="B7" t="str">
-        <v>29.53</v>
+        <v>11.9</v>
       </c>
       <c r="C7" t="str">
-        <v>29.53</v>
+        <v>11.9</v>
       </c>
       <c r="D7" t="str">
         <v>0</v>
@@ -2032,10 +2448,10 @@
         <v>4.29</v>
       </c>
       <c r="F7" t="str">
-        <v>33.5</v>
+        <v>18.5</v>
       </c>
       <c r="G7" t="str">
-        <v>-3.97</v>
+        <v>-6.6</v>
       </c>
       <c r="H7" t="str">
         <v>Shortage</v>
@@ -2046,10 +2462,10 @@
         <v>2025-11-09</v>
       </c>
       <c r="B8" t="str">
-        <v>33.53</v>
+        <v>13.57</v>
       </c>
       <c r="C8" t="str">
-        <v>33.53</v>
+        <v>13.57</v>
       </c>
       <c r="D8" t="str">
         <v>0</v>
@@ -2058,10 +2474,10 @@
         <v>4.29</v>
       </c>
       <c r="F8" t="str">
-        <v>36</v>
+        <v>14.5</v>
       </c>
       <c r="G8" t="str">
-        <v>-2.47</v>
+        <v>-0.93</v>
       </c>
       <c r="H8" t="str">
         <v>Shortage</v>
@@ -2076,7 +2492,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H64"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2109,25 +2525,25 @@
         <v>2025-11-03</v>
       </c>
       <c r="B2" t="str">
-        <v>Addey (GH), Sunny</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="C2" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D2" t="str">
-        <v>10:32-12:31</v>
+        <v>12:00-21:00</v>
       </c>
       <c r="E2" t="str">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="F2" t="str">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="G2" t="str">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="H2" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -2135,7 +2551,7 @@
         <v>2025-11-03</v>
       </c>
       <c r="B3" t="str">
-        <v>Deborah Bright (W) (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="C3" t="str">
         <v>Available</v>
@@ -2144,13 +2560,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E3" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="F3" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="G3" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -2161,22 +2577,22 @@
         <v>2025-11-03</v>
       </c>
       <c r="B4" t="str">
-        <v>Kirstie Quirke (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="C4" t="str">
         <v>Available</v>
       </c>
       <c r="D4" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="E4" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G4" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H4" t="str">
         <v/>
@@ -2187,25 +2603,25 @@
         <v>2025-11-03</v>
       </c>
       <c r="B5" t="str">
-        <v>Kumar (GH), Anish</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="C5" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D5" t="str">
-        <v>14:01-16:02</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E5" t="str">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="F5" t="str">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="G5" t="str">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="H5" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -2213,13 +2629,13 @@
         <v>2025-11-03</v>
       </c>
       <c r="B6" t="str">
-        <v>Mackie (GH), Natalie</v>
+        <v>Hartley-Oliver (GH), Ruby</v>
       </c>
       <c r="C6" t="str">
         <v>Ad-hoc</v>
       </c>
       <c r="D6" t="str">
-        <v>09:29-10:30; 11:30-13:30; 16:05-17:05</v>
+        <v>10:00-12:00</v>
       </c>
       <c r="E6" t="str">
         <v>0</v>
@@ -2239,25 +2655,25 @@
         <v>2025-11-03</v>
       </c>
       <c r="B7" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="C7" t="str">
-        <v>Maternity/Paternity</v>
+        <v>Available</v>
       </c>
       <c r="D7" t="str">
-        <v/>
+        <v>08:00-16:30</v>
       </c>
       <c r="E7" t="str">
-        <v>4.29</v>
+        <v>3.75</v>
       </c>
       <c r="F7" t="str">
-        <v>4.29</v>
+        <v>3.75</v>
       </c>
       <c r="G7" t="str">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="H7" t="str">
-        <v>Ola going on paternity leave (MU 21/10/2025) [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -2265,22 +2681,22 @@
         <v>2025-11-03</v>
       </c>
       <c r="B8" t="str">
-        <v>Sharon Jane Riley (W) (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="C8" t="str">
         <v>Available</v>
       </c>
       <c r="D8" t="str">
-        <v>07:00-22:10</v>
+        <v>09:30-15:00</v>
       </c>
       <c r="E8" t="str">
-        <v>6</v>
+        <v>2.29</v>
       </c>
       <c r="F8" t="str">
-        <v>6</v>
+        <v>2.29</v>
       </c>
       <c r="G8" t="str">
-        <v>6</v>
+        <v>2.29</v>
       </c>
       <c r="H8" t="str">
         <v/>
@@ -2291,48 +2707,48 @@
         <v>2025-11-03</v>
       </c>
       <c r="B9" t="str">
-        <v>Tobiloba Akinlosotu (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="C9" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D9" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E9" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="F9" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="G9" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H9" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-03</v>
       </c>
       <c r="B10" t="str">
-        <v>Chance Devereaux-Colby (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="C10" t="str">
         <v>Available</v>
       </c>
       <c r="D10" t="str">
-        <v>07:00-22:00</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E10" t="str">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="str">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="G10" t="str">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="H10" t="str">
         <v/>
@@ -2340,25 +2756,25 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-03</v>
       </c>
       <c r="B11" t="str">
-        <v>Deborah Bright (W) (GH)</v>
+        <v>Victoria Bateman (GH)</v>
       </c>
       <c r="C11" t="str">
         <v>Available</v>
       </c>
       <c r="D11" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E11" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="F11" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="G11" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -2369,22 +2785,22 @@
         <v>2025-11-04</v>
       </c>
       <c r="B12" t="str">
-        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="C12" t="str">
         <v>Available</v>
       </c>
       <c r="D12" t="str">
-        <v>08:00-21:30</v>
+        <v>12:00-21:00</v>
       </c>
       <c r="E12" t="str">
-        <v>7.5</v>
+        <v>1.67</v>
       </c>
       <c r="F12" t="str">
-        <v>7.5</v>
+        <v>1.67</v>
       </c>
       <c r="G12" t="str">
-        <v>7.5</v>
+        <v>1.67</v>
       </c>
       <c r="H12" t="str">
         <v/>
@@ -2395,7 +2811,7 @@
         <v>2025-11-04</v>
       </c>
       <c r="B13" t="str">
-        <v>Jacqueline Clark</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="C13" t="str">
         <v>Available</v>
@@ -2404,13 +2820,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E13" t="str">
-        <v>4</v>
+        <v>2.86</v>
       </c>
       <c r="F13" t="str">
-        <v>4</v>
+        <v>2.86</v>
       </c>
       <c r="G13" t="str">
-        <v>4</v>
+        <v>2.86</v>
       </c>
       <c r="H13" t="str">
         <v/>
@@ -2421,25 +2837,25 @@
         <v>2025-11-04</v>
       </c>
       <c r="B14" t="str">
-        <v>Mackie (GH), Natalie</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="C14" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D14" t="str">
-        <v>09:26-10:25; 12:53-13:52; 16:00-16:59</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="E14" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F14" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G14" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H14" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -2447,25 +2863,25 @@
         <v>2025-11-04</v>
       </c>
       <c r="B15" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="C15" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D15" t="str">
-        <v/>
+        <v>08:00-18:00</v>
       </c>
       <c r="E15" t="str">
-        <v>4.29</v>
+        <v>2.5</v>
       </c>
       <c r="F15" t="str">
-        <v>4.29</v>
+        <v>2.5</v>
       </c>
       <c r="G15" t="str">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="H15" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -2473,25 +2889,25 @@
         <v>2025-11-04</v>
       </c>
       <c r="B16" t="str">
-        <v>Sharon Jane Riley (W) (GH)</v>
+        <v>Hartley-Oliver (GH), Ruby</v>
       </c>
       <c r="C16" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D16" t="str">
-        <v>07:00-22:10</v>
+        <v>13:59-16:59</v>
       </c>
       <c r="E16" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F16" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G16" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H16" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="17">
@@ -2499,22 +2915,22 @@
         <v>2025-11-04</v>
       </c>
       <c r="B17" t="str">
-        <v>Sunny Addey (GH)</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="C17" t="str">
         <v>Available</v>
       </c>
       <c r="D17" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-16:00</v>
       </c>
       <c r="E17" t="str">
-        <v>7.5</v>
+        <v>3.75</v>
       </c>
       <c r="F17" t="str">
-        <v>7.5</v>
+        <v>3.75</v>
       </c>
       <c r="G17" t="str">
-        <v>7.5</v>
+        <v>3.75</v>
       </c>
       <c r="H17" t="str">
         <v/>
@@ -2525,22 +2941,22 @@
         <v>2025-11-04</v>
       </c>
       <c r="B18" t="str">
-        <v>Tobiloba Akinlosotu (GH)</v>
+        <v>Lorraine Parsons</v>
       </c>
       <c r="C18" t="str">
         <v>Available</v>
       </c>
       <c r="D18" t="str">
-        <v>08:00-21:30</v>
+        <v>09:30-14:30</v>
       </c>
       <c r="E18" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="F18" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="G18" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="H18" t="str">
         <v/>
@@ -2548,51 +2964,51 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-04</v>
       </c>
       <c r="B19" t="str">
-        <v>Bright (W) (GH), Deborah</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="C19" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D19" t="str">
-        <v>09:29-11:30</v>
+        <v>09:30-10:30; 18:30-21:00</v>
       </c>
       <c r="E19" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F19" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G19" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H19" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-04</v>
       </c>
       <c r="B20" t="str">
-        <v>Chance Devereaux-Colby (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="C20" t="str">
         <v>Available</v>
       </c>
       <c r="D20" t="str">
-        <v>07:00-22:00</v>
+        <v>09:30-15:00</v>
       </c>
       <c r="E20" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="F20" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="G20" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -2600,51 +3016,51 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-04</v>
       </c>
       <c r="B21" t="str">
-        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="C21" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D21" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E21" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="F21" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="G21" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H21" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-04</v>
       </c>
       <c r="B22" t="str">
-        <v>Jacqueline Clark</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="C22" t="str">
         <v>Available</v>
       </c>
       <c r="D22" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E22" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F22" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G22" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H22" t="str">
         <v/>
@@ -2652,28 +3068,28 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-04</v>
       </c>
       <c r="B23" t="str">
-        <v>Mackie (GH), Natalie</v>
+        <v>Victoria Bateman (GH)</v>
       </c>
       <c r="C23" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D23" t="str">
-        <v>07:59-09:00; 09:29-10:30; 10:59-12:00; 12:29-13:30; 16:00-16:59</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E23" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="F23" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="G23" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H23" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -2681,25 +3097,25 @@
         <v>2025-11-05</v>
       </c>
       <c r="B24" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="C24" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D24" t="str">
-        <v/>
+        <v>09:15-21:00</v>
       </c>
       <c r="E24" t="str">
-        <v>4.29</v>
+        <v>1.67</v>
       </c>
       <c r="F24" t="str">
-        <v>4.29</v>
+        <v>1.67</v>
       </c>
       <c r="G24" t="str">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="H24" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -2707,22 +3123,22 @@
         <v>2025-11-05</v>
       </c>
       <c r="B25" t="str">
-        <v>Sharon Jane Riley (W) (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="C25" t="str">
         <v>Available</v>
       </c>
       <c r="D25" t="str">
-        <v>07:00-22:10</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E25" t="str">
-        <v>6</v>
+        <v>2.86</v>
       </c>
       <c r="F25" t="str">
-        <v>6</v>
+        <v>2.86</v>
       </c>
       <c r="G25" t="str">
-        <v>6</v>
+        <v>2.86</v>
       </c>
       <c r="H25" t="str">
         <v/>
@@ -2733,22 +3149,22 @@
         <v>2025-11-05</v>
       </c>
       <c r="B26" t="str">
-        <v>Sunny Addey (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="C26" t="str">
         <v>Available</v>
       </c>
       <c r="D26" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="E26" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="F26" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="G26" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="H26" t="str">
         <v/>
@@ -2756,25 +3172,25 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-05</v>
       </c>
       <c r="B27" t="str">
-        <v>Chance Devereaux-Colby (GH)</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="C27" t="str">
         <v>Available</v>
       </c>
       <c r="D27" t="str">
-        <v>07:00-22:00</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E27" t="str">
-        <v>3.2</v>
+        <v>2.5</v>
       </c>
       <c r="F27" t="str">
-        <v>3.2</v>
+        <v>2.5</v>
       </c>
       <c r="G27" t="str">
-        <v>3.2</v>
+        <v>2.5</v>
       </c>
       <c r="H27" t="str">
         <v/>
@@ -2782,25 +3198,25 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-05</v>
       </c>
       <c r="B28" t="str">
-        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
+        <v>Lorraine Parsons</v>
       </c>
       <c r="C28" t="str">
         <v>Available</v>
       </c>
       <c r="D28" t="str">
-        <v>08:00-21:30</v>
+        <v>09:30-14:30</v>
       </c>
       <c r="E28" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="F28" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="G28" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -2808,25 +3224,25 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-05</v>
       </c>
       <c r="B29" t="str">
-        <v>Jacqueline Clark</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="C29" t="str">
         <v>Available</v>
       </c>
       <c r="D29" t="str">
-        <v>08:00-21:30</v>
+        <v>18:30-21:00</v>
       </c>
       <c r="E29" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F29" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G29" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -2834,25 +3250,25 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-05</v>
       </c>
       <c r="B30" t="str">
-        <v>Kirstie Quirke (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="C30" t="str">
         <v>Available</v>
       </c>
       <c r="D30" t="str">
-        <v>08:00-21:30</v>
+        <v>09:30-15:00</v>
       </c>
       <c r="E30" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="F30" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="G30" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="H30" t="str">
         <v/>
@@ -2860,16 +3276,16 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-05</v>
       </c>
       <c r="B31" t="str">
-        <v>Mackie (GH), Natalie</v>
+        <v>Morrison (GH), Helen</v>
       </c>
       <c r="C31" t="str">
         <v>Ad-hoc</v>
       </c>
       <c r="D31" t="str">
-        <v>09:29-10:30; 11:30-13:30</v>
+        <v>07:59-09:00; 09:15-10:14</v>
       </c>
       <c r="E31" t="str">
         <v>0</v>
@@ -2886,10 +3302,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-05</v>
       </c>
       <c r="B32" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="C32" t="str">
         <v>Holiday</v>
@@ -2912,51 +3328,51 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-05</v>
       </c>
       <c r="B33" t="str">
-        <v>Riley (W) (GH), Sharon Jane</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="C33" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D33" t="str">
-        <v>07:59-09:00; 11:44-12:45</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E33" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H33" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-05</v>
       </c>
       <c r="B34" t="str">
-        <v>Sunny Addey (GH)</v>
+        <v>Victoria Bateman (GH)</v>
       </c>
       <c r="C34" t="str">
         <v>Available</v>
       </c>
       <c r="D34" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E34" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="F34" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="G34" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="H34" t="str">
         <v/>
@@ -2964,25 +3380,25 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B35" t="str">
-        <v>Anish Kumar (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="C35" t="str">
         <v>Available</v>
       </c>
       <c r="D35" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-21:00</v>
       </c>
       <c r="E35" t="str">
-        <v>5.33</v>
+        <v>1.67</v>
       </c>
       <c r="F35" t="str">
-        <v>5.33</v>
+        <v>1.67</v>
       </c>
       <c r="G35" t="str">
-        <v>5.33</v>
+        <v>1.67</v>
       </c>
       <c r="H35" t="str">
         <v/>
@@ -2990,10 +3406,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B36" t="str">
-        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="C36" t="str">
         <v>Available</v>
@@ -3002,13 +3418,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E36" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="F36" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="G36" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H36" t="str">
         <v/>
@@ -3016,25 +3432,25 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B37" t="str">
-        <v>Jacqueline Clark</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="C37" t="str">
         <v>Available</v>
       </c>
       <c r="D37" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="E37" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F37" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G37" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H37" t="str">
         <v/>
@@ -3042,25 +3458,25 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B38" t="str">
-        <v>Kirstie Quirke (GH)</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="C38" t="str">
         <v>Available</v>
       </c>
       <c r="D38" t="str">
-        <v>09:00-14:30</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E38" t="str">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="F38" t="str">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="G38" t="str">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="H38" t="str">
         <v/>
@@ -3068,16 +3484,16 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B39" t="str">
-        <v>Mackie (GH), Natalie</v>
+        <v>Hartley-Oliver (GH), Ruby</v>
       </c>
       <c r="C39" t="str">
         <v>Ad-hoc</v>
       </c>
       <c r="D39" t="str">
-        <v>09:29-10:30; 13:00-13:59; 14:15-15:00; 16:00-16:59</v>
+        <v>13:59-16:59</v>
       </c>
       <c r="E39" t="str">
         <v>0</v>
@@ -3094,103 +3510,103 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B40" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="C40" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D40" t="str">
-        <v/>
+        <v>09:30-10:30; 18:30-21:00</v>
       </c>
       <c r="E40" t="str">
-        <v>4.29</v>
+        <v>3</v>
       </c>
       <c r="F40" t="str">
-        <v>4.29</v>
+        <v>3</v>
       </c>
       <c r="G40" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H40" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B41" t="str">
-        <v>Riley (W) (GH), Sharon Jane</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="C41" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D41" t="str">
-        <v>07:59-09:00</v>
+        <v>09:30-15:00</v>
       </c>
       <c r="E41" t="str">
-        <v>0</v>
+        <v>2.29</v>
       </c>
       <c r="F41" t="str">
-        <v>0</v>
+        <v>2.29</v>
       </c>
       <c r="G41" t="str">
-        <v>0</v>
+        <v>2.29</v>
       </c>
       <c r="H41" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B42" t="str">
-        <v>Sunny Addey (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="C42" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D42" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E42" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="F42" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="G42" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H42" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B43" t="str">
-        <v>Anish Kumar (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="C43" t="str">
         <v>Available</v>
       </c>
       <c r="D43" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E43" t="str">
-        <v>5.33</v>
+        <v>1</v>
       </c>
       <c r="F43" t="str">
-        <v>5.33</v>
+        <v>1</v>
       </c>
       <c r="G43" t="str">
-        <v>5.33</v>
+        <v>1</v>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -3198,16 +3614,16 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-06</v>
       </c>
       <c r="B44" t="str">
-        <v>Chance Devereaux-Colby (GH)</v>
+        <v>Victoria Bateman (GH)</v>
       </c>
       <c r="C44" t="str">
         <v>Available</v>
       </c>
       <c r="D44" t="str">
-        <v>07:00-22:00</v>
+        <v>08:00-17:30</v>
       </c>
       <c r="E44" t="str">
         <v>3.2</v>
@@ -3224,36 +3640,36 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B45" t="str">
-        <v>Clark, Jacqueline</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="C45" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D45" t="str">
-        <v>07:59-09:00; 09:29-10:30; 11:35-12:35; 16:00-16:59; 18:00-19:00</v>
+        <v>12:00-17:45</v>
       </c>
       <c r="E45" t="str">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="F45" t="str">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="G45" t="str">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="H45" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B46" t="str">
-        <v>Deborah Bright (W) (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="C46" t="str">
         <v>Available</v>
@@ -3262,13 +3678,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E46" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="F46" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="G46" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H46" t="str">
         <v/>
@@ -3276,103 +3692,103 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B47" t="str">
-        <v>Lazar (GH), Nina</v>
+        <v>Lorraine Parsons</v>
       </c>
       <c r="C47" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D47" t="str">
-        <v>07:59-09:00; 10:00-10:59; 14:15-15:00; 16:30-17:30; 18:00-19:00</v>
+        <v>09:30-16:00</v>
       </c>
       <c r="E47" t="str">
-        <v>0</v>
+        <v>3.33</v>
       </c>
       <c r="F47" t="str">
-        <v>0</v>
+        <v>3.33</v>
       </c>
       <c r="G47" t="str">
-        <v>0</v>
+        <v>3.33</v>
       </c>
       <c r="H47" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B48" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="C48" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D48" t="str">
-        <v/>
+        <v>09:30-15:00</v>
       </c>
       <c r="E48" t="str">
-        <v>4.29</v>
+        <v>2.29</v>
       </c>
       <c r="F48" t="str">
-        <v>4.29</v>
+        <v>2.29</v>
       </c>
       <c r="G48" t="str">
-        <v>0</v>
+        <v>2.29</v>
       </c>
       <c r="H48" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B49" t="str">
-        <v>Sharon Jane Riley (W) (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="C49" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D49" t="str">
-        <v>07:00-22:10</v>
+        <v/>
       </c>
       <c r="E49" t="str">
-        <v>6</v>
+        <v>4.29</v>
       </c>
       <c r="F49" t="str">
-        <v>6</v>
+        <v>4.29</v>
       </c>
       <c r="G49" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H49" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B50" t="str">
-        <v>Tobiloba Akinlosotu (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="C50" t="str">
         <v>Available</v>
       </c>
       <c r="D50" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E50" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="F50" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="G50" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -3380,42 +3796,42 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B51" t="str">
-        <v>Anish Kumar (GH)</v>
+        <v>Vettrino, Marie</v>
       </c>
       <c r="C51" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D51" t="str">
-        <v>08:00-21:30</v>
+        <v>19:00-21:29</v>
       </c>
       <c r="E51" t="str">
-        <v>5.33</v>
+        <v>0</v>
       </c>
       <c r="F51" t="str">
-        <v>5.33</v>
+        <v>0</v>
       </c>
       <c r="G51" t="str">
-        <v>5.33</v>
+        <v>0</v>
       </c>
       <c r="H51" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-07</v>
       </c>
       <c r="B52" t="str">
-        <v>Chance Devereaux-Colby (GH)</v>
+        <v>Victoria Bateman (GH)</v>
       </c>
       <c r="C52" t="str">
         <v>Available</v>
       </c>
       <c r="D52" t="str">
-        <v>07:00-22:00</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E52" t="str">
         <v>3.2</v>
@@ -3432,10 +3848,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-08</v>
       </c>
       <c r="B53" t="str">
-        <v>Deborah Bright (W) (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="C53" t="str">
         <v>Available</v>
@@ -3444,13 +3860,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E53" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="F53" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="G53" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H53" t="str">
         <v/>
@@ -3458,103 +3874,103 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-08</v>
       </c>
       <c r="B54" t="str">
-        <v>Kirstie Quirke (GH)</v>
+        <v>Hartley-Oliver (GH), Ruby</v>
       </c>
       <c r="C54" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D54" t="str">
-        <v>08:00-21:30</v>
+        <v>12:29-15:29</v>
       </c>
       <c r="E54" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F54" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G54" t="str">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H54" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-08</v>
       </c>
       <c r="B55" t="str">
-        <v>Lazar (GH), Nina</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="C55" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D55" t="str">
-        <v>07:59-09:00; 10:00-10:59; 14:15-15:00; 16:30-17:30; 18:00-19:00</v>
+        <v>08:00-16:30</v>
       </c>
       <c r="E55" t="str">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="F55" t="str">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="G55" t="str">
-        <v>0</v>
+        <v>3.75</v>
       </c>
       <c r="H55" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-08</v>
       </c>
       <c r="B56" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="C56" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D56" t="str">
-        <v/>
+        <v>10:30-11:30; 16:45-17:45</v>
       </c>
       <c r="E56" t="str">
-        <v>4.29</v>
+        <v>3</v>
       </c>
       <c r="F56" t="str">
-        <v>4.29</v>
+        <v>3</v>
       </c>
       <c r="G56" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H56" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-08</v>
       </c>
       <c r="B57" t="str">
-        <v>Sharon Jane Riley (W) (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="C57" t="str">
         <v>Available</v>
       </c>
       <c r="D57" t="str">
-        <v>07:00-22:10</v>
+        <v>09:30-15:00</v>
       </c>
       <c r="E57" t="str">
-        <v>6</v>
+        <v>2.29</v>
       </c>
       <c r="F57" t="str">
-        <v>6</v>
+        <v>2.29</v>
       </c>
       <c r="G57" t="str">
-        <v>6</v>
+        <v>2.29</v>
       </c>
       <c r="H57" t="str">
         <v/>
@@ -3562,40 +3978,196 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
+        <v>2025-11-08</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Muhammad Irtaza Tahir (GH)</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Holiday</v>
+      </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
+      <c r="E58" t="str">
+        <v>4.29</v>
+      </c>
+      <c r="F58" t="str">
+        <v>4.29</v>
+      </c>
+      <c r="G58" t="str">
+        <v>0</v>
+      </c>
+      <c r="H58" t="str">
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
         <v>2025-11-09</v>
       </c>
-      <c r="B58" t="str">
-        <v>Tobiloba Akinlosotu (GH)</v>
-      </c>
-      <c r="C58" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D58" t="str">
+      <c r="B59" t="str">
+        <v>Anne Morrison</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D59" t="str">
+        <v>21:00-22:00</v>
+      </c>
+      <c r="E59" t="str">
+        <v>1.67</v>
+      </c>
+      <c r="F59" t="str">
+        <v>1.67</v>
+      </c>
+      <c r="G59" t="str">
+        <v>1.67</v>
+      </c>
+      <c r="H59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>2025-11-09</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Dhaval Mithaiwala</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D60" t="str">
         <v>08:00-21:30</v>
       </c>
-      <c r="E58" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="F58" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="G58" t="str">
-        <v>7.5</v>
-      </c>
-      <c r="H58" t="str">
-        <v/>
+      <c r="E60" t="str">
+        <v>2.86</v>
+      </c>
+      <c r="F60" t="str">
+        <v>2.86</v>
+      </c>
+      <c r="G60" t="str">
+        <v>2.86</v>
+      </c>
+      <c r="H60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>2025-11-09</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Helen Morrison (GH)</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D61" t="str">
+        <v>08:00-16:00</v>
+      </c>
+      <c r="E61" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="F61" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="G61" t="str">
+        <v>3.75</v>
+      </c>
+      <c r="H61" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>2025-11-09</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Marie Vettrino</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D62" t="str">
+        <v>10:30-11:30; 16:45-17:45</v>
+      </c>
+      <c r="E62" t="str">
+        <v>3</v>
+      </c>
+      <c r="F62" t="str">
+        <v>3</v>
+      </c>
+      <c r="G62" t="str">
+        <v>3</v>
+      </c>
+      <c r="H62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2025-11-09</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Mikhaila (W) Calder</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D63" t="str">
+        <v>09:30-15:00</v>
+      </c>
+      <c r="E63" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="F63" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="G63" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="H63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>2025-11-09</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Muhammad Irtaza Tahir (GH)</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Holiday</v>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+      <c r="E64" t="str">
+        <v>4.29</v>
+      </c>
+      <c r="F64" t="str">
+        <v>4.29</v>
+      </c>
+      <c r="G64" t="str">
+        <v>0</v>
+      </c>
+      <c r="H64" t="str">
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H64"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3619,130 +4191,130 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Sunny Addey (GH)</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="B2" t="str">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C2" t="str">
         <v>Driver</v>
       </c>
       <c r="D2" t="str">
-        <v>Mr</v>
+        <v>Mrs</v>
       </c>
       <c r="E2" t="str">
-        <v>male</v>
+        <v>female</v>
       </c>
       <c r="F2" t="str">
-        <v xml:space="preserve">AB24 1UW  </v>
+        <v xml:space="preserve">EH21 6NQ  </v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Tobiloba Akinlosotu (GH)</v>
+        <v>Victoria Bateman (GH)</v>
       </c>
       <c r="B3" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C3" t="str">
         <v>Driver</v>
       </c>
       <c r="D3" t="str">
-        <v>Mr</v>
+        <v>Mrs</v>
       </c>
       <c r="E3" t="str">
-        <v>male</v>
+        <v>female</v>
       </c>
       <c r="F3" t="str">
-        <v xml:space="preserve">AB25 2RF  </v>
+        <v xml:space="preserve">EH23 4NL  </v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Deborah Bright (W) (GH)</v>
+        <v>Amy Brown</v>
       </c>
       <c r="B4" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C4" t="str">
-        <v>Walker</v>
+        <v>Driver</v>
       </c>
       <c r="D4" t="str">
-        <v>Mrs</v>
+        <v>Miss</v>
       </c>
       <c r="E4" t="str">
         <v>female</v>
       </c>
       <c r="F4" t="str">
-        <v xml:space="preserve">AB24 3EX  </v>
+        <v xml:space="preserve">EH21 6DQ  </v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Jacqueline Clark</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B5" t="str">
         <v>16</v>
       </c>
       <c r="C5" t="str">
-        <v>Driver</v>
+        <v>Walker</v>
       </c>
       <c r="D5" t="str">
-        <v>Mrs</v>
+        <v>Miss</v>
       </c>
       <c r="E5" t="str">
         <v>female</v>
       </c>
       <c r="F5" t="str">
-        <v xml:space="preserve">AB11 8BP  </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Chance Devereaux-Colby (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="B6" t="str">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C6" t="str">
         <v>Driver</v>
       </c>
       <c r="D6" t="str">
-        <v>Mr</v>
+        <v>Miss</v>
       </c>
       <c r="E6" t="str">
-        <v>male</v>
+        <v>female</v>
       </c>
       <c r="F6" t="str">
-        <v xml:space="preserve">AB24 2GG  </v>
+        <v xml:space="preserve">EH32 9SS  </v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Olakunle Folarin (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="B7" t="str">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="C7" t="str">
         <v>Driver</v>
       </c>
       <c r="D7" t="str">
-        <v>Mr</v>
+        <v>Miss</v>
       </c>
       <c r="E7" t="str">
-        <v>male</v>
+        <v>female</v>
       </c>
       <c r="F7" t="str">
-        <v xml:space="preserve">AB11 8DQ  </v>
+        <v xml:space="preserve">EH34 5HE  </v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Anish Kumar (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B8" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C8" t="str">
         <v>Driver</v>
@@ -3754,38 +4326,38 @@
         <v>male</v>
       </c>
       <c r="F8" t="str">
-        <v xml:space="preserve">AB25 1GN  </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Kirstie Quirke (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B9" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C9" t="str">
         <v>Driver</v>
       </c>
       <c r="D9" t="str">
-        <v>Miss</v>
+        <v>Mrs</v>
       </c>
       <c r="E9" t="str">
         <v>female</v>
       </c>
       <c r="F9" t="str">
-        <v xml:space="preserve">AB11 8LH  </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Sharon Jane Riley (W) (GH)</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="B10" t="str">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C10" t="str">
-        <v>Walker</v>
+        <v>Driver</v>
       </c>
       <c r="D10" t="str">
         <v>Mrs</v>
@@ -3794,15 +4366,15 @@
         <v>female</v>
       </c>
       <c r="F10" t="str">
-        <v xml:space="preserve">AB12 3WF  </v>
+        <v xml:space="preserve">EH21 6JY  </v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Ifeoma Gabriella Uzoigwe (GH)</v>
+        <v>Lorraine Parsons</v>
       </c>
       <c r="B11" t="str">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C11" t="str">
         <v>Driver</v>
@@ -3814,12 +4386,52 @@
         <v>female</v>
       </c>
       <c r="F11" t="str">
-        <v xml:space="preserve">AB10 7BQ  </v>
+        <v xml:space="preserve">EH22 4FP  </v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Muhammad Irtaza Tahir (GH)</v>
+      </c>
+      <c r="B12" t="str">
+        <v>30</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Mr</v>
+      </c>
+      <c r="E12" t="str">
+        <v>male</v>
+      </c>
+      <c r="F12" t="str">
+        <v xml:space="preserve">EH8 7AD   </v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Marie Vettrino</v>
+      </c>
+      <c r="B13" t="str">
+        <v>15</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E13" t="str">
+        <v>female</v>
+      </c>
+      <c r="F13" t="str">
+        <v xml:space="preserve">EH32 0DG  </v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update capacity dashboard to include canceled visits in filtering
Modified capacity_dashboard.xlsx to alter the filtering logic, now including canceled visits.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -2190,10 +2190,10 @@
         <v>7.5</v>
       </c>
       <c r="F2" t="str">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="G2" t="str">
-        <v>-18.7</v>
+        <v>-0.7</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -2216,13 +2216,13 @@
         <v>11.5</v>
       </c>
       <c r="F3" t="str">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="G3" t="str">
-        <v>-3.7</v>
+        <v>9.3</v>
       </c>
       <c r="H3" t="str">
-        <v>Shortage</v>
+        <v>Sufficient</v>
       </c>
     </row>
     <row r="4">
@@ -2242,10 +2242,10 @@
         <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>66</v>
+        <v>51.5</v>
       </c>
       <c r="G4" t="str">
-        <v>-25.4</v>
+        <v>-10.9</v>
       </c>
       <c r="H4" t="str">
         <v>Shortage</v>
@@ -2268,13 +2268,13 @@
         <v>4</v>
       </c>
       <c r="F5" t="str">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="G5" t="str">
-        <v>-8.73</v>
+        <v>9.27</v>
       </c>
       <c r="H5" t="str">
-        <v>Shortage</v>
+        <v>Sufficient</v>
       </c>
     </row>
     <row r="6">
@@ -2294,13 +2294,13 @@
         <v>9.2</v>
       </c>
       <c r="F6" t="str">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="G6" t="str">
-        <v>-13.93</v>
+        <v>4.07</v>
       </c>
       <c r="H6" t="str">
-        <v>Shortage</v>
+        <v>Sufficient</v>
       </c>
     </row>
     <row r="7">
@@ -2320,10 +2320,10 @@
         <v>9.2</v>
       </c>
       <c r="F7" t="str">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="G7" t="str">
-        <v>-21.5</v>
+        <v>-3.5</v>
       </c>
       <c r="H7" t="str">
         <v>Shortage</v>
@@ -2346,10 +2346,10 @@
         <v>9.2</v>
       </c>
       <c r="F8" t="str">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="G8" t="str">
-        <v>-18.13</v>
+        <v>-0.13</v>
       </c>
       <c r="H8" t="str">
         <v>Shortage</v>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update dashboard to reflect current scheduling capacity
Updated capacity dashboard spreadsheet.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J54"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,16 +442,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="B2" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C2" t="str">
-        <v>4.29</v>
+        <v>4</v>
       </c>
       <c r="D2" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E2" t="str">
         <v>Holiday</v>
@@ -460,7 +460,7 @@
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>4.29</v>
+        <v>4</v>
       </c>
       <c r="H2" t="str">
         <v>0</v>
@@ -469,21 +469,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J2" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK7 7PN   </v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="B3" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C3" t="str">
-        <v>4.29</v>
+        <v>4</v>
       </c>
       <c r="D3" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E3" t="str">
         <v>Holiday</v>
@@ -492,7 +492,7 @@
         <v/>
       </c>
       <c r="G3" t="str">
-        <v>4.29</v>
+        <v>4</v>
       </c>
       <c r="H3" t="str">
         <v>0</v>
@@ -501,21 +501,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J3" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK7 7PN   </v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="B4" t="str">
         <v>30</v>
       </c>
       <c r="C4" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="D4" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E4" t="str">
         <v>Holiday</v>
@@ -524,7 +524,7 @@
         <v/>
       </c>
       <c r="G4" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="H4" t="str">
         <v>0</v>
@@ -533,21 +533,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J4" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK8 1XY   </v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="B5" t="str">
         <v>30</v>
       </c>
       <c r="C5" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="D5" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E5" t="str">
         <v>Holiday</v>
@@ -556,7 +556,7 @@
         <v/>
       </c>
       <c r="G5" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="H5" t="str">
         <v>0</v>
@@ -565,21 +565,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J5" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK8 1XY   </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="B6" t="str">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="C6" t="str">
-        <v>4.29</v>
+        <v>9.2</v>
       </c>
       <c r="D6" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E6" t="str">
         <v>Holiday</v>
@@ -588,7 +588,7 @@
         <v/>
       </c>
       <c r="G6" t="str">
-        <v>4.29</v>
+        <v>9.2</v>
       </c>
       <c r="H6" t="str">
         <v>0</v>
@@ -597,21 +597,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J6" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK8 1RS   </v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="B7" t="str">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="C7" t="str">
-        <v>4.29</v>
+        <v>9.2</v>
       </c>
       <c r="D7" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E7" t="str">
         <v>Holiday</v>
@@ -620,7 +620,7 @@
         <v/>
       </c>
       <c r="G7" t="str">
-        <v>4.29</v>
+        <v>9.2</v>
       </c>
       <c r="H7" t="str">
         <v>0</v>
@@ -629,21 +629,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J7" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK8 1RS   </v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="B8" t="str">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="C8" t="str">
-        <v>4.29</v>
+        <v>9.2</v>
       </c>
       <c r="D8" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E8" t="str">
         <v>Holiday</v>
@@ -652,7 +652,7 @@
         <v/>
       </c>
       <c r="G8" t="str">
-        <v>4.29</v>
+        <v>9.2</v>
       </c>
       <c r="H8" t="str">
         <v>0</v>
@@ -661,693 +661,693 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J8" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK8 1RS   </v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Eilish McNally</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="B9" t="str">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="C9" t="str">
-        <v>3</v>
+        <v>9.2</v>
       </c>
       <c r="D9" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E9" t="str">
-        <v>Available</v>
+        <v>Partial Availability</v>
       </c>
       <c r="F9" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:00-13:00; 17:00-22:00</v>
       </c>
       <c r="G9" t="str">
-        <v>3</v>
+        <v>5.2</v>
       </c>
       <c r="H9" t="str">
-        <v>3</v>
+        <v>5.2</v>
       </c>
       <c r="I9" t="str">
-        <v/>
+        <v>Haseeb is helping out GN</v>
       </c>
       <c r="J9" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">FK2 7ER   </v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Eilish McNally</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="B10" t="str">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="C10" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="D10" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E10" t="str">
         <v>Available</v>
       </c>
       <c r="F10" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>15:30-21:30</v>
       </c>
       <c r="G10" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H10" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="I10" t="str">
         <v/>
       </c>
       <c r="J10" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">FK6 5AE   </v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Eilish McNally</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="B11" t="str">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="C11" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="D11" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E11" t="str">
         <v>Available</v>
       </c>
       <c r="F11" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G11" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H11" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="I11" t="str">
         <v/>
       </c>
       <c r="J11" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">FK6 5AE   </v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Eilish McNally</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="B12" t="str">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="C12" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="D12" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E12" t="str">
         <v>Available</v>
       </c>
       <c r="F12" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G12" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H12" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="I12" t="str">
         <v/>
       </c>
       <c r="J12" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">FK6 5AE   </v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Marie Vettrino</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="B13" t="str">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="C13" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="D13" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E13" t="str">
         <v>Available</v>
       </c>
       <c r="F13" t="str">
-        <v>09:30-10:30; 18:30-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G13" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H13" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="I13" t="str">
         <v/>
       </c>
       <c r="J13" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">FK6 5AE   </v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Marie Vettrino</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="B14" t="str">
-        <v>15</v>
+        <v>37.5</v>
       </c>
       <c r="C14" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="D14" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E14" t="str">
         <v>Available</v>
       </c>
       <c r="F14" t="str">
-        <v>18:30-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G14" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H14" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="I14" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
       <c r="J14" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">FK8 2BQ   </v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Marie Vettrino</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="B15" t="str">
-        <v>15</v>
+        <v>37.5</v>
       </c>
       <c r="C15" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="D15" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E15" t="str">
         <v>Available</v>
       </c>
       <c r="F15" t="str">
-        <v>09:30-10:30; 18:30-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G15" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H15" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="I15" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
       <c r="J15" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">FK8 2BQ   </v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Marie Vettrino</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="B16" t="str">
-        <v>15</v>
+        <v>37.5</v>
       </c>
       <c r="C16" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="D16" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E16" t="str">
         <v>Available</v>
       </c>
       <c r="F16" t="str">
-        <v>10:30-11:30; 16:45-17:45</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G16" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H16" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="I16" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
       <c r="J16" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">FK8 2BQ   </v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Marie Vettrino</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="B17" t="str">
-        <v>15</v>
+        <v>37.5</v>
       </c>
       <c r="C17" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="D17" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E17" t="str">
         <v>Available</v>
       </c>
       <c r="F17" t="str">
-        <v>10:30-11:30; 16:45-17:45</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G17" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H17" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="I17" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
       <c r="J17" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">FK8 2BQ   </v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="B18" t="str">
-        <v>16</v>
+        <v>37.5</v>
       </c>
       <c r="C18" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="D18" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E18" t="str">
         <v>Available</v>
       </c>
       <c r="F18" t="str">
-        <v>09:30-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G18" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="H18" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="I18" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
       <c r="J18" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK8 2BQ   </v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="B19" t="str">
         <v>16</v>
       </c>
       <c r="C19" t="str">
-        <v>2.29</v>
+        <v>4</v>
       </c>
       <c r="D19" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E19" t="str">
         <v>Available</v>
       </c>
       <c r="F19" t="str">
-        <v>09:30-15:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G19" t="str">
-        <v>2.29</v>
+        <v>4</v>
       </c>
       <c r="H19" t="str">
-        <v>2.29</v>
+        <v>4</v>
       </c>
       <c r="I19" t="str">
         <v/>
       </c>
       <c r="J19" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK7 7PN   </v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="B20" t="str">
         <v>16</v>
       </c>
       <c r="C20" t="str">
-        <v>2.29</v>
+        <v>4</v>
       </c>
       <c r="D20" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E20" t="str">
         <v>Available</v>
       </c>
       <c r="F20" t="str">
-        <v>09:30-15:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G20" t="str">
-        <v>2.29</v>
+        <v>4</v>
       </c>
       <c r="H20" t="str">
-        <v>2.29</v>
+        <v>4</v>
       </c>
       <c r="I20" t="str">
         <v/>
       </c>
       <c r="J20" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK7 7PN   </v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="B21" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C21" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="D21" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E21" t="str">
         <v>Available</v>
       </c>
       <c r="F21" t="str">
-        <v>09:30-15:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G21" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="H21" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="I21" t="str">
         <v/>
       </c>
       <c r="J21" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK10 2SR  </v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="B22" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C22" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="D22" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E22" t="str">
         <v>Available</v>
       </c>
       <c r="F22" t="str">
-        <v>09:30-15:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G22" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="H22" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="I22" t="str">
         <v/>
       </c>
       <c r="J22" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK10 2SR  </v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="B23" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C23" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="D23" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E23" t="str">
         <v>Available</v>
       </c>
       <c r="F23" t="str">
-        <v>09:30-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G23" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="H23" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="I23" t="str">
         <v/>
       </c>
       <c r="J23" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK10 2SR  </v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="B24" t="str">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C24" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="D24" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E24" t="str">
         <v>Available</v>
       </c>
       <c r="F24" t="str">
-        <v>09:30-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G24" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="H24" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="I24" t="str">
         <v/>
       </c>
       <c r="J24" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK10 2SR  </v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Romina Ferrara</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="B25" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C25" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D25" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E25" t="str">
         <v>Available</v>
       </c>
       <c r="F25" t="str">
-        <v>09:15-10:15</v>
+        <v>08:15-21:30</v>
       </c>
       <c r="G25" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H25" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I25" t="str">
         <v/>
       </c>
       <c r="J25" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">FK10 1NH  </v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Romina Ferrara</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="B26" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C26" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D26" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E26" t="str">
         <v>Available</v>
       </c>
       <c r="F26" t="str">
-        <v>09:15-10:15</v>
+        <v>08:15-21:30</v>
       </c>
       <c r="G26" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H26" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I26" t="str">
         <v/>
       </c>
       <c r="J26" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">FK10 1NH  </v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Romina Ferrara</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="B27" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C27" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D27" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E27" t="str">
         <v>Available</v>
       </c>
       <c r="F27" t="str">
-        <v>09:15-10:15</v>
+        <v>08:15-17:15</v>
       </c>
       <c r="G27" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H27" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I27" t="str">
         <v/>
       </c>
       <c r="J27" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">FK10 1NH  </v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Romina Ferrara</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="B28" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C28" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D28" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E28" t="str">
         <v>Available</v>
       </c>
       <c r="F28" t="str">
-        <v>09:15-10:15</v>
+        <v>08:15-17:15</v>
       </c>
       <c r="G28" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H28" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I28" t="str">
         <v/>
       </c>
       <c r="J28" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">FK10 1NH  </v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Romina Ferrara</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="B29" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C29" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D29" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E29" t="str">
         <v>Available</v>
       </c>
       <c r="F29" t="str">
-        <v>09:15-10:15</v>
+        <v>08:15-17:15</v>
       </c>
       <c r="G29" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H29" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I29" t="str">
         <v/>
       </c>
       <c r="J29" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">FK10 1NH  </v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="B30" t="str">
         <v>20</v>
       </c>
       <c r="C30" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="D30" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E30" t="str">
         <v>Available</v>
@@ -1356,62 +1356,62 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G30" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="H30" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="I30" t="str">
         <v/>
       </c>
       <c r="J30" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK5 4XD   </v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="B31" t="str">
         <v>20</v>
       </c>
       <c r="C31" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="D31" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E31" t="str">
         <v>Available</v>
       </c>
       <c r="F31" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-14:00</v>
       </c>
       <c r="G31" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="H31" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="I31" t="str">
         <v/>
       </c>
       <c r="J31" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK5 4XD   </v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="B32" t="str">
         <v>20</v>
       </c>
       <c r="C32" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="D32" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E32" t="str">
         <v>Available</v>
@@ -1420,853 +1420,725 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G32" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="H32" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="I32" t="str">
         <v/>
       </c>
       <c r="J32" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK5 4XD   </v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="B33" t="str">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C33" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="D33" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E33" t="str">
         <v>Available</v>
       </c>
       <c r="F33" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="G33" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="H33" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="I33" t="str">
         <v/>
       </c>
       <c r="J33" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK2 7ER   </v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="B34" t="str">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C34" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="D34" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E34" t="str">
         <v>Available</v>
       </c>
       <c r="F34" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="G34" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="H34" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="I34" t="str">
         <v/>
       </c>
       <c r="J34" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK2 7ER   </v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="B35" t="str">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C35" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="D35" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E35" t="str">
         <v>Available</v>
       </c>
       <c r="F35" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="G35" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="H35" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="I35" t="str">
         <v/>
       </c>
       <c r="J35" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK2 7ER   </v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="B36" t="str">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C36" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="D36" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E36" t="str">
         <v>Available</v>
       </c>
       <c r="F36" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="G36" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="H36" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="I36" t="str">
         <v/>
       </c>
       <c r="J36" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK2 7ER   </v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Anne Morrison</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="B37" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C37" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="D37" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E37" t="str">
         <v>Available</v>
       </c>
       <c r="F37" t="str">
-        <v>12:00-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G37" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="H37" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="I37" t="str">
         <v/>
       </c>
       <c r="J37" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK8 1XY   </v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Anne Morrison</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="B38" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C38" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="D38" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E38" t="str">
         <v>Available</v>
       </c>
       <c r="F38" t="str">
-        <v>12:00-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G38" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="H38" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="I38" t="str">
         <v/>
       </c>
       <c r="J38" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK8 1XY   </v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Anne Morrison</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="B39" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C39" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="D39" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E39" t="str">
         <v>Available</v>
       </c>
       <c r="F39" t="str">
-        <v>09:15-21:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G39" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="H39" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="I39" t="str">
         <v/>
       </c>
       <c r="J39" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK10 3HJ  </v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Anne Morrison</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="B40" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C40" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="D40" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E40" t="str">
         <v>Available</v>
       </c>
       <c r="F40" t="str">
-        <v>09:15-21:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G40" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="H40" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="I40" t="str">
         <v/>
       </c>
       <c r="J40" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK10 3HJ  </v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Anne Morrison</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="B41" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C41" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="D41" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E41" t="str">
         <v>Available</v>
       </c>
       <c r="F41" t="str">
-        <v>12:00-17:45</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G41" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="H41" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="I41" t="str">
         <v/>
       </c>
       <c r="J41" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK10 3HJ  </v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Anne Morrison</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="B42" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C42" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="D42" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E42" t="str">
         <v>Available</v>
       </c>
       <c r="F42" t="str">
-        <v>21:00-22:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G42" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="H42" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="I42" t="str">
         <v/>
       </c>
       <c r="J42" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK10 3HJ  </v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="B43" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C43" t="str">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="D43" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E43" t="str">
         <v>Available</v>
       </c>
       <c r="F43" t="str">
-        <v>08:00-18:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G43" t="str">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="H43" t="str">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="I43" t="str">
         <v/>
       </c>
       <c r="J43" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
+        <v xml:space="preserve">FK10 3HJ  </v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="B44" t="str">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="C44" t="str">
-        <v>2.5</v>
+        <v>9.2</v>
       </c>
       <c r="D44" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E44" t="str">
         <v>Available</v>
       </c>
       <c r="F44" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G44" t="str">
-        <v>2.5</v>
+        <v>9.2</v>
       </c>
       <c r="H44" t="str">
-        <v>2.5</v>
+        <v>9.2</v>
       </c>
       <c r="I44" t="str">
         <v/>
       </c>
       <c r="J44" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
+        <v xml:space="preserve">FK8 1RS   </v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="B45" t="str">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="C45" t="str">
-        <v>2.5</v>
+        <v>9.2</v>
       </c>
       <c r="D45" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E45" t="str">
         <v>Available</v>
       </c>
       <c r="F45" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G45" t="str">
-        <v>2.5</v>
+        <v>9.2</v>
       </c>
       <c r="H45" t="str">
-        <v>2.5</v>
+        <v>9.2</v>
       </c>
       <c r="I45" t="str">
         <v/>
       </c>
       <c r="J45" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
+        <v xml:space="preserve">FK8 1RS   </v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="B46" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C46" t="str">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="D46" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E46" t="str">
         <v>Available</v>
       </c>
       <c r="F46" t="str">
-        <v>08:00-18:00</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="G46" t="str">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="H46" t="str">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="I46" t="str">
         <v/>
       </c>
       <c r="J46" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
+        <v xml:space="preserve">FK12 5HG  </v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="B47" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C47" t="str">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="D47" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E47" t="str">
         <v>Available</v>
       </c>
       <c r="F47" t="str">
-        <v>08:00-16:30</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="G47" t="str">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="H47" t="str">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="I47" t="str">
         <v/>
       </c>
       <c r="J47" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
+        <v xml:space="preserve">FK12 5HG  </v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="B48" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C48" t="str">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="D48" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E48" t="str">
         <v>Available</v>
       </c>
       <c r="F48" t="str">
-        <v>08:00-16:00</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="G48" t="str">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="H48" t="str">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="I48" t="str">
         <v/>
       </c>
       <c r="J48" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
+        <v xml:space="preserve">FK12 5HG  </v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="B49" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C49" t="str">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="D49" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E49" t="str">
         <v>Available</v>
       </c>
       <c r="F49" t="str">
-        <v>08:00-16:30</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="G49" t="str">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="H49" t="str">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="I49" t="str">
         <v/>
       </c>
       <c r="J49" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
+        <v xml:space="preserve">FK12 5HG  </v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="B50" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C50" t="str">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="D50" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E50" t="str">
         <v>Available</v>
       </c>
       <c r="F50" t="str">
-        <v>08:00-16:00</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="G50" t="str">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="H50" t="str">
-        <v>3.75</v>
+        <v>3.2</v>
       </c>
       <c r="I50" t="str">
         <v/>
       </c>
       <c r="J50" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
+        <v xml:space="preserve">FK12 5HG  </v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="B51" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C51" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="D51" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E51" t="str">
         <v>Available</v>
       </c>
       <c r="F51" t="str">
-        <v>09:30-14:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G51" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="H51" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="I51" t="str">
         <v/>
       </c>
       <c r="J51" t="str">
-        <v xml:space="preserve">EH22 4FP  </v>
+        <v xml:space="preserve">FK3 8LP   </v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="B52" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C52" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="D52" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E52" t="str">
         <v>Available</v>
       </c>
       <c r="F52" t="str">
-        <v>09:30-14:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G52" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="H52" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="I52" t="str">
         <v/>
       </c>
       <c r="J52" t="str">
-        <v xml:space="preserve">EH22 4FP  </v>
+        <v xml:space="preserve">FK3 8LP   </v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="B53" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C53" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="D53" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E53" t="str">
         <v>Available</v>
       </c>
       <c r="F53" t="str">
-        <v>09:30-16:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G53" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="H53" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="I53" t="str">
         <v/>
       </c>
       <c r="J53" t="str">
-        <v xml:space="preserve">EH22 4FP  </v>
+        <v xml:space="preserve">FK3 8LP   </v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="B54" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C54" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="D54" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E54" t="str">
         <v>Available</v>
       </c>
       <c r="F54" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G54" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H54" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="I54" t="str">
         <v/>
       </c>
       <c r="J54" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="B55" t="str">
-        <v>16</v>
-      </c>
-      <c r="C55" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D55" t="str">
-        <v>2025-11-04</v>
-      </c>
-      <c r="E55" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F55" t="str">
-        <v>08:00-15:30</v>
-      </c>
-      <c r="G55" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H55" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I55" t="str">
-        <v/>
-      </c>
-      <c r="J55" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="B56" t="str">
-        <v>16</v>
-      </c>
-      <c r="C56" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D56" t="str">
-        <v>2025-11-05</v>
-      </c>
-      <c r="E56" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F56" t="str">
-        <v>08:00-15:30</v>
-      </c>
-      <c r="G56" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H56" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I56" t="str">
-        <v/>
-      </c>
-      <c r="J56" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="B57" t="str">
-        <v>16</v>
-      </c>
-      <c r="C57" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D57" t="str">
-        <v>2025-11-06</v>
-      </c>
-      <c r="E57" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F57" t="str">
-        <v>08:00-17:30</v>
-      </c>
-      <c r="G57" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H57" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I57" t="str">
-        <v/>
-      </c>
-      <c r="J57" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="B58" t="str">
-        <v>16</v>
-      </c>
-      <c r="C58" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D58" t="str">
-        <v>2025-11-07</v>
-      </c>
-      <c r="E58" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F58" t="str">
-        <v>08:00-15:30</v>
-      </c>
-      <c r="G58" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H58" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I58" t="str">
-        <v/>
-      </c>
-      <c r="J58" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
+        <v xml:space="preserve">FK3 8LP   </v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J54"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2303,25 +2175,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B2" t="str">
-        <v>20.27</v>
+        <v>34.1</v>
       </c>
       <c r="C2" t="str">
-        <v>20.27</v>
+        <v>39.3</v>
       </c>
       <c r="D2" t="str">
-        <v>0</v>
+        <v>5.2</v>
       </c>
       <c r="E2" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="F2" t="str">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="G2" t="str">
-        <v>-13.73</v>
+        <v>-18.7</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -2329,25 +2201,25 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B3" t="str">
-        <v>26.6</v>
+        <v>58.3</v>
       </c>
       <c r="C3" t="str">
-        <v>26.6</v>
+        <v>58.3</v>
       </c>
       <c r="D3" t="str">
         <v>0</v>
       </c>
       <c r="E3" t="str">
-        <v>4.29</v>
+        <v>11.5</v>
       </c>
       <c r="F3" t="str">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="G3" t="str">
-        <v>-7.4</v>
+        <v>-3.7</v>
       </c>
       <c r="H3" t="str">
         <v>Shortage</v>
@@ -2355,25 +2227,25 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B4" t="str">
-        <v>22.85</v>
+        <v>40.6</v>
       </c>
       <c r="C4" t="str">
-        <v>22.85</v>
+        <v>40.6</v>
       </c>
       <c r="D4" t="str">
         <v>0</v>
       </c>
       <c r="E4" t="str">
-        <v>4.29</v>
+        <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>48.5</v>
+        <v>66</v>
       </c>
       <c r="G4" t="str">
-        <v>-25.65</v>
+        <v>-25.4</v>
       </c>
       <c r="H4" t="str">
         <v>Shortage</v>
@@ -2381,25 +2253,25 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B5" t="str">
-        <v>19.52</v>
+        <v>43.27</v>
       </c>
       <c r="C5" t="str">
-        <v>19.52</v>
+        <v>43.27</v>
       </c>
       <c r="D5" t="str">
         <v>0</v>
       </c>
       <c r="E5" t="str">
-        <v>4.29</v>
+        <v>4</v>
       </c>
       <c r="F5" t="str">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="G5" t="str">
-        <v>-14.48</v>
+        <v>-8.73</v>
       </c>
       <c r="H5" t="str">
         <v>Shortage</v>
@@ -2407,25 +2279,25 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B6" t="str">
-        <v>14.35</v>
+        <v>44.07</v>
       </c>
       <c r="C6" t="str">
-        <v>14.35</v>
+        <v>44.07</v>
       </c>
       <c r="D6" t="str">
         <v>0</v>
       </c>
       <c r="E6" t="str">
-        <v>4.29</v>
+        <v>9.2</v>
       </c>
       <c r="F6" t="str">
-        <v>24.25</v>
+        <v>58</v>
       </c>
       <c r="G6" t="str">
-        <v>-9.9</v>
+        <v>-13.93</v>
       </c>
       <c r="H6" t="str">
         <v>Shortage</v>
@@ -2433,25 +2305,25 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-15</v>
       </c>
       <c r="B7" t="str">
-        <v>11.9</v>
+        <v>27.5</v>
       </c>
       <c r="C7" t="str">
-        <v>11.9</v>
+        <v>27.5</v>
       </c>
       <c r="D7" t="str">
         <v>0</v>
       </c>
       <c r="E7" t="str">
-        <v>4.29</v>
+        <v>9.2</v>
       </c>
       <c r="F7" t="str">
-        <v>18.5</v>
+        <v>49</v>
       </c>
       <c r="G7" t="str">
-        <v>-6.6</v>
+        <v>-21.5</v>
       </c>
       <c r="H7" t="str">
         <v>Shortage</v>
@@ -2459,25 +2331,25 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2025-11-09</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B8" t="str">
-        <v>13.57</v>
+        <v>29.87</v>
       </c>
       <c r="C8" t="str">
-        <v>13.57</v>
+        <v>29.87</v>
       </c>
       <c r="D8" t="str">
         <v>0</v>
       </c>
       <c r="E8" t="str">
-        <v>4.29</v>
+        <v>9.2</v>
       </c>
       <c r="F8" t="str">
-        <v>14.5</v>
+        <v>48</v>
       </c>
       <c r="G8" t="str">
-        <v>-0.93</v>
+        <v>-18.13</v>
       </c>
       <c r="H8" t="str">
         <v>Shortage</v>
@@ -2492,7 +2364,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H57"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2522,25 +2394,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B2" t="str">
-        <v>Anne Morrison</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="C2" t="str">
         <v>Available</v>
       </c>
       <c r="D2" t="str">
-        <v>12:00-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E2" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="F2" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="G2" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -2548,25 +2420,25 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B3" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="C3" t="str">
         <v>Available</v>
       </c>
       <c r="D3" t="str">
-        <v>08:00-21:30</v>
+        <v>15:30-21:30</v>
       </c>
       <c r="E3" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="F3" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="G3" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -2574,51 +2446,51 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B4" t="str">
-        <v>Eilish McNally</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="C4" t="str">
         <v>Available</v>
       </c>
       <c r="D4" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E4" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="F4" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="G4" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B5" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="C5" t="str">
         <v>Available</v>
       </c>
       <c r="D5" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E5" t="str">
-        <v>2.5</v>
+        <v>9.2</v>
       </c>
       <c r="F5" t="str">
-        <v>2.5</v>
+        <v>9.2</v>
       </c>
       <c r="G5" t="str">
-        <v>2.5</v>
+        <v>9.2</v>
       </c>
       <c r="H5" t="str">
         <v/>
@@ -2626,129 +2498,129 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B6" t="str">
-        <v>Hartley-Oliver (GH), Ruby</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="C6" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D6" t="str">
-        <v>10:00-12:00</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="E6" t="str">
-        <v>0</v>
+        <v>9.2</v>
       </c>
       <c r="F6" t="str">
-        <v>0</v>
+        <v>9.2</v>
       </c>
       <c r="G6" t="str">
-        <v>0</v>
+        <v>9.2</v>
       </c>
       <c r="H6" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B7" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="C7" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D7" t="str">
-        <v>08:00-16:30</v>
+        <v/>
       </c>
       <c r="E7" t="str">
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="F7" t="str">
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="G7" t="str">
-        <v>3.75</v>
+        <v>0</v>
       </c>
       <c r="H7" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B8" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="C8" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D8" t="str">
-        <v>09:30-15:00</v>
+        <v/>
       </c>
       <c r="E8" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="F8" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="G8" t="str">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="H8" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B9" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="C9" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D9" t="str">
-        <v/>
+        <v>10:00-14:30</v>
       </c>
       <c r="E9" t="str">
-        <v>4.29</v>
+        <v>3.2</v>
       </c>
       <c r="F9" t="str">
-        <v>4.29</v>
+        <v>3.2</v>
       </c>
       <c r="G9" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H9" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B10" t="str">
-        <v>Romina Ferrara</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="C10" t="str">
         <v>Available</v>
       </c>
       <c r="D10" t="str">
-        <v>09:15-10:15</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E10" t="str">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="F10" t="str">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="G10" t="str">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="H10" t="str">
         <v/>
@@ -2756,25 +2628,25 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2025-11-03</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B11" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="C11" t="str">
         <v>Available</v>
       </c>
       <c r="D11" t="str">
-        <v>08:00-15:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E11" t="str">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="F11" t="str">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="G11" t="str">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -2782,25 +2654,25 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B12" t="str">
-        <v>Anne Morrison</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="C12" t="str">
         <v>Available</v>
       </c>
       <c r="D12" t="str">
-        <v>12:00-21:00</v>
+        <v>08:15-21:30</v>
       </c>
       <c r="E12" t="str">
-        <v>1.67</v>
+        <v>6</v>
       </c>
       <c r="F12" t="str">
-        <v>1.67</v>
+        <v>6</v>
       </c>
       <c r="G12" t="str">
-        <v>1.67</v>
+        <v>6</v>
       </c>
       <c r="H12" t="str">
         <v/>
@@ -2808,51 +2680,51 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B13" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Vidler, Ziyal</v>
       </c>
       <c r="C13" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D13" t="str">
-        <v>08:00-21:30</v>
+        <v>12:29-13:00</v>
       </c>
       <c r="E13" t="str">
-        <v>2.86</v>
+        <v>0</v>
       </c>
       <c r="F13" t="str">
-        <v>2.86</v>
+        <v>0</v>
       </c>
       <c r="G13" t="str">
-        <v>2.86</v>
+        <v>0</v>
       </c>
       <c r="H13" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B14" t="str">
-        <v>Eilish McNally</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="C14" t="str">
         <v>Available</v>
       </c>
       <c r="D14" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E14" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="F14" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="G14" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H14" t="str">
         <v/>
@@ -2860,103 +2732,103 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B15" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="C15" t="str">
         <v>Available</v>
       </c>
       <c r="D15" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E15" t="str">
-        <v>2.5</v>
+        <v>7.5</v>
       </c>
       <c r="F15" t="str">
-        <v>2.5</v>
+        <v>7.5</v>
       </c>
       <c r="G15" t="str">
-        <v>2.5</v>
+        <v>7.5</v>
       </c>
       <c r="H15" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B16" t="str">
-        <v>Hartley-Oliver (GH), Ruby</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="C16" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D16" t="str">
-        <v>13:59-16:59</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="E16" t="str">
-        <v>0</v>
+        <v>9.2</v>
       </c>
       <c r="F16" t="str">
-        <v>0</v>
+        <v>9.2</v>
       </c>
       <c r="G16" t="str">
-        <v>0</v>
+        <v>9.2</v>
       </c>
       <c r="H16" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B17" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="C17" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D17" t="str">
-        <v>08:00-16:00</v>
+        <v/>
       </c>
       <c r="E17" t="str">
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="F17" t="str">
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="G17" t="str">
-        <v>3.75</v>
+        <v>0</v>
       </c>
       <c r="H17" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B18" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="C18" t="str">
         <v>Available</v>
       </c>
       <c r="D18" t="str">
-        <v>09:30-14:30</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="E18" t="str">
-        <v>3.33</v>
+        <v>3.2</v>
       </c>
       <c r="F18" t="str">
-        <v>3.33</v>
+        <v>3.2</v>
       </c>
       <c r="G18" t="str">
-        <v>3.33</v>
+        <v>3.2</v>
       </c>
       <c r="H18" t="str">
         <v/>
@@ -2964,25 +2836,25 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B19" t="str">
-        <v>Marie Vettrino</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="C19" t="str">
         <v>Available</v>
       </c>
       <c r="D19" t="str">
-        <v>09:30-10:30; 18:30-21:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E19" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="F19" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="G19" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H19" t="str">
         <v/>
@@ -2990,25 +2862,25 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B20" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="C20" t="str">
         <v>Available</v>
       </c>
       <c r="D20" t="str">
-        <v>09:30-15:00</v>
+        <v>08:15-17:15</v>
       </c>
       <c r="E20" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="F20" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="G20" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -3016,51 +2888,51 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B21" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="C21" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D21" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E21" t="str">
-        <v>4.29</v>
+        <v>6.67</v>
       </c>
       <c r="F21" t="str">
-        <v>4.29</v>
+        <v>6.67</v>
       </c>
       <c r="G21" t="str">
-        <v>0</v>
+        <v>6.67</v>
       </c>
       <c r="H21" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B22" t="str">
-        <v>Romina Ferrara</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="C22" t="str">
         <v>Available</v>
       </c>
       <c r="D22" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E22" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="F22" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="G22" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="H22" t="str">
         <v/>
@@ -3068,25 +2940,25 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2025-11-04</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B23" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="C23" t="str">
         <v>Available</v>
       </c>
       <c r="D23" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E23" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="F23" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="G23" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="H23" t="str">
         <v/>
@@ -3094,77 +2966,77 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B24" t="str">
-        <v>Anne Morrison</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="C24" t="str">
-        <v>Available</v>
+        <v>Partial Availability</v>
       </c>
       <c r="D24" t="str">
-        <v>09:15-21:00</v>
+        <v>08:00-13:00; 17:00-22:00</v>
       </c>
       <c r="E24" t="str">
-        <v>1.67</v>
+        <v>9.2</v>
       </c>
       <c r="F24" t="str">
-        <v>1.67</v>
+        <v>5.2</v>
       </c>
       <c r="G24" t="str">
-        <v>1.67</v>
+        <v>5.2</v>
       </c>
       <c r="H24" t="str">
-        <v/>
+        <v>Haseeb is helping out GN</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B25" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="C25" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D25" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E25" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="F25" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="G25" t="str">
-        <v>2.86</v>
+        <v>0</v>
       </c>
       <c r="H25" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B26" t="str">
-        <v>Eilish McNally</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="C26" t="str">
         <v>Available</v>
       </c>
       <c r="D26" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="E26" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="F26" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="G26" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H26" t="str">
         <v/>
@@ -3172,25 +3044,25 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B27" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="C27" t="str">
         <v>Available</v>
       </c>
       <c r="D27" t="str">
-        <v>08:00-18:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E27" t="str">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="F27" t="str">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="G27" t="str">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="H27" t="str">
         <v/>
@@ -3198,25 +3070,25 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B28" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="C28" t="str">
         <v>Available</v>
       </c>
       <c r="D28" t="str">
-        <v>09:30-14:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E28" t="str">
-        <v>3.33</v>
+        <v>5</v>
       </c>
       <c r="F28" t="str">
-        <v>3.33</v>
+        <v>5</v>
       </c>
       <c r="G28" t="str">
-        <v>3.33</v>
+        <v>5</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -3224,25 +3096,25 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B29" t="str">
-        <v>Marie Vettrino</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="C29" t="str">
         <v>Available</v>
       </c>
       <c r="D29" t="str">
-        <v>18:30-21:00</v>
+        <v>08:15-21:30</v>
       </c>
       <c r="E29" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F29" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G29" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -3250,129 +3122,129 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B30" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Stevenson (GH), Keri</v>
       </c>
       <c r="C30" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D30" t="str">
-        <v>09:30-15:00</v>
+        <v>09:15-12:15</v>
       </c>
       <c r="E30" t="str">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="F30" t="str">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="G30" t="str">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="H30" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B31" t="str">
-        <v>Morrison (GH), Helen</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="C31" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D31" t="str">
-        <v>07:59-09:00; 09:15-10:14</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E31" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F31" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="G31" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H31" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B32" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="C32" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D32" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E32" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="F32" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="G32" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H32" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v>Created by new employee process.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B33" t="str">
-        <v>Romina Ferrara</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="C33" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D33" t="str">
-        <v>09:15-10:15</v>
+        <v/>
       </c>
       <c r="E33" t="str">
-        <v>1</v>
+        <v>9.2</v>
       </c>
       <c r="F33" t="str">
-        <v>1</v>
+        <v>9.2</v>
       </c>
       <c r="G33" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H33" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2025-11-05</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B34" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="C34" t="str">
         <v>Available</v>
       </c>
       <c r="D34" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="E34" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="F34" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="G34" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="H34" t="str">
         <v/>
@@ -3380,25 +3252,25 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B35" t="str">
-        <v>Anne Morrison</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="C35" t="str">
         <v>Available</v>
       </c>
       <c r="D35" t="str">
-        <v>09:15-21:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E35" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="F35" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="G35" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="H35" t="str">
         <v/>
@@ -3406,25 +3278,25 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B36" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="C36" t="str">
         <v>Available</v>
       </c>
       <c r="D36" t="str">
-        <v>08:00-21:30</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="E36" t="str">
-        <v>2.86</v>
+        <v>3.2</v>
       </c>
       <c r="F36" t="str">
-        <v>2.86</v>
+        <v>3.2</v>
       </c>
       <c r="G36" t="str">
-        <v>2.86</v>
+        <v>3.2</v>
       </c>
       <c r="H36" t="str">
         <v/>
@@ -3432,25 +3304,25 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B37" t="str">
-        <v>Eilish McNally</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="C37" t="str">
         <v>Available</v>
       </c>
       <c r="D37" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:15-17:15</v>
       </c>
       <c r="E37" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F37" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G37" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H37" t="str">
         <v/>
@@ -3458,25 +3330,25 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B38" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="C38" t="str">
         <v>Available</v>
       </c>
       <c r="D38" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-14:00</v>
       </c>
       <c r="E38" t="str">
-        <v>2.5</v>
+        <v>6.67</v>
       </c>
       <c r="F38" t="str">
-        <v>2.5</v>
+        <v>6.67</v>
       </c>
       <c r="G38" t="str">
-        <v>2.5</v>
+        <v>6.67</v>
       </c>
       <c r="H38" t="str">
         <v/>
@@ -3484,129 +3356,129 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-15</v>
       </c>
       <c r="B39" t="str">
-        <v>Hartley-Oliver (GH), Ruby</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="C39" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D39" t="str">
-        <v>13:59-16:59</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E39" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F39" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="G39" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H39" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-15</v>
       </c>
       <c r="B40" t="str">
-        <v>Marie Vettrino</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="C40" t="str">
         <v>Available</v>
       </c>
       <c r="D40" t="str">
-        <v>09:30-10:30; 18:30-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E40" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="F40" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="G40" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H40" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-15</v>
       </c>
       <c r="B41" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="C41" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D41" t="str">
-        <v>09:30-15:00</v>
+        <v/>
       </c>
       <c r="E41" t="str">
-        <v>2.29</v>
+        <v>9.2</v>
       </c>
       <c r="F41" t="str">
-        <v>2.29</v>
+        <v>9.2</v>
       </c>
       <c r="G41" t="str">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="H41" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-15</v>
       </c>
       <c r="B42" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="C42" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D42" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E42" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="F42" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="G42" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H42" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-15</v>
       </c>
       <c r="B43" t="str">
-        <v>Romina Ferrara</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="C43" t="str">
         <v>Available</v>
       </c>
       <c r="D43" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E43" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F43" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G43" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -3614,25 +3486,25 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2025-11-06</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B44" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="C44" t="str">
         <v>Available</v>
       </c>
       <c r="D44" t="str">
-        <v>08:00-17:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E44" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F44" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G44" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H44" t="str">
         <v/>
@@ -3640,36 +3512,36 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B45" t="str">
-        <v>Anne Morrison</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="C45" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D45" t="str">
-        <v>12:00-17:45</v>
+        <v/>
       </c>
       <c r="E45" t="str">
-        <v>1.67</v>
+        <v>9.2</v>
       </c>
       <c r="F45" t="str">
-        <v>1.67</v>
+        <v>9.2</v>
       </c>
       <c r="G45" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="H45" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B46" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="C46" t="str">
         <v>Available</v>
@@ -3678,13 +3550,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E46" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="F46" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="G46" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H46" t="str">
         <v/>
@@ -3692,25 +3564,25 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B47" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="C47" t="str">
         <v>Available</v>
       </c>
       <c r="D47" t="str">
-        <v>09:30-16:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E47" t="str">
-        <v>3.33</v>
+        <v>3.2</v>
       </c>
       <c r="F47" t="str">
-        <v>3.33</v>
+        <v>3.2</v>
       </c>
       <c r="G47" t="str">
-        <v>3.33</v>
+        <v>3.2</v>
       </c>
       <c r="H47" t="str">
         <v/>
@@ -3718,25 +3590,25 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B48" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="C48" t="str">
         <v>Available</v>
       </c>
       <c r="D48" t="str">
-        <v>09:30-15:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E48" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="F48" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="G48" t="str">
-        <v>2.29</v>
+        <v>5</v>
       </c>
       <c r="H48" t="str">
         <v/>
@@ -3744,51 +3616,51 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B49" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="C49" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D49" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E49" t="str">
-        <v>4.29</v>
+        <v>6.67</v>
       </c>
       <c r="F49" t="str">
-        <v>4.29</v>
+        <v>6.67</v>
       </c>
       <c r="G49" t="str">
-        <v>0</v>
+        <v>6.67</v>
       </c>
       <c r="H49" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B50" t="str">
-        <v>Romina Ferrara</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="C50" t="str">
         <v>Available</v>
       </c>
       <c r="D50" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E50" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="F50" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="G50" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -3796,51 +3668,51 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B51" t="str">
-        <v>Vettrino, Marie</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="C51" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D51" t="str">
-        <v>19:00-21:29</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E51" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F51" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="G51" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H51" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v>Created by new employee process.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2025-11-07</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B52" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="C52" t="str">
         <v>Available</v>
       </c>
       <c r="D52" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="E52" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="F52" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="G52" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="H52" t="str">
         <v/>
@@ -3848,25 +3720,25 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B53" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="C53" t="str">
         <v>Available</v>
       </c>
       <c r="D53" t="str">
-        <v>08:00-21:30</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E53" t="str">
-        <v>2.86</v>
+        <v>4</v>
       </c>
       <c r="F53" t="str">
-        <v>2.86</v>
+        <v>4</v>
       </c>
       <c r="G53" t="str">
-        <v>2.86</v>
+        <v>4</v>
       </c>
       <c r="H53" t="str">
         <v/>
@@ -3874,77 +3746,77 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B54" t="str">
-        <v>Hartley-Oliver (GH), Ruby</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="C54" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D54" t="str">
-        <v>12:29-15:29</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="E54" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="F54" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="G54" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H54" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B55" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Onweluzo (GH), Chiamaka</v>
       </c>
       <c r="C55" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D55" t="str">
-        <v>08:00-16:30</v>
+        <v>07:59-09:00; 09:29-14:30</v>
       </c>
       <c r="E55" t="str">
-        <v>3.75</v>
+        <v>0</v>
       </c>
       <c r="F55" t="str">
-        <v>3.75</v>
+        <v>0</v>
       </c>
       <c r="G55" t="str">
-        <v>3.75</v>
+        <v>0</v>
       </c>
       <c r="H55" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B56" t="str">
-        <v>Marie Vettrino</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="C56" t="str">
         <v>Available</v>
       </c>
       <c r="D56" t="str">
-        <v>10:30-11:30; 16:45-17:45</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E56" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="F56" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="G56" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H56" t="str">
         <v/>
@@ -3952,222 +3824,40 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2025-11-08</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B57" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="C57" t="str">
         <v>Available</v>
       </c>
       <c r="D57" t="str">
-        <v>09:30-15:00</v>
+        <v>08:15-17:15</v>
       </c>
       <c r="E57" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="F57" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="G57" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="H57" t="str">
         <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <v>2025-11-08</v>
-      </c>
-      <c r="B58" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
-      </c>
-      <c r="C58" t="str">
-        <v>Holiday</v>
-      </c>
-      <c r="D58" t="str">
-        <v/>
-      </c>
-      <c r="E58" t="str">
-        <v>4.29</v>
-      </c>
-      <c r="F58" t="str">
-        <v>4.29</v>
-      </c>
-      <c r="G58" t="str">
-        <v>0</v>
-      </c>
-      <c r="H58" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <v>2025-11-09</v>
-      </c>
-      <c r="B59" t="str">
-        <v>Anne Morrison</v>
-      </c>
-      <c r="C59" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D59" t="str">
-        <v>21:00-22:00</v>
-      </c>
-      <c r="E59" t="str">
-        <v>1.67</v>
-      </c>
-      <c r="F59" t="str">
-        <v>1.67</v>
-      </c>
-      <c r="G59" t="str">
-        <v>1.67</v>
-      </c>
-      <c r="H59" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <v>2025-11-09</v>
-      </c>
-      <c r="B60" t="str">
-        <v>Dhaval Mithaiwala</v>
-      </c>
-      <c r="C60" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D60" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E60" t="str">
-        <v>2.86</v>
-      </c>
-      <c r="F60" t="str">
-        <v>2.86</v>
-      </c>
-      <c r="G60" t="str">
-        <v>2.86</v>
-      </c>
-      <c r="H60" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="str">
-        <v>2025-11-09</v>
-      </c>
-      <c r="B61" t="str">
-        <v>Helen Morrison (GH)</v>
-      </c>
-      <c r="C61" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D61" t="str">
-        <v>08:00-16:00</v>
-      </c>
-      <c r="E61" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="F61" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="G61" t="str">
-        <v>3.75</v>
-      </c>
-      <c r="H61" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="str">
-        <v>2025-11-09</v>
-      </c>
-      <c r="B62" t="str">
-        <v>Marie Vettrino</v>
-      </c>
-      <c r="C62" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D62" t="str">
-        <v>10:30-11:30; 16:45-17:45</v>
-      </c>
-      <c r="E62" t="str">
-        <v>3</v>
-      </c>
-      <c r="F62" t="str">
-        <v>3</v>
-      </c>
-      <c r="G62" t="str">
-        <v>3</v>
-      </c>
-      <c r="H62" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="str">
-        <v>2025-11-09</v>
-      </c>
-      <c r="B63" t="str">
-        <v>Mikhaila (W) Calder</v>
-      </c>
-      <c r="C63" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D63" t="str">
-        <v>09:30-15:00</v>
-      </c>
-      <c r="E63" t="str">
-        <v>2.29</v>
-      </c>
-      <c r="F63" t="str">
-        <v>2.29</v>
-      </c>
-      <c r="G63" t="str">
-        <v>2.29</v>
-      </c>
-      <c r="H63" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="str">
-        <v>2025-11-09</v>
-      </c>
-      <c r="B64" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
-      </c>
-      <c r="C64" t="str">
-        <v>Holiday</v>
-      </c>
-      <c r="D64" t="str">
-        <v/>
-      </c>
-      <c r="E64" t="str">
-        <v>4.29</v>
-      </c>
-      <c r="F64" t="str">
-        <v>4.29</v>
-      </c>
-      <c r="G64" t="str">
-        <v>0</v>
-      </c>
-      <c r="H64" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H57"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4191,27 +3881,27 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="B2" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C2" t="str">
         <v>Driver</v>
       </c>
       <c r="D2" t="str">
-        <v>Mrs</v>
+        <v>Miss</v>
       </c>
       <c r="E2" t="str">
         <v>female</v>
       </c>
       <c r="F2" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
+        <v xml:space="preserve">FK10 1NH  </v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="B3" t="str">
         <v>16</v>
@@ -4220,81 +3910,81 @@
         <v>Driver</v>
       </c>
       <c r="D3" t="str">
-        <v>Mrs</v>
+        <v>Mr</v>
       </c>
       <c r="E3" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="F3" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
+        <v xml:space="preserve">FK10 3HJ  </v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Amy Brown</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="B4" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C4" t="str">
         <v>Driver</v>
       </c>
       <c r="D4" t="str">
-        <v>Miss</v>
+        <v>Mr</v>
       </c>
       <c r="E4" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="F4" t="str">
-        <v xml:space="preserve">EH21 6DQ  </v>
+        <v xml:space="preserve">FK8 1XY   </v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="B5" t="str">
         <v>16</v>
       </c>
       <c r="C5" t="str">
-        <v>Walker</v>
+        <v>Driver</v>
       </c>
       <c r="D5" t="str">
-        <v>Miss</v>
+        <v>Mrs</v>
       </c>
       <c r="E5" t="str">
         <v>female</v>
       </c>
       <c r="F5" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK12 5HG  </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Romina Ferrara</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="B6" t="str">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C6" t="str">
         <v>Driver</v>
       </c>
       <c r="D6" t="str">
-        <v>Miss</v>
+        <v>Mr</v>
       </c>
       <c r="E6" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="F6" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">FK2 7ER   </v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Eilish McNally</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="B7" t="str">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C7" t="str">
         <v>Driver</v>
@@ -4306,55 +3996,55 @@
         <v>female</v>
       </c>
       <c r="F7" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">FK7 7PN   </v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Clare Mackie</v>
       </c>
       <c r="B8" t="str">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="C8" t="str">
         <v>Driver</v>
       </c>
       <c r="D8" t="str">
-        <v>Mr</v>
+        <v>Miss</v>
       </c>
       <c r="E8" t="str">
-        <v>male</v>
+        <v>female</v>
       </c>
       <c r="F8" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK2 8FD   </v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Anne Morrison</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="B9" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C9" t="str">
         <v>Driver</v>
       </c>
       <c r="D9" t="str">
-        <v>Mrs</v>
+        <v>Miss</v>
       </c>
       <c r="E9" t="str">
         <v>female</v>
       </c>
       <c r="F9" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK6 5AE   </v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="B10" t="str">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="C10" t="str">
         <v>Driver</v>
@@ -4366,32 +4056,32 @@
         <v>female</v>
       </c>
       <c r="F10" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
+        <v xml:space="preserve">FK8 1RS   </v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Emma (NL) Shawcross</v>
       </c>
       <c r="B11" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C11" t="str">
-        <v>Driver</v>
+        <v>Walker</v>
       </c>
       <c r="D11" t="str">
-        <v>Mrs</v>
+        <v>Miss</v>
       </c>
       <c r="E11" t="str">
         <v>female</v>
       </c>
       <c r="F11" t="str">
-        <v xml:space="preserve">EH22 4FP  </v>
+        <v xml:space="preserve">ML6 0JH   </v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="B12" t="str">
         <v>30</v>
@@ -4400,21 +4090,21 @@
         <v>Driver</v>
       </c>
       <c r="D12" t="str">
-        <v>Mr</v>
+        <v>Ms</v>
       </c>
       <c r="E12" t="str">
-        <v>male</v>
+        <v>female</v>
       </c>
       <c r="F12" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK3 8LP   </v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Marie Vettrino</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="B13" t="str">
-        <v>15</v>
+        <v>37.5</v>
       </c>
       <c r="C13" t="str">
         <v>Driver</v>
@@ -4426,12 +4116,52 @@
         <v>female</v>
       </c>
       <c r="F13" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">FK8 2BQ   </v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Rhian Steel</v>
+      </c>
+      <c r="B14" t="str">
+        <v>20</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E14" t="str">
+        <v>female</v>
+      </c>
+      <c r="F14" t="str">
+        <v xml:space="preserve">FK10 2SR  </v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Ziyal Vidler</v>
+      </c>
+      <c r="B15" t="str">
+        <v>20</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E15" t="str">
+        <v>female</v>
+      </c>
+      <c r="F15" t="str">
+        <v xml:space="preserve">FK5 4XD   </v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Improve scheduling logic and address geocoding issues for increased reliability
Adds debug logging for visit processing, enhances geocoding accuracy for employees and clients, and optimizes data extraction for scheduling, addressing previous performance and reliability concerns.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J58"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,16 +442,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Jamie Lee Kane (GH)</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="B2" t="str">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C2" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E2" t="str">
         <v>Holiday</v>
@@ -460,7 +460,7 @@
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H2" t="str">
         <v>0</v>
@@ -469,21 +469,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J2" t="str">
-        <v xml:space="preserve">FK7 7PN   </v>
+        <v xml:space="preserve">EH32 0DG  </v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Jamie Lee Kane (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B3" t="str">
         <v>16</v>
       </c>
       <c r="C3" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="D3" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E3" t="str">
         <v>Holiday</v>
@@ -492,7 +492,7 @@
         <v/>
       </c>
       <c r="G3" t="str">
-        <v>4</v>
+        <v>2.29</v>
       </c>
       <c r="H3" t="str">
         <v>0</v>
@@ -501,21 +501,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J3" t="str">
-        <v xml:space="preserve">FK7 7PN   </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>John Clarke (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B4" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C4" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="D4" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E4" t="str">
         <v>Holiday</v>
@@ -524,7 +524,7 @@
         <v/>
       </c>
       <c r="G4" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="H4" t="str">
         <v>0</v>
@@ -533,21 +533,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J4" t="str">
-        <v xml:space="preserve">FK8 1XY   </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>John Clarke (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B5" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C5" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="D5" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E5" t="str">
         <v>Holiday</v>
@@ -556,7 +556,7 @@
         <v/>
       </c>
       <c r="G5" t="str">
-        <v>7.5</v>
+        <v>2.29</v>
       </c>
       <c r="H5" t="str">
         <v>0</v>
@@ -565,21 +565,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J5" t="str">
-        <v xml:space="preserve">FK8 1XY   </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Chiamaka Onweluzo (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B6" t="str">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="C6" t="str">
-        <v>9.2</v>
+        <v>2.29</v>
       </c>
       <c r="D6" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E6" t="str">
         <v>Holiday</v>
@@ -588,7 +588,7 @@
         <v/>
       </c>
       <c r="G6" t="str">
-        <v>9.2</v>
+        <v>2.29</v>
       </c>
       <c r="H6" t="str">
         <v>0</v>
@@ -597,21 +597,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J6" t="str">
-        <v xml:space="preserve">FK8 1RS   </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Chiamaka Onweluzo (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B7" t="str">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="C7" t="str">
-        <v>9.2</v>
+        <v>2.29</v>
       </c>
       <c r="D7" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E7" t="str">
         <v>Holiday</v>
@@ -620,7 +620,7 @@
         <v/>
       </c>
       <c r="G7" t="str">
-        <v>9.2</v>
+        <v>2.29</v>
       </c>
       <c r="H7" t="str">
         <v>0</v>
@@ -629,21 +629,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J7" t="str">
-        <v xml:space="preserve">FK8 1RS   </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Chiamaka Onweluzo (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B8" t="str">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="C8" t="str">
-        <v>9.2</v>
+        <v>2.29</v>
       </c>
       <c r="D8" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E8" t="str">
         <v>Holiday</v>
@@ -652,7 +652,7 @@
         <v/>
       </c>
       <c r="G8" t="str">
-        <v>9.2</v>
+        <v>2.29</v>
       </c>
       <c r="H8" t="str">
         <v>0</v>
@@ -661,434 +661,434 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J8" t="str">
-        <v xml:space="preserve">FK8 1RS   </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B9" t="str">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="C9" t="str">
-        <v>9.2</v>
+        <v>2.29</v>
       </c>
       <c r="D9" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E9" t="str">
-        <v>Partial Availability</v>
+        <v>Holiday</v>
       </c>
       <c r="F9" t="str">
-        <v>08:00-13:00; 17:00-22:00</v>
+        <v/>
       </c>
       <c r="G9" t="str">
-        <v>5.2</v>
+        <v>2.29</v>
       </c>
       <c r="H9" t="str">
-        <v>5.2</v>
+        <v>0</v>
       </c>
       <c r="I9" t="str">
-        <v>Haseeb is helping out GN</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J9" t="str">
-        <v xml:space="preserve">FK2 7ER   </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Anisa Naeem</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B10" t="str">
         <v>30</v>
       </c>
       <c r="C10" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="D10" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E10" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="F10" t="str">
-        <v>15:30-21:30</v>
+        <v/>
       </c>
       <c r="G10" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="H10" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I10" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J10" t="str">
-        <v xml:space="preserve">FK6 5AE   </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Anisa Naeem</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B11" t="str">
         <v>30</v>
       </c>
       <c r="C11" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="D11" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E11" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="F11" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G11" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="H11" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I11" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J11" t="str">
-        <v xml:space="preserve">FK6 5AE   </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Anisa Naeem</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B12" t="str">
         <v>30</v>
       </c>
       <c r="C12" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="D12" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E12" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="F12" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G12" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="H12" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J12" t="str">
-        <v xml:space="preserve">FK6 5AE   </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Anisa Naeem</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B13" t="str">
         <v>30</v>
       </c>
       <c r="C13" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="D13" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E13" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="F13" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G13" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="H13" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I13" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J13" t="str">
-        <v xml:space="preserve">FK6 5AE   </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Barbora Slabochova (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B14" t="str">
-        <v>37.5</v>
+        <v>30</v>
       </c>
       <c r="C14" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="D14" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E14" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="F14" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G14" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="H14" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I14" t="str">
-        <v>Created by new employee process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J14" t="str">
-        <v xml:space="preserve">FK8 2BQ   </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Barbora Slabochova (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B15" t="str">
-        <v>37.5</v>
+        <v>30</v>
       </c>
       <c r="C15" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="D15" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E15" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="F15" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G15" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="H15" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I15" t="str">
-        <v>Created by new employee process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J15" t="str">
-        <v xml:space="preserve">FK8 2BQ   </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Barbora Slabochova (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B16" t="str">
-        <v>37.5</v>
+        <v>30</v>
       </c>
       <c r="C16" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="D16" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E16" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="F16" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G16" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="H16" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I16" t="str">
-        <v>Created by new employee process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J16" t="str">
-        <v xml:space="preserve">FK8 2BQ   </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Barbora Slabochova (GH)</v>
+        <v>Lorraine Parsons</v>
       </c>
       <c r="B17" t="str">
-        <v>37.5</v>
+        <v>10</v>
       </c>
       <c r="C17" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="D17" t="str">
         <v>2025-11-14</v>
       </c>
       <c r="E17" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="F17" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="G17" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="H17" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I17" t="str">
-        <v>Created by new employee process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J17" t="str">
-        <v xml:space="preserve">FK8 2BQ   </v>
+        <v xml:space="preserve">EH22 4FP  </v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Barbora Slabochova (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="B18" t="str">
-        <v>37.5</v>
+        <v>12</v>
       </c>
       <c r="C18" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="D18" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E18" t="str">
         <v>Available</v>
       </c>
       <c r="F18" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="G18" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="H18" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="I18" t="str">
-        <v>Created by new employee process.</v>
+        <v/>
       </c>
       <c r="J18" t="str">
-        <v xml:space="preserve">FK8 2BQ   </v>
+        <v xml:space="preserve">EH34 5HE  </v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Jamie Lee Kane (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="B19" t="str">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C19" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D19" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E19" t="str">
         <v>Available</v>
       </c>
       <c r="F19" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="G19" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H19" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I19" t="str">
-        <v/>
+        <v>Eilish emailed that she is traveling to Glasgow for her SVQ training (MU 04.11.25)</v>
       </c>
       <c r="J19" t="str">
-        <v xml:space="preserve">FK7 7PN   </v>
+        <v xml:space="preserve">EH34 5HE  </v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Jamie Lee Kane (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="B20" t="str">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C20" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D20" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E20" t="str">
         <v>Available</v>
       </c>
       <c r="F20" t="str">
-        <v>16:45-21:30</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="G20" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H20" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I20" t="str">
         <v/>
       </c>
       <c r="J20" t="str">
-        <v xml:space="preserve">FK7 7PN   </v>
+        <v xml:space="preserve">EH34 5HE  </v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Rhian Steel</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="B21" t="str">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C21" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D21" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E21" t="str">
         <v>Available</v>
       </c>
       <c r="F21" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="G21" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H21" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I21" t="str">
         <v/>
       </c>
       <c r="J21" t="str">
-        <v xml:space="preserve">FK10 2SR  </v>
+        <v xml:space="preserve">EH34 5HE  </v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Rhian Steel</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="B22" t="str">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C22" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D22" t="str">
         <v>2025-11-11</v>
@@ -1097,321 +1097,321 @@
         <v>Available</v>
       </c>
       <c r="F22" t="str">
-        <v>09:15-14:00</v>
+        <v>09:30-12:30; 18:30-21:30</v>
       </c>
       <c r="G22" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H22" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I22" t="str">
         <v/>
       </c>
       <c r="J22" t="str">
-        <v xml:space="preserve">FK10 2SR  </v>
+        <v xml:space="preserve">EH32 0DG  </v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Rhian Steel</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="B23" t="str">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C23" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D23" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E23" t="str">
         <v>Available</v>
       </c>
       <c r="F23" t="str">
-        <v>08:00-21:30</v>
+        <v>10:30-12:30; 18:30-21:30</v>
       </c>
       <c r="G23" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H23" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I23" t="str">
         <v/>
       </c>
       <c r="J23" t="str">
-        <v xml:space="preserve">FK10 2SR  </v>
+        <v xml:space="preserve">EH32 0DG  </v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Rhian Steel</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="B24" t="str">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C24" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D24" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E24" t="str">
         <v>Available</v>
       </c>
       <c r="F24" t="str">
-        <v>08:00-21:30</v>
+        <v>09:30-12:30; 18:30-21:30</v>
       </c>
       <c r="G24" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H24" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I24" t="str">
         <v/>
       </c>
       <c r="J24" t="str">
-        <v xml:space="preserve">FK10 2SR  </v>
+        <v xml:space="preserve">EH32 0DG  </v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="B25" t="str">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C25" t="str">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D25" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E25" t="str">
         <v>Available</v>
       </c>
       <c r="F25" t="str">
-        <v>08:15-21:30</v>
+        <v>10:30-11:30; 16:45-17:45</v>
       </c>
       <c r="G25" t="str">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H25" t="str">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I25" t="str">
         <v/>
       </c>
       <c r="J25" t="str">
-        <v xml:space="preserve">FK10 1NH  </v>
+        <v xml:space="preserve">EH32 0DG  </v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="B26" t="str">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="C26" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D26" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E26" t="str">
         <v>Available</v>
       </c>
       <c r="F26" t="str">
-        <v>08:15-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G26" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H26" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I26" t="str">
         <v/>
       </c>
       <c r="J26" t="str">
-        <v xml:space="preserve">FK10 1NH  </v>
+        <v xml:space="preserve">EH32 9SS  </v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="B27" t="str">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="C27" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D27" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E27" t="str">
         <v>Available</v>
       </c>
       <c r="F27" t="str">
-        <v>08:15-17:15</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G27" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H27" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I27" t="str">
         <v/>
       </c>
       <c r="J27" t="str">
-        <v xml:space="preserve">FK10 1NH  </v>
+        <v xml:space="preserve">EH32 9SS  </v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="B28" t="str">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="C28" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D28" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E28" t="str">
         <v>Available</v>
       </c>
       <c r="F28" t="str">
-        <v>08:15-17:15</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G28" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H28" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I28" t="str">
         <v/>
       </c>
       <c r="J28" t="str">
-        <v xml:space="preserve">FK10 1NH  </v>
+        <v xml:space="preserve">EH32 9SS  </v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="B29" t="str">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="C29" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D29" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E29" t="str">
         <v>Available</v>
       </c>
       <c r="F29" t="str">
-        <v>08:15-17:15</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G29" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H29" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I29" t="str">
         <v/>
       </c>
       <c r="J29" t="str">
-        <v xml:space="preserve">FK10 1NH  </v>
+        <v xml:space="preserve">EH32 9SS  </v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Ziyal Vidler</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="B30" t="str">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="C30" t="str">
-        <v>6.67</v>
+        <v>1</v>
       </c>
       <c r="D30" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E30" t="str">
         <v>Available</v>
       </c>
       <c r="F30" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="G30" t="str">
-        <v>6.67</v>
+        <v>1</v>
       </c>
       <c r="H30" t="str">
-        <v>6.67</v>
+        <v>1</v>
       </c>
       <c r="I30" t="str">
         <v/>
       </c>
       <c r="J30" t="str">
-        <v xml:space="preserve">FK5 4XD   </v>
+        <v xml:space="preserve">EH32 9SS  </v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Ziyal Vidler</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B31" t="str">
         <v>20</v>
       </c>
       <c r="C31" t="str">
-        <v>6.67</v>
+        <v>2.86</v>
       </c>
       <c r="D31" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E31" t="str">
         <v>Available</v>
       </c>
       <c r="F31" t="str">
-        <v>08:00-14:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G31" t="str">
-        <v>6.67</v>
+        <v>2.86</v>
       </c>
       <c r="H31" t="str">
-        <v>6.67</v>
+        <v>2.86</v>
       </c>
       <c r="I31" t="str">
         <v/>
       </c>
       <c r="J31" t="str">
-        <v xml:space="preserve">FK5 4XD   </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Ziyal Vidler</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B32" t="str">
         <v>20</v>
       </c>
       <c r="C32" t="str">
-        <v>6.67</v>
+        <v>2.86</v>
       </c>
       <c r="D32" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E32" t="str">
         <v>Available</v>
@@ -1420,158 +1420,158 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G32" t="str">
-        <v>6.67</v>
+        <v>2.86</v>
       </c>
       <c r="H32" t="str">
-        <v>6.67</v>
+        <v>2.86</v>
       </c>
       <c r="I32" t="str">
         <v/>
       </c>
       <c r="J32" t="str">
-        <v xml:space="preserve">FK5 4XD   </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B33" t="str">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="C33" t="str">
-        <v>9.2</v>
+        <v>2.86</v>
       </c>
       <c r="D33" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E33" t="str">
         <v>Available</v>
       </c>
       <c r="F33" t="str">
-        <v>08:00-22:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G33" t="str">
-        <v>9.2</v>
+        <v>2.86</v>
       </c>
       <c r="H33" t="str">
-        <v>9.2</v>
+        <v>2.86</v>
       </c>
       <c r="I33" t="str">
         <v/>
       </c>
       <c r="J33" t="str">
-        <v xml:space="preserve">FK2 7ER   </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B34" t="str">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="C34" t="str">
-        <v>9.2</v>
+        <v>2.86</v>
       </c>
       <c r="D34" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E34" t="str">
         <v>Available</v>
       </c>
       <c r="F34" t="str">
-        <v>08:00-22:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G34" t="str">
-        <v>9.2</v>
+        <v>2.86</v>
       </c>
       <c r="H34" t="str">
-        <v>9.2</v>
+        <v>2.86</v>
       </c>
       <c r="I34" t="str">
         <v/>
       </c>
       <c r="J34" t="str">
-        <v xml:space="preserve">FK2 7ER   </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B35" t="str">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="C35" t="str">
-        <v>9.2</v>
+        <v>2.86</v>
       </c>
       <c r="D35" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E35" t="str">
         <v>Available</v>
       </c>
       <c r="F35" t="str">
-        <v>08:00-22:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G35" t="str">
-        <v>9.2</v>
+        <v>2.86</v>
       </c>
       <c r="H35" t="str">
-        <v>9.2</v>
+        <v>2.86</v>
       </c>
       <c r="I35" t="str">
         <v/>
       </c>
       <c r="J35" t="str">
-        <v xml:space="preserve">FK2 7ER   </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B36" t="str">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="C36" t="str">
-        <v>9.2</v>
+        <v>2.86</v>
       </c>
       <c r="D36" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E36" t="str">
         <v>Available</v>
       </c>
       <c r="F36" t="str">
-        <v>08:00-22:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G36" t="str">
-        <v>9.2</v>
+        <v>2.86</v>
       </c>
       <c r="H36" t="str">
-        <v>9.2</v>
+        <v>2.86</v>
       </c>
       <c r="I36" t="str">
         <v/>
       </c>
       <c r="J36" t="str">
-        <v xml:space="preserve">FK2 7ER   </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>John Clarke (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B37" t="str">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C37" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="D37" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E37" t="str">
         <v>Available</v>
@@ -1580,187 +1580,187 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G37" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H37" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="I37" t="str">
         <v/>
       </c>
       <c r="J37" t="str">
-        <v xml:space="preserve">FK8 1XY   </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>John Clarke (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B38" t="str">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C38" t="str">
-        <v>7.5</v>
+        <v>1.67</v>
       </c>
       <c r="D38" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E38" t="str">
         <v>Available</v>
       </c>
       <c r="F38" t="str">
-        <v>08:00-21:30</v>
+        <v>12:00-21:00</v>
       </c>
       <c r="G38" t="str">
-        <v>7.5</v>
+        <v>1.67</v>
       </c>
       <c r="H38" t="str">
-        <v>7.5</v>
+        <v>1.67</v>
       </c>
       <c r="I38" t="str">
         <v/>
       </c>
       <c r="J38" t="str">
-        <v xml:space="preserve">FK8 1XY   </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Paul Chalmers (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B39" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C39" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="D39" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E39" t="str">
         <v>Available</v>
       </c>
       <c r="F39" t="str">
-        <v>09:15-15:15</v>
+        <v>12:00-21:00</v>
       </c>
       <c r="G39" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="H39" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="I39" t="str">
         <v/>
       </c>
       <c r="J39" t="str">
-        <v xml:space="preserve">FK10 3HJ  </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Paul Chalmers (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B40" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C40" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="D40" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E40" t="str">
         <v>Available</v>
       </c>
       <c r="F40" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-21:00</v>
       </c>
       <c r="G40" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="H40" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="I40" t="str">
         <v/>
       </c>
       <c r="J40" t="str">
-        <v xml:space="preserve">FK10 3HJ  </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Paul Chalmers (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B41" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C41" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="D41" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E41" t="str">
         <v>Available</v>
       </c>
       <c r="F41" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-21:00</v>
       </c>
       <c r="G41" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="H41" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="I41" t="str">
         <v/>
       </c>
       <c r="J41" t="str">
-        <v xml:space="preserve">FK10 3HJ  </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Paul Chalmers (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B42" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C42" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="D42" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E42" t="str">
         <v>Available</v>
       </c>
       <c r="F42" t="str">
-        <v>09:15-15:15</v>
+        <v>12:00-17:45</v>
       </c>
       <c r="G42" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="H42" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="I42" t="str">
         <v/>
       </c>
       <c r="J42" t="str">
-        <v xml:space="preserve">FK10 3HJ  </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Paul Chalmers (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B43" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C43" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="D43" t="str">
         <v>2025-11-16</v>
@@ -1769,30 +1769,30 @@
         <v>Available</v>
       </c>
       <c r="F43" t="str">
-        <v>09:15-15:15</v>
+        <v>21:00-22:00</v>
       </c>
       <c r="G43" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="H43" t="str">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="I43" t="str">
         <v/>
       </c>
       <c r="J43" t="str">
-        <v xml:space="preserve">FK10 3HJ  </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Chiamaka Onweluzo (GH)</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="B44" t="str">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="C44" t="str">
-        <v>9.2</v>
+        <v>3.33</v>
       </c>
       <c r="D44" t="str">
         <v>2025-11-10</v>
@@ -1801,30 +1801,30 @@
         <v>Available</v>
       </c>
       <c r="F44" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="G44" t="str">
-        <v>9.2</v>
+        <v>3.33</v>
       </c>
       <c r="H44" t="str">
-        <v>9.2</v>
+        <v>3.33</v>
       </c>
       <c r="I44" t="str">
         <v/>
       </c>
       <c r="J44" t="str">
-        <v xml:space="preserve">FK8 1RS   </v>
+        <v xml:space="preserve">EH21 6NQ  </v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Chiamaka Onweluzo (GH)</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="B45" t="str">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="C45" t="str">
-        <v>9.2</v>
+        <v>3.33</v>
       </c>
       <c r="D45" t="str">
         <v>2025-11-11</v>
@@ -1833,222 +1833,222 @@
         <v>Available</v>
       </c>
       <c r="F45" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="G45" t="str">
-        <v>9.2</v>
+        <v>3.33</v>
       </c>
       <c r="H45" t="str">
-        <v>9.2</v>
+        <v>3.33</v>
       </c>
       <c r="I45" t="str">
         <v/>
       </c>
       <c r="J45" t="str">
-        <v xml:space="preserve">FK8 1RS   </v>
+        <v xml:space="preserve">EH21 6NQ  </v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Kristin Earhart</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="B46" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C46" t="str">
-        <v>3.2</v>
+        <v>3.33</v>
       </c>
       <c r="D46" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E46" t="str">
         <v>Available</v>
       </c>
       <c r="F46" t="str">
-        <v>10:00-14:30</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="G46" t="str">
-        <v>3.2</v>
+        <v>3.33</v>
       </c>
       <c r="H46" t="str">
-        <v>3.2</v>
+        <v>3.33</v>
       </c>
       <c r="I46" t="str">
         <v/>
       </c>
       <c r="J46" t="str">
-        <v xml:space="preserve">FK12 5HG  </v>
+        <v xml:space="preserve">EH21 6NQ  </v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Kristin Earhart</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="B47" t="str">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C47" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="D47" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E47" t="str">
         <v>Available</v>
       </c>
       <c r="F47" t="str">
-        <v>10:00-14:30</v>
+        <v>08:00-16:30</v>
       </c>
       <c r="G47" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="H47" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="I47" t="str">
         <v/>
       </c>
       <c r="J47" t="str">
-        <v xml:space="preserve">FK12 5HG  </v>
+        <v xml:space="preserve">EH21 6JY  </v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Kristin Earhart</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="B48" t="str">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C48" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="D48" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E48" t="str">
         <v>Available</v>
       </c>
       <c r="F48" t="str">
-        <v>10:00-14:30</v>
+        <v>08:00-16:00</v>
       </c>
       <c r="G48" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="H48" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="I48" t="str">
         <v/>
       </c>
       <c r="J48" t="str">
-        <v xml:space="preserve">FK12 5HG  </v>
+        <v xml:space="preserve">EH21 6JY  </v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Kristin Earhart</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="B49" t="str">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C49" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="D49" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E49" t="str">
         <v>Available</v>
       </c>
       <c r="F49" t="str">
-        <v>10:00-14:30</v>
+        <v>08:00-16:00</v>
       </c>
       <c r="G49" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="H49" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="I49" t="str">
         <v/>
       </c>
       <c r="J49" t="str">
-        <v xml:space="preserve">FK12 5HG  </v>
+        <v xml:space="preserve">EH21 6JY  </v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Kristin Earhart</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="B50" t="str">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C50" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="D50" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E50" t="str">
         <v>Available</v>
       </c>
       <c r="F50" t="str">
-        <v>10:00-14:30</v>
+        <v>08:00-16:00</v>
       </c>
       <c r="G50" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="H50" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="I50" t="str">
         <v/>
       </c>
       <c r="J50" t="str">
-        <v xml:space="preserve">FK12 5HG  </v>
+        <v xml:space="preserve">EH21 6JY  </v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Alison Shields (GH)</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="B51" t="str">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C51" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="D51" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E51" t="str">
         <v>Available</v>
       </c>
       <c r="F51" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-16:30</v>
       </c>
       <c r="G51" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="H51" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="I51" t="str">
         <v/>
       </c>
       <c r="J51" t="str">
-        <v xml:space="preserve">FK3 8LP   </v>
+        <v xml:space="preserve">EH21 6JY  </v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Alison Shields (GH)</v>
+        <v>Lorraine Parsons</v>
       </c>
       <c r="B52" t="str">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C52" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="D52" t="str">
         <v>2025-11-11</v>
@@ -2057,88 +2057,216 @@
         <v>Available</v>
       </c>
       <c r="F52" t="str">
-        <v>08:00-21:30</v>
+        <v>09:30-14:30</v>
       </c>
       <c r="G52" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="H52" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="I52" t="str">
         <v/>
       </c>
       <c r="J52" t="str">
-        <v xml:space="preserve">FK3 8LP   </v>
+        <v xml:space="preserve">EH22 4FP  </v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Alison Shields (GH)</v>
+        <v>Lorraine Parsons</v>
       </c>
       <c r="B53" t="str">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C53" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="D53" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E53" t="str">
         <v>Available</v>
       </c>
       <c r="F53" t="str">
-        <v>08:00-21:30</v>
+        <v>09:30-14:30</v>
       </c>
       <c r="G53" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="H53" t="str">
-        <v>7.5</v>
+        <v>3.33</v>
       </c>
       <c r="I53" t="str">
         <v/>
       </c>
       <c r="J53" t="str">
-        <v xml:space="preserve">FK3 8LP   </v>
+        <v xml:space="preserve">EH22 4FP  </v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Alison Shields (GH)</v>
+        <v>Victoria Bateman (GH)</v>
       </c>
       <c r="B54" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C54" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="D54" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E54" t="str">
         <v>Available</v>
       </c>
       <c r="F54" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="G54" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="H54" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="I54" t="str">
         <v/>
       </c>
       <c r="J54" t="str">
-        <v xml:space="preserve">FK3 8LP   </v>
+        <v xml:space="preserve">EH23 4NL  </v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Victoria Bateman (GH)</v>
+      </c>
+      <c r="B55" t="str">
+        <v>16</v>
+      </c>
+      <c r="C55" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="D55" t="str">
+        <v>2025-11-11</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F55" t="str">
+        <v>08:00-15:30</v>
+      </c>
+      <c r="G55" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H55" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55" t="str">
+        <v xml:space="preserve">EH23 4NL  </v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Victoria Bateman (GH)</v>
+      </c>
+      <c r="B56" t="str">
+        <v>16</v>
+      </c>
+      <c r="C56" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="D56" t="str">
+        <v>2025-11-12</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F56" t="str">
+        <v>08:00-15:30</v>
+      </c>
+      <c r="G56" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H56" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="I56" t="str">
+        <v/>
+      </c>
+      <c r="J56" t="str">
+        <v xml:space="preserve">EH23 4NL  </v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Victoria Bateman (GH)</v>
+      </c>
+      <c r="B57" t="str">
+        <v>16</v>
+      </c>
+      <c r="C57" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="D57" t="str">
+        <v>2025-11-13</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F57" t="str">
+        <v>08:00-17:30</v>
+      </c>
+      <c r="G57" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H57" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="I57" t="str">
+        <v/>
+      </c>
+      <c r="J57" t="str">
+        <v xml:space="preserve">EH23 4NL  </v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Victoria Bateman (GH)</v>
+      </c>
+      <c r="B58" t="str">
+        <v>16</v>
+      </c>
+      <c r="C58" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="D58" t="str">
+        <v>2025-11-14</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Available</v>
+      </c>
+      <c r="F58" t="str">
+        <v>08:00-15:30</v>
+      </c>
+      <c r="G58" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H58" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="I58" t="str">
+        <v/>
+      </c>
+      <c r="J58" t="str">
+        <v xml:space="preserve">EH23 4NL  </v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J58"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2178,22 +2306,22 @@
         <v>2025-11-10</v>
       </c>
       <c r="B2" t="str">
-        <v>34.1</v>
+        <v>18.06</v>
       </c>
       <c r="C2" t="str">
-        <v>39.3</v>
+        <v>18.06</v>
       </c>
       <c r="D2" t="str">
-        <v>5.2</v>
+        <v>0</v>
       </c>
       <c r="E2" t="str">
-        <v>7.5</v>
+        <v>6.58</v>
       </c>
       <c r="F2" t="str">
-        <v>58</v>
+        <v>25.5</v>
       </c>
       <c r="G2" t="str">
-        <v>-18.7</v>
+        <v>-7.44</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -2204,22 +2332,22 @@
         <v>2025-11-11</v>
       </c>
       <c r="B3" t="str">
-        <v>58.3</v>
+        <v>24.39</v>
       </c>
       <c r="C3" t="str">
-        <v>58.3</v>
+        <v>24.39</v>
       </c>
       <c r="D3" t="str">
         <v>0</v>
       </c>
       <c r="E3" t="str">
-        <v>11.5</v>
+        <v>6.58</v>
       </c>
       <c r="F3" t="str">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="G3" t="str">
-        <v>-3.7</v>
+        <v>-3.61</v>
       </c>
       <c r="H3" t="str">
         <v>Shortage</v>
@@ -2230,22 +2358,22 @@
         <v>2025-11-12</v>
       </c>
       <c r="B4" t="str">
-        <v>40.6</v>
+        <v>21.06</v>
       </c>
       <c r="C4" t="str">
-        <v>40.6</v>
+        <v>21.06</v>
       </c>
       <c r="D4" t="str">
         <v>0</v>
       </c>
       <c r="E4" t="str">
-        <v>0</v>
+        <v>6.58</v>
       </c>
       <c r="F4" t="str">
-        <v>66</v>
+        <v>24.5</v>
       </c>
       <c r="G4" t="str">
-        <v>-25.4</v>
+        <v>-3.44</v>
       </c>
       <c r="H4" t="str">
         <v>Shortage</v>
@@ -2256,22 +2384,22 @@
         <v>2025-11-13</v>
       </c>
       <c r="B5" t="str">
-        <v>43.27</v>
+        <v>21.06</v>
       </c>
       <c r="C5" t="str">
-        <v>43.27</v>
+        <v>21.06</v>
       </c>
       <c r="D5" t="str">
         <v>0</v>
       </c>
       <c r="E5" t="str">
-        <v>4</v>
+        <v>6.58</v>
       </c>
       <c r="F5" t="str">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="G5" t="str">
-        <v>-8.73</v>
+        <v>-4.94</v>
       </c>
       <c r="H5" t="str">
         <v>Shortage</v>
@@ -2282,22 +2410,22 @@
         <v>2025-11-14</v>
       </c>
       <c r="B6" t="str">
-        <v>44.07</v>
+        <v>8.73</v>
       </c>
       <c r="C6" t="str">
-        <v>44.07</v>
+        <v>8.73</v>
       </c>
       <c r="D6" t="str">
         <v>0</v>
       </c>
       <c r="E6" t="str">
-        <v>9.2</v>
+        <v>9.91</v>
       </c>
       <c r="F6" t="str">
-        <v>58</v>
+        <v>21.5</v>
       </c>
       <c r="G6" t="str">
-        <v>-13.93</v>
+        <v>-12.77</v>
       </c>
       <c r="H6" t="str">
         <v>Shortage</v>
@@ -2308,22 +2436,22 @@
         <v>2025-11-15</v>
       </c>
       <c r="B7" t="str">
-        <v>27.5</v>
+        <v>8.86</v>
       </c>
       <c r="C7" t="str">
-        <v>27.5</v>
+        <v>8.86</v>
       </c>
       <c r="D7" t="str">
         <v>0</v>
       </c>
       <c r="E7" t="str">
-        <v>9.2</v>
+        <v>6.58</v>
       </c>
       <c r="F7" t="str">
-        <v>49</v>
+        <v>16.5</v>
       </c>
       <c r="G7" t="str">
-        <v>-21.5</v>
+        <v>-7.64</v>
       </c>
       <c r="H7" t="str">
         <v>Shortage</v>
@@ -2334,22 +2462,22 @@
         <v>2025-11-16</v>
       </c>
       <c r="B8" t="str">
-        <v>29.87</v>
+        <v>4.53</v>
       </c>
       <c r="C8" t="str">
-        <v>29.87</v>
+        <v>4.53</v>
       </c>
       <c r="D8" t="str">
         <v>0</v>
       </c>
       <c r="E8" t="str">
-        <v>9.2</v>
+        <v>8.58</v>
       </c>
       <c r="F8" t="str">
-        <v>48</v>
+        <v>12.5</v>
       </c>
       <c r="G8" t="str">
-        <v>-18.13</v>
+        <v>-7.97</v>
       </c>
       <c r="H8" t="str">
         <v>Shortage</v>
@@ -2364,7 +2492,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H68"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2394,25 +2522,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B2" t="str">
-        <v>Alison Shields (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="C2" t="str">
         <v>Available</v>
       </c>
       <c r="D2" t="str">
-        <v>08:00-21:30</v>
+        <v>21:00-22:00</v>
       </c>
       <c r="E2" t="str">
-        <v>7.5</v>
+        <v>1.67</v>
       </c>
       <c r="F2" t="str">
-        <v>7.5</v>
+        <v>1.67</v>
       </c>
       <c r="G2" t="str">
-        <v>7.5</v>
+        <v>1.67</v>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -2420,25 +2548,25 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B3" t="str">
-        <v>Anisa Naeem</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="C3" t="str">
         <v>Available</v>
       </c>
       <c r="D3" t="str">
-        <v>15:30-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E3" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="F3" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="G3" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -2446,88 +2574,88 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B4" t="str">
-        <v>Barbora Slabochova (GH)</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="C4" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D4" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E4" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="F4" t="str">
-        <v>7.5</v>
+        <v>2</v>
       </c>
       <c r="G4" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H4" t="str">
-        <v>Created by new employee process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B5" t="str">
-        <v>Chiamaka Onweluzo (GH)</v>
+        <v>McNally, Eilish</v>
       </c>
       <c r="C5" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D5" t="str">
-        <v>08:00-21:30</v>
+        <v>19:00-21:29</v>
       </c>
       <c r="E5" t="str">
-        <v>9.2</v>
+        <v>0</v>
       </c>
       <c r="F5" t="str">
-        <v>9.2</v>
+        <v>0</v>
       </c>
       <c r="G5" t="str">
-        <v>9.2</v>
+        <v>0</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B6" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="C6" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D6" t="str">
-        <v>08:00-22:00</v>
+        <v/>
       </c>
       <c r="E6" t="str">
-        <v>9.2</v>
+        <v>2.29</v>
       </c>
       <c r="F6" t="str">
-        <v>9.2</v>
+        <v>2.29</v>
       </c>
       <c r="G6" t="str">
-        <v>9.2</v>
+        <v>0</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B7" t="str">
-        <v>Jamie Lee Kane (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="C7" t="str">
         <v>Holiday</v>
@@ -2536,10 +2664,10 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>4</v>
+        <v>4.29</v>
       </c>
       <c r="F7" t="str">
-        <v>4</v>
+        <v>4.29</v>
       </c>
       <c r="G7" t="str">
         <v>0</v>
@@ -2550,51 +2678,51 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B8" t="str">
-        <v>John Clarke (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="C8" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D8" t="str">
-        <v/>
+        <v>12:00-21:00</v>
       </c>
       <c r="E8" t="str">
-        <v>7.5</v>
+        <v>1.67</v>
       </c>
       <c r="F8" t="str">
-        <v>7.5</v>
+        <v>1.67</v>
       </c>
       <c r="G8" t="str">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="H8" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B9" t="str">
-        <v>Kristin Earhart</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="C9" t="str">
         <v>Available</v>
       </c>
       <c r="D9" t="str">
-        <v>10:00-14:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E9" t="str">
-        <v>3.2</v>
+        <v>2.86</v>
       </c>
       <c r="F9" t="str">
-        <v>3.2</v>
+        <v>2.86</v>
       </c>
       <c r="G9" t="str">
-        <v>3.2</v>
+        <v>2.86</v>
       </c>
       <c r="H9" t="str">
         <v/>
@@ -2602,25 +2730,25 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B10" t="str">
-        <v>Paul Chalmers (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="C10" t="str">
         <v>Available</v>
       </c>
       <c r="D10" t="str">
-        <v>09:15-15:15</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="E10" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="F10" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="G10" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="H10" t="str">
         <v/>
@@ -2628,25 +2756,25 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B11" t="str">
-        <v>Rhian Steel</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="C11" t="str">
         <v>Available</v>
       </c>
       <c r="D11" t="str">
-        <v>09:15-14:00</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E11" t="str">
-        <v>5</v>
+        <v>3.33</v>
       </c>
       <c r="F11" t="str">
-        <v>5</v>
+        <v>3.33</v>
       </c>
       <c r="G11" t="str">
-        <v>5</v>
+        <v>3.33</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -2654,25 +2782,25 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B12" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="C12" t="str">
         <v>Available</v>
       </c>
       <c r="D12" t="str">
-        <v>08:15-21:30</v>
+        <v>08:00-16:30</v>
       </c>
       <c r="E12" t="str">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F12" t="str">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G12" t="str">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H12" t="str">
         <v/>
@@ -2680,103 +2808,103 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B13" t="str">
-        <v>Vidler, Ziyal</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="C13" t="str">
-        <v>Ad-hoc</v>
+        <v>Holiday</v>
       </c>
       <c r="D13" t="str">
-        <v>12:29-13:00</v>
+        <v/>
       </c>
       <c r="E13" t="str">
-        <v>0</v>
+        <v>2.29</v>
       </c>
       <c r="F13" t="str">
-        <v>0</v>
+        <v>2.29</v>
       </c>
       <c r="G13" t="str">
         <v>0</v>
       </c>
       <c r="H13" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B14" t="str">
-        <v>Anisa Naeem</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="C14" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D14" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E14" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="F14" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="G14" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B15" t="str">
-        <v>Barbora Slabochova (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="C15" t="str">
         <v>Available</v>
       </c>
       <c r="D15" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E15" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="F15" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="G15" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="H15" t="str">
-        <v>Created by new employee process.</v>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B16" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>Victoria Bateman (GH)</v>
       </c>
       <c r="C16" t="str">
         <v>Available</v>
       </c>
       <c r="D16" t="str">
-        <v>08:00-22:00</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E16" t="str">
-        <v>9.2</v>
+        <v>3.2</v>
       </c>
       <c r="F16" t="str">
-        <v>9.2</v>
+        <v>3.2</v>
       </c>
       <c r="G16" t="str">
-        <v>9.2</v>
+        <v>3.2</v>
       </c>
       <c r="H16" t="str">
         <v/>
@@ -2784,77 +2912,77 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B17" t="str">
-        <v>Jamie Lee Kane (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="C17" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D17" t="str">
-        <v/>
+        <v>12:00-21:00</v>
       </c>
       <c r="E17" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="F17" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="G17" t="str">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="H17" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B18" t="str">
-        <v>Kristin Earhart</v>
+        <v>Dale (GH), Heather</v>
       </c>
       <c r="C18" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D18" t="str">
-        <v>10:00-14:30</v>
+        <v>09:22-11:53</v>
       </c>
       <c r="E18" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="F18" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="G18" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H18" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B19" t="str">
-        <v>Paul Chalmers (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="C19" t="str">
         <v>Available</v>
       </c>
       <c r="D19" t="str">
-        <v>09:15-15:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E19" t="str">
-        <v>3.2</v>
+        <v>2.86</v>
       </c>
       <c r="F19" t="str">
-        <v>3.2</v>
+        <v>2.86</v>
       </c>
       <c r="G19" t="str">
-        <v>3.2</v>
+        <v>2.86</v>
       </c>
       <c r="H19" t="str">
         <v/>
@@ -2862,51 +2990,51 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B20" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="C20" t="str">
         <v>Available</v>
       </c>
       <c r="D20" t="str">
-        <v>08:15-17:15</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="E20" t="str">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F20" t="str">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G20" t="str">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H20" t="str">
-        <v/>
+        <v>Eilish emailed that she is traveling to Glasgow for her SVQ training (MU 04.11.25)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B21" t="str">
-        <v>Ziyal Vidler</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="C21" t="str">
         <v>Available</v>
       </c>
       <c r="D21" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-18:00</v>
       </c>
       <c r="E21" t="str">
-        <v>6.67</v>
+        <v>3.33</v>
       </c>
       <c r="F21" t="str">
-        <v>6.67</v>
+        <v>3.33</v>
       </c>
       <c r="G21" t="str">
-        <v>6.67</v>
+        <v>3.33</v>
       </c>
       <c r="H21" t="str">
         <v/>
@@ -2914,51 +3042,51 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B22" t="str">
-        <v>Alison Shields (GH)</v>
+        <v>Hartley-Oliver (GH), Ruby</v>
       </c>
       <c r="C22" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D22" t="str">
-        <v>08:00-21:30</v>
+        <v>13:59-16:59</v>
       </c>
       <c r="E22" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="F22" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G22" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H22" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B23" t="str">
-        <v>Chiamaka Onweluzo (GH)</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="C23" t="str">
         <v>Available</v>
       </c>
       <c r="D23" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-16:00</v>
       </c>
       <c r="E23" t="str">
-        <v>9.2</v>
+        <v>3</v>
       </c>
       <c r="F23" t="str">
-        <v>9.2</v>
+        <v>3</v>
       </c>
       <c r="G23" t="str">
-        <v>9.2</v>
+        <v>3</v>
       </c>
       <c r="H23" t="str">
         <v/>
@@ -2966,129 +3094,129 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B24" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>Lorraine Parsons</v>
       </c>
       <c r="C24" t="str">
-        <v>Partial Availability</v>
+        <v>Available</v>
       </c>
       <c r="D24" t="str">
-        <v>08:00-13:00; 17:00-22:00</v>
+        <v>09:30-14:30</v>
       </c>
       <c r="E24" t="str">
-        <v>9.2</v>
+        <v>3.33</v>
       </c>
       <c r="F24" t="str">
-        <v>5.2</v>
+        <v>3.33</v>
       </c>
       <c r="G24" t="str">
-        <v>5.2</v>
+        <v>3.33</v>
       </c>
       <c r="H24" t="str">
-        <v>Haseeb is helping out GN</v>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B25" t="str">
-        <v>John Clarke (GH)</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="C25" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D25" t="str">
-        <v/>
+        <v>09:30-12:30; 18:30-21:30</v>
       </c>
       <c r="E25" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="F25" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="G25" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H25" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B26" t="str">
-        <v>Kristin Earhart</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="C26" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D26" t="str">
-        <v>10:00-14:30</v>
+        <v/>
       </c>
       <c r="E26" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="F26" t="str">
-        <v>3.2</v>
+        <v>2.29</v>
       </c>
       <c r="G26" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H26" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B27" t="str">
-        <v>Paul Chalmers (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="C27" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D27" t="str">
-        <v>09:15-15:15</v>
+        <v/>
       </c>
       <c r="E27" t="str">
-        <v>3.2</v>
+        <v>4.29</v>
       </c>
       <c r="F27" t="str">
-        <v>3.2</v>
+        <v>4.29</v>
       </c>
       <c r="G27" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H27" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B28" t="str">
-        <v>Rhian Steel</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="C28" t="str">
         <v>Available</v>
       </c>
       <c r="D28" t="str">
-        <v>09:15-14:00</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E28" t="str">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F28" t="str">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G28" t="str">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -3096,25 +3224,25 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B29" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Victoria Bateman (GH)</v>
       </c>
       <c r="C29" t="str">
         <v>Available</v>
       </c>
       <c r="D29" t="str">
-        <v>08:15-21:30</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E29" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="F29" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="G29" t="str">
-        <v>6</v>
+        <v>3.2</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -3122,62 +3250,62 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B30" t="str">
-        <v>Stevenson (GH), Keri</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="C30" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D30" t="str">
-        <v>09:15-12:15</v>
+        <v>09:15-21:00</v>
       </c>
       <c r="E30" t="str">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="F30" t="str">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="G30" t="str">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="H30" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B31" t="str">
-        <v>Anisa Naeem</v>
+        <v>Dale (GH), Heather</v>
       </c>
       <c r="C31" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D31" t="str">
-        <v>08:00-21:30</v>
+        <v>09:29-13:30</v>
       </c>
       <c r="E31" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="F31" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G31" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H31" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B32" t="str">
-        <v>Barbora Slabochova (GH)</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="C32" t="str">
         <v>Available</v>
@@ -3186,65 +3314,65 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E32" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="F32" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="G32" t="str">
-        <v>7.5</v>
+        <v>2.86</v>
       </c>
       <c r="H32" t="str">
-        <v>Created by new employee process.</v>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B33" t="str">
-        <v>Chiamaka Onweluzo (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="C33" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D33" t="str">
-        <v/>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="E33" t="str">
-        <v>9.2</v>
+        <v>3</v>
       </c>
       <c r="F33" t="str">
-        <v>9.2</v>
+        <v>3</v>
       </c>
       <c r="G33" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H33" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B34" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="C34" t="str">
         <v>Available</v>
       </c>
       <c r="D34" t="str">
-        <v>08:00-22:00</v>
+        <v>08:00-16:00</v>
       </c>
       <c r="E34" t="str">
-        <v>9.2</v>
+        <v>3</v>
       </c>
       <c r="F34" t="str">
-        <v>9.2</v>
+        <v>3</v>
       </c>
       <c r="G34" t="str">
-        <v>9.2</v>
+        <v>3</v>
       </c>
       <c r="H34" t="str">
         <v/>
@@ -3252,25 +3380,25 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B35" t="str">
-        <v>Jamie Lee Kane (GH)</v>
+        <v>Lorraine Parsons</v>
       </c>
       <c r="C35" t="str">
         <v>Available</v>
       </c>
       <c r="D35" t="str">
-        <v>16:45-21:30</v>
+        <v>09:30-14:30</v>
       </c>
       <c r="E35" t="str">
-        <v>4</v>
+        <v>3.33</v>
       </c>
       <c r="F35" t="str">
-        <v>4</v>
+        <v>3.33</v>
       </c>
       <c r="G35" t="str">
-        <v>4</v>
+        <v>3.33</v>
       </c>
       <c r="H35" t="str">
         <v/>
@@ -3278,25 +3406,25 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B36" t="str">
-        <v>Kristin Earhart</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="C36" t="str">
         <v>Available</v>
       </c>
       <c r="D36" t="str">
-        <v>10:00-14:30</v>
+        <v>10:30-12:30; 18:30-21:30</v>
       </c>
       <c r="E36" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="F36" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="G36" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="H36" t="str">
         <v/>
@@ -3304,77 +3432,77 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B37" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="C37" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D37" t="str">
-        <v>08:15-17:15</v>
+        <v/>
       </c>
       <c r="E37" t="str">
-        <v>6</v>
+        <v>2.29</v>
       </c>
       <c r="F37" t="str">
-        <v>6</v>
+        <v>2.29</v>
       </c>
       <c r="G37" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H37" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B38" t="str">
-        <v>Ziyal Vidler</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="C38" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D38" t="str">
-        <v>08:00-14:00</v>
+        <v/>
       </c>
       <c r="E38" t="str">
-        <v>6.67</v>
+        <v>4.29</v>
       </c>
       <c r="F38" t="str">
-        <v>6.67</v>
+        <v>4.29</v>
       </c>
       <c r="G38" t="str">
-        <v>6.67</v>
+        <v>0</v>
       </c>
       <c r="H38" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B39" t="str">
-        <v>Alison Shields (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="C39" t="str">
         <v>Available</v>
       </c>
       <c r="D39" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E39" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="F39" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="G39" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="H39" t="str">
         <v/>
@@ -3382,88 +3510,88 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B40" t="str">
-        <v>Barbora Slabochova (GH)</v>
+        <v>Victoria Bateman (GH)</v>
       </c>
       <c r="C40" t="str">
         <v>Available</v>
       </c>
       <c r="D40" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-15:30</v>
       </c>
       <c r="E40" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="F40" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="G40" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="H40" t="str">
-        <v>Created by new employee process.</v>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B41" t="str">
-        <v>Chiamaka Onweluzo (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="C41" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D41" t="str">
-        <v/>
+        <v>09:15-21:00</v>
       </c>
       <c r="E41" t="str">
-        <v>9.2</v>
+        <v>1.67</v>
       </c>
       <c r="F41" t="str">
-        <v>9.2</v>
+        <v>1.67</v>
       </c>
       <c r="G41" t="str">
-        <v>0</v>
+        <v>1.67</v>
       </c>
       <c r="H41" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B42" t="str">
-        <v>John Clarke (GH)</v>
+        <v>Dale (GH), Heather</v>
       </c>
       <c r="C42" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D42" t="str">
-        <v>08:00-21:30</v>
+        <v>09:29-12:00</v>
       </c>
       <c r="E42" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="F42" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G42" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H42" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B43" t="str">
-        <v>Rhian Steel</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="C43" t="str">
         <v>Available</v>
@@ -3472,13 +3600,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E43" t="str">
-        <v>5</v>
+        <v>2.86</v>
       </c>
       <c r="F43" t="str">
-        <v>5</v>
+        <v>2.86</v>
       </c>
       <c r="G43" t="str">
-        <v>5</v>
+        <v>2.86</v>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -3486,25 +3614,25 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B44" t="str">
-        <v>Alison Shields (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="C44" t="str">
         <v>Available</v>
       </c>
       <c r="D44" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-10:00; 19:00-21:30</v>
       </c>
       <c r="E44" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="F44" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="G44" t="str">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="H44" t="str">
         <v/>
@@ -3512,77 +3640,77 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B45" t="str">
-        <v>Chiamaka Onweluzo (GH)</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="C45" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D45" t="str">
-        <v/>
+        <v>08:00-18:00</v>
       </c>
       <c r="E45" t="str">
-        <v>9.2</v>
+        <v>3.33</v>
       </c>
       <c r="F45" t="str">
-        <v>9.2</v>
+        <v>3.33</v>
       </c>
       <c r="G45" t="str">
-        <v>0</v>
+        <v>3.33</v>
       </c>
       <c r="H45" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B46" t="str">
-        <v>John Clarke (GH)</v>
+        <v>Hartley-Oliver (GH), Ruby</v>
       </c>
       <c r="C46" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D46" t="str">
-        <v>08:00-21:30</v>
+        <v>13:59-16:59</v>
       </c>
       <c r="E46" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="F46" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G46" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H46" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B47" t="str">
-        <v>Paul Chalmers (GH)</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="C47" t="str">
         <v>Available</v>
       </c>
       <c r="D47" t="str">
-        <v>09:15-15:15</v>
+        <v>08:00-16:00</v>
       </c>
       <c r="E47" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="F47" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="G47" t="str">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="H47" t="str">
         <v/>
@@ -3590,25 +3718,25 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B48" t="str">
-        <v>Rhian Steel</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="C48" t="str">
         <v>Available</v>
       </c>
       <c r="D48" t="str">
-        <v>08:00-21:30</v>
+        <v>09:30-12:30; 18:30-21:30</v>
       </c>
       <c r="E48" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F48" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G48" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H48" t="str">
         <v/>
@@ -3616,103 +3744,103 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B49" t="str">
-        <v>Ziyal Vidler</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="C49" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D49" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E49" t="str">
-        <v>6.67</v>
+        <v>2.29</v>
       </c>
       <c r="F49" t="str">
-        <v>6.67</v>
+        <v>2.29</v>
       </c>
       <c r="G49" t="str">
-        <v>6.67</v>
+        <v>0</v>
       </c>
       <c r="H49" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B50" t="str">
-        <v>Anisa Naeem</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="C50" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D50" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E50" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="F50" t="str">
-        <v>7.5</v>
+        <v>4.29</v>
       </c>
       <c r="G50" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H50" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B51" t="str">
-        <v>Barbora Slabochova (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="C51" t="str">
         <v>Available</v>
       </c>
       <c r="D51" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-10:15</v>
       </c>
       <c r="E51" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="F51" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="G51" t="str">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="H51" t="str">
-        <v>Created by new employee process.</v>
+        <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B52" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>Victoria Bateman (GH)</v>
       </c>
       <c r="C52" t="str">
         <v>Available</v>
       </c>
       <c r="D52" t="str">
-        <v>08:00-22:00</v>
+        <v>08:00-17:30</v>
       </c>
       <c r="E52" t="str">
-        <v>9.2</v>
+        <v>3.2</v>
       </c>
       <c r="F52" t="str">
-        <v>9.2</v>
+        <v>3.2</v>
       </c>
       <c r="G52" t="str">
-        <v>9.2</v>
+        <v>3.2</v>
       </c>
       <c r="H52" t="str">
         <v/>
@@ -3720,25 +3848,25 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B53" t="str">
-        <v>Jamie Lee Kane (GH)</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="C53" t="str">
         <v>Available</v>
       </c>
       <c r="D53" t="str">
-        <v>16:45-21:30</v>
+        <v>12:00-17:45</v>
       </c>
       <c r="E53" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="F53" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="G53" t="str">
-        <v>4</v>
+        <v>1.67</v>
       </c>
       <c r="H53" t="str">
         <v/>
@@ -3746,25 +3874,25 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B54" t="str">
-        <v>Kristin Earhart</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="C54" t="str">
         <v>Available</v>
       </c>
       <c r="D54" t="str">
-        <v>10:00-14:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E54" t="str">
-        <v>3.2</v>
+        <v>2.86</v>
       </c>
       <c r="F54" t="str">
-        <v>3.2</v>
+        <v>2.86</v>
       </c>
       <c r="G54" t="str">
-        <v>3.2</v>
+        <v>2.86</v>
       </c>
       <c r="H54" t="str">
         <v/>
@@ -3772,16 +3900,16 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B55" t="str">
-        <v>Onweluzo (GH), Chiamaka</v>
+        <v>Hartley-Oliver (GH), Ruby</v>
       </c>
       <c r="C55" t="str">
         <v>Ad-hoc</v>
       </c>
       <c r="D55" t="str">
-        <v>07:59-09:00; 09:29-14:30</v>
+        <v>10:45-13:45</v>
       </c>
       <c r="E55" t="str">
         <v>0</v>
@@ -3798,66 +3926,352 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B56" t="str">
-        <v>Paul Chalmers (GH)</v>
+        <v>Lorraine Parsons</v>
       </c>
       <c r="C56" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D56" t="str">
-        <v>09:15-15:15</v>
+        <v/>
       </c>
       <c r="E56" t="str">
-        <v>3.2</v>
+        <v>3.33</v>
       </c>
       <c r="F56" t="str">
-        <v>3.2</v>
+        <v>3.33</v>
       </c>
       <c r="G56" t="str">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="H56" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B57" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="C57" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D57" t="str">
-        <v>08:15-17:15</v>
+        <v/>
       </c>
       <c r="E57" t="str">
-        <v>6</v>
+        <v>2.29</v>
       </c>
       <c r="F57" t="str">
-        <v>6</v>
+        <v>2.29</v>
       </c>
       <c r="G57" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H57" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>2025-11-14</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Morrison (GH), Helen</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Ad-hoc</v>
+      </c>
+      <c r="D58" t="str">
+        <v>07:59-09:00</v>
+      </c>
+      <c r="E58" t="str">
+        <v>0</v>
+      </c>
+      <c r="F58" t="str">
+        <v>0</v>
+      </c>
+      <c r="G58" t="str">
+        <v>0</v>
+      </c>
+      <c r="H58" t="str">
+        <v>Scheduled (no availability record for this day)</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>2025-11-14</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Muhammad Irtaza Tahir (GH)</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Holiday</v>
+      </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
+      <c r="E59" t="str">
+        <v>4.29</v>
+      </c>
+      <c r="F59" t="str">
+        <v>4.29</v>
+      </c>
+      <c r="G59" t="str">
+        <v>0</v>
+      </c>
+      <c r="H59" t="str">
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>2025-11-14</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Romina Ferrara</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D60" t="str">
+        <v>09:15-10:15</v>
+      </c>
+      <c r="E60" t="str">
+        <v>1</v>
+      </c>
+      <c r="F60" t="str">
+        <v>1</v>
+      </c>
+      <c r="G60" t="str">
+        <v>1</v>
+      </c>
+      <c r="H60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>2025-11-14</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Victoria Bateman (GH)</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D61" t="str">
+        <v>08:00-15:30</v>
+      </c>
+      <c r="E61" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="F61" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="G61" t="str">
+        <v>3.2</v>
+      </c>
+      <c r="H61" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>2025-11-15</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Dhaval Mithaiwala</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D62" t="str">
+        <v>08:00-21:30</v>
+      </c>
+      <c r="E62" t="str">
+        <v>2.86</v>
+      </c>
+      <c r="F62" t="str">
+        <v>2.86</v>
+      </c>
+      <c r="G62" t="str">
+        <v>2.86</v>
+      </c>
+      <c r="H62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2025-11-15</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Hartley-Oliver (GH), Ruby</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Ad-hoc</v>
+      </c>
+      <c r="D63" t="str">
+        <v>12:29-15:29</v>
+      </c>
+      <c r="E63" t="str">
+        <v>0</v>
+      </c>
+      <c r="F63" t="str">
+        <v>0</v>
+      </c>
+      <c r="G63" t="str">
+        <v>0</v>
+      </c>
+      <c r="H63" t="str">
+        <v>Scheduled (no availability record for this day)</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>2025-11-15</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Helen Morrison (GH)</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D64" t="str">
+        <v>08:00-16:30</v>
+      </c>
+      <c r="E64" t="str">
+        <v>3</v>
+      </c>
+      <c r="F64" t="str">
+        <v>3</v>
+      </c>
+      <c r="G64" t="str">
+        <v>3</v>
+      </c>
+      <c r="H64" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>2025-11-15</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Marie Vettrino</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Available</v>
+      </c>
+      <c r="D65" t="str">
+        <v>10:30-11:30; 16:45-17:45</v>
+      </c>
+      <c r="E65" t="str">
+        <v>3</v>
+      </c>
+      <c r="F65" t="str">
+        <v>3</v>
+      </c>
+      <c r="G65" t="str">
+        <v>3</v>
+      </c>
+      <c r="H65" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>2025-11-15</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Mikhaila (W) Calder</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Holiday</v>
+      </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
+      <c r="E66" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="F66" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="G66" t="str">
+        <v>0</v>
+      </c>
+      <c r="H66" t="str">
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>2025-11-15</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Morrison, Anne</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Ad-hoc</v>
+      </c>
+      <c r="D67" t="str">
+        <v>19:00-21:29</v>
+      </c>
+      <c r="E67" t="str">
+        <v>0</v>
+      </c>
+      <c r="F67" t="str">
+        <v>0</v>
+      </c>
+      <c r="G67" t="str">
+        <v>0</v>
+      </c>
+      <c r="H67" t="str">
+        <v>Scheduled (no availability record for this day)</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>2025-11-15</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Muhammad Irtaza Tahir (GH)</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Holiday</v>
+      </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
+      <c r="E68" t="str">
+        <v>4.29</v>
+      </c>
+      <c r="F68" t="str">
+        <v>4.29</v>
+      </c>
+      <c r="G68" t="str">
+        <v>0</v>
+      </c>
+      <c r="H68" t="str">
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H68"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3881,27 +4295,27 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Elizabeth Adams</v>
       </c>
       <c r="B2" t="str">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C2" t="str">
         <v>Driver</v>
       </c>
       <c r="D2" t="str">
-        <v>Miss</v>
+        <v>Mrs</v>
       </c>
       <c r="E2" t="str">
         <v>female</v>
       </c>
       <c r="F2" t="str">
-        <v xml:space="preserve">FK10 1NH  </v>
+        <v xml:space="preserve">EH21 6NQ  </v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Paul Chalmers (GH)</v>
+        <v>Victoria Bateman (GH)</v>
       </c>
       <c r="B3" t="str">
         <v>16</v>
@@ -3910,81 +4324,81 @@
         <v>Driver</v>
       </c>
       <c r="D3" t="str">
-        <v>Mr</v>
+        <v>Mrs</v>
       </c>
       <c r="E3" t="str">
-        <v>male</v>
+        <v>female</v>
       </c>
       <c r="F3" t="str">
-        <v xml:space="preserve">FK10 3HJ  </v>
+        <v xml:space="preserve">EH23 4NL  </v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>John Clarke (GH)</v>
+        <v>Amy Brown</v>
       </c>
       <c r="B4" t="str">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C4" t="str">
         <v>Driver</v>
       </c>
       <c r="D4" t="str">
-        <v>Mr</v>
+        <v>Miss</v>
       </c>
       <c r="E4" t="str">
-        <v>male</v>
+        <v>female</v>
       </c>
       <c r="F4" t="str">
-        <v xml:space="preserve">FK8 1XY   </v>
+        <v xml:space="preserve">EH21 6DQ  </v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Kristin Earhart</v>
+        <v>Mikhaila (W) Calder</v>
       </c>
       <c r="B5" t="str">
         <v>16</v>
       </c>
       <c r="C5" t="str">
-        <v>Driver</v>
+        <v>Walker</v>
       </c>
       <c r="D5" t="str">
-        <v>Mrs</v>
+        <v>Miss</v>
       </c>
       <c r="E5" t="str">
         <v>female</v>
       </c>
       <c r="F5" t="str">
-        <v xml:space="preserve">FK12 5HG  </v>
+        <v xml:space="preserve">EH17 7RT  </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>Romina Ferrara</v>
       </c>
       <c r="B6" t="str">
-        <v>46</v>
+        <v>5</v>
       </c>
       <c r="C6" t="str">
         <v>Driver</v>
       </c>
       <c r="D6" t="str">
-        <v>Mr</v>
+        <v>Miss</v>
       </c>
       <c r="E6" t="str">
-        <v>male</v>
+        <v>female</v>
       </c>
       <c r="F6" t="str">
-        <v xml:space="preserve">FK2 7ER   </v>
+        <v xml:space="preserve">EH32 9SS  </v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Jamie Lee Kane (GH)</v>
+        <v>Eilish McNally</v>
       </c>
       <c r="B7" t="str">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C7" t="str">
         <v>Driver</v>
@@ -3996,55 +4410,55 @@
         <v>female</v>
       </c>
       <c r="F7" t="str">
-        <v xml:space="preserve">FK7 7PN   </v>
+        <v xml:space="preserve">EH34 5HE  </v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Clare Mackie</v>
+        <v>Dhaval Mithaiwala</v>
       </c>
       <c r="B8" t="str">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="C8" t="str">
         <v>Driver</v>
       </c>
       <c r="D8" t="str">
-        <v>Miss</v>
+        <v>Mr</v>
       </c>
       <c r="E8" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="F8" t="str">
-        <v xml:space="preserve">FK2 8FD   </v>
+        <v xml:space="preserve">EH11 3JF  </v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Anisa Naeem</v>
+        <v>Anne Morrison</v>
       </c>
       <c r="B9" t="str">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C9" t="str">
         <v>Driver</v>
       </c>
       <c r="D9" t="str">
-        <v>Miss</v>
+        <v>Mrs</v>
       </c>
       <c r="E9" t="str">
         <v>female</v>
       </c>
       <c r="F9" t="str">
-        <v xml:space="preserve">FK6 5AE   </v>
+        <v xml:space="preserve">EH21 7LH  </v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Chiamaka Onweluzo (GH)</v>
+        <v>Helen Morrison (GH)</v>
       </c>
       <c r="B10" t="str">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="C10" t="str">
         <v>Driver</v>
@@ -4056,32 +4470,32 @@
         <v>female</v>
       </c>
       <c r="F10" t="str">
-        <v xml:space="preserve">FK8 1RS   </v>
+        <v xml:space="preserve">EH21 6JY  </v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Emma (NL) Shawcross</v>
+        <v>Lorraine Parsons</v>
       </c>
       <c r="B11" t="str">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C11" t="str">
-        <v>Walker</v>
+        <v>Driver</v>
       </c>
       <c r="D11" t="str">
-        <v>Miss</v>
+        <v>Mrs</v>
       </c>
       <c r="E11" t="str">
         <v>female</v>
       </c>
       <c r="F11" t="str">
-        <v xml:space="preserve">ML6 0JH   </v>
+        <v xml:space="preserve">EH22 4FP  </v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Alison Shields (GH)</v>
+        <v>Muhammad Irtaza Tahir (GH)</v>
       </c>
       <c r="B12" t="str">
         <v>30</v>
@@ -4090,21 +4504,21 @@
         <v>Driver</v>
       </c>
       <c r="D12" t="str">
-        <v>Ms</v>
+        <v>Mr</v>
       </c>
       <c r="E12" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="F12" t="str">
-        <v xml:space="preserve">FK3 8LP   </v>
+        <v xml:space="preserve">EH8 7AD   </v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Barbora Slabochova (GH)</v>
+        <v>Marie Vettrino</v>
       </c>
       <c r="B13" t="str">
-        <v>37.5</v>
+        <v>15</v>
       </c>
       <c r="C13" t="str">
         <v>Driver</v>
@@ -4116,52 +4530,12 @@
         <v>female</v>
       </c>
       <c r="F13" t="str">
-        <v xml:space="preserve">FK8 2BQ   </v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Rhian Steel</v>
-      </c>
-      <c r="B14" t="str">
-        <v>20</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Driver</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Miss</v>
-      </c>
-      <c r="E14" t="str">
-        <v>female</v>
-      </c>
-      <c r="F14" t="str">
-        <v xml:space="preserve">FK10 2SR  </v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Ziyal Vidler</v>
-      </c>
-      <c r="B15" t="str">
-        <v>20</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Driver</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Miss</v>
-      </c>
-      <c r="E15" t="str">
-        <v>female</v>
-      </c>
-      <c r="F15" t="str">
-        <v xml:space="preserve">FK5 4XD   </v>
+        <v xml:space="preserve">EH32 0DG  </v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update dashboard to correctly exclude office hours and night visits
Added new image file `attached_assets/image_1762873766237.png` and updated `capacity_dashboard.xlsx`.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -406,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J54"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,16 +442,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Marie Vettrino</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="B2" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E2" t="str">
         <v>Holiday</v>
@@ -460,7 +460,7 @@
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H2" t="str">
         <v>0</v>
@@ -469,21 +469,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J2" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">FK7 7PN   </v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="B3" t="str">
         <v>16</v>
       </c>
       <c r="C3" t="str">
-        <v>2.29</v>
+        <v>4</v>
       </c>
       <c r="D3" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E3" t="str">
         <v>Holiday</v>
@@ -492,7 +492,7 @@
         <v/>
       </c>
       <c r="G3" t="str">
-        <v>2.29</v>
+        <v>4</v>
       </c>
       <c r="H3" t="str">
         <v>0</v>
@@ -501,21 +501,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J3" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK7 7PN   </v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="B4" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C4" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="D4" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E4" t="str">
         <v>Holiday</v>
@@ -524,7 +524,7 @@
         <v/>
       </c>
       <c r="G4" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="H4" t="str">
         <v>0</v>
@@ -533,21 +533,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J4" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK8 1XY   </v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="B5" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C5" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="D5" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E5" t="str">
         <v>Holiday</v>
@@ -556,7 +556,7 @@
         <v/>
       </c>
       <c r="G5" t="str">
-        <v>2.29</v>
+        <v>7.5</v>
       </c>
       <c r="H5" t="str">
         <v>0</v>
@@ -565,21 +565,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J5" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK8 1XY   </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="B6" t="str">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="C6" t="str">
-        <v>2.29</v>
+        <v>9.2</v>
       </c>
       <c r="D6" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E6" t="str">
         <v>Holiday</v>
@@ -588,7 +588,7 @@
         <v/>
       </c>
       <c r="G6" t="str">
-        <v>2.29</v>
+        <v>9.2</v>
       </c>
       <c r="H6" t="str">
         <v>0</v>
@@ -597,21 +597,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J6" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK8 1RS   </v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="B7" t="str">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="C7" t="str">
-        <v>2.29</v>
+        <v>9.2</v>
       </c>
       <c r="D7" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E7" t="str">
         <v>Holiday</v>
@@ -620,7 +620,7 @@
         <v/>
       </c>
       <c r="G7" t="str">
-        <v>2.29</v>
+        <v>9.2</v>
       </c>
       <c r="H7" t="str">
         <v>0</v>
@@ -629,21 +629,21 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J7" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK8 1RS   </v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="B8" t="str">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="C8" t="str">
-        <v>2.29</v>
+        <v>9.2</v>
       </c>
       <c r="D8" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E8" t="str">
         <v>Holiday</v>
@@ -652,7 +652,7 @@
         <v/>
       </c>
       <c r="G8" t="str">
-        <v>2.29</v>
+        <v>9.2</v>
       </c>
       <c r="H8" t="str">
         <v>0</v>
@@ -661,434 +661,434 @@
         <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
       <c r="J8" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK8 1RS   </v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="B9" t="str">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="C9" t="str">
-        <v>2.29</v>
+        <v>9.2</v>
       </c>
       <c r="D9" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E9" t="str">
-        <v>Holiday</v>
+        <v>Partial Availability</v>
       </c>
       <c r="F9" t="str">
-        <v/>
+        <v>08:00-13:00; 17:00-22:00</v>
       </c>
       <c r="G9" t="str">
-        <v>2.29</v>
+        <v>5.2</v>
       </c>
       <c r="H9" t="str">
-        <v>0</v>
+        <v>5.2</v>
       </c>
       <c r="I9" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v>Haseeb is helping out GN</v>
       </c>
       <c r="J9" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK2 7ER   </v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="B10" t="str">
         <v>30</v>
       </c>
       <c r="C10" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="D10" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E10" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="F10" t="str">
-        <v/>
+        <v>15:30-21:30</v>
       </c>
       <c r="G10" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="H10" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="I10" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
       <c r="J10" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK6 5AE   </v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="B11" t="str">
         <v>30</v>
       </c>
       <c r="C11" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="D11" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E11" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="F11" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G11" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="H11" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="I11" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
       <c r="J11" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK6 5AE   </v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="B12" t="str">
         <v>30</v>
       </c>
       <c r="C12" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="D12" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E12" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="F12" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G12" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="H12" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="I12" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
       <c r="J12" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK6 5AE   </v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="B13" t="str">
         <v>30</v>
       </c>
       <c r="C13" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="D13" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E13" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="F13" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G13" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="H13" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="I13" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
       <c r="J13" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK6 5AE   </v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="B14" t="str">
-        <v>30</v>
+        <v>37.5</v>
       </c>
       <c r="C14" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="D14" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E14" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="F14" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G14" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="H14" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="I14" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v>Created by new employee process.</v>
       </c>
       <c r="J14" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK8 2BQ   </v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="B15" t="str">
-        <v>30</v>
+        <v>37.5</v>
       </c>
       <c r="C15" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="D15" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E15" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="F15" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G15" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="H15" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="I15" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v>Created by new employee process.</v>
       </c>
       <c r="J15" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK8 2BQ   </v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="B16" t="str">
-        <v>30</v>
+        <v>37.5</v>
       </c>
       <c r="C16" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="D16" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E16" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="F16" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G16" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="H16" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="I16" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v>Created by new employee process.</v>
       </c>
       <c r="J16" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK8 2BQ   </v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="B17" t="str">
-        <v>10</v>
+        <v>37.5</v>
       </c>
       <c r="C17" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="D17" t="str">
         <v>2025-11-14</v>
       </c>
       <c r="E17" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="F17" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="G17" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="H17" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="I17" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v>Created by new employee process.</v>
       </c>
       <c r="J17" t="str">
-        <v xml:space="preserve">EH22 4FP  </v>
+        <v xml:space="preserve">FK8 2BQ   </v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Eilish McNally</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="B18" t="str">
-        <v>12</v>
+        <v>37.5</v>
       </c>
       <c r="C18" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="D18" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E18" t="str">
         <v>Available</v>
       </c>
       <c r="F18" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G18" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H18" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="I18" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
       <c r="J18" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">FK8 2BQ   </v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Eilish McNally</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="B19" t="str">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C19" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D19" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E19" t="str">
         <v>Available</v>
       </c>
       <c r="F19" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G19" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H19" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I19" t="str">
-        <v>Eilish emailed that she is traveling to Glasgow for her SVQ training (MU 04.11.25)</v>
+        <v/>
       </c>
       <c r="J19" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">FK7 7PN   </v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Eilish McNally</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="B20" t="str">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C20" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D20" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E20" t="str">
         <v>Available</v>
       </c>
       <c r="F20" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="G20" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H20" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I20" t="str">
         <v/>
       </c>
       <c r="J20" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">FK7 7PN   </v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Eilish McNally</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="B21" t="str">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C21" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D21" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E21" t="str">
         <v>Available</v>
       </c>
       <c r="F21" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G21" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H21" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I21" t="str">
         <v/>
       </c>
       <c r="J21" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">FK10 2SR  </v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Marie Vettrino</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="B22" t="str">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C22" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D22" t="str">
         <v>2025-11-11</v>
@@ -1097,321 +1097,321 @@
         <v>Available</v>
       </c>
       <c r="F22" t="str">
-        <v>09:30-12:30; 18:30-21:30</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="G22" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H22" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I22" t="str">
         <v/>
       </c>
       <c r="J22" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">FK10 2SR  </v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Marie Vettrino</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="B23" t="str">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C23" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D23" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E23" t="str">
         <v>Available</v>
       </c>
       <c r="F23" t="str">
-        <v>10:30-12:30; 18:30-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G23" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H23" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I23" t="str">
         <v/>
       </c>
       <c r="J23" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">FK10 2SR  </v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Marie Vettrino</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="B24" t="str">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C24" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D24" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E24" t="str">
         <v>Available</v>
       </c>
       <c r="F24" t="str">
-        <v>09:30-12:30; 18:30-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G24" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H24" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I24" t="str">
         <v/>
       </c>
       <c r="J24" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">FK10 2SR  </v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Marie Vettrino</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="B25" t="str">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="C25" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D25" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E25" t="str">
         <v>Available</v>
       </c>
       <c r="F25" t="str">
-        <v>10:30-11:30; 16:45-17:45</v>
+        <v>08:15-21:30</v>
       </c>
       <c r="G25" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H25" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I25" t="str">
         <v/>
       </c>
       <c r="J25" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">FK10 1NH  </v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Romina Ferrara</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="B26" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C26" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D26" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E26" t="str">
         <v>Available</v>
       </c>
       <c r="F26" t="str">
-        <v>09:15-10:15</v>
+        <v>08:15-21:30</v>
       </c>
       <c r="G26" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H26" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I26" t="str">
         <v/>
       </c>
       <c r="J26" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">FK10 1NH  </v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Romina Ferrara</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="B27" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C27" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D27" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E27" t="str">
         <v>Available</v>
       </c>
       <c r="F27" t="str">
-        <v>09:15-10:15</v>
+        <v>08:15-17:15</v>
       </c>
       <c r="G27" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H27" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I27" t="str">
         <v/>
       </c>
       <c r="J27" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">FK10 1NH  </v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Romina Ferrara</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="B28" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C28" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D28" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E28" t="str">
         <v>Available</v>
       </c>
       <c r="F28" t="str">
-        <v>09:15-10:15</v>
+        <v>08:15-17:15</v>
       </c>
       <c r="G28" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H28" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I28" t="str">
         <v/>
       </c>
       <c r="J28" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">FK10 1NH  </v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Romina Ferrara</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="B29" t="str">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="C29" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D29" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E29" t="str">
         <v>Available</v>
       </c>
       <c r="F29" t="str">
-        <v>09:15-10:15</v>
+        <v>08:15-17:15</v>
       </c>
       <c r="G29" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H29" t="str">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I29" t="str">
         <v/>
       </c>
       <c r="J29" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">FK10 1NH  </v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Romina Ferrara</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="B30" t="str">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C30" t="str">
-        <v>1</v>
+        <v>6.67</v>
       </c>
       <c r="D30" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E30" t="str">
         <v>Available</v>
       </c>
       <c r="F30" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G30" t="str">
-        <v>1</v>
+        <v>6.67</v>
       </c>
       <c r="H30" t="str">
-        <v>1</v>
+        <v>6.67</v>
       </c>
       <c r="I30" t="str">
         <v/>
       </c>
       <c r="J30" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">FK5 4XD   </v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="B31" t="str">
         <v>20</v>
       </c>
       <c r="C31" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="D31" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E31" t="str">
         <v>Available</v>
       </c>
       <c r="F31" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-14:00</v>
       </c>
       <c r="G31" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="H31" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="I31" t="str">
         <v/>
       </c>
       <c r="J31" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK5 4XD   </v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="B32" t="str">
         <v>20</v>
       </c>
       <c r="C32" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="D32" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E32" t="str">
         <v>Available</v>
@@ -1420,158 +1420,158 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G32" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="H32" t="str">
-        <v>2.86</v>
+        <v>6.67</v>
       </c>
       <c r="I32" t="str">
         <v/>
       </c>
       <c r="J32" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK5 4XD   </v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="B33" t="str">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C33" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="D33" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E33" t="str">
         <v>Available</v>
       </c>
       <c r="F33" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="G33" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="H33" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="I33" t="str">
         <v/>
       </c>
       <c r="J33" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK2 7ER   </v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="B34" t="str">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C34" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="D34" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E34" t="str">
         <v>Available</v>
       </c>
       <c r="F34" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="G34" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="H34" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="I34" t="str">
         <v/>
       </c>
       <c r="J34" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK2 7ER   </v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="B35" t="str">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C35" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="D35" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E35" t="str">
         <v>Available</v>
       </c>
       <c r="F35" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="G35" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="H35" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="I35" t="str">
         <v/>
       </c>
       <c r="J35" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK2 7ER   </v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="B36" t="str">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C36" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="D36" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E36" t="str">
         <v>Available</v>
       </c>
       <c r="F36" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="G36" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="H36" t="str">
-        <v>2.86</v>
+        <v>9.2</v>
       </c>
       <c r="I36" t="str">
         <v/>
       </c>
       <c r="J36" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK2 7ER   </v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="B37" t="str">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C37" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="D37" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E37" t="str">
         <v>Available</v>
@@ -1580,187 +1580,187 @@
         <v>08:00-21:30</v>
       </c>
       <c r="G37" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H37" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="I37" t="str">
         <v/>
       </c>
       <c r="J37" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK8 1XY   </v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Anne Morrison</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="B38" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C38" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="D38" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E38" t="str">
         <v>Available</v>
       </c>
       <c r="F38" t="str">
-        <v>12:00-21:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G38" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="H38" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="I38" t="str">
         <v/>
       </c>
       <c r="J38" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK8 1XY   </v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Anne Morrison</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="B39" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C39" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="D39" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E39" t="str">
         <v>Available</v>
       </c>
       <c r="F39" t="str">
-        <v>12:00-21:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G39" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="H39" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="I39" t="str">
         <v/>
       </c>
       <c r="J39" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK10 3HJ  </v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Anne Morrison</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="B40" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C40" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="D40" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E40" t="str">
         <v>Available</v>
       </c>
       <c r="F40" t="str">
-        <v>09:15-21:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G40" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="H40" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="I40" t="str">
         <v/>
       </c>
       <c r="J40" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK10 3HJ  </v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Anne Morrison</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="B41" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C41" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="D41" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E41" t="str">
         <v>Available</v>
       </c>
       <c r="F41" t="str">
-        <v>09:15-21:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G41" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="H41" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="I41" t="str">
         <v/>
       </c>
       <c r="J41" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK10 3HJ  </v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Anne Morrison</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="B42" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C42" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="D42" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E42" t="str">
         <v>Available</v>
       </c>
       <c r="F42" t="str">
-        <v>12:00-17:45</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G42" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="H42" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="I42" t="str">
         <v/>
       </c>
       <c r="J42" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK10 3HJ  </v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Anne Morrison</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="B43" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C43" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="D43" t="str">
         <v>2025-11-16</v>
@@ -1769,30 +1769,30 @@
         <v>Available</v>
       </c>
       <c r="F43" t="str">
-        <v>21:00-22:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="G43" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="H43" t="str">
-        <v>1.67</v>
+        <v>3.2</v>
       </c>
       <c r="I43" t="str">
         <v/>
       </c>
       <c r="J43" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK10 3HJ  </v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="B44" t="str">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="C44" t="str">
-        <v>3.33</v>
+        <v>9.2</v>
       </c>
       <c r="D44" t="str">
         <v>2025-11-10</v>
@@ -1801,30 +1801,30 @@
         <v>Available</v>
       </c>
       <c r="F44" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G44" t="str">
-        <v>3.33</v>
+        <v>9.2</v>
       </c>
       <c r="H44" t="str">
-        <v>3.33</v>
+        <v>9.2</v>
       </c>
       <c r="I44" t="str">
         <v/>
       </c>
       <c r="J44" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
+        <v xml:space="preserve">FK8 1RS   </v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="B45" t="str">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="C45" t="str">
-        <v>3.33</v>
+        <v>9.2</v>
       </c>
       <c r="D45" t="str">
         <v>2025-11-11</v>
@@ -1833,222 +1833,222 @@
         <v>Available</v>
       </c>
       <c r="F45" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G45" t="str">
-        <v>3.33</v>
+        <v>9.2</v>
       </c>
       <c r="H45" t="str">
-        <v>3.33</v>
+        <v>9.2</v>
       </c>
       <c r="I45" t="str">
         <v/>
       </c>
       <c r="J45" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
+        <v xml:space="preserve">FK8 1RS   </v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="B46" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C46" t="str">
-        <v>3.33</v>
+        <v>3.2</v>
       </c>
       <c r="D46" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E46" t="str">
         <v>Available</v>
       </c>
       <c r="F46" t="str">
-        <v>08:00-18:00</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="G46" t="str">
-        <v>3.33</v>
+        <v>3.2</v>
       </c>
       <c r="H46" t="str">
-        <v>3.33</v>
+        <v>3.2</v>
       </c>
       <c r="I46" t="str">
         <v/>
       </c>
       <c r="J46" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
+        <v xml:space="preserve">FK12 5HG  </v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="B47" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C47" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="D47" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="E47" t="str">
         <v>Available</v>
       </c>
       <c r="F47" t="str">
-        <v>08:00-16:30</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="G47" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H47" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="I47" t="str">
         <v/>
       </c>
       <c r="J47" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
+        <v xml:space="preserve">FK12 5HG  </v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="B48" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C48" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="D48" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-12</v>
       </c>
       <c r="E48" t="str">
         <v>Available</v>
       </c>
       <c r="F48" t="str">
-        <v>08:00-16:00</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="G48" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H48" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="I48" t="str">
         <v/>
       </c>
       <c r="J48" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
+        <v xml:space="preserve">FK12 5HG  </v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="B49" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C49" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="D49" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-13</v>
       </c>
       <c r="E49" t="str">
         <v>Available</v>
       </c>
       <c r="F49" t="str">
-        <v>08:00-16:00</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="G49" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H49" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="I49" t="str">
         <v/>
       </c>
       <c r="J49" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
+        <v xml:space="preserve">FK12 5HG  </v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="B50" t="str">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C50" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="D50" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-14</v>
       </c>
       <c r="E50" t="str">
         <v>Available</v>
       </c>
       <c r="F50" t="str">
-        <v>08:00-16:00</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="G50" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H50" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="I50" t="str">
         <v/>
       </c>
       <c r="J50" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
+        <v xml:space="preserve">FK12 5HG  </v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="B51" t="str">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="C51" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="D51" t="str">
-        <v>2025-11-15</v>
+        <v>2025-11-10</v>
       </c>
       <c r="E51" t="str">
         <v>Available</v>
       </c>
       <c r="F51" t="str">
-        <v>08:00-16:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G51" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H51" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="I51" t="str">
         <v/>
       </c>
       <c r="J51" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
+        <v xml:space="preserve">FK3 8LP   </v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="B52" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C52" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="D52" t="str">
         <v>2025-11-11</v>
@@ -2057,216 +2057,88 @@
         <v>Available</v>
       </c>
       <c r="F52" t="str">
-        <v>09:30-14:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G52" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="H52" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="I52" t="str">
         <v/>
       </c>
       <c r="J52" t="str">
-        <v xml:space="preserve">EH22 4FP  </v>
+        <v xml:space="preserve">FK3 8LP   </v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="B53" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C53" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="D53" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-15</v>
       </c>
       <c r="E53" t="str">
         <v>Available</v>
       </c>
       <c r="F53" t="str">
-        <v>09:30-14:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G53" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="H53" t="str">
-        <v>3.33</v>
+        <v>7.5</v>
       </c>
       <c r="I53" t="str">
         <v/>
       </c>
       <c r="J53" t="str">
-        <v xml:space="preserve">EH22 4FP  </v>
+        <v xml:space="preserve">FK3 8LP   </v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="B54" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C54" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="D54" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-16</v>
       </c>
       <c r="E54" t="str">
         <v>Available</v>
       </c>
       <c r="F54" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="G54" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H54" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="I54" t="str">
         <v/>
       </c>
       <c r="J54" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="B55" t="str">
-        <v>16</v>
-      </c>
-      <c r="C55" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D55" t="str">
-        <v>2025-11-11</v>
-      </c>
-      <c r="E55" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F55" t="str">
-        <v>08:00-15:30</v>
-      </c>
-      <c r="G55" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H55" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I55" t="str">
-        <v/>
-      </c>
-      <c r="J55" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="B56" t="str">
-        <v>16</v>
-      </c>
-      <c r="C56" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D56" t="str">
-        <v>2025-11-12</v>
-      </c>
-      <c r="E56" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F56" t="str">
-        <v>08:00-15:30</v>
-      </c>
-      <c r="G56" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H56" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I56" t="str">
-        <v/>
-      </c>
-      <c r="J56" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="B57" t="str">
-        <v>16</v>
-      </c>
-      <c r="C57" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D57" t="str">
-        <v>2025-11-13</v>
-      </c>
-      <c r="E57" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F57" t="str">
-        <v>08:00-17:30</v>
-      </c>
-      <c r="G57" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H57" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I57" t="str">
-        <v/>
-      </c>
-      <c r="J57" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="B58" t="str">
-        <v>16</v>
-      </c>
-      <c r="C58" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="D58" t="str">
-        <v>2025-11-14</v>
-      </c>
-      <c r="E58" t="str">
-        <v>Available</v>
-      </c>
-      <c r="F58" t="str">
-        <v>08:00-15:30</v>
-      </c>
-      <c r="G58" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H58" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="I58" t="str">
-        <v/>
-      </c>
-      <c r="J58" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
+        <v xml:space="preserve">FK3 8LP   </v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J54"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2306,22 +2178,22 @@
         <v>2025-11-10</v>
       </c>
       <c r="B2" t="str">
-        <v>18.06</v>
+        <v>34.1</v>
       </c>
       <c r="C2" t="str">
-        <v>18.06</v>
+        <v>39.3</v>
       </c>
       <c r="D2" t="str">
-        <v>0</v>
+        <v>5.2</v>
       </c>
       <c r="E2" t="str">
-        <v>6.58</v>
+        <v>7.5</v>
       </c>
       <c r="F2" t="str">
-        <v>25.5</v>
+        <v>58</v>
       </c>
       <c r="G2" t="str">
-        <v>-7.44</v>
+        <v>-18.7</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -2332,22 +2204,22 @@
         <v>2025-11-11</v>
       </c>
       <c r="B3" t="str">
-        <v>24.39</v>
+        <v>58.3</v>
       </c>
       <c r="C3" t="str">
-        <v>24.39</v>
+        <v>58.3</v>
       </c>
       <c r="D3" t="str">
         <v>0</v>
       </c>
       <c r="E3" t="str">
-        <v>6.58</v>
+        <v>11.5</v>
       </c>
       <c r="F3" t="str">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="G3" t="str">
-        <v>-3.61</v>
+        <v>-3.7</v>
       </c>
       <c r="H3" t="str">
         <v>Shortage</v>
@@ -2358,22 +2230,22 @@
         <v>2025-11-12</v>
       </c>
       <c r="B4" t="str">
-        <v>21.06</v>
+        <v>40.6</v>
       </c>
       <c r="C4" t="str">
-        <v>21.06</v>
+        <v>40.6</v>
       </c>
       <c r="D4" t="str">
         <v>0</v>
       </c>
       <c r="E4" t="str">
-        <v>6.58</v>
+        <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>24.5</v>
+        <v>66</v>
       </c>
       <c r="G4" t="str">
-        <v>-3.44</v>
+        <v>-25.4</v>
       </c>
       <c r="H4" t="str">
         <v>Shortage</v>
@@ -2384,22 +2256,22 @@
         <v>2025-11-13</v>
       </c>
       <c r="B5" t="str">
-        <v>21.06</v>
+        <v>43.27</v>
       </c>
       <c r="C5" t="str">
-        <v>21.06</v>
+        <v>43.27</v>
       </c>
       <c r="D5" t="str">
         <v>0</v>
       </c>
       <c r="E5" t="str">
-        <v>6.58</v>
+        <v>4</v>
       </c>
       <c r="F5" t="str">
-        <v>26</v>
+        <v>52</v>
       </c>
       <c r="G5" t="str">
-        <v>-4.94</v>
+        <v>-8.73</v>
       </c>
       <c r="H5" t="str">
         <v>Shortage</v>
@@ -2410,22 +2282,22 @@
         <v>2025-11-14</v>
       </c>
       <c r="B6" t="str">
-        <v>8.73</v>
+        <v>44.07</v>
       </c>
       <c r="C6" t="str">
-        <v>8.73</v>
+        <v>44.07</v>
       </c>
       <c r="D6" t="str">
         <v>0</v>
       </c>
       <c r="E6" t="str">
-        <v>9.91</v>
+        <v>9.2</v>
       </c>
       <c r="F6" t="str">
-        <v>21.5</v>
+        <v>58</v>
       </c>
       <c r="G6" t="str">
-        <v>-12.77</v>
+        <v>-13.93</v>
       </c>
       <c r="H6" t="str">
         <v>Shortage</v>
@@ -2436,22 +2308,22 @@
         <v>2025-11-15</v>
       </c>
       <c r="B7" t="str">
-        <v>8.86</v>
+        <v>27.5</v>
       </c>
       <c r="C7" t="str">
-        <v>8.86</v>
+        <v>27.5</v>
       </c>
       <c r="D7" t="str">
         <v>0</v>
       </c>
       <c r="E7" t="str">
-        <v>6.58</v>
+        <v>9.2</v>
       </c>
       <c r="F7" t="str">
-        <v>16.5</v>
+        <v>49</v>
       </c>
       <c r="G7" t="str">
-        <v>-7.64</v>
+        <v>-21.5</v>
       </c>
       <c r="H7" t="str">
         <v>Shortage</v>
@@ -2462,22 +2334,22 @@
         <v>2025-11-16</v>
       </c>
       <c r="B8" t="str">
-        <v>4.53</v>
+        <v>29.87</v>
       </c>
       <c r="C8" t="str">
-        <v>4.53</v>
+        <v>29.87</v>
       </c>
       <c r="D8" t="str">
         <v>0</v>
       </c>
       <c r="E8" t="str">
-        <v>8.58</v>
+        <v>9.2</v>
       </c>
       <c r="F8" t="str">
-        <v>12.5</v>
+        <v>48</v>
       </c>
       <c r="G8" t="str">
-        <v>-7.97</v>
+        <v>-18.13</v>
       </c>
       <c r="H8" t="str">
         <v>Shortage</v>
@@ -2492,7 +2364,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H57"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2522,25 +2394,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B2" t="str">
-        <v>Anne Morrison</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="C2" t="str">
         <v>Available</v>
       </c>
       <c r="D2" t="str">
-        <v>21:00-22:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E2" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="F2" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="G2" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="H2" t="str">
         <v/>
@@ -2548,25 +2420,25 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B3" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="C3" t="str">
         <v>Available</v>
       </c>
       <c r="D3" t="str">
-        <v>08:00-21:30</v>
+        <v>15:30-21:30</v>
       </c>
       <c r="E3" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="F3" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="G3" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -2574,88 +2446,88 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B4" t="str">
-        <v>Marie Vettrino</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="C4" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D4" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E4" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="F4" t="str">
-        <v>2</v>
+        <v>7.5</v>
       </c>
       <c r="G4" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H4" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v>Created by new employee process.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B5" t="str">
-        <v>McNally, Eilish</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="C5" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D5" t="str">
-        <v>19:00-21:29</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E5" t="str">
-        <v>0</v>
+        <v>9.2</v>
       </c>
       <c r="F5" t="str">
-        <v>0</v>
+        <v>9.2</v>
       </c>
       <c r="G5" t="str">
-        <v>0</v>
+        <v>9.2</v>
       </c>
       <c r="H5" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B6" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="C6" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D6" t="str">
-        <v/>
+        <v>08:00-22:00</v>
       </c>
       <c r="E6" t="str">
-        <v>2.29</v>
+        <v>9.2</v>
       </c>
       <c r="F6" t="str">
-        <v>2.29</v>
+        <v>9.2</v>
       </c>
       <c r="G6" t="str">
-        <v>0</v>
+        <v>9.2</v>
       </c>
       <c r="H6" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2025-11-16</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B7" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="C7" t="str">
         <v>Holiday</v>
@@ -2664,10 +2536,10 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>4.29</v>
+        <v>4</v>
       </c>
       <c r="F7" t="str">
-        <v>4.29</v>
+        <v>4</v>
       </c>
       <c r="G7" t="str">
         <v>0</v>
@@ -2678,51 +2550,51 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B8" t="str">
-        <v>Anne Morrison</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="C8" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D8" t="str">
-        <v>12:00-21:00</v>
+        <v/>
       </c>
       <c r="E8" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="F8" t="str">
-        <v>1.67</v>
+        <v>7.5</v>
       </c>
       <c r="G8" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="H8" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B9" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="C9" t="str">
         <v>Available</v>
       </c>
       <c r="D9" t="str">
-        <v>08:00-21:30</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="E9" t="str">
-        <v>2.86</v>
+        <v>3.2</v>
       </c>
       <c r="F9" t="str">
-        <v>2.86</v>
+        <v>3.2</v>
       </c>
       <c r="G9" t="str">
-        <v>2.86</v>
+        <v>3.2</v>
       </c>
       <c r="H9" t="str">
         <v/>
@@ -2730,25 +2602,25 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B10" t="str">
-        <v>Eilish McNally</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="C10" t="str">
         <v>Available</v>
       </c>
       <c r="D10" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E10" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="F10" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="G10" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H10" t="str">
         <v/>
@@ -2756,25 +2628,25 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B11" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="C11" t="str">
         <v>Available</v>
       </c>
       <c r="D11" t="str">
-        <v>08:00-18:00</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E11" t="str">
-        <v>3.33</v>
+        <v>5</v>
       </c>
       <c r="F11" t="str">
-        <v>3.33</v>
+        <v>5</v>
       </c>
       <c r="G11" t="str">
-        <v>3.33</v>
+        <v>5</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -2782,25 +2654,25 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B12" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="C12" t="str">
         <v>Available</v>
       </c>
       <c r="D12" t="str">
-        <v>08:00-16:30</v>
+        <v>08:15-21:30</v>
       </c>
       <c r="E12" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F12" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G12" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H12" t="str">
         <v/>
@@ -2808,103 +2680,103 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-11</v>
       </c>
       <c r="B13" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Vidler, Ziyal</v>
       </c>
       <c r="C13" t="str">
-        <v>Holiday</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D13" t="str">
-        <v/>
+        <v>12:29-13:00</v>
       </c>
       <c r="E13" t="str">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="F13" t="str">
-        <v>2.29</v>
+        <v>0</v>
       </c>
       <c r="G13" t="str">
         <v>0</v>
       </c>
       <c r="H13" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B14" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="C14" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D14" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E14" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="F14" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="G14" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H14" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B15" t="str">
-        <v>Romina Ferrara</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="C15" t="str">
         <v>Available</v>
       </c>
       <c r="D15" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E15" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="F15" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="G15" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="H15" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B16" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="C16" t="str">
         <v>Available</v>
       </c>
       <c r="D16" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="E16" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="F16" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="G16" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="H16" t="str">
         <v/>
@@ -2912,77 +2784,77 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B17" t="str">
-        <v>Anne Morrison</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="C17" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D17" t="str">
-        <v>12:00-21:00</v>
+        <v/>
       </c>
       <c r="E17" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="F17" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="G17" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="H17" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B18" t="str">
-        <v>Dale (GH), Heather</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="C18" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D18" t="str">
-        <v>09:22-11:53</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="E18" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="F18" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="G18" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H18" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B19" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="C19" t="str">
         <v>Available</v>
       </c>
       <c r="D19" t="str">
-        <v>08:00-21:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E19" t="str">
-        <v>2.86</v>
+        <v>3.2</v>
       </c>
       <c r="F19" t="str">
-        <v>2.86</v>
+        <v>3.2</v>
       </c>
       <c r="G19" t="str">
-        <v>2.86</v>
+        <v>3.2</v>
       </c>
       <c r="H19" t="str">
         <v/>
@@ -2990,51 +2862,51 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B20" t="str">
-        <v>Eilish McNally</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="C20" t="str">
         <v>Available</v>
       </c>
       <c r="D20" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:15-17:15</v>
       </c>
       <c r="E20" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F20" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G20" t="str">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H20" t="str">
-        <v>Eilish emailed that she is traveling to Glasgow for her SVQ training (MU 04.11.25)</v>
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B21" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="C21" t="str">
         <v>Available</v>
       </c>
       <c r="D21" t="str">
-        <v>08:00-18:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E21" t="str">
-        <v>3.33</v>
+        <v>6.67</v>
       </c>
       <c r="F21" t="str">
-        <v>3.33</v>
+        <v>6.67</v>
       </c>
       <c r="G21" t="str">
-        <v>3.33</v>
+        <v>6.67</v>
       </c>
       <c r="H21" t="str">
         <v/>
@@ -3042,51 +2914,51 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B22" t="str">
-        <v>Hartley-Oliver (GH), Ruby</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="C22" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D22" t="str">
-        <v>13:59-16:59</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E22" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F22" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="G22" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H22" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B23" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="C23" t="str">
         <v>Available</v>
       </c>
       <c r="D23" t="str">
-        <v>08:00-16:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E23" t="str">
-        <v>3</v>
+        <v>9.2</v>
       </c>
       <c r="F23" t="str">
-        <v>3</v>
+        <v>9.2</v>
       </c>
       <c r="G23" t="str">
-        <v>3</v>
+        <v>9.2</v>
       </c>
       <c r="H23" t="str">
         <v/>
@@ -3094,129 +2966,129 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B24" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="C24" t="str">
-        <v>Available</v>
+        <v>Partial Availability</v>
       </c>
       <c r="D24" t="str">
-        <v>09:30-14:30</v>
+        <v>08:00-13:00; 17:00-22:00</v>
       </c>
       <c r="E24" t="str">
-        <v>3.33</v>
+        <v>9.2</v>
       </c>
       <c r="F24" t="str">
-        <v>3.33</v>
+        <v>5.2</v>
       </c>
       <c r="G24" t="str">
-        <v>3.33</v>
+        <v>5.2</v>
       </c>
       <c r="H24" t="str">
-        <v/>
+        <v>Haseeb is helping out GN</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B25" t="str">
-        <v>Marie Vettrino</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="C25" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D25" t="str">
-        <v>09:30-12:30; 18:30-21:30</v>
+        <v/>
       </c>
       <c r="E25" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="F25" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="G25" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H25" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B26" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="C26" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D26" t="str">
-        <v/>
+        <v>10:00-14:30</v>
       </c>
       <c r="E26" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="F26" t="str">
-        <v>2.29</v>
+        <v>3.2</v>
       </c>
       <c r="G26" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H26" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B27" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="C27" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D27" t="str">
-        <v/>
+        <v>09:15-15:15</v>
       </c>
       <c r="E27" t="str">
-        <v>4.29</v>
+        <v>3.2</v>
       </c>
       <c r="F27" t="str">
-        <v>4.29</v>
+        <v>3.2</v>
       </c>
       <c r="G27" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H27" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B28" t="str">
-        <v>Romina Ferrara</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="C28" t="str">
         <v>Available</v>
       </c>
       <c r="D28" t="str">
-        <v>09:15-10:15</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E28" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F28" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G28" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -3224,25 +3096,25 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B29" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="C29" t="str">
         <v>Available</v>
       </c>
       <c r="D29" t="str">
-        <v>08:00-15:30</v>
+        <v>08:15-21:30</v>
       </c>
       <c r="E29" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="F29" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="G29" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -3250,62 +3122,62 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B30" t="str">
-        <v>Anne Morrison</v>
+        <v>Stevenson (GH), Keri</v>
       </c>
       <c r="C30" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D30" t="str">
-        <v>09:15-21:00</v>
+        <v>09:15-12:15</v>
       </c>
       <c r="E30" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="F30" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="G30" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="H30" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B31" t="str">
-        <v>Dale (GH), Heather</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="C31" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D31" t="str">
-        <v>09:29-13:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E31" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F31" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="G31" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H31" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B32" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="C32" t="str">
         <v>Available</v>
@@ -3314,65 +3186,65 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E32" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="F32" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="G32" t="str">
-        <v>2.86</v>
+        <v>7.5</v>
       </c>
       <c r="H32" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B33" t="str">
-        <v>Eilish McNally</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="C33" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D33" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v/>
       </c>
       <c r="E33" t="str">
-        <v>3</v>
+        <v>9.2</v>
       </c>
       <c r="F33" t="str">
-        <v>3</v>
+        <v>9.2</v>
       </c>
       <c r="G33" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H33" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B34" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="C34" t="str">
         <v>Available</v>
       </c>
       <c r="D34" t="str">
-        <v>08:00-16:00</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="E34" t="str">
-        <v>3</v>
+        <v>9.2</v>
       </c>
       <c r="F34" t="str">
-        <v>3</v>
+        <v>9.2</v>
       </c>
       <c r="G34" t="str">
-        <v>3</v>
+        <v>9.2</v>
       </c>
       <c r="H34" t="str">
         <v/>
@@ -3380,25 +3252,25 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B35" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="C35" t="str">
         <v>Available</v>
       </c>
       <c r="D35" t="str">
-        <v>09:30-14:30</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E35" t="str">
-        <v>3.33</v>
+        <v>4</v>
       </c>
       <c r="F35" t="str">
-        <v>3.33</v>
+        <v>4</v>
       </c>
       <c r="G35" t="str">
-        <v>3.33</v>
+        <v>4</v>
       </c>
       <c r="H35" t="str">
         <v/>
@@ -3406,25 +3278,25 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B36" t="str">
-        <v>Marie Vettrino</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="C36" t="str">
         <v>Available</v>
       </c>
       <c r="D36" t="str">
-        <v>10:30-12:30; 18:30-21:30</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="E36" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="F36" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="G36" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H36" t="str">
         <v/>
@@ -3432,77 +3304,77 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B37" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="C37" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D37" t="str">
-        <v/>
+        <v>08:15-17:15</v>
       </c>
       <c r="E37" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="F37" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="G37" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H37" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B38" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="C38" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D38" t="str">
-        <v/>
+        <v>08:00-14:00</v>
       </c>
       <c r="E38" t="str">
-        <v>4.29</v>
+        <v>6.67</v>
       </c>
       <c r="F38" t="str">
-        <v>4.29</v>
+        <v>6.67</v>
       </c>
       <c r="G38" t="str">
-        <v>0</v>
+        <v>6.67</v>
       </c>
       <c r="H38" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-15</v>
       </c>
       <c r="B39" t="str">
-        <v>Romina Ferrara</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="C39" t="str">
         <v>Available</v>
       </c>
       <c r="D39" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E39" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="F39" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="G39" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="H39" t="str">
         <v/>
@@ -3510,88 +3382,88 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2025-11-12</v>
+        <v>2025-11-15</v>
       </c>
       <c r="B40" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="C40" t="str">
         <v>Available</v>
       </c>
       <c r="D40" t="str">
-        <v>08:00-15:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E40" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="F40" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="G40" t="str">
-        <v>3.2</v>
+        <v>7.5</v>
       </c>
       <c r="H40" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-15</v>
       </c>
       <c r="B41" t="str">
-        <v>Anne Morrison</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="C41" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D41" t="str">
-        <v>09:15-21:00</v>
+        <v/>
       </c>
       <c r="E41" t="str">
-        <v>1.67</v>
+        <v>9.2</v>
       </c>
       <c r="F41" t="str">
-        <v>1.67</v>
+        <v>9.2</v>
       </c>
       <c r="G41" t="str">
-        <v>1.67</v>
+        <v>0</v>
       </c>
       <c r="H41" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-15</v>
       </c>
       <c r="B42" t="str">
-        <v>Dale (GH), Heather</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="C42" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D42" t="str">
-        <v>09:29-12:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E42" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F42" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="G42" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H42" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-15</v>
       </c>
       <c r="B43" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="C43" t="str">
         <v>Available</v>
@@ -3600,13 +3472,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E43" t="str">
-        <v>2.86</v>
+        <v>5</v>
       </c>
       <c r="F43" t="str">
-        <v>2.86</v>
+        <v>5</v>
       </c>
       <c r="G43" t="str">
-        <v>2.86</v>
+        <v>5</v>
       </c>
       <c r="H43" t="str">
         <v/>
@@ -3614,25 +3486,25 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B44" t="str">
-        <v>Eilish McNally</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="C44" t="str">
         <v>Available</v>
       </c>
       <c r="D44" t="str">
-        <v>08:00-10:00; 19:00-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E44" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="F44" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="G44" t="str">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H44" t="str">
         <v/>
@@ -3640,77 +3512,77 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B45" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="C45" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D45" t="str">
-        <v>08:00-18:00</v>
+        <v/>
       </c>
       <c r="E45" t="str">
-        <v>3.33</v>
+        <v>9.2</v>
       </c>
       <c r="F45" t="str">
-        <v>3.33</v>
+        <v>9.2</v>
       </c>
       <c r="G45" t="str">
-        <v>3.33</v>
+        <v>0</v>
       </c>
       <c r="H45" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B46" t="str">
-        <v>Hartley-Oliver (GH), Ruby</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="C46" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D46" t="str">
-        <v>13:59-16:59</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E46" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F46" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="G46" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H46" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B47" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="C47" t="str">
         <v>Available</v>
       </c>
       <c r="D47" t="str">
-        <v>08:00-16:00</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E47" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="F47" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="G47" t="str">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H47" t="str">
         <v/>
@@ -3718,25 +3590,25 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B48" t="str">
-        <v>Marie Vettrino</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="C48" t="str">
         <v>Available</v>
       </c>
       <c r="D48" t="str">
-        <v>09:30-12:30; 18:30-21:30</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E48" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F48" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G48" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H48" t="str">
         <v/>
@@ -3744,103 +3616,103 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-16</v>
       </c>
       <c r="B49" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="C49" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D49" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E49" t="str">
-        <v>2.29</v>
+        <v>6.67</v>
       </c>
       <c r="F49" t="str">
-        <v>2.29</v>
+        <v>6.67</v>
       </c>
       <c r="G49" t="str">
-        <v>0</v>
+        <v>6.67</v>
       </c>
       <c r="H49" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B50" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="C50" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D50" t="str">
-        <v/>
+        <v>08:00-21:30</v>
       </c>
       <c r="E50" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="F50" t="str">
-        <v>4.29</v>
+        <v>7.5</v>
       </c>
       <c r="G50" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H50" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B51" t="str">
-        <v>Romina Ferrara</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="C51" t="str">
         <v>Available</v>
       </c>
       <c r="D51" t="str">
-        <v>09:15-10:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E51" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="F51" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="G51" t="str">
-        <v>1</v>
+        <v>7.5</v>
       </c>
       <c r="H51" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B52" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="C52" t="str">
         <v>Available</v>
       </c>
       <c r="D52" t="str">
-        <v>08:00-17:30</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="E52" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="F52" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="G52" t="str">
-        <v>3.2</v>
+        <v>9.2</v>
       </c>
       <c r="H52" t="str">
         <v/>
@@ -3848,25 +3720,25 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B53" t="str">
-        <v>Anne Morrison</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="C53" t="str">
         <v>Available</v>
       </c>
       <c r="D53" t="str">
-        <v>12:00-17:45</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E53" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="F53" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="G53" t="str">
-        <v>1.67</v>
+        <v>4</v>
       </c>
       <c r="H53" t="str">
         <v/>
@@ -3874,25 +3746,25 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B54" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="C54" t="str">
         <v>Available</v>
       </c>
       <c r="D54" t="str">
-        <v>08:00-21:30</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="E54" t="str">
-        <v>2.86</v>
+        <v>3.2</v>
       </c>
       <c r="F54" t="str">
-        <v>2.86</v>
+        <v>3.2</v>
       </c>
       <c r="G54" t="str">
-        <v>2.86</v>
+        <v>3.2</v>
       </c>
       <c r="H54" t="str">
         <v/>
@@ -3900,16 +3772,16 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B55" t="str">
-        <v>Hartley-Oliver (GH), Ruby</v>
+        <v>Onweluzo (GH), Chiamaka</v>
       </c>
       <c r="C55" t="str">
         <v>Ad-hoc</v>
       </c>
       <c r="D55" t="str">
-        <v>10:45-13:45</v>
+        <v>07:59-09:00; 09:29-14:30</v>
       </c>
       <c r="E55" t="str">
         <v>0</v>
@@ -3926,352 +3798,66 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B56" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="C56" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D56" t="str">
-        <v/>
+        <v>09:15-15:15</v>
       </c>
       <c r="E56" t="str">
-        <v>3.33</v>
+        <v>3.2</v>
       </c>
       <c r="F56" t="str">
-        <v>3.33</v>
+        <v>3.2</v>
       </c>
       <c r="G56" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H56" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2025-11-14</v>
+        <v>2025-11-12</v>
       </c>
       <c r="B57" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="C57" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D57" t="str">
-        <v/>
+        <v>08:15-17:15</v>
       </c>
       <c r="E57" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="F57" t="str">
-        <v>2.29</v>
+        <v>6</v>
       </c>
       <c r="G57" t="str">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H57" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <v>2025-11-14</v>
-      </c>
-      <c r="B58" t="str">
-        <v>Morrison (GH), Helen</v>
-      </c>
-      <c r="C58" t="str">
-        <v>Ad-hoc</v>
-      </c>
-      <c r="D58" t="str">
-        <v>07:59-09:00</v>
-      </c>
-      <c r="E58" t="str">
-        <v>0</v>
-      </c>
-      <c r="F58" t="str">
-        <v>0</v>
-      </c>
-      <c r="G58" t="str">
-        <v>0</v>
-      </c>
-      <c r="H58" t="str">
-        <v>Scheduled (no availability record for this day)</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <v>2025-11-14</v>
-      </c>
-      <c r="B59" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
-      </c>
-      <c r="C59" t="str">
-        <v>Holiday</v>
-      </c>
-      <c r="D59" t="str">
-        <v/>
-      </c>
-      <c r="E59" t="str">
-        <v>4.29</v>
-      </c>
-      <c r="F59" t="str">
-        <v>4.29</v>
-      </c>
-      <c r="G59" t="str">
-        <v>0</v>
-      </c>
-      <c r="H59" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <v>2025-11-14</v>
-      </c>
-      <c r="B60" t="str">
-        <v>Romina Ferrara</v>
-      </c>
-      <c r="C60" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D60" t="str">
-        <v>09:15-10:15</v>
-      </c>
-      <c r="E60" t="str">
-        <v>1</v>
-      </c>
-      <c r="F60" t="str">
-        <v>1</v>
-      </c>
-      <c r="G60" t="str">
-        <v>1</v>
-      </c>
-      <c r="H60" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="str">
-        <v>2025-11-14</v>
-      </c>
-      <c r="B61" t="str">
-        <v>Victoria Bateman (GH)</v>
-      </c>
-      <c r="C61" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D61" t="str">
-        <v>08:00-15:30</v>
-      </c>
-      <c r="E61" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="F61" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="G61" t="str">
-        <v>3.2</v>
-      </c>
-      <c r="H61" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="str">
-        <v>2025-11-15</v>
-      </c>
-      <c r="B62" t="str">
-        <v>Dhaval Mithaiwala</v>
-      </c>
-      <c r="C62" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D62" t="str">
-        <v>08:00-21:30</v>
-      </c>
-      <c r="E62" t="str">
-        <v>2.86</v>
-      </c>
-      <c r="F62" t="str">
-        <v>2.86</v>
-      </c>
-      <c r="G62" t="str">
-        <v>2.86</v>
-      </c>
-      <c r="H62" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="str">
-        <v>2025-11-15</v>
-      </c>
-      <c r="B63" t="str">
-        <v>Hartley-Oliver (GH), Ruby</v>
-      </c>
-      <c r="C63" t="str">
-        <v>Ad-hoc</v>
-      </c>
-      <c r="D63" t="str">
-        <v>12:29-15:29</v>
-      </c>
-      <c r="E63" t="str">
-        <v>0</v>
-      </c>
-      <c r="F63" t="str">
-        <v>0</v>
-      </c>
-      <c r="G63" t="str">
-        <v>0</v>
-      </c>
-      <c r="H63" t="str">
-        <v>Scheduled (no availability record for this day)</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="str">
-        <v>2025-11-15</v>
-      </c>
-      <c r="B64" t="str">
-        <v>Helen Morrison (GH)</v>
-      </c>
-      <c r="C64" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D64" t="str">
-        <v>08:00-16:30</v>
-      </c>
-      <c r="E64" t="str">
-        <v>3</v>
-      </c>
-      <c r="F64" t="str">
-        <v>3</v>
-      </c>
-      <c r="G64" t="str">
-        <v>3</v>
-      </c>
-      <c r="H64" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="str">
-        <v>2025-11-15</v>
-      </c>
-      <c r="B65" t="str">
-        <v>Marie Vettrino</v>
-      </c>
-      <c r="C65" t="str">
-        <v>Available</v>
-      </c>
-      <c r="D65" t="str">
-        <v>10:30-11:30; 16:45-17:45</v>
-      </c>
-      <c r="E65" t="str">
-        <v>3</v>
-      </c>
-      <c r="F65" t="str">
-        <v>3</v>
-      </c>
-      <c r="G65" t="str">
-        <v>3</v>
-      </c>
-      <c r="H65" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="str">
-        <v>2025-11-15</v>
-      </c>
-      <c r="B66" t="str">
-        <v>Mikhaila (W) Calder</v>
-      </c>
-      <c r="C66" t="str">
-        <v>Holiday</v>
-      </c>
-      <c r="D66" t="str">
-        <v/>
-      </c>
-      <c r="E66" t="str">
-        <v>2.29</v>
-      </c>
-      <c r="F66" t="str">
-        <v>2.29</v>
-      </c>
-      <c r="G66" t="str">
-        <v>0</v>
-      </c>
-      <c r="H66" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="str">
-        <v>2025-11-15</v>
-      </c>
-      <c r="B67" t="str">
-        <v>Morrison, Anne</v>
-      </c>
-      <c r="C67" t="str">
-        <v>Ad-hoc</v>
-      </c>
-      <c r="D67" t="str">
-        <v>19:00-21:29</v>
-      </c>
-      <c r="E67" t="str">
-        <v>0</v>
-      </c>
-      <c r="F67" t="str">
-        <v>0</v>
-      </c>
-      <c r="G67" t="str">
-        <v>0</v>
-      </c>
-      <c r="H67" t="str">
-        <v>Scheduled (no availability record for this day)</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="str">
-        <v>2025-11-15</v>
-      </c>
-      <c r="B68" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
-      </c>
-      <c r="C68" t="str">
-        <v>Holiday</v>
-      </c>
-      <c r="D68" t="str">
-        <v/>
-      </c>
-      <c r="E68" t="str">
-        <v>4.29</v>
-      </c>
-      <c r="F68" t="str">
-        <v>4.29</v>
-      </c>
-      <c r="G68" t="str">
-        <v>0</v>
-      </c>
-      <c r="H68" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H68"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H57"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4295,27 +3881,27 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Elizabeth Adams</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="B2" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C2" t="str">
         <v>Driver</v>
       </c>
       <c r="D2" t="str">
-        <v>Mrs</v>
+        <v>Miss</v>
       </c>
       <c r="E2" t="str">
         <v>female</v>
       </c>
       <c r="F2" t="str">
-        <v xml:space="preserve">EH21 6NQ  </v>
+        <v xml:space="preserve">FK10 1NH  </v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Victoria Bateman (GH)</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="B3" t="str">
         <v>16</v>
@@ -4324,81 +3910,81 @@
         <v>Driver</v>
       </c>
       <c r="D3" t="str">
-        <v>Mrs</v>
+        <v>Mr</v>
       </c>
       <c r="E3" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="F3" t="str">
-        <v xml:space="preserve">EH23 4NL  </v>
+        <v xml:space="preserve">FK10 3HJ  </v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Amy Brown</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="B4" t="str">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="C4" t="str">
         <v>Driver</v>
       </c>
       <c r="D4" t="str">
-        <v>Miss</v>
+        <v>Mr</v>
       </c>
       <c r="E4" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="F4" t="str">
-        <v xml:space="preserve">EH21 6DQ  </v>
+        <v xml:space="preserve">FK8 1XY   </v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Mikhaila (W) Calder</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="B5" t="str">
         <v>16</v>
       </c>
       <c r="C5" t="str">
-        <v>Walker</v>
+        <v>Driver</v>
       </c>
       <c r="D5" t="str">
-        <v>Miss</v>
+        <v>Mrs</v>
       </c>
       <c r="E5" t="str">
         <v>female</v>
       </c>
       <c r="F5" t="str">
-        <v xml:space="preserve">EH17 7RT  </v>
+        <v xml:space="preserve">FK12 5HG  </v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Romina Ferrara</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="B6" t="str">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="C6" t="str">
         <v>Driver</v>
       </c>
       <c r="D6" t="str">
-        <v>Miss</v>
+        <v>Mr</v>
       </c>
       <c r="E6" t="str">
-        <v>female</v>
+        <v>male</v>
       </c>
       <c r="F6" t="str">
-        <v xml:space="preserve">EH32 9SS  </v>
+        <v xml:space="preserve">FK2 7ER   </v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Eilish McNally</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="B7" t="str">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C7" t="str">
         <v>Driver</v>
@@ -4410,55 +3996,55 @@
         <v>female</v>
       </c>
       <c r="F7" t="str">
-        <v xml:space="preserve">EH34 5HE  </v>
+        <v xml:space="preserve">FK7 7PN   </v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Dhaval Mithaiwala</v>
+        <v>Clare Mackie</v>
       </c>
       <c r="B8" t="str">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="C8" t="str">
         <v>Driver</v>
       </c>
       <c r="D8" t="str">
-        <v>Mr</v>
+        <v>Miss</v>
       </c>
       <c r="E8" t="str">
-        <v>male</v>
+        <v>female</v>
       </c>
       <c r="F8" t="str">
-        <v xml:space="preserve">EH11 3JF  </v>
+        <v xml:space="preserve">FK2 8FD   </v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Anne Morrison</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="B9" t="str">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C9" t="str">
         <v>Driver</v>
       </c>
       <c r="D9" t="str">
-        <v>Mrs</v>
+        <v>Miss</v>
       </c>
       <c r="E9" t="str">
         <v>female</v>
       </c>
       <c r="F9" t="str">
-        <v xml:space="preserve">EH21 7LH  </v>
+        <v xml:space="preserve">FK6 5AE   </v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Helen Morrison (GH)</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="B10" t="str">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="C10" t="str">
         <v>Driver</v>
@@ -4470,32 +4056,32 @@
         <v>female</v>
       </c>
       <c r="F10" t="str">
-        <v xml:space="preserve">EH21 6JY  </v>
+        <v xml:space="preserve">FK8 1RS   </v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Lorraine Parsons</v>
+        <v>Emma (NL) Shawcross</v>
       </c>
       <c r="B11" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C11" t="str">
-        <v>Driver</v>
+        <v>Walker</v>
       </c>
       <c r="D11" t="str">
-        <v>Mrs</v>
+        <v>Miss</v>
       </c>
       <c r="E11" t="str">
         <v>female</v>
       </c>
       <c r="F11" t="str">
-        <v xml:space="preserve">EH22 4FP  </v>
+        <v xml:space="preserve">ML6 0JH   </v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Muhammad Irtaza Tahir (GH)</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="B12" t="str">
         <v>30</v>
@@ -4504,21 +4090,21 @@
         <v>Driver</v>
       </c>
       <c r="D12" t="str">
-        <v>Mr</v>
+        <v>Ms</v>
       </c>
       <c r="E12" t="str">
-        <v>male</v>
+        <v>female</v>
       </c>
       <c r="F12" t="str">
-        <v xml:space="preserve">EH8 7AD   </v>
+        <v xml:space="preserve">FK3 8LP   </v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Marie Vettrino</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="B13" t="str">
-        <v>15</v>
+        <v>37.5</v>
       </c>
       <c r="C13" t="str">
         <v>Driver</v>
@@ -4530,12 +4116,52 @@
         <v>female</v>
       </c>
       <c r="F13" t="str">
-        <v xml:space="preserve">EH32 0DG  </v>
+        <v xml:space="preserve">FK8 2BQ   </v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Rhian Steel</v>
+      </c>
+      <c r="B14" t="str">
+        <v>20</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E14" t="str">
+        <v>female</v>
+      </c>
+      <c r="F14" t="str">
+        <v xml:space="preserve">FK10 2SR  </v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Ziyal Vidler</v>
+      </c>
+      <c r="B15" t="str">
+        <v>20</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Driver</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Miss</v>
+      </c>
+      <c r="E15" t="str">
+        <v>female</v>
+      </c>
+      <c r="F15" t="str">
+        <v xml:space="preserve">FK5 4XD   </v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Checkpoint before assistant change: Update capacity dashboard with new performance data
Updated the capacity_dashboard.xlsx file.

Replit-Commit-Author: Assistant
</commit_message>
<xml_diff>
--- a/capacity_dashboard.xlsx
+++ b/capacity_dashboard.xlsx
@@ -2190,10 +2190,10 @@
         <v>7.5</v>
       </c>
       <c r="F2" t="str">
-        <v>58</v>
+        <v>57.5</v>
       </c>
       <c r="G2" t="str">
-        <v>-18.7</v>
+        <v>-18.2</v>
       </c>
       <c r="H2" t="str">
         <v>Shortage</v>
@@ -2216,10 +2216,10 @@
         <v>11.5</v>
       </c>
       <c r="F3" t="str">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G3" t="str">
-        <v>-3.7</v>
+        <v>-0.7</v>
       </c>
       <c r="H3" t="str">
         <v>Shortage</v>
@@ -2242,10 +2242,10 @@
         <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="G4" t="str">
-        <v>-25.4</v>
+        <v>-18.4</v>
       </c>
       <c r="H4" t="str">
         <v>Shortage</v>
@@ -2346,10 +2346,10 @@
         <v>9.2</v>
       </c>
       <c r="F8" t="str">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G8" t="str">
-        <v>-18.13</v>
+        <v>-15.13</v>
       </c>
       <c r="H8" t="str">
         <v>Shortage</v>
@@ -2364,7 +2364,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H56"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2680,28 +2680,28 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2025-11-11</v>
+        <v>2025-11-13</v>
       </c>
       <c r="B13" t="str">
-        <v>Vidler, Ziyal</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="C13" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D13" t="str">
-        <v>12:29-13:00</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E13" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F13" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="G13" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H13" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -2709,7 +2709,7 @@
         <v>2025-11-13</v>
       </c>
       <c r="B14" t="str">
-        <v>Anisa Naeem</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="C14" t="str">
         <v>Available</v>
@@ -2727,7 +2727,7 @@
         <v>7.5</v>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
     </row>
     <row r="15">
@@ -2735,25 +2735,25 @@
         <v>2025-11-13</v>
       </c>
       <c r="B15" t="str">
-        <v>Barbora Slabochova (GH)</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="C15" t="str">
         <v>Available</v>
       </c>
       <c r="D15" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-22:00</v>
       </c>
       <c r="E15" t="str">
-        <v>7.5</v>
+        <v>9.2</v>
       </c>
       <c r="F15" t="str">
-        <v>7.5</v>
+        <v>9.2</v>
       </c>
       <c r="G15" t="str">
-        <v>7.5</v>
+        <v>9.2</v>
       </c>
       <c r="H15" t="str">
-        <v>Created by new employee process.</v>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -2761,25 +2761,25 @@
         <v>2025-11-13</v>
       </c>
       <c r="B16" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="C16" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D16" t="str">
-        <v>08:00-22:00</v>
+        <v/>
       </c>
       <c r="E16" t="str">
-        <v>9.2</v>
+        <v>4</v>
       </c>
       <c r="F16" t="str">
-        <v>9.2</v>
+        <v>4</v>
       </c>
       <c r="G16" t="str">
-        <v>9.2</v>
+        <v>0</v>
       </c>
       <c r="H16" t="str">
-        <v/>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="17">
@@ -2787,25 +2787,25 @@
         <v>2025-11-13</v>
       </c>
       <c r="B17" t="str">
-        <v>Jamie Lee Kane (GH)</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="C17" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D17" t="str">
-        <v/>
+        <v>10:00-14:30</v>
       </c>
       <c r="E17" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="F17" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="G17" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H17" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -2813,13 +2813,13 @@
         <v>2025-11-13</v>
       </c>
       <c r="B18" t="str">
-        <v>Kristin Earhart</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="C18" t="str">
         <v>Available</v>
       </c>
       <c r="D18" t="str">
-        <v>10:00-14:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E18" t="str">
         <v>3.2</v>
@@ -2839,22 +2839,22 @@
         <v>2025-11-13</v>
       </c>
       <c r="B19" t="str">
-        <v>Paul Chalmers (GH)</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="C19" t="str">
         <v>Available</v>
       </c>
       <c r="D19" t="str">
-        <v>09:15-15:15</v>
+        <v>08:15-17:15</v>
       </c>
       <c r="E19" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="F19" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="G19" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H19" t="str">
         <v/>
@@ -2865,22 +2865,22 @@
         <v>2025-11-13</v>
       </c>
       <c r="B20" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="C20" t="str">
         <v>Available</v>
       </c>
       <c r="D20" t="str">
-        <v>08:15-17:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E20" t="str">
-        <v>6</v>
+        <v>6.67</v>
       </c>
       <c r="F20" t="str">
-        <v>6</v>
+        <v>6.67</v>
       </c>
       <c r="G20" t="str">
-        <v>6</v>
+        <v>6.67</v>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -2888,10 +2888,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2025-11-13</v>
+        <v>2025-11-10</v>
       </c>
       <c r="B21" t="str">
-        <v>Ziyal Vidler</v>
+        <v>Alison Shields (GH)</v>
       </c>
       <c r="C21" t="str">
         <v>Available</v>
@@ -2900,13 +2900,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E21" t="str">
-        <v>6.67</v>
+        <v>7.5</v>
       </c>
       <c r="F21" t="str">
-        <v>6.67</v>
+        <v>7.5</v>
       </c>
       <c r="G21" t="str">
-        <v>6.67</v>
+        <v>7.5</v>
       </c>
       <c r="H21" t="str">
         <v/>
@@ -2917,7 +2917,7 @@
         <v>2025-11-10</v>
       </c>
       <c r="B22" t="str">
-        <v>Alison Shields (GH)</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="C22" t="str">
         <v>Available</v>
@@ -2926,13 +2926,13 @@
         <v>08:00-21:30</v>
       </c>
       <c r="E22" t="str">
-        <v>7.5</v>
+        <v>9.2</v>
       </c>
       <c r="F22" t="str">
-        <v>7.5</v>
+        <v>9.2</v>
       </c>
       <c r="G22" t="str">
-        <v>7.5</v>
+        <v>9.2</v>
       </c>
       <c r="H22" t="str">
         <v/>
@@ -2943,25 +2943,25 @@
         <v>2025-11-10</v>
       </c>
       <c r="B23" t="str">
-        <v>Chiamaka Onweluzo (GH)</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="C23" t="str">
-        <v>Available</v>
+        <v>Partial Availability</v>
       </c>
       <c r="D23" t="str">
-        <v>08:00-21:30</v>
+        <v>08:00-13:00; 17:00-22:00</v>
       </c>
       <c r="E23" t="str">
         <v>9.2</v>
       </c>
       <c r="F23" t="str">
-        <v>9.2</v>
+        <v>5.2</v>
       </c>
       <c r="G23" t="str">
-        <v>9.2</v>
+        <v>5.2</v>
       </c>
       <c r="H23" t="str">
-        <v/>
+        <v>Haseeb is helping out GN</v>
       </c>
     </row>
     <row r="24">
@@ -2969,25 +2969,25 @@
         <v>2025-11-10</v>
       </c>
       <c r="B24" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>John Clarke (GH)</v>
       </c>
       <c r="C24" t="str">
-        <v>Partial Availability</v>
+        <v>Holiday</v>
       </c>
       <c r="D24" t="str">
-        <v>08:00-13:00; 17:00-22:00</v>
+        <v/>
       </c>
       <c r="E24" t="str">
-        <v>9.2</v>
+        <v>7.5</v>
       </c>
       <c r="F24" t="str">
-        <v>5.2</v>
+        <v>7.5</v>
       </c>
       <c r="G24" t="str">
-        <v>5.2</v>
+        <v>0</v>
       </c>
       <c r="H24" t="str">
-        <v>Haseeb is helping out GN</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="25">
@@ -2995,25 +2995,25 @@
         <v>2025-11-10</v>
       </c>
       <c r="B25" t="str">
-        <v>John Clarke (GH)</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="C25" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D25" t="str">
-        <v/>
+        <v>10:00-14:30</v>
       </c>
       <c r="E25" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="F25" t="str">
-        <v>7.5</v>
+        <v>3.2</v>
       </c>
       <c r="G25" t="str">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H25" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -3021,13 +3021,13 @@
         <v>2025-11-10</v>
       </c>
       <c r="B26" t="str">
-        <v>Kristin Earhart</v>
+        <v>Paul Chalmers (GH)</v>
       </c>
       <c r="C26" t="str">
         <v>Available</v>
       </c>
       <c r="D26" t="str">
-        <v>10:00-14:30</v>
+        <v>09:15-15:15</v>
       </c>
       <c r="E26" t="str">
         <v>3.2</v>
@@ -3047,22 +3047,22 @@
         <v>2025-11-10</v>
       </c>
       <c r="B27" t="str">
-        <v>Paul Chalmers (GH)</v>
+        <v>Rhian Steel</v>
       </c>
       <c r="C27" t="str">
         <v>Available</v>
       </c>
       <c r="D27" t="str">
-        <v>09:15-15:15</v>
+        <v>09:15-14:00</v>
       </c>
       <c r="E27" t="str">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="F27" t="str">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="G27" t="str">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="H27" t="str">
         <v/>
@@ -3073,22 +3073,22 @@
         <v>2025-11-10</v>
       </c>
       <c r="B28" t="str">
-        <v>Rhian Steel</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="C28" t="str">
         <v>Available</v>
       </c>
       <c r="D28" t="str">
-        <v>09:15-14:00</v>
+        <v>08:15-21:30</v>
       </c>
       <c r="E28" t="str">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F28" t="str">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G28" t="str">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -3099,51 +3099,51 @@
         <v>2025-11-10</v>
       </c>
       <c r="B29" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Stevenson (GH), Keri</v>
       </c>
       <c r="C29" t="str">
-        <v>Available</v>
+        <v>Ad-hoc</v>
       </c>
       <c r="D29" t="str">
-        <v>08:15-21:30</v>
+        <v>09:15-12:15</v>
       </c>
       <c r="E29" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F29" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G29" t="str">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H29" t="str">
-        <v/>
+        <v>Scheduled (no availability record for this day)</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2025-11-10</v>
+        <v>2025-11-14</v>
       </c>
       <c r="B30" t="str">
-        <v>Stevenson (GH), Keri</v>
+        <v>Anisa Naeem</v>
       </c>
       <c r="C30" t="str">
-        <v>Ad-hoc</v>
+        <v>Available</v>
       </c>
       <c r="D30" t="str">
-        <v>09:15-12:15</v>
+        <v>08:00-21:30</v>
       </c>
       <c r="E30" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F30" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="G30" t="str">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="H30" t="str">
-        <v>Scheduled (no availability record for this day)</v>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -3151,7 +3151,7 @@
         <v>2025-11-14</v>
       </c>
       <c r="B31" t="str">
-        <v>Anisa Naeem</v>
+        <v>Barbora Slabochova (GH)</v>
       </c>
       <c r="C31" t="str">
         <v>Available</v>
@@ -3169,7 +3169,7 @@
         <v>7.5</v>
       </c>
       <c r="H31" t="str">
-        <v/>
+        <v>Created by new employee process.</v>
       </c>
     </row>
     <row r="32">
@@ -3177,25 +3177,25 @@
         <v>2025-11-14</v>
       </c>
       <c r="B32" t="str">
-        <v>Barbora Slabochova (GH)</v>
+        <v>Chiamaka Onweluzo (GH)</v>
       </c>
       <c r="C32" t="str">
-        <v>Available</v>
+        <v>Holiday</v>
       </c>
       <c r="D32" t="str">
-        <v>08:00-21:30</v>
+        <v/>
       </c>
       <c r="E32" t="str">
-        <v>7.5</v>
+        <v>9.2</v>
       </c>
       <c r="F32" t="str">
-        <v>7.5</v>
+        <v>9.2</v>
       </c>
       <c r="G32" t="str">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="H32" t="str">
-        <v>Created by new employee process.</v>
+        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
       </c>
     </row>
     <row r="33">
@@ -3203,13 +3203,13 @@
         <v>2025-11-14</v>
       </c>
       <c r="B33" t="str">
-        <v>Chiamaka Onweluzo (GH)</v>
+        <v>Haseeb Halepota (GH)</v>
       </c>
       <c r="C33" t="str">
-        <v>Holiday</v>
+        <v>Available</v>
       </c>
       <c r="D33" t="str">
-        <v/>
+        <v>08:00-22:00</v>
       </c>
       <c r="E33" t="str">
         <v>9.2</v>
@@ -3218,10 +3218,10 @@
         <v>9.2</v>
       </c>
       <c r="G33" t="str">
-        <v>0</v>
+        <v>9.2</v>
       </c>
       <c r="H33" t="str">
-        <v>Created by new vacation process. [availability ignored due to day-level leave]</v>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -3229,22 +3229,22 @@
         <v>2025-11-14</v>
       </c>
       <c r="B34" t="str">
-        <v>Haseeb Halepota (GH)</v>
+        <v>Jamie Lee Kane (GH)</v>
       </c>
       <c r="C34" t="str">
         <v>Available</v>
       </c>
       <c r="D34" t="str">
-        <v>08:00-22:00</v>
+        <v>16:45-21:30</v>
       </c>
       <c r="E34" t="str">
-        <v>9.2</v>
+        <v>4</v>
       </c>
       <c r="F34" t="str">
-        <v>9.2</v>
+        <v>4</v>
       </c>
       <c r="G34" t="str">
-        <v>9.2</v>
+        <v>4</v>
       </c>
       <c r="H34" t="str">
         <v/>
@@ -3255,22 +3255,22 @@
         <v>2025-11-14</v>
       </c>
       <c r="B35" t="str">
-        <v>Jamie Lee Kane (GH)</v>
+        <v>Kristin Earhart</v>
       </c>
       <c r="C35" t="str">
         <v>Available</v>
       </c>
       <c r="D35" t="str">
-        <v>16:45-21:30</v>
+        <v>10:00-14:30</v>
       </c>
       <c r="E35" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="F35" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="G35" t="str">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="H35" t="str">
         <v/>
@@ -3281,22 +3281,22 @@
         <v>2025-11-14</v>
       </c>
       <c r="B36" t="str">
-        <v>Kristin Earhart</v>
+        <v>Rowan Boyle (GH)</v>
       </c>
       <c r="C36" t="str">
         <v>Available</v>
       </c>
       <c r="D36" t="str">
-        <v>10:00-14:30</v>
+        <v>08:15-17:15</v>
       </c>
       <c r="E36" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="F36" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="G36" t="str">
-        <v>3.2</v>
+        <v>6</v>
       </c>
       <c r="H36" t="str">
         <v/>
@@ -3307,22 +3307,22 @@
         <v>2025-11-14</v>
       </c>
       <c r="B37" t="str">
-        <v>Rowan Boyle (GH)</v>
+        <v>Ziyal Vidler</v>
       </c>
       <c r="C37" t="str">
         <v>Available</v>
       </c>
       <c r="D37" t="str">
-        <v>08:15-17:15</v>
+        <v>08:00-14:00</v>
       </c>
       <c r="E37" t="str">
-        <v>6</v>
+        <v>6.67</v>
       </c>
       <c r="F37" t="str">
-        <v>6</v>
+        <v>6.67</v>
       </c>
       <c r="G37" t="str">
-        <v>6</v>
+        <v>6.67</v>
       </c>
       <c r="H37" t="str">
         <v/>
@@ -3330,25 +3330,25 @@
     </row>
     <row r="38">
   